<commit_message>
got data for 23rd march and got predictions for 24th march
</commit_message>
<xml_diff>
--- a/Probability Project.xlsx
+++ b/Probability Project.xlsx
@@ -12,6 +12,7 @@
     <sheet name="AUTO_20260319" sheetId="7" state="visible" r:id="rId7"/>
     <sheet name="AUTO_20260320" sheetId="8" state="visible" r:id="rId8"/>
     <sheet name="AUTO_20260321" sheetId="9" state="visible" r:id="rId9"/>
+    <sheet name="AUTO_20260323" sheetId="10" state="visible" r:id="rId10"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -2520,6 +2521,1042 @@
 </worksheet>
 </file>
 
+<file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:D51"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="24" t="inlineStr">
+        <is>
+          <t>Date</t>
+        </is>
+      </c>
+      <c r="B1" s="24" t="inlineStr">
+        <is>
+          <t>Rank</t>
+        </is>
+      </c>
+      <c r="C1" s="24" t="inlineStr">
+        <is>
+          <t>Song</t>
+        </is>
+      </c>
+      <c r="D1" s="24" t="inlineStr">
+        <is>
+          <t>Artist</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>2026-03-23</t>
+        </is>
+      </c>
+      <c r="B2" t="n">
+        <v>1</v>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>Bairan</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>Banjaare</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>2026-03-23</t>
+        </is>
+      </c>
+      <c r="B3" t="n">
+        <v>2</v>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>Sheesha - Aakhya Mai Aakh Ghali Jo Bairan</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>Mitta Ror, Swara Verma</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>2026-03-23</t>
+        </is>
+      </c>
+      <c r="B4" t="n">
+        <v>3</v>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>Dhurandhar The Revenge - Aari Aari (From "Dhurandhar The Revenge")</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>Shashwat Sachdev, Bombay Rockers, Irshad Kamil, Khan Saab, Reble, Token, Jasmine Sandlas, Sudhir Yaduvanshi</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>2026-03-23</t>
+        </is>
+      </c>
+      <c r="B5" t="n">
+        <v>4</v>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>Gehra Hua</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>Shashwat Sachdev, Arijit Singh, Irshad Kamil, Armaan Khan</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>2026-03-23</t>
+        </is>
+      </c>
+      <c r="B6" t="n">
+        <v>5</v>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>Jaiye Sajana</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>Shashwat Sachdev, Jasmine Sandlas, Satinder Sartaaj</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>2026-03-23</t>
+        </is>
+      </c>
+      <c r="B7" t="n">
+        <v>6</v>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>Khat</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>Navjot Ahuja</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>2026-03-23</t>
+        </is>
+      </c>
+      <c r="B8" t="n">
+        <v>7</v>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>Dooron Dooron</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>Paresh Pahuja, Shiv Tandan, Meghdeep Bose</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>2026-03-23</t>
+        </is>
+      </c>
+      <c r="B9" t="n">
+        <v>8</v>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>Sahiba</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>Aditya Rikhari</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>2026-03-23</t>
+        </is>
+      </c>
+      <c r="B10" t="n">
+        <v>9</v>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>Sitaare (From "Ikkis")</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>Arijit Singh, White Noise Collectives, Amitabh Bhattacharya</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>2026-03-23</t>
+        </is>
+      </c>
+      <c r="B11" t="n">
+        <v>10</v>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>Jaan Se Guzarte Hain</t>
+        </is>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>Shashwat Sachdev, Khan Saab</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>2026-03-23</t>
+        </is>
+      </c>
+      <c r="B12" t="n">
+        <v>11</v>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>Finding Her</t>
+        </is>
+      </c>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>Kushagra, Bharath, Saaheal</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>2026-03-23</t>
+        </is>
+      </c>
+      <c r="B13" t="n">
+        <v>12</v>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>Samjhawan</t>
+        </is>
+      </c>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t>Jawad Ahmad, Shaarib Toshi, Arijit Singh, Shreya Ghoshal</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>2026-03-23</t>
+        </is>
+      </c>
+      <c r="B14" t="n">
+        <v>13</v>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>Apna Bana Le</t>
+        </is>
+      </c>
+      <c r="D14" t="inlineStr">
+        <is>
+          <t>Sachin-Jigar, Arijit Singh, Amitabh Bhattacharya</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>2026-03-23</t>
+        </is>
+      </c>
+      <c r="B15" t="n">
+        <v>14</v>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>Dhurandhar - Title Track</t>
+        </is>
+      </c>
+      <c r="D15" t="inlineStr">
+        <is>
+          <t>Shashwat Sachdev, Hanumankind, Jasmine Sandlas, Sudhir Yaduvanshi, Charanjit Ahuja, Muhammad Sadiq, Ranjit Kaur, Babu Singh Maan</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>2026-03-23</t>
+        </is>
+      </c>
+      <c r="B16" t="n">
+        <v>15</v>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>Shararat</t>
+        </is>
+      </c>
+      <c r="D16" t="inlineStr">
+        <is>
+          <t>Shashwat Sachdev, Madhubanti Bagchi, Jasmine Sandlas</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>2026-03-23</t>
+        </is>
+      </c>
+      <c r="B17" t="n">
+        <v>16</v>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>Arz Kiya Hai | Coke Studio Bharat</t>
+        </is>
+      </c>
+      <c r="D17" t="inlineStr">
+        <is>
+          <t>Anuv Jain</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>2026-03-23</t>
+        </is>
+      </c>
+      <c r="B18" t="n">
+        <v>17</v>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>For A Reason</t>
+        </is>
+      </c>
+      <c r="D18" t="inlineStr">
+        <is>
+          <t>Karan Aujla, Ikky</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>2026-03-23</t>
+        </is>
+      </c>
+      <c r="B19" t="n">
+        <v>18</v>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>Boyfriend</t>
+        </is>
+      </c>
+      <c r="D19" t="inlineStr">
+        <is>
+          <t>Karan Aujla, Ikky</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>2026-03-23</t>
+        </is>
+      </c>
+      <c r="B20" t="n">
+        <v>19</v>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>Pavazha Malli - From "Think Indie"</t>
+        </is>
+      </c>
+      <c r="D20" t="inlineStr">
+        <is>
+          <t>Sai Abhyankkar, Shruti Haasan, Vivek</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>2026-03-23</t>
+        </is>
+      </c>
+      <c r="B21" t="n">
+        <v>20</v>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>Ishq</t>
+        </is>
+      </c>
+      <c r="D21" t="inlineStr">
+        <is>
+          <t>Faheem Abdullah, Rauhan Malik, Amir Ameer</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>2026-03-23</t>
+        </is>
+      </c>
+      <c r="B22" t="n">
+        <v>21</v>
+      </c>
+      <c r="C22" t="inlineStr">
+        <is>
+          <t>Bairi</t>
+        </is>
+      </c>
+      <c r="D22" t="inlineStr">
+        <is>
+          <t>Virat, Pradeep Solanki, Heena</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>2026-03-23</t>
+        </is>
+      </c>
+      <c r="B23" t="n">
+        <v>22</v>
+      </c>
+      <c r="C23" t="inlineStr">
+        <is>
+          <t>Saiyaara</t>
+        </is>
+      </c>
+      <c r="D23" t="inlineStr">
+        <is>
+          <t>Tanishk Bagchi, Faheem Abdullah, Arslan Nizami, Irshad Kamil</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>2026-03-23</t>
+        </is>
+      </c>
+      <c r="B24" t="n">
+        <v>23</v>
+      </c>
+      <c r="C24" t="inlineStr">
+        <is>
+          <t>Ishqa Ve</t>
+        </is>
+      </c>
+      <c r="D24" t="inlineStr">
+        <is>
+          <t>Zeeshan Ali, Yuvraj Tung, Sandeep Aulakh, Honey Dhillon</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>2026-03-23</t>
+        </is>
+      </c>
+      <c r="B25" t="n">
+        <v>24</v>
+      </c>
+      <c r="C25" t="inlineStr">
+        <is>
+          <t>Mann Mera</t>
+        </is>
+      </c>
+      <c r="D25" t="inlineStr">
+        <is>
+          <t>Gajendra Verma</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>2026-03-23</t>
+        </is>
+      </c>
+      <c r="B26" t="n">
+        <v>25</v>
+      </c>
+      <c r="C26" t="inlineStr">
+        <is>
+          <t>SWIM</t>
+        </is>
+      </c>
+      <c r="D26" t="inlineStr">
+        <is>
+          <t>BTS</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>2026-03-23</t>
+        </is>
+      </c>
+      <c r="B27" t="n">
+        <v>26</v>
+      </c>
+      <c r="C27" t="inlineStr">
+        <is>
+          <t>Raanjhan (From "Do Patti")</t>
+        </is>
+      </c>
+      <c r="D27" t="inlineStr">
+        <is>
+          <t>Sachet-Parampara, Parampara Tandon, Kausar Munir</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>2026-03-23</t>
+        </is>
+      </c>
+      <c r="B28" t="n">
+        <v>27</v>
+      </c>
+      <c r="C28" t="inlineStr">
+        <is>
+          <t>Naal Nachna</t>
+        </is>
+      </c>
+      <c r="D28" t="inlineStr">
+        <is>
+          <t>Shashwat Sachdev, Afsana Khan, Irshad Kamil, Reble</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>2026-03-23</t>
+        </is>
+      </c>
+      <c r="B29" t="n">
+        <v>28</v>
+      </c>
+      <c r="C29" t="inlineStr">
+        <is>
+          <t>Tum Ho Toh (From "Saiyaara")</t>
+        </is>
+      </c>
+      <c r="D29" t="inlineStr">
+        <is>
+          <t>Vishal Mishra, Hansika Pareek, Raj Shekhar</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>2026-03-23</t>
+        </is>
+      </c>
+      <c r="B30" t="n">
+        <v>29</v>
+      </c>
+      <c r="C30" t="inlineStr">
+        <is>
+          <t>Deewaana Deewaana</t>
+        </is>
+      </c>
+      <c r="D30" t="inlineStr">
+        <is>
+          <t>A.R. Rahman, Irshad Kamil</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>2026-03-23</t>
+        </is>
+      </c>
+      <c r="B31" t="n">
+        <v>30</v>
+      </c>
+      <c r="C31" t="inlineStr">
+        <is>
+          <t>Tere Liye</t>
+        </is>
+      </c>
+      <c r="D31" t="inlineStr">
+        <is>
+          <t>Atif Aslam, Shreya Ghoshal, Sachin Gupta, Sameer Anjaan</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="inlineStr">
+        <is>
+          <t>2026-03-23</t>
+        </is>
+      </c>
+      <c r="B32" t="n">
+        <v>31</v>
+      </c>
+      <c r="C32" t="inlineStr">
+        <is>
+          <t>Lutt Le Gaya</t>
+        </is>
+      </c>
+      <c r="D32" t="inlineStr">
+        <is>
+          <t>Shashwat Sachdev, Simran Choudhary</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="inlineStr">
+        <is>
+          <t>2026-03-23</t>
+        </is>
+      </c>
+      <c r="B33" t="n">
+        <v>32</v>
+      </c>
+      <c r="C33" t="inlineStr">
+        <is>
+          <t>Aaya Sher (From "The Paradise") (Telugu)</t>
+        </is>
+      </c>
+      <c r="D33" t="inlineStr">
+        <is>
+          <t>Anirudh Ravichander, Jangi Reddy, Arjun Chandy, Kasarla Shyam</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="inlineStr">
+        <is>
+          <t>2026-03-23</t>
+        </is>
+      </c>
+      <c r="B34" t="n">
+        <v>33</v>
+      </c>
+      <c r="C34" t="inlineStr">
+        <is>
+          <t>Ishq Jalakar - Karvaan</t>
+        </is>
+      </c>
+      <c r="D34" t="inlineStr">
+        <is>
+          <t>Shashwat Sachdev, Shahzad Ali, Subhadeep Das Chowdhury, Armaan Khan, Irshad Kamil, Roshan, Sahir Ludhianvi</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="inlineStr">
+        <is>
+          <t>2026-03-23</t>
+        </is>
+      </c>
+      <c r="B35" t="n">
+        <v>34</v>
+      </c>
+      <c r="C35" t="inlineStr">
+        <is>
+          <t>Agar Tum Saath Ho (From "Tamasha")</t>
+        </is>
+      </c>
+      <c r="D35" t="inlineStr">
+        <is>
+          <t>Alka Yagnik, Arijit Singh</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="inlineStr">
+        <is>
+          <t>2026-03-23</t>
+        </is>
+      </c>
+      <c r="B36" t="n">
+        <v>35</v>
+      </c>
+      <c r="C36" t="inlineStr">
+        <is>
+          <t>Tere Bina</t>
+        </is>
+      </c>
+      <c r="D36" t="inlineStr">
+        <is>
+          <t>A.R. Rahman, Chinmayi, Murtuza Khan, Qadir Khan</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="inlineStr">
+        <is>
+          <t>2026-03-23</t>
+        </is>
+      </c>
+      <c r="B37" t="n">
+        <v>36</v>
+      </c>
+      <c r="C37" t="inlineStr">
+        <is>
+          <t>Haseen</t>
+        </is>
+      </c>
+      <c r="D37" t="inlineStr">
+        <is>
+          <t>Talwiinder, NDS, Rippy Grewal</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="inlineStr">
+        <is>
+          <t>2026-03-23</t>
+        </is>
+      </c>
+      <c r="B38" t="n">
+        <v>37</v>
+      </c>
+      <c r="C38" t="inlineStr">
+        <is>
+          <t>Jo Tum Mere Ho</t>
+        </is>
+      </c>
+      <c r="D38" t="inlineStr">
+        <is>
+          <t>Anuv Jain</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="inlineStr">
+        <is>
+          <t>2026-03-23</t>
+        </is>
+      </c>
+      <c r="B39" t="n">
+        <v>38</v>
+      </c>
+      <c r="C39" t="inlineStr">
+        <is>
+          <t>Darkhaast</t>
+        </is>
+      </c>
+      <c r="D39" t="inlineStr">
+        <is>
+          <t>Mithoon, Arijit Singh, Sunidhi Chauhan, Sayeed Quadri</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" t="inlineStr">
+        <is>
+          <t>2026-03-23</t>
+        </is>
+      </c>
+      <c r="B40" t="n">
+        <v>39</v>
+      </c>
+      <c r="C40" t="inlineStr">
+        <is>
+          <t>Main Aur Tu (From "Dhurandhar The Revenge")</t>
+        </is>
+      </c>
+      <c r="D40" t="inlineStr">
+        <is>
+          <t>Shashwat Sachdev, Jasmine Sandlas, Reble</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" t="inlineStr">
+        <is>
+          <t>2026-03-23</t>
+        </is>
+      </c>
+      <c r="B41" t="n">
+        <v>40</v>
+      </c>
+      <c r="C41" t="inlineStr">
+        <is>
+          <t>Ye Tune Kya Kiya</t>
+        </is>
+      </c>
+      <c r="D41" t="inlineStr">
+        <is>
+          <t>Pritam, Javed Bashir, Rajat Arora</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" t="inlineStr">
+        <is>
+          <t>2026-03-23</t>
+        </is>
+      </c>
+      <c r="B42" t="n">
+        <v>41</v>
+      </c>
+      <c r="C42" t="inlineStr">
+        <is>
+          <t>Barbaad (From "Saiyaara")</t>
+        </is>
+      </c>
+      <c r="D42" t="inlineStr">
+        <is>
+          <t>The Rish, Jubin Nautiyal</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" t="inlineStr">
+        <is>
+          <t>2026-03-23</t>
+        </is>
+      </c>
+      <c r="B43" t="n">
+        <v>42</v>
+      </c>
+      <c r="C43" t="inlineStr">
+        <is>
+          <t>Mutta Kalakki (From "Youth")</t>
+        </is>
+      </c>
+      <c r="D43" t="inlineStr">
+        <is>
+          <t>G. V. Prakash, Ken Karunaas</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" t="inlineStr">
+        <is>
+          <t>2026-03-23</t>
+        </is>
+      </c>
+      <c r="B44" t="n">
+        <v>43</v>
+      </c>
+      <c r="C44" t="inlineStr">
+        <is>
+          <t>Not Guilty</t>
+        </is>
+      </c>
+      <c r="D44" t="inlineStr">
+        <is>
+          <t>Dhanda Nyoliwala</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" t="inlineStr">
+        <is>
+          <t>2026-03-23</t>
+        </is>
+      </c>
+      <c r="B45" t="n">
+        <v>44</v>
+      </c>
+      <c r="C45" t="inlineStr">
+        <is>
+          <t>Run Down The City - Monica</t>
+        </is>
+      </c>
+      <c r="D45" t="inlineStr">
+        <is>
+          <t>Shashwat Sachdev, Reble, Asha Bhosle, R. D. Burman, Majrooh Sultanpuri</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" t="inlineStr">
+        <is>
+          <t>2026-03-23</t>
+        </is>
+      </c>
+      <c r="B46" t="n">
+        <v>45</v>
+      </c>
+      <c r="C46" t="inlineStr">
+        <is>
+          <t>Ehsaas</t>
+        </is>
+      </c>
+      <c r="D46" t="inlineStr">
+        <is>
+          <t>Faheem Abdullah, Duha Shah, Vaibhav Pani, Hyder Dar</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" t="inlineStr">
+        <is>
+          <t>2026-03-23</t>
+        </is>
+      </c>
+      <c r="B47" t="n">
+        <v>46</v>
+      </c>
+      <c r="C47" t="inlineStr">
+        <is>
+          <t>Mast Magan (From "2 States)</t>
+        </is>
+      </c>
+      <c r="D47" t="inlineStr">
+        <is>
+          <t>Arijit Singh, Chinmayi</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" t="inlineStr">
+        <is>
+          <t>2026-03-23</t>
+        </is>
+      </c>
+      <c r="B48" t="n">
+        <v>47</v>
+      </c>
+      <c r="C48" t="inlineStr">
+        <is>
+          <t>Teri Deewani</t>
+        </is>
+      </c>
+      <c r="D48" t="inlineStr">
+        <is>
+          <t>Kailash Kher, Paresh Kamath, Naresh Kamath</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" t="inlineStr">
+        <is>
+          <t>2026-03-23</t>
+        </is>
+      </c>
+      <c r="B49" t="n">
+        <v>48</v>
+      </c>
+      <c r="C49" t="inlineStr">
+        <is>
+          <t>Dealer</t>
+        </is>
+      </c>
+      <c r="D49" t="inlineStr">
+        <is>
+          <t>Diljit Dosanjh, Da Future, Virk Andaaz</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" t="inlineStr">
+        <is>
+          <t>2026-03-23</t>
+        </is>
+      </c>
+      <c r="B50" t="n">
+        <v>49</v>
+      </c>
+      <c r="C50" t="inlineStr">
+        <is>
+          <t>Body to Body</t>
+        </is>
+      </c>
+      <c r="D50" t="inlineStr">
+        <is>
+          <t>BTS</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" t="inlineStr">
+        <is>
+          <t>2026-03-23</t>
+        </is>
+      </c>
+      <c r="B51" t="n">
+        <v>50</v>
+      </c>
+      <c r="C51" t="inlineStr">
+        <is>
+          <t>Humdard (From "Ek Villain")</t>
+        </is>
+      </c>
+      <c r="D51" t="inlineStr">
+        <is>
+          <t>Arijit Singh</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
@@ -9804,1000 +10841,1000 @@
       </c>
     </row>
     <row r="2">
-      <c r="A2" t="inlineStr">
+      <c r="A2" s="0" t="inlineStr">
         <is>
           <t>2026-03-21</t>
         </is>
       </c>
-      <c r="B2" t="n">
+      <c r="B2" s="0" t="n">
         <v>1</v>
       </c>
-      <c r="C2" t="inlineStr">
+      <c r="C2" s="0" t="inlineStr">
         <is>
           <t>Bairan</t>
         </is>
       </c>
-      <c r="D2" t="inlineStr">
+      <c r="D2" s="0" t="inlineStr">
         <is>
           <t>Banjaare</t>
         </is>
       </c>
     </row>
     <row r="3">
-      <c r="A3" t="inlineStr">
+      <c r="A3" s="0" t="inlineStr">
         <is>
           <t>2026-03-21</t>
         </is>
       </c>
-      <c r="B3" t="n">
+      <c r="B3" s="0" t="n">
         <v>2</v>
       </c>
-      <c r="C3" t="inlineStr">
+      <c r="C3" s="0" t="inlineStr">
         <is>
           <t>Sheesha - Aakhya Mai Aakh Ghali Jo Bairan</t>
         </is>
       </c>
-      <c r="D3" t="inlineStr">
+      <c r="D3" s="0" t="inlineStr">
         <is>
           <t>Mitta Ror, Swara Verma</t>
         </is>
       </c>
     </row>
     <row r="4">
-      <c r="A4" t="inlineStr">
+      <c r="A4" s="0" t="inlineStr">
         <is>
           <t>2026-03-21</t>
         </is>
       </c>
-      <c r="B4" t="n">
+      <c r="B4" s="0" t="n">
         <v>3</v>
       </c>
-      <c r="C4" t="inlineStr">
+      <c r="C4" s="0" t="inlineStr">
         <is>
           <t>Gehra Hua</t>
         </is>
       </c>
-      <c r="D4" t="inlineStr">
+      <c r="D4" s="0" t="inlineStr">
         <is>
           <t>Shashwat Sachdev, Arijit Singh, Irshad Kamil, Armaan Khan</t>
         </is>
       </c>
     </row>
     <row r="5">
-      <c r="A5" t="inlineStr">
+      <c r="A5" s="0" t="inlineStr">
         <is>
           <t>2026-03-21</t>
         </is>
       </c>
-      <c r="B5" t="n">
+      <c r="B5" s="0" t="n">
         <v>4</v>
       </c>
-      <c r="C5" t="inlineStr">
+      <c r="C5" s="0" t="inlineStr">
         <is>
           <t>Dhurandhar The Revenge - Aari Aari (From "Dhurandhar The Revenge")</t>
         </is>
       </c>
-      <c r="D5" t="inlineStr">
+      <c r="D5" s="0" t="inlineStr">
         <is>
           <t>Shashwat Sachdev, Bombay Rockers, Irshad Kamil, Khan Saab, Reble, Token, Jasmine Sandlas, Sudhir Yaduvanshi</t>
         </is>
       </c>
     </row>
     <row r="6">
-      <c r="A6" t="inlineStr">
+      <c r="A6" s="0" t="inlineStr">
         <is>
           <t>2026-03-21</t>
         </is>
       </c>
-      <c r="B6" t="n">
+      <c r="B6" s="0" t="n">
         <v>5</v>
       </c>
-      <c r="C6" t="inlineStr">
+      <c r="C6" s="0" t="inlineStr">
         <is>
           <t>Khat</t>
         </is>
       </c>
-      <c r="D6" t="inlineStr">
+      <c r="D6" s="0" t="inlineStr">
         <is>
           <t>Navjot Ahuja</t>
         </is>
       </c>
     </row>
     <row r="7">
-      <c r="A7" t="inlineStr">
+      <c r="A7" s="0" t="inlineStr">
         <is>
           <t>2026-03-21</t>
         </is>
       </c>
-      <c r="B7" t="n">
+      <c r="B7" s="0" t="n">
         <v>6</v>
       </c>
-      <c r="C7" t="inlineStr">
+      <c r="C7" s="0" t="inlineStr">
         <is>
           <t>Dooron Dooron</t>
         </is>
       </c>
-      <c r="D7" t="inlineStr">
+      <c r="D7" s="0" t="inlineStr">
         <is>
           <t>Paresh Pahuja, Shiv Tandan, Meghdeep Bose</t>
         </is>
       </c>
     </row>
     <row r="8">
-      <c r="A8" t="inlineStr">
+      <c r="A8" s="0" t="inlineStr">
         <is>
           <t>2026-03-21</t>
         </is>
       </c>
-      <c r="B8" t="n">
+      <c r="B8" s="0" t="n">
         <v>7</v>
       </c>
-      <c r="C8" t="inlineStr">
+      <c r="C8" s="0" t="inlineStr">
         <is>
           <t>Sahiba</t>
         </is>
       </c>
-      <c r="D8" t="inlineStr">
+      <c r="D8" s="0" t="inlineStr">
         <is>
           <t>Aditya Rikhari</t>
         </is>
       </c>
     </row>
     <row r="9">
-      <c r="A9" t="inlineStr">
+      <c r="A9" s="0" t="inlineStr">
         <is>
           <t>2026-03-21</t>
         </is>
       </c>
-      <c r="B9" t="n">
+      <c r="B9" s="0" t="n">
         <v>8</v>
       </c>
-      <c r="C9" t="inlineStr">
+      <c r="C9" s="0" t="inlineStr">
         <is>
           <t>Sitaare (From "Ikkis")</t>
         </is>
       </c>
-      <c r="D9" t="inlineStr">
+      <c r="D9" s="0" t="inlineStr">
         <is>
           <t>Arijit Singh, White Noise Collectives, Amitabh Bhattacharya</t>
         </is>
       </c>
     </row>
     <row r="10">
-      <c r="A10" t="inlineStr">
+      <c r="A10" s="0" t="inlineStr">
         <is>
           <t>2026-03-21</t>
         </is>
       </c>
-      <c r="B10" t="n">
+      <c r="B10" s="0" t="n">
         <v>9</v>
       </c>
-      <c r="C10" t="inlineStr">
+      <c r="C10" s="0" t="inlineStr">
         <is>
           <t>Samjhawan</t>
         </is>
       </c>
-      <c r="D10" t="inlineStr">
+      <c r="D10" s="0" t="inlineStr">
         <is>
           <t>Jawad Ahmad, Shaarib Toshi, Arijit Singh, Shreya Ghoshal</t>
         </is>
       </c>
     </row>
     <row r="11">
-      <c r="A11" t="inlineStr">
+      <c r="A11" s="0" t="inlineStr">
         <is>
           <t>2026-03-21</t>
         </is>
       </c>
-      <c r="B11" t="n">
+      <c r="B11" s="0" t="n">
         <v>10</v>
       </c>
-      <c r="C11" t="inlineStr">
+      <c r="C11" s="0" t="inlineStr">
         <is>
           <t>Finding Her</t>
         </is>
       </c>
-      <c r="D11" t="inlineStr">
+      <c r="D11" s="0" t="inlineStr">
         <is>
           <t>Kushagra, Bharath, Saaheal</t>
         </is>
       </c>
     </row>
     <row r="12">
-      <c r="A12" t="inlineStr">
+      <c r="A12" s="0" t="inlineStr">
         <is>
           <t>2026-03-21</t>
         </is>
       </c>
-      <c r="B12" t="n">
+      <c r="B12" s="0" t="n">
         <v>11</v>
       </c>
-      <c r="C12" t="inlineStr">
+      <c r="C12" s="0" t="inlineStr">
         <is>
           <t>Apna Bana Le</t>
         </is>
       </c>
-      <c r="D12" t="inlineStr">
+      <c r="D12" s="0" t="inlineStr">
         <is>
           <t>Sachin-Jigar, Arijit Singh, Amitabh Bhattacharya</t>
         </is>
       </c>
     </row>
     <row r="13">
-      <c r="A13" t="inlineStr">
+      <c r="A13" s="0" t="inlineStr">
         <is>
           <t>2026-03-21</t>
         </is>
       </c>
-      <c r="B13" t="n">
+      <c r="B13" s="0" t="n">
         <v>12</v>
       </c>
-      <c r="C13" t="inlineStr">
+      <c r="C13" s="0" t="inlineStr">
         <is>
           <t>Shararat</t>
         </is>
       </c>
-      <c r="D13" t="inlineStr">
+      <c r="D13" s="0" t="inlineStr">
         <is>
           <t>Shashwat Sachdev, Madhubanti Bagchi, Jasmine Sandlas</t>
         </is>
       </c>
     </row>
     <row r="14">
-      <c r="A14" t="inlineStr">
+      <c r="A14" s="0" t="inlineStr">
         <is>
           <t>2026-03-21</t>
         </is>
       </c>
-      <c r="B14" t="n">
+      <c r="B14" s="0" t="n">
         <v>13</v>
       </c>
-      <c r="C14" t="inlineStr">
+      <c r="C14" s="0" t="inlineStr">
         <is>
           <t>Dhurandhar - Title Track</t>
         </is>
       </c>
-      <c r="D14" t="inlineStr">
+      <c r="D14" s="0" t="inlineStr">
         <is>
           <t>Shashwat Sachdev, Hanumankind, Jasmine Sandlas, Sudhir Yaduvanshi, Charanjit Ahuja, Muhammad Sadiq, Ranjit Kaur, Babu Singh Maan</t>
         </is>
       </c>
     </row>
     <row r="15">
-      <c r="A15" t="inlineStr">
+      <c r="A15" s="0" t="inlineStr">
         <is>
           <t>2026-03-21</t>
         </is>
       </c>
-      <c r="B15" t="n">
+      <c r="B15" s="0" t="n">
         <v>14</v>
       </c>
-      <c r="C15" t="inlineStr">
+      <c r="C15" s="0" t="inlineStr">
         <is>
           <t>Arz Kiya Hai | Coke Studio Bharat</t>
         </is>
       </c>
-      <c r="D15" t="inlineStr">
+      <c r="D15" s="0" t="inlineStr">
         <is>
           <t>Anuv Jain</t>
         </is>
       </c>
     </row>
     <row r="16">
-      <c r="A16" t="inlineStr">
+      <c r="A16" s="0" t="inlineStr">
         <is>
           <t>2026-03-21</t>
         </is>
       </c>
-      <c r="B16" t="n">
+      <c r="B16" s="0" t="n">
         <v>15</v>
       </c>
-      <c r="C16" t="inlineStr">
+      <c r="C16" s="0" t="inlineStr">
         <is>
           <t>Pavazha Malli - From "Think Indie"</t>
         </is>
       </c>
-      <c r="D16" t="inlineStr">
+      <c r="D16" s="0" t="inlineStr">
         <is>
           <t>Sai Abhyankkar, Shruti Haasan, Vivek</t>
         </is>
       </c>
     </row>
     <row r="17">
-      <c r="A17" t="inlineStr">
+      <c r="A17" s="0" t="inlineStr">
         <is>
           <t>2026-03-21</t>
         </is>
       </c>
-      <c r="B17" t="n">
+      <c r="B17" s="0" t="n">
         <v>16</v>
       </c>
-      <c r="C17" t="inlineStr">
+      <c r="C17" s="0" t="inlineStr">
         <is>
           <t>For A Reason</t>
         </is>
       </c>
-      <c r="D17" t="inlineStr">
+      <c r="D17" s="0" t="inlineStr">
         <is>
           <t>Karan Aujla, Ikky</t>
         </is>
       </c>
     </row>
     <row r="18">
-      <c r="A18" t="inlineStr">
+      <c r="A18" s="0" t="inlineStr">
         <is>
           <t>2026-03-21</t>
         </is>
       </c>
-      <c r="B18" t="n">
+      <c r="B18" s="0" t="n">
         <v>17</v>
       </c>
-      <c r="C18" t="inlineStr">
+      <c r="C18" s="0" t="inlineStr">
         <is>
           <t>Boyfriend</t>
         </is>
       </c>
-      <c r="D18" t="inlineStr">
+      <c r="D18" s="0" t="inlineStr">
         <is>
           <t>Karan Aujla, Ikky</t>
         </is>
       </c>
     </row>
     <row r="19">
-      <c r="A19" t="inlineStr">
+      <c r="A19" s="0" t="inlineStr">
         <is>
           <t>2026-03-21</t>
         </is>
       </c>
-      <c r="B19" t="n">
+      <c r="B19" s="0" t="n">
         <v>18</v>
       </c>
-      <c r="C19" t="inlineStr">
+      <c r="C19" s="0" t="inlineStr">
         <is>
           <t>Bairi</t>
         </is>
       </c>
-      <c r="D19" t="inlineStr">
+      <c r="D19" s="0" t="inlineStr">
         <is>
           <t>Virat, Pradeep Solanki, Heena</t>
         </is>
       </c>
     </row>
     <row r="20">
-      <c r="A20" t="inlineStr">
+      <c r="A20" s="0" t="inlineStr">
         <is>
           <t>2026-03-21</t>
         </is>
       </c>
-      <c r="B20" t="n">
+      <c r="B20" s="0" t="n">
         <v>19</v>
       </c>
-      <c r="C20" t="inlineStr">
+      <c r="C20" s="0" t="inlineStr">
         <is>
           <t>Ishq</t>
         </is>
       </c>
-      <c r="D20" t="inlineStr">
+      <c r="D20" s="0" t="inlineStr">
         <is>
           <t>Faheem Abdullah, Rauhan Malik, Amir Ameer</t>
         </is>
       </c>
     </row>
     <row r="21">
-      <c r="A21" t="inlineStr">
+      <c r="A21" s="0" t="inlineStr">
         <is>
           <t>2026-03-21</t>
         </is>
       </c>
-      <c r="B21" t="n">
+      <c r="B21" s="0" t="n">
         <v>20</v>
       </c>
-      <c r="C21" t="inlineStr">
+      <c r="C21" s="0" t="inlineStr">
         <is>
           <t>Saiyaara</t>
         </is>
       </c>
-      <c r="D21" t="inlineStr">
+      <c r="D21" s="0" t="inlineStr">
         <is>
           <t>Tanishk Bagchi, Faheem Abdullah, Arslan Nizami, Irshad Kamil</t>
         </is>
       </c>
     </row>
     <row r="22">
-      <c r="A22" t="inlineStr">
+      <c r="A22" s="0" t="inlineStr">
         <is>
           <t>2026-03-21</t>
         </is>
       </c>
-      <c r="B22" t="n">
+      <c r="B22" s="0" t="n">
         <v>21</v>
       </c>
-      <c r="C22" t="inlineStr">
+      <c r="C22" s="0" t="inlineStr">
         <is>
           <t>Ishqa Ve</t>
         </is>
       </c>
-      <c r="D22" t="inlineStr">
+      <c r="D22" s="0" t="inlineStr">
         <is>
           <t>Zeeshan Ali, Yuvraj Tung, Sandeep Aulakh, Honey Dhillon</t>
         </is>
       </c>
     </row>
     <row r="23">
-      <c r="A23" t="inlineStr">
+      <c r="A23" s="0" t="inlineStr">
         <is>
           <t>2026-03-21</t>
         </is>
       </c>
-      <c r="B23" t="n">
+      <c r="B23" s="0" t="n">
         <v>22</v>
       </c>
-      <c r="C23" t="inlineStr">
+      <c r="C23" s="0" t="inlineStr">
         <is>
           <t>SWIM</t>
         </is>
       </c>
-      <c r="D23" t="inlineStr">
+      <c r="D23" s="0" t="inlineStr">
         <is>
           <t>BTS</t>
         </is>
       </c>
     </row>
     <row r="24">
-      <c r="A24" t="inlineStr">
+      <c r="A24" s="0" t="inlineStr">
         <is>
           <t>2026-03-21</t>
         </is>
       </c>
-      <c r="B24" t="n">
+      <c r="B24" s="0" t="n">
         <v>23</v>
       </c>
-      <c r="C24" t="inlineStr">
+      <c r="C24" s="0" t="inlineStr">
         <is>
           <t>Mann Mera</t>
         </is>
       </c>
-      <c r="D24" t="inlineStr">
+      <c r="D24" s="0" t="inlineStr">
         <is>
           <t>Gajendra Verma</t>
         </is>
       </c>
     </row>
     <row r="25">
-      <c r="A25" t="inlineStr">
+      <c r="A25" s="0" t="inlineStr">
         <is>
           <t>2026-03-21</t>
         </is>
       </c>
-      <c r="B25" t="n">
+      <c r="B25" s="0" t="n">
         <v>24</v>
       </c>
-      <c r="C25" t="inlineStr">
+      <c r="C25" s="0" t="inlineStr">
         <is>
           <t>Raanjhan (From "Do Patti")</t>
         </is>
       </c>
-      <c r="D25" t="inlineStr">
+      <c r="D25" s="0" t="inlineStr">
         <is>
           <t>Sachet-Parampara, Parampara Tandon, Kausar Munir</t>
         </is>
       </c>
     </row>
     <row r="26">
-      <c r="A26" t="inlineStr">
+      <c r="A26" s="0" t="inlineStr">
         <is>
           <t>2026-03-21</t>
         </is>
       </c>
-      <c r="B26" t="n">
+      <c r="B26" s="0" t="n">
         <v>25</v>
       </c>
-      <c r="C26" t="inlineStr">
+      <c r="C26" s="0" t="inlineStr">
         <is>
           <t>Deewaana Deewaana</t>
         </is>
       </c>
-      <c r="D26" t="inlineStr">
+      <c r="D26" s="0" t="inlineStr">
         <is>
           <t>A.R. Rahman, Irshad Kamil</t>
         </is>
       </c>
     </row>
     <row r="27">
-      <c r="A27" t="inlineStr">
+      <c r="A27" s="0" t="inlineStr">
         <is>
           <t>2026-03-21</t>
         </is>
       </c>
-      <c r="B27" t="n">
+      <c r="B27" s="0" t="n">
         <v>26</v>
       </c>
-      <c r="C27" t="inlineStr">
+      <c r="C27" s="0" t="inlineStr">
         <is>
           <t>Tere Liye</t>
         </is>
       </c>
-      <c r="D27" t="inlineStr">
+      <c r="D27" s="0" t="inlineStr">
         <is>
           <t>Atif Aslam, Shreya Ghoshal, Sachin Gupta, Sameer Anjaan</t>
         </is>
       </c>
     </row>
     <row r="28">
-      <c r="A28" t="inlineStr">
+      <c r="A28" s="0" t="inlineStr">
         <is>
           <t>2026-03-21</t>
         </is>
       </c>
-      <c r="B28" t="n">
+      <c r="B28" s="0" t="n">
         <v>27</v>
       </c>
-      <c r="C28" t="inlineStr">
+      <c r="C28" s="0" t="inlineStr">
         <is>
           <t>Lutt Le Gaya</t>
         </is>
       </c>
-      <c r="D28" t="inlineStr">
+      <c r="D28" s="0" t="inlineStr">
         <is>
           <t>Shashwat Sachdev, Simran Choudhary</t>
         </is>
       </c>
     </row>
     <row r="29">
-      <c r="A29" t="inlineStr">
+      <c r="A29" s="0" t="inlineStr">
         <is>
           <t>2026-03-21</t>
         </is>
       </c>
-      <c r="B29" t="n">
+      <c r="B29" s="0" t="n">
         <v>28</v>
       </c>
-      <c r="C29" t="inlineStr">
+      <c r="C29" s="0" t="inlineStr">
         <is>
           <t>Jaiye Sajana</t>
         </is>
       </c>
-      <c r="D29" t="inlineStr">
+      <c r="D29" s="0" t="inlineStr">
         <is>
           <t>Shashwat Sachdev, Jasmine Sandlas, Satinder Sartaaj</t>
         </is>
       </c>
     </row>
     <row r="30">
-      <c r="A30" t="inlineStr">
+      <c r="A30" s="0" t="inlineStr">
         <is>
           <t>2026-03-21</t>
         </is>
       </c>
-      <c r="B30" t="n">
+      <c r="B30" s="0" t="n">
         <v>29</v>
       </c>
-      <c r="C30" t="inlineStr">
+      <c r="C30" s="0" t="inlineStr">
         <is>
           <t>Naal Nachna</t>
         </is>
       </c>
-      <c r="D30" t="inlineStr">
+      <c r="D30" s="0" t="inlineStr">
         <is>
           <t>Shashwat Sachdev, Afsana Khan, Irshad Kamil, Reble</t>
         </is>
       </c>
     </row>
     <row r="31">
-      <c r="A31" t="inlineStr">
+      <c r="A31" s="0" t="inlineStr">
         <is>
           <t>2026-03-21</t>
         </is>
       </c>
-      <c r="B31" t="n">
+      <c r="B31" s="0" t="n">
         <v>30</v>
       </c>
-      <c r="C31" t="inlineStr">
+      <c r="C31" s="0" t="inlineStr">
         <is>
           <t>Ishq Jalakar - Karvaan</t>
         </is>
       </c>
-      <c r="D31" t="inlineStr">
+      <c r="D31" s="0" t="inlineStr">
         <is>
           <t>Shashwat Sachdev, Shahzad Ali, Subhadeep Das Chowdhury, Armaan Khan, Irshad Kamil, Roshan, Sahir Ludhianvi</t>
         </is>
       </c>
     </row>
     <row r="32">
-      <c r="A32" t="inlineStr">
+      <c r="A32" s="0" t="inlineStr">
         <is>
           <t>2026-03-21</t>
         </is>
       </c>
-      <c r="B32" t="n">
+      <c r="B32" s="0" t="n">
         <v>31</v>
       </c>
-      <c r="C32" t="inlineStr">
+      <c r="C32" s="0" t="inlineStr">
         <is>
           <t>Agar Tum Saath Ho (From "Tamasha")</t>
         </is>
       </c>
-      <c r="D32" t="inlineStr">
+      <c r="D32" s="0" t="inlineStr">
         <is>
           <t>Alka Yagnik, Arijit Singh</t>
         </is>
       </c>
     </row>
     <row r="33">
-      <c r="A33" t="inlineStr">
+      <c r="A33" s="0" t="inlineStr">
         <is>
           <t>2026-03-21</t>
         </is>
       </c>
-      <c r="B33" t="n">
+      <c r="B33" s="0" t="n">
         <v>32</v>
       </c>
-      <c r="C33" t="inlineStr">
+      <c r="C33" s="0" t="inlineStr">
         <is>
           <t>Tere Bina</t>
         </is>
       </c>
-      <c r="D33" t="inlineStr">
+      <c r="D33" s="0" t="inlineStr">
         <is>
           <t>A.R. Rahman, Chinmayi, Murtuza Khan, Qadir Khan</t>
         </is>
       </c>
     </row>
     <row r="34">
-      <c r="A34" t="inlineStr">
+      <c r="A34" s="0" t="inlineStr">
         <is>
           <t>2026-03-21</t>
         </is>
       </c>
-      <c r="B34" t="n">
+      <c r="B34" s="0" t="n">
         <v>33</v>
       </c>
-      <c r="C34" t="inlineStr">
+      <c r="C34" s="0" t="inlineStr">
         <is>
           <t>Mutta Kalakki (From "Youth")</t>
         </is>
       </c>
-      <c r="D34" t="inlineStr">
+      <c r="D34" s="0" t="inlineStr">
         <is>
           <t>G. V. Prakash, Ken Karunaas</t>
         </is>
       </c>
     </row>
     <row r="35">
-      <c r="A35" t="inlineStr">
+      <c r="A35" s="0" t="inlineStr">
         <is>
           <t>2026-03-21</t>
         </is>
       </c>
-      <c r="B35" t="n">
+      <c r="B35" s="0" t="n">
         <v>34</v>
       </c>
-      <c r="C35" t="inlineStr">
+      <c r="C35" s="0" t="inlineStr">
         <is>
           <t>Jo Tum Mere Ho</t>
         </is>
       </c>
-      <c r="D35" t="inlineStr">
+      <c r="D35" s="0" t="inlineStr">
         <is>
           <t>Anuv Jain</t>
         </is>
       </c>
     </row>
     <row r="36">
-      <c r="A36" t="inlineStr">
+      <c r="A36" s="0" t="inlineStr">
         <is>
           <t>2026-03-21</t>
         </is>
       </c>
-      <c r="B36" t="n">
+      <c r="B36" s="0" t="n">
         <v>35</v>
       </c>
-      <c r="C36" t="inlineStr">
+      <c r="C36" s="0" t="inlineStr">
         <is>
           <t>Haseen</t>
         </is>
       </c>
-      <c r="D36" t="inlineStr">
+      <c r="D36" s="0" t="inlineStr">
         <is>
           <t>Talwiinder, NDS, Rippy Grewal</t>
         </is>
       </c>
     </row>
     <row r="37">
-      <c r="A37" t="inlineStr">
+      <c r="A37" s="0" t="inlineStr">
         <is>
           <t>2026-03-21</t>
         </is>
       </c>
-      <c r="B37" t="n">
+      <c r="B37" s="0" t="n">
         <v>36</v>
       </c>
-      <c r="C37" t="inlineStr">
+      <c r="C37" s="0" t="inlineStr">
         <is>
           <t>Aaya Sher (From "The Paradise") (Telugu)</t>
         </is>
       </c>
-      <c r="D37" t="inlineStr">
+      <c r="D37" s="0" t="inlineStr">
         <is>
           <t>Anirudh Ravichander, Jangi Reddy, Arjun Chandy, Kasarla Shyam</t>
         </is>
       </c>
     </row>
     <row r="38">
-      <c r="A38" t="inlineStr">
+      <c r="A38" s="0" t="inlineStr">
         <is>
           <t>2026-03-21</t>
         </is>
       </c>
-      <c r="B38" t="n">
+      <c r="B38" s="0" t="n">
         <v>37</v>
       </c>
-      <c r="C38" t="inlineStr">
+      <c r="C38" s="0" t="inlineStr">
         <is>
           <t>Jaan Se Guzarte Hain</t>
         </is>
       </c>
-      <c r="D38" t="inlineStr">
+      <c r="D38" s="0" t="inlineStr">
         <is>
           <t>Shashwat Sachdev, Khan Saab</t>
         </is>
       </c>
     </row>
     <row r="39">
-      <c r="A39" t="inlineStr">
+      <c r="A39" s="0" t="inlineStr">
         <is>
           <t>2026-03-21</t>
         </is>
       </c>
-      <c r="B39" t="n">
+      <c r="B39" s="0" t="n">
         <v>38</v>
       </c>
-      <c r="C39" t="inlineStr">
+      <c r="C39" s="0" t="inlineStr">
         <is>
           <t>Tum Ho Toh (From "Saiyaara")</t>
         </is>
       </c>
-      <c r="D39" t="inlineStr">
+      <c r="D39" s="0" t="inlineStr">
         <is>
           <t>Vishal Mishra, Hansika Pareek, Raj Shekhar</t>
         </is>
       </c>
     </row>
     <row r="40">
-      <c r="A40" t="inlineStr">
+      <c r="A40" s="0" t="inlineStr">
         <is>
           <t>2026-03-21</t>
         </is>
       </c>
-      <c r="B40" t="n">
+      <c r="B40" s="0" t="n">
         <v>39</v>
       </c>
-      <c r="C40" t="inlineStr">
+      <c r="C40" s="0" t="inlineStr">
         <is>
           <t>Darkhaast</t>
         </is>
       </c>
-      <c r="D40" t="inlineStr">
+      <c r="D40" s="0" t="inlineStr">
         <is>
           <t>Mithoon, Arijit Singh, Sunidhi Chauhan, Sayeed Quadri</t>
         </is>
       </c>
     </row>
     <row r="41">
-      <c r="A41" t="inlineStr">
+      <c r="A41" s="0" t="inlineStr">
         <is>
           <t>2026-03-21</t>
         </is>
       </c>
-      <c r="B41" t="n">
+      <c r="B41" s="0" t="n">
         <v>40</v>
       </c>
-      <c r="C41" t="inlineStr">
+      <c r="C41" s="0" t="inlineStr">
         <is>
           <t>KALYANI</t>
         </is>
       </c>
-      <c r="D41" t="inlineStr">
+      <c r="D41" s="0" t="inlineStr">
         <is>
           <t>ARJN, KDS, FIFTY4, RONN</t>
         </is>
       </c>
     </row>
     <row r="42">
-      <c r="A42" t="inlineStr">
+      <c r="A42" s="0" t="inlineStr">
         <is>
           <t>2026-03-21</t>
         </is>
       </c>
-      <c r="B42" t="n">
+      <c r="B42" s="0" t="n">
         <v>41</v>
       </c>
-      <c r="C42" t="inlineStr">
+      <c r="C42" s="0" t="inlineStr">
         <is>
           <t>Body to Body</t>
         </is>
       </c>
-      <c r="D42" t="inlineStr">
+      <c r="D42" s="0" t="inlineStr">
         <is>
           <t>BTS</t>
         </is>
       </c>
     </row>
     <row r="43">
-      <c r="A43" t="inlineStr">
+      <c r="A43" s="0" t="inlineStr">
         <is>
           <t>2026-03-21</t>
         </is>
       </c>
-      <c r="B43" t="n">
+      <c r="B43" s="0" t="n">
         <v>42</v>
       </c>
-      <c r="C43" t="inlineStr">
+      <c r="C43" s="0" t="inlineStr">
         <is>
           <t>Jogi</t>
         </is>
       </c>
-      <c r="D43" t="inlineStr">
+      <c r="D43" s="0" t="inlineStr">
         <is>
           <t>thiarajxtt, Bir</t>
         </is>
       </c>
     </row>
     <row r="44">
-      <c r="A44" t="inlineStr">
+      <c r="A44" s="0" t="inlineStr">
         <is>
           <t>2026-03-21</t>
         </is>
       </c>
-      <c r="B44" t="n">
+      <c r="B44" s="0" t="n">
         <v>43</v>
       </c>
-      <c r="C44" t="inlineStr">
+      <c r="C44" s="0" t="inlineStr">
         <is>
           <t>Barbaad (From "Saiyaara")</t>
         </is>
       </c>
-      <c r="D44" t="inlineStr">
+      <c r="D44" s="0" t="inlineStr">
         <is>
           <t>The Rish, Jubin Nautiyal</t>
         </is>
       </c>
     </row>
     <row r="45">
-      <c r="A45" t="inlineStr">
+      <c r="A45" s="0" t="inlineStr">
         <is>
           <t>2026-03-21</t>
         </is>
       </c>
-      <c r="B45" t="n">
+      <c r="B45" s="0" t="n">
         <v>44</v>
       </c>
-      <c r="C45" t="inlineStr">
+      <c r="C45" s="0" t="inlineStr">
         <is>
           <t>Not Guilty</t>
         </is>
       </c>
-      <c r="D45" t="inlineStr">
+      <c r="D45" s="0" t="inlineStr">
         <is>
           <t>Dhanda Nyoliwala</t>
         </is>
       </c>
     </row>
     <row r="46">
-      <c r="A46" t="inlineStr">
+      <c r="A46" s="0" t="inlineStr">
         <is>
           <t>2026-03-21</t>
         </is>
       </c>
-      <c r="B46" t="n">
+      <c r="B46" s="0" t="n">
         <v>45</v>
       </c>
-      <c r="C46" t="inlineStr">
+      <c r="C46" s="0" t="inlineStr">
         <is>
           <t>Ye Tune Kya Kiya</t>
         </is>
       </c>
-      <c r="D46" t="inlineStr">
+      <c r="D46" s="0" t="inlineStr">
         <is>
           <t>Pritam, Javed Bashir, Rajat Arora</t>
         </is>
       </c>
     </row>
     <row r="47">
-      <c r="A47" t="inlineStr">
+      <c r="A47" s="0" t="inlineStr">
         <is>
           <t>2026-03-21</t>
         </is>
       </c>
-      <c r="B47" t="n">
+      <c r="B47" s="0" t="n">
         <v>46</v>
       </c>
-      <c r="C47" t="inlineStr">
+      <c r="C47" s="0" t="inlineStr">
         <is>
           <t>Oorum Blood</t>
         </is>
       </c>
-      <c r="D47" t="inlineStr">
+      <c r="D47" s="0" t="inlineStr">
         <is>
           <t>Sai Abhyankkar, Paal Dabba, Bhumi, Deepthi Suresh</t>
         </is>
       </c>
     </row>
     <row r="48">
-      <c r="A48" t="inlineStr">
+      <c r="A48" s="0" t="inlineStr">
         <is>
           <t>2026-03-21</t>
         </is>
       </c>
-      <c r="B48" t="n">
+      <c r="B48" s="0" t="n">
         <v>47</v>
       </c>
-      <c r="C48" t="inlineStr">
+      <c r="C48" s="0" t="inlineStr">
         <is>
           <t>Mast Magan (From "2 States)</t>
         </is>
       </c>
-      <c r="D48" t="inlineStr">
+      <c r="D48" s="0" t="inlineStr">
         <is>
           <t>Arijit Singh, Chinmayi</t>
         </is>
       </c>
     </row>
     <row r="49">
-      <c r="A49" t="inlineStr">
+      <c r="A49" s="0" t="inlineStr">
         <is>
           <t>2026-03-21</t>
         </is>
       </c>
-      <c r="B49" t="n">
+      <c r="B49" s="0" t="n">
         <v>48</v>
       </c>
-      <c r="C49" t="inlineStr">
+      <c r="C49" s="0" t="inlineStr">
         <is>
           <t>Zaalima</t>
         </is>
       </c>
-      <c r="D49" t="inlineStr">
+      <c r="D49" s="0" t="inlineStr">
         <is>
           <t>Arijit Singh, Harshdeep Kaur</t>
         </is>
       </c>
     </row>
     <row r="50">
-      <c r="A50" t="inlineStr">
+      <c r="A50" s="0" t="inlineStr">
         <is>
           <t>2026-03-21</t>
         </is>
       </c>
-      <c r="B50" t="n">
+      <c r="B50" s="0" t="n">
         <v>49</v>
       </c>
-      <c r="C50" t="inlineStr">
+      <c r="C50" s="0" t="inlineStr">
         <is>
           <t>Ehsaas</t>
         </is>
       </c>
-      <c r="D50" t="inlineStr">
+      <c r="D50" s="0" t="inlineStr">
         <is>
           <t>Faheem Abdullah, Duha Shah, Vaibhav Pani, Hyder Dar</t>
         </is>
       </c>
     </row>
     <row r="51">
-      <c r="A51" t="inlineStr">
+      <c r="A51" s="0" t="inlineStr">
         <is>
           <t>2026-03-21</t>
         </is>
       </c>
-      <c r="B51" t="n">
+      <c r="B51" s="0" t="n">
         <v>50</v>
       </c>
-      <c r="C51" t="inlineStr">
+      <c r="C51" s="0" t="inlineStr">
         <is>
           <t>Teri Deewani</t>
         </is>
       </c>
-      <c r="D51" t="inlineStr">
+      <c r="D51" s="0" t="inlineStr">
         <is>
           <t>Kailash Kher, Paresh Kamath, Naresh Kamath</t>
         </is>

</xml_diff>

<commit_message>
got data for 24th , got predictions for 25th
</commit_message>
<xml_diff>
--- a/Probability Project.xlsx
+++ b/Probability Project.xlsx
@@ -13,6 +13,7 @@
     <sheet name="AUTO_20260320" sheetId="8" state="visible" r:id="rId8"/>
     <sheet name="AUTO_20260321" sheetId="9" state="visible" r:id="rId9"/>
     <sheet name="AUTO_20260323" sheetId="10" state="visible" r:id="rId10"/>
+    <sheet name="AUTO_20260324" sheetId="11" state="visible" r:id="rId11"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -2553,9 +2554,1045 @@
       </c>
     </row>
     <row r="2">
+      <c r="A2" s="0" t="inlineStr">
+        <is>
+          <t>2026-03-23</t>
+        </is>
+      </c>
+      <c r="B2" s="0" t="n">
+        <v>1</v>
+      </c>
+      <c r="C2" s="0" t="inlineStr">
+        <is>
+          <t>Bairan</t>
+        </is>
+      </c>
+      <c r="D2" s="0" t="inlineStr">
+        <is>
+          <t>Banjaare</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="0" t="inlineStr">
+        <is>
+          <t>2026-03-23</t>
+        </is>
+      </c>
+      <c r="B3" s="0" t="n">
+        <v>2</v>
+      </c>
+      <c r="C3" s="0" t="inlineStr">
+        <is>
+          <t>Sheesha - Aakhya Mai Aakh Ghali Jo Bairan</t>
+        </is>
+      </c>
+      <c r="D3" s="0" t="inlineStr">
+        <is>
+          <t>Mitta Ror, Swara Verma</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="0" t="inlineStr">
+        <is>
+          <t>2026-03-23</t>
+        </is>
+      </c>
+      <c r="B4" s="0" t="n">
+        <v>3</v>
+      </c>
+      <c r="C4" s="0" t="inlineStr">
+        <is>
+          <t>Dhurandhar The Revenge - Aari Aari (From "Dhurandhar The Revenge")</t>
+        </is>
+      </c>
+      <c r="D4" s="0" t="inlineStr">
+        <is>
+          <t>Shashwat Sachdev, Bombay Rockers, Irshad Kamil, Khan Saab, Reble, Token, Jasmine Sandlas, Sudhir Yaduvanshi</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="0" t="inlineStr">
+        <is>
+          <t>2026-03-23</t>
+        </is>
+      </c>
+      <c r="B5" s="0" t="n">
+        <v>4</v>
+      </c>
+      <c r="C5" s="0" t="inlineStr">
+        <is>
+          <t>Gehra Hua</t>
+        </is>
+      </c>
+      <c r="D5" s="0" t="inlineStr">
+        <is>
+          <t>Shashwat Sachdev, Arijit Singh, Irshad Kamil, Armaan Khan</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="0" t="inlineStr">
+        <is>
+          <t>2026-03-23</t>
+        </is>
+      </c>
+      <c r="B6" s="0" t="n">
+        <v>5</v>
+      </c>
+      <c r="C6" s="0" t="inlineStr">
+        <is>
+          <t>Jaiye Sajana</t>
+        </is>
+      </c>
+      <c r="D6" s="0" t="inlineStr">
+        <is>
+          <t>Shashwat Sachdev, Jasmine Sandlas, Satinder Sartaaj</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="0" t="inlineStr">
+        <is>
+          <t>2026-03-23</t>
+        </is>
+      </c>
+      <c r="B7" s="0" t="n">
+        <v>6</v>
+      </c>
+      <c r="C7" s="0" t="inlineStr">
+        <is>
+          <t>Khat</t>
+        </is>
+      </c>
+      <c r="D7" s="0" t="inlineStr">
+        <is>
+          <t>Navjot Ahuja</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="0" t="inlineStr">
+        <is>
+          <t>2026-03-23</t>
+        </is>
+      </c>
+      <c r="B8" s="0" t="n">
+        <v>7</v>
+      </c>
+      <c r="C8" s="0" t="inlineStr">
+        <is>
+          <t>Dooron Dooron</t>
+        </is>
+      </c>
+      <c r="D8" s="0" t="inlineStr">
+        <is>
+          <t>Paresh Pahuja, Shiv Tandan, Meghdeep Bose</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="0" t="inlineStr">
+        <is>
+          <t>2026-03-23</t>
+        </is>
+      </c>
+      <c r="B9" s="0" t="n">
+        <v>8</v>
+      </c>
+      <c r="C9" s="0" t="inlineStr">
+        <is>
+          <t>Sahiba</t>
+        </is>
+      </c>
+      <c r="D9" s="0" t="inlineStr">
+        <is>
+          <t>Aditya Rikhari</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="0" t="inlineStr">
+        <is>
+          <t>2026-03-23</t>
+        </is>
+      </c>
+      <c r="B10" s="0" t="n">
+        <v>9</v>
+      </c>
+      <c r="C10" s="0" t="inlineStr">
+        <is>
+          <t>Sitaare (From "Ikkis")</t>
+        </is>
+      </c>
+      <c r="D10" s="0" t="inlineStr">
+        <is>
+          <t>Arijit Singh, White Noise Collectives, Amitabh Bhattacharya</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="0" t="inlineStr">
+        <is>
+          <t>2026-03-23</t>
+        </is>
+      </c>
+      <c r="B11" s="0" t="n">
+        <v>10</v>
+      </c>
+      <c r="C11" s="0" t="inlineStr">
+        <is>
+          <t>Jaan Se Guzarte Hain</t>
+        </is>
+      </c>
+      <c r="D11" s="0" t="inlineStr">
+        <is>
+          <t>Shashwat Sachdev, Khan Saab</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="0" t="inlineStr">
+        <is>
+          <t>2026-03-23</t>
+        </is>
+      </c>
+      <c r="B12" s="0" t="n">
+        <v>11</v>
+      </c>
+      <c r="C12" s="0" t="inlineStr">
+        <is>
+          <t>Finding Her</t>
+        </is>
+      </c>
+      <c r="D12" s="0" t="inlineStr">
+        <is>
+          <t>Kushagra, Bharath, Saaheal</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="0" t="inlineStr">
+        <is>
+          <t>2026-03-23</t>
+        </is>
+      </c>
+      <c r="B13" s="0" t="n">
+        <v>12</v>
+      </c>
+      <c r="C13" s="0" t="inlineStr">
+        <is>
+          <t>Samjhawan</t>
+        </is>
+      </c>
+      <c r="D13" s="0" t="inlineStr">
+        <is>
+          <t>Jawad Ahmad, Shaarib Toshi, Arijit Singh, Shreya Ghoshal</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="0" t="inlineStr">
+        <is>
+          <t>2026-03-23</t>
+        </is>
+      </c>
+      <c r="B14" s="0" t="n">
+        <v>13</v>
+      </c>
+      <c r="C14" s="0" t="inlineStr">
+        <is>
+          <t>Apna Bana Le</t>
+        </is>
+      </c>
+      <c r="D14" s="0" t="inlineStr">
+        <is>
+          <t>Sachin-Jigar, Arijit Singh, Amitabh Bhattacharya</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="0" t="inlineStr">
+        <is>
+          <t>2026-03-23</t>
+        </is>
+      </c>
+      <c r="B15" s="0" t="n">
+        <v>14</v>
+      </c>
+      <c r="C15" s="0" t="inlineStr">
+        <is>
+          <t>Dhurandhar - Title Track</t>
+        </is>
+      </c>
+      <c r="D15" s="0" t="inlineStr">
+        <is>
+          <t>Shashwat Sachdev, Hanumankind, Jasmine Sandlas, Sudhir Yaduvanshi, Charanjit Ahuja, Muhammad Sadiq, Ranjit Kaur, Babu Singh Maan</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="0" t="inlineStr">
+        <is>
+          <t>2026-03-23</t>
+        </is>
+      </c>
+      <c r="B16" s="0" t="n">
+        <v>15</v>
+      </c>
+      <c r="C16" s="0" t="inlineStr">
+        <is>
+          <t>Shararat</t>
+        </is>
+      </c>
+      <c r="D16" s="0" t="inlineStr">
+        <is>
+          <t>Shashwat Sachdev, Madhubanti Bagchi, Jasmine Sandlas</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="0" t="inlineStr">
+        <is>
+          <t>2026-03-23</t>
+        </is>
+      </c>
+      <c r="B17" s="0" t="n">
+        <v>16</v>
+      </c>
+      <c r="C17" s="0" t="inlineStr">
+        <is>
+          <t>Arz Kiya Hai | Coke Studio Bharat</t>
+        </is>
+      </c>
+      <c r="D17" s="0" t="inlineStr">
+        <is>
+          <t>Anuv Jain</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="0" t="inlineStr">
+        <is>
+          <t>2026-03-23</t>
+        </is>
+      </c>
+      <c r="B18" s="0" t="n">
+        <v>17</v>
+      </c>
+      <c r="C18" s="0" t="inlineStr">
+        <is>
+          <t>For A Reason</t>
+        </is>
+      </c>
+      <c r="D18" s="0" t="inlineStr">
+        <is>
+          <t>Karan Aujla, Ikky</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="0" t="inlineStr">
+        <is>
+          <t>2026-03-23</t>
+        </is>
+      </c>
+      <c r="B19" s="0" t="n">
+        <v>18</v>
+      </c>
+      <c r="C19" s="0" t="inlineStr">
+        <is>
+          <t>Boyfriend</t>
+        </is>
+      </c>
+      <c r="D19" s="0" t="inlineStr">
+        <is>
+          <t>Karan Aujla, Ikky</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="0" t="inlineStr">
+        <is>
+          <t>2026-03-23</t>
+        </is>
+      </c>
+      <c r="B20" s="0" t="n">
+        <v>19</v>
+      </c>
+      <c r="C20" s="0" t="inlineStr">
+        <is>
+          <t>Pavazha Malli - From "Think Indie"</t>
+        </is>
+      </c>
+      <c r="D20" s="0" t="inlineStr">
+        <is>
+          <t>Sai Abhyankkar, Shruti Haasan, Vivek</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="0" t="inlineStr">
+        <is>
+          <t>2026-03-23</t>
+        </is>
+      </c>
+      <c r="B21" s="0" t="n">
+        <v>20</v>
+      </c>
+      <c r="C21" s="0" t="inlineStr">
+        <is>
+          <t>Ishq</t>
+        </is>
+      </c>
+      <c r="D21" s="0" t="inlineStr">
+        <is>
+          <t>Faheem Abdullah, Rauhan Malik, Amir Ameer</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="0" t="inlineStr">
+        <is>
+          <t>2026-03-23</t>
+        </is>
+      </c>
+      <c r="B22" s="0" t="n">
+        <v>21</v>
+      </c>
+      <c r="C22" s="0" t="inlineStr">
+        <is>
+          <t>Bairi</t>
+        </is>
+      </c>
+      <c r="D22" s="0" t="inlineStr">
+        <is>
+          <t>Virat, Pradeep Solanki, Heena</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="0" t="inlineStr">
+        <is>
+          <t>2026-03-23</t>
+        </is>
+      </c>
+      <c r="B23" s="0" t="n">
+        <v>22</v>
+      </c>
+      <c r="C23" s="0" t="inlineStr">
+        <is>
+          <t>Saiyaara</t>
+        </is>
+      </c>
+      <c r="D23" s="0" t="inlineStr">
+        <is>
+          <t>Tanishk Bagchi, Faheem Abdullah, Arslan Nizami, Irshad Kamil</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="0" t="inlineStr">
+        <is>
+          <t>2026-03-23</t>
+        </is>
+      </c>
+      <c r="B24" s="0" t="n">
+        <v>23</v>
+      </c>
+      <c r="C24" s="0" t="inlineStr">
+        <is>
+          <t>Ishqa Ve</t>
+        </is>
+      </c>
+      <c r="D24" s="0" t="inlineStr">
+        <is>
+          <t>Zeeshan Ali, Yuvraj Tung, Sandeep Aulakh, Honey Dhillon</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="0" t="inlineStr">
+        <is>
+          <t>2026-03-23</t>
+        </is>
+      </c>
+      <c r="B25" s="0" t="n">
+        <v>24</v>
+      </c>
+      <c r="C25" s="0" t="inlineStr">
+        <is>
+          <t>Mann Mera</t>
+        </is>
+      </c>
+      <c r="D25" s="0" t="inlineStr">
+        <is>
+          <t>Gajendra Verma</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="0" t="inlineStr">
+        <is>
+          <t>2026-03-23</t>
+        </is>
+      </c>
+      <c r="B26" s="0" t="n">
+        <v>25</v>
+      </c>
+      <c r="C26" s="0" t="inlineStr">
+        <is>
+          <t>SWIM</t>
+        </is>
+      </c>
+      <c r="D26" s="0" t="inlineStr">
+        <is>
+          <t>BTS</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="0" t="inlineStr">
+        <is>
+          <t>2026-03-23</t>
+        </is>
+      </c>
+      <c r="B27" s="0" t="n">
+        <v>26</v>
+      </c>
+      <c r="C27" s="0" t="inlineStr">
+        <is>
+          <t>Raanjhan (From "Do Patti")</t>
+        </is>
+      </c>
+      <c r="D27" s="0" t="inlineStr">
+        <is>
+          <t>Sachet-Parampara, Parampara Tandon, Kausar Munir</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="0" t="inlineStr">
+        <is>
+          <t>2026-03-23</t>
+        </is>
+      </c>
+      <c r="B28" s="0" t="n">
+        <v>27</v>
+      </c>
+      <c r="C28" s="0" t="inlineStr">
+        <is>
+          <t>Naal Nachna</t>
+        </is>
+      </c>
+      <c r="D28" s="0" t="inlineStr">
+        <is>
+          <t>Shashwat Sachdev, Afsana Khan, Irshad Kamil, Reble</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="0" t="inlineStr">
+        <is>
+          <t>2026-03-23</t>
+        </is>
+      </c>
+      <c r="B29" s="0" t="n">
+        <v>28</v>
+      </c>
+      <c r="C29" s="0" t="inlineStr">
+        <is>
+          <t>Tum Ho Toh (From "Saiyaara")</t>
+        </is>
+      </c>
+      <c r="D29" s="0" t="inlineStr">
+        <is>
+          <t>Vishal Mishra, Hansika Pareek, Raj Shekhar</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="0" t="inlineStr">
+        <is>
+          <t>2026-03-23</t>
+        </is>
+      </c>
+      <c r="B30" s="0" t="n">
+        <v>29</v>
+      </c>
+      <c r="C30" s="0" t="inlineStr">
+        <is>
+          <t>Deewaana Deewaana</t>
+        </is>
+      </c>
+      <c r="D30" s="0" t="inlineStr">
+        <is>
+          <t>A.R. Rahman, Irshad Kamil</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="0" t="inlineStr">
+        <is>
+          <t>2026-03-23</t>
+        </is>
+      </c>
+      <c r="B31" s="0" t="n">
+        <v>30</v>
+      </c>
+      <c r="C31" s="0" t="inlineStr">
+        <is>
+          <t>Tere Liye</t>
+        </is>
+      </c>
+      <c r="D31" s="0" t="inlineStr">
+        <is>
+          <t>Atif Aslam, Shreya Ghoshal, Sachin Gupta, Sameer Anjaan</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="0" t="inlineStr">
+        <is>
+          <t>2026-03-23</t>
+        </is>
+      </c>
+      <c r="B32" s="0" t="n">
+        <v>31</v>
+      </c>
+      <c r="C32" s="0" t="inlineStr">
+        <is>
+          <t>Lutt Le Gaya</t>
+        </is>
+      </c>
+      <c r="D32" s="0" t="inlineStr">
+        <is>
+          <t>Shashwat Sachdev, Simran Choudhary</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="0" t="inlineStr">
+        <is>
+          <t>2026-03-23</t>
+        </is>
+      </c>
+      <c r="B33" s="0" t="n">
+        <v>32</v>
+      </c>
+      <c r="C33" s="0" t="inlineStr">
+        <is>
+          <t>Aaya Sher (From "The Paradise") (Telugu)</t>
+        </is>
+      </c>
+      <c r="D33" s="0" t="inlineStr">
+        <is>
+          <t>Anirudh Ravichander, Jangi Reddy, Arjun Chandy, Kasarla Shyam</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="0" t="inlineStr">
+        <is>
+          <t>2026-03-23</t>
+        </is>
+      </c>
+      <c r="B34" s="0" t="n">
+        <v>33</v>
+      </c>
+      <c r="C34" s="0" t="inlineStr">
+        <is>
+          <t>Ishq Jalakar - Karvaan</t>
+        </is>
+      </c>
+      <c r="D34" s="0" t="inlineStr">
+        <is>
+          <t>Shashwat Sachdev, Shahzad Ali, Subhadeep Das Chowdhury, Armaan Khan, Irshad Kamil, Roshan, Sahir Ludhianvi</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="0" t="inlineStr">
+        <is>
+          <t>2026-03-23</t>
+        </is>
+      </c>
+      <c r="B35" s="0" t="n">
+        <v>34</v>
+      </c>
+      <c r="C35" s="0" t="inlineStr">
+        <is>
+          <t>Agar Tum Saath Ho (From "Tamasha")</t>
+        </is>
+      </c>
+      <c r="D35" s="0" t="inlineStr">
+        <is>
+          <t>Alka Yagnik, Arijit Singh</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="0" t="inlineStr">
+        <is>
+          <t>2026-03-23</t>
+        </is>
+      </c>
+      <c r="B36" s="0" t="n">
+        <v>35</v>
+      </c>
+      <c r="C36" s="0" t="inlineStr">
+        <is>
+          <t>Tere Bina</t>
+        </is>
+      </c>
+      <c r="D36" s="0" t="inlineStr">
+        <is>
+          <t>A.R. Rahman, Chinmayi, Murtuza Khan, Qadir Khan</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="0" t="inlineStr">
+        <is>
+          <t>2026-03-23</t>
+        </is>
+      </c>
+      <c r="B37" s="0" t="n">
+        <v>36</v>
+      </c>
+      <c r="C37" s="0" t="inlineStr">
+        <is>
+          <t>Haseen</t>
+        </is>
+      </c>
+      <c r="D37" s="0" t="inlineStr">
+        <is>
+          <t>Talwiinder, NDS, Rippy Grewal</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="0" t="inlineStr">
+        <is>
+          <t>2026-03-23</t>
+        </is>
+      </c>
+      <c r="B38" s="0" t="n">
+        <v>37</v>
+      </c>
+      <c r="C38" s="0" t="inlineStr">
+        <is>
+          <t>Jo Tum Mere Ho</t>
+        </is>
+      </c>
+      <c r="D38" s="0" t="inlineStr">
+        <is>
+          <t>Anuv Jain</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="0" t="inlineStr">
+        <is>
+          <t>2026-03-23</t>
+        </is>
+      </c>
+      <c r="B39" s="0" t="n">
+        <v>38</v>
+      </c>
+      <c r="C39" s="0" t="inlineStr">
+        <is>
+          <t>Darkhaast</t>
+        </is>
+      </c>
+      <c r="D39" s="0" t="inlineStr">
+        <is>
+          <t>Mithoon, Arijit Singh, Sunidhi Chauhan, Sayeed Quadri</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="0" t="inlineStr">
+        <is>
+          <t>2026-03-23</t>
+        </is>
+      </c>
+      <c r="B40" s="0" t="n">
+        <v>39</v>
+      </c>
+      <c r="C40" s="0" t="inlineStr">
+        <is>
+          <t>Main Aur Tu (From "Dhurandhar The Revenge")</t>
+        </is>
+      </c>
+      <c r="D40" s="0" t="inlineStr">
+        <is>
+          <t>Shashwat Sachdev, Jasmine Sandlas, Reble</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" s="0" t="inlineStr">
+        <is>
+          <t>2026-03-23</t>
+        </is>
+      </c>
+      <c r="B41" s="0" t="n">
+        <v>40</v>
+      </c>
+      <c r="C41" s="0" t="inlineStr">
+        <is>
+          <t>Ye Tune Kya Kiya</t>
+        </is>
+      </c>
+      <c r="D41" s="0" t="inlineStr">
+        <is>
+          <t>Pritam, Javed Bashir, Rajat Arora</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" s="0" t="inlineStr">
+        <is>
+          <t>2026-03-23</t>
+        </is>
+      </c>
+      <c r="B42" s="0" t="n">
+        <v>41</v>
+      </c>
+      <c r="C42" s="0" t="inlineStr">
+        <is>
+          <t>Barbaad (From "Saiyaara")</t>
+        </is>
+      </c>
+      <c r="D42" s="0" t="inlineStr">
+        <is>
+          <t>The Rish, Jubin Nautiyal</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" s="0" t="inlineStr">
+        <is>
+          <t>2026-03-23</t>
+        </is>
+      </c>
+      <c r="B43" s="0" t="n">
+        <v>42</v>
+      </c>
+      <c r="C43" s="0" t="inlineStr">
+        <is>
+          <t>Mutta Kalakki (From "Youth")</t>
+        </is>
+      </c>
+      <c r="D43" s="0" t="inlineStr">
+        <is>
+          <t>G. V. Prakash, Ken Karunaas</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" s="0" t="inlineStr">
+        <is>
+          <t>2026-03-23</t>
+        </is>
+      </c>
+      <c r="B44" s="0" t="n">
+        <v>43</v>
+      </c>
+      <c r="C44" s="0" t="inlineStr">
+        <is>
+          <t>Not Guilty</t>
+        </is>
+      </c>
+      <c r="D44" s="0" t="inlineStr">
+        <is>
+          <t>Dhanda Nyoliwala</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" s="0" t="inlineStr">
+        <is>
+          <t>2026-03-23</t>
+        </is>
+      </c>
+      <c r="B45" s="0" t="n">
+        <v>44</v>
+      </c>
+      <c r="C45" s="0" t="inlineStr">
+        <is>
+          <t>Run Down The City - Monica</t>
+        </is>
+      </c>
+      <c r="D45" s="0" t="inlineStr">
+        <is>
+          <t>Shashwat Sachdev, Reble, Asha Bhosle, R. D. Burman, Majrooh Sultanpuri</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" s="0" t="inlineStr">
+        <is>
+          <t>2026-03-23</t>
+        </is>
+      </c>
+      <c r="B46" s="0" t="n">
+        <v>45</v>
+      </c>
+      <c r="C46" s="0" t="inlineStr">
+        <is>
+          <t>Ehsaas</t>
+        </is>
+      </c>
+      <c r="D46" s="0" t="inlineStr">
+        <is>
+          <t>Faheem Abdullah, Duha Shah, Vaibhav Pani, Hyder Dar</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" s="0" t="inlineStr">
+        <is>
+          <t>2026-03-23</t>
+        </is>
+      </c>
+      <c r="B47" s="0" t="n">
+        <v>46</v>
+      </c>
+      <c r="C47" s="0" t="inlineStr">
+        <is>
+          <t>Mast Magan (From "2 States)</t>
+        </is>
+      </c>
+      <c r="D47" s="0" t="inlineStr">
+        <is>
+          <t>Arijit Singh, Chinmayi</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" s="0" t="inlineStr">
+        <is>
+          <t>2026-03-23</t>
+        </is>
+      </c>
+      <c r="B48" s="0" t="n">
+        <v>47</v>
+      </c>
+      <c r="C48" s="0" t="inlineStr">
+        <is>
+          <t>Teri Deewani</t>
+        </is>
+      </c>
+      <c r="D48" s="0" t="inlineStr">
+        <is>
+          <t>Kailash Kher, Paresh Kamath, Naresh Kamath</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" s="0" t="inlineStr">
+        <is>
+          <t>2026-03-23</t>
+        </is>
+      </c>
+      <c r="B49" s="0" t="n">
+        <v>48</v>
+      </c>
+      <c r="C49" s="0" t="inlineStr">
+        <is>
+          <t>Dealer</t>
+        </is>
+      </c>
+      <c r="D49" s="0" t="inlineStr">
+        <is>
+          <t>Diljit Dosanjh, Da Future, Virk Andaaz</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" s="0" t="inlineStr">
+        <is>
+          <t>2026-03-23</t>
+        </is>
+      </c>
+      <c r="B50" s="0" t="n">
+        <v>49</v>
+      </c>
+      <c r="C50" s="0" t="inlineStr">
+        <is>
+          <t>Body to Body</t>
+        </is>
+      </c>
+      <c r="D50" s="0" t="inlineStr">
+        <is>
+          <t>BTS</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" s="0" t="inlineStr">
+        <is>
+          <t>2026-03-23</t>
+        </is>
+      </c>
+      <c r="B51" s="0" t="n">
+        <v>50</v>
+      </c>
+      <c r="C51" s="0" t="inlineStr">
+        <is>
+          <t>Humdard (From "Ek Villain")</t>
+        </is>
+      </c>
+      <c r="D51" s="0" t="inlineStr">
+        <is>
+          <t>Arijit Singh</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:D51"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="24" t="inlineStr">
+        <is>
+          <t>Date</t>
+        </is>
+      </c>
+      <c r="B1" s="24" t="inlineStr">
+        <is>
+          <t>Rank</t>
+        </is>
+      </c>
+      <c r="C1" s="24" t="inlineStr">
+        <is>
+          <t>Song</t>
+        </is>
+      </c>
+      <c r="D1" s="24" t="inlineStr">
+        <is>
+          <t>Artist</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>2026-03-23</t>
+          <t>2026-03-24</t>
         </is>
       </c>
       <c r="B2" t="n">
@@ -2575,7 +3612,7 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>2026-03-23</t>
+          <t>2026-03-24</t>
         </is>
       </c>
       <c r="B3" t="n">
@@ -2595,7 +3632,7 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>2026-03-23</t>
+          <t>2026-03-24</t>
         </is>
       </c>
       <c r="B4" t="n">
@@ -2603,19 +3640,19 @@
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>Dhurandhar The Revenge - Aari Aari (From "Dhurandhar The Revenge")</t>
+          <t>Jaiye Sajana</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>Shashwat Sachdev, Bombay Rockers, Irshad Kamil, Khan Saab, Reble, Token, Jasmine Sandlas, Sudhir Yaduvanshi</t>
+          <t>Shashwat Sachdev, Jasmine Sandlas, Satinder Sartaaj</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>2026-03-23</t>
+          <t>2026-03-24</t>
         </is>
       </c>
       <c r="B5" t="n">
@@ -2635,7 +3672,7 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>2026-03-23</t>
+          <t>2026-03-24</t>
         </is>
       </c>
       <c r="B6" t="n">
@@ -2643,19 +3680,19 @@
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>Jaiye Sajana</t>
+          <t>Dhurandhar The Revenge - Aari Aari (From "Dhurandhar The Revenge")</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>Shashwat Sachdev, Jasmine Sandlas, Satinder Sartaaj</t>
+          <t>Shashwat Sachdev, Bombay Rockers, Irshad Kamil, Khan Saab, Reble, Token, Jasmine Sandlas, Sudhir Yaduvanshi</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>2026-03-23</t>
+          <t>2026-03-24</t>
         </is>
       </c>
       <c r="B7" t="n">
@@ -2675,7 +3712,7 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>2026-03-23</t>
+          <t>2026-03-24</t>
         </is>
       </c>
       <c r="B8" t="n">
@@ -2683,19 +3720,19 @@
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>Dooron Dooron</t>
+          <t>Jaan Se Guzarte Hain</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>Paresh Pahuja, Shiv Tandan, Meghdeep Bose</t>
+          <t>Shashwat Sachdev, Khan Saab</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>2026-03-23</t>
+          <t>2026-03-24</t>
         </is>
       </c>
       <c r="B9" t="n">
@@ -2715,7 +3752,7 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>2026-03-23</t>
+          <t>2026-03-24</t>
         </is>
       </c>
       <c r="B10" t="n">
@@ -2723,19 +3760,19 @@
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>Sitaare (From "Ikkis")</t>
+          <t>Dooron Dooron</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>Arijit Singh, White Noise Collectives, Amitabh Bhattacharya</t>
+          <t>Paresh Pahuja, Shiv Tandan, Meghdeep Bose</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>2026-03-23</t>
+          <t>2026-03-24</t>
         </is>
       </c>
       <c r="B11" t="n">
@@ -2743,19 +3780,19 @@
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>Jaan Se Guzarte Hain</t>
+          <t>Sitaare (From "Ikkis")</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>Shashwat Sachdev, Khan Saab</t>
+          <t>Arijit Singh, White Noise Collectives, Amitabh Bhattacharya</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>2026-03-23</t>
+          <t>2026-03-24</t>
         </is>
       </c>
       <c r="B12" t="n">
@@ -2775,7 +3812,7 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>2026-03-23</t>
+          <t>2026-03-24</t>
         </is>
       </c>
       <c r="B13" t="n">
@@ -2783,19 +3820,19 @@
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>Samjhawan</t>
+          <t>Apna Bana Le</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>Jawad Ahmad, Shaarib Toshi, Arijit Singh, Shreya Ghoshal</t>
+          <t>Sachin-Jigar, Arijit Singh, Amitabh Bhattacharya</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>2026-03-23</t>
+          <t>2026-03-24</t>
         </is>
       </c>
       <c r="B14" t="n">
@@ -2803,19 +3840,19 @@
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>Apna Bana Le</t>
+          <t>Samjhawan</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>Sachin-Jigar, Arijit Singh, Amitabh Bhattacharya</t>
+          <t>Jawad Ahmad, Shaarib Toshi, Arijit Singh, Shreya Ghoshal</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>2026-03-23</t>
+          <t>2026-03-24</t>
         </is>
       </c>
       <c r="B15" t="n">
@@ -2835,7 +3872,7 @@
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>2026-03-23</t>
+          <t>2026-03-24</t>
         </is>
       </c>
       <c r="B16" t="n">
@@ -2855,7 +3892,7 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>2026-03-23</t>
+          <t>2026-03-24</t>
         </is>
       </c>
       <c r="B17" t="n">
@@ -2875,7 +3912,7 @@
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>2026-03-23</t>
+          <t>2026-03-24</t>
         </is>
       </c>
       <c r="B18" t="n">
@@ -2895,7 +3932,7 @@
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>2026-03-23</t>
+          <t>2026-03-24</t>
         </is>
       </c>
       <c r="B19" t="n">
@@ -2915,7 +3952,7 @@
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>2026-03-23</t>
+          <t>2026-03-24</t>
         </is>
       </c>
       <c r="B20" t="n">
@@ -2923,19 +3960,19 @@
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>Pavazha Malli - From "Think Indie"</t>
+          <t>Ishq</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>Sai Abhyankkar, Shruti Haasan, Vivek</t>
+          <t>Faheem Abdullah, Rauhan Malik, Amir Ameer</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>2026-03-23</t>
+          <t>2026-03-24</t>
         </is>
       </c>
       <c r="B21" t="n">
@@ -2943,19 +3980,19 @@
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>Ishq</t>
+          <t>Pavazha Malli - From "Think Indie"</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>Faheem Abdullah, Rauhan Malik, Amir Ameer</t>
+          <t>Sai Abhyankkar, Shruti Haasan, Vivek</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>2026-03-23</t>
+          <t>2026-03-24</t>
         </is>
       </c>
       <c r="B22" t="n">
@@ -2963,19 +4000,19 @@
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>Bairi</t>
+          <t>Ishqa Ve</t>
         </is>
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>Virat, Pradeep Solanki, Heena</t>
+          <t>Zeeshan Ali, Yuvraj Tung, Sandeep Aulakh, Honey Dhillon</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>2026-03-23</t>
+          <t>2026-03-24</t>
         </is>
       </c>
       <c r="B23" t="n">
@@ -2983,19 +4020,19 @@
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>Saiyaara</t>
+          <t>Mann Mera</t>
         </is>
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>Tanishk Bagchi, Faheem Abdullah, Arslan Nizami, Irshad Kamil</t>
+          <t>Gajendra Verma</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>2026-03-23</t>
+          <t>2026-03-24</t>
         </is>
       </c>
       <c r="B24" t="n">
@@ -3003,19 +4040,19 @@
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>Ishqa Ve</t>
+          <t>Saiyaara</t>
         </is>
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>Zeeshan Ali, Yuvraj Tung, Sandeep Aulakh, Honey Dhillon</t>
+          <t>Tanishk Bagchi, Faheem Abdullah, Arslan Nizami, Irshad Kamil</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>2026-03-23</t>
+          <t>2026-03-24</t>
         </is>
       </c>
       <c r="B25" t="n">
@@ -3023,19 +4060,19 @@
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>Mann Mera</t>
+          <t>Bairi</t>
         </is>
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>Gajendra Verma</t>
+          <t>Virat, Pradeep Solanki, Heena</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>2026-03-23</t>
+          <t>2026-03-24</t>
         </is>
       </c>
       <c r="B26" t="n">
@@ -3043,19 +4080,19 @@
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>SWIM</t>
+          <t>Raanjhan (From "Do Patti")</t>
         </is>
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>BTS</t>
+          <t>Sachet-Parampara, Parampara Tandon, Kausar Munir</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>2026-03-23</t>
+          <t>2026-03-24</t>
         </is>
       </c>
       <c r="B27" t="n">
@@ -3063,19 +4100,19 @@
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>Raanjhan (From "Do Patti")</t>
+          <t>Naal Nachna</t>
         </is>
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t>Sachet-Parampara, Parampara Tandon, Kausar Munir</t>
+          <t>Shashwat Sachdev, Afsana Khan, Irshad Kamil, Reble</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>2026-03-23</t>
+          <t>2026-03-24</t>
         </is>
       </c>
       <c r="B28" t="n">
@@ -3083,19 +4120,19 @@
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>Naal Nachna</t>
+          <t>Jogi</t>
         </is>
       </c>
       <c r="D28" t="inlineStr">
         <is>
-          <t>Shashwat Sachdev, Afsana Khan, Irshad Kamil, Reble</t>
+          <t>thiarajxtt, Bir</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>2026-03-23</t>
+          <t>2026-03-24</t>
         </is>
       </c>
       <c r="B29" t="n">
@@ -3103,19 +4140,19 @@
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>Tum Ho Toh (From "Saiyaara")</t>
+          <t>Deewaana Deewaana</t>
         </is>
       </c>
       <c r="D29" t="inlineStr">
         <is>
-          <t>Vishal Mishra, Hansika Pareek, Raj Shekhar</t>
+          <t>A.R. Rahman, Irshad Kamil</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>2026-03-23</t>
+          <t>2026-03-24</t>
         </is>
       </c>
       <c r="B30" t="n">
@@ -3123,19 +4160,19 @@
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>Deewaana Deewaana</t>
+          <t>SWIM</t>
         </is>
       </c>
       <c r="D30" t="inlineStr">
         <is>
-          <t>A.R. Rahman, Irshad Kamil</t>
+          <t>BTS</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>2026-03-23</t>
+          <t>2026-03-24</t>
         </is>
       </c>
       <c r="B31" t="n">
@@ -3143,19 +4180,19 @@
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>Tere Liye</t>
+          <t>Lutt Le Gaya</t>
         </is>
       </c>
       <c r="D31" t="inlineStr">
         <is>
-          <t>Atif Aslam, Shreya Ghoshal, Sachin Gupta, Sameer Anjaan</t>
+          <t>Shashwat Sachdev, Simran Choudhary</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>2026-03-23</t>
+          <t>2026-03-24</t>
         </is>
       </c>
       <c r="B32" t="n">
@@ -3163,19 +4200,19 @@
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>Lutt Le Gaya</t>
+          <t>Tere Liye</t>
         </is>
       </c>
       <c r="D32" t="inlineStr">
         <is>
-          <t>Shashwat Sachdev, Simran Choudhary</t>
+          <t>Atif Aslam, Shreya Ghoshal, Sachin Gupta, Sameer Anjaan</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>2026-03-23</t>
+          <t>2026-03-24</t>
         </is>
       </c>
       <c r="B33" t="n">
@@ -3183,19 +4220,19 @@
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>Aaya Sher (From "The Paradise") (Telugu)</t>
+          <t>Tum Ho Toh (From "Saiyaara")</t>
         </is>
       </c>
       <c r="D33" t="inlineStr">
         <is>
-          <t>Anirudh Ravichander, Jangi Reddy, Arjun Chandy, Kasarla Shyam</t>
+          <t>Vishal Mishra, Hansika Pareek, Raj Shekhar</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>2026-03-23</t>
+          <t>2026-03-24</t>
         </is>
       </c>
       <c r="B34" t="n">
@@ -3203,19 +4240,19 @@
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>Ishq Jalakar - Karvaan</t>
+          <t>Tere Bina</t>
         </is>
       </c>
       <c r="D34" t="inlineStr">
         <is>
-          <t>Shashwat Sachdev, Shahzad Ali, Subhadeep Das Chowdhury, Armaan Khan, Irshad Kamil, Roshan, Sahir Ludhianvi</t>
+          <t>A.R. Rahman, Chinmayi, Murtuza Khan, Qadir Khan</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>2026-03-23</t>
+          <t>2026-03-24</t>
         </is>
       </c>
       <c r="B35" t="n">
@@ -3223,19 +4260,19 @@
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>Agar Tum Saath Ho (From "Tamasha")</t>
+          <t>Ishq Jalakar - Karvaan</t>
         </is>
       </c>
       <c r="D35" t="inlineStr">
         <is>
-          <t>Alka Yagnik, Arijit Singh</t>
+          <t>Shashwat Sachdev, Shahzad Ali, Subhadeep Das Chowdhury, Armaan Khan, Irshad Kamil, Roshan, Sahir Ludhianvi</t>
         </is>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>2026-03-23</t>
+          <t>2026-03-24</t>
         </is>
       </c>
       <c r="B36" t="n">
@@ -3243,19 +4280,19 @@
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>Tere Bina</t>
+          <t>Haseen</t>
         </is>
       </c>
       <c r="D36" t="inlineStr">
         <is>
-          <t>A.R. Rahman, Chinmayi, Murtuza Khan, Qadir Khan</t>
+          <t>Talwiinder, NDS, Rippy Grewal</t>
         </is>
       </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>2026-03-23</t>
+          <t>2026-03-24</t>
         </is>
       </c>
       <c r="B37" t="n">
@@ -3263,19 +4300,19 @@
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>Haseen</t>
+          <t>Agar Tum Saath Ho (From "Tamasha")</t>
         </is>
       </c>
       <c r="D37" t="inlineStr">
         <is>
-          <t>Talwiinder, NDS, Rippy Grewal</t>
+          <t>Alka Yagnik, Arijit Singh</t>
         </is>
       </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>2026-03-23</t>
+          <t>2026-03-24</t>
         </is>
       </c>
       <c r="B38" t="n">
@@ -3283,19 +4320,19 @@
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>Jo Tum Mere Ho</t>
+          <t>Aaya Sher (From "The Paradise") (Telugu)</t>
         </is>
       </c>
       <c r="D38" t="inlineStr">
         <is>
-          <t>Anuv Jain</t>
+          <t>Anirudh Ravichander, Jangi Reddy, Arjun Chandy, Kasarla Shyam</t>
         </is>
       </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>2026-03-23</t>
+          <t>2026-03-24</t>
         </is>
       </c>
       <c r="B39" t="n">
@@ -3303,19 +4340,19 @@
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>Darkhaast</t>
+          <t>Jo Tum Mere Ho</t>
         </is>
       </c>
       <c r="D39" t="inlineStr">
         <is>
-          <t>Mithoon, Arijit Singh, Sunidhi Chauhan, Sayeed Quadri</t>
+          <t>Anuv Jain</t>
         </is>
       </c>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>2026-03-23</t>
+          <t>2026-03-24</t>
         </is>
       </c>
       <c r="B40" t="n">
@@ -3335,7 +4372,7 @@
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>2026-03-23</t>
+          <t>2026-03-24</t>
         </is>
       </c>
       <c r="B41" t="n">
@@ -3343,19 +4380,19 @@
       </c>
       <c r="C41" t="inlineStr">
         <is>
-          <t>Ye Tune Kya Kiya</t>
+          <t>Darkhaast</t>
         </is>
       </c>
       <c r="D41" t="inlineStr">
         <is>
-          <t>Pritam, Javed Bashir, Rajat Arora</t>
+          <t>Mithoon, Arijit Singh, Sunidhi Chauhan, Sayeed Quadri</t>
         </is>
       </c>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>2026-03-23</t>
+          <t>2026-03-24</t>
         </is>
       </c>
       <c r="B42" t="n">
@@ -3363,19 +4400,19 @@
       </c>
       <c r="C42" t="inlineStr">
         <is>
-          <t>Barbaad (From "Saiyaara")</t>
+          <t>Run Down The City - Monica</t>
         </is>
       </c>
       <c r="D42" t="inlineStr">
         <is>
-          <t>The Rish, Jubin Nautiyal</t>
+          <t>Shashwat Sachdev, Reble, Asha Bhosle, R. D. Burman, Majrooh Sultanpuri</t>
         </is>
       </c>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>2026-03-23</t>
+          <t>2026-03-24</t>
         </is>
       </c>
       <c r="B43" t="n">
@@ -3395,7 +4432,7 @@
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>2026-03-23</t>
+          <t>2026-03-24</t>
         </is>
       </c>
       <c r="B44" t="n">
@@ -3403,19 +4440,19 @@
       </c>
       <c r="C44" t="inlineStr">
         <is>
-          <t>Not Guilty</t>
+          <t>Barbaad (From "Saiyaara")</t>
         </is>
       </c>
       <c r="D44" t="inlineStr">
         <is>
-          <t>Dhanda Nyoliwala</t>
+          <t>The Rish, Jubin Nautiyal</t>
         </is>
       </c>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>2026-03-23</t>
+          <t>2026-03-24</t>
         </is>
       </c>
       <c r="B45" t="n">
@@ -3423,19 +4460,19 @@
       </c>
       <c r="C45" t="inlineStr">
         <is>
-          <t>Run Down The City - Monica</t>
+          <t>Ye Tune Kya Kiya</t>
         </is>
       </c>
       <c r="D45" t="inlineStr">
         <is>
-          <t>Shashwat Sachdev, Reble, Asha Bhosle, R. D. Burman, Majrooh Sultanpuri</t>
+          <t>Pritam, Javed Bashir, Rajat Arora</t>
         </is>
       </c>
     </row>
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>2026-03-23</t>
+          <t>2026-03-24</t>
         </is>
       </c>
       <c r="B46" t="n">
@@ -3443,19 +4480,19 @@
       </c>
       <c r="C46" t="inlineStr">
         <is>
-          <t>Ehsaas</t>
+          <t>Phir Se (From "Dhurandhar The Revenge")</t>
         </is>
       </c>
       <c r="D46" t="inlineStr">
         <is>
-          <t>Faheem Abdullah, Duha Shah, Vaibhav Pani, Hyder Dar</t>
+          <t>Shashwat Sachdev, Arijit Singh, Irshad Kamil</t>
         </is>
       </c>
     </row>
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>2026-03-23</t>
+          <t>2026-03-24</t>
         </is>
       </c>
       <c r="B47" t="n">
@@ -3463,19 +4500,19 @@
       </c>
       <c r="C47" t="inlineStr">
         <is>
-          <t>Mast Magan (From "2 States)</t>
+          <t>Not Guilty</t>
         </is>
       </c>
       <c r="D47" t="inlineStr">
         <is>
-          <t>Arijit Singh, Chinmayi</t>
+          <t>Dhanda Nyoliwala</t>
         </is>
       </c>
     </row>
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>2026-03-23</t>
+          <t>2026-03-24</t>
         </is>
       </c>
       <c r="B48" t="n">
@@ -3483,19 +4520,19 @@
       </c>
       <c r="C48" t="inlineStr">
         <is>
-          <t>Teri Deewani</t>
+          <t>Ehsaas</t>
         </is>
       </c>
       <c r="D48" t="inlineStr">
         <is>
-          <t>Kailash Kher, Paresh Kamath, Naresh Kamath</t>
+          <t>Faheem Abdullah, Duha Shah, Vaibhav Pani, Hyder Dar</t>
         </is>
       </c>
     </row>
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>2026-03-23</t>
+          <t>2026-03-24</t>
         </is>
       </c>
       <c r="B49" t="n">
@@ -3503,19 +4540,19 @@
       </c>
       <c r="C49" t="inlineStr">
         <is>
-          <t>Dealer</t>
+          <t>Mast Magan (From "2 States)</t>
         </is>
       </c>
       <c r="D49" t="inlineStr">
         <is>
-          <t>Diljit Dosanjh, Da Future, Virk Andaaz</t>
+          <t>Arijit Singh, Chinmayi</t>
         </is>
       </c>
     </row>
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>2026-03-23</t>
+          <t>2026-03-24</t>
         </is>
       </c>
       <c r="B50" t="n">
@@ -3523,19 +4560,19 @@
       </c>
       <c r="C50" t="inlineStr">
         <is>
-          <t>Body to Body</t>
+          <t>Thodi Si Daaru</t>
         </is>
       </c>
       <c r="D50" t="inlineStr">
         <is>
-          <t>BTS</t>
+          <t>AP Dhillon, Shreya Ghoshal</t>
         </is>
       </c>
     </row>
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>2026-03-23</t>
+          <t>2026-03-24</t>
         </is>
       </c>
       <c r="B51" t="n">
@@ -3543,12 +4580,12 @@
       </c>
       <c r="C51" t="inlineStr">
         <is>
-          <t>Humdard (From "Ek Villain")</t>
+          <t>Dhun (From "Saiyaara")</t>
         </is>
       </c>
       <c r="D51" t="inlineStr">
         <is>
-          <t>Arijit Singh</t>
+          <t>Mithoon, Arijit Singh</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
added data for 25th , got predictions for 26th march
</commit_message>
<xml_diff>
--- a/Probability Project.xlsx
+++ b/Probability Project.xlsx
@@ -14,6 +14,7 @@
     <sheet name="AUTO_20260321" sheetId="9" state="visible" r:id="rId9"/>
     <sheet name="AUTO_20260323" sheetId="10" state="visible" r:id="rId10"/>
     <sheet name="AUTO_20260324" sheetId="11" state="visible" r:id="rId11"/>
+    <sheet name="AUTO_20260325" sheetId="12" state="visible" r:id="rId12"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -3590,9 +3591,1045 @@
       </c>
     </row>
     <row r="2">
+      <c r="A2" s="0" t="inlineStr">
+        <is>
+          <t>2026-03-24</t>
+        </is>
+      </c>
+      <c r="B2" s="0" t="n">
+        <v>1</v>
+      </c>
+      <c r="C2" s="0" t="inlineStr">
+        <is>
+          <t>Bairan</t>
+        </is>
+      </c>
+      <c r="D2" s="0" t="inlineStr">
+        <is>
+          <t>Banjaare</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="0" t="inlineStr">
+        <is>
+          <t>2026-03-24</t>
+        </is>
+      </c>
+      <c r="B3" s="0" t="n">
+        <v>2</v>
+      </c>
+      <c r="C3" s="0" t="inlineStr">
+        <is>
+          <t>Sheesha - Aakhya Mai Aakh Ghali Jo Bairan</t>
+        </is>
+      </c>
+      <c r="D3" s="0" t="inlineStr">
+        <is>
+          <t>Mitta Ror, Swara Verma</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="0" t="inlineStr">
+        <is>
+          <t>2026-03-24</t>
+        </is>
+      </c>
+      <c r="B4" s="0" t="n">
+        <v>3</v>
+      </c>
+      <c r="C4" s="0" t="inlineStr">
+        <is>
+          <t>Jaiye Sajana</t>
+        </is>
+      </c>
+      <c r="D4" s="0" t="inlineStr">
+        <is>
+          <t>Shashwat Sachdev, Jasmine Sandlas, Satinder Sartaaj</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="0" t="inlineStr">
+        <is>
+          <t>2026-03-24</t>
+        </is>
+      </c>
+      <c r="B5" s="0" t="n">
+        <v>4</v>
+      </c>
+      <c r="C5" s="0" t="inlineStr">
+        <is>
+          <t>Gehra Hua</t>
+        </is>
+      </c>
+      <c r="D5" s="0" t="inlineStr">
+        <is>
+          <t>Shashwat Sachdev, Arijit Singh, Irshad Kamil, Armaan Khan</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="0" t="inlineStr">
+        <is>
+          <t>2026-03-24</t>
+        </is>
+      </c>
+      <c r="B6" s="0" t="n">
+        <v>5</v>
+      </c>
+      <c r="C6" s="0" t="inlineStr">
+        <is>
+          <t>Dhurandhar The Revenge - Aari Aari (From "Dhurandhar The Revenge")</t>
+        </is>
+      </c>
+      <c r="D6" s="0" t="inlineStr">
+        <is>
+          <t>Shashwat Sachdev, Bombay Rockers, Irshad Kamil, Khan Saab, Reble, Token, Jasmine Sandlas, Sudhir Yaduvanshi</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="0" t="inlineStr">
+        <is>
+          <t>2026-03-24</t>
+        </is>
+      </c>
+      <c r="B7" s="0" t="n">
+        <v>6</v>
+      </c>
+      <c r="C7" s="0" t="inlineStr">
+        <is>
+          <t>Khat</t>
+        </is>
+      </c>
+      <c r="D7" s="0" t="inlineStr">
+        <is>
+          <t>Navjot Ahuja</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="0" t="inlineStr">
+        <is>
+          <t>2026-03-24</t>
+        </is>
+      </c>
+      <c r="B8" s="0" t="n">
+        <v>7</v>
+      </c>
+      <c r="C8" s="0" t="inlineStr">
+        <is>
+          <t>Jaan Se Guzarte Hain</t>
+        </is>
+      </c>
+      <c r="D8" s="0" t="inlineStr">
+        <is>
+          <t>Shashwat Sachdev, Khan Saab</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="0" t="inlineStr">
+        <is>
+          <t>2026-03-24</t>
+        </is>
+      </c>
+      <c r="B9" s="0" t="n">
+        <v>8</v>
+      </c>
+      <c r="C9" s="0" t="inlineStr">
+        <is>
+          <t>Sahiba</t>
+        </is>
+      </c>
+      <c r="D9" s="0" t="inlineStr">
+        <is>
+          <t>Aditya Rikhari</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="0" t="inlineStr">
+        <is>
+          <t>2026-03-24</t>
+        </is>
+      </c>
+      <c r="B10" s="0" t="n">
+        <v>9</v>
+      </c>
+      <c r="C10" s="0" t="inlineStr">
+        <is>
+          <t>Dooron Dooron</t>
+        </is>
+      </c>
+      <c r="D10" s="0" t="inlineStr">
+        <is>
+          <t>Paresh Pahuja, Shiv Tandan, Meghdeep Bose</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="0" t="inlineStr">
+        <is>
+          <t>2026-03-24</t>
+        </is>
+      </c>
+      <c r="B11" s="0" t="n">
+        <v>10</v>
+      </c>
+      <c r="C11" s="0" t="inlineStr">
+        <is>
+          <t>Sitaare (From "Ikkis")</t>
+        </is>
+      </c>
+      <c r="D11" s="0" t="inlineStr">
+        <is>
+          <t>Arijit Singh, White Noise Collectives, Amitabh Bhattacharya</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="0" t="inlineStr">
+        <is>
+          <t>2026-03-24</t>
+        </is>
+      </c>
+      <c r="B12" s="0" t="n">
+        <v>11</v>
+      </c>
+      <c r="C12" s="0" t="inlineStr">
+        <is>
+          <t>Finding Her</t>
+        </is>
+      </c>
+      <c r="D12" s="0" t="inlineStr">
+        <is>
+          <t>Kushagra, Bharath, Saaheal</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="0" t="inlineStr">
+        <is>
+          <t>2026-03-24</t>
+        </is>
+      </c>
+      <c r="B13" s="0" t="n">
+        <v>12</v>
+      </c>
+      <c r="C13" s="0" t="inlineStr">
+        <is>
+          <t>Apna Bana Le</t>
+        </is>
+      </c>
+      <c r="D13" s="0" t="inlineStr">
+        <is>
+          <t>Sachin-Jigar, Arijit Singh, Amitabh Bhattacharya</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="0" t="inlineStr">
+        <is>
+          <t>2026-03-24</t>
+        </is>
+      </c>
+      <c r="B14" s="0" t="n">
+        <v>13</v>
+      </c>
+      <c r="C14" s="0" t="inlineStr">
+        <is>
+          <t>Samjhawan</t>
+        </is>
+      </c>
+      <c r="D14" s="0" t="inlineStr">
+        <is>
+          <t>Jawad Ahmad, Shaarib Toshi, Arijit Singh, Shreya Ghoshal</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="0" t="inlineStr">
+        <is>
+          <t>2026-03-24</t>
+        </is>
+      </c>
+      <c r="B15" s="0" t="n">
+        <v>14</v>
+      </c>
+      <c r="C15" s="0" t="inlineStr">
+        <is>
+          <t>Dhurandhar - Title Track</t>
+        </is>
+      </c>
+      <c r="D15" s="0" t="inlineStr">
+        <is>
+          <t>Shashwat Sachdev, Hanumankind, Jasmine Sandlas, Sudhir Yaduvanshi, Charanjit Ahuja, Muhammad Sadiq, Ranjit Kaur, Babu Singh Maan</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="0" t="inlineStr">
+        <is>
+          <t>2026-03-24</t>
+        </is>
+      </c>
+      <c r="B16" s="0" t="n">
+        <v>15</v>
+      </c>
+      <c r="C16" s="0" t="inlineStr">
+        <is>
+          <t>Shararat</t>
+        </is>
+      </c>
+      <c r="D16" s="0" t="inlineStr">
+        <is>
+          <t>Shashwat Sachdev, Madhubanti Bagchi, Jasmine Sandlas</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="0" t="inlineStr">
+        <is>
+          <t>2026-03-24</t>
+        </is>
+      </c>
+      <c r="B17" s="0" t="n">
+        <v>16</v>
+      </c>
+      <c r="C17" s="0" t="inlineStr">
+        <is>
+          <t>Arz Kiya Hai | Coke Studio Bharat</t>
+        </is>
+      </c>
+      <c r="D17" s="0" t="inlineStr">
+        <is>
+          <t>Anuv Jain</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="0" t="inlineStr">
+        <is>
+          <t>2026-03-24</t>
+        </is>
+      </c>
+      <c r="B18" s="0" t="n">
+        <v>17</v>
+      </c>
+      <c r="C18" s="0" t="inlineStr">
+        <is>
+          <t>For A Reason</t>
+        </is>
+      </c>
+      <c r="D18" s="0" t="inlineStr">
+        <is>
+          <t>Karan Aujla, Ikky</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="0" t="inlineStr">
+        <is>
+          <t>2026-03-24</t>
+        </is>
+      </c>
+      <c r="B19" s="0" t="n">
+        <v>18</v>
+      </c>
+      <c r="C19" s="0" t="inlineStr">
+        <is>
+          <t>Boyfriend</t>
+        </is>
+      </c>
+      <c r="D19" s="0" t="inlineStr">
+        <is>
+          <t>Karan Aujla, Ikky</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="0" t="inlineStr">
+        <is>
+          <t>2026-03-24</t>
+        </is>
+      </c>
+      <c r="B20" s="0" t="n">
+        <v>19</v>
+      </c>
+      <c r="C20" s="0" t="inlineStr">
+        <is>
+          <t>Ishq</t>
+        </is>
+      </c>
+      <c r="D20" s="0" t="inlineStr">
+        <is>
+          <t>Faheem Abdullah, Rauhan Malik, Amir Ameer</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="0" t="inlineStr">
+        <is>
+          <t>2026-03-24</t>
+        </is>
+      </c>
+      <c r="B21" s="0" t="n">
+        <v>20</v>
+      </c>
+      <c r="C21" s="0" t="inlineStr">
+        <is>
+          <t>Pavazha Malli - From "Think Indie"</t>
+        </is>
+      </c>
+      <c r="D21" s="0" t="inlineStr">
+        <is>
+          <t>Sai Abhyankkar, Shruti Haasan, Vivek</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="0" t="inlineStr">
+        <is>
+          <t>2026-03-24</t>
+        </is>
+      </c>
+      <c r="B22" s="0" t="n">
+        <v>21</v>
+      </c>
+      <c r="C22" s="0" t="inlineStr">
+        <is>
+          <t>Ishqa Ve</t>
+        </is>
+      </c>
+      <c r="D22" s="0" t="inlineStr">
+        <is>
+          <t>Zeeshan Ali, Yuvraj Tung, Sandeep Aulakh, Honey Dhillon</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="0" t="inlineStr">
+        <is>
+          <t>2026-03-24</t>
+        </is>
+      </c>
+      <c r="B23" s="0" t="n">
+        <v>22</v>
+      </c>
+      <c r="C23" s="0" t="inlineStr">
+        <is>
+          <t>Mann Mera</t>
+        </is>
+      </c>
+      <c r="D23" s="0" t="inlineStr">
+        <is>
+          <t>Gajendra Verma</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="0" t="inlineStr">
+        <is>
+          <t>2026-03-24</t>
+        </is>
+      </c>
+      <c r="B24" s="0" t="n">
+        <v>23</v>
+      </c>
+      <c r="C24" s="0" t="inlineStr">
+        <is>
+          <t>Saiyaara</t>
+        </is>
+      </c>
+      <c r="D24" s="0" t="inlineStr">
+        <is>
+          <t>Tanishk Bagchi, Faheem Abdullah, Arslan Nizami, Irshad Kamil</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="0" t="inlineStr">
+        <is>
+          <t>2026-03-24</t>
+        </is>
+      </c>
+      <c r="B25" s="0" t="n">
+        <v>24</v>
+      </c>
+      <c r="C25" s="0" t="inlineStr">
+        <is>
+          <t>Bairi</t>
+        </is>
+      </c>
+      <c r="D25" s="0" t="inlineStr">
+        <is>
+          <t>Virat, Pradeep Solanki, Heena</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="0" t="inlineStr">
+        <is>
+          <t>2026-03-24</t>
+        </is>
+      </c>
+      <c r="B26" s="0" t="n">
+        <v>25</v>
+      </c>
+      <c r="C26" s="0" t="inlineStr">
+        <is>
+          <t>Raanjhan (From "Do Patti")</t>
+        </is>
+      </c>
+      <c r="D26" s="0" t="inlineStr">
+        <is>
+          <t>Sachet-Parampara, Parampara Tandon, Kausar Munir</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="0" t="inlineStr">
+        <is>
+          <t>2026-03-24</t>
+        </is>
+      </c>
+      <c r="B27" s="0" t="n">
+        <v>26</v>
+      </c>
+      <c r="C27" s="0" t="inlineStr">
+        <is>
+          <t>Naal Nachna</t>
+        </is>
+      </c>
+      <c r="D27" s="0" t="inlineStr">
+        <is>
+          <t>Shashwat Sachdev, Afsana Khan, Irshad Kamil, Reble</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="0" t="inlineStr">
+        <is>
+          <t>2026-03-24</t>
+        </is>
+      </c>
+      <c r="B28" s="0" t="n">
+        <v>27</v>
+      </c>
+      <c r="C28" s="0" t="inlineStr">
+        <is>
+          <t>Jogi</t>
+        </is>
+      </c>
+      <c r="D28" s="0" t="inlineStr">
+        <is>
+          <t>thiarajxtt, Bir</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="0" t="inlineStr">
+        <is>
+          <t>2026-03-24</t>
+        </is>
+      </c>
+      <c r="B29" s="0" t="n">
+        <v>28</v>
+      </c>
+      <c r="C29" s="0" t="inlineStr">
+        <is>
+          <t>Deewaana Deewaana</t>
+        </is>
+      </c>
+      <c r="D29" s="0" t="inlineStr">
+        <is>
+          <t>A.R. Rahman, Irshad Kamil</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="0" t="inlineStr">
+        <is>
+          <t>2026-03-24</t>
+        </is>
+      </c>
+      <c r="B30" s="0" t="n">
+        <v>29</v>
+      </c>
+      <c r="C30" s="0" t="inlineStr">
+        <is>
+          <t>SWIM</t>
+        </is>
+      </c>
+      <c r="D30" s="0" t="inlineStr">
+        <is>
+          <t>BTS</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="0" t="inlineStr">
+        <is>
+          <t>2026-03-24</t>
+        </is>
+      </c>
+      <c r="B31" s="0" t="n">
+        <v>30</v>
+      </c>
+      <c r="C31" s="0" t="inlineStr">
+        <is>
+          <t>Lutt Le Gaya</t>
+        </is>
+      </c>
+      <c r="D31" s="0" t="inlineStr">
+        <is>
+          <t>Shashwat Sachdev, Simran Choudhary</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="0" t="inlineStr">
+        <is>
+          <t>2026-03-24</t>
+        </is>
+      </c>
+      <c r="B32" s="0" t="n">
+        <v>31</v>
+      </c>
+      <c r="C32" s="0" t="inlineStr">
+        <is>
+          <t>Tere Liye</t>
+        </is>
+      </c>
+      <c r="D32" s="0" t="inlineStr">
+        <is>
+          <t>Atif Aslam, Shreya Ghoshal, Sachin Gupta, Sameer Anjaan</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="0" t="inlineStr">
+        <is>
+          <t>2026-03-24</t>
+        </is>
+      </c>
+      <c r="B33" s="0" t="n">
+        <v>32</v>
+      </c>
+      <c r="C33" s="0" t="inlineStr">
+        <is>
+          <t>Tum Ho Toh (From "Saiyaara")</t>
+        </is>
+      </c>
+      <c r="D33" s="0" t="inlineStr">
+        <is>
+          <t>Vishal Mishra, Hansika Pareek, Raj Shekhar</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="0" t="inlineStr">
+        <is>
+          <t>2026-03-24</t>
+        </is>
+      </c>
+      <c r="B34" s="0" t="n">
+        <v>33</v>
+      </c>
+      <c r="C34" s="0" t="inlineStr">
+        <is>
+          <t>Tere Bina</t>
+        </is>
+      </c>
+      <c r="D34" s="0" t="inlineStr">
+        <is>
+          <t>A.R. Rahman, Chinmayi, Murtuza Khan, Qadir Khan</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="0" t="inlineStr">
+        <is>
+          <t>2026-03-24</t>
+        </is>
+      </c>
+      <c r="B35" s="0" t="n">
+        <v>34</v>
+      </c>
+      <c r="C35" s="0" t="inlineStr">
+        <is>
+          <t>Ishq Jalakar - Karvaan</t>
+        </is>
+      </c>
+      <c r="D35" s="0" t="inlineStr">
+        <is>
+          <t>Shashwat Sachdev, Shahzad Ali, Subhadeep Das Chowdhury, Armaan Khan, Irshad Kamil, Roshan, Sahir Ludhianvi</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="0" t="inlineStr">
+        <is>
+          <t>2026-03-24</t>
+        </is>
+      </c>
+      <c r="B36" s="0" t="n">
+        <v>35</v>
+      </c>
+      <c r="C36" s="0" t="inlineStr">
+        <is>
+          <t>Haseen</t>
+        </is>
+      </c>
+      <c r="D36" s="0" t="inlineStr">
+        <is>
+          <t>Talwiinder, NDS, Rippy Grewal</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="0" t="inlineStr">
+        <is>
+          <t>2026-03-24</t>
+        </is>
+      </c>
+      <c r="B37" s="0" t="n">
+        <v>36</v>
+      </c>
+      <c r="C37" s="0" t="inlineStr">
+        <is>
+          <t>Agar Tum Saath Ho (From "Tamasha")</t>
+        </is>
+      </c>
+      <c r="D37" s="0" t="inlineStr">
+        <is>
+          <t>Alka Yagnik, Arijit Singh</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="0" t="inlineStr">
+        <is>
+          <t>2026-03-24</t>
+        </is>
+      </c>
+      <c r="B38" s="0" t="n">
+        <v>37</v>
+      </c>
+      <c r="C38" s="0" t="inlineStr">
+        <is>
+          <t>Aaya Sher (From "The Paradise") (Telugu)</t>
+        </is>
+      </c>
+      <c r="D38" s="0" t="inlineStr">
+        <is>
+          <t>Anirudh Ravichander, Jangi Reddy, Arjun Chandy, Kasarla Shyam</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="0" t="inlineStr">
+        <is>
+          <t>2026-03-24</t>
+        </is>
+      </c>
+      <c r="B39" s="0" t="n">
+        <v>38</v>
+      </c>
+      <c r="C39" s="0" t="inlineStr">
+        <is>
+          <t>Jo Tum Mere Ho</t>
+        </is>
+      </c>
+      <c r="D39" s="0" t="inlineStr">
+        <is>
+          <t>Anuv Jain</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="0" t="inlineStr">
+        <is>
+          <t>2026-03-24</t>
+        </is>
+      </c>
+      <c r="B40" s="0" t="n">
+        <v>39</v>
+      </c>
+      <c r="C40" s="0" t="inlineStr">
+        <is>
+          <t>Main Aur Tu (From "Dhurandhar The Revenge")</t>
+        </is>
+      </c>
+      <c r="D40" s="0" t="inlineStr">
+        <is>
+          <t>Shashwat Sachdev, Jasmine Sandlas, Reble</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" s="0" t="inlineStr">
+        <is>
+          <t>2026-03-24</t>
+        </is>
+      </c>
+      <c r="B41" s="0" t="n">
+        <v>40</v>
+      </c>
+      <c r="C41" s="0" t="inlineStr">
+        <is>
+          <t>Darkhaast</t>
+        </is>
+      </c>
+      <c r="D41" s="0" t="inlineStr">
+        <is>
+          <t>Mithoon, Arijit Singh, Sunidhi Chauhan, Sayeed Quadri</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" s="0" t="inlineStr">
+        <is>
+          <t>2026-03-24</t>
+        </is>
+      </c>
+      <c r="B42" s="0" t="n">
+        <v>41</v>
+      </c>
+      <c r="C42" s="0" t="inlineStr">
+        <is>
+          <t>Run Down The City - Monica</t>
+        </is>
+      </c>
+      <c r="D42" s="0" t="inlineStr">
+        <is>
+          <t>Shashwat Sachdev, Reble, Asha Bhosle, R. D. Burman, Majrooh Sultanpuri</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" s="0" t="inlineStr">
+        <is>
+          <t>2026-03-24</t>
+        </is>
+      </c>
+      <c r="B43" s="0" t="n">
+        <v>42</v>
+      </c>
+      <c r="C43" s="0" t="inlineStr">
+        <is>
+          <t>Mutta Kalakki (From "Youth")</t>
+        </is>
+      </c>
+      <c r="D43" s="0" t="inlineStr">
+        <is>
+          <t>G. V. Prakash, Ken Karunaas</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" s="0" t="inlineStr">
+        <is>
+          <t>2026-03-24</t>
+        </is>
+      </c>
+      <c r="B44" s="0" t="n">
+        <v>43</v>
+      </c>
+      <c r="C44" s="0" t="inlineStr">
+        <is>
+          <t>Barbaad (From "Saiyaara")</t>
+        </is>
+      </c>
+      <c r="D44" s="0" t="inlineStr">
+        <is>
+          <t>The Rish, Jubin Nautiyal</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" s="0" t="inlineStr">
+        <is>
+          <t>2026-03-24</t>
+        </is>
+      </c>
+      <c r="B45" s="0" t="n">
+        <v>44</v>
+      </c>
+      <c r="C45" s="0" t="inlineStr">
+        <is>
+          <t>Ye Tune Kya Kiya</t>
+        </is>
+      </c>
+      <c r="D45" s="0" t="inlineStr">
+        <is>
+          <t>Pritam, Javed Bashir, Rajat Arora</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" s="0" t="inlineStr">
+        <is>
+          <t>2026-03-24</t>
+        </is>
+      </c>
+      <c r="B46" s="0" t="n">
+        <v>45</v>
+      </c>
+      <c r="C46" s="0" t="inlineStr">
+        <is>
+          <t>Phir Se (From "Dhurandhar The Revenge")</t>
+        </is>
+      </c>
+      <c r="D46" s="0" t="inlineStr">
+        <is>
+          <t>Shashwat Sachdev, Arijit Singh, Irshad Kamil</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" s="0" t="inlineStr">
+        <is>
+          <t>2026-03-24</t>
+        </is>
+      </c>
+      <c r="B47" s="0" t="n">
+        <v>46</v>
+      </c>
+      <c r="C47" s="0" t="inlineStr">
+        <is>
+          <t>Not Guilty</t>
+        </is>
+      </c>
+      <c r="D47" s="0" t="inlineStr">
+        <is>
+          <t>Dhanda Nyoliwala</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" s="0" t="inlineStr">
+        <is>
+          <t>2026-03-24</t>
+        </is>
+      </c>
+      <c r="B48" s="0" t="n">
+        <v>47</v>
+      </c>
+      <c r="C48" s="0" t="inlineStr">
+        <is>
+          <t>Ehsaas</t>
+        </is>
+      </c>
+      <c r="D48" s="0" t="inlineStr">
+        <is>
+          <t>Faheem Abdullah, Duha Shah, Vaibhav Pani, Hyder Dar</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" s="0" t="inlineStr">
+        <is>
+          <t>2026-03-24</t>
+        </is>
+      </c>
+      <c r="B49" s="0" t="n">
+        <v>48</v>
+      </c>
+      <c r="C49" s="0" t="inlineStr">
+        <is>
+          <t>Mast Magan (From "2 States)</t>
+        </is>
+      </c>
+      <c r="D49" s="0" t="inlineStr">
+        <is>
+          <t>Arijit Singh, Chinmayi</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" s="0" t="inlineStr">
+        <is>
+          <t>2026-03-24</t>
+        </is>
+      </c>
+      <c r="B50" s="0" t="n">
+        <v>49</v>
+      </c>
+      <c r="C50" s="0" t="inlineStr">
+        <is>
+          <t>Thodi Si Daaru</t>
+        </is>
+      </c>
+      <c r="D50" s="0" t="inlineStr">
+        <is>
+          <t>AP Dhillon, Shreya Ghoshal</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" s="0" t="inlineStr">
+        <is>
+          <t>2026-03-24</t>
+        </is>
+      </c>
+      <c r="B51" s="0" t="n">
+        <v>50</v>
+      </c>
+      <c r="C51" s="0" t="inlineStr">
+        <is>
+          <t>Dhun (From "Saiyaara")</t>
+        </is>
+      </c>
+      <c r="D51" s="0" t="inlineStr">
+        <is>
+          <t>Mithoon, Arijit Singh</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:D51"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="24" t="inlineStr">
+        <is>
+          <t>Date</t>
+        </is>
+      </c>
+      <c r="B1" s="24" t="inlineStr">
+        <is>
+          <t>Rank</t>
+        </is>
+      </c>
+      <c r="C1" s="24" t="inlineStr">
+        <is>
+          <t>Song</t>
+        </is>
+      </c>
+      <c r="D1" s="24" t="inlineStr">
+        <is>
+          <t>Artist</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>2026-03-24</t>
+          <t>2026-03-25</t>
         </is>
       </c>
       <c r="B2" t="n">
@@ -3612,7 +4649,7 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>2026-03-24</t>
+          <t>2026-03-25</t>
         </is>
       </c>
       <c r="B3" t="n">
@@ -3620,19 +4657,19 @@
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>Sheesha - Aakhya Mai Aakh Ghali Jo Bairan</t>
+          <t>Jaiye Sajana</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>Mitta Ror, Swara Verma</t>
+          <t>Shashwat Sachdev, Jasmine Sandlas, Satinder Sartaaj</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>2026-03-24</t>
+          <t>2026-03-25</t>
         </is>
       </c>
       <c r="B4" t="n">
@@ -3640,19 +4677,19 @@
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>Jaiye Sajana</t>
+          <t>Sheesha - Aakhya Mai Aakh Ghali Jo Bairan</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>Shashwat Sachdev, Jasmine Sandlas, Satinder Sartaaj</t>
+          <t>Mitta Ror, Swara Verma</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>2026-03-24</t>
+          <t>2026-03-25</t>
         </is>
       </c>
       <c r="B5" t="n">
@@ -3672,7 +4709,7 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>2026-03-24</t>
+          <t>2026-03-25</t>
         </is>
       </c>
       <c r="B6" t="n">
@@ -3680,7 +4717,7 @@
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>Dhurandhar The Revenge - Aari Aari (From "Dhurandhar The Revenge")</t>
+          <t>Dhurandhar The Revenge - Aari Aari</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
@@ -3692,7 +4729,7 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>2026-03-24</t>
+          <t>2026-03-25</t>
         </is>
       </c>
       <c r="B7" t="n">
@@ -3712,7 +4749,7 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>2026-03-24</t>
+          <t>2026-03-25</t>
         </is>
       </c>
       <c r="B8" t="n">
@@ -3732,7 +4769,7 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>2026-03-24</t>
+          <t>2026-03-25</t>
         </is>
       </c>
       <c r="B9" t="n">
@@ -3740,19 +4777,19 @@
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>Sahiba</t>
+          <t>Dooron Dooron</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>Aditya Rikhari</t>
+          <t>Paresh Pahuja, Shiv Tandan, Meghdeep Bose</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>2026-03-24</t>
+          <t>2026-03-25</t>
         </is>
       </c>
       <c r="B10" t="n">
@@ -3760,19 +4797,19 @@
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>Dooron Dooron</t>
+          <t>Sitaare (From "Ikkis")</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>Paresh Pahuja, Shiv Tandan, Meghdeep Bose</t>
+          <t>Arijit Singh, White Noise Collectives, Amitabh Bhattacharya</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>2026-03-24</t>
+          <t>2026-03-25</t>
         </is>
       </c>
       <c r="B11" t="n">
@@ -3780,19 +4817,19 @@
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>Sitaare (From "Ikkis")</t>
+          <t>Sahiba</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>Arijit Singh, White Noise Collectives, Amitabh Bhattacharya</t>
+          <t>Aditya Rikhari</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>2026-03-24</t>
+          <t>2026-03-25</t>
         </is>
       </c>
       <c r="B12" t="n">
@@ -3812,7 +4849,7 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>2026-03-24</t>
+          <t>2026-03-25</t>
         </is>
       </c>
       <c r="B13" t="n">
@@ -3832,7 +4869,7 @@
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>2026-03-24</t>
+          <t>2026-03-25</t>
         </is>
       </c>
       <c r="B14" t="n">
@@ -3840,19 +4877,19 @@
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>Samjhawan</t>
+          <t>Shararat</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>Jawad Ahmad, Shaarib Toshi, Arijit Singh, Shreya Ghoshal</t>
+          <t>Shashwat Sachdev, Madhubanti Bagchi, Jasmine Sandlas</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>2026-03-24</t>
+          <t>2026-03-25</t>
         </is>
       </c>
       <c r="B15" t="n">
@@ -3860,19 +4897,19 @@
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>Dhurandhar - Title Track</t>
+          <t>Samjhawan</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>Shashwat Sachdev, Hanumankind, Jasmine Sandlas, Sudhir Yaduvanshi, Charanjit Ahuja, Muhammad Sadiq, Ranjit Kaur, Babu Singh Maan</t>
+          <t>Jawad Ahmad, Shaarib Toshi, Arijit Singh, Shreya Ghoshal</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>2026-03-24</t>
+          <t>2026-03-25</t>
         </is>
       </c>
       <c r="B16" t="n">
@@ -3880,19 +4917,19 @@
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>Shararat</t>
+          <t>Dhurandhar - Title Track</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>Shashwat Sachdev, Madhubanti Bagchi, Jasmine Sandlas</t>
+          <t>Shashwat Sachdev, Hanumankind, Jasmine Sandlas, Sudhir Yaduvanshi, Charanjit Ahuja, Muhammad Sadiq, Ranjit Kaur, Babu Singh Maan</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>2026-03-24</t>
+          <t>2026-03-25</t>
         </is>
       </c>
       <c r="B17" t="n">
@@ -3912,7 +4949,7 @@
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>2026-03-24</t>
+          <t>2026-03-25</t>
         </is>
       </c>
       <c r="B18" t="n">
@@ -3920,19 +4957,19 @@
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>For A Reason</t>
+          <t>Ishqa Ve</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>Karan Aujla, Ikky</t>
+          <t>Zeeshan Ali, Yuvraj Tung, Sandeep Aulakh, Honey Dhillon</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>2026-03-24</t>
+          <t>2026-03-25</t>
         </is>
       </c>
       <c r="B19" t="n">
@@ -3940,7 +4977,7 @@
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>Boyfriend</t>
+          <t>For A Reason</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
@@ -3952,7 +4989,7 @@
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>2026-03-24</t>
+          <t>2026-03-25</t>
         </is>
       </c>
       <c r="B20" t="n">
@@ -3960,19 +4997,19 @@
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>Ishq</t>
+          <t>Boyfriend</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>Faheem Abdullah, Rauhan Malik, Amir Ameer</t>
+          <t>Karan Aujla, Ikky</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>2026-03-24</t>
+          <t>2026-03-25</t>
         </is>
       </c>
       <c r="B21" t="n">
@@ -3992,7 +5029,7 @@
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>2026-03-24</t>
+          <t>2026-03-25</t>
         </is>
       </c>
       <c r="B22" t="n">
@@ -4000,19 +5037,19 @@
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>Ishqa Ve</t>
+          <t>Mann Mera</t>
         </is>
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>Zeeshan Ali, Yuvraj Tung, Sandeep Aulakh, Honey Dhillon</t>
+          <t>Gajendra Verma</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>2026-03-24</t>
+          <t>2026-03-25</t>
         </is>
       </c>
       <c r="B23" t="n">
@@ -4020,19 +5057,19 @@
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>Mann Mera</t>
+          <t>Bairi</t>
         </is>
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>Gajendra Verma</t>
+          <t>Virat, Pradeep Solanki, Heena</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>2026-03-24</t>
+          <t>2026-03-25</t>
         </is>
       </c>
       <c r="B24" t="n">
@@ -4040,19 +5077,19 @@
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>Saiyaara</t>
+          <t>Ishq</t>
         </is>
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>Tanishk Bagchi, Faheem Abdullah, Arslan Nizami, Irshad Kamil</t>
+          <t>Faheem Abdullah, Rauhan Malik, Amir Ameer</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>2026-03-24</t>
+          <t>2026-03-25</t>
         </is>
       </c>
       <c r="B25" t="n">
@@ -4060,19 +5097,19 @@
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>Bairi</t>
+          <t>Saiyaara</t>
         </is>
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>Virat, Pradeep Solanki, Heena</t>
+          <t>Tanishk Bagchi, Faheem Abdullah, Arslan Nizami, Irshad Kamil</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>2026-03-24</t>
+          <t>2026-03-25</t>
         </is>
       </c>
       <c r="B26" t="n">
@@ -4080,19 +5117,19 @@
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>Raanjhan (From "Do Patti")</t>
+          <t>Naal Nachna</t>
         </is>
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>Sachet-Parampara, Parampara Tandon, Kausar Munir</t>
+          <t>Shashwat Sachdev, Afsana Khan, Irshad Kamil, Reble</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>2026-03-24</t>
+          <t>2026-03-25</t>
         </is>
       </c>
       <c r="B27" t="n">
@@ -4100,19 +5137,19 @@
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>Naal Nachna</t>
+          <t>SWIM</t>
         </is>
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t>Shashwat Sachdev, Afsana Khan, Irshad Kamil, Reble</t>
+          <t>BTS</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>2026-03-24</t>
+          <t>2026-03-25</t>
         </is>
       </c>
       <c r="B28" t="n">
@@ -4120,19 +5157,19 @@
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>Jogi</t>
+          <t>Raanjhan (From "Do Patti")</t>
         </is>
       </c>
       <c r="D28" t="inlineStr">
         <is>
-          <t>thiarajxtt, Bir</t>
+          <t>Sachet-Parampara, Parampara Tandon, Kausar Munir</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>2026-03-24</t>
+          <t>2026-03-25</t>
         </is>
       </c>
       <c r="B29" t="n">
@@ -4140,19 +5177,19 @@
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>Deewaana Deewaana</t>
+          <t>Phir Se</t>
         </is>
       </c>
       <c r="D29" t="inlineStr">
         <is>
-          <t>A.R. Rahman, Irshad Kamil</t>
+          <t>Shashwat Sachdev, Arijit Singh, Irshad Kamil</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>2026-03-24</t>
+          <t>2026-03-25</t>
         </is>
       </c>
       <c r="B30" t="n">
@@ -4160,19 +5197,19 @@
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>SWIM</t>
+          <t>Main Aur Tu</t>
         </is>
       </c>
       <c r="D30" t="inlineStr">
         <is>
-          <t>BTS</t>
+          <t>Shashwat Sachdev, Jasmine Sandlas, Reble</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>2026-03-24</t>
+          <t>2026-03-25</t>
         </is>
       </c>
       <c r="B31" t="n">
@@ -4180,19 +5217,19 @@
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>Lutt Le Gaya</t>
+          <t>Deewaana Deewaana</t>
         </is>
       </c>
       <c r="D31" t="inlineStr">
         <is>
-          <t>Shashwat Sachdev, Simran Choudhary</t>
+          <t>A.R. Rahman, Irshad Kamil</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>2026-03-24</t>
+          <t>2026-03-25</t>
         </is>
       </c>
       <c r="B32" t="n">
@@ -4200,19 +5237,19 @@
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>Tere Liye</t>
+          <t>Lutt Le Gaya</t>
         </is>
       </c>
       <c r="D32" t="inlineStr">
         <is>
-          <t>Atif Aslam, Shreya Ghoshal, Sachin Gupta, Sameer Anjaan</t>
+          <t>Shashwat Sachdev, Simran Choudhary</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>2026-03-24</t>
+          <t>2026-03-25</t>
         </is>
       </c>
       <c r="B33" t="n">
@@ -4232,7 +5269,7 @@
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>2026-03-24</t>
+          <t>2026-03-25</t>
         </is>
       </c>
       <c r="B34" t="n">
@@ -4240,19 +5277,19 @@
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>Tere Bina</t>
+          <t>Darkhaast</t>
         </is>
       </c>
       <c r="D34" t="inlineStr">
         <is>
-          <t>A.R. Rahman, Chinmayi, Murtuza Khan, Qadir Khan</t>
+          <t>Mithoon, Arijit Singh, Sunidhi Chauhan, Sayeed Quadri</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>2026-03-24</t>
+          <t>2026-03-25</t>
         </is>
       </c>
       <c r="B35" t="n">
@@ -4260,19 +5297,19 @@
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>Ishq Jalakar - Karvaan</t>
+          <t>Tere Liye</t>
         </is>
       </c>
       <c r="D35" t="inlineStr">
         <is>
-          <t>Shashwat Sachdev, Shahzad Ali, Subhadeep Das Chowdhury, Armaan Khan, Irshad Kamil, Roshan, Sahir Ludhianvi</t>
+          <t>Atif Aslam, Shreya Ghoshal, Sachin Gupta, Sameer Anjaan</t>
         </is>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>2026-03-24</t>
+          <t>2026-03-25</t>
         </is>
       </c>
       <c r="B36" t="n">
@@ -4280,19 +5317,19 @@
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>Haseen</t>
+          <t>Ishq Jalakar - Karvaan</t>
         </is>
       </c>
       <c r="D36" t="inlineStr">
         <is>
-          <t>Talwiinder, NDS, Rippy Grewal</t>
+          <t>Shashwat Sachdev, Shahzad Ali, Subhadeep Das Chowdhury, Armaan Khan, Irshad Kamil, Roshan, Sahir Ludhianvi</t>
         </is>
       </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>2026-03-24</t>
+          <t>2026-03-25</t>
         </is>
       </c>
       <c r="B37" t="n">
@@ -4300,19 +5337,19 @@
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>Agar Tum Saath Ho (From "Tamasha")</t>
+          <t>Aaya Sher (From "The Paradise") (Telugu)</t>
         </is>
       </c>
       <c r="D37" t="inlineStr">
         <is>
-          <t>Alka Yagnik, Arijit Singh</t>
+          <t>Anirudh Ravichander, Jangi Reddy, Arjun Chandy, Kasarla Shyam</t>
         </is>
       </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>2026-03-24</t>
+          <t>2026-03-25</t>
         </is>
       </c>
       <c r="B38" t="n">
@@ -4320,19 +5357,19 @@
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>Aaya Sher (From "The Paradise") (Telugu)</t>
+          <t>Jo Tum Mere Ho</t>
         </is>
       </c>
       <c r="D38" t="inlineStr">
         <is>
-          <t>Anirudh Ravichander, Jangi Reddy, Arjun Chandy, Kasarla Shyam</t>
+          <t>Anuv Jain</t>
         </is>
       </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>2026-03-24</t>
+          <t>2026-03-25</t>
         </is>
       </c>
       <c r="B39" t="n">
@@ -4340,19 +5377,19 @@
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>Jo Tum Mere Ho</t>
+          <t>Run Down The City - Monica</t>
         </is>
       </c>
       <c r="D39" t="inlineStr">
         <is>
-          <t>Anuv Jain</t>
+          <t>Shashwat Sachdev, Reble, Asha Bhosle, R. D. Burman, Majrooh Sultanpuri</t>
         </is>
       </c>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>2026-03-24</t>
+          <t>2026-03-25</t>
         </is>
       </c>
       <c r="B40" t="n">
@@ -4360,19 +5397,19 @@
       </c>
       <c r="C40" t="inlineStr">
         <is>
-          <t>Main Aur Tu (From "Dhurandhar The Revenge")</t>
+          <t>Jogi</t>
         </is>
       </c>
       <c r="D40" t="inlineStr">
         <is>
-          <t>Shashwat Sachdev, Jasmine Sandlas, Reble</t>
+          <t>thiarajxtt, Bir</t>
         </is>
       </c>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>2026-03-24</t>
+          <t>2026-03-25</t>
         </is>
       </c>
       <c r="B41" t="n">
@@ -4380,19 +5417,19 @@
       </c>
       <c r="C41" t="inlineStr">
         <is>
-          <t>Darkhaast</t>
+          <t>Haseen</t>
         </is>
       </c>
       <c r="D41" t="inlineStr">
         <is>
-          <t>Mithoon, Arijit Singh, Sunidhi Chauhan, Sayeed Quadri</t>
+          <t>Talwiinder, NDS, Rippy Grewal</t>
         </is>
       </c>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>2026-03-24</t>
+          <t>2026-03-25</t>
         </is>
       </c>
       <c r="B42" t="n">
@@ -4400,19 +5437,19 @@
       </c>
       <c r="C42" t="inlineStr">
         <is>
-          <t>Run Down The City - Monica</t>
+          <t>Agar Tum Saath Ho (From "Tamasha")</t>
         </is>
       </c>
       <c r="D42" t="inlineStr">
         <is>
-          <t>Shashwat Sachdev, Reble, Asha Bhosle, R. D. Burman, Majrooh Sultanpuri</t>
+          <t>Alka Yagnik, Arijit Singh</t>
         </is>
       </c>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>2026-03-24</t>
+          <t>2026-03-25</t>
         </is>
       </c>
       <c r="B43" t="n">
@@ -4420,19 +5457,19 @@
       </c>
       <c r="C43" t="inlineStr">
         <is>
-          <t>Mutta Kalakki (From "Youth")</t>
+          <t>Tere Bina</t>
         </is>
       </c>
       <c r="D43" t="inlineStr">
         <is>
-          <t>G. V. Prakash, Ken Karunaas</t>
+          <t>A.R. Rahman, Chinmayi, Murtuza Khan, Qadir Khan</t>
         </is>
       </c>
     </row>
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>2026-03-24</t>
+          <t>2026-03-25</t>
         </is>
       </c>
       <c r="B44" t="n">
@@ -4452,7 +5489,7 @@
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>2026-03-24</t>
+          <t>2026-03-25</t>
         </is>
       </c>
       <c r="B45" t="n">
@@ -4460,19 +5497,19 @@
       </c>
       <c r="C45" t="inlineStr">
         <is>
-          <t>Ye Tune Kya Kiya</t>
+          <t>Not Guilty</t>
         </is>
       </c>
       <c r="D45" t="inlineStr">
         <is>
-          <t>Pritam, Javed Bashir, Rajat Arora</t>
+          <t>Dhanda Nyoliwala</t>
         </is>
       </c>
     </row>
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>2026-03-24</t>
+          <t>2026-03-25</t>
         </is>
       </c>
       <c r="B46" t="n">
@@ -4480,19 +5517,19 @@
       </c>
       <c r="C46" t="inlineStr">
         <is>
-          <t>Phir Se (From "Dhurandhar The Revenge")</t>
+          <t>Mutta Kalakki (From "Youth")</t>
         </is>
       </c>
       <c r="D46" t="inlineStr">
         <is>
-          <t>Shashwat Sachdev, Arijit Singh, Irshad Kamil</t>
+          <t>G. V. Prakash, Ken Karunaas</t>
         </is>
       </c>
     </row>
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>2026-03-24</t>
+          <t>2026-03-25</t>
         </is>
       </c>
       <c r="B47" t="n">
@@ -4500,19 +5537,19 @@
       </c>
       <c r="C47" t="inlineStr">
         <is>
-          <t>Not Guilty</t>
+          <t>Ehsaas</t>
         </is>
       </c>
       <c r="D47" t="inlineStr">
         <is>
-          <t>Dhanda Nyoliwala</t>
+          <t>Faheem Abdullah, Duha Shah, Vaibhav Pani, Hyder Dar</t>
         </is>
       </c>
     </row>
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>2026-03-24</t>
+          <t>2026-03-25</t>
         </is>
       </c>
       <c r="B48" t="n">
@@ -4520,19 +5557,19 @@
       </c>
       <c r="C48" t="inlineStr">
         <is>
-          <t>Ehsaas</t>
+          <t>Ye Tune Kya Kiya</t>
         </is>
       </c>
       <c r="D48" t="inlineStr">
         <is>
-          <t>Faheem Abdullah, Duha Shah, Vaibhav Pani, Hyder Dar</t>
+          <t>Pritam, Javed Bashir, Rajat Arora</t>
         </is>
       </c>
     </row>
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>2026-03-24</t>
+          <t>2026-03-25</t>
         </is>
       </c>
       <c r="B49" t="n">
@@ -4540,19 +5577,19 @@
       </c>
       <c r="C49" t="inlineStr">
         <is>
-          <t>Mast Magan (From "2 States)</t>
+          <t>Thodi Si Daaru</t>
         </is>
       </c>
       <c r="D49" t="inlineStr">
         <is>
-          <t>Arijit Singh, Chinmayi</t>
+          <t>AP Dhillon, Shreya Ghoshal</t>
         </is>
       </c>
     </row>
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>2026-03-24</t>
+          <t>2026-03-25</t>
         </is>
       </c>
       <c r="B50" t="n">
@@ -4560,19 +5597,19 @@
       </c>
       <c r="C50" t="inlineStr">
         <is>
-          <t>Thodi Si Daaru</t>
+          <t>Teri Deewani</t>
         </is>
       </c>
       <c r="D50" t="inlineStr">
         <is>
-          <t>AP Dhillon, Shreya Ghoshal</t>
+          <t>Kailash Kher, Paresh Kamath, Naresh Kamath</t>
         </is>
       </c>
     </row>
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>2026-03-24</t>
+          <t>2026-03-25</t>
         </is>
       </c>
       <c r="B51" t="n">
@@ -4580,12 +5617,12 @@
       </c>
       <c r="C51" t="inlineStr">
         <is>
-          <t>Dhun (From "Saiyaara")</t>
+          <t>Mast Magan (From "2 States)</t>
         </is>
       </c>
       <c r="D51" t="inlineStr">
         <is>
-          <t>Mithoon, Arijit Singh</t>
+          <t>Arijit Singh, Chinmayi</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
added data for 26th and got predictions for 27th march
</commit_message>
<xml_diff>
--- a/Probability Project.xlsx
+++ b/Probability Project.xlsx
@@ -15,6 +15,7 @@
     <sheet name="AUTO_20260323" sheetId="10" state="visible" r:id="rId10"/>
     <sheet name="AUTO_20260324" sheetId="11" state="visible" r:id="rId11"/>
     <sheet name="AUTO_20260325" sheetId="12" state="visible" r:id="rId12"/>
+    <sheet name="AUTO_20260326" sheetId="13" state="visible" r:id="rId13"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -4627,9 +4628,1045 @@
       </c>
     </row>
     <row r="2">
+      <c r="A2" s="0" t="inlineStr">
+        <is>
+          <t>2026-03-25</t>
+        </is>
+      </c>
+      <c r="B2" s="0" t="n">
+        <v>1</v>
+      </c>
+      <c r="C2" s="0" t="inlineStr">
+        <is>
+          <t>Bairan</t>
+        </is>
+      </c>
+      <c r="D2" s="0" t="inlineStr">
+        <is>
+          <t>Banjaare</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="0" t="inlineStr">
+        <is>
+          <t>2026-03-25</t>
+        </is>
+      </c>
+      <c r="B3" s="0" t="n">
+        <v>2</v>
+      </c>
+      <c r="C3" s="0" t="inlineStr">
+        <is>
+          <t>Jaiye Sajana</t>
+        </is>
+      </c>
+      <c r="D3" s="0" t="inlineStr">
+        <is>
+          <t>Shashwat Sachdev, Jasmine Sandlas, Satinder Sartaaj</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="0" t="inlineStr">
+        <is>
+          <t>2026-03-25</t>
+        </is>
+      </c>
+      <c r="B4" s="0" t="n">
+        <v>3</v>
+      </c>
+      <c r="C4" s="0" t="inlineStr">
+        <is>
+          <t>Sheesha - Aakhya Mai Aakh Ghali Jo Bairan</t>
+        </is>
+      </c>
+      <c r="D4" s="0" t="inlineStr">
+        <is>
+          <t>Mitta Ror, Swara Verma</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="0" t="inlineStr">
+        <is>
+          <t>2026-03-25</t>
+        </is>
+      </c>
+      <c r="B5" s="0" t="n">
+        <v>4</v>
+      </c>
+      <c r="C5" s="0" t="inlineStr">
+        <is>
+          <t>Gehra Hua</t>
+        </is>
+      </c>
+      <c r="D5" s="0" t="inlineStr">
+        <is>
+          <t>Shashwat Sachdev, Arijit Singh, Irshad Kamil, Armaan Khan</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="0" t="inlineStr">
+        <is>
+          <t>2026-03-25</t>
+        </is>
+      </c>
+      <c r="B6" s="0" t="n">
+        <v>5</v>
+      </c>
+      <c r="C6" s="0" t="inlineStr">
+        <is>
+          <t>Dhurandhar The Revenge - Aari Aari</t>
+        </is>
+      </c>
+      <c r="D6" s="0" t="inlineStr">
+        <is>
+          <t>Shashwat Sachdev, Bombay Rockers, Irshad Kamil, Khan Saab, Reble, Token, Jasmine Sandlas, Sudhir Yaduvanshi</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="0" t="inlineStr">
+        <is>
+          <t>2026-03-25</t>
+        </is>
+      </c>
+      <c r="B7" s="0" t="n">
+        <v>6</v>
+      </c>
+      <c r="C7" s="0" t="inlineStr">
+        <is>
+          <t>Khat</t>
+        </is>
+      </c>
+      <c r="D7" s="0" t="inlineStr">
+        <is>
+          <t>Navjot Ahuja</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="0" t="inlineStr">
+        <is>
+          <t>2026-03-25</t>
+        </is>
+      </c>
+      <c r="B8" s="0" t="n">
+        <v>7</v>
+      </c>
+      <c r="C8" s="0" t="inlineStr">
+        <is>
+          <t>Jaan Se Guzarte Hain</t>
+        </is>
+      </c>
+      <c r="D8" s="0" t="inlineStr">
+        <is>
+          <t>Shashwat Sachdev, Khan Saab</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="0" t="inlineStr">
+        <is>
+          <t>2026-03-25</t>
+        </is>
+      </c>
+      <c r="B9" s="0" t="n">
+        <v>8</v>
+      </c>
+      <c r="C9" s="0" t="inlineStr">
+        <is>
+          <t>Dooron Dooron</t>
+        </is>
+      </c>
+      <c r="D9" s="0" t="inlineStr">
+        <is>
+          <t>Paresh Pahuja, Shiv Tandan, Meghdeep Bose</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="0" t="inlineStr">
+        <is>
+          <t>2026-03-25</t>
+        </is>
+      </c>
+      <c r="B10" s="0" t="n">
+        <v>9</v>
+      </c>
+      <c r="C10" s="0" t="inlineStr">
+        <is>
+          <t>Sitaare (From "Ikkis")</t>
+        </is>
+      </c>
+      <c r="D10" s="0" t="inlineStr">
+        <is>
+          <t>Arijit Singh, White Noise Collectives, Amitabh Bhattacharya</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="0" t="inlineStr">
+        <is>
+          <t>2026-03-25</t>
+        </is>
+      </c>
+      <c r="B11" s="0" t="n">
+        <v>10</v>
+      </c>
+      <c r="C11" s="0" t="inlineStr">
+        <is>
+          <t>Sahiba</t>
+        </is>
+      </c>
+      <c r="D11" s="0" t="inlineStr">
+        <is>
+          <t>Aditya Rikhari</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="0" t="inlineStr">
+        <is>
+          <t>2026-03-25</t>
+        </is>
+      </c>
+      <c r="B12" s="0" t="n">
+        <v>11</v>
+      </c>
+      <c r="C12" s="0" t="inlineStr">
+        <is>
+          <t>Finding Her</t>
+        </is>
+      </c>
+      <c r="D12" s="0" t="inlineStr">
+        <is>
+          <t>Kushagra, Bharath, Saaheal</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="0" t="inlineStr">
+        <is>
+          <t>2026-03-25</t>
+        </is>
+      </c>
+      <c r="B13" s="0" t="n">
+        <v>12</v>
+      </c>
+      <c r="C13" s="0" t="inlineStr">
+        <is>
+          <t>Apna Bana Le</t>
+        </is>
+      </c>
+      <c r="D13" s="0" t="inlineStr">
+        <is>
+          <t>Sachin-Jigar, Arijit Singh, Amitabh Bhattacharya</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="0" t="inlineStr">
+        <is>
+          <t>2026-03-25</t>
+        </is>
+      </c>
+      <c r="B14" s="0" t="n">
+        <v>13</v>
+      </c>
+      <c r="C14" s="0" t="inlineStr">
+        <is>
+          <t>Shararat</t>
+        </is>
+      </c>
+      <c r="D14" s="0" t="inlineStr">
+        <is>
+          <t>Shashwat Sachdev, Madhubanti Bagchi, Jasmine Sandlas</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="0" t="inlineStr">
+        <is>
+          <t>2026-03-25</t>
+        </is>
+      </c>
+      <c r="B15" s="0" t="n">
+        <v>14</v>
+      </c>
+      <c r="C15" s="0" t="inlineStr">
+        <is>
+          <t>Samjhawan</t>
+        </is>
+      </c>
+      <c r="D15" s="0" t="inlineStr">
+        <is>
+          <t>Jawad Ahmad, Shaarib Toshi, Arijit Singh, Shreya Ghoshal</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="0" t="inlineStr">
+        <is>
+          <t>2026-03-25</t>
+        </is>
+      </c>
+      <c r="B16" s="0" t="n">
+        <v>15</v>
+      </c>
+      <c r="C16" s="0" t="inlineStr">
+        <is>
+          <t>Dhurandhar - Title Track</t>
+        </is>
+      </c>
+      <c r="D16" s="0" t="inlineStr">
+        <is>
+          <t>Shashwat Sachdev, Hanumankind, Jasmine Sandlas, Sudhir Yaduvanshi, Charanjit Ahuja, Muhammad Sadiq, Ranjit Kaur, Babu Singh Maan</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="0" t="inlineStr">
+        <is>
+          <t>2026-03-25</t>
+        </is>
+      </c>
+      <c r="B17" s="0" t="n">
+        <v>16</v>
+      </c>
+      <c r="C17" s="0" t="inlineStr">
+        <is>
+          <t>Arz Kiya Hai | Coke Studio Bharat</t>
+        </is>
+      </c>
+      <c r="D17" s="0" t="inlineStr">
+        <is>
+          <t>Anuv Jain</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="0" t="inlineStr">
+        <is>
+          <t>2026-03-25</t>
+        </is>
+      </c>
+      <c r="B18" s="0" t="n">
+        <v>17</v>
+      </c>
+      <c r="C18" s="0" t="inlineStr">
+        <is>
+          <t>Ishqa Ve</t>
+        </is>
+      </c>
+      <c r="D18" s="0" t="inlineStr">
+        <is>
+          <t>Zeeshan Ali, Yuvraj Tung, Sandeep Aulakh, Honey Dhillon</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="0" t="inlineStr">
+        <is>
+          <t>2026-03-25</t>
+        </is>
+      </c>
+      <c r="B19" s="0" t="n">
+        <v>18</v>
+      </c>
+      <c r="C19" s="0" t="inlineStr">
+        <is>
+          <t>For A Reason</t>
+        </is>
+      </c>
+      <c r="D19" s="0" t="inlineStr">
+        <is>
+          <t>Karan Aujla, Ikky</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="0" t="inlineStr">
+        <is>
+          <t>2026-03-25</t>
+        </is>
+      </c>
+      <c r="B20" s="0" t="n">
+        <v>19</v>
+      </c>
+      <c r="C20" s="0" t="inlineStr">
+        <is>
+          <t>Boyfriend</t>
+        </is>
+      </c>
+      <c r="D20" s="0" t="inlineStr">
+        <is>
+          <t>Karan Aujla, Ikky</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="0" t="inlineStr">
+        <is>
+          <t>2026-03-25</t>
+        </is>
+      </c>
+      <c r="B21" s="0" t="n">
+        <v>20</v>
+      </c>
+      <c r="C21" s="0" t="inlineStr">
+        <is>
+          <t>Pavazha Malli - From "Think Indie"</t>
+        </is>
+      </c>
+      <c r="D21" s="0" t="inlineStr">
+        <is>
+          <t>Sai Abhyankkar, Shruti Haasan, Vivek</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="0" t="inlineStr">
+        <is>
+          <t>2026-03-25</t>
+        </is>
+      </c>
+      <c r="B22" s="0" t="n">
+        <v>21</v>
+      </c>
+      <c r="C22" s="0" t="inlineStr">
+        <is>
+          <t>Mann Mera</t>
+        </is>
+      </c>
+      <c r="D22" s="0" t="inlineStr">
+        <is>
+          <t>Gajendra Verma</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="0" t="inlineStr">
+        <is>
+          <t>2026-03-25</t>
+        </is>
+      </c>
+      <c r="B23" s="0" t="n">
+        <v>22</v>
+      </c>
+      <c r="C23" s="0" t="inlineStr">
+        <is>
+          <t>Bairi</t>
+        </is>
+      </c>
+      <c r="D23" s="0" t="inlineStr">
+        <is>
+          <t>Virat, Pradeep Solanki, Heena</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="0" t="inlineStr">
+        <is>
+          <t>2026-03-25</t>
+        </is>
+      </c>
+      <c r="B24" s="0" t="n">
+        <v>23</v>
+      </c>
+      <c r="C24" s="0" t="inlineStr">
+        <is>
+          <t>Ishq</t>
+        </is>
+      </c>
+      <c r="D24" s="0" t="inlineStr">
+        <is>
+          <t>Faheem Abdullah, Rauhan Malik, Amir Ameer</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="0" t="inlineStr">
+        <is>
+          <t>2026-03-25</t>
+        </is>
+      </c>
+      <c r="B25" s="0" t="n">
+        <v>24</v>
+      </c>
+      <c r="C25" s="0" t="inlineStr">
+        <is>
+          <t>Saiyaara</t>
+        </is>
+      </c>
+      <c r="D25" s="0" t="inlineStr">
+        <is>
+          <t>Tanishk Bagchi, Faheem Abdullah, Arslan Nizami, Irshad Kamil</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="0" t="inlineStr">
+        <is>
+          <t>2026-03-25</t>
+        </is>
+      </c>
+      <c r="B26" s="0" t="n">
+        <v>25</v>
+      </c>
+      <c r="C26" s="0" t="inlineStr">
+        <is>
+          <t>Naal Nachna</t>
+        </is>
+      </c>
+      <c r="D26" s="0" t="inlineStr">
+        <is>
+          <t>Shashwat Sachdev, Afsana Khan, Irshad Kamil, Reble</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="0" t="inlineStr">
+        <is>
+          <t>2026-03-25</t>
+        </is>
+      </c>
+      <c r="B27" s="0" t="n">
+        <v>26</v>
+      </c>
+      <c r="C27" s="0" t="inlineStr">
+        <is>
+          <t>SWIM</t>
+        </is>
+      </c>
+      <c r="D27" s="0" t="inlineStr">
+        <is>
+          <t>BTS</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="0" t="inlineStr">
+        <is>
+          <t>2026-03-25</t>
+        </is>
+      </c>
+      <c r="B28" s="0" t="n">
+        <v>27</v>
+      </c>
+      <c r="C28" s="0" t="inlineStr">
+        <is>
+          <t>Raanjhan (From "Do Patti")</t>
+        </is>
+      </c>
+      <c r="D28" s="0" t="inlineStr">
+        <is>
+          <t>Sachet-Parampara, Parampara Tandon, Kausar Munir</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="0" t="inlineStr">
+        <is>
+          <t>2026-03-25</t>
+        </is>
+      </c>
+      <c r="B29" s="0" t="n">
+        <v>28</v>
+      </c>
+      <c r="C29" s="0" t="inlineStr">
+        <is>
+          <t>Phir Se</t>
+        </is>
+      </c>
+      <c r="D29" s="0" t="inlineStr">
+        <is>
+          <t>Shashwat Sachdev, Arijit Singh, Irshad Kamil</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="0" t="inlineStr">
+        <is>
+          <t>2026-03-25</t>
+        </is>
+      </c>
+      <c r="B30" s="0" t="n">
+        <v>29</v>
+      </c>
+      <c r="C30" s="0" t="inlineStr">
+        <is>
+          <t>Main Aur Tu</t>
+        </is>
+      </c>
+      <c r="D30" s="0" t="inlineStr">
+        <is>
+          <t>Shashwat Sachdev, Jasmine Sandlas, Reble</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="0" t="inlineStr">
+        <is>
+          <t>2026-03-25</t>
+        </is>
+      </c>
+      <c r="B31" s="0" t="n">
+        <v>30</v>
+      </c>
+      <c r="C31" s="0" t="inlineStr">
+        <is>
+          <t>Deewaana Deewaana</t>
+        </is>
+      </c>
+      <c r="D31" s="0" t="inlineStr">
+        <is>
+          <t>A.R. Rahman, Irshad Kamil</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="0" t="inlineStr">
+        <is>
+          <t>2026-03-25</t>
+        </is>
+      </c>
+      <c r="B32" s="0" t="n">
+        <v>31</v>
+      </c>
+      <c r="C32" s="0" t="inlineStr">
+        <is>
+          <t>Lutt Le Gaya</t>
+        </is>
+      </c>
+      <c r="D32" s="0" t="inlineStr">
+        <is>
+          <t>Shashwat Sachdev, Simran Choudhary</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="0" t="inlineStr">
+        <is>
+          <t>2026-03-25</t>
+        </is>
+      </c>
+      <c r="B33" s="0" t="n">
+        <v>32</v>
+      </c>
+      <c r="C33" s="0" t="inlineStr">
+        <is>
+          <t>Tum Ho Toh (From "Saiyaara")</t>
+        </is>
+      </c>
+      <c r="D33" s="0" t="inlineStr">
+        <is>
+          <t>Vishal Mishra, Hansika Pareek, Raj Shekhar</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="0" t="inlineStr">
+        <is>
+          <t>2026-03-25</t>
+        </is>
+      </c>
+      <c r="B34" s="0" t="n">
+        <v>33</v>
+      </c>
+      <c r="C34" s="0" t="inlineStr">
+        <is>
+          <t>Darkhaast</t>
+        </is>
+      </c>
+      <c r="D34" s="0" t="inlineStr">
+        <is>
+          <t>Mithoon, Arijit Singh, Sunidhi Chauhan, Sayeed Quadri</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="0" t="inlineStr">
+        <is>
+          <t>2026-03-25</t>
+        </is>
+      </c>
+      <c r="B35" s="0" t="n">
+        <v>34</v>
+      </c>
+      <c r="C35" s="0" t="inlineStr">
+        <is>
+          <t>Tere Liye</t>
+        </is>
+      </c>
+      <c r="D35" s="0" t="inlineStr">
+        <is>
+          <t>Atif Aslam, Shreya Ghoshal, Sachin Gupta, Sameer Anjaan</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="0" t="inlineStr">
+        <is>
+          <t>2026-03-25</t>
+        </is>
+      </c>
+      <c r="B36" s="0" t="n">
+        <v>35</v>
+      </c>
+      <c r="C36" s="0" t="inlineStr">
+        <is>
+          <t>Ishq Jalakar - Karvaan</t>
+        </is>
+      </c>
+      <c r="D36" s="0" t="inlineStr">
+        <is>
+          <t>Shashwat Sachdev, Shahzad Ali, Subhadeep Das Chowdhury, Armaan Khan, Irshad Kamil, Roshan, Sahir Ludhianvi</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="0" t="inlineStr">
+        <is>
+          <t>2026-03-25</t>
+        </is>
+      </c>
+      <c r="B37" s="0" t="n">
+        <v>36</v>
+      </c>
+      <c r="C37" s="0" t="inlineStr">
+        <is>
+          <t>Aaya Sher (From "The Paradise") (Telugu)</t>
+        </is>
+      </c>
+      <c r="D37" s="0" t="inlineStr">
+        <is>
+          <t>Anirudh Ravichander, Jangi Reddy, Arjun Chandy, Kasarla Shyam</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="0" t="inlineStr">
+        <is>
+          <t>2026-03-25</t>
+        </is>
+      </c>
+      <c r="B38" s="0" t="n">
+        <v>37</v>
+      </c>
+      <c r="C38" s="0" t="inlineStr">
+        <is>
+          <t>Jo Tum Mere Ho</t>
+        </is>
+      </c>
+      <c r="D38" s="0" t="inlineStr">
+        <is>
+          <t>Anuv Jain</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="0" t="inlineStr">
+        <is>
+          <t>2026-03-25</t>
+        </is>
+      </c>
+      <c r="B39" s="0" t="n">
+        <v>38</v>
+      </c>
+      <c r="C39" s="0" t="inlineStr">
+        <is>
+          <t>Run Down The City - Monica</t>
+        </is>
+      </c>
+      <c r="D39" s="0" t="inlineStr">
+        <is>
+          <t>Shashwat Sachdev, Reble, Asha Bhosle, R. D. Burman, Majrooh Sultanpuri</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="0" t="inlineStr">
+        <is>
+          <t>2026-03-25</t>
+        </is>
+      </c>
+      <c r="B40" s="0" t="n">
+        <v>39</v>
+      </c>
+      <c r="C40" s="0" t="inlineStr">
+        <is>
+          <t>Jogi</t>
+        </is>
+      </c>
+      <c r="D40" s="0" t="inlineStr">
+        <is>
+          <t>thiarajxtt, Bir</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" s="0" t="inlineStr">
+        <is>
+          <t>2026-03-25</t>
+        </is>
+      </c>
+      <c r="B41" s="0" t="n">
+        <v>40</v>
+      </c>
+      <c r="C41" s="0" t="inlineStr">
+        <is>
+          <t>Haseen</t>
+        </is>
+      </c>
+      <c r="D41" s="0" t="inlineStr">
+        <is>
+          <t>Talwiinder, NDS, Rippy Grewal</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" s="0" t="inlineStr">
+        <is>
+          <t>2026-03-25</t>
+        </is>
+      </c>
+      <c r="B42" s="0" t="n">
+        <v>41</v>
+      </c>
+      <c r="C42" s="0" t="inlineStr">
+        <is>
+          <t>Agar Tum Saath Ho (From "Tamasha")</t>
+        </is>
+      </c>
+      <c r="D42" s="0" t="inlineStr">
+        <is>
+          <t>Alka Yagnik, Arijit Singh</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" s="0" t="inlineStr">
+        <is>
+          <t>2026-03-25</t>
+        </is>
+      </c>
+      <c r="B43" s="0" t="n">
+        <v>42</v>
+      </c>
+      <c r="C43" s="0" t="inlineStr">
+        <is>
+          <t>Tere Bina</t>
+        </is>
+      </c>
+      <c r="D43" s="0" t="inlineStr">
+        <is>
+          <t>A.R. Rahman, Chinmayi, Murtuza Khan, Qadir Khan</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" s="0" t="inlineStr">
+        <is>
+          <t>2026-03-25</t>
+        </is>
+      </c>
+      <c r="B44" s="0" t="n">
+        <v>43</v>
+      </c>
+      <c r="C44" s="0" t="inlineStr">
+        <is>
+          <t>Barbaad (From "Saiyaara")</t>
+        </is>
+      </c>
+      <c r="D44" s="0" t="inlineStr">
+        <is>
+          <t>The Rish, Jubin Nautiyal</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" s="0" t="inlineStr">
+        <is>
+          <t>2026-03-25</t>
+        </is>
+      </c>
+      <c r="B45" s="0" t="n">
+        <v>44</v>
+      </c>
+      <c r="C45" s="0" t="inlineStr">
+        <is>
+          <t>Not Guilty</t>
+        </is>
+      </c>
+      <c r="D45" s="0" t="inlineStr">
+        <is>
+          <t>Dhanda Nyoliwala</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" s="0" t="inlineStr">
+        <is>
+          <t>2026-03-25</t>
+        </is>
+      </c>
+      <c r="B46" s="0" t="n">
+        <v>45</v>
+      </c>
+      <c r="C46" s="0" t="inlineStr">
+        <is>
+          <t>Mutta Kalakki (From "Youth")</t>
+        </is>
+      </c>
+      <c r="D46" s="0" t="inlineStr">
+        <is>
+          <t>G. V. Prakash, Ken Karunaas</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" s="0" t="inlineStr">
+        <is>
+          <t>2026-03-25</t>
+        </is>
+      </c>
+      <c r="B47" s="0" t="n">
+        <v>46</v>
+      </c>
+      <c r="C47" s="0" t="inlineStr">
+        <is>
+          <t>Ehsaas</t>
+        </is>
+      </c>
+      <c r="D47" s="0" t="inlineStr">
+        <is>
+          <t>Faheem Abdullah, Duha Shah, Vaibhav Pani, Hyder Dar</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" s="0" t="inlineStr">
+        <is>
+          <t>2026-03-25</t>
+        </is>
+      </c>
+      <c r="B48" s="0" t="n">
+        <v>47</v>
+      </c>
+      <c r="C48" s="0" t="inlineStr">
+        <is>
+          <t>Ye Tune Kya Kiya</t>
+        </is>
+      </c>
+      <c r="D48" s="0" t="inlineStr">
+        <is>
+          <t>Pritam, Javed Bashir, Rajat Arora</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" s="0" t="inlineStr">
+        <is>
+          <t>2026-03-25</t>
+        </is>
+      </c>
+      <c r="B49" s="0" t="n">
+        <v>48</v>
+      </c>
+      <c r="C49" s="0" t="inlineStr">
+        <is>
+          <t>Thodi Si Daaru</t>
+        </is>
+      </c>
+      <c r="D49" s="0" t="inlineStr">
+        <is>
+          <t>AP Dhillon, Shreya Ghoshal</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" s="0" t="inlineStr">
+        <is>
+          <t>2026-03-25</t>
+        </is>
+      </c>
+      <c r="B50" s="0" t="n">
+        <v>49</v>
+      </c>
+      <c r="C50" s="0" t="inlineStr">
+        <is>
+          <t>Teri Deewani</t>
+        </is>
+      </c>
+      <c r="D50" s="0" t="inlineStr">
+        <is>
+          <t>Kailash Kher, Paresh Kamath, Naresh Kamath</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" s="0" t="inlineStr">
+        <is>
+          <t>2026-03-25</t>
+        </is>
+      </c>
+      <c r="B51" s="0" t="n">
+        <v>50</v>
+      </c>
+      <c r="C51" s="0" t="inlineStr">
+        <is>
+          <t>Mast Magan (From "2 States)</t>
+        </is>
+      </c>
+      <c r="D51" s="0" t="inlineStr">
+        <is>
+          <t>Arijit Singh, Chinmayi</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet13.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:D51"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="24" t="inlineStr">
+        <is>
+          <t>Date</t>
+        </is>
+      </c>
+      <c r="B1" s="24" t="inlineStr">
+        <is>
+          <t>Rank</t>
+        </is>
+      </c>
+      <c r="C1" s="24" t="inlineStr">
+        <is>
+          <t>Song</t>
+        </is>
+      </c>
+      <c r="D1" s="24" t="inlineStr">
+        <is>
+          <t>Artist</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>2026-03-25</t>
+          <t>2026-03-26</t>
         </is>
       </c>
       <c r="B2" t="n">
@@ -4649,7 +5686,7 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>2026-03-25</t>
+          <t>2026-03-26</t>
         </is>
       </c>
       <c r="B3" t="n">
@@ -4669,7 +5706,7 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>2026-03-25</t>
+          <t>2026-03-26</t>
         </is>
       </c>
       <c r="B4" t="n">
@@ -4689,7 +5726,7 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>2026-03-25</t>
+          <t>2026-03-26</t>
         </is>
       </c>
       <c r="B5" t="n">
@@ -4709,7 +5746,7 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>2026-03-25</t>
+          <t>2026-03-26</t>
         </is>
       </c>
       <c r="B6" t="n">
@@ -4729,7 +5766,7 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>2026-03-25</t>
+          <t>2026-03-26</t>
         </is>
       </c>
       <c r="B7" t="n">
@@ -4737,19 +5774,19 @@
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>Khat</t>
+          <t>Jaan Se Guzarte Hain</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>Navjot Ahuja</t>
+          <t>Shashwat Sachdev, Khan Saab, Nusrat Fateh Ali Khan</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>2026-03-25</t>
+          <t>2026-03-26</t>
         </is>
       </c>
       <c r="B8" t="n">
@@ -4757,19 +5794,19 @@
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>Jaan Se Guzarte Hain</t>
+          <t>Khat</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>Shashwat Sachdev, Khan Saab</t>
+          <t>Navjot Ahuja</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>2026-03-25</t>
+          <t>2026-03-26</t>
         </is>
       </c>
       <c r="B9" t="n">
@@ -4789,7 +5826,7 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>2026-03-25</t>
+          <t>2026-03-26</t>
         </is>
       </c>
       <c r="B10" t="n">
@@ -4809,7 +5846,7 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>2026-03-25</t>
+          <t>2026-03-26</t>
         </is>
       </c>
       <c r="B11" t="n">
@@ -4829,7 +5866,7 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>2026-03-25</t>
+          <t>2026-03-26</t>
         </is>
       </c>
       <c r="B12" t="n">
@@ -4837,19 +5874,19 @@
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>Finding Her</t>
+          <t>Apna Bana Le</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>Kushagra, Bharath, Saaheal</t>
+          <t>Sachin-Jigar, Arijit Singh, Amitabh Bhattacharya</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>2026-03-25</t>
+          <t>2026-03-26</t>
         </is>
       </c>
       <c r="B13" t="n">
@@ -4857,19 +5894,19 @@
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>Apna Bana Le</t>
+          <t>Samjhawan</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>Sachin-Jigar, Arijit Singh, Amitabh Bhattacharya</t>
+          <t>Jawad Ahmad, Shaarib Toshi, Arijit Singh, Shreya Ghoshal</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>2026-03-25</t>
+          <t>2026-03-26</t>
         </is>
       </c>
       <c r="B14" t="n">
@@ -4877,19 +5914,19 @@
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>Shararat</t>
+          <t>Finding Her</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>Shashwat Sachdev, Madhubanti Bagchi, Jasmine Sandlas</t>
+          <t>Kushagra, Bharath, Saaheal</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>2026-03-25</t>
+          <t>2026-03-26</t>
         </is>
       </c>
       <c r="B15" t="n">
@@ -4897,19 +5934,19 @@
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>Samjhawan</t>
+          <t>Shararat</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>Jawad Ahmad, Shaarib Toshi, Arijit Singh, Shreya Ghoshal</t>
+          <t>Shashwat Sachdev, Madhubanti Bagchi, Jasmine Sandlas</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>2026-03-25</t>
+          <t>2026-03-26</t>
         </is>
       </c>
       <c r="B16" t="n">
@@ -4929,7 +5966,7 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>2026-03-25</t>
+          <t>2026-03-26</t>
         </is>
       </c>
       <c r="B17" t="n">
@@ -4949,7 +5986,7 @@
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>2026-03-25</t>
+          <t>2026-03-26</t>
         </is>
       </c>
       <c r="B18" t="n">
@@ -4957,19 +5994,19 @@
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>Ishqa Ve</t>
+          <t>Pavazha Malli - From "Think Indie"</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>Zeeshan Ali, Yuvraj Tung, Sandeep Aulakh, Honey Dhillon</t>
+          <t>Sai Abhyankkar, Shruti Haasan, Vivek</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>2026-03-25</t>
+          <t>2026-03-26</t>
         </is>
       </c>
       <c r="B19" t="n">
@@ -4977,19 +6014,19 @@
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>For A Reason</t>
+          <t>Ishq</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>Karan Aujla, Ikky</t>
+          <t>Faheem Abdullah, Rauhan Malik, Amir Ameer</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>2026-03-25</t>
+          <t>2026-03-26</t>
         </is>
       </c>
       <c r="B20" t="n">
@@ -4997,19 +6034,19 @@
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>Boyfriend</t>
+          <t>Mann Mera</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>Karan Aujla, Ikky</t>
+          <t>Gajendra Verma</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>2026-03-25</t>
+          <t>2026-03-26</t>
         </is>
       </c>
       <c r="B21" t="n">
@@ -5017,19 +6054,19 @@
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>Pavazha Malli - From "Think Indie"</t>
+          <t>For A Reason</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>Sai Abhyankkar, Shruti Haasan, Vivek</t>
+          <t>Karan Aujla, Ikky</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>2026-03-25</t>
+          <t>2026-03-26</t>
         </is>
       </c>
       <c r="B22" t="n">
@@ -5037,19 +6074,19 @@
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>Mann Mera</t>
+          <t>Boyfriend</t>
         </is>
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>Gajendra Verma</t>
+          <t>Karan Aujla, Ikky</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>2026-03-25</t>
+          <t>2026-03-26</t>
         </is>
       </c>
       <c r="B23" t="n">
@@ -5057,19 +6094,19 @@
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>Bairi</t>
+          <t>Phir Se</t>
         </is>
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>Virat, Pradeep Solanki, Heena</t>
+          <t>Shashwat Sachdev, Arijit Singh, Irshad Kamil</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>2026-03-25</t>
+          <t>2026-03-26</t>
         </is>
       </c>
       <c r="B24" t="n">
@@ -5077,19 +6114,19 @@
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>Ishq</t>
+          <t>Bairi</t>
         </is>
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>Faheem Abdullah, Rauhan Malik, Amir Ameer</t>
+          <t>Virat, Pradeep Solanki, Heena</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>2026-03-25</t>
+          <t>2026-03-26</t>
         </is>
       </c>
       <c r="B25" t="n">
@@ -5109,7 +6146,7 @@
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>2026-03-25</t>
+          <t>2026-03-26</t>
         </is>
       </c>
       <c r="B26" t="n">
@@ -5117,19 +6154,19 @@
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>Naal Nachna</t>
+          <t>Ishqa Ve</t>
         </is>
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>Shashwat Sachdev, Afsana Khan, Irshad Kamil, Reble</t>
+          <t>Zeeshan Ali, Yuvraj Tung, Sandeep Aulakh, Honey Dhillon</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>2026-03-25</t>
+          <t>2026-03-26</t>
         </is>
       </c>
       <c r="B27" t="n">
@@ -5137,19 +6174,19 @@
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>SWIM</t>
+          <t>Naal Nachna</t>
         </is>
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t>BTS</t>
+          <t>Shashwat Sachdev, Afsana Khan, Irshad Kamil, Reble</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>2026-03-25</t>
+          <t>2026-03-26</t>
         </is>
       </c>
       <c r="B28" t="n">
@@ -5157,19 +6194,19 @@
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>Raanjhan (From "Do Patti")</t>
+          <t>Main Aur Tu</t>
         </is>
       </c>
       <c r="D28" t="inlineStr">
         <is>
-          <t>Sachet-Parampara, Parampara Tandon, Kausar Munir</t>
+          <t>Jasmine Sandlas, Shashwat Sachdev, Reble</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>2026-03-25</t>
+          <t>2026-03-26</t>
         </is>
       </c>
       <c r="B29" t="n">
@@ -5177,19 +6214,19 @@
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>Phir Se</t>
+          <t>Raanjhan (From "Do Patti")</t>
         </is>
       </c>
       <c r="D29" t="inlineStr">
         <is>
-          <t>Shashwat Sachdev, Arijit Singh, Irshad Kamil</t>
+          <t>Sachet-Parampara, Parampara Tandon, Kausar Munir</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>2026-03-25</t>
+          <t>2026-03-26</t>
         </is>
       </c>
       <c r="B30" t="n">
@@ -5197,19 +6234,19 @@
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>Main Aur Tu</t>
+          <t>Deewaana Deewaana</t>
         </is>
       </c>
       <c r="D30" t="inlineStr">
         <is>
-          <t>Shashwat Sachdev, Jasmine Sandlas, Reble</t>
+          <t>A.R. Rahman, Irshad Kamil</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>2026-03-25</t>
+          <t>2026-03-26</t>
         </is>
       </c>
       <c r="B31" t="n">
@@ -5217,19 +6254,19 @@
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>Deewaana Deewaana</t>
+          <t>Tere Liye</t>
         </is>
       </c>
       <c r="D31" t="inlineStr">
         <is>
-          <t>A.R. Rahman, Irshad Kamil</t>
+          <t>Atif Aslam, Shreya Ghoshal, Sachin Gupta, Sameer Anjaan</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>2026-03-25</t>
+          <t>2026-03-26</t>
         </is>
       </c>
       <c r="B32" t="n">
@@ -5249,7 +6286,7 @@
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>2026-03-25</t>
+          <t>2026-03-26</t>
         </is>
       </c>
       <c r="B33" t="n">
@@ -5257,19 +6294,19 @@
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>Tum Ho Toh (From "Saiyaara")</t>
+          <t>SWIM</t>
         </is>
       </c>
       <c r="D33" t="inlineStr">
         <is>
-          <t>Vishal Mishra, Hansika Pareek, Raj Shekhar</t>
+          <t>BTS</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>2026-03-25</t>
+          <t>2026-03-26</t>
         </is>
       </c>
       <c r="B34" t="n">
@@ -5277,19 +6314,19 @@
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>Darkhaast</t>
+          <t>Jogi</t>
         </is>
       </c>
       <c r="D34" t="inlineStr">
         <is>
-          <t>Mithoon, Arijit Singh, Sunidhi Chauhan, Sayeed Quadri</t>
+          <t>thiarajxtt, Bir</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>2026-03-25</t>
+          <t>2026-03-26</t>
         </is>
       </c>
       <c r="B35" t="n">
@@ -5297,19 +6334,19 @@
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>Tere Liye</t>
+          <t>Ishq Jalakar - Karvaan</t>
         </is>
       </c>
       <c r="D35" t="inlineStr">
         <is>
-          <t>Atif Aslam, Shreya Ghoshal, Sachin Gupta, Sameer Anjaan</t>
+          <t>Shashwat Sachdev, Shahzad Ali, Subhadeep Das Chowdhury, Armaan Khan, Irshad Kamil, Roshan, Sahir Ludhianvi</t>
         </is>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>2026-03-25</t>
+          <t>2026-03-26</t>
         </is>
       </c>
       <c r="B36" t="n">
@@ -5317,19 +6354,19 @@
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>Ishq Jalakar - Karvaan</t>
+          <t>Aaya Sher (From "The Paradise") (Telugu)</t>
         </is>
       </c>
       <c r="D36" t="inlineStr">
         <is>
-          <t>Shashwat Sachdev, Shahzad Ali, Subhadeep Das Chowdhury, Armaan Khan, Irshad Kamil, Roshan, Sahir Ludhianvi</t>
+          <t>Anirudh Ravichander, Jangi Reddy, Arjun Chandy, Kasarla Shyam</t>
         </is>
       </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>2026-03-25</t>
+          <t>2026-03-26</t>
         </is>
       </c>
       <c r="B37" t="n">
@@ -5337,19 +6374,19 @@
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>Aaya Sher (From "The Paradise") (Telugu)</t>
+          <t>Tum Ho Toh (From "Saiyaara")</t>
         </is>
       </c>
       <c r="D37" t="inlineStr">
         <is>
-          <t>Anirudh Ravichander, Jangi Reddy, Arjun Chandy, Kasarla Shyam</t>
+          <t>Vishal Mishra, Hansika Pareek, Raj Shekhar</t>
         </is>
       </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>2026-03-25</t>
+          <t>2026-03-26</t>
         </is>
       </c>
       <c r="B38" t="n">
@@ -5357,19 +6394,19 @@
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>Jo Tum Mere Ho</t>
+          <t>Tere Bina</t>
         </is>
       </c>
       <c r="D38" t="inlineStr">
         <is>
-          <t>Anuv Jain</t>
+          <t>A.R. Rahman, Chinmayi, Murtuza Khan, Qadir Khan</t>
         </is>
       </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>2026-03-25</t>
+          <t>2026-03-26</t>
         </is>
       </c>
       <c r="B39" t="n">
@@ -5377,19 +6414,19 @@
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>Run Down The City - Monica</t>
+          <t>Jo Tum Mere Ho</t>
         </is>
       </c>
       <c r="D39" t="inlineStr">
         <is>
-          <t>Shashwat Sachdev, Reble, Asha Bhosle, R. D. Burman, Majrooh Sultanpuri</t>
+          <t>Anuv Jain</t>
         </is>
       </c>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>2026-03-25</t>
+          <t>2026-03-26</t>
         </is>
       </c>
       <c r="B40" t="n">
@@ -5397,19 +6434,19 @@
       </c>
       <c r="C40" t="inlineStr">
         <is>
-          <t>Jogi</t>
+          <t>Agar Tum Saath Ho (From "Tamasha")</t>
         </is>
       </c>
       <c r="D40" t="inlineStr">
         <is>
-          <t>thiarajxtt, Bir</t>
+          <t>Alka Yagnik, Arijit Singh</t>
         </is>
       </c>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>2026-03-25</t>
+          <t>2026-03-26</t>
         </is>
       </c>
       <c r="B41" t="n">
@@ -5417,19 +6454,19 @@
       </c>
       <c r="C41" t="inlineStr">
         <is>
-          <t>Haseen</t>
+          <t>Run Down The City - Monica</t>
         </is>
       </c>
       <c r="D41" t="inlineStr">
         <is>
-          <t>Talwiinder, NDS, Rippy Grewal</t>
+          <t>Shashwat Sachdev, Reble, Asha Bhosle, R. D. Burman, Majrooh Sultanpuri</t>
         </is>
       </c>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>2026-03-25</t>
+          <t>2026-03-26</t>
         </is>
       </c>
       <c r="B42" t="n">
@@ -5437,19 +6474,19 @@
       </c>
       <c r="C42" t="inlineStr">
         <is>
-          <t>Agar Tum Saath Ho (From "Tamasha")</t>
+          <t>Darkhaast</t>
         </is>
       </c>
       <c r="D42" t="inlineStr">
         <is>
-          <t>Alka Yagnik, Arijit Singh</t>
+          <t>Mithoon, Arijit Singh, Sunidhi Chauhan, Sayeed Quadri</t>
         </is>
       </c>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>2026-03-25</t>
+          <t>2026-03-26</t>
         </is>
       </c>
       <c r="B43" t="n">
@@ -5457,19 +6494,19 @@
       </c>
       <c r="C43" t="inlineStr">
         <is>
-          <t>Tere Bina</t>
+          <t>Haseen</t>
         </is>
       </c>
       <c r="D43" t="inlineStr">
         <is>
-          <t>A.R. Rahman, Chinmayi, Murtuza Khan, Qadir Khan</t>
+          <t>Talwiinder, NDS, Rippy Grewal</t>
         </is>
       </c>
     </row>
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>2026-03-25</t>
+          <t>2026-03-26</t>
         </is>
       </c>
       <c r="B44" t="n">
@@ -5477,19 +6514,19 @@
       </c>
       <c r="C44" t="inlineStr">
         <is>
-          <t>Barbaad (From "Saiyaara")</t>
+          <t>Mutta Kalakki (From "Youth")</t>
         </is>
       </c>
       <c r="D44" t="inlineStr">
         <is>
-          <t>The Rish, Jubin Nautiyal</t>
+          <t>G. V. Prakash, Ken Karunaas</t>
         </is>
       </c>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>2026-03-25</t>
+          <t>2026-03-26</t>
         </is>
       </c>
       <c r="B45" t="n">
@@ -5497,19 +6534,19 @@
       </c>
       <c r="C45" t="inlineStr">
         <is>
-          <t>Not Guilty</t>
+          <t>Barbaad (From "Saiyaara")</t>
         </is>
       </c>
       <c r="D45" t="inlineStr">
         <is>
-          <t>Dhanda Nyoliwala</t>
+          <t>The Rish, Jubin Nautiyal</t>
         </is>
       </c>
     </row>
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>2026-03-25</t>
+          <t>2026-03-26</t>
         </is>
       </c>
       <c r="B46" t="n">
@@ -5517,19 +6554,19 @@
       </c>
       <c r="C46" t="inlineStr">
         <is>
-          <t>Mutta Kalakki (From "Youth")</t>
+          <t>Ye Tune Kya Kiya</t>
         </is>
       </c>
       <c r="D46" t="inlineStr">
         <is>
-          <t>G. V. Prakash, Ken Karunaas</t>
+          <t>Pritam, Javed Bashir, Rajat Arora</t>
         </is>
       </c>
     </row>
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>2026-03-25</t>
+          <t>2026-03-26</t>
         </is>
       </c>
       <c r="B47" t="n">
@@ -5537,19 +6574,19 @@
       </c>
       <c r="C47" t="inlineStr">
         <is>
-          <t>Ehsaas</t>
+          <t>Not Guilty</t>
         </is>
       </c>
       <c r="D47" t="inlineStr">
         <is>
-          <t>Faheem Abdullah, Duha Shah, Vaibhav Pani, Hyder Dar</t>
+          <t>Dhanda Nyoliwala</t>
         </is>
       </c>
     </row>
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>2026-03-25</t>
+          <t>2026-03-26</t>
         </is>
       </c>
       <c r="B48" t="n">
@@ -5557,19 +6594,19 @@
       </c>
       <c r="C48" t="inlineStr">
         <is>
-          <t>Ye Tune Kya Kiya</t>
+          <t>Ehsaas</t>
         </is>
       </c>
       <c r="D48" t="inlineStr">
         <is>
-          <t>Pritam, Javed Bashir, Rajat Arora</t>
+          <t>Faheem Abdullah, Duha Shah, Vaibhav Pani, Hyder Dar</t>
         </is>
       </c>
     </row>
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>2026-03-25</t>
+          <t>2026-03-26</t>
         </is>
       </c>
       <c r="B49" t="n">
@@ -5577,19 +6614,19 @@
       </c>
       <c r="C49" t="inlineStr">
         <is>
-          <t>Thodi Si Daaru</t>
+          <t>Aakhri Ishq</t>
         </is>
       </c>
       <c r="D49" t="inlineStr">
         <is>
-          <t>AP Dhillon, Shreya Ghoshal</t>
+          <t>Shashwat Sachdev, Jubin Nautiyal, Irshad Kamil</t>
         </is>
       </c>
     </row>
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>2026-03-25</t>
+          <t>2026-03-26</t>
         </is>
       </c>
       <c r="B50" t="n">
@@ -5609,7 +6646,7 @@
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>2026-03-25</t>
+          <t>2026-03-26</t>
         </is>
       </c>
       <c r="B51" t="n">
@@ -5617,12 +6654,12 @@
       </c>
       <c r="C51" t="inlineStr">
         <is>
-          <t>Mast Magan (From "2 States)</t>
+          <t>Hum Pyaar Karne Wale</t>
         </is>
       </c>
       <c r="D51" t="inlineStr">
         <is>
-          <t>Arijit Singh, Chinmayi</t>
+          <t>Shashwat Sachdev, Anuradha Paudwal, Udit Narayan, Anand-Milind, Sameer Anjaan, Qveen Herby</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
added data for 27th and got predictions for 28th march
</commit_message>
<xml_diff>
--- a/Probability Project.xlsx
+++ b/Probability Project.xlsx
@@ -16,6 +16,7 @@
     <sheet name="AUTO_20260324" sheetId="11" state="visible" r:id="rId11"/>
     <sheet name="AUTO_20260325" sheetId="12" state="visible" r:id="rId12"/>
     <sheet name="AUTO_20260326" sheetId="13" state="visible" r:id="rId13"/>
+    <sheet name="AUTO_20260327" sheetId="14" state="visible" r:id="rId14"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -5664,9 +5665,1045 @@
       </c>
     </row>
     <row r="2">
+      <c r="A2" s="0" t="inlineStr">
+        <is>
+          <t>2026-03-26</t>
+        </is>
+      </c>
+      <c r="B2" s="0" t="n">
+        <v>1</v>
+      </c>
+      <c r="C2" s="0" t="inlineStr">
+        <is>
+          <t>Bairan</t>
+        </is>
+      </c>
+      <c r="D2" s="0" t="inlineStr">
+        <is>
+          <t>Banjaare</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="0" t="inlineStr">
+        <is>
+          <t>2026-03-26</t>
+        </is>
+      </c>
+      <c r="B3" s="0" t="n">
+        <v>2</v>
+      </c>
+      <c r="C3" s="0" t="inlineStr">
+        <is>
+          <t>Jaiye Sajana</t>
+        </is>
+      </c>
+      <c r="D3" s="0" t="inlineStr">
+        <is>
+          <t>Shashwat Sachdev, Jasmine Sandlas, Satinder Sartaaj</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="0" t="inlineStr">
+        <is>
+          <t>2026-03-26</t>
+        </is>
+      </c>
+      <c r="B4" s="0" t="n">
+        <v>3</v>
+      </c>
+      <c r="C4" s="0" t="inlineStr">
+        <is>
+          <t>Sheesha - Aakhya Mai Aakh Ghali Jo Bairan</t>
+        </is>
+      </c>
+      <c r="D4" s="0" t="inlineStr">
+        <is>
+          <t>Mitta Ror, Swara Verma</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="0" t="inlineStr">
+        <is>
+          <t>2026-03-26</t>
+        </is>
+      </c>
+      <c r="B5" s="0" t="n">
+        <v>4</v>
+      </c>
+      <c r="C5" s="0" t="inlineStr">
+        <is>
+          <t>Gehra Hua</t>
+        </is>
+      </c>
+      <c r="D5" s="0" t="inlineStr">
+        <is>
+          <t>Shashwat Sachdev, Arijit Singh, Irshad Kamil, Armaan Khan</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="0" t="inlineStr">
+        <is>
+          <t>2026-03-26</t>
+        </is>
+      </c>
+      <c r="B6" s="0" t="n">
+        <v>5</v>
+      </c>
+      <c r="C6" s="0" t="inlineStr">
+        <is>
+          <t>Dhurandhar The Revenge - Aari Aari</t>
+        </is>
+      </c>
+      <c r="D6" s="0" t="inlineStr">
+        <is>
+          <t>Shashwat Sachdev, Bombay Rockers, Irshad Kamil, Khan Saab, Reble, Token, Jasmine Sandlas, Sudhir Yaduvanshi</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="0" t="inlineStr">
+        <is>
+          <t>2026-03-26</t>
+        </is>
+      </c>
+      <c r="B7" s="0" t="n">
+        <v>6</v>
+      </c>
+      <c r="C7" s="0" t="inlineStr">
+        <is>
+          <t>Jaan Se Guzarte Hain</t>
+        </is>
+      </c>
+      <c r="D7" s="0" t="inlineStr">
+        <is>
+          <t>Shashwat Sachdev, Khan Saab, Nusrat Fateh Ali Khan</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="0" t="inlineStr">
+        <is>
+          <t>2026-03-26</t>
+        </is>
+      </c>
+      <c r="B8" s="0" t="n">
+        <v>7</v>
+      </c>
+      <c r="C8" s="0" t="inlineStr">
+        <is>
+          <t>Khat</t>
+        </is>
+      </c>
+      <c r="D8" s="0" t="inlineStr">
+        <is>
+          <t>Navjot Ahuja</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="0" t="inlineStr">
+        <is>
+          <t>2026-03-26</t>
+        </is>
+      </c>
+      <c r="B9" s="0" t="n">
+        <v>8</v>
+      </c>
+      <c r="C9" s="0" t="inlineStr">
+        <is>
+          <t>Dooron Dooron</t>
+        </is>
+      </c>
+      <c r="D9" s="0" t="inlineStr">
+        <is>
+          <t>Paresh Pahuja, Shiv Tandan, Meghdeep Bose</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="0" t="inlineStr">
+        <is>
+          <t>2026-03-26</t>
+        </is>
+      </c>
+      <c r="B10" s="0" t="n">
+        <v>9</v>
+      </c>
+      <c r="C10" s="0" t="inlineStr">
+        <is>
+          <t>Sitaare (From "Ikkis")</t>
+        </is>
+      </c>
+      <c r="D10" s="0" t="inlineStr">
+        <is>
+          <t>Arijit Singh, White Noise Collectives, Amitabh Bhattacharya</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="0" t="inlineStr">
+        <is>
+          <t>2026-03-26</t>
+        </is>
+      </c>
+      <c r="B11" s="0" t="n">
+        <v>10</v>
+      </c>
+      <c r="C11" s="0" t="inlineStr">
+        <is>
+          <t>Sahiba</t>
+        </is>
+      </c>
+      <c r="D11" s="0" t="inlineStr">
+        <is>
+          <t>Aditya Rikhari</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="0" t="inlineStr">
+        <is>
+          <t>2026-03-26</t>
+        </is>
+      </c>
+      <c r="B12" s="0" t="n">
+        <v>11</v>
+      </c>
+      <c r="C12" s="0" t="inlineStr">
+        <is>
+          <t>Apna Bana Le</t>
+        </is>
+      </c>
+      <c r="D12" s="0" t="inlineStr">
+        <is>
+          <t>Sachin-Jigar, Arijit Singh, Amitabh Bhattacharya</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="0" t="inlineStr">
+        <is>
+          <t>2026-03-26</t>
+        </is>
+      </c>
+      <c r="B13" s="0" t="n">
+        <v>12</v>
+      </c>
+      <c r="C13" s="0" t="inlineStr">
+        <is>
+          <t>Samjhawan</t>
+        </is>
+      </c>
+      <c r="D13" s="0" t="inlineStr">
+        <is>
+          <t>Jawad Ahmad, Shaarib Toshi, Arijit Singh, Shreya Ghoshal</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="0" t="inlineStr">
+        <is>
+          <t>2026-03-26</t>
+        </is>
+      </c>
+      <c r="B14" s="0" t="n">
+        <v>13</v>
+      </c>
+      <c r="C14" s="0" t="inlineStr">
+        <is>
+          <t>Finding Her</t>
+        </is>
+      </c>
+      <c r="D14" s="0" t="inlineStr">
+        <is>
+          <t>Kushagra, Bharath, Saaheal</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="0" t="inlineStr">
+        <is>
+          <t>2026-03-26</t>
+        </is>
+      </c>
+      <c r="B15" s="0" t="n">
+        <v>14</v>
+      </c>
+      <c r="C15" s="0" t="inlineStr">
+        <is>
+          <t>Shararat</t>
+        </is>
+      </c>
+      <c r="D15" s="0" t="inlineStr">
+        <is>
+          <t>Shashwat Sachdev, Madhubanti Bagchi, Jasmine Sandlas</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="0" t="inlineStr">
+        <is>
+          <t>2026-03-26</t>
+        </is>
+      </c>
+      <c r="B16" s="0" t="n">
+        <v>15</v>
+      </c>
+      <c r="C16" s="0" t="inlineStr">
+        <is>
+          <t>Dhurandhar - Title Track</t>
+        </is>
+      </c>
+      <c r="D16" s="0" t="inlineStr">
+        <is>
+          <t>Shashwat Sachdev, Hanumankind, Jasmine Sandlas, Sudhir Yaduvanshi, Charanjit Ahuja, Muhammad Sadiq, Ranjit Kaur, Babu Singh Maan</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="0" t="inlineStr">
+        <is>
+          <t>2026-03-26</t>
+        </is>
+      </c>
+      <c r="B17" s="0" t="n">
+        <v>16</v>
+      </c>
+      <c r="C17" s="0" t="inlineStr">
+        <is>
+          <t>Arz Kiya Hai | Coke Studio Bharat</t>
+        </is>
+      </c>
+      <c r="D17" s="0" t="inlineStr">
+        <is>
+          <t>Anuv Jain</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="0" t="inlineStr">
+        <is>
+          <t>2026-03-26</t>
+        </is>
+      </c>
+      <c r="B18" s="0" t="n">
+        <v>17</v>
+      </c>
+      <c r="C18" s="0" t="inlineStr">
+        <is>
+          <t>Pavazha Malli - From "Think Indie"</t>
+        </is>
+      </c>
+      <c r="D18" s="0" t="inlineStr">
+        <is>
+          <t>Sai Abhyankkar, Shruti Haasan, Vivek</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="0" t="inlineStr">
+        <is>
+          <t>2026-03-26</t>
+        </is>
+      </c>
+      <c r="B19" s="0" t="n">
+        <v>18</v>
+      </c>
+      <c r="C19" s="0" t="inlineStr">
+        <is>
+          <t>Ishq</t>
+        </is>
+      </c>
+      <c r="D19" s="0" t="inlineStr">
+        <is>
+          <t>Faheem Abdullah, Rauhan Malik, Amir Ameer</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="0" t="inlineStr">
+        <is>
+          <t>2026-03-26</t>
+        </is>
+      </c>
+      <c r="B20" s="0" t="n">
+        <v>19</v>
+      </c>
+      <c r="C20" s="0" t="inlineStr">
+        <is>
+          <t>Mann Mera</t>
+        </is>
+      </c>
+      <c r="D20" s="0" t="inlineStr">
+        <is>
+          <t>Gajendra Verma</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="0" t="inlineStr">
+        <is>
+          <t>2026-03-26</t>
+        </is>
+      </c>
+      <c r="B21" s="0" t="n">
+        <v>20</v>
+      </c>
+      <c r="C21" s="0" t="inlineStr">
+        <is>
+          <t>For A Reason</t>
+        </is>
+      </c>
+      <c r="D21" s="0" t="inlineStr">
+        <is>
+          <t>Karan Aujla, Ikky</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="0" t="inlineStr">
+        <is>
+          <t>2026-03-26</t>
+        </is>
+      </c>
+      <c r="B22" s="0" t="n">
+        <v>21</v>
+      </c>
+      <c r="C22" s="0" t="inlineStr">
+        <is>
+          <t>Boyfriend</t>
+        </is>
+      </c>
+      <c r="D22" s="0" t="inlineStr">
+        <is>
+          <t>Karan Aujla, Ikky</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="0" t="inlineStr">
+        <is>
+          <t>2026-03-26</t>
+        </is>
+      </c>
+      <c r="B23" s="0" t="n">
+        <v>22</v>
+      </c>
+      <c r="C23" s="0" t="inlineStr">
+        <is>
+          <t>Phir Se</t>
+        </is>
+      </c>
+      <c r="D23" s="0" t="inlineStr">
+        <is>
+          <t>Shashwat Sachdev, Arijit Singh, Irshad Kamil</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="0" t="inlineStr">
+        <is>
+          <t>2026-03-26</t>
+        </is>
+      </c>
+      <c r="B24" s="0" t="n">
+        <v>23</v>
+      </c>
+      <c r="C24" s="0" t="inlineStr">
+        <is>
+          <t>Bairi</t>
+        </is>
+      </c>
+      <c r="D24" s="0" t="inlineStr">
+        <is>
+          <t>Virat, Pradeep Solanki, Heena</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="0" t="inlineStr">
+        <is>
+          <t>2026-03-26</t>
+        </is>
+      </c>
+      <c r="B25" s="0" t="n">
+        <v>24</v>
+      </c>
+      <c r="C25" s="0" t="inlineStr">
+        <is>
+          <t>Saiyaara</t>
+        </is>
+      </c>
+      <c r="D25" s="0" t="inlineStr">
+        <is>
+          <t>Tanishk Bagchi, Faheem Abdullah, Arslan Nizami, Irshad Kamil</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="0" t="inlineStr">
+        <is>
+          <t>2026-03-26</t>
+        </is>
+      </c>
+      <c r="B26" s="0" t="n">
+        <v>25</v>
+      </c>
+      <c r="C26" s="0" t="inlineStr">
+        <is>
+          <t>Ishqa Ve</t>
+        </is>
+      </c>
+      <c r="D26" s="0" t="inlineStr">
+        <is>
+          <t>Zeeshan Ali, Yuvraj Tung, Sandeep Aulakh, Honey Dhillon</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="0" t="inlineStr">
+        <is>
+          <t>2026-03-26</t>
+        </is>
+      </c>
+      <c r="B27" s="0" t="n">
+        <v>26</v>
+      </c>
+      <c r="C27" s="0" t="inlineStr">
+        <is>
+          <t>Naal Nachna</t>
+        </is>
+      </c>
+      <c r="D27" s="0" t="inlineStr">
+        <is>
+          <t>Shashwat Sachdev, Afsana Khan, Irshad Kamil, Reble</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="0" t="inlineStr">
+        <is>
+          <t>2026-03-26</t>
+        </is>
+      </c>
+      <c r="B28" s="0" t="n">
+        <v>27</v>
+      </c>
+      <c r="C28" s="0" t="inlineStr">
+        <is>
+          <t>Main Aur Tu</t>
+        </is>
+      </c>
+      <c r="D28" s="0" t="inlineStr">
+        <is>
+          <t>Jasmine Sandlas, Shashwat Sachdev, Reble</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="0" t="inlineStr">
+        <is>
+          <t>2026-03-26</t>
+        </is>
+      </c>
+      <c r="B29" s="0" t="n">
+        <v>28</v>
+      </c>
+      <c r="C29" s="0" t="inlineStr">
+        <is>
+          <t>Raanjhan (From "Do Patti")</t>
+        </is>
+      </c>
+      <c r="D29" s="0" t="inlineStr">
+        <is>
+          <t>Sachet-Parampara, Parampara Tandon, Kausar Munir</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="0" t="inlineStr">
+        <is>
+          <t>2026-03-26</t>
+        </is>
+      </c>
+      <c r="B30" s="0" t="n">
+        <v>29</v>
+      </c>
+      <c r="C30" s="0" t="inlineStr">
+        <is>
+          <t>Deewaana Deewaana</t>
+        </is>
+      </c>
+      <c r="D30" s="0" t="inlineStr">
+        <is>
+          <t>A.R. Rahman, Irshad Kamil</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="0" t="inlineStr">
+        <is>
+          <t>2026-03-26</t>
+        </is>
+      </c>
+      <c r="B31" s="0" t="n">
+        <v>30</v>
+      </c>
+      <c r="C31" s="0" t="inlineStr">
+        <is>
+          <t>Tere Liye</t>
+        </is>
+      </c>
+      <c r="D31" s="0" t="inlineStr">
+        <is>
+          <t>Atif Aslam, Shreya Ghoshal, Sachin Gupta, Sameer Anjaan</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="0" t="inlineStr">
+        <is>
+          <t>2026-03-26</t>
+        </is>
+      </c>
+      <c r="B32" s="0" t="n">
+        <v>31</v>
+      </c>
+      <c r="C32" s="0" t="inlineStr">
+        <is>
+          <t>Lutt Le Gaya</t>
+        </is>
+      </c>
+      <c r="D32" s="0" t="inlineStr">
+        <is>
+          <t>Shashwat Sachdev, Simran Choudhary</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="0" t="inlineStr">
+        <is>
+          <t>2026-03-26</t>
+        </is>
+      </c>
+      <c r="B33" s="0" t="n">
+        <v>32</v>
+      </c>
+      <c r="C33" s="0" t="inlineStr">
+        <is>
+          <t>SWIM</t>
+        </is>
+      </c>
+      <c r="D33" s="0" t="inlineStr">
+        <is>
+          <t>BTS</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="0" t="inlineStr">
+        <is>
+          <t>2026-03-26</t>
+        </is>
+      </c>
+      <c r="B34" s="0" t="n">
+        <v>33</v>
+      </c>
+      <c r="C34" s="0" t="inlineStr">
+        <is>
+          <t>Jogi</t>
+        </is>
+      </c>
+      <c r="D34" s="0" t="inlineStr">
+        <is>
+          <t>thiarajxtt, Bir</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="0" t="inlineStr">
+        <is>
+          <t>2026-03-26</t>
+        </is>
+      </c>
+      <c r="B35" s="0" t="n">
+        <v>34</v>
+      </c>
+      <c r="C35" s="0" t="inlineStr">
+        <is>
+          <t>Ishq Jalakar - Karvaan</t>
+        </is>
+      </c>
+      <c r="D35" s="0" t="inlineStr">
+        <is>
+          <t>Shashwat Sachdev, Shahzad Ali, Subhadeep Das Chowdhury, Armaan Khan, Irshad Kamil, Roshan, Sahir Ludhianvi</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="0" t="inlineStr">
+        <is>
+          <t>2026-03-26</t>
+        </is>
+      </c>
+      <c r="B36" s="0" t="n">
+        <v>35</v>
+      </c>
+      <c r="C36" s="0" t="inlineStr">
+        <is>
+          <t>Aaya Sher (From "The Paradise") (Telugu)</t>
+        </is>
+      </c>
+      <c r="D36" s="0" t="inlineStr">
+        <is>
+          <t>Anirudh Ravichander, Jangi Reddy, Arjun Chandy, Kasarla Shyam</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="0" t="inlineStr">
+        <is>
+          <t>2026-03-26</t>
+        </is>
+      </c>
+      <c r="B37" s="0" t="n">
+        <v>36</v>
+      </c>
+      <c r="C37" s="0" t="inlineStr">
+        <is>
+          <t>Tum Ho Toh (From "Saiyaara")</t>
+        </is>
+      </c>
+      <c r="D37" s="0" t="inlineStr">
+        <is>
+          <t>Vishal Mishra, Hansika Pareek, Raj Shekhar</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="0" t="inlineStr">
+        <is>
+          <t>2026-03-26</t>
+        </is>
+      </c>
+      <c r="B38" s="0" t="n">
+        <v>37</v>
+      </c>
+      <c r="C38" s="0" t="inlineStr">
+        <is>
+          <t>Tere Bina</t>
+        </is>
+      </c>
+      <c r="D38" s="0" t="inlineStr">
+        <is>
+          <t>A.R. Rahman, Chinmayi, Murtuza Khan, Qadir Khan</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="0" t="inlineStr">
+        <is>
+          <t>2026-03-26</t>
+        </is>
+      </c>
+      <c r="B39" s="0" t="n">
+        <v>38</v>
+      </c>
+      <c r="C39" s="0" t="inlineStr">
+        <is>
+          <t>Jo Tum Mere Ho</t>
+        </is>
+      </c>
+      <c r="D39" s="0" t="inlineStr">
+        <is>
+          <t>Anuv Jain</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="0" t="inlineStr">
+        <is>
+          <t>2026-03-26</t>
+        </is>
+      </c>
+      <c r="B40" s="0" t="n">
+        <v>39</v>
+      </c>
+      <c r="C40" s="0" t="inlineStr">
+        <is>
+          <t>Agar Tum Saath Ho (From "Tamasha")</t>
+        </is>
+      </c>
+      <c r="D40" s="0" t="inlineStr">
+        <is>
+          <t>Alka Yagnik, Arijit Singh</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" s="0" t="inlineStr">
+        <is>
+          <t>2026-03-26</t>
+        </is>
+      </c>
+      <c r="B41" s="0" t="n">
+        <v>40</v>
+      </c>
+      <c r="C41" s="0" t="inlineStr">
+        <is>
+          <t>Run Down The City - Monica</t>
+        </is>
+      </c>
+      <c r="D41" s="0" t="inlineStr">
+        <is>
+          <t>Shashwat Sachdev, Reble, Asha Bhosle, R. D. Burman, Majrooh Sultanpuri</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" s="0" t="inlineStr">
+        <is>
+          <t>2026-03-26</t>
+        </is>
+      </c>
+      <c r="B42" s="0" t="n">
+        <v>41</v>
+      </c>
+      <c r="C42" s="0" t="inlineStr">
+        <is>
+          <t>Darkhaast</t>
+        </is>
+      </c>
+      <c r="D42" s="0" t="inlineStr">
+        <is>
+          <t>Mithoon, Arijit Singh, Sunidhi Chauhan, Sayeed Quadri</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" s="0" t="inlineStr">
+        <is>
+          <t>2026-03-26</t>
+        </is>
+      </c>
+      <c r="B43" s="0" t="n">
+        <v>42</v>
+      </c>
+      <c r="C43" s="0" t="inlineStr">
+        <is>
+          <t>Haseen</t>
+        </is>
+      </c>
+      <c r="D43" s="0" t="inlineStr">
+        <is>
+          <t>Talwiinder, NDS, Rippy Grewal</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" s="0" t="inlineStr">
+        <is>
+          <t>2026-03-26</t>
+        </is>
+      </c>
+      <c r="B44" s="0" t="n">
+        <v>43</v>
+      </c>
+      <c r="C44" s="0" t="inlineStr">
+        <is>
+          <t>Mutta Kalakki (From "Youth")</t>
+        </is>
+      </c>
+      <c r="D44" s="0" t="inlineStr">
+        <is>
+          <t>G. V. Prakash, Ken Karunaas</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" s="0" t="inlineStr">
+        <is>
+          <t>2026-03-26</t>
+        </is>
+      </c>
+      <c r="B45" s="0" t="n">
+        <v>44</v>
+      </c>
+      <c r="C45" s="0" t="inlineStr">
+        <is>
+          <t>Barbaad (From "Saiyaara")</t>
+        </is>
+      </c>
+      <c r="D45" s="0" t="inlineStr">
+        <is>
+          <t>The Rish, Jubin Nautiyal</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" s="0" t="inlineStr">
+        <is>
+          <t>2026-03-26</t>
+        </is>
+      </c>
+      <c r="B46" s="0" t="n">
+        <v>45</v>
+      </c>
+      <c r="C46" s="0" t="inlineStr">
+        <is>
+          <t>Ye Tune Kya Kiya</t>
+        </is>
+      </c>
+      <c r="D46" s="0" t="inlineStr">
+        <is>
+          <t>Pritam, Javed Bashir, Rajat Arora</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" s="0" t="inlineStr">
+        <is>
+          <t>2026-03-26</t>
+        </is>
+      </c>
+      <c r="B47" s="0" t="n">
+        <v>46</v>
+      </c>
+      <c r="C47" s="0" t="inlineStr">
+        <is>
+          <t>Not Guilty</t>
+        </is>
+      </c>
+      <c r="D47" s="0" t="inlineStr">
+        <is>
+          <t>Dhanda Nyoliwala</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" s="0" t="inlineStr">
+        <is>
+          <t>2026-03-26</t>
+        </is>
+      </c>
+      <c r="B48" s="0" t="n">
+        <v>47</v>
+      </c>
+      <c r="C48" s="0" t="inlineStr">
+        <is>
+          <t>Ehsaas</t>
+        </is>
+      </c>
+      <c r="D48" s="0" t="inlineStr">
+        <is>
+          <t>Faheem Abdullah, Duha Shah, Vaibhav Pani, Hyder Dar</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" s="0" t="inlineStr">
+        <is>
+          <t>2026-03-26</t>
+        </is>
+      </c>
+      <c r="B49" s="0" t="n">
+        <v>48</v>
+      </c>
+      <c r="C49" s="0" t="inlineStr">
+        <is>
+          <t>Aakhri Ishq</t>
+        </is>
+      </c>
+      <c r="D49" s="0" t="inlineStr">
+        <is>
+          <t>Shashwat Sachdev, Jubin Nautiyal, Irshad Kamil</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" s="0" t="inlineStr">
+        <is>
+          <t>2026-03-26</t>
+        </is>
+      </c>
+      <c r="B50" s="0" t="n">
+        <v>49</v>
+      </c>
+      <c r="C50" s="0" t="inlineStr">
+        <is>
+          <t>Teri Deewani</t>
+        </is>
+      </c>
+      <c r="D50" s="0" t="inlineStr">
+        <is>
+          <t>Kailash Kher, Paresh Kamath, Naresh Kamath</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" s="0" t="inlineStr">
+        <is>
+          <t>2026-03-26</t>
+        </is>
+      </c>
+      <c r="B51" s="0" t="n">
+        <v>50</v>
+      </c>
+      <c r="C51" s="0" t="inlineStr">
+        <is>
+          <t>Hum Pyaar Karne Wale</t>
+        </is>
+      </c>
+      <c r="D51" s="0" t="inlineStr">
+        <is>
+          <t>Shashwat Sachdev, Anuradha Paudwal, Udit Narayan, Anand-Milind, Sameer Anjaan, Qveen Herby</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet14.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:D51"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="24" t="inlineStr">
+        <is>
+          <t>Date</t>
+        </is>
+      </c>
+      <c r="B1" s="24" t="inlineStr">
+        <is>
+          <t>Rank</t>
+        </is>
+      </c>
+      <c r="C1" s="24" t="inlineStr">
+        <is>
+          <t>Song</t>
+        </is>
+      </c>
+      <c r="D1" s="24" t="inlineStr">
+        <is>
+          <t>Artist</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>2026-03-26</t>
+          <t>2026-03-27</t>
         </is>
       </c>
       <c r="B2" t="n">
@@ -5686,7 +6723,7 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>2026-03-26</t>
+          <t>2026-03-27</t>
         </is>
       </c>
       <c r="B3" t="n">
@@ -5706,7 +6743,7 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>2026-03-26</t>
+          <t>2026-03-27</t>
         </is>
       </c>
       <c r="B4" t="n">
@@ -5726,7 +6763,7 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>2026-03-26</t>
+          <t>2026-03-27</t>
         </is>
       </c>
       <c r="B5" t="n">
@@ -5746,7 +6783,7 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>2026-03-26</t>
+          <t>2026-03-27</t>
         </is>
       </c>
       <c r="B6" t="n">
@@ -5766,7 +6803,7 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>2026-03-26</t>
+          <t>2026-03-27</t>
         </is>
       </c>
       <c r="B7" t="n">
@@ -5786,7 +6823,7 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>2026-03-26</t>
+          <t>2026-03-27</t>
         </is>
       </c>
       <c r="B8" t="n">
@@ -5806,7 +6843,7 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>2026-03-26</t>
+          <t>2026-03-27</t>
         </is>
       </c>
       <c r="B9" t="n">
@@ -5814,19 +6851,19 @@
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>Dooron Dooron</t>
+          <t>Sitaare (From "Ikkis")</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>Paresh Pahuja, Shiv Tandan, Meghdeep Bose</t>
+          <t>Arijit Singh, White Noise Collectives, Amitabh Bhattacharya</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>2026-03-26</t>
+          <t>2026-03-27</t>
         </is>
       </c>
       <c r="B10" t="n">
@@ -5834,19 +6871,19 @@
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>Sitaare (From "Ikkis")</t>
+          <t>Dooron Dooron</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>Arijit Singh, White Noise Collectives, Amitabh Bhattacharya</t>
+          <t>Paresh Pahuja, Shiv Tandan, Meghdeep Bose</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>2026-03-26</t>
+          <t>2026-03-27</t>
         </is>
       </c>
       <c r="B11" t="n">
@@ -5866,7 +6903,7 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>2026-03-26</t>
+          <t>2026-03-27</t>
         </is>
       </c>
       <c r="B12" t="n">
@@ -5886,7 +6923,7 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>2026-03-26</t>
+          <t>2026-03-27</t>
         </is>
       </c>
       <c r="B13" t="n">
@@ -5894,19 +6931,19 @@
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>Samjhawan</t>
+          <t>Shararat</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>Jawad Ahmad, Shaarib Toshi, Arijit Singh, Shreya Ghoshal</t>
+          <t>Shashwat Sachdev, Madhubanti Bagchi, Jasmine Sandlas</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>2026-03-26</t>
+          <t>2026-03-27</t>
         </is>
       </c>
       <c r="B14" t="n">
@@ -5914,19 +6951,19 @@
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>Finding Her</t>
+          <t>Samjhawan</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>Kushagra, Bharath, Saaheal</t>
+          <t>Jawad Ahmad, Shaarib Toshi, Arijit Singh, Shreya Ghoshal</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>2026-03-26</t>
+          <t>2026-03-27</t>
         </is>
       </c>
       <c r="B15" t="n">
@@ -5934,19 +6971,19 @@
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>Shararat</t>
+          <t>Finding Her</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>Shashwat Sachdev, Madhubanti Bagchi, Jasmine Sandlas</t>
+          <t>Kushagra, Bharath, Saaheal</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>2026-03-26</t>
+          <t>2026-03-27</t>
         </is>
       </c>
       <c r="B16" t="n">
@@ -5966,7 +7003,7 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>2026-03-26</t>
+          <t>2026-03-27</t>
         </is>
       </c>
       <c r="B17" t="n">
@@ -5986,7 +7023,7 @@
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>2026-03-26</t>
+          <t>2026-03-27</t>
         </is>
       </c>
       <c r="B18" t="n">
@@ -6006,7 +7043,7 @@
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>2026-03-26</t>
+          <t>2026-03-27</t>
         </is>
       </c>
       <c r="B19" t="n">
@@ -6014,19 +7051,19 @@
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>Ishq</t>
+          <t>Boyfriend</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>Faheem Abdullah, Rauhan Malik, Amir Ameer</t>
+          <t>Karan Aujla, Ikky</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>2026-03-26</t>
+          <t>2026-03-27</t>
         </is>
       </c>
       <c r="B20" t="n">
@@ -6034,19 +7071,19 @@
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>Mann Mera</t>
+          <t>Ishq</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>Gajendra Verma</t>
+          <t>Faheem Abdullah, Rauhan Malik, Amir Ameer</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>2026-03-26</t>
+          <t>2026-03-27</t>
         </is>
       </c>
       <c r="B21" t="n">
@@ -6066,7 +7103,7 @@
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>2026-03-26</t>
+          <t>2026-03-27</t>
         </is>
       </c>
       <c r="B22" t="n">
@@ -6074,19 +7111,19 @@
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>Boyfriend</t>
+          <t>Naal Nachna</t>
         </is>
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>Karan Aujla, Ikky</t>
+          <t>Shashwat Sachdev, Afsana Khan, Irshad Kamil, Reble</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>2026-03-26</t>
+          <t>2026-03-27</t>
         </is>
       </c>
       <c r="B23" t="n">
@@ -6094,19 +7131,19 @@
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>Phir Se</t>
+          <t>Bairi</t>
         </is>
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>Shashwat Sachdev, Arijit Singh, Irshad Kamil</t>
+          <t>Virat, Pradeep Solanki, Heena</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>2026-03-26</t>
+          <t>2026-03-27</t>
         </is>
       </c>
       <c r="B24" t="n">
@@ -6114,19 +7151,19 @@
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>Bairi</t>
+          <t>Mann Mera</t>
         </is>
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>Virat, Pradeep Solanki, Heena</t>
+          <t>Gajendra Verma</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>2026-03-26</t>
+          <t>2026-03-27</t>
         </is>
       </c>
       <c r="B25" t="n">
@@ -6146,7 +7183,7 @@
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>2026-03-26</t>
+          <t>2026-03-27</t>
         </is>
       </c>
       <c r="B26" t="n">
@@ -6166,7 +7203,7 @@
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>2026-03-26</t>
+          <t>2026-03-27</t>
         </is>
       </c>
       <c r="B27" t="n">
@@ -6174,19 +7211,19 @@
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>Naal Nachna</t>
+          <t>Tere Liye</t>
         </is>
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t>Shashwat Sachdev, Afsana Khan, Irshad Kamil, Reble</t>
+          <t>Atif Aslam, Shreya Ghoshal, Sachin Gupta, Sameer Anjaan</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>2026-03-26</t>
+          <t>2026-03-27</t>
         </is>
       </c>
       <c r="B28" t="n">
@@ -6194,19 +7231,19 @@
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>Main Aur Tu</t>
+          <t>Deewaana Deewaana</t>
         </is>
       </c>
       <c r="D28" t="inlineStr">
         <is>
-          <t>Jasmine Sandlas, Shashwat Sachdev, Reble</t>
+          <t>A.R. Rahman, Irshad Kamil</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>2026-03-26</t>
+          <t>2026-03-27</t>
         </is>
       </c>
       <c r="B29" t="n">
@@ -6214,19 +7251,19 @@
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>Raanjhan (From "Do Patti")</t>
+          <t>Phir Se</t>
         </is>
       </c>
       <c r="D29" t="inlineStr">
         <is>
-          <t>Sachet-Parampara, Parampara Tandon, Kausar Munir</t>
+          <t>Shashwat Sachdev, Arijit Singh, Irshad Kamil</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>2026-03-26</t>
+          <t>2026-03-27</t>
         </is>
       </c>
       <c r="B30" t="n">
@@ -6234,19 +7271,19 @@
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>Deewaana Deewaana</t>
+          <t>Raanjhan (From "Do Patti")</t>
         </is>
       </c>
       <c r="D30" t="inlineStr">
         <is>
-          <t>A.R. Rahman, Irshad Kamil</t>
+          <t>Sachet-Parampara, Parampara Tandon, Kausar Munir</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>2026-03-26</t>
+          <t>2026-03-27</t>
         </is>
       </c>
       <c r="B31" t="n">
@@ -6254,19 +7291,19 @@
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>Tere Liye</t>
+          <t>Lutt Le Gaya</t>
         </is>
       </c>
       <c r="D31" t="inlineStr">
         <is>
-          <t>Atif Aslam, Shreya Ghoshal, Sachin Gupta, Sameer Anjaan</t>
+          <t>Shashwat Sachdev, Simran Choudhary</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>2026-03-26</t>
+          <t>2026-03-27</t>
         </is>
       </c>
       <c r="B32" t="n">
@@ -6274,19 +7311,19 @@
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>Lutt Le Gaya</t>
+          <t>Main Aur Tu (From "Dhurandhar The Revenge")</t>
         </is>
       </c>
       <c r="D32" t="inlineStr">
         <is>
-          <t>Shashwat Sachdev, Simran Choudhary</t>
+          <t>Shashwat Sachdev, Jasmine Sandlas, Reble</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>2026-03-26</t>
+          <t>2026-03-27</t>
         </is>
       </c>
       <c r="B33" t="n">
@@ -6294,19 +7331,19 @@
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>SWIM</t>
+          <t>Darkhaast</t>
         </is>
       </c>
       <c r="D33" t="inlineStr">
         <is>
-          <t>BTS</t>
+          <t>Mithoon, Arijit Singh, Sunidhi Chauhan, Sayeed Quadri</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>2026-03-26</t>
+          <t>2026-03-27</t>
         </is>
       </c>
       <c r="B34" t="n">
@@ -6314,19 +7351,19 @@
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>Jogi</t>
+          <t>Run Down The City - Monica</t>
         </is>
       </c>
       <c r="D34" t="inlineStr">
         <is>
-          <t>thiarajxtt, Bir</t>
+          <t>Shashwat Sachdev, Reble, Asha Bhosle, R. D. Burman, Majrooh Sultanpuri</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>2026-03-26</t>
+          <t>2026-03-27</t>
         </is>
       </c>
       <c r="B35" t="n">
@@ -6334,19 +7371,19 @@
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>Ishq Jalakar - Karvaan</t>
+          <t>Tere Bina</t>
         </is>
       </c>
       <c r="D35" t="inlineStr">
         <is>
-          <t>Shashwat Sachdev, Shahzad Ali, Subhadeep Das Chowdhury, Armaan Khan, Irshad Kamil, Roshan, Sahir Ludhianvi</t>
+          <t>A.R. Rahman, Chinmayi, Murtuza Khan, Qadir Khan</t>
         </is>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>2026-03-26</t>
+          <t>2026-03-27</t>
         </is>
       </c>
       <c r="B36" t="n">
@@ -6354,19 +7391,19 @@
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>Aaya Sher (From "The Paradise") (Telugu)</t>
+          <t>Tum Ho Toh (From "Saiyaara")</t>
         </is>
       </c>
       <c r="D36" t="inlineStr">
         <is>
-          <t>Anirudh Ravichander, Jangi Reddy, Arjun Chandy, Kasarla Shyam</t>
+          <t>Vishal Mishra, Hansika Pareek, Raj Shekhar</t>
         </is>
       </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>2026-03-26</t>
+          <t>2026-03-27</t>
         </is>
       </c>
       <c r="B37" t="n">
@@ -6374,19 +7411,19 @@
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>Tum Ho Toh (From "Saiyaara")</t>
+          <t>Ishq Jalakar - Karvaan</t>
         </is>
       </c>
       <c r="D37" t="inlineStr">
         <is>
-          <t>Vishal Mishra, Hansika Pareek, Raj Shekhar</t>
+          <t>Shashwat Sachdev, Shahzad Ali, Subhadeep Das Chowdhury, Armaan Khan, Irshad Kamil, Roshan, Sahir Ludhianvi</t>
         </is>
       </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>2026-03-26</t>
+          <t>2026-03-27</t>
         </is>
       </c>
       <c r="B38" t="n">
@@ -6394,19 +7431,19 @@
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>Tere Bina</t>
+          <t>Jogi</t>
         </is>
       </c>
       <c r="D38" t="inlineStr">
         <is>
-          <t>A.R. Rahman, Chinmayi, Murtuza Khan, Qadir Khan</t>
+          <t>thiarajxtt, Bir</t>
         </is>
       </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>2026-03-26</t>
+          <t>2026-03-27</t>
         </is>
       </c>
       <c r="B39" t="n">
@@ -6414,19 +7451,19 @@
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>Jo Tum Mere Ho</t>
+          <t>Agar Tum Saath Ho (From "Tamasha")</t>
         </is>
       </c>
       <c r="D39" t="inlineStr">
         <is>
-          <t>Anuv Jain</t>
+          <t>Alka Yagnik, Arijit Singh</t>
         </is>
       </c>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>2026-03-26</t>
+          <t>2026-03-27</t>
         </is>
       </c>
       <c r="B40" t="n">
@@ -6434,19 +7471,19 @@
       </c>
       <c r="C40" t="inlineStr">
         <is>
-          <t>Agar Tum Saath Ho (From "Tamasha")</t>
+          <t>SWIM</t>
         </is>
       </c>
       <c r="D40" t="inlineStr">
         <is>
-          <t>Alka Yagnik, Arijit Singh</t>
+          <t>BTS</t>
         </is>
       </c>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>2026-03-26</t>
+          <t>2026-03-27</t>
         </is>
       </c>
       <c r="B41" t="n">
@@ -6454,19 +7491,19 @@
       </c>
       <c r="C41" t="inlineStr">
         <is>
-          <t>Run Down The City - Monica</t>
+          <t>Aaya Sher (From "The Paradise") (Telugu)</t>
         </is>
       </c>
       <c r="D41" t="inlineStr">
         <is>
-          <t>Shashwat Sachdev, Reble, Asha Bhosle, R. D. Burman, Majrooh Sultanpuri</t>
+          <t>Anirudh Ravichander, Jangi Reddy, Arjun Chandy, Kasarla Shyam</t>
         </is>
       </c>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>2026-03-26</t>
+          <t>2026-03-27</t>
         </is>
       </c>
       <c r="B42" t="n">
@@ -6474,19 +7511,19 @@
       </c>
       <c r="C42" t="inlineStr">
         <is>
-          <t>Darkhaast</t>
+          <t>Jo Tum Mere Ho</t>
         </is>
       </c>
       <c r="D42" t="inlineStr">
         <is>
-          <t>Mithoon, Arijit Singh, Sunidhi Chauhan, Sayeed Quadri</t>
+          <t>Anuv Jain</t>
         </is>
       </c>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>2026-03-26</t>
+          <t>2026-03-27</t>
         </is>
       </c>
       <c r="B43" t="n">
@@ -6494,19 +7531,19 @@
       </c>
       <c r="C43" t="inlineStr">
         <is>
-          <t>Haseen</t>
+          <t>Mutta Kalakki (From "Youth")</t>
         </is>
       </c>
       <c r="D43" t="inlineStr">
         <is>
-          <t>Talwiinder, NDS, Rippy Grewal</t>
+          <t>G. V. Prakash, Ken Karunaas</t>
         </is>
       </c>
     </row>
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>2026-03-26</t>
+          <t>2026-03-27</t>
         </is>
       </c>
       <c r="B44" t="n">
@@ -6514,19 +7551,19 @@
       </c>
       <c r="C44" t="inlineStr">
         <is>
-          <t>Mutta Kalakki (From "Youth")</t>
+          <t>Ye Tune Kya Kiya</t>
         </is>
       </c>
       <c r="D44" t="inlineStr">
         <is>
-          <t>G. V. Prakash, Ken Karunaas</t>
+          <t>Pritam, Javed Bashir, Rajat Arora</t>
         </is>
       </c>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>2026-03-26</t>
+          <t>2026-03-27</t>
         </is>
       </c>
       <c r="B45" t="n">
@@ -6534,19 +7571,19 @@
       </c>
       <c r="C45" t="inlineStr">
         <is>
-          <t>Barbaad (From "Saiyaara")</t>
+          <t>Haseen</t>
         </is>
       </c>
       <c r="D45" t="inlineStr">
         <is>
-          <t>The Rish, Jubin Nautiyal</t>
+          <t>Talwiinder, NDS, Rippy Grewal</t>
         </is>
       </c>
     </row>
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>2026-03-26</t>
+          <t>2026-03-27</t>
         </is>
       </c>
       <c r="B46" t="n">
@@ -6554,19 +7591,19 @@
       </c>
       <c r="C46" t="inlineStr">
         <is>
-          <t>Ye Tune Kya Kiya</t>
+          <t>Not Guilty</t>
         </is>
       </c>
       <c r="D46" t="inlineStr">
         <is>
-          <t>Pritam, Javed Bashir, Rajat Arora</t>
+          <t>Dhanda Nyoliwala</t>
         </is>
       </c>
     </row>
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>2026-03-26</t>
+          <t>2026-03-27</t>
         </is>
       </c>
       <c r="B47" t="n">
@@ -6574,19 +7611,19 @@
       </c>
       <c r="C47" t="inlineStr">
         <is>
-          <t>Not Guilty</t>
+          <t>Ehsaas</t>
         </is>
       </c>
       <c r="D47" t="inlineStr">
         <is>
-          <t>Dhanda Nyoliwala</t>
+          <t>Faheem Abdullah, Duha Shah, Vaibhav Pani, Hyder Dar</t>
         </is>
       </c>
     </row>
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>2026-03-26</t>
+          <t>2026-03-27</t>
         </is>
       </c>
       <c r="B48" t="n">
@@ -6594,19 +7631,19 @@
       </c>
       <c r="C48" t="inlineStr">
         <is>
-          <t>Ehsaas</t>
+          <t>Barbaad (From "Saiyaara")</t>
         </is>
       </c>
       <c r="D48" t="inlineStr">
         <is>
-          <t>Faheem Abdullah, Duha Shah, Vaibhav Pani, Hyder Dar</t>
+          <t>The Rish, Jubin Nautiyal</t>
         </is>
       </c>
     </row>
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>2026-03-26</t>
+          <t>2026-03-27</t>
         </is>
       </c>
       <c r="B49" t="n">
@@ -6614,19 +7651,19 @@
       </c>
       <c r="C49" t="inlineStr">
         <is>
-          <t>Aakhri Ishq</t>
+          <t>Hum Pyaar Karne Wale</t>
         </is>
       </c>
       <c r="D49" t="inlineStr">
         <is>
-          <t>Shashwat Sachdev, Jubin Nautiyal, Irshad Kamil</t>
+          <t>Shashwat Sachdev, Anuradha Paudwal, Udit Narayan, Anand-Milind, Sameer Anjaan, Qveen Herby</t>
         </is>
       </c>
     </row>
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>2026-03-26</t>
+          <t>2026-03-27</t>
         </is>
       </c>
       <c r="B50" t="n">
@@ -6634,19 +7671,19 @@
       </c>
       <c r="C50" t="inlineStr">
         <is>
-          <t>Teri Deewani</t>
+          <t>Mast Magan (From "2 States)</t>
         </is>
       </c>
       <c r="D50" t="inlineStr">
         <is>
-          <t>Kailash Kher, Paresh Kamath, Naresh Kamath</t>
+          <t>Arijit Singh, Chinmayi</t>
         </is>
       </c>
     </row>
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>2026-03-26</t>
+          <t>2026-03-27</t>
         </is>
       </c>
       <c r="B51" t="n">
@@ -6654,12 +7691,12 @@
       </c>
       <c r="C51" t="inlineStr">
         <is>
-          <t>Hum Pyaar Karne Wale</t>
+          <t>Teri Deewani</t>
         </is>
       </c>
       <c r="D51" t="inlineStr">
         <is>
-          <t>Shashwat Sachdev, Anuradha Paudwal, Udit Narayan, Anand-Milind, Sameer Anjaan, Qveen Herby</t>
+          <t>Kailash Kher, Paresh Kamath, Naresh Kamath</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
added data for 28th and got predictions for 29th march
</commit_message>
<xml_diff>
--- a/Probability Project.xlsx
+++ b/Probability Project.xlsx
@@ -17,6 +17,7 @@
     <sheet name="AUTO_20260325" sheetId="12" state="visible" r:id="rId12"/>
     <sheet name="AUTO_20260326" sheetId="13" state="visible" r:id="rId13"/>
     <sheet name="AUTO_20260327" sheetId="14" state="visible" r:id="rId14"/>
+    <sheet name="AUTO_20260328" sheetId="15" state="visible" r:id="rId15"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -6701,9 +6702,1045 @@
       </c>
     </row>
     <row r="2">
+      <c r="A2" s="0" t="inlineStr">
+        <is>
+          <t>2026-03-27</t>
+        </is>
+      </c>
+      <c r="B2" s="0" t="n">
+        <v>1</v>
+      </c>
+      <c r="C2" s="0" t="inlineStr">
+        <is>
+          <t>Bairan</t>
+        </is>
+      </c>
+      <c r="D2" s="0" t="inlineStr">
+        <is>
+          <t>Banjaare</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="0" t="inlineStr">
+        <is>
+          <t>2026-03-27</t>
+        </is>
+      </c>
+      <c r="B3" s="0" t="n">
+        <v>2</v>
+      </c>
+      <c r="C3" s="0" t="inlineStr">
+        <is>
+          <t>Jaiye Sajana</t>
+        </is>
+      </c>
+      <c r="D3" s="0" t="inlineStr">
+        <is>
+          <t>Shashwat Sachdev, Jasmine Sandlas, Satinder Sartaaj</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="0" t="inlineStr">
+        <is>
+          <t>2026-03-27</t>
+        </is>
+      </c>
+      <c r="B4" s="0" t="n">
+        <v>3</v>
+      </c>
+      <c r="C4" s="0" t="inlineStr">
+        <is>
+          <t>Sheesha - Aakhya Mai Aakh Ghali Jo Bairan</t>
+        </is>
+      </c>
+      <c r="D4" s="0" t="inlineStr">
+        <is>
+          <t>Mitta Ror, Swara Verma</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="0" t="inlineStr">
+        <is>
+          <t>2026-03-27</t>
+        </is>
+      </c>
+      <c r="B5" s="0" t="n">
+        <v>4</v>
+      </c>
+      <c r="C5" s="0" t="inlineStr">
+        <is>
+          <t>Gehra Hua</t>
+        </is>
+      </c>
+      <c r="D5" s="0" t="inlineStr">
+        <is>
+          <t>Shashwat Sachdev, Arijit Singh, Irshad Kamil, Armaan Khan</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="0" t="inlineStr">
+        <is>
+          <t>2026-03-27</t>
+        </is>
+      </c>
+      <c r="B6" s="0" t="n">
+        <v>5</v>
+      </c>
+      <c r="C6" s="0" t="inlineStr">
+        <is>
+          <t>Dhurandhar The Revenge - Aari Aari</t>
+        </is>
+      </c>
+      <c r="D6" s="0" t="inlineStr">
+        <is>
+          <t>Shashwat Sachdev, Bombay Rockers, Irshad Kamil, Khan Saab, Reble, Token, Jasmine Sandlas, Sudhir Yaduvanshi</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="0" t="inlineStr">
+        <is>
+          <t>2026-03-27</t>
+        </is>
+      </c>
+      <c r="B7" s="0" t="n">
+        <v>6</v>
+      </c>
+      <c r="C7" s="0" t="inlineStr">
+        <is>
+          <t>Jaan Se Guzarte Hain</t>
+        </is>
+      </c>
+      <c r="D7" s="0" t="inlineStr">
+        <is>
+          <t>Shashwat Sachdev, Khan Saab, Nusrat Fateh Ali Khan</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="0" t="inlineStr">
+        <is>
+          <t>2026-03-27</t>
+        </is>
+      </c>
+      <c r="B8" s="0" t="n">
+        <v>7</v>
+      </c>
+      <c r="C8" s="0" t="inlineStr">
+        <is>
+          <t>Khat</t>
+        </is>
+      </c>
+      <c r="D8" s="0" t="inlineStr">
+        <is>
+          <t>Navjot Ahuja</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="0" t="inlineStr">
+        <is>
+          <t>2026-03-27</t>
+        </is>
+      </c>
+      <c r="B9" s="0" t="n">
+        <v>8</v>
+      </c>
+      <c r="C9" s="0" t="inlineStr">
+        <is>
+          <t>Sitaare (From "Ikkis")</t>
+        </is>
+      </c>
+      <c r="D9" s="0" t="inlineStr">
+        <is>
+          <t>Arijit Singh, White Noise Collectives, Amitabh Bhattacharya</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="0" t="inlineStr">
+        <is>
+          <t>2026-03-27</t>
+        </is>
+      </c>
+      <c r="B10" s="0" t="n">
+        <v>9</v>
+      </c>
+      <c r="C10" s="0" t="inlineStr">
+        <is>
+          <t>Dooron Dooron</t>
+        </is>
+      </c>
+      <c r="D10" s="0" t="inlineStr">
+        <is>
+          <t>Paresh Pahuja, Shiv Tandan, Meghdeep Bose</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="0" t="inlineStr">
+        <is>
+          <t>2026-03-27</t>
+        </is>
+      </c>
+      <c r="B11" s="0" t="n">
+        <v>10</v>
+      </c>
+      <c r="C11" s="0" t="inlineStr">
+        <is>
+          <t>Sahiba</t>
+        </is>
+      </c>
+      <c r="D11" s="0" t="inlineStr">
+        <is>
+          <t>Aditya Rikhari</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="0" t="inlineStr">
+        <is>
+          <t>2026-03-27</t>
+        </is>
+      </c>
+      <c r="B12" s="0" t="n">
+        <v>11</v>
+      </c>
+      <c r="C12" s="0" t="inlineStr">
+        <is>
+          <t>Apna Bana Le</t>
+        </is>
+      </c>
+      <c r="D12" s="0" t="inlineStr">
+        <is>
+          <t>Sachin-Jigar, Arijit Singh, Amitabh Bhattacharya</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="0" t="inlineStr">
+        <is>
+          <t>2026-03-27</t>
+        </is>
+      </c>
+      <c r="B13" s="0" t="n">
+        <v>12</v>
+      </c>
+      <c r="C13" s="0" t="inlineStr">
+        <is>
+          <t>Shararat</t>
+        </is>
+      </c>
+      <c r="D13" s="0" t="inlineStr">
+        <is>
+          <t>Shashwat Sachdev, Madhubanti Bagchi, Jasmine Sandlas</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="0" t="inlineStr">
+        <is>
+          <t>2026-03-27</t>
+        </is>
+      </c>
+      <c r="B14" s="0" t="n">
+        <v>13</v>
+      </c>
+      <c r="C14" s="0" t="inlineStr">
+        <is>
+          <t>Samjhawan</t>
+        </is>
+      </c>
+      <c r="D14" s="0" t="inlineStr">
+        <is>
+          <t>Jawad Ahmad, Shaarib Toshi, Arijit Singh, Shreya Ghoshal</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="0" t="inlineStr">
+        <is>
+          <t>2026-03-27</t>
+        </is>
+      </c>
+      <c r="B15" s="0" t="n">
+        <v>14</v>
+      </c>
+      <c r="C15" s="0" t="inlineStr">
+        <is>
+          <t>Finding Her</t>
+        </is>
+      </c>
+      <c r="D15" s="0" t="inlineStr">
+        <is>
+          <t>Kushagra, Bharath, Saaheal</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="0" t="inlineStr">
+        <is>
+          <t>2026-03-27</t>
+        </is>
+      </c>
+      <c r="B16" s="0" t="n">
+        <v>15</v>
+      </c>
+      <c r="C16" s="0" t="inlineStr">
+        <is>
+          <t>Dhurandhar - Title Track</t>
+        </is>
+      </c>
+      <c r="D16" s="0" t="inlineStr">
+        <is>
+          <t>Shashwat Sachdev, Hanumankind, Jasmine Sandlas, Sudhir Yaduvanshi, Charanjit Ahuja, Muhammad Sadiq, Ranjit Kaur, Babu Singh Maan</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="0" t="inlineStr">
+        <is>
+          <t>2026-03-27</t>
+        </is>
+      </c>
+      <c r="B17" s="0" t="n">
+        <v>16</v>
+      </c>
+      <c r="C17" s="0" t="inlineStr">
+        <is>
+          <t>Arz Kiya Hai | Coke Studio Bharat</t>
+        </is>
+      </c>
+      <c r="D17" s="0" t="inlineStr">
+        <is>
+          <t>Anuv Jain</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="0" t="inlineStr">
+        <is>
+          <t>2026-03-27</t>
+        </is>
+      </c>
+      <c r="B18" s="0" t="n">
+        <v>17</v>
+      </c>
+      <c r="C18" s="0" t="inlineStr">
+        <is>
+          <t>Pavazha Malli - From "Think Indie"</t>
+        </is>
+      </c>
+      <c r="D18" s="0" t="inlineStr">
+        <is>
+          <t>Sai Abhyankkar, Shruti Haasan, Vivek</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="0" t="inlineStr">
+        <is>
+          <t>2026-03-27</t>
+        </is>
+      </c>
+      <c r="B19" s="0" t="n">
+        <v>18</v>
+      </c>
+      <c r="C19" s="0" t="inlineStr">
+        <is>
+          <t>Boyfriend</t>
+        </is>
+      </c>
+      <c r="D19" s="0" t="inlineStr">
+        <is>
+          <t>Karan Aujla, Ikky</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="0" t="inlineStr">
+        <is>
+          <t>2026-03-27</t>
+        </is>
+      </c>
+      <c r="B20" s="0" t="n">
+        <v>19</v>
+      </c>
+      <c r="C20" s="0" t="inlineStr">
+        <is>
+          <t>Ishq</t>
+        </is>
+      </c>
+      <c r="D20" s="0" t="inlineStr">
+        <is>
+          <t>Faheem Abdullah, Rauhan Malik, Amir Ameer</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="0" t="inlineStr">
+        <is>
+          <t>2026-03-27</t>
+        </is>
+      </c>
+      <c r="B21" s="0" t="n">
+        <v>20</v>
+      </c>
+      <c r="C21" s="0" t="inlineStr">
+        <is>
+          <t>For A Reason</t>
+        </is>
+      </c>
+      <c r="D21" s="0" t="inlineStr">
+        <is>
+          <t>Karan Aujla, Ikky</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="0" t="inlineStr">
+        <is>
+          <t>2026-03-27</t>
+        </is>
+      </c>
+      <c r="B22" s="0" t="n">
+        <v>21</v>
+      </c>
+      <c r="C22" s="0" t="inlineStr">
+        <is>
+          <t>Naal Nachna</t>
+        </is>
+      </c>
+      <c r="D22" s="0" t="inlineStr">
+        <is>
+          <t>Shashwat Sachdev, Afsana Khan, Irshad Kamil, Reble</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="0" t="inlineStr">
+        <is>
+          <t>2026-03-27</t>
+        </is>
+      </c>
+      <c r="B23" s="0" t="n">
+        <v>22</v>
+      </c>
+      <c r="C23" s="0" t="inlineStr">
+        <is>
+          <t>Bairi</t>
+        </is>
+      </c>
+      <c r="D23" s="0" t="inlineStr">
+        <is>
+          <t>Virat, Pradeep Solanki, Heena</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="0" t="inlineStr">
+        <is>
+          <t>2026-03-27</t>
+        </is>
+      </c>
+      <c r="B24" s="0" t="n">
+        <v>23</v>
+      </c>
+      <c r="C24" s="0" t="inlineStr">
+        <is>
+          <t>Mann Mera</t>
+        </is>
+      </c>
+      <c r="D24" s="0" t="inlineStr">
+        <is>
+          <t>Gajendra Verma</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="0" t="inlineStr">
+        <is>
+          <t>2026-03-27</t>
+        </is>
+      </c>
+      <c r="B25" s="0" t="n">
+        <v>24</v>
+      </c>
+      <c r="C25" s="0" t="inlineStr">
+        <is>
+          <t>Saiyaara</t>
+        </is>
+      </c>
+      <c r="D25" s="0" t="inlineStr">
+        <is>
+          <t>Tanishk Bagchi, Faheem Abdullah, Arslan Nizami, Irshad Kamil</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="0" t="inlineStr">
+        <is>
+          <t>2026-03-27</t>
+        </is>
+      </c>
+      <c r="B26" s="0" t="n">
+        <v>25</v>
+      </c>
+      <c r="C26" s="0" t="inlineStr">
+        <is>
+          <t>Ishqa Ve</t>
+        </is>
+      </c>
+      <c r="D26" s="0" t="inlineStr">
+        <is>
+          <t>Zeeshan Ali, Yuvraj Tung, Sandeep Aulakh, Honey Dhillon</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="0" t="inlineStr">
+        <is>
+          <t>2026-03-27</t>
+        </is>
+      </c>
+      <c r="B27" s="0" t="n">
+        <v>26</v>
+      </c>
+      <c r="C27" s="0" t="inlineStr">
+        <is>
+          <t>Tere Liye</t>
+        </is>
+      </c>
+      <c r="D27" s="0" t="inlineStr">
+        <is>
+          <t>Atif Aslam, Shreya Ghoshal, Sachin Gupta, Sameer Anjaan</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="0" t="inlineStr">
+        <is>
+          <t>2026-03-27</t>
+        </is>
+      </c>
+      <c r="B28" s="0" t="n">
+        <v>27</v>
+      </c>
+      <c r="C28" s="0" t="inlineStr">
+        <is>
+          <t>Deewaana Deewaana</t>
+        </is>
+      </c>
+      <c r="D28" s="0" t="inlineStr">
+        <is>
+          <t>A.R. Rahman, Irshad Kamil</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="0" t="inlineStr">
+        <is>
+          <t>2026-03-27</t>
+        </is>
+      </c>
+      <c r="B29" s="0" t="n">
+        <v>28</v>
+      </c>
+      <c r="C29" s="0" t="inlineStr">
+        <is>
+          <t>Phir Se</t>
+        </is>
+      </c>
+      <c r="D29" s="0" t="inlineStr">
+        <is>
+          <t>Shashwat Sachdev, Arijit Singh, Irshad Kamil</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="0" t="inlineStr">
+        <is>
+          <t>2026-03-27</t>
+        </is>
+      </c>
+      <c r="B30" s="0" t="n">
+        <v>29</v>
+      </c>
+      <c r="C30" s="0" t="inlineStr">
+        <is>
+          <t>Raanjhan (From "Do Patti")</t>
+        </is>
+      </c>
+      <c r="D30" s="0" t="inlineStr">
+        <is>
+          <t>Sachet-Parampara, Parampara Tandon, Kausar Munir</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="0" t="inlineStr">
+        <is>
+          <t>2026-03-27</t>
+        </is>
+      </c>
+      <c r="B31" s="0" t="n">
+        <v>30</v>
+      </c>
+      <c r="C31" s="0" t="inlineStr">
+        <is>
+          <t>Lutt Le Gaya</t>
+        </is>
+      </c>
+      <c r="D31" s="0" t="inlineStr">
+        <is>
+          <t>Shashwat Sachdev, Simran Choudhary</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="0" t="inlineStr">
+        <is>
+          <t>2026-03-27</t>
+        </is>
+      </c>
+      <c r="B32" s="0" t="n">
+        <v>31</v>
+      </c>
+      <c r="C32" s="0" t="inlineStr">
+        <is>
+          <t>Main Aur Tu (From "Dhurandhar The Revenge")</t>
+        </is>
+      </c>
+      <c r="D32" s="0" t="inlineStr">
+        <is>
+          <t>Shashwat Sachdev, Jasmine Sandlas, Reble</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="0" t="inlineStr">
+        <is>
+          <t>2026-03-27</t>
+        </is>
+      </c>
+      <c r="B33" s="0" t="n">
+        <v>32</v>
+      </c>
+      <c r="C33" s="0" t="inlineStr">
+        <is>
+          <t>Darkhaast</t>
+        </is>
+      </c>
+      <c r="D33" s="0" t="inlineStr">
+        <is>
+          <t>Mithoon, Arijit Singh, Sunidhi Chauhan, Sayeed Quadri</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="0" t="inlineStr">
+        <is>
+          <t>2026-03-27</t>
+        </is>
+      </c>
+      <c r="B34" s="0" t="n">
+        <v>33</v>
+      </c>
+      <c r="C34" s="0" t="inlineStr">
+        <is>
+          <t>Run Down The City - Monica</t>
+        </is>
+      </c>
+      <c r="D34" s="0" t="inlineStr">
+        <is>
+          <t>Shashwat Sachdev, Reble, Asha Bhosle, R. D. Burman, Majrooh Sultanpuri</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="0" t="inlineStr">
+        <is>
+          <t>2026-03-27</t>
+        </is>
+      </c>
+      <c r="B35" s="0" t="n">
+        <v>34</v>
+      </c>
+      <c r="C35" s="0" t="inlineStr">
+        <is>
+          <t>Tere Bina</t>
+        </is>
+      </c>
+      <c r="D35" s="0" t="inlineStr">
+        <is>
+          <t>A.R. Rahman, Chinmayi, Murtuza Khan, Qadir Khan</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="0" t="inlineStr">
+        <is>
+          <t>2026-03-27</t>
+        </is>
+      </c>
+      <c r="B36" s="0" t="n">
+        <v>35</v>
+      </c>
+      <c r="C36" s="0" t="inlineStr">
+        <is>
+          <t>Tum Ho Toh (From "Saiyaara")</t>
+        </is>
+      </c>
+      <c r="D36" s="0" t="inlineStr">
+        <is>
+          <t>Vishal Mishra, Hansika Pareek, Raj Shekhar</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="0" t="inlineStr">
+        <is>
+          <t>2026-03-27</t>
+        </is>
+      </c>
+      <c r="B37" s="0" t="n">
+        <v>36</v>
+      </c>
+      <c r="C37" s="0" t="inlineStr">
+        <is>
+          <t>Ishq Jalakar - Karvaan</t>
+        </is>
+      </c>
+      <c r="D37" s="0" t="inlineStr">
+        <is>
+          <t>Shashwat Sachdev, Shahzad Ali, Subhadeep Das Chowdhury, Armaan Khan, Irshad Kamil, Roshan, Sahir Ludhianvi</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="0" t="inlineStr">
+        <is>
+          <t>2026-03-27</t>
+        </is>
+      </c>
+      <c r="B38" s="0" t="n">
+        <v>37</v>
+      </c>
+      <c r="C38" s="0" t="inlineStr">
+        <is>
+          <t>Jogi</t>
+        </is>
+      </c>
+      <c r="D38" s="0" t="inlineStr">
+        <is>
+          <t>thiarajxtt, Bir</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="0" t="inlineStr">
+        <is>
+          <t>2026-03-27</t>
+        </is>
+      </c>
+      <c r="B39" s="0" t="n">
+        <v>38</v>
+      </c>
+      <c r="C39" s="0" t="inlineStr">
+        <is>
+          <t>Agar Tum Saath Ho (From "Tamasha")</t>
+        </is>
+      </c>
+      <c r="D39" s="0" t="inlineStr">
+        <is>
+          <t>Alka Yagnik, Arijit Singh</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="0" t="inlineStr">
+        <is>
+          <t>2026-03-27</t>
+        </is>
+      </c>
+      <c r="B40" s="0" t="n">
+        <v>39</v>
+      </c>
+      <c r="C40" s="0" t="inlineStr">
+        <is>
+          <t>SWIM</t>
+        </is>
+      </c>
+      <c r="D40" s="0" t="inlineStr">
+        <is>
+          <t>BTS</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" s="0" t="inlineStr">
+        <is>
+          <t>2026-03-27</t>
+        </is>
+      </c>
+      <c r="B41" s="0" t="n">
+        <v>40</v>
+      </c>
+      <c r="C41" s="0" t="inlineStr">
+        <is>
+          <t>Aaya Sher (From "The Paradise") (Telugu)</t>
+        </is>
+      </c>
+      <c r="D41" s="0" t="inlineStr">
+        <is>
+          <t>Anirudh Ravichander, Jangi Reddy, Arjun Chandy, Kasarla Shyam</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" s="0" t="inlineStr">
+        <is>
+          <t>2026-03-27</t>
+        </is>
+      </c>
+      <c r="B42" s="0" t="n">
+        <v>41</v>
+      </c>
+      <c r="C42" s="0" t="inlineStr">
+        <is>
+          <t>Jo Tum Mere Ho</t>
+        </is>
+      </c>
+      <c r="D42" s="0" t="inlineStr">
+        <is>
+          <t>Anuv Jain</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" s="0" t="inlineStr">
+        <is>
+          <t>2026-03-27</t>
+        </is>
+      </c>
+      <c r="B43" s="0" t="n">
+        <v>42</v>
+      </c>
+      <c r="C43" s="0" t="inlineStr">
+        <is>
+          <t>Mutta Kalakki (From "Youth")</t>
+        </is>
+      </c>
+      <c r="D43" s="0" t="inlineStr">
+        <is>
+          <t>G. V. Prakash, Ken Karunaas</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" s="0" t="inlineStr">
+        <is>
+          <t>2026-03-27</t>
+        </is>
+      </c>
+      <c r="B44" s="0" t="n">
+        <v>43</v>
+      </c>
+      <c r="C44" s="0" t="inlineStr">
+        <is>
+          <t>Ye Tune Kya Kiya</t>
+        </is>
+      </c>
+      <c r="D44" s="0" t="inlineStr">
+        <is>
+          <t>Pritam, Javed Bashir, Rajat Arora</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" s="0" t="inlineStr">
+        <is>
+          <t>2026-03-27</t>
+        </is>
+      </c>
+      <c r="B45" s="0" t="n">
+        <v>44</v>
+      </c>
+      <c r="C45" s="0" t="inlineStr">
+        <is>
+          <t>Haseen</t>
+        </is>
+      </c>
+      <c r="D45" s="0" t="inlineStr">
+        <is>
+          <t>Talwiinder, NDS, Rippy Grewal</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" s="0" t="inlineStr">
+        <is>
+          <t>2026-03-27</t>
+        </is>
+      </c>
+      <c r="B46" s="0" t="n">
+        <v>45</v>
+      </c>
+      <c r="C46" s="0" t="inlineStr">
+        <is>
+          <t>Not Guilty</t>
+        </is>
+      </c>
+      <c r="D46" s="0" t="inlineStr">
+        <is>
+          <t>Dhanda Nyoliwala</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" s="0" t="inlineStr">
+        <is>
+          <t>2026-03-27</t>
+        </is>
+      </c>
+      <c r="B47" s="0" t="n">
+        <v>46</v>
+      </c>
+      <c r="C47" s="0" t="inlineStr">
+        <is>
+          <t>Ehsaas</t>
+        </is>
+      </c>
+      <c r="D47" s="0" t="inlineStr">
+        <is>
+          <t>Faheem Abdullah, Duha Shah, Vaibhav Pani, Hyder Dar</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" s="0" t="inlineStr">
+        <is>
+          <t>2026-03-27</t>
+        </is>
+      </c>
+      <c r="B48" s="0" t="n">
+        <v>47</v>
+      </c>
+      <c r="C48" s="0" t="inlineStr">
+        <is>
+          <t>Barbaad (From "Saiyaara")</t>
+        </is>
+      </c>
+      <c r="D48" s="0" t="inlineStr">
+        <is>
+          <t>The Rish, Jubin Nautiyal</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" s="0" t="inlineStr">
+        <is>
+          <t>2026-03-27</t>
+        </is>
+      </c>
+      <c r="B49" s="0" t="n">
+        <v>48</v>
+      </c>
+      <c r="C49" s="0" t="inlineStr">
+        <is>
+          <t>Hum Pyaar Karne Wale</t>
+        </is>
+      </c>
+      <c r="D49" s="0" t="inlineStr">
+        <is>
+          <t>Shashwat Sachdev, Anuradha Paudwal, Udit Narayan, Anand-Milind, Sameer Anjaan, Qveen Herby</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" s="0" t="inlineStr">
+        <is>
+          <t>2026-03-27</t>
+        </is>
+      </c>
+      <c r="B50" s="0" t="n">
+        <v>49</v>
+      </c>
+      <c r="C50" s="0" t="inlineStr">
+        <is>
+          <t>Mast Magan (From "2 States)</t>
+        </is>
+      </c>
+      <c r="D50" s="0" t="inlineStr">
+        <is>
+          <t>Arijit Singh, Chinmayi</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" s="0" t="inlineStr">
+        <is>
+          <t>2026-03-27</t>
+        </is>
+      </c>
+      <c r="B51" s="0" t="n">
+        <v>50</v>
+      </c>
+      <c r="C51" s="0" t="inlineStr">
+        <is>
+          <t>Teri Deewani</t>
+        </is>
+      </c>
+      <c r="D51" s="0" t="inlineStr">
+        <is>
+          <t>Kailash Kher, Paresh Kamath, Naresh Kamath</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet15.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:D51"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="24" t="inlineStr">
+        <is>
+          <t>Date</t>
+        </is>
+      </c>
+      <c r="B1" s="24" t="inlineStr">
+        <is>
+          <t>Rank</t>
+        </is>
+      </c>
+      <c r="C1" s="24" t="inlineStr">
+        <is>
+          <t>Song</t>
+        </is>
+      </c>
+      <c r="D1" s="24" t="inlineStr">
+        <is>
+          <t>Artist</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>2026-03-27</t>
+          <t>2026-03-28</t>
         </is>
       </c>
       <c r="B2" t="n">
@@ -6723,7 +7760,7 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>2026-03-27</t>
+          <t>2026-03-28</t>
         </is>
       </c>
       <c r="B3" t="n">
@@ -6743,7 +7780,7 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>2026-03-27</t>
+          <t>2026-03-28</t>
         </is>
       </c>
       <c r="B4" t="n">
@@ -6751,19 +7788,19 @@
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>Sheesha - Aakhya Mai Aakh Ghali Jo Bairan</t>
+          <t>Gehra Hua</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>Mitta Ror, Swara Verma</t>
+          <t>Shashwat Sachdev, Arijit Singh, Irshad Kamil, Armaan Khan</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>2026-03-27</t>
+          <t>2026-03-28</t>
         </is>
       </c>
       <c r="B5" t="n">
@@ -6771,19 +7808,19 @@
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>Gehra Hua</t>
+          <t>Sheesha - Aakhya Mai Aakh Ghali Jo Bairan</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>Shashwat Sachdev, Arijit Singh, Irshad Kamil, Armaan Khan</t>
+          <t>Mitta Ror, Swara Verma</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>2026-03-27</t>
+          <t>2026-03-28</t>
         </is>
       </c>
       <c r="B6" t="n">
@@ -6803,7 +7840,7 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>2026-03-27</t>
+          <t>2026-03-28</t>
         </is>
       </c>
       <c r="B7" t="n">
@@ -6811,19 +7848,19 @@
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>Jaan Se Guzarte Hain</t>
+          <t>Khat</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>Shashwat Sachdev, Khan Saab, Nusrat Fateh Ali Khan</t>
+          <t>Navjot Ahuja</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>2026-03-27</t>
+          <t>2026-03-28</t>
         </is>
       </c>
       <c r="B8" t="n">
@@ -6831,19 +7868,19 @@
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>Khat</t>
+          <t>Jaan Se Guzarte Hain</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>Navjot Ahuja</t>
+          <t>Shashwat Sachdev, Khan Saab, Nusrat Fateh Ali Khan</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>2026-03-27</t>
+          <t>2026-03-28</t>
         </is>
       </c>
       <c r="B9" t="n">
@@ -6863,7 +7900,7 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>2026-03-27</t>
+          <t>2026-03-28</t>
         </is>
       </c>
       <c r="B10" t="n">
@@ -6883,7 +7920,7 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>2026-03-27</t>
+          <t>2026-03-28</t>
         </is>
       </c>
       <c r="B11" t="n">
@@ -6903,7 +7940,7 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>2026-03-27</t>
+          <t>2026-03-28</t>
         </is>
       </c>
       <c r="B12" t="n">
@@ -6911,19 +7948,19 @@
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>Apna Bana Le</t>
+          <t>Shararat</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>Sachin-Jigar, Arijit Singh, Amitabh Bhattacharya</t>
+          <t>Shashwat Sachdev, Madhubanti Bagchi, Jasmine Sandlas</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>2026-03-27</t>
+          <t>2026-03-28</t>
         </is>
       </c>
       <c r="B13" t="n">
@@ -6931,19 +7968,19 @@
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>Shararat</t>
+          <t>Finding Her</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>Shashwat Sachdev, Madhubanti Bagchi, Jasmine Sandlas</t>
+          <t>Kushagra, Bharath, Saaheal</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>2026-03-27</t>
+          <t>2026-03-28</t>
         </is>
       </c>
       <c r="B14" t="n">
@@ -6951,19 +7988,19 @@
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>Samjhawan</t>
+          <t>Apna Bana Le</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>Jawad Ahmad, Shaarib Toshi, Arijit Singh, Shreya Ghoshal</t>
+          <t>Sachin-Jigar, Arijit Singh, Amitabh Bhattacharya</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>2026-03-27</t>
+          <t>2026-03-28</t>
         </is>
       </c>
       <c r="B15" t="n">
@@ -6971,19 +8008,19 @@
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>Finding Her</t>
+          <t>Samjhawan</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>Kushagra, Bharath, Saaheal</t>
+          <t>Jawad Ahmad, Shaarib Toshi, Arijit Singh, Shreya Ghoshal</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>2026-03-27</t>
+          <t>2026-03-28</t>
         </is>
       </c>
       <c r="B16" t="n">
@@ -7003,7 +8040,7 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>2026-03-27</t>
+          <t>2026-03-28</t>
         </is>
       </c>
       <c r="B17" t="n">
@@ -7011,19 +8048,19 @@
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>Arz Kiya Hai | Coke Studio Bharat</t>
+          <t>Pavazha Malli - From "Think Indie"</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>Anuv Jain</t>
+          <t>Sai Abhyankkar, Shruti Haasan, Vivek</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>2026-03-27</t>
+          <t>2026-03-28</t>
         </is>
       </c>
       <c r="B18" t="n">
@@ -7031,19 +8068,19 @@
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>Pavazha Malli - From "Think Indie"</t>
+          <t>Ishq</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>Sai Abhyankkar, Shruti Haasan, Vivek</t>
+          <t>Faheem Abdullah, Rauhan Malik, Amir Ameer</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>2026-03-27</t>
+          <t>2026-03-28</t>
         </is>
       </c>
       <c r="B19" t="n">
@@ -7051,19 +8088,19 @@
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>Boyfriend</t>
+          <t>Arz Kiya Hai | Coke Studio Bharat</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>Karan Aujla, Ikky</t>
+          <t>Anuv Jain</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>2026-03-27</t>
+          <t>2026-03-28</t>
         </is>
       </c>
       <c r="B20" t="n">
@@ -7071,19 +8108,19 @@
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>Ishq</t>
+          <t>For A Reason</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>Faheem Abdullah, Rauhan Malik, Amir Ameer</t>
+          <t>Karan Aujla, Ikky</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>2026-03-27</t>
+          <t>2026-03-28</t>
         </is>
       </c>
       <c r="B21" t="n">
@@ -7091,7 +8128,7 @@
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>For A Reason</t>
+          <t>Boyfriend</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
@@ -7103,7 +8140,7 @@
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>2026-03-27</t>
+          <t>2026-03-28</t>
         </is>
       </c>
       <c r="B22" t="n">
@@ -7111,19 +8148,19 @@
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>Naal Nachna</t>
+          <t>Mann Mera</t>
         </is>
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>Shashwat Sachdev, Afsana Khan, Irshad Kamil, Reble</t>
+          <t>Gajendra Verma</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>2026-03-27</t>
+          <t>2026-03-28</t>
         </is>
       </c>
       <c r="B23" t="n">
@@ -7131,19 +8168,19 @@
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>Bairi</t>
+          <t>Naal Nachna</t>
         </is>
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>Virat, Pradeep Solanki, Heena</t>
+          <t>Shashwat Sachdev, Afsana Khan, Irshad Kamil, Reble</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>2026-03-27</t>
+          <t>2026-03-28</t>
         </is>
       </c>
       <c r="B24" t="n">
@@ -7151,19 +8188,19 @@
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>Mann Mera</t>
+          <t>Bairi</t>
         </is>
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>Gajendra Verma</t>
+          <t>Virat, Pradeep Solanki, Heena</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>2026-03-27</t>
+          <t>2026-03-28</t>
         </is>
       </c>
       <c r="B25" t="n">
@@ -7183,7 +8220,7 @@
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>2026-03-27</t>
+          <t>2026-03-28</t>
         </is>
       </c>
       <c r="B26" t="n">
@@ -7191,19 +8228,19 @@
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>Ishqa Ve</t>
+          <t>Phir Se</t>
         </is>
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>Zeeshan Ali, Yuvraj Tung, Sandeep Aulakh, Honey Dhillon</t>
+          <t>Shashwat Sachdev, Arijit Singh, Irshad Kamil</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>2026-03-27</t>
+          <t>2026-03-28</t>
         </is>
       </c>
       <c r="B27" t="n">
@@ -7211,19 +8248,19 @@
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>Tere Liye</t>
+          <t>Ishqa Ve</t>
         </is>
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t>Atif Aslam, Shreya Ghoshal, Sachin Gupta, Sameer Anjaan</t>
+          <t>Zeeshan Ali, Yuvraj Tung, Sandeep Aulakh, Honey Dhillon</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>2026-03-27</t>
+          <t>2026-03-28</t>
         </is>
       </c>
       <c r="B28" t="n">
@@ -7231,19 +8268,19 @@
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>Deewaana Deewaana</t>
+          <t>Tere Liye</t>
         </is>
       </c>
       <c r="D28" t="inlineStr">
         <is>
-          <t>A.R. Rahman, Irshad Kamil</t>
+          <t>Atif Aslam, Shreya Ghoshal, Sachin Gupta, Sameer Anjaan</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>2026-03-27</t>
+          <t>2026-03-28</t>
         </is>
       </c>
       <c r="B29" t="n">
@@ -7251,19 +8288,19 @@
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>Phir Se</t>
+          <t>Deewaana Deewaana</t>
         </is>
       </c>
       <c r="D29" t="inlineStr">
         <is>
-          <t>Shashwat Sachdev, Arijit Singh, Irshad Kamil</t>
+          <t>A.R. Rahman, Irshad Kamil</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>2026-03-27</t>
+          <t>2026-03-28</t>
         </is>
       </c>
       <c r="B30" t="n">
@@ -7271,19 +8308,19 @@
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>Raanjhan (From "Do Patti")</t>
+          <t>Lutt Le Gaya</t>
         </is>
       </c>
       <c r="D30" t="inlineStr">
         <is>
-          <t>Sachet-Parampara, Parampara Tandon, Kausar Munir</t>
+          <t>Shashwat Sachdev, Simran Choudhary</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>2026-03-27</t>
+          <t>2026-03-28</t>
         </is>
       </c>
       <c r="B31" t="n">
@@ -7291,19 +8328,19 @@
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>Lutt Le Gaya</t>
+          <t>Main Aur Tu (From "Dhurandhar The Revenge")</t>
         </is>
       </c>
       <c r="D31" t="inlineStr">
         <is>
-          <t>Shashwat Sachdev, Simran Choudhary</t>
+          <t>Shashwat Sachdev, Jasmine Sandlas, Reble</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>2026-03-27</t>
+          <t>2026-03-28</t>
         </is>
       </c>
       <c r="B32" t="n">
@@ -7311,19 +8348,19 @@
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>Main Aur Tu (From "Dhurandhar The Revenge")</t>
+          <t>Raanjhan (From "Do Patti")</t>
         </is>
       </c>
       <c r="D32" t="inlineStr">
         <is>
-          <t>Shashwat Sachdev, Jasmine Sandlas, Reble</t>
+          <t>Sachet-Parampara, Parampara Tandon, Kausar Munir</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>2026-03-27</t>
+          <t>2026-03-28</t>
         </is>
       </c>
       <c r="B33" t="n">
@@ -7331,19 +8368,19 @@
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>Darkhaast</t>
+          <t>Ishq Jalakar - Karvaan</t>
         </is>
       </c>
       <c r="D33" t="inlineStr">
         <is>
-          <t>Mithoon, Arijit Singh, Sunidhi Chauhan, Sayeed Quadri</t>
+          <t>Shashwat Sachdev, Shahzad Ali, Subhadeep Das Chowdhury, Armaan Khan, Irshad Kamil, Roshan, Sahir Ludhianvi</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>2026-03-27</t>
+          <t>2026-03-28</t>
         </is>
       </c>
       <c r="B34" t="n">
@@ -7363,7 +8400,7 @@
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>2026-03-27</t>
+          <t>2026-03-28</t>
         </is>
       </c>
       <c r="B35" t="n">
@@ -7371,19 +8408,19 @@
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>Tere Bina</t>
+          <t>Tum Ho Toh (From "Saiyaara")</t>
         </is>
       </c>
       <c r="D35" t="inlineStr">
         <is>
-          <t>A.R. Rahman, Chinmayi, Murtuza Khan, Qadir Khan</t>
+          <t>Vishal Mishra, Hansika Pareek, Raj Shekhar</t>
         </is>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>2026-03-27</t>
+          <t>2026-03-28</t>
         </is>
       </c>
       <c r="B36" t="n">
@@ -7391,19 +8428,19 @@
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>Tum Ho Toh (From "Saiyaara")</t>
+          <t>Darkhaast</t>
         </is>
       </c>
       <c r="D36" t="inlineStr">
         <is>
-          <t>Vishal Mishra, Hansika Pareek, Raj Shekhar</t>
+          <t>Mithoon, Arijit Singh, Sunidhi Chauhan, Sayeed Quadri</t>
         </is>
       </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>2026-03-27</t>
+          <t>2026-03-28</t>
         </is>
       </c>
       <c r="B37" t="n">
@@ -7411,19 +8448,19 @@
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>Ishq Jalakar - Karvaan</t>
+          <t>Agar Tum Saath Ho (From "Tamasha")</t>
         </is>
       </c>
       <c r="D37" t="inlineStr">
         <is>
-          <t>Shashwat Sachdev, Shahzad Ali, Subhadeep Das Chowdhury, Armaan Khan, Irshad Kamil, Roshan, Sahir Ludhianvi</t>
+          <t>Alka Yagnik, Arijit Singh</t>
         </is>
       </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>2026-03-27</t>
+          <t>2026-03-28</t>
         </is>
       </c>
       <c r="B38" t="n">
@@ -7431,19 +8468,19 @@
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>Jogi</t>
+          <t>Tere Bina</t>
         </is>
       </c>
       <c r="D38" t="inlineStr">
         <is>
-          <t>thiarajxtt, Bir</t>
+          <t>A.R. Rahman, Chinmayi, Murtuza Khan, Qadir Khan</t>
         </is>
       </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>2026-03-27</t>
+          <t>2026-03-28</t>
         </is>
       </c>
       <c r="B39" t="n">
@@ -7451,19 +8488,19 @@
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>Agar Tum Saath Ho (From "Tamasha")</t>
+          <t>Jo Tum Mere Ho</t>
         </is>
       </c>
       <c r="D39" t="inlineStr">
         <is>
-          <t>Alka Yagnik, Arijit Singh</t>
+          <t>Anuv Jain</t>
         </is>
       </c>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>2026-03-27</t>
+          <t>2026-03-28</t>
         </is>
       </c>
       <c r="B40" t="n">
@@ -7471,19 +8508,19 @@
       </c>
       <c r="C40" t="inlineStr">
         <is>
-          <t>SWIM</t>
+          <t>Aaya Sher (From "The Paradise") (Telugu)</t>
         </is>
       </c>
       <c r="D40" t="inlineStr">
         <is>
-          <t>BTS</t>
+          <t>Anirudh Ravichander, Jangi Reddy, Arjun Chandy, Kasarla Shyam</t>
         </is>
       </c>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>2026-03-27</t>
+          <t>2026-03-28</t>
         </is>
       </c>
       <c r="B41" t="n">
@@ -7491,19 +8528,19 @@
       </c>
       <c r="C41" t="inlineStr">
         <is>
-          <t>Aaya Sher (From "The Paradise") (Telugu)</t>
+          <t>Mutta Kalakki (From "Youth")</t>
         </is>
       </c>
       <c r="D41" t="inlineStr">
         <is>
-          <t>Anirudh Ravichander, Jangi Reddy, Arjun Chandy, Kasarla Shyam</t>
+          <t>G. V. Prakash, Ken Karunaas</t>
         </is>
       </c>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>2026-03-27</t>
+          <t>2026-03-28</t>
         </is>
       </c>
       <c r="B42" t="n">
@@ -7511,19 +8548,19 @@
       </c>
       <c r="C42" t="inlineStr">
         <is>
-          <t>Jo Tum Mere Ho</t>
+          <t>Ye Tune Kya Kiya</t>
         </is>
       </c>
       <c r="D42" t="inlineStr">
         <is>
-          <t>Anuv Jain</t>
+          <t>Pritam, Javed Bashir, Rajat Arora</t>
         </is>
       </c>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>2026-03-27</t>
+          <t>2026-03-28</t>
         </is>
       </c>
       <c r="B43" t="n">
@@ -7531,19 +8568,19 @@
       </c>
       <c r="C43" t="inlineStr">
         <is>
-          <t>Mutta Kalakki (From "Youth")</t>
+          <t>Haseen</t>
         </is>
       </c>
       <c r="D43" t="inlineStr">
         <is>
-          <t>G. V. Prakash, Ken Karunaas</t>
+          <t>Talwiinder, NDS, Rippy Grewal</t>
         </is>
       </c>
     </row>
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>2026-03-27</t>
+          <t>2026-03-28</t>
         </is>
       </c>
       <c r="B44" t="n">
@@ -7551,19 +8588,19 @@
       </c>
       <c r="C44" t="inlineStr">
         <is>
-          <t>Ye Tune Kya Kiya</t>
+          <t>SWIM</t>
         </is>
       </c>
       <c r="D44" t="inlineStr">
         <is>
-          <t>Pritam, Javed Bashir, Rajat Arora</t>
+          <t>BTS</t>
         </is>
       </c>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>2026-03-27</t>
+          <t>2026-03-28</t>
         </is>
       </c>
       <c r="B45" t="n">
@@ -7571,19 +8608,19 @@
       </c>
       <c r="C45" t="inlineStr">
         <is>
-          <t>Haseen</t>
+          <t>Not Guilty</t>
         </is>
       </c>
       <c r="D45" t="inlineStr">
         <is>
-          <t>Talwiinder, NDS, Rippy Grewal</t>
+          <t>Dhanda Nyoliwala</t>
         </is>
       </c>
     </row>
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>2026-03-27</t>
+          <t>2026-03-28</t>
         </is>
       </c>
       <c r="B46" t="n">
@@ -7591,19 +8628,19 @@
       </c>
       <c r="C46" t="inlineStr">
         <is>
-          <t>Not Guilty</t>
+          <t>Ehsaas</t>
         </is>
       </c>
       <c r="D46" t="inlineStr">
         <is>
-          <t>Dhanda Nyoliwala</t>
+          <t>Faheem Abdullah, Duha Shah, Vaibhav Pani, Hyder Dar</t>
         </is>
       </c>
     </row>
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>2026-03-27</t>
+          <t>2026-03-28</t>
         </is>
       </c>
       <c r="B47" t="n">
@@ -7611,19 +8648,19 @@
       </c>
       <c r="C47" t="inlineStr">
         <is>
-          <t>Ehsaas</t>
+          <t>Jogi</t>
         </is>
       </c>
       <c r="D47" t="inlineStr">
         <is>
-          <t>Faheem Abdullah, Duha Shah, Vaibhav Pani, Hyder Dar</t>
+          <t>thiarajxtt, Bir</t>
         </is>
       </c>
     </row>
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>2026-03-27</t>
+          <t>2026-03-28</t>
         </is>
       </c>
       <c r="B48" t="n">
@@ -7643,7 +8680,7 @@
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>2026-03-27</t>
+          <t>2026-03-28</t>
         </is>
       </c>
       <c r="B49" t="n">
@@ -7651,19 +8688,19 @@
       </c>
       <c r="C49" t="inlineStr">
         <is>
-          <t>Hum Pyaar Karne Wale</t>
+          <t>Mann Mera - Original Version</t>
         </is>
       </c>
       <c r="D49" t="inlineStr">
         <is>
-          <t>Shashwat Sachdev, Anuradha Paudwal, Udit Narayan, Anand-Milind, Sameer Anjaan, Qveen Herby</t>
+          <t>Gajendra Verma</t>
         </is>
       </c>
     </row>
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>2026-03-27</t>
+          <t>2026-03-28</t>
         </is>
       </c>
       <c r="B50" t="n">
@@ -7671,19 +8708,19 @@
       </c>
       <c r="C50" t="inlineStr">
         <is>
-          <t>Mast Magan (From "2 States)</t>
+          <t>Hum Pyaar Karne Wale</t>
         </is>
       </c>
       <c r="D50" t="inlineStr">
         <is>
-          <t>Arijit Singh, Chinmayi</t>
+          <t>Shashwat Sachdev, Anuradha Paudwal, Udit Narayan, Anand-Milind, Sameer Anjaan, Qveen Herby</t>
         </is>
       </c>
     </row>
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>2026-03-27</t>
+          <t>2026-03-28</t>
         </is>
       </c>
       <c r="B51" t="n">

</xml_diff>

<commit_message>
added data of 29th march and 30th march and got predictions for 31st march
</commit_message>
<xml_diff>
--- a/Probability Project.xlsx
+++ b/Probability Project.xlsx
@@ -18,6 +18,8 @@
     <sheet name="AUTO_20260326" sheetId="13" state="visible" r:id="rId13"/>
     <sheet name="AUTO_20260327" sheetId="14" state="visible" r:id="rId14"/>
     <sheet name="AUTO_20260328" sheetId="15" state="visible" r:id="rId15"/>
+    <sheet name="AUTO_20260330" sheetId="16" state="visible" r:id="rId16"/>
+    <sheet name="AUTO_20260329" sheetId="17" state="visible" r:id="rId17"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -7738,9 +7740,2081 @@
       </c>
     </row>
     <row r="2">
+      <c r="A2" s="0" t="inlineStr">
+        <is>
+          <t>2026-03-28</t>
+        </is>
+      </c>
+      <c r="B2" s="0" t="n">
+        <v>1</v>
+      </c>
+      <c r="C2" s="0" t="inlineStr">
+        <is>
+          <t>Bairan</t>
+        </is>
+      </c>
+      <c r="D2" s="0" t="inlineStr">
+        <is>
+          <t>Banjaare</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="0" t="inlineStr">
+        <is>
+          <t>2026-03-28</t>
+        </is>
+      </c>
+      <c r="B3" s="0" t="n">
+        <v>2</v>
+      </c>
+      <c r="C3" s="0" t="inlineStr">
+        <is>
+          <t>Jaiye Sajana</t>
+        </is>
+      </c>
+      <c r="D3" s="0" t="inlineStr">
+        <is>
+          <t>Shashwat Sachdev, Jasmine Sandlas, Satinder Sartaaj</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="0" t="inlineStr">
+        <is>
+          <t>2026-03-28</t>
+        </is>
+      </c>
+      <c r="B4" s="0" t="n">
+        <v>3</v>
+      </c>
+      <c r="C4" s="0" t="inlineStr">
+        <is>
+          <t>Gehra Hua</t>
+        </is>
+      </c>
+      <c r="D4" s="0" t="inlineStr">
+        <is>
+          <t>Shashwat Sachdev, Arijit Singh, Irshad Kamil, Armaan Khan</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="0" t="inlineStr">
+        <is>
+          <t>2026-03-28</t>
+        </is>
+      </c>
+      <c r="B5" s="0" t="n">
+        <v>4</v>
+      </c>
+      <c r="C5" s="0" t="inlineStr">
+        <is>
+          <t>Sheesha - Aakhya Mai Aakh Ghali Jo Bairan</t>
+        </is>
+      </c>
+      <c r="D5" s="0" t="inlineStr">
+        <is>
+          <t>Mitta Ror, Swara Verma</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="0" t="inlineStr">
+        <is>
+          <t>2026-03-28</t>
+        </is>
+      </c>
+      <c r="B6" s="0" t="n">
+        <v>5</v>
+      </c>
+      <c r="C6" s="0" t="inlineStr">
+        <is>
+          <t>Dhurandhar The Revenge - Aari Aari</t>
+        </is>
+      </c>
+      <c r="D6" s="0" t="inlineStr">
+        <is>
+          <t>Shashwat Sachdev, Bombay Rockers, Irshad Kamil, Khan Saab, Reble, Token, Jasmine Sandlas, Sudhir Yaduvanshi</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="0" t="inlineStr">
+        <is>
+          <t>2026-03-28</t>
+        </is>
+      </c>
+      <c r="B7" s="0" t="n">
+        <v>6</v>
+      </c>
+      <c r="C7" s="0" t="inlineStr">
+        <is>
+          <t>Khat</t>
+        </is>
+      </c>
+      <c r="D7" s="0" t="inlineStr">
+        <is>
+          <t>Navjot Ahuja</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="0" t="inlineStr">
+        <is>
+          <t>2026-03-28</t>
+        </is>
+      </c>
+      <c r="B8" s="0" t="n">
+        <v>7</v>
+      </c>
+      <c r="C8" s="0" t="inlineStr">
+        <is>
+          <t>Jaan Se Guzarte Hain</t>
+        </is>
+      </c>
+      <c r="D8" s="0" t="inlineStr">
+        <is>
+          <t>Shashwat Sachdev, Khan Saab, Nusrat Fateh Ali Khan</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="0" t="inlineStr">
+        <is>
+          <t>2026-03-28</t>
+        </is>
+      </c>
+      <c r="B9" s="0" t="n">
+        <v>8</v>
+      </c>
+      <c r="C9" s="0" t="inlineStr">
+        <is>
+          <t>Sitaare (From "Ikkis")</t>
+        </is>
+      </c>
+      <c r="D9" s="0" t="inlineStr">
+        <is>
+          <t>Arijit Singh, White Noise Collectives, Amitabh Bhattacharya</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="0" t="inlineStr">
+        <is>
+          <t>2026-03-28</t>
+        </is>
+      </c>
+      <c r="B10" s="0" t="n">
+        <v>9</v>
+      </c>
+      <c r="C10" s="0" t="inlineStr">
+        <is>
+          <t>Dooron Dooron</t>
+        </is>
+      </c>
+      <c r="D10" s="0" t="inlineStr">
+        <is>
+          <t>Paresh Pahuja, Shiv Tandan, Meghdeep Bose</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="0" t="inlineStr">
+        <is>
+          <t>2026-03-28</t>
+        </is>
+      </c>
+      <c r="B11" s="0" t="n">
+        <v>10</v>
+      </c>
+      <c r="C11" s="0" t="inlineStr">
+        <is>
+          <t>Sahiba</t>
+        </is>
+      </c>
+      <c r="D11" s="0" t="inlineStr">
+        <is>
+          <t>Aditya Rikhari</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="0" t="inlineStr">
+        <is>
+          <t>2026-03-28</t>
+        </is>
+      </c>
+      <c r="B12" s="0" t="n">
+        <v>11</v>
+      </c>
+      <c r="C12" s="0" t="inlineStr">
+        <is>
+          <t>Shararat</t>
+        </is>
+      </c>
+      <c r="D12" s="0" t="inlineStr">
+        <is>
+          <t>Shashwat Sachdev, Madhubanti Bagchi, Jasmine Sandlas</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="0" t="inlineStr">
+        <is>
+          <t>2026-03-28</t>
+        </is>
+      </c>
+      <c r="B13" s="0" t="n">
+        <v>12</v>
+      </c>
+      <c r="C13" s="0" t="inlineStr">
+        <is>
+          <t>Finding Her</t>
+        </is>
+      </c>
+      <c r="D13" s="0" t="inlineStr">
+        <is>
+          <t>Kushagra, Bharath, Saaheal</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="0" t="inlineStr">
+        <is>
+          <t>2026-03-28</t>
+        </is>
+      </c>
+      <c r="B14" s="0" t="n">
+        <v>13</v>
+      </c>
+      <c r="C14" s="0" t="inlineStr">
+        <is>
+          <t>Apna Bana Le</t>
+        </is>
+      </c>
+      <c r="D14" s="0" t="inlineStr">
+        <is>
+          <t>Sachin-Jigar, Arijit Singh, Amitabh Bhattacharya</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="0" t="inlineStr">
+        <is>
+          <t>2026-03-28</t>
+        </is>
+      </c>
+      <c r="B15" s="0" t="n">
+        <v>14</v>
+      </c>
+      <c r="C15" s="0" t="inlineStr">
+        <is>
+          <t>Samjhawan</t>
+        </is>
+      </c>
+      <c r="D15" s="0" t="inlineStr">
+        <is>
+          <t>Jawad Ahmad, Shaarib Toshi, Arijit Singh, Shreya Ghoshal</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="0" t="inlineStr">
+        <is>
+          <t>2026-03-28</t>
+        </is>
+      </c>
+      <c r="B16" s="0" t="n">
+        <v>15</v>
+      </c>
+      <c r="C16" s="0" t="inlineStr">
+        <is>
+          <t>Dhurandhar - Title Track</t>
+        </is>
+      </c>
+      <c r="D16" s="0" t="inlineStr">
+        <is>
+          <t>Shashwat Sachdev, Hanumankind, Jasmine Sandlas, Sudhir Yaduvanshi, Charanjit Ahuja, Muhammad Sadiq, Ranjit Kaur, Babu Singh Maan</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="0" t="inlineStr">
+        <is>
+          <t>2026-03-28</t>
+        </is>
+      </c>
+      <c r="B17" s="0" t="n">
+        <v>16</v>
+      </c>
+      <c r="C17" s="0" t="inlineStr">
+        <is>
+          <t>Pavazha Malli - From "Think Indie"</t>
+        </is>
+      </c>
+      <c r="D17" s="0" t="inlineStr">
+        <is>
+          <t>Sai Abhyankkar, Shruti Haasan, Vivek</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="0" t="inlineStr">
+        <is>
+          <t>2026-03-28</t>
+        </is>
+      </c>
+      <c r="B18" s="0" t="n">
+        <v>17</v>
+      </c>
+      <c r="C18" s="0" t="inlineStr">
+        <is>
+          <t>Ishq</t>
+        </is>
+      </c>
+      <c r="D18" s="0" t="inlineStr">
+        <is>
+          <t>Faheem Abdullah, Rauhan Malik, Amir Ameer</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="0" t="inlineStr">
+        <is>
+          <t>2026-03-28</t>
+        </is>
+      </c>
+      <c r="B19" s="0" t="n">
+        <v>18</v>
+      </c>
+      <c r="C19" s="0" t="inlineStr">
+        <is>
+          <t>Arz Kiya Hai | Coke Studio Bharat</t>
+        </is>
+      </c>
+      <c r="D19" s="0" t="inlineStr">
+        <is>
+          <t>Anuv Jain</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="0" t="inlineStr">
+        <is>
+          <t>2026-03-28</t>
+        </is>
+      </c>
+      <c r="B20" s="0" t="n">
+        <v>19</v>
+      </c>
+      <c r="C20" s="0" t="inlineStr">
+        <is>
+          <t>For A Reason</t>
+        </is>
+      </c>
+      <c r="D20" s="0" t="inlineStr">
+        <is>
+          <t>Karan Aujla, Ikky</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="0" t="inlineStr">
+        <is>
+          <t>2026-03-28</t>
+        </is>
+      </c>
+      <c r="B21" s="0" t="n">
+        <v>20</v>
+      </c>
+      <c r="C21" s="0" t="inlineStr">
+        <is>
+          <t>Boyfriend</t>
+        </is>
+      </c>
+      <c r="D21" s="0" t="inlineStr">
+        <is>
+          <t>Karan Aujla, Ikky</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="0" t="inlineStr">
+        <is>
+          <t>2026-03-28</t>
+        </is>
+      </c>
+      <c r="B22" s="0" t="n">
+        <v>21</v>
+      </c>
+      <c r="C22" s="0" t="inlineStr">
+        <is>
+          <t>Mann Mera</t>
+        </is>
+      </c>
+      <c r="D22" s="0" t="inlineStr">
+        <is>
+          <t>Gajendra Verma</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="0" t="inlineStr">
+        <is>
+          <t>2026-03-28</t>
+        </is>
+      </c>
+      <c r="B23" s="0" t="n">
+        <v>22</v>
+      </c>
+      <c r="C23" s="0" t="inlineStr">
+        <is>
+          <t>Naal Nachna</t>
+        </is>
+      </c>
+      <c r="D23" s="0" t="inlineStr">
+        <is>
+          <t>Shashwat Sachdev, Afsana Khan, Irshad Kamil, Reble</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="0" t="inlineStr">
+        <is>
+          <t>2026-03-28</t>
+        </is>
+      </c>
+      <c r="B24" s="0" t="n">
+        <v>23</v>
+      </c>
+      <c r="C24" s="0" t="inlineStr">
+        <is>
+          <t>Bairi</t>
+        </is>
+      </c>
+      <c r="D24" s="0" t="inlineStr">
+        <is>
+          <t>Virat, Pradeep Solanki, Heena</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="0" t="inlineStr">
+        <is>
+          <t>2026-03-28</t>
+        </is>
+      </c>
+      <c r="B25" s="0" t="n">
+        <v>24</v>
+      </c>
+      <c r="C25" s="0" t="inlineStr">
+        <is>
+          <t>Saiyaara</t>
+        </is>
+      </c>
+      <c r="D25" s="0" t="inlineStr">
+        <is>
+          <t>Tanishk Bagchi, Faheem Abdullah, Arslan Nizami, Irshad Kamil</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="0" t="inlineStr">
+        <is>
+          <t>2026-03-28</t>
+        </is>
+      </c>
+      <c r="B26" s="0" t="n">
+        <v>25</v>
+      </c>
+      <c r="C26" s="0" t="inlineStr">
+        <is>
+          <t>Phir Se</t>
+        </is>
+      </c>
+      <c r="D26" s="0" t="inlineStr">
+        <is>
+          <t>Shashwat Sachdev, Arijit Singh, Irshad Kamil</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="0" t="inlineStr">
+        <is>
+          <t>2026-03-28</t>
+        </is>
+      </c>
+      <c r="B27" s="0" t="n">
+        <v>26</v>
+      </c>
+      <c r="C27" s="0" t="inlineStr">
+        <is>
+          <t>Ishqa Ve</t>
+        </is>
+      </c>
+      <c r="D27" s="0" t="inlineStr">
+        <is>
+          <t>Zeeshan Ali, Yuvraj Tung, Sandeep Aulakh, Honey Dhillon</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="0" t="inlineStr">
+        <is>
+          <t>2026-03-28</t>
+        </is>
+      </c>
+      <c r="B28" s="0" t="n">
+        <v>27</v>
+      </c>
+      <c r="C28" s="0" t="inlineStr">
+        <is>
+          <t>Tere Liye</t>
+        </is>
+      </c>
+      <c r="D28" s="0" t="inlineStr">
+        <is>
+          <t>Atif Aslam, Shreya Ghoshal, Sachin Gupta, Sameer Anjaan</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="0" t="inlineStr">
+        <is>
+          <t>2026-03-28</t>
+        </is>
+      </c>
+      <c r="B29" s="0" t="n">
+        <v>28</v>
+      </c>
+      <c r="C29" s="0" t="inlineStr">
+        <is>
+          <t>Deewaana Deewaana</t>
+        </is>
+      </c>
+      <c r="D29" s="0" t="inlineStr">
+        <is>
+          <t>A.R. Rahman, Irshad Kamil</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="0" t="inlineStr">
+        <is>
+          <t>2026-03-28</t>
+        </is>
+      </c>
+      <c r="B30" s="0" t="n">
+        <v>29</v>
+      </c>
+      <c r="C30" s="0" t="inlineStr">
+        <is>
+          <t>Lutt Le Gaya</t>
+        </is>
+      </c>
+      <c r="D30" s="0" t="inlineStr">
+        <is>
+          <t>Shashwat Sachdev, Simran Choudhary</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="0" t="inlineStr">
+        <is>
+          <t>2026-03-28</t>
+        </is>
+      </c>
+      <c r="B31" s="0" t="n">
+        <v>30</v>
+      </c>
+      <c r="C31" s="0" t="inlineStr">
+        <is>
+          <t>Main Aur Tu (From "Dhurandhar The Revenge")</t>
+        </is>
+      </c>
+      <c r="D31" s="0" t="inlineStr">
+        <is>
+          <t>Shashwat Sachdev, Jasmine Sandlas, Reble</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="0" t="inlineStr">
+        <is>
+          <t>2026-03-28</t>
+        </is>
+      </c>
+      <c r="B32" s="0" t="n">
+        <v>31</v>
+      </c>
+      <c r="C32" s="0" t="inlineStr">
+        <is>
+          <t>Raanjhan (From "Do Patti")</t>
+        </is>
+      </c>
+      <c r="D32" s="0" t="inlineStr">
+        <is>
+          <t>Sachet-Parampara, Parampara Tandon, Kausar Munir</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="0" t="inlineStr">
+        <is>
+          <t>2026-03-28</t>
+        </is>
+      </c>
+      <c r="B33" s="0" t="n">
+        <v>32</v>
+      </c>
+      <c r="C33" s="0" t="inlineStr">
+        <is>
+          <t>Ishq Jalakar - Karvaan</t>
+        </is>
+      </c>
+      <c r="D33" s="0" t="inlineStr">
+        <is>
+          <t>Shashwat Sachdev, Shahzad Ali, Subhadeep Das Chowdhury, Armaan Khan, Irshad Kamil, Roshan, Sahir Ludhianvi</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="0" t="inlineStr">
+        <is>
+          <t>2026-03-28</t>
+        </is>
+      </c>
+      <c r="B34" s="0" t="n">
+        <v>33</v>
+      </c>
+      <c r="C34" s="0" t="inlineStr">
+        <is>
+          <t>Run Down The City - Monica</t>
+        </is>
+      </c>
+      <c r="D34" s="0" t="inlineStr">
+        <is>
+          <t>Shashwat Sachdev, Reble, Asha Bhosle, R. D. Burman, Majrooh Sultanpuri</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="0" t="inlineStr">
+        <is>
+          <t>2026-03-28</t>
+        </is>
+      </c>
+      <c r="B35" s="0" t="n">
+        <v>34</v>
+      </c>
+      <c r="C35" s="0" t="inlineStr">
+        <is>
+          <t>Tum Ho Toh (From "Saiyaara")</t>
+        </is>
+      </c>
+      <c r="D35" s="0" t="inlineStr">
+        <is>
+          <t>Vishal Mishra, Hansika Pareek, Raj Shekhar</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="0" t="inlineStr">
+        <is>
+          <t>2026-03-28</t>
+        </is>
+      </c>
+      <c r="B36" s="0" t="n">
+        <v>35</v>
+      </c>
+      <c r="C36" s="0" t="inlineStr">
+        <is>
+          <t>Darkhaast</t>
+        </is>
+      </c>
+      <c r="D36" s="0" t="inlineStr">
+        <is>
+          <t>Mithoon, Arijit Singh, Sunidhi Chauhan, Sayeed Quadri</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="0" t="inlineStr">
+        <is>
+          <t>2026-03-28</t>
+        </is>
+      </c>
+      <c r="B37" s="0" t="n">
+        <v>36</v>
+      </c>
+      <c r="C37" s="0" t="inlineStr">
+        <is>
+          <t>Agar Tum Saath Ho (From "Tamasha")</t>
+        </is>
+      </c>
+      <c r="D37" s="0" t="inlineStr">
+        <is>
+          <t>Alka Yagnik, Arijit Singh</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="0" t="inlineStr">
+        <is>
+          <t>2026-03-28</t>
+        </is>
+      </c>
+      <c r="B38" s="0" t="n">
+        <v>37</v>
+      </c>
+      <c r="C38" s="0" t="inlineStr">
+        <is>
+          <t>Tere Bina</t>
+        </is>
+      </c>
+      <c r="D38" s="0" t="inlineStr">
+        <is>
+          <t>A.R. Rahman, Chinmayi, Murtuza Khan, Qadir Khan</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="0" t="inlineStr">
+        <is>
+          <t>2026-03-28</t>
+        </is>
+      </c>
+      <c r="B39" s="0" t="n">
+        <v>38</v>
+      </c>
+      <c r="C39" s="0" t="inlineStr">
+        <is>
+          <t>Jo Tum Mere Ho</t>
+        </is>
+      </c>
+      <c r="D39" s="0" t="inlineStr">
+        <is>
+          <t>Anuv Jain</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="0" t="inlineStr">
+        <is>
+          <t>2026-03-28</t>
+        </is>
+      </c>
+      <c r="B40" s="0" t="n">
+        <v>39</v>
+      </c>
+      <c r="C40" s="0" t="inlineStr">
+        <is>
+          <t>Aaya Sher (From "The Paradise") (Telugu)</t>
+        </is>
+      </c>
+      <c r="D40" s="0" t="inlineStr">
+        <is>
+          <t>Anirudh Ravichander, Jangi Reddy, Arjun Chandy, Kasarla Shyam</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" s="0" t="inlineStr">
+        <is>
+          <t>2026-03-28</t>
+        </is>
+      </c>
+      <c r="B41" s="0" t="n">
+        <v>40</v>
+      </c>
+      <c r="C41" s="0" t="inlineStr">
+        <is>
+          <t>Mutta Kalakki (From "Youth")</t>
+        </is>
+      </c>
+      <c r="D41" s="0" t="inlineStr">
+        <is>
+          <t>G. V. Prakash, Ken Karunaas</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" s="0" t="inlineStr">
+        <is>
+          <t>2026-03-28</t>
+        </is>
+      </c>
+      <c r="B42" s="0" t="n">
+        <v>41</v>
+      </c>
+      <c r="C42" s="0" t="inlineStr">
+        <is>
+          <t>Ye Tune Kya Kiya</t>
+        </is>
+      </c>
+      <c r="D42" s="0" t="inlineStr">
+        <is>
+          <t>Pritam, Javed Bashir, Rajat Arora</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" s="0" t="inlineStr">
+        <is>
+          <t>2026-03-28</t>
+        </is>
+      </c>
+      <c r="B43" s="0" t="n">
+        <v>42</v>
+      </c>
+      <c r="C43" s="0" t="inlineStr">
+        <is>
+          <t>Haseen</t>
+        </is>
+      </c>
+      <c r="D43" s="0" t="inlineStr">
+        <is>
+          <t>Talwiinder, NDS, Rippy Grewal</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" s="0" t="inlineStr">
+        <is>
+          <t>2026-03-28</t>
+        </is>
+      </c>
+      <c r="B44" s="0" t="n">
+        <v>43</v>
+      </c>
+      <c r="C44" s="0" t="inlineStr">
+        <is>
+          <t>SWIM</t>
+        </is>
+      </c>
+      <c r="D44" s="0" t="inlineStr">
+        <is>
+          <t>BTS</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" s="0" t="inlineStr">
+        <is>
+          <t>2026-03-28</t>
+        </is>
+      </c>
+      <c r="B45" s="0" t="n">
+        <v>44</v>
+      </c>
+      <c r="C45" s="0" t="inlineStr">
+        <is>
+          <t>Not Guilty</t>
+        </is>
+      </c>
+      <c r="D45" s="0" t="inlineStr">
+        <is>
+          <t>Dhanda Nyoliwala</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" s="0" t="inlineStr">
+        <is>
+          <t>2026-03-28</t>
+        </is>
+      </c>
+      <c r="B46" s="0" t="n">
+        <v>45</v>
+      </c>
+      <c r="C46" s="0" t="inlineStr">
+        <is>
+          <t>Ehsaas</t>
+        </is>
+      </c>
+      <c r="D46" s="0" t="inlineStr">
+        <is>
+          <t>Faheem Abdullah, Duha Shah, Vaibhav Pani, Hyder Dar</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" s="0" t="inlineStr">
+        <is>
+          <t>2026-03-28</t>
+        </is>
+      </c>
+      <c r="B47" s="0" t="n">
+        <v>46</v>
+      </c>
+      <c r="C47" s="0" t="inlineStr">
+        <is>
+          <t>Jogi</t>
+        </is>
+      </c>
+      <c r="D47" s="0" t="inlineStr">
+        <is>
+          <t>thiarajxtt, Bir</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" s="0" t="inlineStr">
+        <is>
+          <t>2026-03-28</t>
+        </is>
+      </c>
+      <c r="B48" s="0" t="n">
+        <v>47</v>
+      </c>
+      <c r="C48" s="0" t="inlineStr">
+        <is>
+          <t>Barbaad (From "Saiyaara")</t>
+        </is>
+      </c>
+      <c r="D48" s="0" t="inlineStr">
+        <is>
+          <t>The Rish, Jubin Nautiyal</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" s="0" t="inlineStr">
+        <is>
+          <t>2026-03-28</t>
+        </is>
+      </c>
+      <c r="B49" s="0" t="n">
+        <v>48</v>
+      </c>
+      <c r="C49" s="0" t="inlineStr">
+        <is>
+          <t>Mann Mera - Original Version</t>
+        </is>
+      </c>
+      <c r="D49" s="0" t="inlineStr">
+        <is>
+          <t>Gajendra Verma</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" s="0" t="inlineStr">
+        <is>
+          <t>2026-03-28</t>
+        </is>
+      </c>
+      <c r="B50" s="0" t="n">
+        <v>49</v>
+      </c>
+      <c r="C50" s="0" t="inlineStr">
+        <is>
+          <t>Hum Pyaar Karne Wale</t>
+        </is>
+      </c>
+      <c r="D50" s="0" t="inlineStr">
+        <is>
+          <t>Shashwat Sachdev, Anuradha Paudwal, Udit Narayan, Anand-Milind, Sameer Anjaan, Qveen Herby</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" s="0" t="inlineStr">
+        <is>
+          <t>2026-03-28</t>
+        </is>
+      </c>
+      <c r="B51" s="0" t="n">
+        <v>50</v>
+      </c>
+      <c r="C51" s="0" t="inlineStr">
+        <is>
+          <t>Teri Deewani</t>
+        </is>
+      </c>
+      <c r="D51" s="0" t="inlineStr">
+        <is>
+          <t>Kailash Kher, Paresh Kamath, Naresh Kamath</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet16.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:D51"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="24" t="inlineStr">
+        <is>
+          <t>Date</t>
+        </is>
+      </c>
+      <c r="B1" s="24" t="inlineStr">
+        <is>
+          <t>Rank</t>
+        </is>
+      </c>
+      <c r="C1" s="24" t="inlineStr">
+        <is>
+          <t>Song</t>
+        </is>
+      </c>
+      <c r="D1" s="24" t="inlineStr">
+        <is>
+          <t>Artist</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="0" t="inlineStr">
+        <is>
+          <t>2026-03-30</t>
+        </is>
+      </c>
+      <c r="B2" s="0" t="n">
+        <v>1</v>
+      </c>
+      <c r="C2" s="0" t="inlineStr">
+        <is>
+          <t>Bairan</t>
+        </is>
+      </c>
+      <c r="D2" s="0" t="inlineStr">
+        <is>
+          <t>Banjaare</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="0" t="inlineStr">
+        <is>
+          <t>2026-03-30</t>
+        </is>
+      </c>
+      <c r="B3" s="0" t="n">
+        <v>2</v>
+      </c>
+      <c r="C3" s="0" t="inlineStr">
+        <is>
+          <t>Jaiye Sajana</t>
+        </is>
+      </c>
+      <c r="D3" s="0" t="inlineStr">
+        <is>
+          <t>Shashwat Sachdev, Jasmine Sandlas, Satinder Sartaaj</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="0" t="inlineStr">
+        <is>
+          <t>2026-03-30</t>
+        </is>
+      </c>
+      <c r="B4" s="0" t="n">
+        <v>3</v>
+      </c>
+      <c r="C4" s="0" t="inlineStr">
+        <is>
+          <t>Gehra Hua</t>
+        </is>
+      </c>
+      <c r="D4" s="0" t="inlineStr">
+        <is>
+          <t>Shashwat Sachdev, Arijit Singh, Irshad Kamil, Armaan Khan</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="0" t="inlineStr">
+        <is>
+          <t>2026-03-30</t>
+        </is>
+      </c>
+      <c r="B5" s="0" t="n">
+        <v>4</v>
+      </c>
+      <c r="C5" s="0" t="inlineStr">
+        <is>
+          <t>Sheesha - Aakhya Mai Aakh Ghali Jo Bairan</t>
+        </is>
+      </c>
+      <c r="D5" s="0" t="inlineStr">
+        <is>
+          <t>Mitta Ror, Swara Verma</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="0" t="inlineStr">
+        <is>
+          <t>2026-03-30</t>
+        </is>
+      </c>
+      <c r="B6" s="0" t="n">
+        <v>5</v>
+      </c>
+      <c r="C6" s="0" t="inlineStr">
+        <is>
+          <t>Dhurandhar The Revenge - Aari Aari</t>
+        </is>
+      </c>
+      <c r="D6" s="0" t="inlineStr">
+        <is>
+          <t>Shashwat Sachdev, Bombay Rockers, Irshad Kamil, Khan Saab, Reble, Token, Jasmine Sandlas, Sudhir Yaduvanshi</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="0" t="inlineStr">
+        <is>
+          <t>2026-03-30</t>
+        </is>
+      </c>
+      <c r="B7" s="0" t="n">
+        <v>6</v>
+      </c>
+      <c r="C7" s="0" t="inlineStr">
+        <is>
+          <t>Khat</t>
+        </is>
+      </c>
+      <c r="D7" s="0" t="inlineStr">
+        <is>
+          <t>Navjot Ahuja</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="0" t="inlineStr">
+        <is>
+          <t>2026-03-30</t>
+        </is>
+      </c>
+      <c r="B8" s="0" t="n">
+        <v>7</v>
+      </c>
+      <c r="C8" s="0" t="inlineStr">
+        <is>
+          <t>Jaan Se Guzarte Hain</t>
+        </is>
+      </c>
+      <c r="D8" s="0" t="inlineStr">
+        <is>
+          <t>Shashwat Sachdev, Khan Saab, Nusrat Fateh Ali Khan</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="0" t="inlineStr">
+        <is>
+          <t>2026-03-30</t>
+        </is>
+      </c>
+      <c r="B9" s="0" t="n">
+        <v>8</v>
+      </c>
+      <c r="C9" s="0" t="inlineStr">
+        <is>
+          <t>Sitaare (From "Ikkis")</t>
+        </is>
+      </c>
+      <c r="D9" s="0" t="inlineStr">
+        <is>
+          <t>Arijit Singh, White Noise Collectives, Amitabh Bhattacharya</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="0" t="inlineStr">
+        <is>
+          <t>2026-03-30</t>
+        </is>
+      </c>
+      <c r="B10" s="0" t="n">
+        <v>9</v>
+      </c>
+      <c r="C10" s="0" t="inlineStr">
+        <is>
+          <t>Dooron Dooron</t>
+        </is>
+      </c>
+      <c r="D10" s="0" t="inlineStr">
+        <is>
+          <t>Paresh Pahuja, Shiv Tandan, Meghdeep Bose</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="0" t="inlineStr">
+        <is>
+          <t>2026-03-30</t>
+        </is>
+      </c>
+      <c r="B11" s="0" t="n">
+        <v>10</v>
+      </c>
+      <c r="C11" s="0" t="inlineStr">
+        <is>
+          <t>Sahiba</t>
+        </is>
+      </c>
+      <c r="D11" s="0" t="inlineStr">
+        <is>
+          <t>Aditya Rikhari</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="0" t="inlineStr">
+        <is>
+          <t>2026-03-30</t>
+        </is>
+      </c>
+      <c r="B12" s="0" t="n">
+        <v>11</v>
+      </c>
+      <c r="C12" s="0" t="inlineStr">
+        <is>
+          <t>Samjhawan</t>
+        </is>
+      </c>
+      <c r="D12" s="0" t="inlineStr">
+        <is>
+          <t>Jawad Ahmad, Shaarib Toshi, Arijit Singh, Shreya Ghoshal</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="0" t="inlineStr">
+        <is>
+          <t>2026-03-30</t>
+        </is>
+      </c>
+      <c r="B13" s="0" t="n">
+        <v>12</v>
+      </c>
+      <c r="C13" s="0" t="inlineStr">
+        <is>
+          <t>Apna Bana Le</t>
+        </is>
+      </c>
+      <c r="D13" s="0" t="inlineStr">
+        <is>
+          <t>Sachin-Jigar, Arijit Singh, Amitabh Bhattacharya</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="0" t="inlineStr">
+        <is>
+          <t>2026-03-30</t>
+        </is>
+      </c>
+      <c r="B14" s="0" t="n">
+        <v>13</v>
+      </c>
+      <c r="C14" s="0" t="inlineStr">
+        <is>
+          <t>Shararat</t>
+        </is>
+      </c>
+      <c r="D14" s="0" t="inlineStr">
+        <is>
+          <t>Shashwat Sachdev, Madhubanti Bagchi, Jasmine Sandlas</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="0" t="inlineStr">
+        <is>
+          <t>2026-03-30</t>
+        </is>
+      </c>
+      <c r="B15" s="0" t="n">
+        <v>14</v>
+      </c>
+      <c r="C15" s="0" t="inlineStr">
+        <is>
+          <t>Finding Her</t>
+        </is>
+      </c>
+      <c r="D15" s="0" t="inlineStr">
+        <is>
+          <t>Kushagra, Bharath, Saaheal</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="0" t="inlineStr">
+        <is>
+          <t>2026-03-30</t>
+        </is>
+      </c>
+      <c r="B16" s="0" t="n">
+        <v>15</v>
+      </c>
+      <c r="C16" s="0" t="inlineStr">
+        <is>
+          <t>Arz Kiya Hai | Coke Studio Bharat</t>
+        </is>
+      </c>
+      <c r="D16" s="0" t="inlineStr">
+        <is>
+          <t>Anuv Jain</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="0" t="inlineStr">
+        <is>
+          <t>2026-03-30</t>
+        </is>
+      </c>
+      <c r="B17" s="0" t="n">
+        <v>16</v>
+      </c>
+      <c r="C17" s="0" t="inlineStr">
+        <is>
+          <t>Dhurandhar - Title Track</t>
+        </is>
+      </c>
+      <c r="D17" s="0" t="inlineStr">
+        <is>
+          <t>Shashwat Sachdev, Hanumankind, Jasmine Sandlas, Sudhir Yaduvanshi, Charanjit Ahuja, Muhammad Sadiq, Ranjit Kaur, Babu Singh Maan</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="0" t="inlineStr">
+        <is>
+          <t>2026-03-30</t>
+        </is>
+      </c>
+      <c r="B18" s="0" t="n">
+        <v>17</v>
+      </c>
+      <c r="C18" s="0" t="inlineStr">
+        <is>
+          <t>For A Reason</t>
+        </is>
+      </c>
+      <c r="D18" s="0" t="inlineStr">
+        <is>
+          <t>Karan Aujla, Ikky</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="0" t="inlineStr">
+        <is>
+          <t>2026-03-30</t>
+        </is>
+      </c>
+      <c r="B19" s="0" t="n">
+        <v>18</v>
+      </c>
+      <c r="C19" s="0" t="inlineStr">
+        <is>
+          <t>Pavazha Malli - From "Think Indie"</t>
+        </is>
+      </c>
+      <c r="D19" s="0" t="inlineStr">
+        <is>
+          <t>Sai Abhyankkar, Shruti Haasan, Vivek</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="0" t="inlineStr">
+        <is>
+          <t>2026-03-30</t>
+        </is>
+      </c>
+      <c r="B20" s="0" t="n">
+        <v>19</v>
+      </c>
+      <c r="C20" s="0" t="inlineStr">
+        <is>
+          <t>Boyfriend</t>
+        </is>
+      </c>
+      <c r="D20" s="0" t="inlineStr">
+        <is>
+          <t>Karan Aujla, Ikky</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="0" t="inlineStr">
+        <is>
+          <t>2026-03-30</t>
+        </is>
+      </c>
+      <c r="B21" s="0" t="n">
+        <v>20</v>
+      </c>
+      <c r="C21" s="0" t="inlineStr">
+        <is>
+          <t>Ishq</t>
+        </is>
+      </c>
+      <c r="D21" s="0" t="inlineStr">
+        <is>
+          <t>Faheem Abdullah, Rauhan Malik, Amir Ameer</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="0" t="inlineStr">
+        <is>
+          <t>2026-03-30</t>
+        </is>
+      </c>
+      <c r="B22" s="0" t="n">
+        <v>21</v>
+      </c>
+      <c r="C22" s="0" t="inlineStr">
+        <is>
+          <t>Mann Mera</t>
+        </is>
+      </c>
+      <c r="D22" s="0" t="inlineStr">
+        <is>
+          <t>Gajendra Verma</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="0" t="inlineStr">
+        <is>
+          <t>2026-03-30</t>
+        </is>
+      </c>
+      <c r="B23" s="0" t="n">
+        <v>22</v>
+      </c>
+      <c r="C23" s="0" t="inlineStr">
+        <is>
+          <t>Phir Se</t>
+        </is>
+      </c>
+      <c r="D23" s="0" t="inlineStr">
+        <is>
+          <t>Shashwat Sachdev, Arijit Singh, Irshad Kamil</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="0" t="inlineStr">
+        <is>
+          <t>2026-03-30</t>
+        </is>
+      </c>
+      <c r="B24" s="0" t="n">
+        <v>23</v>
+      </c>
+      <c r="C24" s="0" t="inlineStr">
+        <is>
+          <t>Bairi</t>
+        </is>
+      </c>
+      <c r="D24" s="0" t="inlineStr">
+        <is>
+          <t>Virat, Pradeep Solanki, Heena</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="0" t="inlineStr">
+        <is>
+          <t>2026-03-30</t>
+        </is>
+      </c>
+      <c r="B25" s="0" t="n">
+        <v>24</v>
+      </c>
+      <c r="C25" s="0" t="inlineStr">
+        <is>
+          <t>Naal Nachna</t>
+        </is>
+      </c>
+      <c r="D25" s="0" t="inlineStr">
+        <is>
+          <t>Shashwat Sachdev, Afsana Khan, Irshad Kamil, Reble</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="0" t="inlineStr">
+        <is>
+          <t>2026-03-30</t>
+        </is>
+      </c>
+      <c r="B26" s="0" t="n">
+        <v>25</v>
+      </c>
+      <c r="C26" s="0" t="inlineStr">
+        <is>
+          <t>Ishqa Ve</t>
+        </is>
+      </c>
+      <c r="D26" s="0" t="inlineStr">
+        <is>
+          <t>Zeeshan Ali, Yuvraj Tung, Sandeep Aulakh, Honey Dhillon</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="0" t="inlineStr">
+        <is>
+          <t>2026-03-30</t>
+        </is>
+      </c>
+      <c r="B27" s="0" t="n">
+        <v>26</v>
+      </c>
+      <c r="C27" s="0" t="inlineStr">
+        <is>
+          <t>Saiyaara</t>
+        </is>
+      </c>
+      <c r="D27" s="0" t="inlineStr">
+        <is>
+          <t>Tanishk Bagchi, Faheem Abdullah, Arslan Nizami, Irshad Kamil</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="0" t="inlineStr">
+        <is>
+          <t>2026-03-30</t>
+        </is>
+      </c>
+      <c r="B28" s="0" t="n">
+        <v>27</v>
+      </c>
+      <c r="C28" s="0" t="inlineStr">
+        <is>
+          <t>Tere Liye</t>
+        </is>
+      </c>
+      <c r="D28" s="0" t="inlineStr">
+        <is>
+          <t>Atif Aslam, Shreya Ghoshal, Sachin Gupta, Sameer Anjaan</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="0" t="inlineStr">
+        <is>
+          <t>2026-03-30</t>
+        </is>
+      </c>
+      <c r="B29" s="0" t="n">
+        <v>28</v>
+      </c>
+      <c r="C29" s="0" t="inlineStr">
+        <is>
+          <t>Deewaana Deewaana</t>
+        </is>
+      </c>
+      <c r="D29" s="0" t="inlineStr">
+        <is>
+          <t>A.R. Rahman, Irshad Kamil</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="0" t="inlineStr">
+        <is>
+          <t>2026-03-30</t>
+        </is>
+      </c>
+      <c r="B30" s="0" t="n">
+        <v>29</v>
+      </c>
+      <c r="C30" s="0" t="inlineStr">
+        <is>
+          <t>Darkhaast</t>
+        </is>
+      </c>
+      <c r="D30" s="0" t="inlineStr">
+        <is>
+          <t>Mithoon, Arijit Singh, Sunidhi Chauhan, Sayeed Quadri</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="0" t="inlineStr">
+        <is>
+          <t>2026-03-30</t>
+        </is>
+      </c>
+      <c r="B31" s="0" t="n">
+        <v>30</v>
+      </c>
+      <c r="C31" s="0" t="inlineStr">
+        <is>
+          <t>Tum Ho Toh (From "Saiyaara")</t>
+        </is>
+      </c>
+      <c r="D31" s="0" t="inlineStr">
+        <is>
+          <t>Vishal Mishra, Hansika Pareek, Raj Shekhar</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="0" t="inlineStr">
+        <is>
+          <t>2026-03-30</t>
+        </is>
+      </c>
+      <c r="B32" s="0" t="n">
+        <v>31</v>
+      </c>
+      <c r="C32" s="0" t="inlineStr">
+        <is>
+          <t>Main Aur Tu</t>
+        </is>
+      </c>
+      <c r="D32" s="0" t="inlineStr">
+        <is>
+          <t>Shashwat Sachdev, Jasmine Sandlas, Reble</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="0" t="inlineStr">
+        <is>
+          <t>2026-03-30</t>
+        </is>
+      </c>
+      <c r="B33" s="0" t="n">
+        <v>32</v>
+      </c>
+      <c r="C33" s="0" t="inlineStr">
+        <is>
+          <t>Lutt Le Gaya</t>
+        </is>
+      </c>
+      <c r="D33" s="0" t="inlineStr">
+        <is>
+          <t>Shashwat Sachdev, Simran Choudhary</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="0" t="inlineStr">
+        <is>
+          <t>2026-03-30</t>
+        </is>
+      </c>
+      <c r="B34" s="0" t="n">
+        <v>33</v>
+      </c>
+      <c r="C34" s="0" t="inlineStr">
+        <is>
+          <t>Tere Bina</t>
+        </is>
+      </c>
+      <c r="D34" s="0" t="inlineStr">
+        <is>
+          <t>A.R. Rahman, Chinmayi, Murtuza Khan, Qadir Khan</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="0" t="inlineStr">
+        <is>
+          <t>2026-03-30</t>
+        </is>
+      </c>
+      <c r="B35" s="0" t="n">
+        <v>34</v>
+      </c>
+      <c r="C35" s="0" t="inlineStr">
+        <is>
+          <t>Jo Tum Mere Ho</t>
+        </is>
+      </c>
+      <c r="D35" s="0" t="inlineStr">
+        <is>
+          <t>Anuv Jain</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="0" t="inlineStr">
+        <is>
+          <t>2026-03-30</t>
+        </is>
+      </c>
+      <c r="B36" s="0" t="n">
+        <v>35</v>
+      </c>
+      <c r="C36" s="0" t="inlineStr">
+        <is>
+          <t>Raanjhan (From "Do Patti")</t>
+        </is>
+      </c>
+      <c r="D36" s="0" t="inlineStr">
+        <is>
+          <t>Sachet-Parampara, Parampara Tandon, Kausar Munir</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="0" t="inlineStr">
+        <is>
+          <t>2026-03-30</t>
+        </is>
+      </c>
+      <c r="B37" s="0" t="n">
+        <v>36</v>
+      </c>
+      <c r="C37" s="0" t="inlineStr">
+        <is>
+          <t>Run Down The City - Monica</t>
+        </is>
+      </c>
+      <c r="D37" s="0" t="inlineStr">
+        <is>
+          <t>Shashwat Sachdev, Reble, Asha Bhosle, R. D. Burman, Majrooh Sultanpuri</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="0" t="inlineStr">
+        <is>
+          <t>2026-03-30</t>
+        </is>
+      </c>
+      <c r="B38" s="0" t="n">
+        <v>37</v>
+      </c>
+      <c r="C38" s="0" t="inlineStr">
+        <is>
+          <t>Haseen</t>
+        </is>
+      </c>
+      <c r="D38" s="0" t="inlineStr">
+        <is>
+          <t>Talwiinder, NDS, Rippy Grewal</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="0" t="inlineStr">
+        <is>
+          <t>2026-03-30</t>
+        </is>
+      </c>
+      <c r="B39" s="0" t="n">
+        <v>38</v>
+      </c>
+      <c r="C39" s="0" t="inlineStr">
+        <is>
+          <t>Agar Tum Saath Ho (From "Tamasha")</t>
+        </is>
+      </c>
+      <c r="D39" s="0" t="inlineStr">
+        <is>
+          <t>Alka Yagnik, Arijit Singh</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="0" t="inlineStr">
+        <is>
+          <t>2026-03-30</t>
+        </is>
+      </c>
+      <c r="B40" s="0" t="n">
+        <v>39</v>
+      </c>
+      <c r="C40" s="0" t="inlineStr">
+        <is>
+          <t>Ishq Jalakar - Karvaan</t>
+        </is>
+      </c>
+      <c r="D40" s="0" t="inlineStr">
+        <is>
+          <t>Shashwat Sachdev, Shahzad Ali, Subhadeep Das Chowdhury, Armaan Khan, Irshad Kamil, Roshan, Sahir Ludhianvi</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" s="0" t="inlineStr">
+        <is>
+          <t>2026-03-30</t>
+        </is>
+      </c>
+      <c r="B41" s="0" t="n">
+        <v>40</v>
+      </c>
+      <c r="C41" s="0" t="inlineStr">
+        <is>
+          <t>Ye Tune Kya Kiya</t>
+        </is>
+      </c>
+      <c r="D41" s="0" t="inlineStr">
+        <is>
+          <t>Pritam, Javed Bashir, Rajat Arora</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" s="0" t="inlineStr">
+        <is>
+          <t>2026-03-30</t>
+        </is>
+      </c>
+      <c r="B42" s="0" t="n">
+        <v>41</v>
+      </c>
+      <c r="C42" s="0" t="inlineStr">
+        <is>
+          <t>Vaari Jaavan</t>
+        </is>
+      </c>
+      <c r="D42" s="0" t="inlineStr">
+        <is>
+          <t>Shashwat Sachdev, Jyoti Nooran, Jasmine Sandlas, Reble</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" s="0" t="inlineStr">
+        <is>
+          <t>2026-03-30</t>
+        </is>
+      </c>
+      <c r="B43" s="0" t="n">
+        <v>42</v>
+      </c>
+      <c r="C43" s="0" t="inlineStr">
+        <is>
+          <t>Barbaad (From "Saiyaara")</t>
+        </is>
+      </c>
+      <c r="D43" s="0" t="inlineStr">
+        <is>
+          <t>The Rish, Jubin Nautiyal</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" s="0" t="inlineStr">
+        <is>
+          <t>2026-03-30</t>
+        </is>
+      </c>
+      <c r="B44" s="0" t="n">
+        <v>43</v>
+      </c>
+      <c r="C44" s="0" t="inlineStr">
+        <is>
+          <t>Not Guilty</t>
+        </is>
+      </c>
+      <c r="D44" s="0" t="inlineStr">
+        <is>
+          <t>Dhanda Nyoliwala</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" s="0" t="inlineStr">
+        <is>
+          <t>2026-03-30</t>
+        </is>
+      </c>
+      <c r="B45" s="0" t="n">
+        <v>44</v>
+      </c>
+      <c r="C45" s="0" t="inlineStr">
+        <is>
+          <t>Jogi</t>
+        </is>
+      </c>
+      <c r="D45" s="0" t="inlineStr">
+        <is>
+          <t>thiarajxtt, Bir</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" s="0" t="inlineStr">
+        <is>
+          <t>2026-03-30</t>
+        </is>
+      </c>
+      <c r="B46" s="0" t="n">
+        <v>45</v>
+      </c>
+      <c r="C46" s="0" t="inlineStr">
+        <is>
+          <t>Aaya Sher (From "The Paradise") (Telugu)</t>
+        </is>
+      </c>
+      <c r="D46" s="0" t="inlineStr">
+        <is>
+          <t>Anirudh Ravichander, Jangi Reddy, Arjun Chandy, Kasarla Shyam</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" s="0" t="inlineStr">
+        <is>
+          <t>2026-03-30</t>
+        </is>
+      </c>
+      <c r="B47" s="0" t="n">
+        <v>46</v>
+      </c>
+      <c r="C47" s="0" t="inlineStr">
+        <is>
+          <t>Mutta Kalakki (From "Youth")</t>
+        </is>
+      </c>
+      <c r="D47" s="0" t="inlineStr">
+        <is>
+          <t>G. V. Prakash, Ken Karunaas</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" s="0" t="inlineStr">
+        <is>
+          <t>2026-03-30</t>
+        </is>
+      </c>
+      <c r="B48" s="0" t="n">
+        <v>47</v>
+      </c>
+      <c r="C48" s="0" t="inlineStr">
+        <is>
+          <t>Hum Pyaar Karne Wale</t>
+        </is>
+      </c>
+      <c r="D48" s="0" t="inlineStr">
+        <is>
+          <t>Shashwat Sachdev, Anuradha Paudwal, Udit Narayan, Anand-Milind, Sameer Anjaan, Qveen Herby</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" s="0" t="inlineStr">
+        <is>
+          <t>2026-03-30</t>
+        </is>
+      </c>
+      <c r="B49" s="0" t="n">
+        <v>48</v>
+      </c>
+      <c r="C49" s="0" t="inlineStr">
+        <is>
+          <t>Ehsaas</t>
+        </is>
+      </c>
+      <c r="D49" s="0" t="inlineStr">
+        <is>
+          <t>Faheem Abdullah, Duha Shah, Vaibhav Pani, Hyder Dar</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" s="0" t="inlineStr">
+        <is>
+          <t>2026-03-30</t>
+        </is>
+      </c>
+      <c r="B50" s="0" t="n">
+        <v>49</v>
+      </c>
+      <c r="C50" s="0" t="inlineStr">
+        <is>
+          <t>Teri Deewani</t>
+        </is>
+      </c>
+      <c r="D50" s="0" t="inlineStr">
+        <is>
+          <t>Kailash Kher, Paresh Kamath, Naresh Kamath</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" s="0" t="inlineStr">
+        <is>
+          <t>2026-03-30</t>
+        </is>
+      </c>
+      <c r="B51" s="0" t="n">
+        <v>50</v>
+      </c>
+      <c r="C51" s="0" t="inlineStr">
+        <is>
+          <t>SWIM</t>
+        </is>
+      </c>
+      <c r="D51" s="0" t="inlineStr">
+        <is>
+          <t>BTS</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet17.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:D51"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="24" t="inlineStr">
+        <is>
+          <t>Date</t>
+        </is>
+      </c>
+      <c r="B1" s="24" t="inlineStr">
+        <is>
+          <t>Rank</t>
+        </is>
+      </c>
+      <c r="C1" s="24" t="inlineStr">
+        <is>
+          <t>Song</t>
+        </is>
+      </c>
+      <c r="D1" s="24" t="inlineStr">
+        <is>
+          <t>Artist</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>2026-03-28</t>
+          <t>2026-03-29</t>
         </is>
       </c>
       <c r="B2" t="n">
@@ -7760,7 +9834,7 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>2026-03-28</t>
+          <t>2026-03-29</t>
         </is>
       </c>
       <c r="B3" t="n">
@@ -7780,7 +9854,7 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>2026-03-28</t>
+          <t>2026-03-29</t>
         </is>
       </c>
       <c r="B4" t="n">
@@ -7800,7 +9874,7 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>2026-03-28</t>
+          <t>2026-03-29</t>
         </is>
       </c>
       <c r="B5" t="n">
@@ -7820,7 +9894,7 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>2026-03-28</t>
+          <t>2026-03-29</t>
         </is>
       </c>
       <c r="B6" t="n">
@@ -7840,7 +9914,7 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>2026-03-28</t>
+          <t>2026-03-29</t>
         </is>
       </c>
       <c r="B7" t="n">
@@ -7860,7 +9934,7 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>2026-03-28</t>
+          <t>2026-03-29</t>
         </is>
       </c>
       <c r="B8" t="n">
@@ -7880,7 +9954,7 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>2026-03-28</t>
+          <t>2026-03-29</t>
         </is>
       </c>
       <c r="B9" t="n">
@@ -7900,7 +9974,7 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>2026-03-28</t>
+          <t>2026-03-29</t>
         </is>
       </c>
       <c r="B10" t="n">
@@ -7920,7 +9994,7 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>2026-03-28</t>
+          <t>2026-03-29</t>
         </is>
       </c>
       <c r="B11" t="n">
@@ -7940,7 +10014,7 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>2026-03-28</t>
+          <t>2026-03-29</t>
         </is>
       </c>
       <c r="B12" t="n">
@@ -7948,19 +10022,19 @@
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>Shararat</t>
+          <t>Samjhawan</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>Shashwat Sachdev, Madhubanti Bagchi, Jasmine Sandlas</t>
+          <t>Jawad Ahmad, Shaarib Toshi, Arijit Singh, Shreya Ghoshal</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>2026-03-28</t>
+          <t>2026-03-29</t>
         </is>
       </c>
       <c r="B13" t="n">
@@ -7968,19 +10042,19 @@
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>Finding Her</t>
+          <t>Shararat</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>Kushagra, Bharath, Saaheal</t>
+          <t>Shashwat Sachdev, Madhubanti Bagchi, Jasmine Sandlas</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>2026-03-28</t>
+          <t>2026-03-29</t>
         </is>
       </c>
       <c r="B14" t="n">
@@ -8000,7 +10074,7 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>2026-03-28</t>
+          <t>2026-03-29</t>
         </is>
       </c>
       <c r="B15" t="n">
@@ -8008,19 +10082,19 @@
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>Samjhawan</t>
+          <t>Finding Her</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>Jawad Ahmad, Shaarib Toshi, Arijit Singh, Shreya Ghoshal</t>
+          <t>Kushagra, Bharath, Saaheal</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>2026-03-28</t>
+          <t>2026-03-29</t>
         </is>
       </c>
       <c r="B16" t="n">
@@ -8040,7 +10114,7 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>2026-03-28</t>
+          <t>2026-03-29</t>
         </is>
       </c>
       <c r="B17" t="n">
@@ -8048,19 +10122,19 @@
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>Pavazha Malli - From "Think Indie"</t>
+          <t>Arz Kiya Hai | Coke Studio Bharat</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>Sai Abhyankkar, Shruti Haasan, Vivek</t>
+          <t>Anuv Jain</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>2026-03-28</t>
+          <t>2026-03-29</t>
         </is>
       </c>
       <c r="B18" t="n">
@@ -8068,19 +10142,19 @@
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>Ishq</t>
+          <t>For A Reason</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>Faheem Abdullah, Rauhan Malik, Amir Ameer</t>
+          <t>Karan Aujla, Ikky</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>2026-03-28</t>
+          <t>2026-03-29</t>
         </is>
       </c>
       <c r="B19" t="n">
@@ -8088,19 +10162,19 @@
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>Arz Kiya Hai | Coke Studio Bharat</t>
+          <t>Pavazha Malli - From "Think Indie"</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>Anuv Jain</t>
+          <t>Sai Abhyankkar, Shruti Haasan, Vivek</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>2026-03-28</t>
+          <t>2026-03-29</t>
         </is>
       </c>
       <c r="B20" t="n">
@@ -8108,19 +10182,19 @@
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>For A Reason</t>
+          <t>Ishq</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>Karan Aujla, Ikky</t>
+          <t>Faheem Abdullah, Rauhan Malik, Amir Ameer</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>2026-03-28</t>
+          <t>2026-03-29</t>
         </is>
       </c>
       <c r="B21" t="n">
@@ -8140,7 +10214,7 @@
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>2026-03-28</t>
+          <t>2026-03-29</t>
         </is>
       </c>
       <c r="B22" t="n">
@@ -8160,7 +10234,7 @@
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>2026-03-28</t>
+          <t>2026-03-29</t>
         </is>
       </c>
       <c r="B23" t="n">
@@ -8168,19 +10242,19 @@
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>Naal Nachna</t>
+          <t>Bairi</t>
         </is>
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>Shashwat Sachdev, Afsana Khan, Irshad Kamil, Reble</t>
+          <t>Virat, Pradeep Solanki, Heena</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>2026-03-28</t>
+          <t>2026-03-29</t>
         </is>
       </c>
       <c r="B24" t="n">
@@ -8188,19 +10262,19 @@
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>Bairi</t>
+          <t>Ishqa Ve</t>
         </is>
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>Virat, Pradeep Solanki, Heena</t>
+          <t>Zeeshan Ali, Yuvraj Tung, Sandeep Aulakh, Honey Dhillon</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>2026-03-28</t>
+          <t>2026-03-29</t>
         </is>
       </c>
       <c r="B25" t="n">
@@ -8208,19 +10282,19 @@
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>Saiyaara</t>
+          <t>Naal Nachna</t>
         </is>
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>Tanishk Bagchi, Faheem Abdullah, Arslan Nizami, Irshad Kamil</t>
+          <t>Shashwat Sachdev, Afsana Khan, Irshad Kamil, Reble</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>2026-03-28</t>
+          <t>2026-03-29</t>
         </is>
       </c>
       <c r="B26" t="n">
@@ -8240,7 +10314,7 @@
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>2026-03-28</t>
+          <t>2026-03-29</t>
         </is>
       </c>
       <c r="B27" t="n">
@@ -8248,19 +10322,19 @@
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>Ishqa Ve</t>
+          <t>Saiyaara</t>
         </is>
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t>Zeeshan Ali, Yuvraj Tung, Sandeep Aulakh, Honey Dhillon</t>
+          <t>Tanishk Bagchi, Faheem Abdullah, Arslan Nizami, Irshad Kamil</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>2026-03-28</t>
+          <t>2026-03-29</t>
         </is>
       </c>
       <c r="B28" t="n">
@@ -8268,19 +10342,19 @@
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>Tere Liye</t>
+          <t>Deewaana Deewaana</t>
         </is>
       </c>
       <c r="D28" t="inlineStr">
         <is>
-          <t>Atif Aslam, Shreya Ghoshal, Sachin Gupta, Sameer Anjaan</t>
+          <t>A.R. Rahman, Irshad Kamil</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>2026-03-28</t>
+          <t>2026-03-29</t>
         </is>
       </c>
       <c r="B29" t="n">
@@ -8288,19 +10362,19 @@
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>Deewaana Deewaana</t>
+          <t>Tere Liye</t>
         </is>
       </c>
       <c r="D29" t="inlineStr">
         <is>
-          <t>A.R. Rahman, Irshad Kamil</t>
+          <t>Atif Aslam, Shreya Ghoshal, Sachin Gupta, Sameer Anjaan</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>2026-03-28</t>
+          <t>2026-03-29</t>
         </is>
       </c>
       <c r="B30" t="n">
@@ -8320,7 +10394,7 @@
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>2026-03-28</t>
+          <t>2026-03-29</t>
         </is>
       </c>
       <c r="B31" t="n">
@@ -8328,19 +10402,19 @@
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>Main Aur Tu (From "Dhurandhar The Revenge")</t>
+          <t>Raanjhan (From "Do Patti")</t>
         </is>
       </c>
       <c r="D31" t="inlineStr">
         <is>
-          <t>Shashwat Sachdev, Jasmine Sandlas, Reble</t>
+          <t>Sachet-Parampara, Parampara Tandon, Kausar Munir</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>2026-03-28</t>
+          <t>2026-03-29</t>
         </is>
       </c>
       <c r="B32" t="n">
@@ -8348,19 +10422,19 @@
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>Raanjhan (From "Do Patti")</t>
+          <t>Tum Ho Toh (From "Saiyaara")</t>
         </is>
       </c>
       <c r="D32" t="inlineStr">
         <is>
-          <t>Sachet-Parampara, Parampara Tandon, Kausar Munir</t>
+          <t>Vishal Mishra, Hansika Pareek, Raj Shekhar</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>2026-03-28</t>
+          <t>2026-03-29</t>
         </is>
       </c>
       <c r="B33" t="n">
@@ -8368,19 +10442,19 @@
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>Ishq Jalakar - Karvaan</t>
+          <t>Main Aur Tu (From "Dhurandhar The Revenge")</t>
         </is>
       </c>
       <c r="D33" t="inlineStr">
         <is>
-          <t>Shashwat Sachdev, Shahzad Ali, Subhadeep Das Chowdhury, Armaan Khan, Irshad Kamil, Roshan, Sahir Ludhianvi</t>
+          <t>Shashwat Sachdev, Jasmine Sandlas, Reble</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>2026-03-28</t>
+          <t>2026-03-29</t>
         </is>
       </c>
       <c r="B34" t="n">
@@ -8388,19 +10462,19 @@
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>Run Down The City - Monica</t>
+          <t>Ishq Jalakar - Karvaan</t>
         </is>
       </c>
       <c r="D34" t="inlineStr">
         <is>
-          <t>Shashwat Sachdev, Reble, Asha Bhosle, R. D. Burman, Majrooh Sultanpuri</t>
+          <t>Shashwat Sachdev, Shahzad Ali, Subhadeep Das Chowdhury, Armaan Khan, Irshad Kamil, Roshan, Sahir Ludhianvi</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>2026-03-28</t>
+          <t>2026-03-29</t>
         </is>
       </c>
       <c r="B35" t="n">
@@ -8408,19 +10482,19 @@
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>Tum Ho Toh (From "Saiyaara")</t>
+          <t>Darkhaast</t>
         </is>
       </c>
       <c r="D35" t="inlineStr">
         <is>
-          <t>Vishal Mishra, Hansika Pareek, Raj Shekhar</t>
+          <t>Mithoon, Arijit Singh, Sunidhi Chauhan, Sayeed Quadri</t>
         </is>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>2026-03-28</t>
+          <t>2026-03-29</t>
         </is>
       </c>
       <c r="B36" t="n">
@@ -8428,19 +10502,19 @@
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>Darkhaast</t>
+          <t>Jo Tum Mere Ho</t>
         </is>
       </c>
       <c r="D36" t="inlineStr">
         <is>
-          <t>Mithoon, Arijit Singh, Sunidhi Chauhan, Sayeed Quadri</t>
+          <t>Anuv Jain</t>
         </is>
       </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>2026-03-28</t>
+          <t>2026-03-29</t>
         </is>
       </c>
       <c r="B37" t="n">
@@ -8448,19 +10522,19 @@
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>Agar Tum Saath Ho (From "Tamasha")</t>
+          <t>Tere Bina</t>
         </is>
       </c>
       <c r="D37" t="inlineStr">
         <is>
-          <t>Alka Yagnik, Arijit Singh</t>
+          <t>A.R. Rahman, Chinmayi, Murtuza Khan, Qadir Khan</t>
         </is>
       </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>2026-03-28</t>
+          <t>2026-03-29</t>
         </is>
       </c>
       <c r="B38" t="n">
@@ -8468,19 +10542,19 @@
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>Tere Bina</t>
+          <t>Run Down The City - Monica</t>
         </is>
       </c>
       <c r="D38" t="inlineStr">
         <is>
-          <t>A.R. Rahman, Chinmayi, Murtuza Khan, Qadir Khan</t>
+          <t>Shashwat Sachdev, Reble, Asha Bhosle, R. D. Burman, Majrooh Sultanpuri</t>
         </is>
       </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>2026-03-28</t>
+          <t>2026-03-29</t>
         </is>
       </c>
       <c r="B39" t="n">
@@ -8488,19 +10562,19 @@
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>Jo Tum Mere Ho</t>
+          <t>Haseen</t>
         </is>
       </c>
       <c r="D39" t="inlineStr">
         <is>
-          <t>Anuv Jain</t>
+          <t>Talwiinder, NDS, Rippy Grewal</t>
         </is>
       </c>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>2026-03-28</t>
+          <t>2026-03-29</t>
         </is>
       </c>
       <c r="B40" t="n">
@@ -8508,19 +10582,19 @@
       </c>
       <c r="C40" t="inlineStr">
         <is>
-          <t>Aaya Sher (From "The Paradise") (Telugu)</t>
+          <t>Agar Tum Saath Ho (From "Tamasha")</t>
         </is>
       </c>
       <c r="D40" t="inlineStr">
         <is>
-          <t>Anirudh Ravichander, Jangi Reddy, Arjun Chandy, Kasarla Shyam</t>
+          <t>Alka Yagnik, Arijit Singh</t>
         </is>
       </c>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>2026-03-28</t>
+          <t>2026-03-29</t>
         </is>
       </c>
       <c r="B41" t="n">
@@ -8528,19 +10602,19 @@
       </c>
       <c r="C41" t="inlineStr">
         <is>
-          <t>Mutta Kalakki (From "Youth")</t>
+          <t>Ye Tune Kya Kiya</t>
         </is>
       </c>
       <c r="D41" t="inlineStr">
         <is>
-          <t>G. V. Prakash, Ken Karunaas</t>
+          <t>Pritam, Javed Bashir, Rajat Arora</t>
         </is>
       </c>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>2026-03-28</t>
+          <t>2026-03-29</t>
         </is>
       </c>
       <c r="B42" t="n">
@@ -8548,19 +10622,19 @@
       </c>
       <c r="C42" t="inlineStr">
         <is>
-          <t>Ye Tune Kya Kiya</t>
+          <t>Aaya Sher (From "The Paradise") (Telugu)</t>
         </is>
       </c>
       <c r="D42" t="inlineStr">
         <is>
-          <t>Pritam, Javed Bashir, Rajat Arora</t>
+          <t>Anirudh Ravichander, Jangi Reddy, Arjun Chandy, Kasarla Shyam</t>
         </is>
       </c>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>2026-03-28</t>
+          <t>2026-03-29</t>
         </is>
       </c>
       <c r="B43" t="n">
@@ -8568,19 +10642,19 @@
       </c>
       <c r="C43" t="inlineStr">
         <is>
-          <t>Haseen</t>
+          <t>Mutta Kalakki (From "Youth")</t>
         </is>
       </c>
       <c r="D43" t="inlineStr">
         <is>
-          <t>Talwiinder, NDS, Rippy Grewal</t>
+          <t>G. V. Prakash, Ken Karunaas</t>
         </is>
       </c>
     </row>
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>2026-03-28</t>
+          <t>2026-03-29</t>
         </is>
       </c>
       <c r="B44" t="n">
@@ -8600,7 +10674,7 @@
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>2026-03-28</t>
+          <t>2026-03-29</t>
         </is>
       </c>
       <c r="B45" t="n">
@@ -8608,19 +10682,19 @@
       </c>
       <c r="C45" t="inlineStr">
         <is>
-          <t>Not Guilty</t>
+          <t>Barbaad (From "Saiyaara")</t>
         </is>
       </c>
       <c r="D45" t="inlineStr">
         <is>
-          <t>Dhanda Nyoliwala</t>
+          <t>The Rish, Jubin Nautiyal</t>
         </is>
       </c>
     </row>
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>2026-03-28</t>
+          <t>2026-03-29</t>
         </is>
       </c>
       <c r="B46" t="n">
@@ -8628,19 +10702,19 @@
       </c>
       <c r="C46" t="inlineStr">
         <is>
-          <t>Ehsaas</t>
+          <t>Not Guilty</t>
         </is>
       </c>
       <c r="D46" t="inlineStr">
         <is>
-          <t>Faheem Abdullah, Duha Shah, Vaibhav Pani, Hyder Dar</t>
+          <t>Dhanda Nyoliwala</t>
         </is>
       </c>
     </row>
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>2026-03-28</t>
+          <t>2026-03-29</t>
         </is>
       </c>
       <c r="B47" t="n">
@@ -8660,7 +10734,7 @@
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>2026-03-28</t>
+          <t>2026-03-29</t>
         </is>
       </c>
       <c r="B48" t="n">
@@ -8668,19 +10742,19 @@
       </c>
       <c r="C48" t="inlineStr">
         <is>
-          <t>Barbaad (From "Saiyaara")</t>
+          <t>Mann Mera - Original Version</t>
         </is>
       </c>
       <c r="D48" t="inlineStr">
         <is>
-          <t>The Rish, Jubin Nautiyal</t>
+          <t>Gajendra Verma</t>
         </is>
       </c>
     </row>
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>2026-03-28</t>
+          <t>2026-03-29</t>
         </is>
       </c>
       <c r="B49" t="n">
@@ -8688,19 +10762,19 @@
       </c>
       <c r="C49" t="inlineStr">
         <is>
-          <t>Mann Mera - Original Version</t>
+          <t>Ehsaas</t>
         </is>
       </c>
       <c r="D49" t="inlineStr">
         <is>
-          <t>Gajendra Verma</t>
+          <t>Faheem Abdullah, Duha Shah, Vaibhav Pani, Hyder Dar</t>
         </is>
       </c>
     </row>
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>2026-03-28</t>
+          <t>2026-03-29</t>
         </is>
       </c>
       <c r="B50" t="n">
@@ -8708,19 +10782,19 @@
       </c>
       <c r="C50" t="inlineStr">
         <is>
-          <t>Hum Pyaar Karne Wale</t>
+          <t>Teri Deewani</t>
         </is>
       </c>
       <c r="D50" t="inlineStr">
         <is>
-          <t>Shashwat Sachdev, Anuradha Paudwal, Udit Narayan, Anand-Milind, Sameer Anjaan, Qveen Herby</t>
+          <t>Kailash Kher, Paresh Kamath, Naresh Kamath</t>
         </is>
       </c>
     </row>
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>2026-03-28</t>
+          <t>2026-03-29</t>
         </is>
       </c>
       <c r="B51" t="n">
@@ -8728,12 +10802,12 @@
       </c>
       <c r="C51" t="inlineStr">
         <is>
-          <t>Teri Deewani</t>
+          <t>Dealer</t>
         </is>
       </c>
       <c r="D51" t="inlineStr">
         <is>
-          <t>Kailash Kher, Paresh Kamath, Naresh Kamath</t>
+          <t>Diljit Dosanjh, Da Future, Virk Andaaz</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
added data for 31st march got predictions for 1st april
</commit_message>
<xml_diff>
--- a/Probability Project.xlsx
+++ b/Probability Project.xlsx
@@ -20,6 +20,7 @@
     <sheet name="AUTO_20260328" sheetId="15" state="visible" r:id="rId15"/>
     <sheet name="AUTO_20260330" sheetId="16" state="visible" r:id="rId16"/>
     <sheet name="AUTO_20260329" sheetId="17" state="visible" r:id="rId17"/>
+    <sheet name="AUTO_20260331" sheetId="18" state="visible" r:id="rId18"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -9812,9 +9813,1045 @@
       </c>
     </row>
     <row r="2">
+      <c r="A2" s="0" t="inlineStr">
+        <is>
+          <t>2026-03-29</t>
+        </is>
+      </c>
+      <c r="B2" s="0" t="n">
+        <v>1</v>
+      </c>
+      <c r="C2" s="0" t="inlineStr">
+        <is>
+          <t>Bairan</t>
+        </is>
+      </c>
+      <c r="D2" s="0" t="inlineStr">
+        <is>
+          <t>Banjaare</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="0" t="inlineStr">
+        <is>
+          <t>2026-03-29</t>
+        </is>
+      </c>
+      <c r="B3" s="0" t="n">
+        <v>2</v>
+      </c>
+      <c r="C3" s="0" t="inlineStr">
+        <is>
+          <t>Jaiye Sajana</t>
+        </is>
+      </c>
+      <c r="D3" s="0" t="inlineStr">
+        <is>
+          <t>Shashwat Sachdev, Jasmine Sandlas, Satinder Sartaaj</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="0" t="inlineStr">
+        <is>
+          <t>2026-03-29</t>
+        </is>
+      </c>
+      <c r="B4" s="0" t="n">
+        <v>3</v>
+      </c>
+      <c r="C4" s="0" t="inlineStr">
+        <is>
+          <t>Gehra Hua</t>
+        </is>
+      </c>
+      <c r="D4" s="0" t="inlineStr">
+        <is>
+          <t>Shashwat Sachdev, Arijit Singh, Irshad Kamil, Armaan Khan</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="0" t="inlineStr">
+        <is>
+          <t>2026-03-29</t>
+        </is>
+      </c>
+      <c r="B5" s="0" t="n">
+        <v>4</v>
+      </c>
+      <c r="C5" s="0" t="inlineStr">
+        <is>
+          <t>Sheesha - Aakhya Mai Aakh Ghali Jo Bairan</t>
+        </is>
+      </c>
+      <c r="D5" s="0" t="inlineStr">
+        <is>
+          <t>Mitta Ror, Swara Verma</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="0" t="inlineStr">
+        <is>
+          <t>2026-03-29</t>
+        </is>
+      </c>
+      <c r="B6" s="0" t="n">
+        <v>5</v>
+      </c>
+      <c r="C6" s="0" t="inlineStr">
+        <is>
+          <t>Dhurandhar The Revenge - Aari Aari</t>
+        </is>
+      </c>
+      <c r="D6" s="0" t="inlineStr">
+        <is>
+          <t>Shashwat Sachdev, Bombay Rockers, Irshad Kamil, Khan Saab, Reble, Token, Jasmine Sandlas, Sudhir Yaduvanshi</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="0" t="inlineStr">
+        <is>
+          <t>2026-03-29</t>
+        </is>
+      </c>
+      <c r="B7" s="0" t="n">
+        <v>6</v>
+      </c>
+      <c r="C7" s="0" t="inlineStr">
+        <is>
+          <t>Khat</t>
+        </is>
+      </c>
+      <c r="D7" s="0" t="inlineStr">
+        <is>
+          <t>Navjot Ahuja</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="0" t="inlineStr">
+        <is>
+          <t>2026-03-29</t>
+        </is>
+      </c>
+      <c r="B8" s="0" t="n">
+        <v>7</v>
+      </c>
+      <c r="C8" s="0" t="inlineStr">
+        <is>
+          <t>Jaan Se Guzarte Hain</t>
+        </is>
+      </c>
+      <c r="D8" s="0" t="inlineStr">
+        <is>
+          <t>Shashwat Sachdev, Khan Saab, Nusrat Fateh Ali Khan</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="0" t="inlineStr">
+        <is>
+          <t>2026-03-29</t>
+        </is>
+      </c>
+      <c r="B9" s="0" t="n">
+        <v>8</v>
+      </c>
+      <c r="C9" s="0" t="inlineStr">
+        <is>
+          <t>Sitaare (From "Ikkis")</t>
+        </is>
+      </c>
+      <c r="D9" s="0" t="inlineStr">
+        <is>
+          <t>Arijit Singh, White Noise Collectives, Amitabh Bhattacharya</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="0" t="inlineStr">
+        <is>
+          <t>2026-03-29</t>
+        </is>
+      </c>
+      <c r="B10" s="0" t="n">
+        <v>9</v>
+      </c>
+      <c r="C10" s="0" t="inlineStr">
+        <is>
+          <t>Dooron Dooron</t>
+        </is>
+      </c>
+      <c r="D10" s="0" t="inlineStr">
+        <is>
+          <t>Paresh Pahuja, Shiv Tandan, Meghdeep Bose</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="0" t="inlineStr">
+        <is>
+          <t>2026-03-29</t>
+        </is>
+      </c>
+      <c r="B11" s="0" t="n">
+        <v>10</v>
+      </c>
+      <c r="C11" s="0" t="inlineStr">
+        <is>
+          <t>Sahiba</t>
+        </is>
+      </c>
+      <c r="D11" s="0" t="inlineStr">
+        <is>
+          <t>Aditya Rikhari</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="0" t="inlineStr">
+        <is>
+          <t>2026-03-29</t>
+        </is>
+      </c>
+      <c r="B12" s="0" t="n">
+        <v>11</v>
+      </c>
+      <c r="C12" s="0" t="inlineStr">
+        <is>
+          <t>Samjhawan</t>
+        </is>
+      </c>
+      <c r="D12" s="0" t="inlineStr">
+        <is>
+          <t>Jawad Ahmad, Shaarib Toshi, Arijit Singh, Shreya Ghoshal</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="0" t="inlineStr">
+        <is>
+          <t>2026-03-29</t>
+        </is>
+      </c>
+      <c r="B13" s="0" t="n">
+        <v>12</v>
+      </c>
+      <c r="C13" s="0" t="inlineStr">
+        <is>
+          <t>Shararat</t>
+        </is>
+      </c>
+      <c r="D13" s="0" t="inlineStr">
+        <is>
+          <t>Shashwat Sachdev, Madhubanti Bagchi, Jasmine Sandlas</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="0" t="inlineStr">
+        <is>
+          <t>2026-03-29</t>
+        </is>
+      </c>
+      <c r="B14" s="0" t="n">
+        <v>13</v>
+      </c>
+      <c r="C14" s="0" t="inlineStr">
+        <is>
+          <t>Apna Bana Le</t>
+        </is>
+      </c>
+      <c r="D14" s="0" t="inlineStr">
+        <is>
+          <t>Sachin-Jigar, Arijit Singh, Amitabh Bhattacharya</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="0" t="inlineStr">
+        <is>
+          <t>2026-03-29</t>
+        </is>
+      </c>
+      <c r="B15" s="0" t="n">
+        <v>14</v>
+      </c>
+      <c r="C15" s="0" t="inlineStr">
+        <is>
+          <t>Finding Her</t>
+        </is>
+      </c>
+      <c r="D15" s="0" t="inlineStr">
+        <is>
+          <t>Kushagra, Bharath, Saaheal</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="0" t="inlineStr">
+        <is>
+          <t>2026-03-29</t>
+        </is>
+      </c>
+      <c r="B16" s="0" t="n">
+        <v>15</v>
+      </c>
+      <c r="C16" s="0" t="inlineStr">
+        <is>
+          <t>Dhurandhar - Title Track</t>
+        </is>
+      </c>
+      <c r="D16" s="0" t="inlineStr">
+        <is>
+          <t>Shashwat Sachdev, Hanumankind, Jasmine Sandlas, Sudhir Yaduvanshi, Charanjit Ahuja, Muhammad Sadiq, Ranjit Kaur, Babu Singh Maan</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="0" t="inlineStr">
+        <is>
+          <t>2026-03-29</t>
+        </is>
+      </c>
+      <c r="B17" s="0" t="n">
+        <v>16</v>
+      </c>
+      <c r="C17" s="0" t="inlineStr">
+        <is>
+          <t>Arz Kiya Hai | Coke Studio Bharat</t>
+        </is>
+      </c>
+      <c r="D17" s="0" t="inlineStr">
+        <is>
+          <t>Anuv Jain</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="0" t="inlineStr">
+        <is>
+          <t>2026-03-29</t>
+        </is>
+      </c>
+      <c r="B18" s="0" t="n">
+        <v>17</v>
+      </c>
+      <c r="C18" s="0" t="inlineStr">
+        <is>
+          <t>For A Reason</t>
+        </is>
+      </c>
+      <c r="D18" s="0" t="inlineStr">
+        <is>
+          <t>Karan Aujla, Ikky</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="0" t="inlineStr">
+        <is>
+          <t>2026-03-29</t>
+        </is>
+      </c>
+      <c r="B19" s="0" t="n">
+        <v>18</v>
+      </c>
+      <c r="C19" s="0" t="inlineStr">
+        <is>
+          <t>Pavazha Malli - From "Think Indie"</t>
+        </is>
+      </c>
+      <c r="D19" s="0" t="inlineStr">
+        <is>
+          <t>Sai Abhyankkar, Shruti Haasan, Vivek</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="0" t="inlineStr">
+        <is>
+          <t>2026-03-29</t>
+        </is>
+      </c>
+      <c r="B20" s="0" t="n">
+        <v>19</v>
+      </c>
+      <c r="C20" s="0" t="inlineStr">
+        <is>
+          <t>Ishq</t>
+        </is>
+      </c>
+      <c r="D20" s="0" t="inlineStr">
+        <is>
+          <t>Faheem Abdullah, Rauhan Malik, Amir Ameer</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="0" t="inlineStr">
+        <is>
+          <t>2026-03-29</t>
+        </is>
+      </c>
+      <c r="B21" s="0" t="n">
+        <v>20</v>
+      </c>
+      <c r="C21" s="0" t="inlineStr">
+        <is>
+          <t>Boyfriend</t>
+        </is>
+      </c>
+      <c r="D21" s="0" t="inlineStr">
+        <is>
+          <t>Karan Aujla, Ikky</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="0" t="inlineStr">
+        <is>
+          <t>2026-03-29</t>
+        </is>
+      </c>
+      <c r="B22" s="0" t="n">
+        <v>21</v>
+      </c>
+      <c r="C22" s="0" t="inlineStr">
+        <is>
+          <t>Mann Mera</t>
+        </is>
+      </c>
+      <c r="D22" s="0" t="inlineStr">
+        <is>
+          <t>Gajendra Verma</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="0" t="inlineStr">
+        <is>
+          <t>2026-03-29</t>
+        </is>
+      </c>
+      <c r="B23" s="0" t="n">
+        <v>22</v>
+      </c>
+      <c r="C23" s="0" t="inlineStr">
+        <is>
+          <t>Bairi</t>
+        </is>
+      </c>
+      <c r="D23" s="0" t="inlineStr">
+        <is>
+          <t>Virat, Pradeep Solanki, Heena</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="0" t="inlineStr">
+        <is>
+          <t>2026-03-29</t>
+        </is>
+      </c>
+      <c r="B24" s="0" t="n">
+        <v>23</v>
+      </c>
+      <c r="C24" s="0" t="inlineStr">
+        <is>
+          <t>Ishqa Ve</t>
+        </is>
+      </c>
+      <c r="D24" s="0" t="inlineStr">
+        <is>
+          <t>Zeeshan Ali, Yuvraj Tung, Sandeep Aulakh, Honey Dhillon</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="0" t="inlineStr">
+        <is>
+          <t>2026-03-29</t>
+        </is>
+      </c>
+      <c r="B25" s="0" t="n">
+        <v>24</v>
+      </c>
+      <c r="C25" s="0" t="inlineStr">
+        <is>
+          <t>Naal Nachna</t>
+        </is>
+      </c>
+      <c r="D25" s="0" t="inlineStr">
+        <is>
+          <t>Shashwat Sachdev, Afsana Khan, Irshad Kamil, Reble</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="0" t="inlineStr">
+        <is>
+          <t>2026-03-29</t>
+        </is>
+      </c>
+      <c r="B26" s="0" t="n">
+        <v>25</v>
+      </c>
+      <c r="C26" s="0" t="inlineStr">
+        <is>
+          <t>Phir Se</t>
+        </is>
+      </c>
+      <c r="D26" s="0" t="inlineStr">
+        <is>
+          <t>Shashwat Sachdev, Arijit Singh, Irshad Kamil</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="0" t="inlineStr">
+        <is>
+          <t>2026-03-29</t>
+        </is>
+      </c>
+      <c r="B27" s="0" t="n">
+        <v>26</v>
+      </c>
+      <c r="C27" s="0" t="inlineStr">
+        <is>
+          <t>Saiyaara</t>
+        </is>
+      </c>
+      <c r="D27" s="0" t="inlineStr">
+        <is>
+          <t>Tanishk Bagchi, Faheem Abdullah, Arslan Nizami, Irshad Kamil</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="0" t="inlineStr">
+        <is>
+          <t>2026-03-29</t>
+        </is>
+      </c>
+      <c r="B28" s="0" t="n">
+        <v>27</v>
+      </c>
+      <c r="C28" s="0" t="inlineStr">
+        <is>
+          <t>Deewaana Deewaana</t>
+        </is>
+      </c>
+      <c r="D28" s="0" t="inlineStr">
+        <is>
+          <t>A.R. Rahman, Irshad Kamil</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="0" t="inlineStr">
+        <is>
+          <t>2026-03-29</t>
+        </is>
+      </c>
+      <c r="B29" s="0" t="n">
+        <v>28</v>
+      </c>
+      <c r="C29" s="0" t="inlineStr">
+        <is>
+          <t>Tere Liye</t>
+        </is>
+      </c>
+      <c r="D29" s="0" t="inlineStr">
+        <is>
+          <t>Atif Aslam, Shreya Ghoshal, Sachin Gupta, Sameer Anjaan</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="0" t="inlineStr">
+        <is>
+          <t>2026-03-29</t>
+        </is>
+      </c>
+      <c r="B30" s="0" t="n">
+        <v>29</v>
+      </c>
+      <c r="C30" s="0" t="inlineStr">
+        <is>
+          <t>Lutt Le Gaya</t>
+        </is>
+      </c>
+      <c r="D30" s="0" t="inlineStr">
+        <is>
+          <t>Shashwat Sachdev, Simran Choudhary</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="0" t="inlineStr">
+        <is>
+          <t>2026-03-29</t>
+        </is>
+      </c>
+      <c r="B31" s="0" t="n">
+        <v>30</v>
+      </c>
+      <c r="C31" s="0" t="inlineStr">
+        <is>
+          <t>Raanjhan (From "Do Patti")</t>
+        </is>
+      </c>
+      <c r="D31" s="0" t="inlineStr">
+        <is>
+          <t>Sachet-Parampara, Parampara Tandon, Kausar Munir</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="0" t="inlineStr">
+        <is>
+          <t>2026-03-29</t>
+        </is>
+      </c>
+      <c r="B32" s="0" t="n">
+        <v>31</v>
+      </c>
+      <c r="C32" s="0" t="inlineStr">
+        <is>
+          <t>Tum Ho Toh (From "Saiyaara")</t>
+        </is>
+      </c>
+      <c r="D32" s="0" t="inlineStr">
+        <is>
+          <t>Vishal Mishra, Hansika Pareek, Raj Shekhar</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="0" t="inlineStr">
+        <is>
+          <t>2026-03-29</t>
+        </is>
+      </c>
+      <c r="B33" s="0" t="n">
+        <v>32</v>
+      </c>
+      <c r="C33" s="0" t="inlineStr">
+        <is>
+          <t>Main Aur Tu (From "Dhurandhar The Revenge")</t>
+        </is>
+      </c>
+      <c r="D33" s="0" t="inlineStr">
+        <is>
+          <t>Shashwat Sachdev, Jasmine Sandlas, Reble</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="0" t="inlineStr">
+        <is>
+          <t>2026-03-29</t>
+        </is>
+      </c>
+      <c r="B34" s="0" t="n">
+        <v>33</v>
+      </c>
+      <c r="C34" s="0" t="inlineStr">
+        <is>
+          <t>Ishq Jalakar - Karvaan</t>
+        </is>
+      </c>
+      <c r="D34" s="0" t="inlineStr">
+        <is>
+          <t>Shashwat Sachdev, Shahzad Ali, Subhadeep Das Chowdhury, Armaan Khan, Irshad Kamil, Roshan, Sahir Ludhianvi</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="0" t="inlineStr">
+        <is>
+          <t>2026-03-29</t>
+        </is>
+      </c>
+      <c r="B35" s="0" t="n">
+        <v>34</v>
+      </c>
+      <c r="C35" s="0" t="inlineStr">
+        <is>
+          <t>Darkhaast</t>
+        </is>
+      </c>
+      <c r="D35" s="0" t="inlineStr">
+        <is>
+          <t>Mithoon, Arijit Singh, Sunidhi Chauhan, Sayeed Quadri</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="0" t="inlineStr">
+        <is>
+          <t>2026-03-29</t>
+        </is>
+      </c>
+      <c r="B36" s="0" t="n">
+        <v>35</v>
+      </c>
+      <c r="C36" s="0" t="inlineStr">
+        <is>
+          <t>Jo Tum Mere Ho</t>
+        </is>
+      </c>
+      <c r="D36" s="0" t="inlineStr">
+        <is>
+          <t>Anuv Jain</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="0" t="inlineStr">
+        <is>
+          <t>2026-03-29</t>
+        </is>
+      </c>
+      <c r="B37" s="0" t="n">
+        <v>36</v>
+      </c>
+      <c r="C37" s="0" t="inlineStr">
+        <is>
+          <t>Tere Bina</t>
+        </is>
+      </c>
+      <c r="D37" s="0" t="inlineStr">
+        <is>
+          <t>A.R. Rahman, Chinmayi, Murtuza Khan, Qadir Khan</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="0" t="inlineStr">
+        <is>
+          <t>2026-03-29</t>
+        </is>
+      </c>
+      <c r="B38" s="0" t="n">
+        <v>37</v>
+      </c>
+      <c r="C38" s="0" t="inlineStr">
+        <is>
+          <t>Run Down The City - Monica</t>
+        </is>
+      </c>
+      <c r="D38" s="0" t="inlineStr">
+        <is>
+          <t>Shashwat Sachdev, Reble, Asha Bhosle, R. D. Burman, Majrooh Sultanpuri</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="0" t="inlineStr">
+        <is>
+          <t>2026-03-29</t>
+        </is>
+      </c>
+      <c r="B39" s="0" t="n">
+        <v>38</v>
+      </c>
+      <c r="C39" s="0" t="inlineStr">
+        <is>
+          <t>Haseen</t>
+        </is>
+      </c>
+      <c r="D39" s="0" t="inlineStr">
+        <is>
+          <t>Talwiinder, NDS, Rippy Grewal</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="0" t="inlineStr">
+        <is>
+          <t>2026-03-29</t>
+        </is>
+      </c>
+      <c r="B40" s="0" t="n">
+        <v>39</v>
+      </c>
+      <c r="C40" s="0" t="inlineStr">
+        <is>
+          <t>Agar Tum Saath Ho (From "Tamasha")</t>
+        </is>
+      </c>
+      <c r="D40" s="0" t="inlineStr">
+        <is>
+          <t>Alka Yagnik, Arijit Singh</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" s="0" t="inlineStr">
+        <is>
+          <t>2026-03-29</t>
+        </is>
+      </c>
+      <c r="B41" s="0" t="n">
+        <v>40</v>
+      </c>
+      <c r="C41" s="0" t="inlineStr">
+        <is>
+          <t>Ye Tune Kya Kiya</t>
+        </is>
+      </c>
+      <c r="D41" s="0" t="inlineStr">
+        <is>
+          <t>Pritam, Javed Bashir, Rajat Arora</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" s="0" t="inlineStr">
+        <is>
+          <t>2026-03-29</t>
+        </is>
+      </c>
+      <c r="B42" s="0" t="n">
+        <v>41</v>
+      </c>
+      <c r="C42" s="0" t="inlineStr">
+        <is>
+          <t>Aaya Sher (From "The Paradise") (Telugu)</t>
+        </is>
+      </c>
+      <c r="D42" s="0" t="inlineStr">
+        <is>
+          <t>Anirudh Ravichander, Jangi Reddy, Arjun Chandy, Kasarla Shyam</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" s="0" t="inlineStr">
+        <is>
+          <t>2026-03-29</t>
+        </is>
+      </c>
+      <c r="B43" s="0" t="n">
+        <v>42</v>
+      </c>
+      <c r="C43" s="0" t="inlineStr">
+        <is>
+          <t>Mutta Kalakki (From "Youth")</t>
+        </is>
+      </c>
+      <c r="D43" s="0" t="inlineStr">
+        <is>
+          <t>G. V. Prakash, Ken Karunaas</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" s="0" t="inlineStr">
+        <is>
+          <t>2026-03-29</t>
+        </is>
+      </c>
+      <c r="B44" s="0" t="n">
+        <v>43</v>
+      </c>
+      <c r="C44" s="0" t="inlineStr">
+        <is>
+          <t>SWIM</t>
+        </is>
+      </c>
+      <c r="D44" s="0" t="inlineStr">
+        <is>
+          <t>BTS</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" s="0" t="inlineStr">
+        <is>
+          <t>2026-03-29</t>
+        </is>
+      </c>
+      <c r="B45" s="0" t="n">
+        <v>44</v>
+      </c>
+      <c r="C45" s="0" t="inlineStr">
+        <is>
+          <t>Barbaad (From "Saiyaara")</t>
+        </is>
+      </c>
+      <c r="D45" s="0" t="inlineStr">
+        <is>
+          <t>The Rish, Jubin Nautiyal</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" s="0" t="inlineStr">
+        <is>
+          <t>2026-03-29</t>
+        </is>
+      </c>
+      <c r="B46" s="0" t="n">
+        <v>45</v>
+      </c>
+      <c r="C46" s="0" t="inlineStr">
+        <is>
+          <t>Not Guilty</t>
+        </is>
+      </c>
+      <c r="D46" s="0" t="inlineStr">
+        <is>
+          <t>Dhanda Nyoliwala</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" s="0" t="inlineStr">
+        <is>
+          <t>2026-03-29</t>
+        </is>
+      </c>
+      <c r="B47" s="0" t="n">
+        <v>46</v>
+      </c>
+      <c r="C47" s="0" t="inlineStr">
+        <is>
+          <t>Jogi</t>
+        </is>
+      </c>
+      <c r="D47" s="0" t="inlineStr">
+        <is>
+          <t>thiarajxtt, Bir</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" s="0" t="inlineStr">
+        <is>
+          <t>2026-03-29</t>
+        </is>
+      </c>
+      <c r="B48" s="0" t="n">
+        <v>47</v>
+      </c>
+      <c r="C48" s="0" t="inlineStr">
+        <is>
+          <t>Mann Mera - Original Version</t>
+        </is>
+      </c>
+      <c r="D48" s="0" t="inlineStr">
+        <is>
+          <t>Gajendra Verma</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" s="0" t="inlineStr">
+        <is>
+          <t>2026-03-29</t>
+        </is>
+      </c>
+      <c r="B49" s="0" t="n">
+        <v>48</v>
+      </c>
+      <c r="C49" s="0" t="inlineStr">
+        <is>
+          <t>Ehsaas</t>
+        </is>
+      </c>
+      <c r="D49" s="0" t="inlineStr">
+        <is>
+          <t>Faheem Abdullah, Duha Shah, Vaibhav Pani, Hyder Dar</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" s="0" t="inlineStr">
+        <is>
+          <t>2026-03-29</t>
+        </is>
+      </c>
+      <c r="B50" s="0" t="n">
+        <v>49</v>
+      </c>
+      <c r="C50" s="0" t="inlineStr">
+        <is>
+          <t>Teri Deewani</t>
+        </is>
+      </c>
+      <c r="D50" s="0" t="inlineStr">
+        <is>
+          <t>Kailash Kher, Paresh Kamath, Naresh Kamath</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" s="0" t="inlineStr">
+        <is>
+          <t>2026-03-29</t>
+        </is>
+      </c>
+      <c r="B51" s="0" t="n">
+        <v>50</v>
+      </c>
+      <c r="C51" s="0" t="inlineStr">
+        <is>
+          <t>Dealer</t>
+        </is>
+      </c>
+      <c r="D51" s="0" t="inlineStr">
+        <is>
+          <t>Diljit Dosanjh, Da Future, Virk Andaaz</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet18.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:D51"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="24" t="inlineStr">
+        <is>
+          <t>Date</t>
+        </is>
+      </c>
+      <c r="B1" s="24" t="inlineStr">
+        <is>
+          <t>Rank</t>
+        </is>
+      </c>
+      <c r="C1" s="24" t="inlineStr">
+        <is>
+          <t>Song</t>
+        </is>
+      </c>
+      <c r="D1" s="24" t="inlineStr">
+        <is>
+          <t>Artist</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>2026-03-29</t>
+          <t>2026-03-31</t>
         </is>
       </c>
       <c r="B2" t="n">
@@ -9834,7 +10871,7 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>2026-03-29</t>
+          <t>2026-03-31</t>
         </is>
       </c>
       <c r="B3" t="n">
@@ -9854,7 +10891,7 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>2026-03-29</t>
+          <t>2026-03-31</t>
         </is>
       </c>
       <c r="B4" t="n">
@@ -9874,7 +10911,7 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>2026-03-29</t>
+          <t>2026-03-31</t>
         </is>
       </c>
       <c r="B5" t="n">
@@ -9894,7 +10931,7 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>2026-03-29</t>
+          <t>2026-03-31</t>
         </is>
       </c>
       <c r="B6" t="n">
@@ -9902,19 +10939,19 @@
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>Dhurandhar The Revenge - Aari Aari</t>
+          <t>Khat</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>Shashwat Sachdev, Bombay Rockers, Irshad Kamil, Khan Saab, Reble, Token, Jasmine Sandlas, Sudhir Yaduvanshi</t>
+          <t>Navjot Ahuja</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>2026-03-29</t>
+          <t>2026-03-31</t>
         </is>
       </c>
       <c r="B7" t="n">
@@ -9922,19 +10959,19 @@
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>Khat</t>
+          <t>Dhurandhar The Revenge - Aari Aari</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>Navjot Ahuja</t>
+          <t>Shashwat Sachdev, Bombay Rockers, Irshad Kamil, Khan Saab, Reble, Token, Jasmine Sandlas, Sudhir Yaduvanshi</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>2026-03-29</t>
+          <t>2026-03-31</t>
         </is>
       </c>
       <c r="B8" t="n">
@@ -9954,7 +10991,7 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>2026-03-29</t>
+          <t>2026-03-31</t>
         </is>
       </c>
       <c r="B9" t="n">
@@ -9974,7 +11011,7 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>2026-03-29</t>
+          <t>2026-03-31</t>
         </is>
       </c>
       <c r="B10" t="n">
@@ -9994,7 +11031,7 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>2026-03-29</t>
+          <t>2026-03-31</t>
         </is>
       </c>
       <c r="B11" t="n">
@@ -10002,19 +11039,19 @@
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>Sahiba</t>
+          <t>Samjhawan</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>Aditya Rikhari</t>
+          <t>Jawad Ahmad, Shaarib Toshi, Arijit Singh, Shreya Ghoshal</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>2026-03-29</t>
+          <t>2026-03-31</t>
         </is>
       </c>
       <c r="B12" t="n">
@@ -10022,19 +11059,19 @@
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>Samjhawan</t>
+          <t>Sahiba</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>Jawad Ahmad, Shaarib Toshi, Arijit Singh, Shreya Ghoshal</t>
+          <t>Aditya Rikhari</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>2026-03-29</t>
+          <t>2026-03-31</t>
         </is>
       </c>
       <c r="B13" t="n">
@@ -10042,19 +11079,19 @@
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>Shararat</t>
+          <t>Apna Bana Le</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>Shashwat Sachdev, Madhubanti Bagchi, Jasmine Sandlas</t>
+          <t>Sachin-Jigar, Arijit Singh, Amitabh Bhattacharya</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>2026-03-29</t>
+          <t>2026-03-31</t>
         </is>
       </c>
       <c r="B14" t="n">
@@ -10062,19 +11099,19 @@
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>Apna Bana Le</t>
+          <t>Shararat</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>Sachin-Jigar, Arijit Singh, Amitabh Bhattacharya</t>
+          <t>Shashwat Sachdev, Madhubanti Bagchi, Jasmine Sandlas</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>2026-03-29</t>
+          <t>2026-03-31</t>
         </is>
       </c>
       <c r="B15" t="n">
@@ -10094,7 +11131,7 @@
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>2026-03-29</t>
+          <t>2026-03-31</t>
         </is>
       </c>
       <c r="B16" t="n">
@@ -10102,19 +11139,19 @@
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>Dhurandhar - Title Track</t>
+          <t>Arz Kiya Hai | Coke Studio Bharat</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>Shashwat Sachdev, Hanumankind, Jasmine Sandlas, Sudhir Yaduvanshi, Charanjit Ahuja, Muhammad Sadiq, Ranjit Kaur, Babu Singh Maan</t>
+          <t>Anuv Jain</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>2026-03-29</t>
+          <t>2026-03-31</t>
         </is>
       </c>
       <c r="B17" t="n">
@@ -10122,19 +11159,19 @@
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>Arz Kiya Hai | Coke Studio Bharat</t>
+          <t>Pavazha Malli - From "Think Indie"</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>Anuv Jain</t>
+          <t>Sai Abhyankkar, Shruti Haasan, Vivek</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>2026-03-29</t>
+          <t>2026-03-31</t>
         </is>
       </c>
       <c r="B18" t="n">
@@ -10142,19 +11179,19 @@
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>For A Reason</t>
+          <t>Dhurandhar - Title Track</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>Karan Aujla, Ikky</t>
+          <t>Shashwat Sachdev, Hanumankind, Jasmine Sandlas, Sudhir Yaduvanshi, Charanjit Ahuja, Muhammad Sadiq, Ranjit Kaur, Babu Singh Maan</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>2026-03-29</t>
+          <t>2026-03-31</t>
         </is>
       </c>
       <c r="B19" t="n">
@@ -10162,19 +11199,19 @@
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>Pavazha Malli - From "Think Indie"</t>
+          <t>For A Reason</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>Sai Abhyankkar, Shruti Haasan, Vivek</t>
+          <t>Karan Aujla, Ikky</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>2026-03-29</t>
+          <t>2026-03-31</t>
         </is>
       </c>
       <c r="B20" t="n">
@@ -10182,19 +11219,19 @@
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>Ishq</t>
+          <t>Boyfriend</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>Faheem Abdullah, Rauhan Malik, Amir Ameer</t>
+          <t>Karan Aujla, Ikky</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>2026-03-29</t>
+          <t>2026-03-31</t>
         </is>
       </c>
       <c r="B21" t="n">
@@ -10202,19 +11239,19 @@
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>Boyfriend</t>
+          <t>Ishq</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>Karan Aujla, Ikky</t>
+          <t>Faheem Abdullah, Rauhan Malik, Amir Ameer</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>2026-03-29</t>
+          <t>2026-03-31</t>
         </is>
       </c>
       <c r="B22" t="n">
@@ -10222,19 +11259,19 @@
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>Mann Mera</t>
+          <t>Phir Se</t>
         </is>
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>Gajendra Verma</t>
+          <t>Shashwat Sachdev, Arijit Singh, Irshad Kamil</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>2026-03-29</t>
+          <t>2026-03-31</t>
         </is>
       </c>
       <c r="B23" t="n">
@@ -10242,19 +11279,19 @@
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>Bairi</t>
+          <t>Mann Mera</t>
         </is>
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>Virat, Pradeep Solanki, Heena</t>
+          <t>Gajendra Verma</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>2026-03-29</t>
+          <t>2026-03-31</t>
         </is>
       </c>
       <c r="B24" t="n">
@@ -10274,7 +11311,7 @@
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>2026-03-29</t>
+          <t>2026-03-31</t>
         </is>
       </c>
       <c r="B25" t="n">
@@ -10282,19 +11319,19 @@
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>Naal Nachna</t>
+          <t>Bairi</t>
         </is>
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>Shashwat Sachdev, Afsana Khan, Irshad Kamil, Reble</t>
+          <t>Virat, Pradeep Solanki, Heena</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>2026-03-29</t>
+          <t>2026-03-31</t>
         </is>
       </c>
       <c r="B26" t="n">
@@ -10302,19 +11339,19 @@
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>Phir Se</t>
+          <t>Saiyaara</t>
         </is>
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>Shashwat Sachdev, Arijit Singh, Irshad Kamil</t>
+          <t>Tanishk Bagchi, Faheem Abdullah, Arslan Nizami, Irshad Kamil</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>2026-03-29</t>
+          <t>2026-03-31</t>
         </is>
       </c>
       <c r="B27" t="n">
@@ -10322,19 +11359,19 @@
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>Saiyaara</t>
+          <t>Naal Nachna</t>
         </is>
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t>Tanishk Bagchi, Faheem Abdullah, Arslan Nizami, Irshad Kamil</t>
+          <t>Shashwat Sachdev, Afsana Khan, Irshad Kamil, Reble</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>2026-03-29</t>
+          <t>2026-03-31</t>
         </is>
       </c>
       <c r="B28" t="n">
@@ -10354,7 +11391,7 @@
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>2026-03-29</t>
+          <t>2026-03-31</t>
         </is>
       </c>
       <c r="B29" t="n">
@@ -10374,7 +11411,7 @@
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>2026-03-29</t>
+          <t>2026-03-31</t>
         </is>
       </c>
       <c r="B30" t="n">
@@ -10382,19 +11419,19 @@
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>Lutt Le Gaya</t>
+          <t>Tum Ho Toh (From "Saiyaara")</t>
         </is>
       </c>
       <c r="D30" t="inlineStr">
         <is>
-          <t>Shashwat Sachdev, Simran Choudhary</t>
+          <t>Vishal Mishra, Hansika Pareek, Raj Shekhar</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>2026-03-29</t>
+          <t>2026-03-31</t>
         </is>
       </c>
       <c r="B31" t="n">
@@ -10402,19 +11439,19 @@
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>Raanjhan (From "Do Patti")</t>
+          <t>Tere Bina</t>
         </is>
       </c>
       <c r="D31" t="inlineStr">
         <is>
-          <t>Sachet-Parampara, Parampara Tandon, Kausar Munir</t>
+          <t>A.R. Rahman, Chinmayi, Murtuza Khan, Qadir Khan</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>2026-03-29</t>
+          <t>2026-03-31</t>
         </is>
       </c>
       <c r="B32" t="n">
@@ -10422,19 +11459,19 @@
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>Tum Ho Toh (From "Saiyaara")</t>
+          <t>Darkhaast</t>
         </is>
       </c>
       <c r="D32" t="inlineStr">
         <is>
-          <t>Vishal Mishra, Hansika Pareek, Raj Shekhar</t>
+          <t>Mithoon, Arijit Singh, Sunidhi Chauhan, Sayeed Quadri</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>2026-03-29</t>
+          <t>2026-03-31</t>
         </is>
       </c>
       <c r="B33" t="n">
@@ -10442,19 +11479,19 @@
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>Main Aur Tu (From "Dhurandhar The Revenge")</t>
+          <t>Lutt Le Gaya</t>
         </is>
       </c>
       <c r="D33" t="inlineStr">
         <is>
-          <t>Shashwat Sachdev, Jasmine Sandlas, Reble</t>
+          <t>Shashwat Sachdev, Simran Choudhary</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>2026-03-29</t>
+          <t>2026-03-31</t>
         </is>
       </c>
       <c r="B34" t="n">
@@ -10462,19 +11499,19 @@
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>Ishq Jalakar - Karvaan</t>
+          <t>Run Down The City - Monica</t>
         </is>
       </c>
       <c r="D34" t="inlineStr">
         <is>
-          <t>Shashwat Sachdev, Shahzad Ali, Subhadeep Das Chowdhury, Armaan Khan, Irshad Kamil, Roshan, Sahir Ludhianvi</t>
+          <t>Shashwat Sachdev, Reble, Asha Bhosle, R. D. Burman, Majrooh Sultanpuri</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>2026-03-29</t>
+          <t>2026-03-31</t>
         </is>
       </c>
       <c r="B35" t="n">
@@ -10482,19 +11519,19 @@
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>Darkhaast</t>
+          <t>Main Aur Tu</t>
         </is>
       </c>
       <c r="D35" t="inlineStr">
         <is>
-          <t>Mithoon, Arijit Singh, Sunidhi Chauhan, Sayeed Quadri</t>
+          <t>Shashwat Sachdev, Jasmine Sandlas, Reble</t>
         </is>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>2026-03-29</t>
+          <t>2026-03-31</t>
         </is>
       </c>
       <c r="B36" t="n">
@@ -10502,19 +11539,19 @@
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>Jo Tum Mere Ho</t>
+          <t>Raanjhan (From "Do Patti")</t>
         </is>
       </c>
       <c r="D36" t="inlineStr">
         <is>
-          <t>Anuv Jain</t>
+          <t>Sachet-Parampara, Parampara Tandon, Kausar Munir</t>
         </is>
       </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>2026-03-29</t>
+          <t>2026-03-31</t>
         </is>
       </c>
       <c r="B37" t="n">
@@ -10522,19 +11559,19 @@
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>Tere Bina</t>
+          <t>Agar Tum Saath Ho (From "Tamasha")</t>
         </is>
       </c>
       <c r="D37" t="inlineStr">
         <is>
-          <t>A.R. Rahman, Chinmayi, Murtuza Khan, Qadir Khan</t>
+          <t>Alka Yagnik, Arijit Singh</t>
         </is>
       </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>2026-03-29</t>
+          <t>2026-03-31</t>
         </is>
       </c>
       <c r="B38" t="n">
@@ -10542,19 +11579,19 @@
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>Run Down The City - Monica</t>
+          <t>Jo Tum Mere Ho</t>
         </is>
       </c>
       <c r="D38" t="inlineStr">
         <is>
-          <t>Shashwat Sachdev, Reble, Asha Bhosle, R. D. Burman, Majrooh Sultanpuri</t>
+          <t>Anuv Jain</t>
         </is>
       </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>2026-03-29</t>
+          <t>2026-03-31</t>
         </is>
       </c>
       <c r="B39" t="n">
@@ -10562,19 +11599,19 @@
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>Haseen</t>
+          <t>Ishq Jalakar - Karvaan</t>
         </is>
       </c>
       <c r="D39" t="inlineStr">
         <is>
-          <t>Talwiinder, NDS, Rippy Grewal</t>
+          <t>Shashwat Sachdev, Shahzad Ali, Subhadeep Das Chowdhury, Armaan Khan, Irshad Kamil, Roshan, Sahir Ludhianvi</t>
         </is>
       </c>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>2026-03-29</t>
+          <t>2026-03-31</t>
         </is>
       </c>
       <c r="B40" t="n">
@@ -10582,19 +11619,19 @@
       </c>
       <c r="C40" t="inlineStr">
         <is>
-          <t>Agar Tum Saath Ho (From "Tamasha")</t>
+          <t>Haseen</t>
         </is>
       </c>
       <c r="D40" t="inlineStr">
         <is>
-          <t>Alka Yagnik, Arijit Singh</t>
+          <t>Talwiinder, NDS, Rippy Grewal</t>
         </is>
       </c>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>2026-03-29</t>
+          <t>2026-03-31</t>
         </is>
       </c>
       <c r="B41" t="n">
@@ -10614,7 +11651,7 @@
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>2026-03-29</t>
+          <t>2026-03-31</t>
         </is>
       </c>
       <c r="B42" t="n">
@@ -10622,19 +11659,19 @@
       </c>
       <c r="C42" t="inlineStr">
         <is>
-          <t>Aaya Sher (From "The Paradise") (Telugu)</t>
+          <t>Barbaad (From "Saiyaara")</t>
         </is>
       </c>
       <c r="D42" t="inlineStr">
         <is>
-          <t>Anirudh Ravichander, Jangi Reddy, Arjun Chandy, Kasarla Shyam</t>
+          <t>The Rish, Jubin Nautiyal</t>
         </is>
       </c>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>2026-03-29</t>
+          <t>2026-03-31</t>
         </is>
       </c>
       <c r="B43" t="n">
@@ -10654,7 +11691,7 @@
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>2026-03-29</t>
+          <t>2026-03-31</t>
         </is>
       </c>
       <c r="B44" t="n">
@@ -10662,19 +11699,19 @@
       </c>
       <c r="C44" t="inlineStr">
         <is>
-          <t>SWIM</t>
+          <t>Vaari Jaavan</t>
         </is>
       </c>
       <c r="D44" t="inlineStr">
         <is>
-          <t>BTS</t>
+          <t>Shashwat Sachdev, Jyoti Nooran, Jasmine Sandlas, Reble</t>
         </is>
       </c>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>2026-03-29</t>
+          <t>2026-03-31</t>
         </is>
       </c>
       <c r="B45" t="n">
@@ -10682,19 +11719,19 @@
       </c>
       <c r="C45" t="inlineStr">
         <is>
-          <t>Barbaad (From "Saiyaara")</t>
+          <t>Jogi</t>
         </is>
       </c>
       <c r="D45" t="inlineStr">
         <is>
-          <t>The Rish, Jubin Nautiyal</t>
+          <t>thiarajxtt, Bir</t>
         </is>
       </c>
     </row>
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>2026-03-29</t>
+          <t>2026-03-31</t>
         </is>
       </c>
       <c r="B46" t="n">
@@ -10702,19 +11739,19 @@
       </c>
       <c r="C46" t="inlineStr">
         <is>
-          <t>Not Guilty</t>
+          <t>Aaya Sher (From "The Paradise") (Telugu)</t>
         </is>
       </c>
       <c r="D46" t="inlineStr">
         <is>
-          <t>Dhanda Nyoliwala</t>
+          <t>Anirudh Ravichander, Jangi Reddy, Arjun Chandy, Kasarla Shyam</t>
         </is>
       </c>
     </row>
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>2026-03-29</t>
+          <t>2026-03-31</t>
         </is>
       </c>
       <c r="B47" t="n">
@@ -10722,19 +11759,19 @@
       </c>
       <c r="C47" t="inlineStr">
         <is>
-          <t>Jogi</t>
+          <t>Ehsaas</t>
         </is>
       </c>
       <c r="D47" t="inlineStr">
         <is>
-          <t>thiarajxtt, Bir</t>
+          <t>Faheem Abdullah, Duha Shah, Vaibhav Pani, Hyder Dar</t>
         </is>
       </c>
     </row>
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>2026-03-29</t>
+          <t>2026-03-31</t>
         </is>
       </c>
       <c r="B48" t="n">
@@ -10742,19 +11779,19 @@
       </c>
       <c r="C48" t="inlineStr">
         <is>
-          <t>Mann Mera - Original Version</t>
+          <t>SWIM</t>
         </is>
       </c>
       <c r="D48" t="inlineStr">
         <is>
-          <t>Gajendra Verma</t>
+          <t>BTS</t>
         </is>
       </c>
     </row>
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>2026-03-29</t>
+          <t>2026-03-31</t>
         </is>
       </c>
       <c r="B49" t="n">
@@ -10762,19 +11799,19 @@
       </c>
       <c r="C49" t="inlineStr">
         <is>
-          <t>Ehsaas</t>
+          <t>Hum Pyaar Karne Wale</t>
         </is>
       </c>
       <c r="D49" t="inlineStr">
         <is>
-          <t>Faheem Abdullah, Duha Shah, Vaibhav Pani, Hyder Dar</t>
+          <t>Shashwat Sachdev, Anuradha Paudwal, Udit Narayan, Anand-Milind, Sameer Anjaan, Qveen Herby</t>
         </is>
       </c>
     </row>
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>2026-03-29</t>
+          <t>2026-03-31</t>
         </is>
       </c>
       <c r="B50" t="n">
@@ -10794,7 +11831,7 @@
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>2026-03-29</t>
+          <t>2026-03-31</t>
         </is>
       </c>
       <c r="B51" t="n">
@@ -10802,12 +11839,12 @@
       </c>
       <c r="C51" t="inlineStr">
         <is>
-          <t>Dealer</t>
+          <t>Mast Magan (From "2 States)</t>
         </is>
       </c>
       <c r="D51" t="inlineStr">
         <is>
-          <t>Diljit Dosanjh, Da Future, Virk Andaaz</t>
+          <t>Arijit Singh, Chinmayi</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
added data for 1st got predictions for 2nd april
</commit_message>
<xml_diff>
--- a/Probability Project.xlsx
+++ b/Probability Project.xlsx
@@ -21,6 +21,7 @@
     <sheet name="AUTO_20260330" sheetId="16" state="visible" r:id="rId16"/>
     <sheet name="AUTO_20260329" sheetId="17" state="visible" r:id="rId17"/>
     <sheet name="AUTO_20260331" sheetId="18" state="visible" r:id="rId18"/>
+    <sheet name="AUTO_20260401" sheetId="19" state="visible" r:id="rId19"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -10849,9 +10850,1045 @@
       </c>
     </row>
     <row r="2">
+      <c r="A2" s="0" t="inlineStr">
+        <is>
+          <t>2026-03-31</t>
+        </is>
+      </c>
+      <c r="B2" s="0" t="n">
+        <v>1</v>
+      </c>
+      <c r="C2" s="0" t="inlineStr">
+        <is>
+          <t>Bairan</t>
+        </is>
+      </c>
+      <c r="D2" s="0" t="inlineStr">
+        <is>
+          <t>Banjaare</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="0" t="inlineStr">
+        <is>
+          <t>2026-03-31</t>
+        </is>
+      </c>
+      <c r="B3" s="0" t="n">
+        <v>2</v>
+      </c>
+      <c r="C3" s="0" t="inlineStr">
+        <is>
+          <t>Jaiye Sajana</t>
+        </is>
+      </c>
+      <c r="D3" s="0" t="inlineStr">
+        <is>
+          <t>Shashwat Sachdev, Jasmine Sandlas, Satinder Sartaaj</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="0" t="inlineStr">
+        <is>
+          <t>2026-03-31</t>
+        </is>
+      </c>
+      <c r="B4" s="0" t="n">
+        <v>3</v>
+      </c>
+      <c r="C4" s="0" t="inlineStr">
+        <is>
+          <t>Gehra Hua</t>
+        </is>
+      </c>
+      <c r="D4" s="0" t="inlineStr">
+        <is>
+          <t>Shashwat Sachdev, Arijit Singh, Irshad Kamil, Armaan Khan</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="0" t="inlineStr">
+        <is>
+          <t>2026-03-31</t>
+        </is>
+      </c>
+      <c r="B5" s="0" t="n">
+        <v>4</v>
+      </c>
+      <c r="C5" s="0" t="inlineStr">
+        <is>
+          <t>Sheesha - Aakhya Mai Aakh Ghali Jo Bairan</t>
+        </is>
+      </c>
+      <c r="D5" s="0" t="inlineStr">
+        <is>
+          <t>Mitta Ror, Swara Verma</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="0" t="inlineStr">
+        <is>
+          <t>2026-03-31</t>
+        </is>
+      </c>
+      <c r="B6" s="0" t="n">
+        <v>5</v>
+      </c>
+      <c r="C6" s="0" t="inlineStr">
+        <is>
+          <t>Khat</t>
+        </is>
+      </c>
+      <c r="D6" s="0" t="inlineStr">
+        <is>
+          <t>Navjot Ahuja</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="0" t="inlineStr">
+        <is>
+          <t>2026-03-31</t>
+        </is>
+      </c>
+      <c r="B7" s="0" t="n">
+        <v>6</v>
+      </c>
+      <c r="C7" s="0" t="inlineStr">
+        <is>
+          <t>Dhurandhar The Revenge - Aari Aari</t>
+        </is>
+      </c>
+      <c r="D7" s="0" t="inlineStr">
+        <is>
+          <t>Shashwat Sachdev, Bombay Rockers, Irshad Kamil, Khan Saab, Reble, Token, Jasmine Sandlas, Sudhir Yaduvanshi</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="0" t="inlineStr">
+        <is>
+          <t>2026-03-31</t>
+        </is>
+      </c>
+      <c r="B8" s="0" t="n">
+        <v>7</v>
+      </c>
+      <c r="C8" s="0" t="inlineStr">
+        <is>
+          <t>Jaan Se Guzarte Hain</t>
+        </is>
+      </c>
+      <c r="D8" s="0" t="inlineStr">
+        <is>
+          <t>Shashwat Sachdev, Khan Saab, Nusrat Fateh Ali Khan</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="0" t="inlineStr">
+        <is>
+          <t>2026-03-31</t>
+        </is>
+      </c>
+      <c r="B9" s="0" t="n">
+        <v>8</v>
+      </c>
+      <c r="C9" s="0" t="inlineStr">
+        <is>
+          <t>Sitaare (From "Ikkis")</t>
+        </is>
+      </c>
+      <c r="D9" s="0" t="inlineStr">
+        <is>
+          <t>Arijit Singh, White Noise Collectives, Amitabh Bhattacharya</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="0" t="inlineStr">
+        <is>
+          <t>2026-03-31</t>
+        </is>
+      </c>
+      <c r="B10" s="0" t="n">
+        <v>9</v>
+      </c>
+      <c r="C10" s="0" t="inlineStr">
+        <is>
+          <t>Dooron Dooron</t>
+        </is>
+      </c>
+      <c r="D10" s="0" t="inlineStr">
+        <is>
+          <t>Paresh Pahuja, Shiv Tandan, Meghdeep Bose</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="0" t="inlineStr">
+        <is>
+          <t>2026-03-31</t>
+        </is>
+      </c>
+      <c r="B11" s="0" t="n">
+        <v>10</v>
+      </c>
+      <c r="C11" s="0" t="inlineStr">
+        <is>
+          <t>Samjhawan</t>
+        </is>
+      </c>
+      <c r="D11" s="0" t="inlineStr">
+        <is>
+          <t>Jawad Ahmad, Shaarib Toshi, Arijit Singh, Shreya Ghoshal</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="0" t="inlineStr">
+        <is>
+          <t>2026-03-31</t>
+        </is>
+      </c>
+      <c r="B12" s="0" t="n">
+        <v>11</v>
+      </c>
+      <c r="C12" s="0" t="inlineStr">
+        <is>
+          <t>Sahiba</t>
+        </is>
+      </c>
+      <c r="D12" s="0" t="inlineStr">
+        <is>
+          <t>Aditya Rikhari</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="0" t="inlineStr">
+        <is>
+          <t>2026-03-31</t>
+        </is>
+      </c>
+      <c r="B13" s="0" t="n">
+        <v>12</v>
+      </c>
+      <c r="C13" s="0" t="inlineStr">
+        <is>
+          <t>Apna Bana Le</t>
+        </is>
+      </c>
+      <c r="D13" s="0" t="inlineStr">
+        <is>
+          <t>Sachin-Jigar, Arijit Singh, Amitabh Bhattacharya</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="0" t="inlineStr">
+        <is>
+          <t>2026-03-31</t>
+        </is>
+      </c>
+      <c r="B14" s="0" t="n">
+        <v>13</v>
+      </c>
+      <c r="C14" s="0" t="inlineStr">
+        <is>
+          <t>Shararat</t>
+        </is>
+      </c>
+      <c r="D14" s="0" t="inlineStr">
+        <is>
+          <t>Shashwat Sachdev, Madhubanti Bagchi, Jasmine Sandlas</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="0" t="inlineStr">
+        <is>
+          <t>2026-03-31</t>
+        </is>
+      </c>
+      <c r="B15" s="0" t="n">
+        <v>14</v>
+      </c>
+      <c r="C15" s="0" t="inlineStr">
+        <is>
+          <t>Finding Her</t>
+        </is>
+      </c>
+      <c r="D15" s="0" t="inlineStr">
+        <is>
+          <t>Kushagra, Bharath, Saaheal</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="0" t="inlineStr">
+        <is>
+          <t>2026-03-31</t>
+        </is>
+      </c>
+      <c r="B16" s="0" t="n">
+        <v>15</v>
+      </c>
+      <c r="C16" s="0" t="inlineStr">
+        <is>
+          <t>Arz Kiya Hai | Coke Studio Bharat</t>
+        </is>
+      </c>
+      <c r="D16" s="0" t="inlineStr">
+        <is>
+          <t>Anuv Jain</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="0" t="inlineStr">
+        <is>
+          <t>2026-03-31</t>
+        </is>
+      </c>
+      <c r="B17" s="0" t="n">
+        <v>16</v>
+      </c>
+      <c r="C17" s="0" t="inlineStr">
+        <is>
+          <t>Pavazha Malli - From "Think Indie"</t>
+        </is>
+      </c>
+      <c r="D17" s="0" t="inlineStr">
+        <is>
+          <t>Sai Abhyankkar, Shruti Haasan, Vivek</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="0" t="inlineStr">
+        <is>
+          <t>2026-03-31</t>
+        </is>
+      </c>
+      <c r="B18" s="0" t="n">
+        <v>17</v>
+      </c>
+      <c r="C18" s="0" t="inlineStr">
+        <is>
+          <t>Dhurandhar - Title Track</t>
+        </is>
+      </c>
+      <c r="D18" s="0" t="inlineStr">
+        <is>
+          <t>Shashwat Sachdev, Hanumankind, Jasmine Sandlas, Sudhir Yaduvanshi, Charanjit Ahuja, Muhammad Sadiq, Ranjit Kaur, Babu Singh Maan</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="0" t="inlineStr">
+        <is>
+          <t>2026-03-31</t>
+        </is>
+      </c>
+      <c r="B19" s="0" t="n">
+        <v>18</v>
+      </c>
+      <c r="C19" s="0" t="inlineStr">
+        <is>
+          <t>For A Reason</t>
+        </is>
+      </c>
+      <c r="D19" s="0" t="inlineStr">
+        <is>
+          <t>Karan Aujla, Ikky</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="0" t="inlineStr">
+        <is>
+          <t>2026-03-31</t>
+        </is>
+      </c>
+      <c r="B20" s="0" t="n">
+        <v>19</v>
+      </c>
+      <c r="C20" s="0" t="inlineStr">
+        <is>
+          <t>Boyfriend</t>
+        </is>
+      </c>
+      <c r="D20" s="0" t="inlineStr">
+        <is>
+          <t>Karan Aujla, Ikky</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="0" t="inlineStr">
+        <is>
+          <t>2026-03-31</t>
+        </is>
+      </c>
+      <c r="B21" s="0" t="n">
+        <v>20</v>
+      </c>
+      <c r="C21" s="0" t="inlineStr">
+        <is>
+          <t>Ishq</t>
+        </is>
+      </c>
+      <c r="D21" s="0" t="inlineStr">
+        <is>
+          <t>Faheem Abdullah, Rauhan Malik, Amir Ameer</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="0" t="inlineStr">
+        <is>
+          <t>2026-03-31</t>
+        </is>
+      </c>
+      <c r="B22" s="0" t="n">
+        <v>21</v>
+      </c>
+      <c r="C22" s="0" t="inlineStr">
+        <is>
+          <t>Phir Se</t>
+        </is>
+      </c>
+      <c r="D22" s="0" t="inlineStr">
+        <is>
+          <t>Shashwat Sachdev, Arijit Singh, Irshad Kamil</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="0" t="inlineStr">
+        <is>
+          <t>2026-03-31</t>
+        </is>
+      </c>
+      <c r="B23" s="0" t="n">
+        <v>22</v>
+      </c>
+      <c r="C23" s="0" t="inlineStr">
+        <is>
+          <t>Mann Mera</t>
+        </is>
+      </c>
+      <c r="D23" s="0" t="inlineStr">
+        <is>
+          <t>Gajendra Verma</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="0" t="inlineStr">
+        <is>
+          <t>2026-03-31</t>
+        </is>
+      </c>
+      <c r="B24" s="0" t="n">
+        <v>23</v>
+      </c>
+      <c r="C24" s="0" t="inlineStr">
+        <is>
+          <t>Ishqa Ve</t>
+        </is>
+      </c>
+      <c r="D24" s="0" t="inlineStr">
+        <is>
+          <t>Zeeshan Ali, Yuvraj Tung, Sandeep Aulakh, Honey Dhillon</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="0" t="inlineStr">
+        <is>
+          <t>2026-03-31</t>
+        </is>
+      </c>
+      <c r="B25" s="0" t="n">
+        <v>24</v>
+      </c>
+      <c r="C25" s="0" t="inlineStr">
+        <is>
+          <t>Bairi</t>
+        </is>
+      </c>
+      <c r="D25" s="0" t="inlineStr">
+        <is>
+          <t>Virat, Pradeep Solanki, Heena</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="0" t="inlineStr">
+        <is>
+          <t>2026-03-31</t>
+        </is>
+      </c>
+      <c r="B26" s="0" t="n">
+        <v>25</v>
+      </c>
+      <c r="C26" s="0" t="inlineStr">
+        <is>
+          <t>Saiyaara</t>
+        </is>
+      </c>
+      <c r="D26" s="0" t="inlineStr">
+        <is>
+          <t>Tanishk Bagchi, Faheem Abdullah, Arslan Nizami, Irshad Kamil</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="0" t="inlineStr">
+        <is>
+          <t>2026-03-31</t>
+        </is>
+      </c>
+      <c r="B27" s="0" t="n">
+        <v>26</v>
+      </c>
+      <c r="C27" s="0" t="inlineStr">
+        <is>
+          <t>Naal Nachna</t>
+        </is>
+      </c>
+      <c r="D27" s="0" t="inlineStr">
+        <is>
+          <t>Shashwat Sachdev, Afsana Khan, Irshad Kamil, Reble</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="0" t="inlineStr">
+        <is>
+          <t>2026-03-31</t>
+        </is>
+      </c>
+      <c r="B28" s="0" t="n">
+        <v>27</v>
+      </c>
+      <c r="C28" s="0" t="inlineStr">
+        <is>
+          <t>Deewaana Deewaana</t>
+        </is>
+      </c>
+      <c r="D28" s="0" t="inlineStr">
+        <is>
+          <t>A.R. Rahman, Irshad Kamil</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="0" t="inlineStr">
+        <is>
+          <t>2026-03-31</t>
+        </is>
+      </c>
+      <c r="B29" s="0" t="n">
+        <v>28</v>
+      </c>
+      <c r="C29" s="0" t="inlineStr">
+        <is>
+          <t>Tere Liye</t>
+        </is>
+      </c>
+      <c r="D29" s="0" t="inlineStr">
+        <is>
+          <t>Atif Aslam, Shreya Ghoshal, Sachin Gupta, Sameer Anjaan</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="0" t="inlineStr">
+        <is>
+          <t>2026-03-31</t>
+        </is>
+      </c>
+      <c r="B30" s="0" t="n">
+        <v>29</v>
+      </c>
+      <c r="C30" s="0" t="inlineStr">
+        <is>
+          <t>Tum Ho Toh (From "Saiyaara")</t>
+        </is>
+      </c>
+      <c r="D30" s="0" t="inlineStr">
+        <is>
+          <t>Vishal Mishra, Hansika Pareek, Raj Shekhar</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="0" t="inlineStr">
+        <is>
+          <t>2026-03-31</t>
+        </is>
+      </c>
+      <c r="B31" s="0" t="n">
+        <v>30</v>
+      </c>
+      <c r="C31" s="0" t="inlineStr">
+        <is>
+          <t>Tere Bina</t>
+        </is>
+      </c>
+      <c r="D31" s="0" t="inlineStr">
+        <is>
+          <t>A.R. Rahman, Chinmayi, Murtuza Khan, Qadir Khan</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="0" t="inlineStr">
+        <is>
+          <t>2026-03-31</t>
+        </is>
+      </c>
+      <c r="B32" s="0" t="n">
+        <v>31</v>
+      </c>
+      <c r="C32" s="0" t="inlineStr">
+        <is>
+          <t>Darkhaast</t>
+        </is>
+      </c>
+      <c r="D32" s="0" t="inlineStr">
+        <is>
+          <t>Mithoon, Arijit Singh, Sunidhi Chauhan, Sayeed Quadri</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="0" t="inlineStr">
+        <is>
+          <t>2026-03-31</t>
+        </is>
+      </c>
+      <c r="B33" s="0" t="n">
+        <v>32</v>
+      </c>
+      <c r="C33" s="0" t="inlineStr">
+        <is>
+          <t>Lutt Le Gaya</t>
+        </is>
+      </c>
+      <c r="D33" s="0" t="inlineStr">
+        <is>
+          <t>Shashwat Sachdev, Simran Choudhary</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="0" t="inlineStr">
+        <is>
+          <t>2026-03-31</t>
+        </is>
+      </c>
+      <c r="B34" s="0" t="n">
+        <v>33</v>
+      </c>
+      <c r="C34" s="0" t="inlineStr">
+        <is>
+          <t>Run Down The City - Monica</t>
+        </is>
+      </c>
+      <c r="D34" s="0" t="inlineStr">
+        <is>
+          <t>Shashwat Sachdev, Reble, Asha Bhosle, R. D. Burman, Majrooh Sultanpuri</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="0" t="inlineStr">
+        <is>
+          <t>2026-03-31</t>
+        </is>
+      </c>
+      <c r="B35" s="0" t="n">
+        <v>34</v>
+      </c>
+      <c r="C35" s="0" t="inlineStr">
+        <is>
+          <t>Main Aur Tu</t>
+        </is>
+      </c>
+      <c r="D35" s="0" t="inlineStr">
+        <is>
+          <t>Shashwat Sachdev, Jasmine Sandlas, Reble</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="0" t="inlineStr">
+        <is>
+          <t>2026-03-31</t>
+        </is>
+      </c>
+      <c r="B36" s="0" t="n">
+        <v>35</v>
+      </c>
+      <c r="C36" s="0" t="inlineStr">
+        <is>
+          <t>Raanjhan (From "Do Patti")</t>
+        </is>
+      </c>
+      <c r="D36" s="0" t="inlineStr">
+        <is>
+          <t>Sachet-Parampara, Parampara Tandon, Kausar Munir</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="0" t="inlineStr">
+        <is>
+          <t>2026-03-31</t>
+        </is>
+      </c>
+      <c r="B37" s="0" t="n">
+        <v>36</v>
+      </c>
+      <c r="C37" s="0" t="inlineStr">
+        <is>
+          <t>Agar Tum Saath Ho (From "Tamasha")</t>
+        </is>
+      </c>
+      <c r="D37" s="0" t="inlineStr">
+        <is>
+          <t>Alka Yagnik, Arijit Singh</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="0" t="inlineStr">
+        <is>
+          <t>2026-03-31</t>
+        </is>
+      </c>
+      <c r="B38" s="0" t="n">
+        <v>37</v>
+      </c>
+      <c r="C38" s="0" t="inlineStr">
+        <is>
+          <t>Jo Tum Mere Ho</t>
+        </is>
+      </c>
+      <c r="D38" s="0" t="inlineStr">
+        <is>
+          <t>Anuv Jain</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="0" t="inlineStr">
+        <is>
+          <t>2026-03-31</t>
+        </is>
+      </c>
+      <c r="B39" s="0" t="n">
+        <v>38</v>
+      </c>
+      <c r="C39" s="0" t="inlineStr">
+        <is>
+          <t>Ishq Jalakar - Karvaan</t>
+        </is>
+      </c>
+      <c r="D39" s="0" t="inlineStr">
+        <is>
+          <t>Shashwat Sachdev, Shahzad Ali, Subhadeep Das Chowdhury, Armaan Khan, Irshad Kamil, Roshan, Sahir Ludhianvi</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="0" t="inlineStr">
+        <is>
+          <t>2026-03-31</t>
+        </is>
+      </c>
+      <c r="B40" s="0" t="n">
+        <v>39</v>
+      </c>
+      <c r="C40" s="0" t="inlineStr">
+        <is>
+          <t>Haseen</t>
+        </is>
+      </c>
+      <c r="D40" s="0" t="inlineStr">
+        <is>
+          <t>Talwiinder, NDS, Rippy Grewal</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" s="0" t="inlineStr">
+        <is>
+          <t>2026-03-31</t>
+        </is>
+      </c>
+      <c r="B41" s="0" t="n">
+        <v>40</v>
+      </c>
+      <c r="C41" s="0" t="inlineStr">
+        <is>
+          <t>Ye Tune Kya Kiya</t>
+        </is>
+      </c>
+      <c r="D41" s="0" t="inlineStr">
+        <is>
+          <t>Pritam, Javed Bashir, Rajat Arora</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" s="0" t="inlineStr">
+        <is>
+          <t>2026-03-31</t>
+        </is>
+      </c>
+      <c r="B42" s="0" t="n">
+        <v>41</v>
+      </c>
+      <c r="C42" s="0" t="inlineStr">
+        <is>
+          <t>Barbaad (From "Saiyaara")</t>
+        </is>
+      </c>
+      <c r="D42" s="0" t="inlineStr">
+        <is>
+          <t>The Rish, Jubin Nautiyal</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" s="0" t="inlineStr">
+        <is>
+          <t>2026-03-31</t>
+        </is>
+      </c>
+      <c r="B43" s="0" t="n">
+        <v>42</v>
+      </c>
+      <c r="C43" s="0" t="inlineStr">
+        <is>
+          <t>Mutta Kalakki (From "Youth")</t>
+        </is>
+      </c>
+      <c r="D43" s="0" t="inlineStr">
+        <is>
+          <t>G. V. Prakash, Ken Karunaas</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" s="0" t="inlineStr">
+        <is>
+          <t>2026-03-31</t>
+        </is>
+      </c>
+      <c r="B44" s="0" t="n">
+        <v>43</v>
+      </c>
+      <c r="C44" s="0" t="inlineStr">
+        <is>
+          <t>Vaari Jaavan</t>
+        </is>
+      </c>
+      <c r="D44" s="0" t="inlineStr">
+        <is>
+          <t>Shashwat Sachdev, Jyoti Nooran, Jasmine Sandlas, Reble</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" s="0" t="inlineStr">
+        <is>
+          <t>2026-03-31</t>
+        </is>
+      </c>
+      <c r="B45" s="0" t="n">
+        <v>44</v>
+      </c>
+      <c r="C45" s="0" t="inlineStr">
+        <is>
+          <t>Jogi</t>
+        </is>
+      </c>
+      <c r="D45" s="0" t="inlineStr">
+        <is>
+          <t>thiarajxtt, Bir</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" s="0" t="inlineStr">
+        <is>
+          <t>2026-03-31</t>
+        </is>
+      </c>
+      <c r="B46" s="0" t="n">
+        <v>45</v>
+      </c>
+      <c r="C46" s="0" t="inlineStr">
+        <is>
+          <t>Aaya Sher (From "The Paradise") (Telugu)</t>
+        </is>
+      </c>
+      <c r="D46" s="0" t="inlineStr">
+        <is>
+          <t>Anirudh Ravichander, Jangi Reddy, Arjun Chandy, Kasarla Shyam</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" s="0" t="inlineStr">
+        <is>
+          <t>2026-03-31</t>
+        </is>
+      </c>
+      <c r="B47" s="0" t="n">
+        <v>46</v>
+      </c>
+      <c r="C47" s="0" t="inlineStr">
+        <is>
+          <t>Ehsaas</t>
+        </is>
+      </c>
+      <c r="D47" s="0" t="inlineStr">
+        <is>
+          <t>Faheem Abdullah, Duha Shah, Vaibhav Pani, Hyder Dar</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" s="0" t="inlineStr">
+        <is>
+          <t>2026-03-31</t>
+        </is>
+      </c>
+      <c r="B48" s="0" t="n">
+        <v>47</v>
+      </c>
+      <c r="C48" s="0" t="inlineStr">
+        <is>
+          <t>SWIM</t>
+        </is>
+      </c>
+      <c r="D48" s="0" t="inlineStr">
+        <is>
+          <t>BTS</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" s="0" t="inlineStr">
+        <is>
+          <t>2026-03-31</t>
+        </is>
+      </c>
+      <c r="B49" s="0" t="n">
+        <v>48</v>
+      </c>
+      <c r="C49" s="0" t="inlineStr">
+        <is>
+          <t>Hum Pyaar Karne Wale</t>
+        </is>
+      </c>
+      <c r="D49" s="0" t="inlineStr">
+        <is>
+          <t>Shashwat Sachdev, Anuradha Paudwal, Udit Narayan, Anand-Milind, Sameer Anjaan, Qveen Herby</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" s="0" t="inlineStr">
+        <is>
+          <t>2026-03-31</t>
+        </is>
+      </c>
+      <c r="B50" s="0" t="n">
+        <v>49</v>
+      </c>
+      <c r="C50" s="0" t="inlineStr">
+        <is>
+          <t>Teri Deewani</t>
+        </is>
+      </c>
+      <c r="D50" s="0" t="inlineStr">
+        <is>
+          <t>Kailash Kher, Paresh Kamath, Naresh Kamath</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" s="0" t="inlineStr">
+        <is>
+          <t>2026-03-31</t>
+        </is>
+      </c>
+      <c r="B51" s="0" t="n">
+        <v>50</v>
+      </c>
+      <c r="C51" s="0" t="inlineStr">
+        <is>
+          <t>Mast Magan (From "2 States)</t>
+        </is>
+      </c>
+      <c r="D51" s="0" t="inlineStr">
+        <is>
+          <t>Arijit Singh, Chinmayi</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet19.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:D51"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="24" t="inlineStr">
+        <is>
+          <t>Date</t>
+        </is>
+      </c>
+      <c r="B1" s="24" t="inlineStr">
+        <is>
+          <t>Rank</t>
+        </is>
+      </c>
+      <c r="C1" s="24" t="inlineStr">
+        <is>
+          <t>Song</t>
+        </is>
+      </c>
+      <c r="D1" s="24" t="inlineStr">
+        <is>
+          <t>Artist</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>2026-03-31</t>
+          <t>2026-04-01</t>
         </is>
       </c>
       <c r="B2" t="n">
@@ -10871,7 +11908,7 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>2026-03-31</t>
+          <t>2026-04-01</t>
         </is>
       </c>
       <c r="B3" t="n">
@@ -10891,7 +11928,7 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>2026-03-31</t>
+          <t>2026-04-01</t>
         </is>
       </c>
       <c r="B4" t="n">
@@ -10899,19 +11936,19 @@
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>Gehra Hua</t>
+          <t>Sheesha - Aakhya Mai Aakh Ghali Jo Bairan</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>Shashwat Sachdev, Arijit Singh, Irshad Kamil, Armaan Khan</t>
+          <t>Mitta Ror, Swara Verma</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>2026-03-31</t>
+          <t>2026-04-01</t>
         </is>
       </c>
       <c r="B5" t="n">
@@ -10919,19 +11956,19 @@
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>Sheesha - Aakhya Mai Aakh Ghali Jo Bairan</t>
+          <t>Gehra Hua</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>Mitta Ror, Swara Verma</t>
+          <t>Shashwat Sachdev, Arijit Singh, Irshad Kamil, Armaan Khan</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>2026-03-31</t>
+          <t>2026-04-01</t>
         </is>
       </c>
       <c r="B6" t="n">
@@ -10951,7 +11988,7 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>2026-03-31</t>
+          <t>2026-04-01</t>
         </is>
       </c>
       <c r="B7" t="n">
@@ -10971,7 +12008,7 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>2026-03-31</t>
+          <t>2026-04-01</t>
         </is>
       </c>
       <c r="B8" t="n">
@@ -10991,7 +12028,7 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>2026-03-31</t>
+          <t>2026-04-01</t>
         </is>
       </c>
       <c r="B9" t="n">
@@ -10999,19 +12036,19 @@
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>Sitaare (From "Ikkis")</t>
+          <t>Dooron Dooron</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>Arijit Singh, White Noise Collectives, Amitabh Bhattacharya</t>
+          <t>Paresh Pahuja, Shiv Tandan, Meghdeep Bose</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>2026-03-31</t>
+          <t>2026-04-01</t>
         </is>
       </c>
       <c r="B10" t="n">
@@ -11019,19 +12056,19 @@
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>Dooron Dooron</t>
+          <t>Sitaare (From "Ikkis")</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>Paresh Pahuja, Shiv Tandan, Meghdeep Bose</t>
+          <t>Arijit Singh, White Noise Collectives, Amitabh Bhattacharya</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>2026-03-31</t>
+          <t>2026-04-01</t>
         </is>
       </c>
       <c r="B11" t="n">
@@ -11039,19 +12076,19 @@
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>Samjhawan</t>
+          <t>Sahiba</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>Jawad Ahmad, Shaarib Toshi, Arijit Singh, Shreya Ghoshal</t>
+          <t>Aditya Rikhari</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>2026-03-31</t>
+          <t>2026-04-01</t>
         </is>
       </c>
       <c r="B12" t="n">
@@ -11059,19 +12096,19 @@
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>Sahiba</t>
+          <t>Apna Bana Le</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>Aditya Rikhari</t>
+          <t>Sachin-Jigar, Arijit Singh, Amitabh Bhattacharya</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>2026-03-31</t>
+          <t>2026-04-01</t>
         </is>
       </c>
       <c r="B13" t="n">
@@ -11079,19 +12116,19 @@
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>Apna Bana Le</t>
+          <t>Pavazha Malli - From "Think Indie"</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>Sachin-Jigar, Arijit Singh, Amitabh Bhattacharya</t>
+          <t>Sai Abhyankkar, Shruti Haasan, Vivek</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>2026-03-31</t>
+          <t>2026-04-01</t>
         </is>
       </c>
       <c r="B14" t="n">
@@ -11099,19 +12136,19 @@
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>Shararat</t>
+          <t>Samjhawan</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>Shashwat Sachdev, Madhubanti Bagchi, Jasmine Sandlas</t>
+          <t>Jawad Ahmad, Shaarib Toshi, Arijit Singh, Shreya Ghoshal</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>2026-03-31</t>
+          <t>2026-04-01</t>
         </is>
       </c>
       <c r="B15" t="n">
@@ -11131,7 +12168,7 @@
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>2026-03-31</t>
+          <t>2026-04-01</t>
         </is>
       </c>
       <c r="B16" t="n">
@@ -11139,19 +12176,19 @@
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>Arz Kiya Hai | Coke Studio Bharat</t>
+          <t>Shararat</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>Anuv Jain</t>
+          <t>Shashwat Sachdev, Madhubanti Bagchi, Jasmine Sandlas</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>2026-03-31</t>
+          <t>2026-04-01</t>
         </is>
       </c>
       <c r="B17" t="n">
@@ -11159,19 +12196,19 @@
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>Pavazha Malli - From "Think Indie"</t>
+          <t>Arz Kiya Hai | Coke Studio Bharat</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>Sai Abhyankkar, Shruti Haasan, Vivek</t>
+          <t>Anuv Jain</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>2026-03-31</t>
+          <t>2026-04-01</t>
         </is>
       </c>
       <c r="B18" t="n">
@@ -11191,7 +12228,7 @@
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>2026-03-31</t>
+          <t>2026-04-01</t>
         </is>
       </c>
       <c r="B19" t="n">
@@ -11199,7 +12236,7 @@
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>For A Reason</t>
+          <t>Boyfriend</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
@@ -11211,7 +12248,7 @@
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>2026-03-31</t>
+          <t>2026-04-01</t>
         </is>
       </c>
       <c r="B20" t="n">
@@ -11219,19 +12256,19 @@
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>Boyfriend</t>
+          <t>Ishq</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>Karan Aujla, Ikky</t>
+          <t>Faheem Abdullah, Rauhan Malik, Amir Ameer</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>2026-03-31</t>
+          <t>2026-04-01</t>
         </is>
       </c>
       <c r="B21" t="n">
@@ -11239,19 +12276,19 @@
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>Ishq</t>
+          <t>Phir Se</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>Faheem Abdullah, Rauhan Malik, Amir Ameer</t>
+          <t>Shashwat Sachdev, Arijit Singh, Irshad Kamil</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>2026-03-31</t>
+          <t>2026-04-01</t>
         </is>
       </c>
       <c r="B22" t="n">
@@ -11259,19 +12296,19 @@
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>Phir Se</t>
+          <t>Mann Mera</t>
         </is>
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>Shashwat Sachdev, Arijit Singh, Irshad Kamil</t>
+          <t>Gajendra Verma</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>2026-03-31</t>
+          <t>2026-04-01</t>
         </is>
       </c>
       <c r="B23" t="n">
@@ -11279,19 +12316,19 @@
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>Mann Mera</t>
+          <t>Bairi</t>
         </is>
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>Gajendra Verma</t>
+          <t>Virat, Pradeep Solanki, Heena</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>2026-03-31</t>
+          <t>2026-04-01</t>
         </is>
       </c>
       <c r="B24" t="n">
@@ -11299,19 +12336,19 @@
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>Ishqa Ve</t>
+          <t>Naal Nachna</t>
         </is>
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>Zeeshan Ali, Yuvraj Tung, Sandeep Aulakh, Honey Dhillon</t>
+          <t>Shashwat Sachdev, Afsana Khan, Irshad Kamil, Reble</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>2026-03-31</t>
+          <t>2026-04-01</t>
         </is>
       </c>
       <c r="B25" t="n">
@@ -11319,19 +12356,19 @@
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>Bairi</t>
+          <t>Saiyaara</t>
         </is>
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>Virat, Pradeep Solanki, Heena</t>
+          <t>Tanishk Bagchi, Faheem Abdullah, Arslan Nizami, Irshad Kamil</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>2026-03-31</t>
+          <t>2026-04-01</t>
         </is>
       </c>
       <c r="B26" t="n">
@@ -11339,19 +12376,19 @@
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>Saiyaara</t>
+          <t>For A Reason</t>
         </is>
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>Tanishk Bagchi, Faheem Abdullah, Arslan Nizami, Irshad Kamil</t>
+          <t>Karan Aujla, Ikky</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>2026-03-31</t>
+          <t>2026-04-01</t>
         </is>
       </c>
       <c r="B27" t="n">
@@ -11359,19 +12396,19 @@
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>Naal Nachna</t>
+          <t>Run Down The City - Monica</t>
         </is>
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t>Shashwat Sachdev, Afsana Khan, Irshad Kamil, Reble</t>
+          <t>Shashwat Sachdev, Reble, Asha Bhosle, R. D. Burman, Majrooh Sultanpuri</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>2026-03-31</t>
+          <t>2026-04-01</t>
         </is>
       </c>
       <c r="B28" t="n">
@@ -11379,19 +12416,19 @@
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>Deewaana Deewaana</t>
+          <t>Darkhaast</t>
         </is>
       </c>
       <c r="D28" t="inlineStr">
         <is>
-          <t>A.R. Rahman, Irshad Kamil</t>
+          <t>Mithoon, Arijit Singh, Sunidhi Chauhan, Sayeed Quadri</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>2026-03-31</t>
+          <t>2026-04-01</t>
         </is>
       </c>
       <c r="B29" t="n">
@@ -11399,19 +12436,19 @@
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>Tere Liye</t>
+          <t>Ishqa Ve</t>
         </is>
       </c>
       <c r="D29" t="inlineStr">
         <is>
-          <t>Atif Aslam, Shreya Ghoshal, Sachin Gupta, Sameer Anjaan</t>
+          <t>Zeeshan Ali, Yuvraj Tung, Sandeep Aulakh, Honey Dhillon</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>2026-03-31</t>
+          <t>2026-04-01</t>
         </is>
       </c>
       <c r="B30" t="n">
@@ -11431,7 +12468,7 @@
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>2026-03-31</t>
+          <t>2026-04-01</t>
         </is>
       </c>
       <c r="B31" t="n">
@@ -11439,19 +12476,19 @@
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>Tere Bina</t>
+          <t>Deewaana Deewaana</t>
         </is>
       </c>
       <c r="D31" t="inlineStr">
         <is>
-          <t>A.R. Rahman, Chinmayi, Murtuza Khan, Qadir Khan</t>
+          <t>A.R. Rahman, Irshad Kamil</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>2026-03-31</t>
+          <t>2026-04-01</t>
         </is>
       </c>
       <c r="B32" t="n">
@@ -11459,19 +12496,19 @@
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>Darkhaast</t>
+          <t>Tere Liye</t>
         </is>
       </c>
       <c r="D32" t="inlineStr">
         <is>
-          <t>Mithoon, Arijit Singh, Sunidhi Chauhan, Sayeed Quadri</t>
+          <t>Atif Aslam, Shreya Ghoshal, Sachin Gupta, Sameer Anjaan</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>2026-03-31</t>
+          <t>2026-04-01</t>
         </is>
       </c>
       <c r="B33" t="n">
@@ -11491,7 +12528,7 @@
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>2026-03-31</t>
+          <t>2026-04-01</t>
         </is>
       </c>
       <c r="B34" t="n">
@@ -11499,19 +12536,19 @@
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>Run Down The City - Monica</t>
+          <t>Raanjhan (From "Do Patti")</t>
         </is>
       </c>
       <c r="D34" t="inlineStr">
         <is>
-          <t>Shashwat Sachdev, Reble, Asha Bhosle, R. D. Burman, Majrooh Sultanpuri</t>
+          <t>Sachet-Parampara, Parampara Tandon, Kausar Munir</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>2026-03-31</t>
+          <t>2026-04-01</t>
         </is>
       </c>
       <c r="B35" t="n">
@@ -11531,7 +12568,7 @@
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>2026-03-31</t>
+          <t>2026-04-01</t>
         </is>
       </c>
       <c r="B36" t="n">
@@ -11539,19 +12576,19 @@
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>Raanjhan (From "Do Patti")</t>
+          <t>Haseen</t>
         </is>
       </c>
       <c r="D36" t="inlineStr">
         <is>
-          <t>Sachet-Parampara, Parampara Tandon, Kausar Munir</t>
+          <t>Talwiinder, NDS, Rippy Grewal</t>
         </is>
       </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>2026-03-31</t>
+          <t>2026-04-01</t>
         </is>
       </c>
       <c r="B37" t="n">
@@ -11559,19 +12596,19 @@
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>Agar Tum Saath Ho (From "Tamasha")</t>
+          <t>Jo Tum Mere Ho</t>
         </is>
       </c>
       <c r="D37" t="inlineStr">
         <is>
-          <t>Alka Yagnik, Arijit Singh</t>
+          <t>Anuv Jain</t>
         </is>
       </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>2026-03-31</t>
+          <t>2026-04-01</t>
         </is>
       </c>
       <c r="B38" t="n">
@@ -11579,19 +12616,19 @@
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>Jo Tum Mere Ho</t>
+          <t>Agar Tum Saath Ho (From "Tamasha")</t>
         </is>
       </c>
       <c r="D38" t="inlineStr">
         <is>
-          <t>Anuv Jain</t>
+          <t>Alka Yagnik, Arijit Singh</t>
         </is>
       </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>2026-03-31</t>
+          <t>2026-04-01</t>
         </is>
       </c>
       <c r="B39" t="n">
@@ -11599,19 +12636,19 @@
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>Ishq Jalakar - Karvaan</t>
+          <t>Tere Bina</t>
         </is>
       </c>
       <c r="D39" t="inlineStr">
         <is>
-          <t>Shashwat Sachdev, Shahzad Ali, Subhadeep Das Chowdhury, Armaan Khan, Irshad Kamil, Roshan, Sahir Ludhianvi</t>
+          <t>A.R. Rahman, Chinmayi, Murtuza Khan, Qadir Khan</t>
         </is>
       </c>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>2026-03-31</t>
+          <t>2026-04-01</t>
         </is>
       </c>
       <c r="B40" t="n">
@@ -11619,19 +12656,19 @@
       </c>
       <c r="C40" t="inlineStr">
         <is>
-          <t>Haseen</t>
+          <t>Barbaad (From "Saiyaara")</t>
         </is>
       </c>
       <c r="D40" t="inlineStr">
         <is>
-          <t>Talwiinder, NDS, Rippy Grewal</t>
+          <t>The Rish, Jubin Nautiyal</t>
         </is>
       </c>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>2026-03-31</t>
+          <t>2026-04-01</t>
         </is>
       </c>
       <c r="B41" t="n">
@@ -11639,19 +12676,19 @@
       </c>
       <c r="C41" t="inlineStr">
         <is>
-          <t>Ye Tune Kya Kiya</t>
+          <t>Ishq Jalakar - Karvaan</t>
         </is>
       </c>
       <c r="D41" t="inlineStr">
         <is>
-          <t>Pritam, Javed Bashir, Rajat Arora</t>
+          <t>Shashwat Sachdev, Shahzad Ali, Subhadeep Das Chowdhury, Armaan Khan, Irshad Kamil, Roshan, Sahir Ludhianvi</t>
         </is>
       </c>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>2026-03-31</t>
+          <t>2026-04-01</t>
         </is>
       </c>
       <c r="B42" t="n">
@@ -11659,19 +12696,19 @@
       </c>
       <c r="C42" t="inlineStr">
         <is>
-          <t>Barbaad (From "Saiyaara")</t>
+          <t>Ye Tune Kya Kiya</t>
         </is>
       </c>
       <c r="D42" t="inlineStr">
         <is>
-          <t>The Rish, Jubin Nautiyal</t>
+          <t>Pritam, Javed Bashir, Rajat Arora</t>
         </is>
       </c>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>2026-03-31</t>
+          <t>2026-04-01</t>
         </is>
       </c>
       <c r="B43" t="n">
@@ -11679,19 +12716,19 @@
       </c>
       <c r="C43" t="inlineStr">
         <is>
-          <t>Mutta Kalakki (From "Youth")</t>
+          <t>Aaya Sher (From "The Paradise") (Telugu)</t>
         </is>
       </c>
       <c r="D43" t="inlineStr">
         <is>
-          <t>G. V. Prakash, Ken Karunaas</t>
+          <t>Anirudh Ravichander, Jangi Reddy, Arjun Chandy, Kasarla Shyam</t>
         </is>
       </c>
     </row>
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>2026-03-31</t>
+          <t>2026-04-01</t>
         </is>
       </c>
       <c r="B44" t="n">
@@ -11699,19 +12736,19 @@
       </c>
       <c r="C44" t="inlineStr">
         <is>
-          <t>Vaari Jaavan</t>
+          <t>Teri Deewani</t>
         </is>
       </c>
       <c r="D44" t="inlineStr">
         <is>
-          <t>Shashwat Sachdev, Jyoti Nooran, Jasmine Sandlas, Reble</t>
+          <t>Kailash Kher, Paresh Kamath, Naresh Kamath</t>
         </is>
       </c>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>2026-03-31</t>
+          <t>2026-04-01</t>
         </is>
       </c>
       <c r="B45" t="n">
@@ -11719,19 +12756,19 @@
       </c>
       <c r="C45" t="inlineStr">
         <is>
-          <t>Jogi</t>
+          <t>Mast Magan (From "2 States)</t>
         </is>
       </c>
       <c r="D45" t="inlineStr">
         <is>
-          <t>thiarajxtt, Bir</t>
+          <t>Arijit Singh, Chinmayi</t>
         </is>
       </c>
     </row>
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>2026-03-31</t>
+          <t>2026-04-01</t>
         </is>
       </c>
       <c r="B46" t="n">
@@ -11739,19 +12776,19 @@
       </c>
       <c r="C46" t="inlineStr">
         <is>
-          <t>Aaya Sher (From "The Paradise") (Telugu)</t>
+          <t>Vaari Jaavan</t>
         </is>
       </c>
       <c r="D46" t="inlineStr">
         <is>
-          <t>Anirudh Ravichander, Jangi Reddy, Arjun Chandy, Kasarla Shyam</t>
+          <t>Shashwat Sachdev, Jyoti Nooran, Jasmine Sandlas, Reble</t>
         </is>
       </c>
     </row>
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>2026-03-31</t>
+          <t>2026-04-01</t>
         </is>
       </c>
       <c r="B47" t="n">
@@ -11771,7 +12808,7 @@
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>2026-03-31</t>
+          <t>2026-04-01</t>
         </is>
       </c>
       <c r="B48" t="n">
@@ -11779,19 +12816,19 @@
       </c>
       <c r="C48" t="inlineStr">
         <is>
-          <t>SWIM</t>
+          <t>Mann Mera - Original Version</t>
         </is>
       </c>
       <c r="D48" t="inlineStr">
         <is>
-          <t>BTS</t>
+          <t>Gajendra Verma</t>
         </is>
       </c>
     </row>
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>2026-03-31</t>
+          <t>2026-04-01</t>
         </is>
       </c>
       <c r="B49" t="n">
@@ -11811,7 +12848,7 @@
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>2026-03-31</t>
+          <t>2026-04-01</t>
         </is>
       </c>
       <c r="B50" t="n">
@@ -11819,19 +12856,19 @@
       </c>
       <c r="C50" t="inlineStr">
         <is>
-          <t>Teri Deewani</t>
+          <t>Not Guilty</t>
         </is>
       </c>
       <c r="D50" t="inlineStr">
         <is>
-          <t>Kailash Kher, Paresh Kamath, Naresh Kamath</t>
+          <t>Dhanda Nyoliwala</t>
         </is>
       </c>
     </row>
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>2026-03-31</t>
+          <t>2026-04-01</t>
         </is>
       </c>
       <c r="B51" t="n">
@@ -11839,12 +12876,12 @@
       </c>
       <c r="C51" t="inlineStr">
         <is>
-          <t>Mast Magan (From "2 States)</t>
+          <t>Jogi</t>
         </is>
       </c>
       <c r="D51" t="inlineStr">
         <is>
-          <t>Arijit Singh, Chinmayi</t>
+          <t>thiarajxtt, Bir</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
added data for 2nd got predictions for 3rd april
</commit_message>
<xml_diff>
--- a/Probability Project.xlsx
+++ b/Probability Project.xlsx
@@ -22,6 +22,7 @@
     <sheet name="AUTO_20260329" sheetId="17" state="visible" r:id="rId17"/>
     <sheet name="AUTO_20260331" sheetId="18" state="visible" r:id="rId18"/>
     <sheet name="AUTO_20260401" sheetId="19" state="visible" r:id="rId19"/>
+    <sheet name="AUTO_20260402" sheetId="20" state="visible" r:id="rId20"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -11886,1000 +11887,1000 @@
       </c>
     </row>
     <row r="2">
-      <c r="A2" t="inlineStr">
+      <c r="A2" s="0" t="inlineStr">
         <is>
           <t>2026-04-01</t>
         </is>
       </c>
-      <c r="B2" t="n">
+      <c r="B2" s="0" t="n">
         <v>1</v>
       </c>
-      <c r="C2" t="inlineStr">
+      <c r="C2" s="0" t="inlineStr">
         <is>
           <t>Bairan</t>
         </is>
       </c>
-      <c r="D2" t="inlineStr">
+      <c r="D2" s="0" t="inlineStr">
         <is>
           <t>Banjaare</t>
         </is>
       </c>
     </row>
     <row r="3">
-      <c r="A3" t="inlineStr">
+      <c r="A3" s="0" t="inlineStr">
         <is>
           <t>2026-04-01</t>
         </is>
       </c>
-      <c r="B3" t="n">
+      <c r="B3" s="0" t="n">
         <v>2</v>
       </c>
-      <c r="C3" t="inlineStr">
+      <c r="C3" s="0" t="inlineStr">
         <is>
           <t>Jaiye Sajana</t>
         </is>
       </c>
-      <c r="D3" t="inlineStr">
+      <c r="D3" s="0" t="inlineStr">
         <is>
           <t>Shashwat Sachdev, Jasmine Sandlas, Satinder Sartaaj</t>
         </is>
       </c>
     </row>
     <row r="4">
-      <c r="A4" t="inlineStr">
+      <c r="A4" s="0" t="inlineStr">
         <is>
           <t>2026-04-01</t>
         </is>
       </c>
-      <c r="B4" t="n">
+      <c r="B4" s="0" t="n">
         <v>3</v>
       </c>
-      <c r="C4" t="inlineStr">
+      <c r="C4" s="0" t="inlineStr">
         <is>
           <t>Sheesha - Aakhya Mai Aakh Ghali Jo Bairan</t>
         </is>
       </c>
-      <c r="D4" t="inlineStr">
+      <c r="D4" s="0" t="inlineStr">
         <is>
           <t>Mitta Ror, Swara Verma</t>
         </is>
       </c>
     </row>
     <row r="5">
-      <c r="A5" t="inlineStr">
+      <c r="A5" s="0" t="inlineStr">
         <is>
           <t>2026-04-01</t>
         </is>
       </c>
-      <c r="B5" t="n">
+      <c r="B5" s="0" t="n">
         <v>4</v>
       </c>
-      <c r="C5" t="inlineStr">
+      <c r="C5" s="0" t="inlineStr">
         <is>
           <t>Gehra Hua</t>
         </is>
       </c>
-      <c r="D5" t="inlineStr">
+      <c r="D5" s="0" t="inlineStr">
         <is>
           <t>Shashwat Sachdev, Arijit Singh, Irshad Kamil, Armaan Khan</t>
         </is>
       </c>
     </row>
     <row r="6">
-      <c r="A6" t="inlineStr">
+      <c r="A6" s="0" t="inlineStr">
         <is>
           <t>2026-04-01</t>
         </is>
       </c>
-      <c r="B6" t="n">
+      <c r="B6" s="0" t="n">
         <v>5</v>
       </c>
-      <c r="C6" t="inlineStr">
+      <c r="C6" s="0" t="inlineStr">
         <is>
           <t>Khat</t>
         </is>
       </c>
-      <c r="D6" t="inlineStr">
+      <c r="D6" s="0" t="inlineStr">
         <is>
           <t>Navjot Ahuja</t>
         </is>
       </c>
     </row>
     <row r="7">
-      <c r="A7" t="inlineStr">
+      <c r="A7" s="0" t="inlineStr">
         <is>
           <t>2026-04-01</t>
         </is>
       </c>
-      <c r="B7" t="n">
+      <c r="B7" s="0" t="n">
         <v>6</v>
       </c>
-      <c r="C7" t="inlineStr">
+      <c r="C7" s="0" t="inlineStr">
         <is>
           <t>Dhurandhar The Revenge - Aari Aari</t>
         </is>
       </c>
-      <c r="D7" t="inlineStr">
+      <c r="D7" s="0" t="inlineStr">
         <is>
           <t>Shashwat Sachdev, Bombay Rockers, Irshad Kamil, Khan Saab, Reble, Token, Jasmine Sandlas, Sudhir Yaduvanshi</t>
         </is>
       </c>
     </row>
     <row r="8">
-      <c r="A8" t="inlineStr">
+      <c r="A8" s="0" t="inlineStr">
         <is>
           <t>2026-04-01</t>
         </is>
       </c>
-      <c r="B8" t="n">
+      <c r="B8" s="0" t="n">
         <v>7</v>
       </c>
-      <c r="C8" t="inlineStr">
+      <c r="C8" s="0" t="inlineStr">
         <is>
           <t>Jaan Se Guzarte Hain</t>
         </is>
       </c>
-      <c r="D8" t="inlineStr">
+      <c r="D8" s="0" t="inlineStr">
         <is>
           <t>Shashwat Sachdev, Khan Saab, Nusrat Fateh Ali Khan</t>
         </is>
       </c>
     </row>
     <row r="9">
-      <c r="A9" t="inlineStr">
+      <c r="A9" s="0" t="inlineStr">
         <is>
           <t>2026-04-01</t>
         </is>
       </c>
-      <c r="B9" t="n">
+      <c r="B9" s="0" t="n">
         <v>8</v>
       </c>
-      <c r="C9" t="inlineStr">
+      <c r="C9" s="0" t="inlineStr">
         <is>
           <t>Dooron Dooron</t>
         </is>
       </c>
-      <c r="D9" t="inlineStr">
+      <c r="D9" s="0" t="inlineStr">
         <is>
           <t>Paresh Pahuja, Shiv Tandan, Meghdeep Bose</t>
         </is>
       </c>
     </row>
     <row r="10">
-      <c r="A10" t="inlineStr">
+      <c r="A10" s="0" t="inlineStr">
         <is>
           <t>2026-04-01</t>
         </is>
       </c>
-      <c r="B10" t="n">
+      <c r="B10" s="0" t="n">
         <v>9</v>
       </c>
-      <c r="C10" t="inlineStr">
+      <c r="C10" s="0" t="inlineStr">
         <is>
           <t>Sitaare (From "Ikkis")</t>
         </is>
       </c>
-      <c r="D10" t="inlineStr">
+      <c r="D10" s="0" t="inlineStr">
         <is>
           <t>Arijit Singh, White Noise Collectives, Amitabh Bhattacharya</t>
         </is>
       </c>
     </row>
     <row r="11">
-      <c r="A11" t="inlineStr">
+      <c r="A11" s="0" t="inlineStr">
         <is>
           <t>2026-04-01</t>
         </is>
       </c>
-      <c r="B11" t="n">
+      <c r="B11" s="0" t="n">
         <v>10</v>
       </c>
-      <c r="C11" t="inlineStr">
+      <c r="C11" s="0" t="inlineStr">
         <is>
           <t>Sahiba</t>
         </is>
       </c>
-      <c r="D11" t="inlineStr">
+      <c r="D11" s="0" t="inlineStr">
         <is>
           <t>Aditya Rikhari</t>
         </is>
       </c>
     </row>
     <row r="12">
-      <c r="A12" t="inlineStr">
+      <c r="A12" s="0" t="inlineStr">
         <is>
           <t>2026-04-01</t>
         </is>
       </c>
-      <c r="B12" t="n">
+      <c r="B12" s="0" t="n">
         <v>11</v>
       </c>
-      <c r="C12" t="inlineStr">
+      <c r="C12" s="0" t="inlineStr">
         <is>
           <t>Apna Bana Le</t>
         </is>
       </c>
-      <c r="D12" t="inlineStr">
+      <c r="D12" s="0" t="inlineStr">
         <is>
           <t>Sachin-Jigar, Arijit Singh, Amitabh Bhattacharya</t>
         </is>
       </c>
     </row>
     <row r="13">
-      <c r="A13" t="inlineStr">
+      <c r="A13" s="0" t="inlineStr">
         <is>
           <t>2026-04-01</t>
         </is>
       </c>
-      <c r="B13" t="n">
+      <c r="B13" s="0" t="n">
         <v>12</v>
       </c>
-      <c r="C13" t="inlineStr">
+      <c r="C13" s="0" t="inlineStr">
         <is>
           <t>Pavazha Malli - From "Think Indie"</t>
         </is>
       </c>
-      <c r="D13" t="inlineStr">
+      <c r="D13" s="0" t="inlineStr">
         <is>
           <t>Sai Abhyankkar, Shruti Haasan, Vivek</t>
         </is>
       </c>
     </row>
     <row r="14">
-      <c r="A14" t="inlineStr">
+      <c r="A14" s="0" t="inlineStr">
         <is>
           <t>2026-04-01</t>
         </is>
       </c>
-      <c r="B14" t="n">
+      <c r="B14" s="0" t="n">
         <v>13</v>
       </c>
-      <c r="C14" t="inlineStr">
+      <c r="C14" s="0" t="inlineStr">
         <is>
           <t>Samjhawan</t>
         </is>
       </c>
-      <c r="D14" t="inlineStr">
+      <c r="D14" s="0" t="inlineStr">
         <is>
           <t>Jawad Ahmad, Shaarib Toshi, Arijit Singh, Shreya Ghoshal</t>
         </is>
       </c>
     </row>
     <row r="15">
-      <c r="A15" t="inlineStr">
+      <c r="A15" s="0" t="inlineStr">
         <is>
           <t>2026-04-01</t>
         </is>
       </c>
-      <c r="B15" t="n">
+      <c r="B15" s="0" t="n">
         <v>14</v>
       </c>
-      <c r="C15" t="inlineStr">
+      <c r="C15" s="0" t="inlineStr">
         <is>
           <t>Finding Her</t>
         </is>
       </c>
-      <c r="D15" t="inlineStr">
+      <c r="D15" s="0" t="inlineStr">
         <is>
           <t>Kushagra, Bharath, Saaheal</t>
         </is>
       </c>
     </row>
     <row r="16">
-      <c r="A16" t="inlineStr">
+      <c r="A16" s="0" t="inlineStr">
         <is>
           <t>2026-04-01</t>
         </is>
       </c>
-      <c r="B16" t="n">
+      <c r="B16" s="0" t="n">
         <v>15</v>
       </c>
-      <c r="C16" t="inlineStr">
+      <c r="C16" s="0" t="inlineStr">
         <is>
           <t>Shararat</t>
         </is>
       </c>
-      <c r="D16" t="inlineStr">
+      <c r="D16" s="0" t="inlineStr">
         <is>
           <t>Shashwat Sachdev, Madhubanti Bagchi, Jasmine Sandlas</t>
         </is>
       </c>
     </row>
     <row r="17">
-      <c r="A17" t="inlineStr">
+      <c r="A17" s="0" t="inlineStr">
         <is>
           <t>2026-04-01</t>
         </is>
       </c>
-      <c r="B17" t="n">
+      <c r="B17" s="0" t="n">
         <v>16</v>
       </c>
-      <c r="C17" t="inlineStr">
+      <c r="C17" s="0" t="inlineStr">
         <is>
           <t>Arz Kiya Hai | Coke Studio Bharat</t>
         </is>
       </c>
-      <c r="D17" t="inlineStr">
+      <c r="D17" s="0" t="inlineStr">
         <is>
           <t>Anuv Jain</t>
         </is>
       </c>
     </row>
     <row r="18">
-      <c r="A18" t="inlineStr">
+      <c r="A18" s="0" t="inlineStr">
         <is>
           <t>2026-04-01</t>
         </is>
       </c>
-      <c r="B18" t="n">
+      <c r="B18" s="0" t="n">
         <v>17</v>
       </c>
-      <c r="C18" t="inlineStr">
+      <c r="C18" s="0" t="inlineStr">
         <is>
           <t>Dhurandhar - Title Track</t>
         </is>
       </c>
-      <c r="D18" t="inlineStr">
+      <c r="D18" s="0" t="inlineStr">
         <is>
           <t>Shashwat Sachdev, Hanumankind, Jasmine Sandlas, Sudhir Yaduvanshi, Charanjit Ahuja, Muhammad Sadiq, Ranjit Kaur, Babu Singh Maan</t>
         </is>
       </c>
     </row>
     <row r="19">
-      <c r="A19" t="inlineStr">
+      <c r="A19" s="0" t="inlineStr">
         <is>
           <t>2026-04-01</t>
         </is>
       </c>
-      <c r="B19" t="n">
+      <c r="B19" s="0" t="n">
         <v>18</v>
       </c>
-      <c r="C19" t="inlineStr">
+      <c r="C19" s="0" t="inlineStr">
         <is>
           <t>Boyfriend</t>
         </is>
       </c>
-      <c r="D19" t="inlineStr">
+      <c r="D19" s="0" t="inlineStr">
         <is>
           <t>Karan Aujla, Ikky</t>
         </is>
       </c>
     </row>
     <row r="20">
-      <c r="A20" t="inlineStr">
+      <c r="A20" s="0" t="inlineStr">
         <is>
           <t>2026-04-01</t>
         </is>
       </c>
-      <c r="B20" t="n">
+      <c r="B20" s="0" t="n">
         <v>19</v>
       </c>
-      <c r="C20" t="inlineStr">
+      <c r="C20" s="0" t="inlineStr">
         <is>
           <t>Ishq</t>
         </is>
       </c>
-      <c r="D20" t="inlineStr">
+      <c r="D20" s="0" t="inlineStr">
         <is>
           <t>Faheem Abdullah, Rauhan Malik, Amir Ameer</t>
         </is>
       </c>
     </row>
     <row r="21">
-      <c r="A21" t="inlineStr">
+      <c r="A21" s="0" t="inlineStr">
         <is>
           <t>2026-04-01</t>
         </is>
       </c>
-      <c r="B21" t="n">
+      <c r="B21" s="0" t="n">
         <v>20</v>
       </c>
-      <c r="C21" t="inlineStr">
+      <c r="C21" s="0" t="inlineStr">
         <is>
           <t>Phir Se</t>
         </is>
       </c>
-      <c r="D21" t="inlineStr">
+      <c r="D21" s="0" t="inlineStr">
         <is>
           <t>Shashwat Sachdev, Arijit Singh, Irshad Kamil</t>
         </is>
       </c>
     </row>
     <row r="22">
-      <c r="A22" t="inlineStr">
+      <c r="A22" s="0" t="inlineStr">
         <is>
           <t>2026-04-01</t>
         </is>
       </c>
-      <c r="B22" t="n">
+      <c r="B22" s="0" t="n">
         <v>21</v>
       </c>
-      <c r="C22" t="inlineStr">
+      <c r="C22" s="0" t="inlineStr">
         <is>
           <t>Mann Mera</t>
         </is>
       </c>
-      <c r="D22" t="inlineStr">
+      <c r="D22" s="0" t="inlineStr">
         <is>
           <t>Gajendra Verma</t>
         </is>
       </c>
     </row>
     <row r="23">
-      <c r="A23" t="inlineStr">
+      <c r="A23" s="0" t="inlineStr">
         <is>
           <t>2026-04-01</t>
         </is>
       </c>
-      <c r="B23" t="n">
+      <c r="B23" s="0" t="n">
         <v>22</v>
       </c>
-      <c r="C23" t="inlineStr">
+      <c r="C23" s="0" t="inlineStr">
         <is>
           <t>Bairi</t>
         </is>
       </c>
-      <c r="D23" t="inlineStr">
+      <c r="D23" s="0" t="inlineStr">
         <is>
           <t>Virat, Pradeep Solanki, Heena</t>
         </is>
       </c>
     </row>
     <row r="24">
-      <c r="A24" t="inlineStr">
+      <c r="A24" s="0" t="inlineStr">
         <is>
           <t>2026-04-01</t>
         </is>
       </c>
-      <c r="B24" t="n">
+      <c r="B24" s="0" t="n">
         <v>23</v>
       </c>
-      <c r="C24" t="inlineStr">
+      <c r="C24" s="0" t="inlineStr">
         <is>
           <t>Naal Nachna</t>
         </is>
       </c>
-      <c r="D24" t="inlineStr">
+      <c r="D24" s="0" t="inlineStr">
         <is>
           <t>Shashwat Sachdev, Afsana Khan, Irshad Kamil, Reble</t>
         </is>
       </c>
     </row>
     <row r="25">
-      <c r="A25" t="inlineStr">
+      <c r="A25" s="0" t="inlineStr">
         <is>
           <t>2026-04-01</t>
         </is>
       </c>
-      <c r="B25" t="n">
+      <c r="B25" s="0" t="n">
         <v>24</v>
       </c>
-      <c r="C25" t="inlineStr">
+      <c r="C25" s="0" t="inlineStr">
         <is>
           <t>Saiyaara</t>
         </is>
       </c>
-      <c r="D25" t="inlineStr">
+      <c r="D25" s="0" t="inlineStr">
         <is>
           <t>Tanishk Bagchi, Faheem Abdullah, Arslan Nizami, Irshad Kamil</t>
         </is>
       </c>
     </row>
     <row r="26">
-      <c r="A26" t="inlineStr">
+      <c r="A26" s="0" t="inlineStr">
         <is>
           <t>2026-04-01</t>
         </is>
       </c>
-      <c r="B26" t="n">
+      <c r="B26" s="0" t="n">
         <v>25</v>
       </c>
-      <c r="C26" t="inlineStr">
+      <c r="C26" s="0" t="inlineStr">
         <is>
           <t>For A Reason</t>
         </is>
       </c>
-      <c r="D26" t="inlineStr">
+      <c r="D26" s="0" t="inlineStr">
         <is>
           <t>Karan Aujla, Ikky</t>
         </is>
       </c>
     </row>
     <row r="27">
-      <c r="A27" t="inlineStr">
+      <c r="A27" s="0" t="inlineStr">
         <is>
           <t>2026-04-01</t>
         </is>
       </c>
-      <c r="B27" t="n">
+      <c r="B27" s="0" t="n">
         <v>26</v>
       </c>
-      <c r="C27" t="inlineStr">
+      <c r="C27" s="0" t="inlineStr">
         <is>
           <t>Run Down The City - Monica</t>
         </is>
       </c>
-      <c r="D27" t="inlineStr">
+      <c r="D27" s="0" t="inlineStr">
         <is>
           <t>Shashwat Sachdev, Reble, Asha Bhosle, R. D. Burman, Majrooh Sultanpuri</t>
         </is>
       </c>
     </row>
     <row r="28">
-      <c r="A28" t="inlineStr">
+      <c r="A28" s="0" t="inlineStr">
         <is>
           <t>2026-04-01</t>
         </is>
       </c>
-      <c r="B28" t="n">
+      <c r="B28" s="0" t="n">
         <v>27</v>
       </c>
-      <c r="C28" t="inlineStr">
+      <c r="C28" s="0" t="inlineStr">
         <is>
           <t>Darkhaast</t>
         </is>
       </c>
-      <c r="D28" t="inlineStr">
+      <c r="D28" s="0" t="inlineStr">
         <is>
           <t>Mithoon, Arijit Singh, Sunidhi Chauhan, Sayeed Quadri</t>
         </is>
       </c>
     </row>
     <row r="29">
-      <c r="A29" t="inlineStr">
+      <c r="A29" s="0" t="inlineStr">
         <is>
           <t>2026-04-01</t>
         </is>
       </c>
-      <c r="B29" t="n">
+      <c r="B29" s="0" t="n">
         <v>28</v>
       </c>
-      <c r="C29" t="inlineStr">
+      <c r="C29" s="0" t="inlineStr">
         <is>
           <t>Ishqa Ve</t>
         </is>
       </c>
-      <c r="D29" t="inlineStr">
+      <c r="D29" s="0" t="inlineStr">
         <is>
           <t>Zeeshan Ali, Yuvraj Tung, Sandeep Aulakh, Honey Dhillon</t>
         </is>
       </c>
     </row>
     <row r="30">
-      <c r="A30" t="inlineStr">
+      <c r="A30" s="0" t="inlineStr">
         <is>
           <t>2026-04-01</t>
         </is>
       </c>
-      <c r="B30" t="n">
+      <c r="B30" s="0" t="n">
         <v>29</v>
       </c>
-      <c r="C30" t="inlineStr">
+      <c r="C30" s="0" t="inlineStr">
         <is>
           <t>Tum Ho Toh (From "Saiyaara")</t>
         </is>
       </c>
-      <c r="D30" t="inlineStr">
+      <c r="D30" s="0" t="inlineStr">
         <is>
           <t>Vishal Mishra, Hansika Pareek, Raj Shekhar</t>
         </is>
       </c>
     </row>
     <row r="31">
-      <c r="A31" t="inlineStr">
+      <c r="A31" s="0" t="inlineStr">
         <is>
           <t>2026-04-01</t>
         </is>
       </c>
-      <c r="B31" t="n">
+      <c r="B31" s="0" t="n">
         <v>30</v>
       </c>
-      <c r="C31" t="inlineStr">
+      <c r="C31" s="0" t="inlineStr">
         <is>
           <t>Deewaana Deewaana</t>
         </is>
       </c>
-      <c r="D31" t="inlineStr">
+      <c r="D31" s="0" t="inlineStr">
         <is>
           <t>A.R. Rahman, Irshad Kamil</t>
         </is>
       </c>
     </row>
     <row r="32">
-      <c r="A32" t="inlineStr">
+      <c r="A32" s="0" t="inlineStr">
         <is>
           <t>2026-04-01</t>
         </is>
       </c>
-      <c r="B32" t="n">
+      <c r="B32" s="0" t="n">
         <v>31</v>
       </c>
-      <c r="C32" t="inlineStr">
+      <c r="C32" s="0" t="inlineStr">
         <is>
           <t>Tere Liye</t>
         </is>
       </c>
-      <c r="D32" t="inlineStr">
+      <c r="D32" s="0" t="inlineStr">
         <is>
           <t>Atif Aslam, Shreya Ghoshal, Sachin Gupta, Sameer Anjaan</t>
         </is>
       </c>
     </row>
     <row r="33">
-      <c r="A33" t="inlineStr">
+      <c r="A33" s="0" t="inlineStr">
         <is>
           <t>2026-04-01</t>
         </is>
       </c>
-      <c r="B33" t="n">
+      <c r="B33" s="0" t="n">
         <v>32</v>
       </c>
-      <c r="C33" t="inlineStr">
+      <c r="C33" s="0" t="inlineStr">
         <is>
           <t>Lutt Le Gaya</t>
         </is>
       </c>
-      <c r="D33" t="inlineStr">
+      <c r="D33" s="0" t="inlineStr">
         <is>
           <t>Shashwat Sachdev, Simran Choudhary</t>
         </is>
       </c>
     </row>
     <row r="34">
-      <c r="A34" t="inlineStr">
+      <c r="A34" s="0" t="inlineStr">
         <is>
           <t>2026-04-01</t>
         </is>
       </c>
-      <c r="B34" t="n">
+      <c r="B34" s="0" t="n">
         <v>33</v>
       </c>
-      <c r="C34" t="inlineStr">
+      <c r="C34" s="0" t="inlineStr">
         <is>
           <t>Raanjhan (From "Do Patti")</t>
         </is>
       </c>
-      <c r="D34" t="inlineStr">
+      <c r="D34" s="0" t="inlineStr">
         <is>
           <t>Sachet-Parampara, Parampara Tandon, Kausar Munir</t>
         </is>
       </c>
     </row>
     <row r="35">
-      <c r="A35" t="inlineStr">
+      <c r="A35" s="0" t="inlineStr">
         <is>
           <t>2026-04-01</t>
         </is>
       </c>
-      <c r="B35" t="n">
+      <c r="B35" s="0" t="n">
         <v>34</v>
       </c>
-      <c r="C35" t="inlineStr">
+      <c r="C35" s="0" t="inlineStr">
         <is>
           <t>Main Aur Tu</t>
         </is>
       </c>
-      <c r="D35" t="inlineStr">
+      <c r="D35" s="0" t="inlineStr">
         <is>
           <t>Shashwat Sachdev, Jasmine Sandlas, Reble</t>
         </is>
       </c>
     </row>
     <row r="36">
-      <c r="A36" t="inlineStr">
+      <c r="A36" s="0" t="inlineStr">
         <is>
           <t>2026-04-01</t>
         </is>
       </c>
-      <c r="B36" t="n">
+      <c r="B36" s="0" t="n">
         <v>35</v>
       </c>
-      <c r="C36" t="inlineStr">
+      <c r="C36" s="0" t="inlineStr">
         <is>
           <t>Haseen</t>
         </is>
       </c>
-      <c r="D36" t="inlineStr">
+      <c r="D36" s="0" t="inlineStr">
         <is>
           <t>Talwiinder, NDS, Rippy Grewal</t>
         </is>
       </c>
     </row>
     <row r="37">
-      <c r="A37" t="inlineStr">
+      <c r="A37" s="0" t="inlineStr">
         <is>
           <t>2026-04-01</t>
         </is>
       </c>
-      <c r="B37" t="n">
+      <c r="B37" s="0" t="n">
         <v>36</v>
       </c>
-      <c r="C37" t="inlineStr">
+      <c r="C37" s="0" t="inlineStr">
         <is>
           <t>Jo Tum Mere Ho</t>
         </is>
       </c>
-      <c r="D37" t="inlineStr">
+      <c r="D37" s="0" t="inlineStr">
         <is>
           <t>Anuv Jain</t>
         </is>
       </c>
     </row>
     <row r="38">
-      <c r="A38" t="inlineStr">
+      <c r="A38" s="0" t="inlineStr">
         <is>
           <t>2026-04-01</t>
         </is>
       </c>
-      <c r="B38" t="n">
+      <c r="B38" s="0" t="n">
         <v>37</v>
       </c>
-      <c r="C38" t="inlineStr">
+      <c r="C38" s="0" t="inlineStr">
         <is>
           <t>Agar Tum Saath Ho (From "Tamasha")</t>
         </is>
       </c>
-      <c r="D38" t="inlineStr">
+      <c r="D38" s="0" t="inlineStr">
         <is>
           <t>Alka Yagnik, Arijit Singh</t>
         </is>
       </c>
     </row>
     <row r="39">
-      <c r="A39" t="inlineStr">
+      <c r="A39" s="0" t="inlineStr">
         <is>
           <t>2026-04-01</t>
         </is>
       </c>
-      <c r="B39" t="n">
+      <c r="B39" s="0" t="n">
         <v>38</v>
       </c>
-      <c r="C39" t="inlineStr">
+      <c r="C39" s="0" t="inlineStr">
         <is>
           <t>Tere Bina</t>
         </is>
       </c>
-      <c r="D39" t="inlineStr">
+      <c r="D39" s="0" t="inlineStr">
         <is>
           <t>A.R. Rahman, Chinmayi, Murtuza Khan, Qadir Khan</t>
         </is>
       </c>
     </row>
     <row r="40">
-      <c r="A40" t="inlineStr">
+      <c r="A40" s="0" t="inlineStr">
         <is>
           <t>2026-04-01</t>
         </is>
       </c>
-      <c r="B40" t="n">
+      <c r="B40" s="0" t="n">
         <v>39</v>
       </c>
-      <c r="C40" t="inlineStr">
+      <c r="C40" s="0" t="inlineStr">
         <is>
           <t>Barbaad (From "Saiyaara")</t>
         </is>
       </c>
-      <c r="D40" t="inlineStr">
+      <c r="D40" s="0" t="inlineStr">
         <is>
           <t>The Rish, Jubin Nautiyal</t>
         </is>
       </c>
     </row>
     <row r="41">
-      <c r="A41" t="inlineStr">
+      <c r="A41" s="0" t="inlineStr">
         <is>
           <t>2026-04-01</t>
         </is>
       </c>
-      <c r="B41" t="n">
+      <c r="B41" s="0" t="n">
         <v>40</v>
       </c>
-      <c r="C41" t="inlineStr">
+      <c r="C41" s="0" t="inlineStr">
         <is>
           <t>Ishq Jalakar - Karvaan</t>
         </is>
       </c>
-      <c r="D41" t="inlineStr">
+      <c r="D41" s="0" t="inlineStr">
         <is>
           <t>Shashwat Sachdev, Shahzad Ali, Subhadeep Das Chowdhury, Armaan Khan, Irshad Kamil, Roshan, Sahir Ludhianvi</t>
         </is>
       </c>
     </row>
     <row r="42">
-      <c r="A42" t="inlineStr">
+      <c r="A42" s="0" t="inlineStr">
         <is>
           <t>2026-04-01</t>
         </is>
       </c>
-      <c r="B42" t="n">
+      <c r="B42" s="0" t="n">
         <v>41</v>
       </c>
-      <c r="C42" t="inlineStr">
+      <c r="C42" s="0" t="inlineStr">
         <is>
           <t>Ye Tune Kya Kiya</t>
         </is>
       </c>
-      <c r="D42" t="inlineStr">
+      <c r="D42" s="0" t="inlineStr">
         <is>
           <t>Pritam, Javed Bashir, Rajat Arora</t>
         </is>
       </c>
     </row>
     <row r="43">
-      <c r="A43" t="inlineStr">
+      <c r="A43" s="0" t="inlineStr">
         <is>
           <t>2026-04-01</t>
         </is>
       </c>
-      <c r="B43" t="n">
+      <c r="B43" s="0" t="n">
         <v>42</v>
       </c>
-      <c r="C43" t="inlineStr">
+      <c r="C43" s="0" t="inlineStr">
         <is>
           <t>Aaya Sher (From "The Paradise") (Telugu)</t>
         </is>
       </c>
-      <c r="D43" t="inlineStr">
+      <c r="D43" s="0" t="inlineStr">
         <is>
           <t>Anirudh Ravichander, Jangi Reddy, Arjun Chandy, Kasarla Shyam</t>
         </is>
       </c>
     </row>
     <row r="44">
-      <c r="A44" t="inlineStr">
+      <c r="A44" s="0" t="inlineStr">
         <is>
           <t>2026-04-01</t>
         </is>
       </c>
-      <c r="B44" t="n">
+      <c r="B44" s="0" t="n">
         <v>43</v>
       </c>
-      <c r="C44" t="inlineStr">
+      <c r="C44" s="0" t="inlineStr">
         <is>
           <t>Teri Deewani</t>
         </is>
       </c>
-      <c r="D44" t="inlineStr">
+      <c r="D44" s="0" t="inlineStr">
         <is>
           <t>Kailash Kher, Paresh Kamath, Naresh Kamath</t>
         </is>
       </c>
     </row>
     <row r="45">
-      <c r="A45" t="inlineStr">
+      <c r="A45" s="0" t="inlineStr">
         <is>
           <t>2026-04-01</t>
         </is>
       </c>
-      <c r="B45" t="n">
+      <c r="B45" s="0" t="n">
         <v>44</v>
       </c>
-      <c r="C45" t="inlineStr">
+      <c r="C45" s="0" t="inlineStr">
         <is>
           <t>Mast Magan (From "2 States)</t>
         </is>
       </c>
-      <c r="D45" t="inlineStr">
+      <c r="D45" s="0" t="inlineStr">
         <is>
           <t>Arijit Singh, Chinmayi</t>
         </is>
       </c>
     </row>
     <row r="46">
-      <c r="A46" t="inlineStr">
+      <c r="A46" s="0" t="inlineStr">
         <is>
           <t>2026-04-01</t>
         </is>
       </c>
-      <c r="B46" t="n">
+      <c r="B46" s="0" t="n">
         <v>45</v>
       </c>
-      <c r="C46" t="inlineStr">
+      <c r="C46" s="0" t="inlineStr">
         <is>
           <t>Vaari Jaavan</t>
         </is>
       </c>
-      <c r="D46" t="inlineStr">
+      <c r="D46" s="0" t="inlineStr">
         <is>
           <t>Shashwat Sachdev, Jyoti Nooran, Jasmine Sandlas, Reble</t>
         </is>
       </c>
     </row>
     <row r="47">
-      <c r="A47" t="inlineStr">
+      <c r="A47" s="0" t="inlineStr">
         <is>
           <t>2026-04-01</t>
         </is>
       </c>
-      <c r="B47" t="n">
+      <c r="B47" s="0" t="n">
         <v>46</v>
       </c>
-      <c r="C47" t="inlineStr">
+      <c r="C47" s="0" t="inlineStr">
         <is>
           <t>Ehsaas</t>
         </is>
       </c>
-      <c r="D47" t="inlineStr">
+      <c r="D47" s="0" t="inlineStr">
         <is>
           <t>Faheem Abdullah, Duha Shah, Vaibhav Pani, Hyder Dar</t>
         </is>
       </c>
     </row>
     <row r="48">
-      <c r="A48" t="inlineStr">
+      <c r="A48" s="0" t="inlineStr">
         <is>
           <t>2026-04-01</t>
         </is>
       </c>
-      <c r="B48" t="n">
+      <c r="B48" s="0" t="n">
         <v>47</v>
       </c>
-      <c r="C48" t="inlineStr">
+      <c r="C48" s="0" t="inlineStr">
         <is>
           <t>Mann Mera - Original Version</t>
         </is>
       </c>
-      <c r="D48" t="inlineStr">
+      <c r="D48" s="0" t="inlineStr">
         <is>
           <t>Gajendra Verma</t>
         </is>
       </c>
     </row>
     <row r="49">
-      <c r="A49" t="inlineStr">
+      <c r="A49" s="0" t="inlineStr">
         <is>
           <t>2026-04-01</t>
         </is>
       </c>
-      <c r="B49" t="n">
+      <c r="B49" s="0" t="n">
         <v>48</v>
       </c>
-      <c r="C49" t="inlineStr">
+      <c r="C49" s="0" t="inlineStr">
         <is>
           <t>Hum Pyaar Karne Wale</t>
         </is>
       </c>
-      <c r="D49" t="inlineStr">
+      <c r="D49" s="0" t="inlineStr">
         <is>
           <t>Shashwat Sachdev, Anuradha Paudwal, Udit Narayan, Anand-Milind, Sameer Anjaan, Qveen Herby</t>
         </is>
       </c>
     </row>
     <row r="50">
-      <c r="A50" t="inlineStr">
+      <c r="A50" s="0" t="inlineStr">
         <is>
           <t>2026-04-01</t>
         </is>
       </c>
-      <c r="B50" t="n">
+      <c r="B50" s="0" t="n">
         <v>49</v>
       </c>
-      <c r="C50" t="inlineStr">
+      <c r="C50" s="0" t="inlineStr">
         <is>
           <t>Not Guilty</t>
         </is>
       </c>
-      <c r="D50" t="inlineStr">
+      <c r="D50" s="0" t="inlineStr">
         <is>
           <t>Dhanda Nyoliwala</t>
         </is>
       </c>
     </row>
     <row r="51">
-      <c r="A51" t="inlineStr">
+      <c r="A51" s="0" t="inlineStr">
         <is>
           <t>2026-04-01</t>
         </is>
       </c>
-      <c r="B51" t="n">
+      <c r="B51" s="0" t="n">
         <v>50</v>
       </c>
-      <c r="C51" t="inlineStr">
+      <c r="C51" s="0" t="inlineStr">
         <is>
           <t>Jogi</t>
         </is>
       </c>
-      <c r="D51" t="inlineStr">
+      <c r="D51" s="0" t="inlineStr">
         <is>
           <t>thiarajxtt, Bir</t>
         </is>
@@ -13926,6 +13927,1042 @@
 </worksheet>
 </file>
 
+<file path=xl/worksheets/sheet20.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:D51"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="24" t="inlineStr">
+        <is>
+          <t>Date</t>
+        </is>
+      </c>
+      <c r="B1" s="24" t="inlineStr">
+        <is>
+          <t>Rank</t>
+        </is>
+      </c>
+      <c r="C1" s="24" t="inlineStr">
+        <is>
+          <t>Song</t>
+        </is>
+      </c>
+      <c r="D1" s="24" t="inlineStr">
+        <is>
+          <t>Artist</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>2026-04-02</t>
+        </is>
+      </c>
+      <c r="B2" t="n">
+        <v>1</v>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>Bairan</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>Banjaare</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>2026-04-02</t>
+        </is>
+      </c>
+      <c r="B3" t="n">
+        <v>2</v>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>Jaiye Sajana</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>Shashwat Sachdev, Jasmine Sandlas, Satinder Sartaaj</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>2026-04-02</t>
+        </is>
+      </c>
+      <c r="B4" t="n">
+        <v>3</v>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>Sheesha - Aakhya Mai Aakh Ghali Jo Bairan</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>Mitta Ror, Swara Verma</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>2026-04-02</t>
+        </is>
+      </c>
+      <c r="B5" t="n">
+        <v>4</v>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>Gehra Hua</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>Shashwat Sachdev, Arijit Singh, Irshad Kamil, Armaan Khan</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>2026-04-02</t>
+        </is>
+      </c>
+      <c r="B6" t="n">
+        <v>5</v>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>Khat</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>Navjot Ahuja</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>2026-04-02</t>
+        </is>
+      </c>
+      <c r="B7" t="n">
+        <v>6</v>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>Dhurandhar The Revenge - Aari Aari</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>Shashwat Sachdev, Bombay Rockers, Irshad Kamil, Khan Saab, Reble, Token, Jasmine Sandlas, Sudhir Yaduvanshi</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>2026-04-02</t>
+        </is>
+      </c>
+      <c r="B8" t="n">
+        <v>7</v>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>Jaan Se Guzarte Hain</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>Shashwat Sachdev, Khan Saab, Nusrat Fateh Ali Khan</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>2026-04-02</t>
+        </is>
+      </c>
+      <c r="B9" t="n">
+        <v>8</v>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>Sitaare (From "Ikkis")</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>Arijit Singh, White Noise Collectives, Amitabh Bhattacharya</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>2026-04-02</t>
+        </is>
+      </c>
+      <c r="B10" t="n">
+        <v>9</v>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>Dooron Dooron</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>Paresh Pahuja, Shiv Tandan, Meghdeep Bose</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>2026-04-02</t>
+        </is>
+      </c>
+      <c r="B11" t="n">
+        <v>10</v>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>Sahiba</t>
+        </is>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>Aditya Rikhari</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>2026-04-02</t>
+        </is>
+      </c>
+      <c r="B12" t="n">
+        <v>11</v>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>Pavazha Malli - From "Think Indie"</t>
+        </is>
+      </c>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>Sai Abhyankkar, Shruti Haasan, Vivek</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>2026-04-02</t>
+        </is>
+      </c>
+      <c r="B13" t="n">
+        <v>12</v>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>Apna Bana Le</t>
+        </is>
+      </c>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t>Sachin-Jigar, Arijit Singh, Amitabh Bhattacharya</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>2026-04-02</t>
+        </is>
+      </c>
+      <c r="B14" t="n">
+        <v>13</v>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>Shree Hanuman Chalisa</t>
+        </is>
+      </c>
+      <c r="D14" t="inlineStr">
+        <is>
+          <t>Hariharan, Lalit Sen, Chander</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>2026-04-02</t>
+        </is>
+      </c>
+      <c r="B15" t="n">
+        <v>14</v>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>Samjhawan</t>
+        </is>
+      </c>
+      <c r="D15" t="inlineStr">
+        <is>
+          <t>Jawad Ahmad, Shaarib Toshi, Arijit Singh, Shreya Ghoshal</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>2026-04-02</t>
+        </is>
+      </c>
+      <c r="B16" t="n">
+        <v>15</v>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>Finding Her</t>
+        </is>
+      </c>
+      <c r="D16" t="inlineStr">
+        <is>
+          <t>Kushagra, Bharath, Saaheal</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>2026-04-02</t>
+        </is>
+      </c>
+      <c r="B17" t="n">
+        <v>16</v>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>Shararat</t>
+        </is>
+      </c>
+      <c r="D17" t="inlineStr">
+        <is>
+          <t>Shashwat Sachdev, Madhubanti Bagchi, Jasmine Sandlas</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>2026-04-02</t>
+        </is>
+      </c>
+      <c r="B18" t="n">
+        <v>17</v>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>Arz Kiya Hai | Coke Studio Bharat</t>
+        </is>
+      </c>
+      <c r="D18" t="inlineStr">
+        <is>
+          <t>Anuv Jain</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>2026-04-02</t>
+        </is>
+      </c>
+      <c r="B19" t="n">
+        <v>18</v>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>Dhurandhar - Title Track</t>
+        </is>
+      </c>
+      <c r="D19" t="inlineStr">
+        <is>
+          <t>Shashwat Sachdev, Hanumankind, Jasmine Sandlas, Sudhir Yaduvanshi, Charanjit Ahuja, Muhammad Sadiq, Ranjit Kaur, Babu Singh Maan</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>2026-04-02</t>
+        </is>
+      </c>
+      <c r="B20" t="n">
+        <v>19</v>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>Ishq</t>
+        </is>
+      </c>
+      <c r="D20" t="inlineStr">
+        <is>
+          <t>Faheem Abdullah, Rauhan Malik, Amir Ameer</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>2026-04-02</t>
+        </is>
+      </c>
+      <c r="B21" t="n">
+        <v>20</v>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>Boyfriend</t>
+        </is>
+      </c>
+      <c r="D21" t="inlineStr">
+        <is>
+          <t>Karan Aujla, Ikky</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>2026-04-02</t>
+        </is>
+      </c>
+      <c r="B22" t="n">
+        <v>21</v>
+      </c>
+      <c r="C22" t="inlineStr">
+        <is>
+          <t>Phir Se</t>
+        </is>
+      </c>
+      <c r="D22" t="inlineStr">
+        <is>
+          <t>Shashwat Sachdev, Arijit Singh, Irshad Kamil</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>2026-04-02</t>
+        </is>
+      </c>
+      <c r="B23" t="n">
+        <v>22</v>
+      </c>
+      <c r="C23" t="inlineStr">
+        <is>
+          <t>Mann Mera</t>
+        </is>
+      </c>
+      <c r="D23" t="inlineStr">
+        <is>
+          <t>Gajendra Verma</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>2026-04-02</t>
+        </is>
+      </c>
+      <c r="B24" t="n">
+        <v>23</v>
+      </c>
+      <c r="C24" t="inlineStr">
+        <is>
+          <t>Saiyaara</t>
+        </is>
+      </c>
+      <c r="D24" t="inlineStr">
+        <is>
+          <t>Tanishk Bagchi, Faheem Abdullah, Arslan Nizami, Irshad Kamil</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>2026-04-02</t>
+        </is>
+      </c>
+      <c r="B25" t="n">
+        <v>24</v>
+      </c>
+      <c r="C25" t="inlineStr">
+        <is>
+          <t>Ishqa Ve</t>
+        </is>
+      </c>
+      <c r="D25" t="inlineStr">
+        <is>
+          <t>Zeeshan Ali, Yuvraj Tung, Sandeep Aulakh, Honey Dhillon</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>2026-04-02</t>
+        </is>
+      </c>
+      <c r="B26" t="n">
+        <v>25</v>
+      </c>
+      <c r="C26" t="inlineStr">
+        <is>
+          <t>Bairi</t>
+        </is>
+      </c>
+      <c r="D26" t="inlineStr">
+        <is>
+          <t>Virat, Pradeep Solanki, Heena</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>2026-04-02</t>
+        </is>
+      </c>
+      <c r="B27" t="n">
+        <v>26</v>
+      </c>
+      <c r="C27" t="inlineStr">
+        <is>
+          <t>For A Reason</t>
+        </is>
+      </c>
+      <c r="D27" t="inlineStr">
+        <is>
+          <t>Karan Aujla, Ikky</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>2026-04-02</t>
+        </is>
+      </c>
+      <c r="B28" t="n">
+        <v>27</v>
+      </c>
+      <c r="C28" t="inlineStr">
+        <is>
+          <t>Naal Nachna</t>
+        </is>
+      </c>
+      <c r="D28" t="inlineStr">
+        <is>
+          <t>Shashwat Sachdev, Afsana Khan, Irshad Kamil, Reble</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>2026-04-02</t>
+        </is>
+      </c>
+      <c r="B29" t="n">
+        <v>28</v>
+      </c>
+      <c r="C29" t="inlineStr">
+        <is>
+          <t>Deewaana Deewaana</t>
+        </is>
+      </c>
+      <c r="D29" t="inlineStr">
+        <is>
+          <t>A.R. Rahman, Irshad Kamil</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>2026-04-02</t>
+        </is>
+      </c>
+      <c r="B30" t="n">
+        <v>29</v>
+      </c>
+      <c r="C30" t="inlineStr">
+        <is>
+          <t>Run Down The City - Monica</t>
+        </is>
+      </c>
+      <c r="D30" t="inlineStr">
+        <is>
+          <t>Shashwat Sachdev, Reble, Asha Bhosle, R. D. Burman, Majrooh Sultanpuri</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>2026-04-02</t>
+        </is>
+      </c>
+      <c r="B31" t="n">
+        <v>30</v>
+      </c>
+      <c r="C31" t="inlineStr">
+        <is>
+          <t>Darkhaast</t>
+        </is>
+      </c>
+      <c r="D31" t="inlineStr">
+        <is>
+          <t>Mithoon, Arijit Singh, Sunidhi Chauhan, Sayeed Quadri</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="inlineStr">
+        <is>
+          <t>2026-04-02</t>
+        </is>
+      </c>
+      <c r="B32" t="n">
+        <v>31</v>
+      </c>
+      <c r="C32" t="inlineStr">
+        <is>
+          <t>Tum Ho Toh (From "Saiyaara")</t>
+        </is>
+      </c>
+      <c r="D32" t="inlineStr">
+        <is>
+          <t>Vishal Mishra, Hansika Pareek, Raj Shekhar</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="inlineStr">
+        <is>
+          <t>2026-04-02</t>
+        </is>
+      </c>
+      <c r="B33" t="n">
+        <v>32</v>
+      </c>
+      <c r="C33" t="inlineStr">
+        <is>
+          <t>Tere Liye</t>
+        </is>
+      </c>
+      <c r="D33" t="inlineStr">
+        <is>
+          <t>Atif Aslam, Shreya Ghoshal, Sachin Gupta, Sameer Anjaan</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="inlineStr">
+        <is>
+          <t>2026-04-02</t>
+        </is>
+      </c>
+      <c r="B34" t="n">
+        <v>33</v>
+      </c>
+      <c r="C34" t="inlineStr">
+        <is>
+          <t>Raanjhan (From "Do Patti")</t>
+        </is>
+      </c>
+      <c r="D34" t="inlineStr">
+        <is>
+          <t>Sachet-Parampara, Parampara Tandon, Kausar Munir</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="inlineStr">
+        <is>
+          <t>2026-04-02</t>
+        </is>
+      </c>
+      <c r="B35" t="n">
+        <v>34</v>
+      </c>
+      <c r="C35" t="inlineStr">
+        <is>
+          <t>Tere Bina</t>
+        </is>
+      </c>
+      <c r="D35" t="inlineStr">
+        <is>
+          <t>A.R. Rahman, Chinmayi, Murtuza Khan, Qadir Khan</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="inlineStr">
+        <is>
+          <t>2026-04-02</t>
+        </is>
+      </c>
+      <c r="B36" t="n">
+        <v>35</v>
+      </c>
+      <c r="C36" t="inlineStr">
+        <is>
+          <t>Lutt Le Gaya</t>
+        </is>
+      </c>
+      <c r="D36" t="inlineStr">
+        <is>
+          <t>Shashwat Sachdev, Simran Choudhary</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="inlineStr">
+        <is>
+          <t>2026-04-02</t>
+        </is>
+      </c>
+      <c r="B37" t="n">
+        <v>36</v>
+      </c>
+      <c r="C37" t="inlineStr">
+        <is>
+          <t>Agar Tum Saath Ho (From "Tamasha")</t>
+        </is>
+      </c>
+      <c r="D37" t="inlineStr">
+        <is>
+          <t>Alka Yagnik, Arijit Singh</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="inlineStr">
+        <is>
+          <t>2026-04-02</t>
+        </is>
+      </c>
+      <c r="B38" t="n">
+        <v>37</v>
+      </c>
+      <c r="C38" t="inlineStr">
+        <is>
+          <t>Jo Tum Mere Ho</t>
+        </is>
+      </c>
+      <c r="D38" t="inlineStr">
+        <is>
+          <t>Anuv Jain</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="inlineStr">
+        <is>
+          <t>2026-04-02</t>
+        </is>
+      </c>
+      <c r="B39" t="n">
+        <v>38</v>
+      </c>
+      <c r="C39" t="inlineStr">
+        <is>
+          <t>Haseen</t>
+        </is>
+      </c>
+      <c r="D39" t="inlineStr">
+        <is>
+          <t>Talwiinder, NDS, Rippy Grewal</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" t="inlineStr">
+        <is>
+          <t>2026-04-02</t>
+        </is>
+      </c>
+      <c r="B40" t="n">
+        <v>39</v>
+      </c>
+      <c r="C40" t="inlineStr">
+        <is>
+          <t>Barbaad (From "Saiyaara")</t>
+        </is>
+      </c>
+      <c r="D40" t="inlineStr">
+        <is>
+          <t>The Rish, Jubin Nautiyal</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" t="inlineStr">
+        <is>
+          <t>2026-04-02</t>
+        </is>
+      </c>
+      <c r="B41" t="n">
+        <v>40</v>
+      </c>
+      <c r="C41" t="inlineStr">
+        <is>
+          <t>Main Aur Tu</t>
+        </is>
+      </c>
+      <c r="D41" t="inlineStr">
+        <is>
+          <t>Shashwat Sachdev, Jasmine Sandlas, Reble</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" t="inlineStr">
+        <is>
+          <t>2026-04-02</t>
+        </is>
+      </c>
+      <c r="B42" t="n">
+        <v>41</v>
+      </c>
+      <c r="C42" t="inlineStr">
+        <is>
+          <t>Ishq Jalakar - Karvaan</t>
+        </is>
+      </c>
+      <c r="D42" t="inlineStr">
+        <is>
+          <t>Shashwat Sachdev, Shahzad Ali, Subhadeep Das Chowdhury, Armaan Khan, Irshad Kamil, Roshan, Sahir Ludhianvi</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" t="inlineStr">
+        <is>
+          <t>2026-04-02</t>
+        </is>
+      </c>
+      <c r="B43" t="n">
+        <v>42</v>
+      </c>
+      <c r="C43" t="inlineStr">
+        <is>
+          <t>Teri Deewani</t>
+        </is>
+      </c>
+      <c r="D43" t="inlineStr">
+        <is>
+          <t>Kailash Kher, Paresh Kamath, Naresh Kamath</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" t="inlineStr">
+        <is>
+          <t>2026-04-02</t>
+        </is>
+      </c>
+      <c r="B44" t="n">
+        <v>43</v>
+      </c>
+      <c r="C44" t="inlineStr">
+        <is>
+          <t>Ye Tune Kya Kiya</t>
+        </is>
+      </c>
+      <c r="D44" t="inlineStr">
+        <is>
+          <t>Pritam, Javed Bashir, Rajat Arora</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" t="inlineStr">
+        <is>
+          <t>2026-04-02</t>
+        </is>
+      </c>
+      <c r="B45" t="n">
+        <v>44</v>
+      </c>
+      <c r="C45" t="inlineStr">
+        <is>
+          <t>Mann Mera - Original Version</t>
+        </is>
+      </c>
+      <c r="D45" t="inlineStr">
+        <is>
+          <t>Gajendra Verma</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" t="inlineStr">
+        <is>
+          <t>2026-04-02</t>
+        </is>
+      </c>
+      <c r="B46" t="n">
+        <v>45</v>
+      </c>
+      <c r="C46" t="inlineStr">
+        <is>
+          <t>Aaya Sher (From "The Paradise") (Telugu)</t>
+        </is>
+      </c>
+      <c r="D46" t="inlineStr">
+        <is>
+          <t>Anirudh Ravichander, Jangi Reddy, Arjun Chandy, Kasarla Shyam</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" t="inlineStr">
+        <is>
+          <t>2026-04-02</t>
+        </is>
+      </c>
+      <c r="B47" t="n">
+        <v>46</v>
+      </c>
+      <c r="C47" t="inlineStr">
+        <is>
+          <t>Not Guilty</t>
+        </is>
+      </c>
+      <c r="D47" t="inlineStr">
+        <is>
+          <t>Dhanda Nyoliwala</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" t="inlineStr">
+        <is>
+          <t>2026-04-02</t>
+        </is>
+      </c>
+      <c r="B48" t="n">
+        <v>47</v>
+      </c>
+      <c r="C48" t="inlineStr">
+        <is>
+          <t>Mutta Kalakki (From "Youth")</t>
+        </is>
+      </c>
+      <c r="D48" t="inlineStr">
+        <is>
+          <t>G. V. Prakash, Ken Karunaas</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" t="inlineStr">
+        <is>
+          <t>2026-04-02</t>
+        </is>
+      </c>
+      <c r="B49" t="n">
+        <v>48</v>
+      </c>
+      <c r="C49" t="inlineStr">
+        <is>
+          <t>Vaari Jaavan</t>
+        </is>
+      </c>
+      <c r="D49" t="inlineStr">
+        <is>
+          <t>Shashwat Sachdev, Jyoti Nooran, Jasmine Sandlas, Reble</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" t="inlineStr">
+        <is>
+          <t>2026-04-02</t>
+        </is>
+      </c>
+      <c r="B50" t="n">
+        <v>49</v>
+      </c>
+      <c r="C50" t="inlineStr">
+        <is>
+          <t>Hum Pyaar Karne Wale</t>
+        </is>
+      </c>
+      <c r="D50" t="inlineStr">
+        <is>
+          <t>Shashwat Sachdev, Anuradha Paudwal, Udit Narayan, Anand-Milind, Sameer Anjaan, Qveen Herby</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" t="inlineStr">
+        <is>
+          <t>2026-04-02</t>
+        </is>
+      </c>
+      <c r="B51" t="n">
+        <v>50</v>
+      </c>
+      <c r="C51" t="inlineStr">
+        <is>
+          <t>Ehsaas</t>
+        </is>
+      </c>
+      <c r="D51" t="inlineStr">
+        <is>
+          <t>Faheem Abdullah, Duha Shah, Vaibhav Pani, Hyder Dar</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>

</xml_diff>

<commit_message>
added data for 3rd got predictions for 4th april
</commit_message>
<xml_diff>
--- a/Probability Project.xlsx
+++ b/Probability Project.xlsx
@@ -23,6 +23,7 @@
     <sheet name="AUTO_20260331" sheetId="18" state="visible" r:id="rId18"/>
     <sheet name="AUTO_20260401" sheetId="19" state="visible" r:id="rId19"/>
     <sheet name="AUTO_20260402" sheetId="20" state="visible" r:id="rId20"/>
+    <sheet name="AUTO_20260403" sheetId="21" state="visible" r:id="rId21"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -13959,9 +13960,1045 @@
       </c>
     </row>
     <row r="2">
+      <c r="A2" s="0" t="inlineStr">
+        <is>
+          <t>2026-04-02</t>
+        </is>
+      </c>
+      <c r="B2" s="0" t="n">
+        <v>1</v>
+      </c>
+      <c r="C2" s="0" t="inlineStr">
+        <is>
+          <t>Bairan</t>
+        </is>
+      </c>
+      <c r="D2" s="0" t="inlineStr">
+        <is>
+          <t>Banjaare</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="0" t="inlineStr">
+        <is>
+          <t>2026-04-02</t>
+        </is>
+      </c>
+      <c r="B3" s="0" t="n">
+        <v>2</v>
+      </c>
+      <c r="C3" s="0" t="inlineStr">
+        <is>
+          <t>Jaiye Sajana</t>
+        </is>
+      </c>
+      <c r="D3" s="0" t="inlineStr">
+        <is>
+          <t>Shashwat Sachdev, Jasmine Sandlas, Satinder Sartaaj</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="0" t="inlineStr">
+        <is>
+          <t>2026-04-02</t>
+        </is>
+      </c>
+      <c r="B4" s="0" t="n">
+        <v>3</v>
+      </c>
+      <c r="C4" s="0" t="inlineStr">
+        <is>
+          <t>Sheesha - Aakhya Mai Aakh Ghali Jo Bairan</t>
+        </is>
+      </c>
+      <c r="D4" s="0" t="inlineStr">
+        <is>
+          <t>Mitta Ror, Swara Verma</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="0" t="inlineStr">
+        <is>
+          <t>2026-04-02</t>
+        </is>
+      </c>
+      <c r="B5" s="0" t="n">
+        <v>4</v>
+      </c>
+      <c r="C5" s="0" t="inlineStr">
+        <is>
+          <t>Gehra Hua</t>
+        </is>
+      </c>
+      <c r="D5" s="0" t="inlineStr">
+        <is>
+          <t>Shashwat Sachdev, Arijit Singh, Irshad Kamil, Armaan Khan</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="0" t="inlineStr">
+        <is>
+          <t>2026-04-02</t>
+        </is>
+      </c>
+      <c r="B6" s="0" t="n">
+        <v>5</v>
+      </c>
+      <c r="C6" s="0" t="inlineStr">
+        <is>
+          <t>Khat</t>
+        </is>
+      </c>
+      <c r="D6" s="0" t="inlineStr">
+        <is>
+          <t>Navjot Ahuja</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="0" t="inlineStr">
+        <is>
+          <t>2026-04-02</t>
+        </is>
+      </c>
+      <c r="B7" s="0" t="n">
+        <v>6</v>
+      </c>
+      <c r="C7" s="0" t="inlineStr">
+        <is>
+          <t>Dhurandhar The Revenge - Aari Aari</t>
+        </is>
+      </c>
+      <c r="D7" s="0" t="inlineStr">
+        <is>
+          <t>Shashwat Sachdev, Bombay Rockers, Irshad Kamil, Khan Saab, Reble, Token, Jasmine Sandlas, Sudhir Yaduvanshi</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="0" t="inlineStr">
+        <is>
+          <t>2026-04-02</t>
+        </is>
+      </c>
+      <c r="B8" s="0" t="n">
+        <v>7</v>
+      </c>
+      <c r="C8" s="0" t="inlineStr">
+        <is>
+          <t>Jaan Se Guzarte Hain</t>
+        </is>
+      </c>
+      <c r="D8" s="0" t="inlineStr">
+        <is>
+          <t>Shashwat Sachdev, Khan Saab, Nusrat Fateh Ali Khan</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="0" t="inlineStr">
+        <is>
+          <t>2026-04-02</t>
+        </is>
+      </c>
+      <c r="B9" s="0" t="n">
+        <v>8</v>
+      </c>
+      <c r="C9" s="0" t="inlineStr">
+        <is>
+          <t>Sitaare (From "Ikkis")</t>
+        </is>
+      </c>
+      <c r="D9" s="0" t="inlineStr">
+        <is>
+          <t>Arijit Singh, White Noise Collectives, Amitabh Bhattacharya</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="0" t="inlineStr">
+        <is>
+          <t>2026-04-02</t>
+        </is>
+      </c>
+      <c r="B10" s="0" t="n">
+        <v>9</v>
+      </c>
+      <c r="C10" s="0" t="inlineStr">
+        <is>
+          <t>Dooron Dooron</t>
+        </is>
+      </c>
+      <c r="D10" s="0" t="inlineStr">
+        <is>
+          <t>Paresh Pahuja, Shiv Tandan, Meghdeep Bose</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="0" t="inlineStr">
+        <is>
+          <t>2026-04-02</t>
+        </is>
+      </c>
+      <c r="B11" s="0" t="n">
+        <v>10</v>
+      </c>
+      <c r="C11" s="0" t="inlineStr">
+        <is>
+          <t>Sahiba</t>
+        </is>
+      </c>
+      <c r="D11" s="0" t="inlineStr">
+        <is>
+          <t>Aditya Rikhari</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="0" t="inlineStr">
+        <is>
+          <t>2026-04-02</t>
+        </is>
+      </c>
+      <c r="B12" s="0" t="n">
+        <v>11</v>
+      </c>
+      <c r="C12" s="0" t="inlineStr">
+        <is>
+          <t>Pavazha Malli - From "Think Indie"</t>
+        </is>
+      </c>
+      <c r="D12" s="0" t="inlineStr">
+        <is>
+          <t>Sai Abhyankkar, Shruti Haasan, Vivek</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="0" t="inlineStr">
+        <is>
+          <t>2026-04-02</t>
+        </is>
+      </c>
+      <c r="B13" s="0" t="n">
+        <v>12</v>
+      </c>
+      <c r="C13" s="0" t="inlineStr">
+        <is>
+          <t>Apna Bana Le</t>
+        </is>
+      </c>
+      <c r="D13" s="0" t="inlineStr">
+        <is>
+          <t>Sachin-Jigar, Arijit Singh, Amitabh Bhattacharya</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="0" t="inlineStr">
+        <is>
+          <t>2026-04-02</t>
+        </is>
+      </c>
+      <c r="B14" s="0" t="n">
+        <v>13</v>
+      </c>
+      <c r="C14" s="0" t="inlineStr">
+        <is>
+          <t>Shree Hanuman Chalisa</t>
+        </is>
+      </c>
+      <c r="D14" s="0" t="inlineStr">
+        <is>
+          <t>Hariharan, Lalit Sen, Chander</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="0" t="inlineStr">
+        <is>
+          <t>2026-04-02</t>
+        </is>
+      </c>
+      <c r="B15" s="0" t="n">
+        <v>14</v>
+      </c>
+      <c r="C15" s="0" t="inlineStr">
+        <is>
+          <t>Samjhawan</t>
+        </is>
+      </c>
+      <c r="D15" s="0" t="inlineStr">
+        <is>
+          <t>Jawad Ahmad, Shaarib Toshi, Arijit Singh, Shreya Ghoshal</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="0" t="inlineStr">
+        <is>
+          <t>2026-04-02</t>
+        </is>
+      </c>
+      <c r="B16" s="0" t="n">
+        <v>15</v>
+      </c>
+      <c r="C16" s="0" t="inlineStr">
+        <is>
+          <t>Finding Her</t>
+        </is>
+      </c>
+      <c r="D16" s="0" t="inlineStr">
+        <is>
+          <t>Kushagra, Bharath, Saaheal</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="0" t="inlineStr">
+        <is>
+          <t>2026-04-02</t>
+        </is>
+      </c>
+      <c r="B17" s="0" t="n">
+        <v>16</v>
+      </c>
+      <c r="C17" s="0" t="inlineStr">
+        <is>
+          <t>Shararat</t>
+        </is>
+      </c>
+      <c r="D17" s="0" t="inlineStr">
+        <is>
+          <t>Shashwat Sachdev, Madhubanti Bagchi, Jasmine Sandlas</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="0" t="inlineStr">
+        <is>
+          <t>2026-04-02</t>
+        </is>
+      </c>
+      <c r="B18" s="0" t="n">
+        <v>17</v>
+      </c>
+      <c r="C18" s="0" t="inlineStr">
+        <is>
+          <t>Arz Kiya Hai | Coke Studio Bharat</t>
+        </is>
+      </c>
+      <c r="D18" s="0" t="inlineStr">
+        <is>
+          <t>Anuv Jain</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="0" t="inlineStr">
+        <is>
+          <t>2026-04-02</t>
+        </is>
+      </c>
+      <c r="B19" s="0" t="n">
+        <v>18</v>
+      </c>
+      <c r="C19" s="0" t="inlineStr">
+        <is>
+          <t>Dhurandhar - Title Track</t>
+        </is>
+      </c>
+      <c r="D19" s="0" t="inlineStr">
+        <is>
+          <t>Shashwat Sachdev, Hanumankind, Jasmine Sandlas, Sudhir Yaduvanshi, Charanjit Ahuja, Muhammad Sadiq, Ranjit Kaur, Babu Singh Maan</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="0" t="inlineStr">
+        <is>
+          <t>2026-04-02</t>
+        </is>
+      </c>
+      <c r="B20" s="0" t="n">
+        <v>19</v>
+      </c>
+      <c r="C20" s="0" t="inlineStr">
+        <is>
+          <t>Ishq</t>
+        </is>
+      </c>
+      <c r="D20" s="0" t="inlineStr">
+        <is>
+          <t>Faheem Abdullah, Rauhan Malik, Amir Ameer</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="0" t="inlineStr">
+        <is>
+          <t>2026-04-02</t>
+        </is>
+      </c>
+      <c r="B21" s="0" t="n">
+        <v>20</v>
+      </c>
+      <c r="C21" s="0" t="inlineStr">
+        <is>
+          <t>Boyfriend</t>
+        </is>
+      </c>
+      <c r="D21" s="0" t="inlineStr">
+        <is>
+          <t>Karan Aujla, Ikky</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="0" t="inlineStr">
+        <is>
+          <t>2026-04-02</t>
+        </is>
+      </c>
+      <c r="B22" s="0" t="n">
+        <v>21</v>
+      </c>
+      <c r="C22" s="0" t="inlineStr">
+        <is>
+          <t>Phir Se</t>
+        </is>
+      </c>
+      <c r="D22" s="0" t="inlineStr">
+        <is>
+          <t>Shashwat Sachdev, Arijit Singh, Irshad Kamil</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="0" t="inlineStr">
+        <is>
+          <t>2026-04-02</t>
+        </is>
+      </c>
+      <c r="B23" s="0" t="n">
+        <v>22</v>
+      </c>
+      <c r="C23" s="0" t="inlineStr">
+        <is>
+          <t>Mann Mera</t>
+        </is>
+      </c>
+      <c r="D23" s="0" t="inlineStr">
+        <is>
+          <t>Gajendra Verma</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="0" t="inlineStr">
+        <is>
+          <t>2026-04-02</t>
+        </is>
+      </c>
+      <c r="B24" s="0" t="n">
+        <v>23</v>
+      </c>
+      <c r="C24" s="0" t="inlineStr">
+        <is>
+          <t>Saiyaara</t>
+        </is>
+      </c>
+      <c r="D24" s="0" t="inlineStr">
+        <is>
+          <t>Tanishk Bagchi, Faheem Abdullah, Arslan Nizami, Irshad Kamil</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="0" t="inlineStr">
+        <is>
+          <t>2026-04-02</t>
+        </is>
+      </c>
+      <c r="B25" s="0" t="n">
+        <v>24</v>
+      </c>
+      <c r="C25" s="0" t="inlineStr">
+        <is>
+          <t>Ishqa Ve</t>
+        </is>
+      </c>
+      <c r="D25" s="0" t="inlineStr">
+        <is>
+          <t>Zeeshan Ali, Yuvraj Tung, Sandeep Aulakh, Honey Dhillon</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="0" t="inlineStr">
+        <is>
+          <t>2026-04-02</t>
+        </is>
+      </c>
+      <c r="B26" s="0" t="n">
+        <v>25</v>
+      </c>
+      <c r="C26" s="0" t="inlineStr">
+        <is>
+          <t>Bairi</t>
+        </is>
+      </c>
+      <c r="D26" s="0" t="inlineStr">
+        <is>
+          <t>Virat, Pradeep Solanki, Heena</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="0" t="inlineStr">
+        <is>
+          <t>2026-04-02</t>
+        </is>
+      </c>
+      <c r="B27" s="0" t="n">
+        <v>26</v>
+      </c>
+      <c r="C27" s="0" t="inlineStr">
+        <is>
+          <t>For A Reason</t>
+        </is>
+      </c>
+      <c r="D27" s="0" t="inlineStr">
+        <is>
+          <t>Karan Aujla, Ikky</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="0" t="inlineStr">
+        <is>
+          <t>2026-04-02</t>
+        </is>
+      </c>
+      <c r="B28" s="0" t="n">
+        <v>27</v>
+      </c>
+      <c r="C28" s="0" t="inlineStr">
+        <is>
+          <t>Naal Nachna</t>
+        </is>
+      </c>
+      <c r="D28" s="0" t="inlineStr">
+        <is>
+          <t>Shashwat Sachdev, Afsana Khan, Irshad Kamil, Reble</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="0" t="inlineStr">
+        <is>
+          <t>2026-04-02</t>
+        </is>
+      </c>
+      <c r="B29" s="0" t="n">
+        <v>28</v>
+      </c>
+      <c r="C29" s="0" t="inlineStr">
+        <is>
+          <t>Deewaana Deewaana</t>
+        </is>
+      </c>
+      <c r="D29" s="0" t="inlineStr">
+        <is>
+          <t>A.R. Rahman, Irshad Kamil</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="0" t="inlineStr">
+        <is>
+          <t>2026-04-02</t>
+        </is>
+      </c>
+      <c r="B30" s="0" t="n">
+        <v>29</v>
+      </c>
+      <c r="C30" s="0" t="inlineStr">
+        <is>
+          <t>Run Down The City - Monica</t>
+        </is>
+      </c>
+      <c r="D30" s="0" t="inlineStr">
+        <is>
+          <t>Shashwat Sachdev, Reble, Asha Bhosle, R. D. Burman, Majrooh Sultanpuri</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="0" t="inlineStr">
+        <is>
+          <t>2026-04-02</t>
+        </is>
+      </c>
+      <c r="B31" s="0" t="n">
+        <v>30</v>
+      </c>
+      <c r="C31" s="0" t="inlineStr">
+        <is>
+          <t>Darkhaast</t>
+        </is>
+      </c>
+      <c r="D31" s="0" t="inlineStr">
+        <is>
+          <t>Mithoon, Arijit Singh, Sunidhi Chauhan, Sayeed Quadri</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="0" t="inlineStr">
+        <is>
+          <t>2026-04-02</t>
+        </is>
+      </c>
+      <c r="B32" s="0" t="n">
+        <v>31</v>
+      </c>
+      <c r="C32" s="0" t="inlineStr">
+        <is>
+          <t>Tum Ho Toh (From "Saiyaara")</t>
+        </is>
+      </c>
+      <c r="D32" s="0" t="inlineStr">
+        <is>
+          <t>Vishal Mishra, Hansika Pareek, Raj Shekhar</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="0" t="inlineStr">
+        <is>
+          <t>2026-04-02</t>
+        </is>
+      </c>
+      <c r="B33" s="0" t="n">
+        <v>32</v>
+      </c>
+      <c r="C33" s="0" t="inlineStr">
+        <is>
+          <t>Tere Liye</t>
+        </is>
+      </c>
+      <c r="D33" s="0" t="inlineStr">
+        <is>
+          <t>Atif Aslam, Shreya Ghoshal, Sachin Gupta, Sameer Anjaan</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="0" t="inlineStr">
+        <is>
+          <t>2026-04-02</t>
+        </is>
+      </c>
+      <c r="B34" s="0" t="n">
+        <v>33</v>
+      </c>
+      <c r="C34" s="0" t="inlineStr">
+        <is>
+          <t>Raanjhan (From "Do Patti")</t>
+        </is>
+      </c>
+      <c r="D34" s="0" t="inlineStr">
+        <is>
+          <t>Sachet-Parampara, Parampara Tandon, Kausar Munir</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="0" t="inlineStr">
+        <is>
+          <t>2026-04-02</t>
+        </is>
+      </c>
+      <c r="B35" s="0" t="n">
+        <v>34</v>
+      </c>
+      <c r="C35" s="0" t="inlineStr">
+        <is>
+          <t>Tere Bina</t>
+        </is>
+      </c>
+      <c r="D35" s="0" t="inlineStr">
+        <is>
+          <t>A.R. Rahman, Chinmayi, Murtuza Khan, Qadir Khan</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="0" t="inlineStr">
+        <is>
+          <t>2026-04-02</t>
+        </is>
+      </c>
+      <c r="B36" s="0" t="n">
+        <v>35</v>
+      </c>
+      <c r="C36" s="0" t="inlineStr">
+        <is>
+          <t>Lutt Le Gaya</t>
+        </is>
+      </c>
+      <c r="D36" s="0" t="inlineStr">
+        <is>
+          <t>Shashwat Sachdev, Simran Choudhary</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="0" t="inlineStr">
+        <is>
+          <t>2026-04-02</t>
+        </is>
+      </c>
+      <c r="B37" s="0" t="n">
+        <v>36</v>
+      </c>
+      <c r="C37" s="0" t="inlineStr">
+        <is>
+          <t>Agar Tum Saath Ho (From "Tamasha")</t>
+        </is>
+      </c>
+      <c r="D37" s="0" t="inlineStr">
+        <is>
+          <t>Alka Yagnik, Arijit Singh</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="0" t="inlineStr">
+        <is>
+          <t>2026-04-02</t>
+        </is>
+      </c>
+      <c r="B38" s="0" t="n">
+        <v>37</v>
+      </c>
+      <c r="C38" s="0" t="inlineStr">
+        <is>
+          <t>Jo Tum Mere Ho</t>
+        </is>
+      </c>
+      <c r="D38" s="0" t="inlineStr">
+        <is>
+          <t>Anuv Jain</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="0" t="inlineStr">
+        <is>
+          <t>2026-04-02</t>
+        </is>
+      </c>
+      <c r="B39" s="0" t="n">
+        <v>38</v>
+      </c>
+      <c r="C39" s="0" t="inlineStr">
+        <is>
+          <t>Haseen</t>
+        </is>
+      </c>
+      <c r="D39" s="0" t="inlineStr">
+        <is>
+          <t>Talwiinder, NDS, Rippy Grewal</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="0" t="inlineStr">
+        <is>
+          <t>2026-04-02</t>
+        </is>
+      </c>
+      <c r="B40" s="0" t="n">
+        <v>39</v>
+      </c>
+      <c r="C40" s="0" t="inlineStr">
+        <is>
+          <t>Barbaad (From "Saiyaara")</t>
+        </is>
+      </c>
+      <c r="D40" s="0" t="inlineStr">
+        <is>
+          <t>The Rish, Jubin Nautiyal</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" s="0" t="inlineStr">
+        <is>
+          <t>2026-04-02</t>
+        </is>
+      </c>
+      <c r="B41" s="0" t="n">
+        <v>40</v>
+      </c>
+      <c r="C41" s="0" t="inlineStr">
+        <is>
+          <t>Main Aur Tu</t>
+        </is>
+      </c>
+      <c r="D41" s="0" t="inlineStr">
+        <is>
+          <t>Shashwat Sachdev, Jasmine Sandlas, Reble</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" s="0" t="inlineStr">
+        <is>
+          <t>2026-04-02</t>
+        </is>
+      </c>
+      <c r="B42" s="0" t="n">
+        <v>41</v>
+      </c>
+      <c r="C42" s="0" t="inlineStr">
+        <is>
+          <t>Ishq Jalakar - Karvaan</t>
+        </is>
+      </c>
+      <c r="D42" s="0" t="inlineStr">
+        <is>
+          <t>Shashwat Sachdev, Shahzad Ali, Subhadeep Das Chowdhury, Armaan Khan, Irshad Kamil, Roshan, Sahir Ludhianvi</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" s="0" t="inlineStr">
+        <is>
+          <t>2026-04-02</t>
+        </is>
+      </c>
+      <c r="B43" s="0" t="n">
+        <v>42</v>
+      </c>
+      <c r="C43" s="0" t="inlineStr">
+        <is>
+          <t>Teri Deewani</t>
+        </is>
+      </c>
+      <c r="D43" s="0" t="inlineStr">
+        <is>
+          <t>Kailash Kher, Paresh Kamath, Naresh Kamath</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" s="0" t="inlineStr">
+        <is>
+          <t>2026-04-02</t>
+        </is>
+      </c>
+      <c r="B44" s="0" t="n">
+        <v>43</v>
+      </c>
+      <c r="C44" s="0" t="inlineStr">
+        <is>
+          <t>Ye Tune Kya Kiya</t>
+        </is>
+      </c>
+      <c r="D44" s="0" t="inlineStr">
+        <is>
+          <t>Pritam, Javed Bashir, Rajat Arora</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" s="0" t="inlineStr">
+        <is>
+          <t>2026-04-02</t>
+        </is>
+      </c>
+      <c r="B45" s="0" t="n">
+        <v>44</v>
+      </c>
+      <c r="C45" s="0" t="inlineStr">
+        <is>
+          <t>Mann Mera - Original Version</t>
+        </is>
+      </c>
+      <c r="D45" s="0" t="inlineStr">
+        <is>
+          <t>Gajendra Verma</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" s="0" t="inlineStr">
+        <is>
+          <t>2026-04-02</t>
+        </is>
+      </c>
+      <c r="B46" s="0" t="n">
+        <v>45</v>
+      </c>
+      <c r="C46" s="0" t="inlineStr">
+        <is>
+          <t>Aaya Sher (From "The Paradise") (Telugu)</t>
+        </is>
+      </c>
+      <c r="D46" s="0" t="inlineStr">
+        <is>
+          <t>Anirudh Ravichander, Jangi Reddy, Arjun Chandy, Kasarla Shyam</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" s="0" t="inlineStr">
+        <is>
+          <t>2026-04-02</t>
+        </is>
+      </c>
+      <c r="B47" s="0" t="n">
+        <v>46</v>
+      </c>
+      <c r="C47" s="0" t="inlineStr">
+        <is>
+          <t>Not Guilty</t>
+        </is>
+      </c>
+      <c r="D47" s="0" t="inlineStr">
+        <is>
+          <t>Dhanda Nyoliwala</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" s="0" t="inlineStr">
+        <is>
+          <t>2026-04-02</t>
+        </is>
+      </c>
+      <c r="B48" s="0" t="n">
+        <v>47</v>
+      </c>
+      <c r="C48" s="0" t="inlineStr">
+        <is>
+          <t>Mutta Kalakki (From "Youth")</t>
+        </is>
+      </c>
+      <c r="D48" s="0" t="inlineStr">
+        <is>
+          <t>G. V. Prakash, Ken Karunaas</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" s="0" t="inlineStr">
+        <is>
+          <t>2026-04-02</t>
+        </is>
+      </c>
+      <c r="B49" s="0" t="n">
+        <v>48</v>
+      </c>
+      <c r="C49" s="0" t="inlineStr">
+        <is>
+          <t>Vaari Jaavan</t>
+        </is>
+      </c>
+      <c r="D49" s="0" t="inlineStr">
+        <is>
+          <t>Shashwat Sachdev, Jyoti Nooran, Jasmine Sandlas, Reble</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" s="0" t="inlineStr">
+        <is>
+          <t>2026-04-02</t>
+        </is>
+      </c>
+      <c r="B50" s="0" t="n">
+        <v>49</v>
+      </c>
+      <c r="C50" s="0" t="inlineStr">
+        <is>
+          <t>Hum Pyaar Karne Wale</t>
+        </is>
+      </c>
+      <c r="D50" s="0" t="inlineStr">
+        <is>
+          <t>Shashwat Sachdev, Anuradha Paudwal, Udit Narayan, Anand-Milind, Sameer Anjaan, Qveen Herby</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" s="0" t="inlineStr">
+        <is>
+          <t>2026-04-02</t>
+        </is>
+      </c>
+      <c r="B51" s="0" t="n">
+        <v>50</v>
+      </c>
+      <c r="C51" s="0" t="inlineStr">
+        <is>
+          <t>Ehsaas</t>
+        </is>
+      </c>
+      <c r="D51" s="0" t="inlineStr">
+        <is>
+          <t>Faheem Abdullah, Duha Shah, Vaibhav Pani, Hyder Dar</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet21.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:D51"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="24" t="inlineStr">
+        <is>
+          <t>Date</t>
+        </is>
+      </c>
+      <c r="B1" s="24" t="inlineStr">
+        <is>
+          <t>Rank</t>
+        </is>
+      </c>
+      <c r="C1" s="24" t="inlineStr">
+        <is>
+          <t>Song</t>
+        </is>
+      </c>
+      <c r="D1" s="24" t="inlineStr">
+        <is>
+          <t>Artist</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>2026-04-02</t>
+          <t>2026-04-03</t>
         </is>
       </c>
       <c r="B2" t="n">
@@ -13981,7 +15018,7 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>2026-04-02</t>
+          <t>2026-04-03</t>
         </is>
       </c>
       <c r="B3" t="n">
@@ -14001,7 +15038,7 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>2026-04-02</t>
+          <t>2026-04-03</t>
         </is>
       </c>
       <c r="B4" t="n">
@@ -14009,19 +15046,19 @@
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>Sheesha - Aakhya Mai Aakh Ghali Jo Bairan</t>
+          <t>Gehra Hua</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>Mitta Ror, Swara Verma</t>
+          <t>Shashwat Sachdev, Arijit Singh, Irshad Kamil, Armaan Khan</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>2026-04-02</t>
+          <t>2026-04-03</t>
         </is>
       </c>
       <c r="B5" t="n">
@@ -14029,19 +15066,19 @@
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>Gehra Hua</t>
+          <t>Sheesha - Aakhya Mai Aakh Ghali Jo Bairan</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>Shashwat Sachdev, Arijit Singh, Irshad Kamil, Armaan Khan</t>
+          <t>Mitta Ror, Swara Verma</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>2026-04-02</t>
+          <t>2026-04-03</t>
         </is>
       </c>
       <c r="B6" t="n">
@@ -14061,7 +15098,7 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>2026-04-02</t>
+          <t>2026-04-03</t>
         </is>
       </c>
       <c r="B7" t="n">
@@ -14081,7 +15118,7 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>2026-04-02</t>
+          <t>2026-04-03</t>
         </is>
       </c>
       <c r="B8" t="n">
@@ -14089,19 +15126,19 @@
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>Jaan Se Guzarte Hain</t>
+          <t>Sahiba</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>Shashwat Sachdev, Khan Saab, Nusrat Fateh Ali Khan</t>
+          <t>Aditya Rikhari</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>2026-04-02</t>
+          <t>2026-04-03</t>
         </is>
       </c>
       <c r="B9" t="n">
@@ -14109,19 +15146,19 @@
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>Sitaare (From "Ikkis")</t>
+          <t>Jaan Se Guzarte Hain</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>Arijit Singh, White Noise Collectives, Amitabh Bhattacharya</t>
+          <t>Shashwat Sachdev, Khan Saab, Nusrat Fateh Ali Khan</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>2026-04-02</t>
+          <t>2026-04-03</t>
         </is>
       </c>
       <c r="B10" t="n">
@@ -14141,7 +15178,7 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>2026-04-02</t>
+          <t>2026-04-03</t>
         </is>
       </c>
       <c r="B11" t="n">
@@ -14149,19 +15186,19 @@
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>Sahiba</t>
+          <t>Sitaare (From "Ikkis")</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>Aditya Rikhari</t>
+          <t>Arijit Singh, White Noise Collectives, Amitabh Bhattacharya</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>2026-04-02</t>
+          <t>2026-04-03</t>
         </is>
       </c>
       <c r="B12" t="n">
@@ -14169,19 +15206,19 @@
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>Pavazha Malli - From "Think Indie"</t>
+          <t>Apna Bana Le</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>Sai Abhyankkar, Shruti Haasan, Vivek</t>
+          <t>Sachin-Jigar, Arijit Singh, Amitabh Bhattacharya</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>2026-04-02</t>
+          <t>2026-04-03</t>
         </is>
       </c>
       <c r="B13" t="n">
@@ -14189,19 +15226,19 @@
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>Apna Bana Le</t>
+          <t>Samjhawan</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>Sachin-Jigar, Arijit Singh, Amitabh Bhattacharya</t>
+          <t>Jawad Ahmad, Shaarib Toshi, Arijit Singh, Shreya Ghoshal</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>2026-04-02</t>
+          <t>2026-04-03</t>
         </is>
       </c>
       <c r="B14" t="n">
@@ -14209,19 +15246,19 @@
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>Shree Hanuman Chalisa</t>
+          <t>Pavazha Malli - From "Think Indie"</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>Hariharan, Lalit Sen, Chander</t>
+          <t>Sai Abhyankkar, Shruti Haasan, Vivek</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>2026-04-02</t>
+          <t>2026-04-03</t>
         </is>
       </c>
       <c r="B15" t="n">
@@ -14229,19 +15266,19 @@
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>Samjhawan</t>
+          <t>Finding Her</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>Jawad Ahmad, Shaarib Toshi, Arijit Singh, Shreya Ghoshal</t>
+          <t>Kushagra, Bharath, Saaheal</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>2026-04-02</t>
+          <t>2026-04-03</t>
         </is>
       </c>
       <c r="B16" t="n">
@@ -14249,19 +15286,19 @@
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>Finding Her</t>
+          <t>Shararat</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>Kushagra, Bharath, Saaheal</t>
+          <t>Shashwat Sachdev, Madhubanti Bagchi, Jasmine Sandlas</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>2026-04-02</t>
+          <t>2026-04-03</t>
         </is>
       </c>
       <c r="B17" t="n">
@@ -14269,19 +15306,19 @@
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>Shararat</t>
+          <t>Boyfriend</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>Shashwat Sachdev, Madhubanti Bagchi, Jasmine Sandlas</t>
+          <t>Karan Aujla, Ikky</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>2026-04-02</t>
+          <t>2026-04-03</t>
         </is>
       </c>
       <c r="B18" t="n">
@@ -14289,19 +15326,19 @@
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>Arz Kiya Hai | Coke Studio Bharat</t>
+          <t>Dhurandhar - Title Track</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>Anuv Jain</t>
+          <t>Shashwat Sachdev, Hanumankind, Jasmine Sandlas, Sudhir Yaduvanshi, Charanjit Ahuja, Muhammad Sadiq, Ranjit Kaur, Babu Singh Maan</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>2026-04-02</t>
+          <t>2026-04-03</t>
         </is>
       </c>
       <c r="B19" t="n">
@@ -14309,19 +15346,19 @@
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>Dhurandhar - Title Track</t>
+          <t>Arz Kiya Hai | Coke Studio Bharat</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>Shashwat Sachdev, Hanumankind, Jasmine Sandlas, Sudhir Yaduvanshi, Charanjit Ahuja, Muhammad Sadiq, Ranjit Kaur, Babu Singh Maan</t>
+          <t>Anuv Jain</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>2026-04-02</t>
+          <t>2026-04-03</t>
         </is>
       </c>
       <c r="B20" t="n">
@@ -14341,7 +15378,7 @@
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>2026-04-02</t>
+          <t>2026-04-03</t>
         </is>
       </c>
       <c r="B21" t="n">
@@ -14349,19 +15386,19 @@
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>Boyfriend</t>
+          <t>Mann Mera</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>Karan Aujla, Ikky</t>
+          <t>Gajendra Verma</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>2026-04-02</t>
+          <t>2026-04-03</t>
         </is>
       </c>
       <c r="B22" t="n">
@@ -14381,7 +15418,7 @@
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>2026-04-02</t>
+          <t>2026-04-03</t>
         </is>
       </c>
       <c r="B23" t="n">
@@ -14389,19 +15426,19 @@
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>Mann Mera</t>
+          <t>For A Reason</t>
         </is>
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>Gajendra Verma</t>
+          <t>Karan Aujla, Ikky</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>2026-04-02</t>
+          <t>2026-04-03</t>
         </is>
       </c>
       <c r="B24" t="n">
@@ -14421,7 +15458,7 @@
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>2026-04-02</t>
+          <t>2026-04-03</t>
         </is>
       </c>
       <c r="B25" t="n">
@@ -14429,19 +15466,19 @@
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>Ishqa Ve</t>
+          <t>Naal Nachna</t>
         </is>
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>Zeeshan Ali, Yuvraj Tung, Sandeep Aulakh, Honey Dhillon</t>
+          <t>Shashwat Sachdev, Afsana Khan, Irshad Kamil, Reble</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>2026-04-02</t>
+          <t>2026-04-03</t>
         </is>
       </c>
       <c r="B26" t="n">
@@ -14449,19 +15486,19 @@
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>Bairi</t>
+          <t>Run Down The City - Monica</t>
         </is>
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>Virat, Pradeep Solanki, Heena</t>
+          <t>Shashwat Sachdev, Reble, Asha Bhosle, R. D. Burman, Majrooh Sultanpuri</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>2026-04-02</t>
+          <t>2026-04-03</t>
         </is>
       </c>
       <c r="B27" t="n">
@@ -14469,19 +15506,19 @@
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>For A Reason</t>
+          <t>Bairi</t>
         </is>
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t>Karan Aujla, Ikky</t>
+          <t>Virat, Pradeep Solanki, Heena</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>2026-04-02</t>
+          <t>2026-04-03</t>
         </is>
       </c>
       <c r="B28" t="n">
@@ -14489,19 +15526,19 @@
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>Naal Nachna</t>
+          <t>Ishqa Ve</t>
         </is>
       </c>
       <c r="D28" t="inlineStr">
         <is>
-          <t>Shashwat Sachdev, Afsana Khan, Irshad Kamil, Reble</t>
+          <t>Zeeshan Ali, Yuvraj Tung, Sandeep Aulakh, Honey Dhillon</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>2026-04-02</t>
+          <t>2026-04-03</t>
         </is>
       </c>
       <c r="B29" t="n">
@@ -14509,19 +15546,19 @@
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>Deewaana Deewaana</t>
+          <t>Tere Liye</t>
         </is>
       </c>
       <c r="D29" t="inlineStr">
         <is>
-          <t>A.R. Rahman, Irshad Kamil</t>
+          <t>Atif Aslam, Shreya Ghoshal, Sachin Gupta, Sameer Anjaan</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>2026-04-02</t>
+          <t>2026-04-03</t>
         </is>
       </c>
       <c r="B30" t="n">
@@ -14529,19 +15566,19 @@
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>Run Down The City - Monica</t>
+          <t>Deewaana Deewaana</t>
         </is>
       </c>
       <c r="D30" t="inlineStr">
         <is>
-          <t>Shashwat Sachdev, Reble, Asha Bhosle, R. D. Burman, Majrooh Sultanpuri</t>
+          <t>A.R. Rahman, Irshad Kamil</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>2026-04-02</t>
+          <t>2026-04-03</t>
         </is>
       </c>
       <c r="B31" t="n">
@@ -14549,19 +15586,19 @@
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>Darkhaast</t>
+          <t>Raanjhan (From "Do Patti")</t>
         </is>
       </c>
       <c r="D31" t="inlineStr">
         <is>
-          <t>Mithoon, Arijit Singh, Sunidhi Chauhan, Sayeed Quadri</t>
+          <t>Sachet-Parampara, Parampara Tandon, Kausar Munir</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>2026-04-02</t>
+          <t>2026-04-03</t>
         </is>
       </c>
       <c r="B32" t="n">
@@ -14569,19 +15606,19 @@
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>Tum Ho Toh (From "Saiyaara")</t>
+          <t>Tere Bina</t>
         </is>
       </c>
       <c r="D32" t="inlineStr">
         <is>
-          <t>Vishal Mishra, Hansika Pareek, Raj Shekhar</t>
+          <t>A.R. Rahman, Chinmayi, Murtuza Khan, Qadir Khan</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>2026-04-02</t>
+          <t>2026-04-03</t>
         </is>
       </c>
       <c r="B33" t="n">
@@ -14589,19 +15626,19 @@
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>Tere Liye</t>
+          <t>Tum Ho Toh (From "Saiyaara")</t>
         </is>
       </c>
       <c r="D33" t="inlineStr">
         <is>
-          <t>Atif Aslam, Shreya Ghoshal, Sachin Gupta, Sameer Anjaan</t>
+          <t>Vishal Mishra, Hansika Pareek, Raj Shekhar</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>2026-04-02</t>
+          <t>2026-04-03</t>
         </is>
       </c>
       <c r="B34" t="n">
@@ -14609,19 +15646,19 @@
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>Raanjhan (From "Do Patti")</t>
+          <t>Darkhaast</t>
         </is>
       </c>
       <c r="D34" t="inlineStr">
         <is>
-          <t>Sachet-Parampara, Parampara Tandon, Kausar Munir</t>
+          <t>Mithoon, Arijit Singh, Sunidhi Chauhan, Sayeed Quadri</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>2026-04-02</t>
+          <t>2026-04-03</t>
         </is>
       </c>
       <c r="B35" t="n">
@@ -14629,19 +15666,19 @@
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>Tere Bina</t>
+          <t>Jo Tum Mere Ho</t>
         </is>
       </c>
       <c r="D35" t="inlineStr">
         <is>
-          <t>A.R. Rahman, Chinmayi, Murtuza Khan, Qadir Khan</t>
+          <t>Anuv Jain</t>
         </is>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>2026-04-02</t>
+          <t>2026-04-03</t>
         </is>
       </c>
       <c r="B36" t="n">
@@ -14661,7 +15698,7 @@
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>2026-04-02</t>
+          <t>2026-04-03</t>
         </is>
       </c>
       <c r="B37" t="n">
@@ -14669,19 +15706,19 @@
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>Agar Tum Saath Ho (From "Tamasha")</t>
+          <t>Haseen</t>
         </is>
       </c>
       <c r="D37" t="inlineStr">
         <is>
-          <t>Alka Yagnik, Arijit Singh</t>
+          <t>Talwiinder, NDS, Rippy Grewal</t>
         </is>
       </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>2026-04-02</t>
+          <t>2026-04-03</t>
         </is>
       </c>
       <c r="B38" t="n">
@@ -14689,19 +15726,19 @@
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>Jo Tum Mere Ho</t>
+          <t>Agar Tum Saath Ho (From "Tamasha")</t>
         </is>
       </c>
       <c r="D38" t="inlineStr">
         <is>
-          <t>Anuv Jain</t>
+          <t>Alka Yagnik, Arijit Singh</t>
         </is>
       </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>2026-04-02</t>
+          <t>2026-04-03</t>
         </is>
       </c>
       <c r="B39" t="n">
@@ -14709,19 +15746,19 @@
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>Haseen</t>
+          <t>Mann Mera - Original Version</t>
         </is>
       </c>
       <c r="D39" t="inlineStr">
         <is>
-          <t>Talwiinder, NDS, Rippy Grewal</t>
+          <t>Gajendra Verma</t>
         </is>
       </c>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>2026-04-02</t>
+          <t>2026-04-03</t>
         </is>
       </c>
       <c r="B40" t="n">
@@ -14729,19 +15766,19 @@
       </c>
       <c r="C40" t="inlineStr">
         <is>
-          <t>Barbaad (From "Saiyaara")</t>
+          <t>Ye Tune Kya Kiya</t>
         </is>
       </c>
       <c r="D40" t="inlineStr">
         <is>
-          <t>The Rish, Jubin Nautiyal</t>
+          <t>Pritam, Javed Bashir, Rajat Arora</t>
         </is>
       </c>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>2026-04-02</t>
+          <t>2026-04-03</t>
         </is>
       </c>
       <c r="B41" t="n">
@@ -14761,7 +15798,7 @@
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>2026-04-02</t>
+          <t>2026-04-03</t>
         </is>
       </c>
       <c r="B42" t="n">
@@ -14769,19 +15806,19 @@
       </c>
       <c r="C42" t="inlineStr">
         <is>
-          <t>Ishq Jalakar - Karvaan</t>
+          <t>Mutta Kalakki (From "Youth")</t>
         </is>
       </c>
       <c r="D42" t="inlineStr">
         <is>
-          <t>Shashwat Sachdev, Shahzad Ali, Subhadeep Das Chowdhury, Armaan Khan, Irshad Kamil, Roshan, Sahir Ludhianvi</t>
+          <t>G. V. Prakash, Ken Karunaas</t>
         </is>
       </c>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>2026-04-02</t>
+          <t>2026-04-03</t>
         </is>
       </c>
       <c r="B43" t="n">
@@ -14789,19 +15826,19 @@
       </c>
       <c r="C43" t="inlineStr">
         <is>
-          <t>Teri Deewani</t>
+          <t>Ishq Jalakar - Karvaan</t>
         </is>
       </c>
       <c r="D43" t="inlineStr">
         <is>
-          <t>Kailash Kher, Paresh Kamath, Naresh Kamath</t>
+          <t>Shashwat Sachdev, Shahzad Ali, Subhadeep Das Chowdhury, Armaan Khan, Irshad Kamil, Roshan, Sahir Ludhianvi</t>
         </is>
       </c>
     </row>
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>2026-04-02</t>
+          <t>2026-04-03</t>
         </is>
       </c>
       <c r="B44" t="n">
@@ -14809,19 +15846,19 @@
       </c>
       <c r="C44" t="inlineStr">
         <is>
-          <t>Ye Tune Kya Kiya</t>
+          <t>Barbaad (From "Saiyaara")</t>
         </is>
       </c>
       <c r="D44" t="inlineStr">
         <is>
-          <t>Pritam, Javed Bashir, Rajat Arora</t>
+          <t>The Rish, Jubin Nautiyal</t>
         </is>
       </c>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>2026-04-02</t>
+          <t>2026-04-03</t>
         </is>
       </c>
       <c r="B45" t="n">
@@ -14829,19 +15866,19 @@
       </c>
       <c r="C45" t="inlineStr">
         <is>
-          <t>Mann Mera - Original Version</t>
+          <t>Aaya Sher (From "The Paradise") (Telugu)</t>
         </is>
       </c>
       <c r="D45" t="inlineStr">
         <is>
-          <t>Gajendra Verma</t>
+          <t>Anirudh Ravichander, Jangi Reddy, Arjun Chandy, Kasarla Shyam</t>
         </is>
       </c>
     </row>
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>2026-04-02</t>
+          <t>2026-04-03</t>
         </is>
       </c>
       <c r="B46" t="n">
@@ -14849,19 +15886,19 @@
       </c>
       <c r="C46" t="inlineStr">
         <is>
-          <t>Aaya Sher (From "The Paradise") (Telugu)</t>
+          <t>Not Guilty</t>
         </is>
       </c>
       <c r="D46" t="inlineStr">
         <is>
-          <t>Anirudh Ravichander, Jangi Reddy, Arjun Chandy, Kasarla Shyam</t>
+          <t>Dhanda Nyoliwala</t>
         </is>
       </c>
     </row>
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>2026-04-02</t>
+          <t>2026-04-03</t>
         </is>
       </c>
       <c r="B47" t="n">
@@ -14869,19 +15906,19 @@
       </c>
       <c r="C47" t="inlineStr">
         <is>
-          <t>Not Guilty</t>
+          <t>Teri Deewani</t>
         </is>
       </c>
       <c r="D47" t="inlineStr">
         <is>
-          <t>Dhanda Nyoliwala</t>
+          <t>Kailash Kher, Paresh Kamath, Naresh Kamath</t>
         </is>
       </c>
     </row>
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>2026-04-02</t>
+          <t>2026-04-03</t>
         </is>
       </c>
       <c r="B48" t="n">
@@ -14889,19 +15926,19 @@
       </c>
       <c r="C48" t="inlineStr">
         <is>
-          <t>Mutta Kalakki (From "Youth")</t>
+          <t>Hum Pyaar Karne Wale</t>
         </is>
       </c>
       <c r="D48" t="inlineStr">
         <is>
-          <t>G. V. Prakash, Ken Karunaas</t>
+          <t>Shashwat Sachdev, Anuradha Paudwal, Udit Narayan, Anand-Milind, Sameer Anjaan, Qveen Herby</t>
         </is>
       </c>
     </row>
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>2026-04-02</t>
+          <t>2026-04-03</t>
         </is>
       </c>
       <c r="B49" t="n">
@@ -14909,19 +15946,19 @@
       </c>
       <c r="C49" t="inlineStr">
         <is>
-          <t>Vaari Jaavan</t>
+          <t>Ehsaas</t>
         </is>
       </c>
       <c r="D49" t="inlineStr">
         <is>
-          <t>Shashwat Sachdev, Jyoti Nooran, Jasmine Sandlas, Reble</t>
+          <t>Faheem Abdullah, Duha Shah, Vaibhav Pani, Hyder Dar</t>
         </is>
       </c>
     </row>
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>2026-04-02</t>
+          <t>2026-04-03</t>
         </is>
       </c>
       <c r="B50" t="n">
@@ -14929,19 +15966,19 @@
       </c>
       <c r="C50" t="inlineStr">
         <is>
-          <t>Hum Pyaar Karne Wale</t>
+          <t>Vaari Jaavan</t>
         </is>
       </c>
       <c r="D50" t="inlineStr">
         <is>
-          <t>Shashwat Sachdev, Anuradha Paudwal, Udit Narayan, Anand-Milind, Sameer Anjaan, Qveen Herby</t>
+          <t>Shashwat Sachdev, Jyoti Nooran, Jasmine Sandlas, Reble</t>
         </is>
       </c>
     </row>
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>2026-04-02</t>
+          <t>2026-04-03</t>
         </is>
       </c>
       <c r="B51" t="n">
@@ -14949,12 +15986,12 @@
       </c>
       <c r="C51" t="inlineStr">
         <is>
-          <t>Ehsaas</t>
+          <t>Mast Magan (From "2 States)</t>
         </is>
       </c>
       <c r="D51" t="inlineStr">
         <is>
-          <t>Faheem Abdullah, Duha Shah, Vaibhav Pani, Hyder Dar</t>
+          <t>Arijit Singh, Chinmayi</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
added data for 4th got predictions for 5th april
</commit_message>
<xml_diff>
--- a/Probability Project.xlsx
+++ b/Probability Project.xlsx
@@ -24,6 +24,7 @@
     <sheet name="AUTO_20260401" sheetId="19" state="visible" r:id="rId19"/>
     <sheet name="AUTO_20260402" sheetId="20" state="visible" r:id="rId20"/>
     <sheet name="AUTO_20260403" sheetId="21" state="visible" r:id="rId21"/>
+    <sheet name="AUTO_20260404" sheetId="22" state="visible" r:id="rId22"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -14996,9 +14997,1045 @@
       </c>
     </row>
     <row r="2">
+      <c r="A2" s="0" t="inlineStr">
+        <is>
+          <t>2026-04-03</t>
+        </is>
+      </c>
+      <c r="B2" s="0" t="n">
+        <v>1</v>
+      </c>
+      <c r="C2" s="0" t="inlineStr">
+        <is>
+          <t>Bairan</t>
+        </is>
+      </c>
+      <c r="D2" s="0" t="inlineStr">
+        <is>
+          <t>Banjaare</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="0" t="inlineStr">
+        <is>
+          <t>2026-04-03</t>
+        </is>
+      </c>
+      <c r="B3" s="0" t="n">
+        <v>2</v>
+      </c>
+      <c r="C3" s="0" t="inlineStr">
+        <is>
+          <t>Jaiye Sajana</t>
+        </is>
+      </c>
+      <c r="D3" s="0" t="inlineStr">
+        <is>
+          <t>Shashwat Sachdev, Jasmine Sandlas, Satinder Sartaaj</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="0" t="inlineStr">
+        <is>
+          <t>2026-04-03</t>
+        </is>
+      </c>
+      <c r="B4" s="0" t="n">
+        <v>3</v>
+      </c>
+      <c r="C4" s="0" t="inlineStr">
+        <is>
+          <t>Gehra Hua</t>
+        </is>
+      </c>
+      <c r="D4" s="0" t="inlineStr">
+        <is>
+          <t>Shashwat Sachdev, Arijit Singh, Irshad Kamil, Armaan Khan</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="0" t="inlineStr">
+        <is>
+          <t>2026-04-03</t>
+        </is>
+      </c>
+      <c r="B5" s="0" t="n">
+        <v>4</v>
+      </c>
+      <c r="C5" s="0" t="inlineStr">
+        <is>
+          <t>Sheesha - Aakhya Mai Aakh Ghali Jo Bairan</t>
+        </is>
+      </c>
+      <c r="D5" s="0" t="inlineStr">
+        <is>
+          <t>Mitta Ror, Swara Verma</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="0" t="inlineStr">
+        <is>
+          <t>2026-04-03</t>
+        </is>
+      </c>
+      <c r="B6" s="0" t="n">
+        <v>5</v>
+      </c>
+      <c r="C6" s="0" t="inlineStr">
+        <is>
+          <t>Khat</t>
+        </is>
+      </c>
+      <c r="D6" s="0" t="inlineStr">
+        <is>
+          <t>Navjot Ahuja</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="0" t="inlineStr">
+        <is>
+          <t>2026-04-03</t>
+        </is>
+      </c>
+      <c r="B7" s="0" t="n">
+        <v>6</v>
+      </c>
+      <c r="C7" s="0" t="inlineStr">
+        <is>
+          <t>Dhurandhar The Revenge - Aari Aari</t>
+        </is>
+      </c>
+      <c r="D7" s="0" t="inlineStr">
+        <is>
+          <t>Shashwat Sachdev, Bombay Rockers, Irshad Kamil, Khan Saab, Reble, Token, Jasmine Sandlas, Sudhir Yaduvanshi</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="0" t="inlineStr">
+        <is>
+          <t>2026-04-03</t>
+        </is>
+      </c>
+      <c r="B8" s="0" t="n">
+        <v>7</v>
+      </c>
+      <c r="C8" s="0" t="inlineStr">
+        <is>
+          <t>Sahiba</t>
+        </is>
+      </c>
+      <c r="D8" s="0" t="inlineStr">
+        <is>
+          <t>Aditya Rikhari</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="0" t="inlineStr">
+        <is>
+          <t>2026-04-03</t>
+        </is>
+      </c>
+      <c r="B9" s="0" t="n">
+        <v>8</v>
+      </c>
+      <c r="C9" s="0" t="inlineStr">
+        <is>
+          <t>Jaan Se Guzarte Hain</t>
+        </is>
+      </c>
+      <c r="D9" s="0" t="inlineStr">
+        <is>
+          <t>Shashwat Sachdev, Khan Saab, Nusrat Fateh Ali Khan</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="0" t="inlineStr">
+        <is>
+          <t>2026-04-03</t>
+        </is>
+      </c>
+      <c r="B10" s="0" t="n">
+        <v>9</v>
+      </c>
+      <c r="C10" s="0" t="inlineStr">
+        <is>
+          <t>Dooron Dooron</t>
+        </is>
+      </c>
+      <c r="D10" s="0" t="inlineStr">
+        <is>
+          <t>Paresh Pahuja, Shiv Tandan, Meghdeep Bose</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="0" t="inlineStr">
+        <is>
+          <t>2026-04-03</t>
+        </is>
+      </c>
+      <c r="B11" s="0" t="n">
+        <v>10</v>
+      </c>
+      <c r="C11" s="0" t="inlineStr">
+        <is>
+          <t>Sitaare (From "Ikkis")</t>
+        </is>
+      </c>
+      <c r="D11" s="0" t="inlineStr">
+        <is>
+          <t>Arijit Singh, White Noise Collectives, Amitabh Bhattacharya</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="0" t="inlineStr">
+        <is>
+          <t>2026-04-03</t>
+        </is>
+      </c>
+      <c r="B12" s="0" t="n">
+        <v>11</v>
+      </c>
+      <c r="C12" s="0" t="inlineStr">
+        <is>
+          <t>Apna Bana Le</t>
+        </is>
+      </c>
+      <c r="D12" s="0" t="inlineStr">
+        <is>
+          <t>Sachin-Jigar, Arijit Singh, Amitabh Bhattacharya</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="0" t="inlineStr">
+        <is>
+          <t>2026-04-03</t>
+        </is>
+      </c>
+      <c r="B13" s="0" t="n">
+        <v>12</v>
+      </c>
+      <c r="C13" s="0" t="inlineStr">
+        <is>
+          <t>Samjhawan</t>
+        </is>
+      </c>
+      <c r="D13" s="0" t="inlineStr">
+        <is>
+          <t>Jawad Ahmad, Shaarib Toshi, Arijit Singh, Shreya Ghoshal</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="0" t="inlineStr">
+        <is>
+          <t>2026-04-03</t>
+        </is>
+      </c>
+      <c r="B14" s="0" t="n">
+        <v>13</v>
+      </c>
+      <c r="C14" s="0" t="inlineStr">
+        <is>
+          <t>Pavazha Malli - From "Think Indie"</t>
+        </is>
+      </c>
+      <c r="D14" s="0" t="inlineStr">
+        <is>
+          <t>Sai Abhyankkar, Shruti Haasan, Vivek</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="0" t="inlineStr">
+        <is>
+          <t>2026-04-03</t>
+        </is>
+      </c>
+      <c r="B15" s="0" t="n">
+        <v>14</v>
+      </c>
+      <c r="C15" s="0" t="inlineStr">
+        <is>
+          <t>Finding Her</t>
+        </is>
+      </c>
+      <c r="D15" s="0" t="inlineStr">
+        <is>
+          <t>Kushagra, Bharath, Saaheal</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="0" t="inlineStr">
+        <is>
+          <t>2026-04-03</t>
+        </is>
+      </c>
+      <c r="B16" s="0" t="n">
+        <v>15</v>
+      </c>
+      <c r="C16" s="0" t="inlineStr">
+        <is>
+          <t>Shararat</t>
+        </is>
+      </c>
+      <c r="D16" s="0" t="inlineStr">
+        <is>
+          <t>Shashwat Sachdev, Madhubanti Bagchi, Jasmine Sandlas</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="0" t="inlineStr">
+        <is>
+          <t>2026-04-03</t>
+        </is>
+      </c>
+      <c r="B17" s="0" t="n">
+        <v>16</v>
+      </c>
+      <c r="C17" s="0" t="inlineStr">
+        <is>
+          <t>Boyfriend</t>
+        </is>
+      </c>
+      <c r="D17" s="0" t="inlineStr">
+        <is>
+          <t>Karan Aujla, Ikky</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="0" t="inlineStr">
+        <is>
+          <t>2026-04-03</t>
+        </is>
+      </c>
+      <c r="B18" s="0" t="n">
+        <v>17</v>
+      </c>
+      <c r="C18" s="0" t="inlineStr">
+        <is>
+          <t>Dhurandhar - Title Track</t>
+        </is>
+      </c>
+      <c r="D18" s="0" t="inlineStr">
+        <is>
+          <t>Shashwat Sachdev, Hanumankind, Jasmine Sandlas, Sudhir Yaduvanshi, Charanjit Ahuja, Muhammad Sadiq, Ranjit Kaur, Babu Singh Maan</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="0" t="inlineStr">
+        <is>
+          <t>2026-04-03</t>
+        </is>
+      </c>
+      <c r="B19" s="0" t="n">
+        <v>18</v>
+      </c>
+      <c r="C19" s="0" t="inlineStr">
+        <is>
+          <t>Arz Kiya Hai | Coke Studio Bharat</t>
+        </is>
+      </c>
+      <c r="D19" s="0" t="inlineStr">
+        <is>
+          <t>Anuv Jain</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="0" t="inlineStr">
+        <is>
+          <t>2026-04-03</t>
+        </is>
+      </c>
+      <c r="B20" s="0" t="n">
+        <v>19</v>
+      </c>
+      <c r="C20" s="0" t="inlineStr">
+        <is>
+          <t>Ishq</t>
+        </is>
+      </c>
+      <c r="D20" s="0" t="inlineStr">
+        <is>
+          <t>Faheem Abdullah, Rauhan Malik, Amir Ameer</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="0" t="inlineStr">
+        <is>
+          <t>2026-04-03</t>
+        </is>
+      </c>
+      <c r="B21" s="0" t="n">
+        <v>20</v>
+      </c>
+      <c r="C21" s="0" t="inlineStr">
+        <is>
+          <t>Mann Mera</t>
+        </is>
+      </c>
+      <c r="D21" s="0" t="inlineStr">
+        <is>
+          <t>Gajendra Verma</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="0" t="inlineStr">
+        <is>
+          <t>2026-04-03</t>
+        </is>
+      </c>
+      <c r="B22" s="0" t="n">
+        <v>21</v>
+      </c>
+      <c r="C22" s="0" t="inlineStr">
+        <is>
+          <t>Phir Se</t>
+        </is>
+      </c>
+      <c r="D22" s="0" t="inlineStr">
+        <is>
+          <t>Shashwat Sachdev, Arijit Singh, Irshad Kamil</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="0" t="inlineStr">
+        <is>
+          <t>2026-04-03</t>
+        </is>
+      </c>
+      <c r="B23" s="0" t="n">
+        <v>22</v>
+      </c>
+      <c r="C23" s="0" t="inlineStr">
+        <is>
+          <t>For A Reason</t>
+        </is>
+      </c>
+      <c r="D23" s="0" t="inlineStr">
+        <is>
+          <t>Karan Aujla, Ikky</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="0" t="inlineStr">
+        <is>
+          <t>2026-04-03</t>
+        </is>
+      </c>
+      <c r="B24" s="0" t="n">
+        <v>23</v>
+      </c>
+      <c r="C24" s="0" t="inlineStr">
+        <is>
+          <t>Saiyaara</t>
+        </is>
+      </c>
+      <c r="D24" s="0" t="inlineStr">
+        <is>
+          <t>Tanishk Bagchi, Faheem Abdullah, Arslan Nizami, Irshad Kamil</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="0" t="inlineStr">
+        <is>
+          <t>2026-04-03</t>
+        </is>
+      </c>
+      <c r="B25" s="0" t="n">
+        <v>24</v>
+      </c>
+      <c r="C25" s="0" t="inlineStr">
+        <is>
+          <t>Naal Nachna</t>
+        </is>
+      </c>
+      <c r="D25" s="0" t="inlineStr">
+        <is>
+          <t>Shashwat Sachdev, Afsana Khan, Irshad Kamil, Reble</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="0" t="inlineStr">
+        <is>
+          <t>2026-04-03</t>
+        </is>
+      </c>
+      <c r="B26" s="0" t="n">
+        <v>25</v>
+      </c>
+      <c r="C26" s="0" t="inlineStr">
+        <is>
+          <t>Run Down The City - Monica</t>
+        </is>
+      </c>
+      <c r="D26" s="0" t="inlineStr">
+        <is>
+          <t>Shashwat Sachdev, Reble, Asha Bhosle, R. D. Burman, Majrooh Sultanpuri</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="0" t="inlineStr">
+        <is>
+          <t>2026-04-03</t>
+        </is>
+      </c>
+      <c r="B27" s="0" t="n">
+        <v>26</v>
+      </c>
+      <c r="C27" s="0" t="inlineStr">
+        <is>
+          <t>Bairi</t>
+        </is>
+      </c>
+      <c r="D27" s="0" t="inlineStr">
+        <is>
+          <t>Virat, Pradeep Solanki, Heena</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="0" t="inlineStr">
+        <is>
+          <t>2026-04-03</t>
+        </is>
+      </c>
+      <c r="B28" s="0" t="n">
+        <v>27</v>
+      </c>
+      <c r="C28" s="0" t="inlineStr">
+        <is>
+          <t>Ishqa Ve</t>
+        </is>
+      </c>
+      <c r="D28" s="0" t="inlineStr">
+        <is>
+          <t>Zeeshan Ali, Yuvraj Tung, Sandeep Aulakh, Honey Dhillon</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="0" t="inlineStr">
+        <is>
+          <t>2026-04-03</t>
+        </is>
+      </c>
+      <c r="B29" s="0" t="n">
+        <v>28</v>
+      </c>
+      <c r="C29" s="0" t="inlineStr">
+        <is>
+          <t>Tere Liye</t>
+        </is>
+      </c>
+      <c r="D29" s="0" t="inlineStr">
+        <is>
+          <t>Atif Aslam, Shreya Ghoshal, Sachin Gupta, Sameer Anjaan</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="0" t="inlineStr">
+        <is>
+          <t>2026-04-03</t>
+        </is>
+      </c>
+      <c r="B30" s="0" t="n">
+        <v>29</v>
+      </c>
+      <c r="C30" s="0" t="inlineStr">
+        <is>
+          <t>Deewaana Deewaana</t>
+        </is>
+      </c>
+      <c r="D30" s="0" t="inlineStr">
+        <is>
+          <t>A.R. Rahman, Irshad Kamil</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="0" t="inlineStr">
+        <is>
+          <t>2026-04-03</t>
+        </is>
+      </c>
+      <c r="B31" s="0" t="n">
+        <v>30</v>
+      </c>
+      <c r="C31" s="0" t="inlineStr">
+        <is>
+          <t>Raanjhan (From "Do Patti")</t>
+        </is>
+      </c>
+      <c r="D31" s="0" t="inlineStr">
+        <is>
+          <t>Sachet-Parampara, Parampara Tandon, Kausar Munir</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="0" t="inlineStr">
+        <is>
+          <t>2026-04-03</t>
+        </is>
+      </c>
+      <c r="B32" s="0" t="n">
+        <v>31</v>
+      </c>
+      <c r="C32" s="0" t="inlineStr">
+        <is>
+          <t>Tere Bina</t>
+        </is>
+      </c>
+      <c r="D32" s="0" t="inlineStr">
+        <is>
+          <t>A.R. Rahman, Chinmayi, Murtuza Khan, Qadir Khan</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="0" t="inlineStr">
+        <is>
+          <t>2026-04-03</t>
+        </is>
+      </c>
+      <c r="B33" s="0" t="n">
+        <v>32</v>
+      </c>
+      <c r="C33" s="0" t="inlineStr">
+        <is>
+          <t>Tum Ho Toh (From "Saiyaara")</t>
+        </is>
+      </c>
+      <c r="D33" s="0" t="inlineStr">
+        <is>
+          <t>Vishal Mishra, Hansika Pareek, Raj Shekhar</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="0" t="inlineStr">
+        <is>
+          <t>2026-04-03</t>
+        </is>
+      </c>
+      <c r="B34" s="0" t="n">
+        <v>33</v>
+      </c>
+      <c r="C34" s="0" t="inlineStr">
+        <is>
+          <t>Darkhaast</t>
+        </is>
+      </c>
+      <c r="D34" s="0" t="inlineStr">
+        <is>
+          <t>Mithoon, Arijit Singh, Sunidhi Chauhan, Sayeed Quadri</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="0" t="inlineStr">
+        <is>
+          <t>2026-04-03</t>
+        </is>
+      </c>
+      <c r="B35" s="0" t="n">
+        <v>34</v>
+      </c>
+      <c r="C35" s="0" t="inlineStr">
+        <is>
+          <t>Jo Tum Mere Ho</t>
+        </is>
+      </c>
+      <c r="D35" s="0" t="inlineStr">
+        <is>
+          <t>Anuv Jain</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="0" t="inlineStr">
+        <is>
+          <t>2026-04-03</t>
+        </is>
+      </c>
+      <c r="B36" s="0" t="n">
+        <v>35</v>
+      </c>
+      <c r="C36" s="0" t="inlineStr">
+        <is>
+          <t>Lutt Le Gaya</t>
+        </is>
+      </c>
+      <c r="D36" s="0" t="inlineStr">
+        <is>
+          <t>Shashwat Sachdev, Simran Choudhary</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="0" t="inlineStr">
+        <is>
+          <t>2026-04-03</t>
+        </is>
+      </c>
+      <c r="B37" s="0" t="n">
+        <v>36</v>
+      </c>
+      <c r="C37" s="0" t="inlineStr">
+        <is>
+          <t>Haseen</t>
+        </is>
+      </c>
+      <c r="D37" s="0" t="inlineStr">
+        <is>
+          <t>Talwiinder, NDS, Rippy Grewal</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="0" t="inlineStr">
+        <is>
+          <t>2026-04-03</t>
+        </is>
+      </c>
+      <c r="B38" s="0" t="n">
+        <v>37</v>
+      </c>
+      <c r="C38" s="0" t="inlineStr">
+        <is>
+          <t>Agar Tum Saath Ho (From "Tamasha")</t>
+        </is>
+      </c>
+      <c r="D38" s="0" t="inlineStr">
+        <is>
+          <t>Alka Yagnik, Arijit Singh</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="0" t="inlineStr">
+        <is>
+          <t>2026-04-03</t>
+        </is>
+      </c>
+      <c r="B39" s="0" t="n">
+        <v>38</v>
+      </c>
+      <c r="C39" s="0" t="inlineStr">
+        <is>
+          <t>Mann Mera - Original Version</t>
+        </is>
+      </c>
+      <c r="D39" s="0" t="inlineStr">
+        <is>
+          <t>Gajendra Verma</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="0" t="inlineStr">
+        <is>
+          <t>2026-04-03</t>
+        </is>
+      </c>
+      <c r="B40" s="0" t="n">
+        <v>39</v>
+      </c>
+      <c r="C40" s="0" t="inlineStr">
+        <is>
+          <t>Ye Tune Kya Kiya</t>
+        </is>
+      </c>
+      <c r="D40" s="0" t="inlineStr">
+        <is>
+          <t>Pritam, Javed Bashir, Rajat Arora</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" s="0" t="inlineStr">
+        <is>
+          <t>2026-04-03</t>
+        </is>
+      </c>
+      <c r="B41" s="0" t="n">
+        <v>40</v>
+      </c>
+      <c r="C41" s="0" t="inlineStr">
+        <is>
+          <t>Main Aur Tu</t>
+        </is>
+      </c>
+      <c r="D41" s="0" t="inlineStr">
+        <is>
+          <t>Shashwat Sachdev, Jasmine Sandlas, Reble</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" s="0" t="inlineStr">
+        <is>
+          <t>2026-04-03</t>
+        </is>
+      </c>
+      <c r="B42" s="0" t="n">
+        <v>41</v>
+      </c>
+      <c r="C42" s="0" t="inlineStr">
+        <is>
+          <t>Mutta Kalakki (From "Youth")</t>
+        </is>
+      </c>
+      <c r="D42" s="0" t="inlineStr">
+        <is>
+          <t>G. V. Prakash, Ken Karunaas</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" s="0" t="inlineStr">
+        <is>
+          <t>2026-04-03</t>
+        </is>
+      </c>
+      <c r="B43" s="0" t="n">
+        <v>42</v>
+      </c>
+      <c r="C43" s="0" t="inlineStr">
+        <is>
+          <t>Ishq Jalakar - Karvaan</t>
+        </is>
+      </c>
+      <c r="D43" s="0" t="inlineStr">
+        <is>
+          <t>Shashwat Sachdev, Shahzad Ali, Subhadeep Das Chowdhury, Armaan Khan, Irshad Kamil, Roshan, Sahir Ludhianvi</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" s="0" t="inlineStr">
+        <is>
+          <t>2026-04-03</t>
+        </is>
+      </c>
+      <c r="B44" s="0" t="n">
+        <v>43</v>
+      </c>
+      <c r="C44" s="0" t="inlineStr">
+        <is>
+          <t>Barbaad (From "Saiyaara")</t>
+        </is>
+      </c>
+      <c r="D44" s="0" t="inlineStr">
+        <is>
+          <t>The Rish, Jubin Nautiyal</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" s="0" t="inlineStr">
+        <is>
+          <t>2026-04-03</t>
+        </is>
+      </c>
+      <c r="B45" s="0" t="n">
+        <v>44</v>
+      </c>
+      <c r="C45" s="0" t="inlineStr">
+        <is>
+          <t>Aaya Sher (From "The Paradise") (Telugu)</t>
+        </is>
+      </c>
+      <c r="D45" s="0" t="inlineStr">
+        <is>
+          <t>Anirudh Ravichander, Jangi Reddy, Arjun Chandy, Kasarla Shyam</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" s="0" t="inlineStr">
+        <is>
+          <t>2026-04-03</t>
+        </is>
+      </c>
+      <c r="B46" s="0" t="n">
+        <v>45</v>
+      </c>
+      <c r="C46" s="0" t="inlineStr">
+        <is>
+          <t>Not Guilty</t>
+        </is>
+      </c>
+      <c r="D46" s="0" t="inlineStr">
+        <is>
+          <t>Dhanda Nyoliwala</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" s="0" t="inlineStr">
+        <is>
+          <t>2026-04-03</t>
+        </is>
+      </c>
+      <c r="B47" s="0" t="n">
+        <v>46</v>
+      </c>
+      <c r="C47" s="0" t="inlineStr">
+        <is>
+          <t>Teri Deewani</t>
+        </is>
+      </c>
+      <c r="D47" s="0" t="inlineStr">
+        <is>
+          <t>Kailash Kher, Paresh Kamath, Naresh Kamath</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" s="0" t="inlineStr">
+        <is>
+          <t>2026-04-03</t>
+        </is>
+      </c>
+      <c r="B48" s="0" t="n">
+        <v>47</v>
+      </c>
+      <c r="C48" s="0" t="inlineStr">
+        <is>
+          <t>Hum Pyaar Karne Wale</t>
+        </is>
+      </c>
+      <c r="D48" s="0" t="inlineStr">
+        <is>
+          <t>Shashwat Sachdev, Anuradha Paudwal, Udit Narayan, Anand-Milind, Sameer Anjaan, Qveen Herby</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" s="0" t="inlineStr">
+        <is>
+          <t>2026-04-03</t>
+        </is>
+      </c>
+      <c r="B49" s="0" t="n">
+        <v>48</v>
+      </c>
+      <c r="C49" s="0" t="inlineStr">
+        <is>
+          <t>Ehsaas</t>
+        </is>
+      </c>
+      <c r="D49" s="0" t="inlineStr">
+        <is>
+          <t>Faheem Abdullah, Duha Shah, Vaibhav Pani, Hyder Dar</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" s="0" t="inlineStr">
+        <is>
+          <t>2026-04-03</t>
+        </is>
+      </c>
+      <c r="B50" s="0" t="n">
+        <v>49</v>
+      </c>
+      <c r="C50" s="0" t="inlineStr">
+        <is>
+          <t>Vaari Jaavan</t>
+        </is>
+      </c>
+      <c r="D50" s="0" t="inlineStr">
+        <is>
+          <t>Shashwat Sachdev, Jyoti Nooran, Jasmine Sandlas, Reble</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" s="0" t="inlineStr">
+        <is>
+          <t>2026-04-03</t>
+        </is>
+      </c>
+      <c r="B51" s="0" t="n">
+        <v>50</v>
+      </c>
+      <c r="C51" s="0" t="inlineStr">
+        <is>
+          <t>Mast Magan (From "2 States)</t>
+        </is>
+      </c>
+      <c r="D51" s="0" t="inlineStr">
+        <is>
+          <t>Arijit Singh, Chinmayi</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet22.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:D51"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="24" t="inlineStr">
+        <is>
+          <t>Date</t>
+        </is>
+      </c>
+      <c r="B1" s="24" t="inlineStr">
+        <is>
+          <t>Rank</t>
+        </is>
+      </c>
+      <c r="C1" s="24" t="inlineStr">
+        <is>
+          <t>Song</t>
+        </is>
+      </c>
+      <c r="D1" s="24" t="inlineStr">
+        <is>
+          <t>Artist</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>2026-04-03</t>
+          <t>2026-04-04</t>
         </is>
       </c>
       <c r="B2" t="n">
@@ -15018,7 +16055,7 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>2026-04-03</t>
+          <t>2026-04-04</t>
         </is>
       </c>
       <c r="B3" t="n">
@@ -15038,7 +16075,7 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>2026-04-03</t>
+          <t>2026-04-04</t>
         </is>
       </c>
       <c r="B4" t="n">
@@ -15058,7 +16095,7 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>2026-04-03</t>
+          <t>2026-04-04</t>
         </is>
       </c>
       <c r="B5" t="n">
@@ -15078,7 +16115,7 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>2026-04-03</t>
+          <t>2026-04-04</t>
         </is>
       </c>
       <c r="B6" t="n">
@@ -15098,7 +16135,7 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>2026-04-03</t>
+          <t>2026-04-04</t>
         </is>
       </c>
       <c r="B7" t="n">
@@ -15118,7 +16155,7 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>2026-04-03</t>
+          <t>2026-04-04</t>
         </is>
       </c>
       <c r="B8" t="n">
@@ -15138,7 +16175,7 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>2026-04-03</t>
+          <t>2026-04-04</t>
         </is>
       </c>
       <c r="B9" t="n">
@@ -15146,19 +16183,19 @@
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>Jaan Se Guzarte Hain</t>
+          <t>Dooron Dooron</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>Shashwat Sachdev, Khan Saab, Nusrat Fateh Ali Khan</t>
+          <t>Paresh Pahuja, Shiv Tandan, Meghdeep Bose</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>2026-04-03</t>
+          <t>2026-04-04</t>
         </is>
       </c>
       <c r="B10" t="n">
@@ -15166,19 +16203,19 @@
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>Dooron Dooron</t>
+          <t>Jaan Se Guzarte Hain</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>Paresh Pahuja, Shiv Tandan, Meghdeep Bose</t>
+          <t>Shashwat Sachdev, Khan Saab, Nusrat Fateh Ali Khan</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>2026-04-03</t>
+          <t>2026-04-04</t>
         </is>
       </c>
       <c r="B11" t="n">
@@ -15186,19 +16223,19 @@
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>Sitaare (From "Ikkis")</t>
+          <t>Apna Bana Le</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>Arijit Singh, White Noise Collectives, Amitabh Bhattacharya</t>
+          <t>Sachin-Jigar, Arijit Singh, Amitabh Bhattacharya</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>2026-04-03</t>
+          <t>2026-04-04</t>
         </is>
       </c>
       <c r="B12" t="n">
@@ -15206,19 +16243,19 @@
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>Apna Bana Le</t>
+          <t>Samjhawan</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>Sachin-Jigar, Arijit Singh, Amitabh Bhattacharya</t>
+          <t>Jawad Ahmad, Shaarib Toshi, Arijit Singh, Shreya Ghoshal</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>2026-04-03</t>
+          <t>2026-04-04</t>
         </is>
       </c>
       <c r="B13" t="n">
@@ -15226,19 +16263,19 @@
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>Samjhawan</t>
+          <t>Sitaare (From "Ikkis")</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>Jawad Ahmad, Shaarib Toshi, Arijit Singh, Shreya Ghoshal</t>
+          <t>Arijit Singh, White Noise Collectives, Amitabh Bhattacharya</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>2026-04-03</t>
+          <t>2026-04-04</t>
         </is>
       </c>
       <c r="B14" t="n">
@@ -15258,7 +16295,7 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>2026-04-03</t>
+          <t>2026-04-04</t>
         </is>
       </c>
       <c r="B15" t="n">
@@ -15278,7 +16315,7 @@
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>2026-04-03</t>
+          <t>2026-04-04</t>
         </is>
       </c>
       <c r="B16" t="n">
@@ -15298,7 +16335,7 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>2026-04-03</t>
+          <t>2026-04-04</t>
         </is>
       </c>
       <c r="B17" t="n">
@@ -15306,19 +16343,19 @@
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>Boyfriend</t>
+          <t>Dhurandhar - Title Track</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>Karan Aujla, Ikky</t>
+          <t>Shashwat Sachdev, Hanumankind, Jasmine Sandlas, Sudhir Yaduvanshi, Charanjit Ahuja, Muhammad Sadiq, Ranjit Kaur, Babu Singh Maan</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>2026-04-03</t>
+          <t>2026-04-04</t>
         </is>
       </c>
       <c r="B18" t="n">
@@ -15326,19 +16363,19 @@
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>Dhurandhar - Title Track</t>
+          <t>Arz Kiya Hai | Coke Studio Bharat</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>Shashwat Sachdev, Hanumankind, Jasmine Sandlas, Sudhir Yaduvanshi, Charanjit Ahuja, Muhammad Sadiq, Ranjit Kaur, Babu Singh Maan</t>
+          <t>Anuv Jain</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>2026-04-03</t>
+          <t>2026-04-04</t>
         </is>
       </c>
       <c r="B19" t="n">
@@ -15346,19 +16383,19 @@
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>Arz Kiya Hai | Coke Studio Bharat</t>
+          <t>Boyfriend</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>Anuv Jain</t>
+          <t>Karan Aujla, Ikky</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>2026-04-03</t>
+          <t>2026-04-04</t>
         </is>
       </c>
       <c r="B20" t="n">
@@ -15378,7 +16415,7 @@
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>2026-04-03</t>
+          <t>2026-04-04</t>
         </is>
       </c>
       <c r="B21" t="n">
@@ -15398,7 +16435,7 @@
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>2026-04-03</t>
+          <t>2026-04-04</t>
         </is>
       </c>
       <c r="B22" t="n">
@@ -15406,19 +16443,19 @@
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>Phir Se</t>
+          <t>Saiyaara</t>
         </is>
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>Shashwat Sachdev, Arijit Singh, Irshad Kamil</t>
+          <t>Tanishk Bagchi, Faheem Abdullah, Arslan Nizami, Irshad Kamil</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>2026-04-03</t>
+          <t>2026-04-04</t>
         </is>
       </c>
       <c r="B23" t="n">
@@ -15426,19 +16463,19 @@
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>For A Reason</t>
+          <t>Ishqa Ve</t>
         </is>
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>Karan Aujla, Ikky</t>
+          <t>Zeeshan Ali, Yuvraj Tung, Sandeep Aulakh, Honey Dhillon</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>2026-04-03</t>
+          <t>2026-04-04</t>
         </is>
       </c>
       <c r="B24" t="n">
@@ -15446,19 +16483,19 @@
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>Saiyaara</t>
+          <t>For A Reason</t>
         </is>
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>Tanishk Bagchi, Faheem Abdullah, Arslan Nizami, Irshad Kamil</t>
+          <t>Karan Aujla, Ikky</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>2026-04-03</t>
+          <t>2026-04-04</t>
         </is>
       </c>
       <c r="B25" t="n">
@@ -15466,19 +16503,19 @@
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>Naal Nachna</t>
+          <t>Tere Bina</t>
         </is>
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>Shashwat Sachdev, Afsana Khan, Irshad Kamil, Reble</t>
+          <t>A.R. Rahman, Chinmayi, Murtuza Khan, Qadir Khan</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>2026-04-03</t>
+          <t>2026-04-04</t>
         </is>
       </c>
       <c r="B26" t="n">
@@ -15486,19 +16523,19 @@
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>Run Down The City - Monica</t>
+          <t>Naal Nachna</t>
         </is>
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>Shashwat Sachdev, Reble, Asha Bhosle, R. D. Burman, Majrooh Sultanpuri</t>
+          <t>Shashwat Sachdev, Afsana Khan, Irshad Kamil, Reble</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>2026-04-03</t>
+          <t>2026-04-04</t>
         </is>
       </c>
       <c r="B27" t="n">
@@ -15518,7 +16555,7 @@
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>2026-04-03</t>
+          <t>2026-04-04</t>
         </is>
       </c>
       <c r="B28" t="n">
@@ -15526,19 +16563,19 @@
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>Ishqa Ve</t>
+          <t>Run Down The City - Monica</t>
         </is>
       </c>
       <c r="D28" t="inlineStr">
         <is>
-          <t>Zeeshan Ali, Yuvraj Tung, Sandeep Aulakh, Honey Dhillon</t>
+          <t>Shashwat Sachdev, Reble, Asha Bhosle, R. D. Burman, Majrooh Sultanpuri</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>2026-04-03</t>
+          <t>2026-04-04</t>
         </is>
       </c>
       <c r="B29" t="n">
@@ -15546,19 +16583,19 @@
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>Tere Liye</t>
+          <t>Phir Se</t>
         </is>
       </c>
       <c r="D29" t="inlineStr">
         <is>
-          <t>Atif Aslam, Shreya Ghoshal, Sachin Gupta, Sameer Anjaan</t>
+          <t>Shashwat Sachdev, Arijit Singh, Irshad Kamil</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>2026-04-03</t>
+          <t>2026-04-04</t>
         </is>
       </c>
       <c r="B30" t="n">
@@ -15578,7 +16615,7 @@
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>2026-04-03</t>
+          <t>2026-04-04</t>
         </is>
       </c>
       <c r="B31" t="n">
@@ -15586,19 +16623,19 @@
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>Raanjhan (From "Do Patti")</t>
+          <t>Tere Liye</t>
         </is>
       </c>
       <c r="D31" t="inlineStr">
         <is>
-          <t>Sachet-Parampara, Parampara Tandon, Kausar Munir</t>
+          <t>Atif Aslam, Shreya Ghoshal, Sachin Gupta, Sameer Anjaan</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>2026-04-03</t>
+          <t>2026-04-04</t>
         </is>
       </c>
       <c r="B32" t="n">
@@ -15606,19 +16643,19 @@
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>Tere Bina</t>
+          <t>Raanjhan (From "Do Patti")</t>
         </is>
       </c>
       <c r="D32" t="inlineStr">
         <is>
-          <t>A.R. Rahman, Chinmayi, Murtuza Khan, Qadir Khan</t>
+          <t>Sachet-Parampara, Parampara Tandon, Kausar Munir</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>2026-04-03</t>
+          <t>2026-04-04</t>
         </is>
       </c>
       <c r="B33" t="n">
@@ -15626,19 +16663,19 @@
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>Tum Ho Toh (From "Saiyaara")</t>
+          <t>Jo Tum Mere Ho</t>
         </is>
       </c>
       <c r="D33" t="inlineStr">
         <is>
-          <t>Vishal Mishra, Hansika Pareek, Raj Shekhar</t>
+          <t>Anuv Jain</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>2026-04-03</t>
+          <t>2026-04-04</t>
         </is>
       </c>
       <c r="B34" t="n">
@@ -15646,19 +16683,19 @@
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>Darkhaast</t>
+          <t>Tum Ho Toh (From "Saiyaara")</t>
         </is>
       </c>
       <c r="D34" t="inlineStr">
         <is>
-          <t>Mithoon, Arijit Singh, Sunidhi Chauhan, Sayeed Quadri</t>
+          <t>Vishal Mishra, Hansika Pareek, Raj Shekhar</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>2026-04-03</t>
+          <t>2026-04-04</t>
         </is>
       </c>
       <c r="B35" t="n">
@@ -15666,19 +16703,19 @@
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>Jo Tum Mere Ho</t>
+          <t>Haseen</t>
         </is>
       </c>
       <c r="D35" t="inlineStr">
         <is>
-          <t>Anuv Jain</t>
+          <t>Talwiinder, NDS, Rippy Grewal</t>
         </is>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>2026-04-03</t>
+          <t>2026-04-04</t>
         </is>
       </c>
       <c r="B36" t="n">
@@ -15686,19 +16723,19 @@
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>Lutt Le Gaya</t>
+          <t>Darkhaast</t>
         </is>
       </c>
       <c r="D36" t="inlineStr">
         <is>
-          <t>Shashwat Sachdev, Simran Choudhary</t>
+          <t>Mithoon, Arijit Singh, Sunidhi Chauhan, Sayeed Quadri</t>
         </is>
       </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>2026-04-03</t>
+          <t>2026-04-04</t>
         </is>
       </c>
       <c r="B37" t="n">
@@ -15706,19 +16743,19 @@
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>Haseen</t>
+          <t>Lutt Le Gaya</t>
         </is>
       </c>
       <c r="D37" t="inlineStr">
         <is>
-          <t>Talwiinder, NDS, Rippy Grewal</t>
+          <t>Shashwat Sachdev, Simran Choudhary</t>
         </is>
       </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>2026-04-03</t>
+          <t>2026-04-04</t>
         </is>
       </c>
       <c r="B38" t="n">
@@ -15726,19 +16763,19 @@
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>Agar Tum Saath Ho (From "Tamasha")</t>
+          <t>Ye Tune Kya Kiya</t>
         </is>
       </c>
       <c r="D38" t="inlineStr">
         <is>
-          <t>Alka Yagnik, Arijit Singh</t>
+          <t>Pritam, Javed Bashir, Rajat Arora</t>
         </is>
       </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>2026-04-03</t>
+          <t>2026-04-04</t>
         </is>
       </c>
       <c r="B39" t="n">
@@ -15758,7 +16795,7 @@
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>2026-04-03</t>
+          <t>2026-04-04</t>
         </is>
       </c>
       <c r="B40" t="n">
@@ -15766,19 +16803,19 @@
       </c>
       <c r="C40" t="inlineStr">
         <is>
-          <t>Ye Tune Kya Kiya</t>
+          <t>Agar Tum Saath Ho (From "Tamasha")</t>
         </is>
       </c>
       <c r="D40" t="inlineStr">
         <is>
-          <t>Pritam, Javed Bashir, Rajat Arora</t>
+          <t>Alka Yagnik, Arijit Singh</t>
         </is>
       </c>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>2026-04-03</t>
+          <t>2026-04-04</t>
         </is>
       </c>
       <c r="B41" t="n">
@@ -15786,19 +16823,19 @@
       </c>
       <c r="C41" t="inlineStr">
         <is>
-          <t>Main Aur Tu</t>
+          <t>Ishq Jalakar - Karvaan</t>
         </is>
       </c>
       <c r="D41" t="inlineStr">
         <is>
-          <t>Shashwat Sachdev, Jasmine Sandlas, Reble</t>
+          <t>Shashwat Sachdev, Shahzad Ali, Subhadeep Das Chowdhury, Armaan Khan, Irshad Kamil, Roshan, Sahir Ludhianvi</t>
         </is>
       </c>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>2026-04-03</t>
+          <t>2026-04-04</t>
         </is>
       </c>
       <c r="B42" t="n">
@@ -15818,7 +16855,7 @@
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>2026-04-03</t>
+          <t>2026-04-04</t>
         </is>
       </c>
       <c r="B43" t="n">
@@ -15826,19 +16863,19 @@
       </c>
       <c r="C43" t="inlineStr">
         <is>
-          <t>Ishq Jalakar - Karvaan</t>
+          <t>Teri Deewani</t>
         </is>
       </c>
       <c r="D43" t="inlineStr">
         <is>
-          <t>Shashwat Sachdev, Shahzad Ali, Subhadeep Das Chowdhury, Armaan Khan, Irshad Kamil, Roshan, Sahir Ludhianvi</t>
+          <t>Kailash Kher, Paresh Kamath, Naresh Kamath</t>
         </is>
       </c>
     </row>
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>2026-04-03</t>
+          <t>2026-04-04</t>
         </is>
       </c>
       <c r="B44" t="n">
@@ -15858,7 +16895,7 @@
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>2026-04-03</t>
+          <t>2026-04-04</t>
         </is>
       </c>
       <c r="B45" t="n">
@@ -15866,19 +16903,19 @@
       </c>
       <c r="C45" t="inlineStr">
         <is>
-          <t>Aaya Sher (From "The Paradise") (Telugu)</t>
+          <t>Main Aur Tu</t>
         </is>
       </c>
       <c r="D45" t="inlineStr">
         <is>
-          <t>Anirudh Ravichander, Jangi Reddy, Arjun Chandy, Kasarla Shyam</t>
+          <t>Shashwat Sachdev, Jasmine Sandlas, Reble</t>
         </is>
       </c>
     </row>
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>2026-04-03</t>
+          <t>2026-04-04</t>
         </is>
       </c>
       <c r="B46" t="n">
@@ -15886,19 +16923,19 @@
       </c>
       <c r="C46" t="inlineStr">
         <is>
-          <t>Not Guilty</t>
+          <t>Ehsaas</t>
         </is>
       </c>
       <c r="D46" t="inlineStr">
         <is>
-          <t>Dhanda Nyoliwala</t>
+          <t>Faheem Abdullah, Duha Shah, Vaibhav Pani, Hyder Dar</t>
         </is>
       </c>
     </row>
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>2026-04-03</t>
+          <t>2026-04-04</t>
         </is>
       </c>
       <c r="B47" t="n">
@@ -15906,19 +16943,19 @@
       </c>
       <c r="C47" t="inlineStr">
         <is>
-          <t>Teri Deewani</t>
+          <t>Aaya Sher (From "The Paradise") (Telugu)</t>
         </is>
       </c>
       <c r="D47" t="inlineStr">
         <is>
-          <t>Kailash Kher, Paresh Kamath, Naresh Kamath</t>
+          <t>Anirudh Ravichander, Jangi Reddy, Arjun Chandy, Kasarla Shyam</t>
         </is>
       </c>
     </row>
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>2026-04-03</t>
+          <t>2026-04-04</t>
         </is>
       </c>
       <c r="B48" t="n">
@@ -15926,19 +16963,19 @@
       </c>
       <c r="C48" t="inlineStr">
         <is>
-          <t>Hum Pyaar Karne Wale</t>
+          <t>Not Guilty</t>
         </is>
       </c>
       <c r="D48" t="inlineStr">
         <is>
-          <t>Shashwat Sachdev, Anuradha Paudwal, Udit Narayan, Anand-Milind, Sameer Anjaan, Qveen Herby</t>
+          <t>Dhanda Nyoliwala</t>
         </is>
       </c>
     </row>
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>2026-04-03</t>
+          <t>2026-04-04</t>
         </is>
       </c>
       <c r="B49" t="n">
@@ -15946,19 +16983,19 @@
       </c>
       <c r="C49" t="inlineStr">
         <is>
-          <t>Ehsaas</t>
+          <t>Mast Magan (From "2 States)</t>
         </is>
       </c>
       <c r="D49" t="inlineStr">
         <is>
-          <t>Faheem Abdullah, Duha Shah, Vaibhav Pani, Hyder Dar</t>
+          <t>Arijit Singh, Chinmayi</t>
         </is>
       </c>
     </row>
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>2026-04-03</t>
+          <t>2026-04-04</t>
         </is>
       </c>
       <c r="B50" t="n">
@@ -15966,19 +17003,19 @@
       </c>
       <c r="C50" t="inlineStr">
         <is>
-          <t>Vaari Jaavan</t>
+          <t>Thodi Si Daaru</t>
         </is>
       </c>
       <c r="D50" t="inlineStr">
         <is>
-          <t>Shashwat Sachdev, Jyoti Nooran, Jasmine Sandlas, Reble</t>
+          <t>AP Dhillon, Shreya Ghoshal</t>
         </is>
       </c>
     </row>
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>2026-04-03</t>
+          <t>2026-04-04</t>
         </is>
       </c>
       <c r="B51" t="n">
@@ -15986,12 +17023,12 @@
       </c>
       <c r="C51" t="inlineStr">
         <is>
-          <t>Mast Magan (From "2 States)</t>
+          <t>Zaalima</t>
         </is>
       </c>
       <c r="D51" t="inlineStr">
         <is>
-          <t>Arijit Singh, Chinmayi</t>
+          <t>Arijit Singh, Harshdeep Kaur</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
added data for 5th got predictions for 6th april
</commit_message>
<xml_diff>
--- a/Probability Project.xlsx
+++ b/Probability Project.xlsx
@@ -25,6 +25,7 @@
     <sheet name="AUTO_20260402" sheetId="20" state="visible" r:id="rId20"/>
     <sheet name="AUTO_20260403" sheetId="21" state="visible" r:id="rId21"/>
     <sheet name="AUTO_20260404" sheetId="22" state="visible" r:id="rId22"/>
+    <sheet name="AUTO_20260405" sheetId="23" state="visible" r:id="rId23"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -16033,9 +16034,1045 @@
       </c>
     </row>
     <row r="2">
+      <c r="A2" s="0" t="inlineStr">
+        <is>
+          <t>2026-04-04</t>
+        </is>
+      </c>
+      <c r="B2" s="0" t="n">
+        <v>1</v>
+      </c>
+      <c r="C2" s="0" t="inlineStr">
+        <is>
+          <t>Bairan</t>
+        </is>
+      </c>
+      <c r="D2" s="0" t="inlineStr">
+        <is>
+          <t>Banjaare</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="0" t="inlineStr">
+        <is>
+          <t>2026-04-04</t>
+        </is>
+      </c>
+      <c r="B3" s="0" t="n">
+        <v>2</v>
+      </c>
+      <c r="C3" s="0" t="inlineStr">
+        <is>
+          <t>Jaiye Sajana</t>
+        </is>
+      </c>
+      <c r="D3" s="0" t="inlineStr">
+        <is>
+          <t>Shashwat Sachdev, Jasmine Sandlas, Satinder Sartaaj</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="0" t="inlineStr">
+        <is>
+          <t>2026-04-04</t>
+        </is>
+      </c>
+      <c r="B4" s="0" t="n">
+        <v>3</v>
+      </c>
+      <c r="C4" s="0" t="inlineStr">
+        <is>
+          <t>Gehra Hua</t>
+        </is>
+      </c>
+      <c r="D4" s="0" t="inlineStr">
+        <is>
+          <t>Shashwat Sachdev, Arijit Singh, Irshad Kamil, Armaan Khan</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="0" t="inlineStr">
+        <is>
+          <t>2026-04-04</t>
+        </is>
+      </c>
+      <c r="B5" s="0" t="n">
+        <v>4</v>
+      </c>
+      <c r="C5" s="0" t="inlineStr">
+        <is>
+          <t>Sheesha - Aakhya Mai Aakh Ghali Jo Bairan</t>
+        </is>
+      </c>
+      <c r="D5" s="0" t="inlineStr">
+        <is>
+          <t>Mitta Ror, Swara Verma</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="0" t="inlineStr">
+        <is>
+          <t>2026-04-04</t>
+        </is>
+      </c>
+      <c r="B6" s="0" t="n">
+        <v>5</v>
+      </c>
+      <c r="C6" s="0" t="inlineStr">
+        <is>
+          <t>Khat</t>
+        </is>
+      </c>
+      <c r="D6" s="0" t="inlineStr">
+        <is>
+          <t>Navjot Ahuja</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="0" t="inlineStr">
+        <is>
+          <t>2026-04-04</t>
+        </is>
+      </c>
+      <c r="B7" s="0" t="n">
+        <v>6</v>
+      </c>
+      <c r="C7" s="0" t="inlineStr">
+        <is>
+          <t>Dhurandhar The Revenge - Aari Aari</t>
+        </is>
+      </c>
+      <c r="D7" s="0" t="inlineStr">
+        <is>
+          <t>Shashwat Sachdev, Bombay Rockers, Irshad Kamil, Khan Saab, Reble, Token, Jasmine Sandlas, Sudhir Yaduvanshi</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="0" t="inlineStr">
+        <is>
+          <t>2026-04-04</t>
+        </is>
+      </c>
+      <c r="B8" s="0" t="n">
+        <v>7</v>
+      </c>
+      <c r="C8" s="0" t="inlineStr">
+        <is>
+          <t>Sahiba</t>
+        </is>
+      </c>
+      <c r="D8" s="0" t="inlineStr">
+        <is>
+          <t>Aditya Rikhari</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="0" t="inlineStr">
+        <is>
+          <t>2026-04-04</t>
+        </is>
+      </c>
+      <c r="B9" s="0" t="n">
+        <v>8</v>
+      </c>
+      <c r="C9" s="0" t="inlineStr">
+        <is>
+          <t>Dooron Dooron</t>
+        </is>
+      </c>
+      <c r="D9" s="0" t="inlineStr">
+        <is>
+          <t>Paresh Pahuja, Shiv Tandan, Meghdeep Bose</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="0" t="inlineStr">
+        <is>
+          <t>2026-04-04</t>
+        </is>
+      </c>
+      <c r="B10" s="0" t="n">
+        <v>9</v>
+      </c>
+      <c r="C10" s="0" t="inlineStr">
+        <is>
+          <t>Jaan Se Guzarte Hain</t>
+        </is>
+      </c>
+      <c r="D10" s="0" t="inlineStr">
+        <is>
+          <t>Shashwat Sachdev, Khan Saab, Nusrat Fateh Ali Khan</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="0" t="inlineStr">
+        <is>
+          <t>2026-04-04</t>
+        </is>
+      </c>
+      <c r="B11" s="0" t="n">
+        <v>10</v>
+      </c>
+      <c r="C11" s="0" t="inlineStr">
+        <is>
+          <t>Apna Bana Le</t>
+        </is>
+      </c>
+      <c r="D11" s="0" t="inlineStr">
+        <is>
+          <t>Sachin-Jigar, Arijit Singh, Amitabh Bhattacharya</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="0" t="inlineStr">
+        <is>
+          <t>2026-04-04</t>
+        </is>
+      </c>
+      <c r="B12" s="0" t="n">
+        <v>11</v>
+      </c>
+      <c r="C12" s="0" t="inlineStr">
+        <is>
+          <t>Samjhawan</t>
+        </is>
+      </c>
+      <c r="D12" s="0" t="inlineStr">
+        <is>
+          <t>Jawad Ahmad, Shaarib Toshi, Arijit Singh, Shreya Ghoshal</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="0" t="inlineStr">
+        <is>
+          <t>2026-04-04</t>
+        </is>
+      </c>
+      <c r="B13" s="0" t="n">
+        <v>12</v>
+      </c>
+      <c r="C13" s="0" t="inlineStr">
+        <is>
+          <t>Sitaare (From "Ikkis")</t>
+        </is>
+      </c>
+      <c r="D13" s="0" t="inlineStr">
+        <is>
+          <t>Arijit Singh, White Noise Collectives, Amitabh Bhattacharya</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="0" t="inlineStr">
+        <is>
+          <t>2026-04-04</t>
+        </is>
+      </c>
+      <c r="B14" s="0" t="n">
+        <v>13</v>
+      </c>
+      <c r="C14" s="0" t="inlineStr">
+        <is>
+          <t>Pavazha Malli - From "Think Indie"</t>
+        </is>
+      </c>
+      <c r="D14" s="0" t="inlineStr">
+        <is>
+          <t>Sai Abhyankkar, Shruti Haasan, Vivek</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="0" t="inlineStr">
+        <is>
+          <t>2026-04-04</t>
+        </is>
+      </c>
+      <c r="B15" s="0" t="n">
+        <v>14</v>
+      </c>
+      <c r="C15" s="0" t="inlineStr">
+        <is>
+          <t>Finding Her</t>
+        </is>
+      </c>
+      <c r="D15" s="0" t="inlineStr">
+        <is>
+          <t>Kushagra, Bharath, Saaheal</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="0" t="inlineStr">
+        <is>
+          <t>2026-04-04</t>
+        </is>
+      </c>
+      <c r="B16" s="0" t="n">
+        <v>15</v>
+      </c>
+      <c r="C16" s="0" t="inlineStr">
+        <is>
+          <t>Shararat</t>
+        </is>
+      </c>
+      <c r="D16" s="0" t="inlineStr">
+        <is>
+          <t>Shashwat Sachdev, Madhubanti Bagchi, Jasmine Sandlas</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="0" t="inlineStr">
+        <is>
+          <t>2026-04-04</t>
+        </is>
+      </c>
+      <c r="B17" s="0" t="n">
+        <v>16</v>
+      </c>
+      <c r="C17" s="0" t="inlineStr">
+        <is>
+          <t>Dhurandhar - Title Track</t>
+        </is>
+      </c>
+      <c r="D17" s="0" t="inlineStr">
+        <is>
+          <t>Shashwat Sachdev, Hanumankind, Jasmine Sandlas, Sudhir Yaduvanshi, Charanjit Ahuja, Muhammad Sadiq, Ranjit Kaur, Babu Singh Maan</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="0" t="inlineStr">
+        <is>
+          <t>2026-04-04</t>
+        </is>
+      </c>
+      <c r="B18" s="0" t="n">
+        <v>17</v>
+      </c>
+      <c r="C18" s="0" t="inlineStr">
+        <is>
+          <t>Arz Kiya Hai | Coke Studio Bharat</t>
+        </is>
+      </c>
+      <c r="D18" s="0" t="inlineStr">
+        <is>
+          <t>Anuv Jain</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="0" t="inlineStr">
+        <is>
+          <t>2026-04-04</t>
+        </is>
+      </c>
+      <c r="B19" s="0" t="n">
+        <v>18</v>
+      </c>
+      <c r="C19" s="0" t="inlineStr">
+        <is>
+          <t>Boyfriend</t>
+        </is>
+      </c>
+      <c r="D19" s="0" t="inlineStr">
+        <is>
+          <t>Karan Aujla, Ikky</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="0" t="inlineStr">
+        <is>
+          <t>2026-04-04</t>
+        </is>
+      </c>
+      <c r="B20" s="0" t="n">
+        <v>19</v>
+      </c>
+      <c r="C20" s="0" t="inlineStr">
+        <is>
+          <t>Ishq</t>
+        </is>
+      </c>
+      <c r="D20" s="0" t="inlineStr">
+        <is>
+          <t>Faheem Abdullah, Rauhan Malik, Amir Ameer</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="0" t="inlineStr">
+        <is>
+          <t>2026-04-04</t>
+        </is>
+      </c>
+      <c r="B21" s="0" t="n">
+        <v>20</v>
+      </c>
+      <c r="C21" s="0" t="inlineStr">
+        <is>
+          <t>Mann Mera</t>
+        </is>
+      </c>
+      <c r="D21" s="0" t="inlineStr">
+        <is>
+          <t>Gajendra Verma</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="0" t="inlineStr">
+        <is>
+          <t>2026-04-04</t>
+        </is>
+      </c>
+      <c r="B22" s="0" t="n">
+        <v>21</v>
+      </c>
+      <c r="C22" s="0" t="inlineStr">
+        <is>
+          <t>Saiyaara</t>
+        </is>
+      </c>
+      <c r="D22" s="0" t="inlineStr">
+        <is>
+          <t>Tanishk Bagchi, Faheem Abdullah, Arslan Nizami, Irshad Kamil</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="0" t="inlineStr">
+        <is>
+          <t>2026-04-04</t>
+        </is>
+      </c>
+      <c r="B23" s="0" t="n">
+        <v>22</v>
+      </c>
+      <c r="C23" s="0" t="inlineStr">
+        <is>
+          <t>Ishqa Ve</t>
+        </is>
+      </c>
+      <c r="D23" s="0" t="inlineStr">
+        <is>
+          <t>Zeeshan Ali, Yuvraj Tung, Sandeep Aulakh, Honey Dhillon</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="0" t="inlineStr">
+        <is>
+          <t>2026-04-04</t>
+        </is>
+      </c>
+      <c r="B24" s="0" t="n">
+        <v>23</v>
+      </c>
+      <c r="C24" s="0" t="inlineStr">
+        <is>
+          <t>For A Reason</t>
+        </is>
+      </c>
+      <c r="D24" s="0" t="inlineStr">
+        <is>
+          <t>Karan Aujla, Ikky</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="0" t="inlineStr">
+        <is>
+          <t>2026-04-04</t>
+        </is>
+      </c>
+      <c r="B25" s="0" t="n">
+        <v>24</v>
+      </c>
+      <c r="C25" s="0" t="inlineStr">
+        <is>
+          <t>Tere Bina</t>
+        </is>
+      </c>
+      <c r="D25" s="0" t="inlineStr">
+        <is>
+          <t>A.R. Rahman, Chinmayi, Murtuza Khan, Qadir Khan</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="0" t="inlineStr">
+        <is>
+          <t>2026-04-04</t>
+        </is>
+      </c>
+      <c r="B26" s="0" t="n">
+        <v>25</v>
+      </c>
+      <c r="C26" s="0" t="inlineStr">
+        <is>
+          <t>Naal Nachna</t>
+        </is>
+      </c>
+      <c r="D26" s="0" t="inlineStr">
+        <is>
+          <t>Shashwat Sachdev, Afsana Khan, Irshad Kamil, Reble</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="0" t="inlineStr">
+        <is>
+          <t>2026-04-04</t>
+        </is>
+      </c>
+      <c r="B27" s="0" t="n">
+        <v>26</v>
+      </c>
+      <c r="C27" s="0" t="inlineStr">
+        <is>
+          <t>Bairi</t>
+        </is>
+      </c>
+      <c r="D27" s="0" t="inlineStr">
+        <is>
+          <t>Virat, Pradeep Solanki, Heena</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="0" t="inlineStr">
+        <is>
+          <t>2026-04-04</t>
+        </is>
+      </c>
+      <c r="B28" s="0" t="n">
+        <v>27</v>
+      </c>
+      <c r="C28" s="0" t="inlineStr">
+        <is>
+          <t>Run Down The City - Monica</t>
+        </is>
+      </c>
+      <c r="D28" s="0" t="inlineStr">
+        <is>
+          <t>Shashwat Sachdev, Reble, Asha Bhosle, R. D. Burman, Majrooh Sultanpuri</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="0" t="inlineStr">
+        <is>
+          <t>2026-04-04</t>
+        </is>
+      </c>
+      <c r="B29" s="0" t="n">
+        <v>28</v>
+      </c>
+      <c r="C29" s="0" t="inlineStr">
+        <is>
+          <t>Phir Se</t>
+        </is>
+      </c>
+      <c r="D29" s="0" t="inlineStr">
+        <is>
+          <t>Shashwat Sachdev, Arijit Singh, Irshad Kamil</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="0" t="inlineStr">
+        <is>
+          <t>2026-04-04</t>
+        </is>
+      </c>
+      <c r="B30" s="0" t="n">
+        <v>29</v>
+      </c>
+      <c r="C30" s="0" t="inlineStr">
+        <is>
+          <t>Deewaana Deewaana</t>
+        </is>
+      </c>
+      <c r="D30" s="0" t="inlineStr">
+        <is>
+          <t>A.R. Rahman, Irshad Kamil</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="0" t="inlineStr">
+        <is>
+          <t>2026-04-04</t>
+        </is>
+      </c>
+      <c r="B31" s="0" t="n">
+        <v>30</v>
+      </c>
+      <c r="C31" s="0" t="inlineStr">
+        <is>
+          <t>Tere Liye</t>
+        </is>
+      </c>
+      <c r="D31" s="0" t="inlineStr">
+        <is>
+          <t>Atif Aslam, Shreya Ghoshal, Sachin Gupta, Sameer Anjaan</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="0" t="inlineStr">
+        <is>
+          <t>2026-04-04</t>
+        </is>
+      </c>
+      <c r="B32" s="0" t="n">
+        <v>31</v>
+      </c>
+      <c r="C32" s="0" t="inlineStr">
+        <is>
+          <t>Raanjhan (From "Do Patti")</t>
+        </is>
+      </c>
+      <c r="D32" s="0" t="inlineStr">
+        <is>
+          <t>Sachet-Parampara, Parampara Tandon, Kausar Munir</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="0" t="inlineStr">
+        <is>
+          <t>2026-04-04</t>
+        </is>
+      </c>
+      <c r="B33" s="0" t="n">
+        <v>32</v>
+      </c>
+      <c r="C33" s="0" t="inlineStr">
+        <is>
+          <t>Jo Tum Mere Ho</t>
+        </is>
+      </c>
+      <c r="D33" s="0" t="inlineStr">
+        <is>
+          <t>Anuv Jain</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="0" t="inlineStr">
+        <is>
+          <t>2026-04-04</t>
+        </is>
+      </c>
+      <c r="B34" s="0" t="n">
+        <v>33</v>
+      </c>
+      <c r="C34" s="0" t="inlineStr">
+        <is>
+          <t>Tum Ho Toh (From "Saiyaara")</t>
+        </is>
+      </c>
+      <c r="D34" s="0" t="inlineStr">
+        <is>
+          <t>Vishal Mishra, Hansika Pareek, Raj Shekhar</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="0" t="inlineStr">
+        <is>
+          <t>2026-04-04</t>
+        </is>
+      </c>
+      <c r="B35" s="0" t="n">
+        <v>34</v>
+      </c>
+      <c r="C35" s="0" t="inlineStr">
+        <is>
+          <t>Haseen</t>
+        </is>
+      </c>
+      <c r="D35" s="0" t="inlineStr">
+        <is>
+          <t>Talwiinder, NDS, Rippy Grewal</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="0" t="inlineStr">
+        <is>
+          <t>2026-04-04</t>
+        </is>
+      </c>
+      <c r="B36" s="0" t="n">
+        <v>35</v>
+      </c>
+      <c r="C36" s="0" t="inlineStr">
+        <is>
+          <t>Darkhaast</t>
+        </is>
+      </c>
+      <c r="D36" s="0" t="inlineStr">
+        <is>
+          <t>Mithoon, Arijit Singh, Sunidhi Chauhan, Sayeed Quadri</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="0" t="inlineStr">
+        <is>
+          <t>2026-04-04</t>
+        </is>
+      </c>
+      <c r="B37" s="0" t="n">
+        <v>36</v>
+      </c>
+      <c r="C37" s="0" t="inlineStr">
+        <is>
+          <t>Lutt Le Gaya</t>
+        </is>
+      </c>
+      <c r="D37" s="0" t="inlineStr">
+        <is>
+          <t>Shashwat Sachdev, Simran Choudhary</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="0" t="inlineStr">
+        <is>
+          <t>2026-04-04</t>
+        </is>
+      </c>
+      <c r="B38" s="0" t="n">
+        <v>37</v>
+      </c>
+      <c r="C38" s="0" t="inlineStr">
+        <is>
+          <t>Ye Tune Kya Kiya</t>
+        </is>
+      </c>
+      <c r="D38" s="0" t="inlineStr">
+        <is>
+          <t>Pritam, Javed Bashir, Rajat Arora</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="0" t="inlineStr">
+        <is>
+          <t>2026-04-04</t>
+        </is>
+      </c>
+      <c r="B39" s="0" t="n">
+        <v>38</v>
+      </c>
+      <c r="C39" s="0" t="inlineStr">
+        <is>
+          <t>Mann Mera - Original Version</t>
+        </is>
+      </c>
+      <c r="D39" s="0" t="inlineStr">
+        <is>
+          <t>Gajendra Verma</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="0" t="inlineStr">
+        <is>
+          <t>2026-04-04</t>
+        </is>
+      </c>
+      <c r="B40" s="0" t="n">
+        <v>39</v>
+      </c>
+      <c r="C40" s="0" t="inlineStr">
+        <is>
+          <t>Agar Tum Saath Ho (From "Tamasha")</t>
+        </is>
+      </c>
+      <c r="D40" s="0" t="inlineStr">
+        <is>
+          <t>Alka Yagnik, Arijit Singh</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" s="0" t="inlineStr">
+        <is>
+          <t>2026-04-04</t>
+        </is>
+      </c>
+      <c r="B41" s="0" t="n">
+        <v>40</v>
+      </c>
+      <c r="C41" s="0" t="inlineStr">
+        <is>
+          <t>Ishq Jalakar - Karvaan</t>
+        </is>
+      </c>
+      <c r="D41" s="0" t="inlineStr">
+        <is>
+          <t>Shashwat Sachdev, Shahzad Ali, Subhadeep Das Chowdhury, Armaan Khan, Irshad Kamil, Roshan, Sahir Ludhianvi</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" s="0" t="inlineStr">
+        <is>
+          <t>2026-04-04</t>
+        </is>
+      </c>
+      <c r="B42" s="0" t="n">
+        <v>41</v>
+      </c>
+      <c r="C42" s="0" t="inlineStr">
+        <is>
+          <t>Mutta Kalakki (From "Youth")</t>
+        </is>
+      </c>
+      <c r="D42" s="0" t="inlineStr">
+        <is>
+          <t>G. V. Prakash, Ken Karunaas</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" s="0" t="inlineStr">
+        <is>
+          <t>2026-04-04</t>
+        </is>
+      </c>
+      <c r="B43" s="0" t="n">
+        <v>42</v>
+      </c>
+      <c r="C43" s="0" t="inlineStr">
+        <is>
+          <t>Teri Deewani</t>
+        </is>
+      </c>
+      <c r="D43" s="0" t="inlineStr">
+        <is>
+          <t>Kailash Kher, Paresh Kamath, Naresh Kamath</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" s="0" t="inlineStr">
+        <is>
+          <t>2026-04-04</t>
+        </is>
+      </c>
+      <c r="B44" s="0" t="n">
+        <v>43</v>
+      </c>
+      <c r="C44" s="0" t="inlineStr">
+        <is>
+          <t>Barbaad (From "Saiyaara")</t>
+        </is>
+      </c>
+      <c r="D44" s="0" t="inlineStr">
+        <is>
+          <t>The Rish, Jubin Nautiyal</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" s="0" t="inlineStr">
+        <is>
+          <t>2026-04-04</t>
+        </is>
+      </c>
+      <c r="B45" s="0" t="n">
+        <v>44</v>
+      </c>
+      <c r="C45" s="0" t="inlineStr">
+        <is>
+          <t>Main Aur Tu</t>
+        </is>
+      </c>
+      <c r="D45" s="0" t="inlineStr">
+        <is>
+          <t>Shashwat Sachdev, Jasmine Sandlas, Reble</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" s="0" t="inlineStr">
+        <is>
+          <t>2026-04-04</t>
+        </is>
+      </c>
+      <c r="B46" s="0" t="n">
+        <v>45</v>
+      </c>
+      <c r="C46" s="0" t="inlineStr">
+        <is>
+          <t>Ehsaas</t>
+        </is>
+      </c>
+      <c r="D46" s="0" t="inlineStr">
+        <is>
+          <t>Faheem Abdullah, Duha Shah, Vaibhav Pani, Hyder Dar</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" s="0" t="inlineStr">
+        <is>
+          <t>2026-04-04</t>
+        </is>
+      </c>
+      <c r="B47" s="0" t="n">
+        <v>46</v>
+      </c>
+      <c r="C47" s="0" t="inlineStr">
+        <is>
+          <t>Aaya Sher (From "The Paradise") (Telugu)</t>
+        </is>
+      </c>
+      <c r="D47" s="0" t="inlineStr">
+        <is>
+          <t>Anirudh Ravichander, Jangi Reddy, Arjun Chandy, Kasarla Shyam</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" s="0" t="inlineStr">
+        <is>
+          <t>2026-04-04</t>
+        </is>
+      </c>
+      <c r="B48" s="0" t="n">
+        <v>47</v>
+      </c>
+      <c r="C48" s="0" t="inlineStr">
+        <is>
+          <t>Not Guilty</t>
+        </is>
+      </c>
+      <c r="D48" s="0" t="inlineStr">
+        <is>
+          <t>Dhanda Nyoliwala</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" s="0" t="inlineStr">
+        <is>
+          <t>2026-04-04</t>
+        </is>
+      </c>
+      <c r="B49" s="0" t="n">
+        <v>48</v>
+      </c>
+      <c r="C49" s="0" t="inlineStr">
+        <is>
+          <t>Mast Magan (From "2 States)</t>
+        </is>
+      </c>
+      <c r="D49" s="0" t="inlineStr">
+        <is>
+          <t>Arijit Singh, Chinmayi</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" s="0" t="inlineStr">
+        <is>
+          <t>2026-04-04</t>
+        </is>
+      </c>
+      <c r="B50" s="0" t="n">
+        <v>49</v>
+      </c>
+      <c r="C50" s="0" t="inlineStr">
+        <is>
+          <t>Thodi Si Daaru</t>
+        </is>
+      </c>
+      <c r="D50" s="0" t="inlineStr">
+        <is>
+          <t>AP Dhillon, Shreya Ghoshal</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" s="0" t="inlineStr">
+        <is>
+          <t>2026-04-04</t>
+        </is>
+      </c>
+      <c r="B51" s="0" t="n">
+        <v>50</v>
+      </c>
+      <c r="C51" s="0" t="inlineStr">
+        <is>
+          <t>Zaalima</t>
+        </is>
+      </c>
+      <c r="D51" s="0" t="inlineStr">
+        <is>
+          <t>Arijit Singh, Harshdeep Kaur</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet23.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:D51"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="24" t="inlineStr">
+        <is>
+          <t>Date</t>
+        </is>
+      </c>
+      <c r="B1" s="24" t="inlineStr">
+        <is>
+          <t>Rank</t>
+        </is>
+      </c>
+      <c r="C1" s="24" t="inlineStr">
+        <is>
+          <t>Song</t>
+        </is>
+      </c>
+      <c r="D1" s="24" t="inlineStr">
+        <is>
+          <t>Artist</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>2026-04-04</t>
+          <t>2026-04-05</t>
         </is>
       </c>
       <c r="B2" t="n">
@@ -16055,7 +17092,7 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>2026-04-04</t>
+          <t>2026-04-05</t>
         </is>
       </c>
       <c r="B3" t="n">
@@ -16068,14 +17105,14 @@
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>Shashwat Sachdev, Jasmine Sandlas, Satinder Sartaaj</t>
+          <t>Shashwat Sachdev</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>2026-04-04</t>
+          <t>2026-04-05</t>
         </is>
       </c>
       <c r="B4" t="n">
@@ -16088,14 +17125,14 @@
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>Shashwat Sachdev, Arijit Singh, Irshad Kamil, Armaan Khan</t>
+          <t>Shashwat Sachdev</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>2026-04-04</t>
+          <t>2026-04-05</t>
         </is>
       </c>
       <c r="B5" t="n">
@@ -16108,14 +17145,14 @@
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>Mitta Ror, Swara Verma</t>
+          <t>Mitta Ror</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>2026-04-04</t>
+          <t>2026-04-05</t>
         </is>
       </c>
       <c r="B6" t="n">
@@ -16135,7 +17172,7 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>2026-04-04</t>
+          <t>2026-04-05</t>
         </is>
       </c>
       <c r="B7" t="n">
@@ -16148,14 +17185,14 @@
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>Shashwat Sachdev, Bombay Rockers, Irshad Kamil, Khan Saab, Reble, Token, Jasmine Sandlas, Sudhir Yaduvanshi</t>
+          <t>Shashwat Sachdev</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>2026-04-04</t>
+          <t>2026-04-05</t>
         </is>
       </c>
       <c r="B8" t="n">
@@ -16175,7 +17212,7 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>2026-04-04</t>
+          <t>2026-04-05</t>
         </is>
       </c>
       <c r="B9" t="n">
@@ -16188,14 +17225,14 @@
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>Paresh Pahuja, Shiv Tandan, Meghdeep Bose</t>
+          <t>Paresh Pahuja</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>2026-04-04</t>
+          <t>2026-04-05</t>
         </is>
       </c>
       <c r="B10" t="n">
@@ -16203,19 +17240,19 @@
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>Jaan Se Guzarte Hain</t>
+          <t>Sitaare</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>Shashwat Sachdev, Khan Saab, Nusrat Fateh Ali Khan</t>
+          <t>Arijit Singh</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>2026-04-04</t>
+          <t>2026-04-05</t>
         </is>
       </c>
       <c r="B11" t="n">
@@ -16228,14 +17265,14 @@
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>Sachin-Jigar, Arijit Singh, Amitabh Bhattacharya</t>
+          <t>Sachin-Jigar</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>2026-04-04</t>
+          <t>2026-04-05</t>
         </is>
       </c>
       <c r="B12" t="n">
@@ -16243,19 +17280,19 @@
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>Samjhawan</t>
+          <t>Jaan Se Guzarte Hain</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>Jawad Ahmad, Shaarib Toshi, Arijit Singh, Shreya Ghoshal</t>
+          <t>Shashwat Sachdev</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>2026-04-04</t>
+          <t>2026-04-05</t>
         </is>
       </c>
       <c r="B13" t="n">
@@ -16263,19 +17300,19 @@
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>Sitaare (From "Ikkis")</t>
+          <t>Pavazha Malli</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>Arijit Singh, White Noise Collectives, Amitabh Bhattacharya</t>
+          <t>Sai Abhyankkar</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>2026-04-04</t>
+          <t>2026-04-05</t>
         </is>
       </c>
       <c r="B14" t="n">
@@ -16283,19 +17320,19 @@
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>Pavazha Malli - From "Think Indie"</t>
+          <t>Finding Her</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>Sai Abhyankkar, Shruti Haasan, Vivek</t>
+          <t>Kushagra</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>2026-04-04</t>
+          <t>2026-04-05</t>
         </is>
       </c>
       <c r="B15" t="n">
@@ -16303,19 +17340,19 @@
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>Finding Her</t>
+          <t>Samjhawan</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>Kushagra, Bharath, Saaheal</t>
+          <t>Jawad Ahmad</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>2026-04-04</t>
+          <t>2026-04-05</t>
         </is>
       </c>
       <c r="B16" t="n">
@@ -16328,14 +17365,14 @@
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>Shashwat Sachdev, Madhubanti Bagchi, Jasmine Sandlas</t>
+          <t>Shashwat Sachdev</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>2026-04-04</t>
+          <t>2026-04-05</t>
         </is>
       </c>
       <c r="B17" t="n">
@@ -16343,19 +17380,19 @@
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>Dhurandhar - Title Track</t>
+          <t>Arz Kiya Hai | Coke Studio Bharat</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>Shashwat Sachdev, Hanumankind, Jasmine Sandlas, Sudhir Yaduvanshi, Charanjit Ahuja, Muhammad Sadiq, Ranjit Kaur, Babu Singh Maan</t>
+          <t>Anuv Jain</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>2026-04-04</t>
+          <t>2026-04-05</t>
         </is>
       </c>
       <c r="B18" t="n">
@@ -16363,19 +17400,19 @@
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>Arz Kiya Hai | Coke Studio Bharat</t>
+          <t>Boyfriend</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>Anuv Jain</t>
+          <t>Karan Aujla</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>2026-04-04</t>
+          <t>2026-04-05</t>
         </is>
       </c>
       <c r="B19" t="n">
@@ -16383,19 +17420,19 @@
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>Boyfriend</t>
+          <t>Dhurandhar - Title Track</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>Karan Aujla, Ikky</t>
+          <t>Shashwat Sachdev</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>2026-04-04</t>
+          <t>2026-04-05</t>
         </is>
       </c>
       <c r="B20" t="n">
@@ -16408,14 +17445,14 @@
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>Faheem Abdullah, Rauhan Malik, Amir Ameer</t>
+          <t>Faheem Abdullah</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>2026-04-04</t>
+          <t>2026-04-05</t>
         </is>
       </c>
       <c r="B21" t="n">
@@ -16435,7 +17472,7 @@
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>2026-04-04</t>
+          <t>2026-04-05</t>
         </is>
       </c>
       <c r="B22" t="n">
@@ -16448,14 +17485,14 @@
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>Tanishk Bagchi, Faheem Abdullah, Arslan Nizami, Irshad Kamil</t>
+          <t>Tanishk Bagchi</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>2026-04-04</t>
+          <t>2026-04-05</t>
         </is>
       </c>
       <c r="B23" t="n">
@@ -16463,19 +17500,19 @@
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>Ishqa Ve</t>
+          <t>For A Reason</t>
         </is>
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>Zeeshan Ali, Yuvraj Tung, Sandeep Aulakh, Honey Dhillon</t>
+          <t>Karan Aujla</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>2026-04-04</t>
+          <t>2026-04-05</t>
         </is>
       </c>
       <c r="B24" t="n">
@@ -16483,19 +17520,19 @@
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>For A Reason</t>
+          <t>Bairi</t>
         </is>
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>Karan Aujla, Ikky</t>
+          <t>Virat</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>2026-04-04</t>
+          <t>2026-04-05</t>
         </is>
       </c>
       <c r="B25" t="n">
@@ -16503,19 +17540,19 @@
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>Tere Bina</t>
+          <t>Deewaana Deewaana</t>
         </is>
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>A.R. Rahman, Chinmayi, Murtuza Khan, Qadir Khan</t>
+          <t>A.R. Rahman</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>2026-04-04</t>
+          <t>2026-04-05</t>
         </is>
       </c>
       <c r="B26" t="n">
@@ -16523,19 +17560,19 @@
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>Naal Nachna</t>
+          <t>Raanjhan</t>
         </is>
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>Shashwat Sachdev, Afsana Khan, Irshad Kamil, Reble</t>
+          <t>Sachet-Parampara</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>2026-04-04</t>
+          <t>2026-04-05</t>
         </is>
       </c>
       <c r="B27" t="n">
@@ -16543,19 +17580,19 @@
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>Bairi</t>
+          <t>Naal Nachna</t>
         </is>
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t>Virat, Pradeep Solanki, Heena</t>
+          <t>Shashwat Sachdev</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>2026-04-04</t>
+          <t>2026-04-05</t>
         </is>
       </c>
       <c r="B28" t="n">
@@ -16563,19 +17600,19 @@
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>Run Down The City - Monica</t>
+          <t>Ishqa Ve</t>
         </is>
       </c>
       <c r="D28" t="inlineStr">
         <is>
-          <t>Shashwat Sachdev, Reble, Asha Bhosle, R. D. Burman, Majrooh Sultanpuri</t>
+          <t>Zeeshan Ali</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>2026-04-04</t>
+          <t>2026-04-05</t>
         </is>
       </c>
       <c r="B29" t="n">
@@ -16588,14 +17625,14 @@
       </c>
       <c r="D29" t="inlineStr">
         <is>
-          <t>Shashwat Sachdev, Arijit Singh, Irshad Kamil</t>
+          <t>Shashwat Sachdev</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>2026-04-04</t>
+          <t>2026-04-05</t>
         </is>
       </c>
       <c r="B30" t="n">
@@ -16603,19 +17640,19 @@
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>Deewaana Deewaana</t>
+          <t>Tum Ho Toh</t>
         </is>
       </c>
       <c r="D30" t="inlineStr">
         <is>
-          <t>A.R. Rahman, Irshad Kamil</t>
+          <t>Vishal Mishra</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>2026-04-04</t>
+          <t>2026-04-05</t>
         </is>
       </c>
       <c r="B31" t="n">
@@ -16628,14 +17665,14 @@
       </c>
       <c r="D31" t="inlineStr">
         <is>
-          <t>Atif Aslam, Shreya Ghoshal, Sachin Gupta, Sameer Anjaan</t>
+          <t>Atif Aslam</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>2026-04-04</t>
+          <t>2026-04-05</t>
         </is>
       </c>
       <c r="B32" t="n">
@@ -16643,19 +17680,19 @@
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>Raanjhan (From "Do Patti")</t>
+          <t>Darkhaast</t>
         </is>
       </c>
       <c r="D32" t="inlineStr">
         <is>
-          <t>Sachet-Parampara, Parampara Tandon, Kausar Munir</t>
+          <t>Mithoon</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>2026-04-04</t>
+          <t>2026-04-05</t>
         </is>
       </c>
       <c r="B33" t="n">
@@ -16663,19 +17700,19 @@
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>Jo Tum Mere Ho</t>
+          <t>Run Down The City - Monica</t>
         </is>
       </c>
       <c r="D33" t="inlineStr">
         <is>
-          <t>Anuv Jain</t>
+          <t>Shashwat Sachdev</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>2026-04-04</t>
+          <t>2026-04-05</t>
         </is>
       </c>
       <c r="B34" t="n">
@@ -16683,19 +17720,19 @@
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>Tum Ho Toh (From "Saiyaara")</t>
+          <t>Lutt Le Gaya</t>
         </is>
       </c>
       <c r="D34" t="inlineStr">
         <is>
-          <t>Vishal Mishra, Hansika Pareek, Raj Shekhar</t>
+          <t>Shashwat Sachdev</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>2026-04-04</t>
+          <t>2026-04-05</t>
         </is>
       </c>
       <c r="B35" t="n">
@@ -16708,14 +17745,14 @@
       </c>
       <c r="D35" t="inlineStr">
         <is>
-          <t>Talwiinder, NDS, Rippy Grewal</t>
+          <t>Talwiinder</t>
         </is>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>2026-04-04</t>
+          <t>2026-04-05</t>
         </is>
       </c>
       <c r="B36" t="n">
@@ -16723,19 +17760,19 @@
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>Darkhaast</t>
+          <t>Jo Tum Mere Ho</t>
         </is>
       </c>
       <c r="D36" t="inlineStr">
         <is>
-          <t>Mithoon, Arijit Singh, Sunidhi Chauhan, Sayeed Quadri</t>
+          <t>Anuv Jain</t>
         </is>
       </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>2026-04-04</t>
+          <t>2026-04-05</t>
         </is>
       </c>
       <c r="B37" t="n">
@@ -16743,19 +17780,19 @@
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>Lutt Le Gaya</t>
+          <t>Tere Bina</t>
         </is>
       </c>
       <c r="D37" t="inlineStr">
         <is>
-          <t>Shashwat Sachdev, Simran Choudhary</t>
+          <t>A.R. Rahman</t>
         </is>
       </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>2026-04-04</t>
+          <t>2026-04-05</t>
         </is>
       </c>
       <c r="B38" t="n">
@@ -16763,19 +17800,19 @@
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>Ye Tune Kya Kiya</t>
+          <t>Agar Tum Saath Ho</t>
         </is>
       </c>
       <c r="D38" t="inlineStr">
         <is>
-          <t>Pritam, Javed Bashir, Rajat Arora</t>
+          <t>Alka Yagnik</t>
         </is>
       </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>2026-04-04</t>
+          <t>2026-04-05</t>
         </is>
       </c>
       <c r="B39" t="n">
@@ -16783,19 +17820,19 @@
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>Mann Mera - Original Version</t>
+          <t>Barbaad</t>
         </is>
       </c>
       <c r="D39" t="inlineStr">
         <is>
-          <t>Gajendra Verma</t>
+          <t>The Rish</t>
         </is>
       </c>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>2026-04-04</t>
+          <t>2026-04-05</t>
         </is>
       </c>
       <c r="B40" t="n">
@@ -16803,19 +17840,19 @@
       </c>
       <c r="C40" t="inlineStr">
         <is>
-          <t>Agar Tum Saath Ho (From "Tamasha")</t>
+          <t>Mutta Kalakki</t>
         </is>
       </c>
       <c r="D40" t="inlineStr">
         <is>
-          <t>Alka Yagnik, Arijit Singh</t>
+          <t>G. V. Prakash</t>
         </is>
       </c>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>2026-04-04</t>
+          <t>2026-04-05</t>
         </is>
       </c>
       <c r="B41" t="n">
@@ -16828,14 +17865,14 @@
       </c>
       <c r="D41" t="inlineStr">
         <is>
-          <t>Shashwat Sachdev, Shahzad Ali, Subhadeep Das Chowdhury, Armaan Khan, Irshad Kamil, Roshan, Sahir Ludhianvi</t>
+          <t>Shashwat Sachdev</t>
         </is>
       </c>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>2026-04-04</t>
+          <t>2026-04-05</t>
         </is>
       </c>
       <c r="B42" t="n">
@@ -16843,19 +17880,19 @@
       </c>
       <c r="C42" t="inlineStr">
         <is>
-          <t>Mutta Kalakki (From "Youth")</t>
+          <t>Teri Deewani</t>
         </is>
       </c>
       <c r="D42" t="inlineStr">
         <is>
-          <t>G. V. Prakash, Ken Karunaas</t>
+          <t>Kailash Kher</t>
         </is>
       </c>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>2026-04-04</t>
+          <t>2026-04-05</t>
         </is>
       </c>
       <c r="B43" t="n">
@@ -16863,19 +17900,19 @@
       </c>
       <c r="C43" t="inlineStr">
         <is>
-          <t>Teri Deewani</t>
+          <t>Mann Mera - Original Version</t>
         </is>
       </c>
       <c r="D43" t="inlineStr">
         <is>
-          <t>Kailash Kher, Paresh Kamath, Naresh Kamath</t>
+          <t>Gajendra Verma</t>
         </is>
       </c>
     </row>
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>2026-04-04</t>
+          <t>2026-04-05</t>
         </is>
       </c>
       <c r="B44" t="n">
@@ -16883,19 +17920,19 @@
       </c>
       <c r="C44" t="inlineStr">
         <is>
-          <t>Barbaad (From "Saiyaara")</t>
+          <t>Ye Tune Kya Kiya</t>
         </is>
       </c>
       <c r="D44" t="inlineStr">
         <is>
-          <t>The Rish, Jubin Nautiyal</t>
+          <t>Pritam</t>
         </is>
       </c>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>2026-04-04</t>
+          <t>2026-04-05</t>
         </is>
       </c>
       <c r="B45" t="n">
@@ -16903,19 +17940,19 @@
       </c>
       <c r="C45" t="inlineStr">
         <is>
-          <t>Main Aur Tu</t>
+          <t>Ehsaas</t>
         </is>
       </c>
       <c r="D45" t="inlineStr">
         <is>
-          <t>Shashwat Sachdev, Jasmine Sandlas, Reble</t>
+          <t>Faheem Abdullah</t>
         </is>
       </c>
     </row>
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>2026-04-04</t>
+          <t>2026-04-05</t>
         </is>
       </c>
       <c r="B46" t="n">
@@ -16923,19 +17960,19 @@
       </c>
       <c r="C46" t="inlineStr">
         <is>
-          <t>Ehsaas</t>
+          <t>Aaya Sher</t>
         </is>
       </c>
       <c r="D46" t="inlineStr">
         <is>
-          <t>Faheem Abdullah, Duha Shah, Vaibhav Pani, Hyder Dar</t>
+          <t>Anirudh Ravichander</t>
         </is>
       </c>
     </row>
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>2026-04-04</t>
+          <t>2026-04-05</t>
         </is>
       </c>
       <c r="B47" t="n">
@@ -16943,19 +17980,19 @@
       </c>
       <c r="C47" t="inlineStr">
         <is>
-          <t>Aaya Sher (From "The Paradise") (Telugu)</t>
+          <t>Main Aur Tu</t>
         </is>
       </c>
       <c r="D47" t="inlineStr">
         <is>
-          <t>Anirudh Ravichander, Jangi Reddy, Arjun Chandy, Kasarla Shyam</t>
+          <t>Shashwat Sachdev</t>
         </is>
       </c>
     </row>
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>2026-04-04</t>
+          <t>2026-04-05</t>
         </is>
       </c>
       <c r="B48" t="n">
@@ -16975,7 +18012,7 @@
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>2026-04-04</t>
+          <t>2026-04-05</t>
         </is>
       </c>
       <c r="B49" t="n">
@@ -16983,19 +18020,19 @@
       </c>
       <c r="C49" t="inlineStr">
         <is>
-          <t>Mast Magan (From "2 States)</t>
+          <t>Dhun</t>
         </is>
       </c>
       <c r="D49" t="inlineStr">
         <is>
-          <t>Arijit Singh, Chinmayi</t>
+          <t>Mithoon</t>
         </is>
       </c>
     </row>
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>2026-04-04</t>
+          <t>2026-04-05</t>
         </is>
       </c>
       <c r="B50" t="n">
@@ -17003,19 +18040,19 @@
       </c>
       <c r="C50" t="inlineStr">
         <is>
-          <t>Thodi Si Daaru</t>
+          <t>Zaalima</t>
         </is>
       </c>
       <c r="D50" t="inlineStr">
         <is>
-          <t>AP Dhillon, Shreya Ghoshal</t>
+          <t>Arijit Singh</t>
         </is>
       </c>
     </row>
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>2026-04-04</t>
+          <t>2026-04-05</t>
         </is>
       </c>
       <c r="B51" t="n">
@@ -17023,12 +18060,12 @@
       </c>
       <c r="C51" t="inlineStr">
         <is>
-          <t>Zaalima</t>
+          <t>Humdard</t>
         </is>
       </c>
       <c r="D51" t="inlineStr">
         <is>
-          <t>Arijit Singh, Harshdeep Kaur</t>
+          <t>Arijit Singh</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
added data for 6th got predictions for 7th april
</commit_message>
<xml_diff>
--- a/Probability Project.xlsx
+++ b/Probability Project.xlsx
@@ -26,6 +26,7 @@
     <sheet name="AUTO_20260403" sheetId="21" state="visible" r:id="rId21"/>
     <sheet name="AUTO_20260404" sheetId="22" state="visible" r:id="rId22"/>
     <sheet name="AUTO_20260405" sheetId="23" state="visible" r:id="rId23"/>
+    <sheet name="AUTO_20260406" sheetId="24" state="visible" r:id="rId24"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -17070,9 +17071,1045 @@
       </c>
     </row>
     <row r="2">
+      <c r="A2" s="0" t="inlineStr">
+        <is>
+          <t>2026-04-05</t>
+        </is>
+      </c>
+      <c r="B2" s="0" t="n">
+        <v>1</v>
+      </c>
+      <c r="C2" s="0" t="inlineStr">
+        <is>
+          <t>Bairan</t>
+        </is>
+      </c>
+      <c r="D2" s="0" t="inlineStr">
+        <is>
+          <t>Banjaare</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="0" t="inlineStr">
+        <is>
+          <t>2026-04-05</t>
+        </is>
+      </c>
+      <c r="B3" s="0" t="n">
+        <v>2</v>
+      </c>
+      <c r="C3" s="0" t="inlineStr">
+        <is>
+          <t>Jaiye Sajana</t>
+        </is>
+      </c>
+      <c r="D3" s="0" t="inlineStr">
+        <is>
+          <t>Shashwat Sachdev</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="0" t="inlineStr">
+        <is>
+          <t>2026-04-05</t>
+        </is>
+      </c>
+      <c r="B4" s="0" t="n">
+        <v>3</v>
+      </c>
+      <c r="C4" s="0" t="inlineStr">
+        <is>
+          <t>Gehra Hua</t>
+        </is>
+      </c>
+      <c r="D4" s="0" t="inlineStr">
+        <is>
+          <t>Shashwat Sachdev</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="0" t="inlineStr">
+        <is>
+          <t>2026-04-05</t>
+        </is>
+      </c>
+      <c r="B5" s="0" t="n">
+        <v>4</v>
+      </c>
+      <c r="C5" s="0" t="inlineStr">
+        <is>
+          <t>Sheesha - Aakhya Mai Aakh Ghali Jo Bairan</t>
+        </is>
+      </c>
+      <c r="D5" s="0" t="inlineStr">
+        <is>
+          <t>Mitta Ror</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="0" t="inlineStr">
+        <is>
+          <t>2026-04-05</t>
+        </is>
+      </c>
+      <c r="B6" s="0" t="n">
+        <v>5</v>
+      </c>
+      <c r="C6" s="0" t="inlineStr">
+        <is>
+          <t>Khat</t>
+        </is>
+      </c>
+      <c r="D6" s="0" t="inlineStr">
+        <is>
+          <t>Navjot Ahuja</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="0" t="inlineStr">
+        <is>
+          <t>2026-04-05</t>
+        </is>
+      </c>
+      <c r="B7" s="0" t="n">
+        <v>6</v>
+      </c>
+      <c r="C7" s="0" t="inlineStr">
+        <is>
+          <t>Dhurandhar The Revenge - Aari Aari</t>
+        </is>
+      </c>
+      <c r="D7" s="0" t="inlineStr">
+        <is>
+          <t>Shashwat Sachdev</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="0" t="inlineStr">
+        <is>
+          <t>2026-04-05</t>
+        </is>
+      </c>
+      <c r="B8" s="0" t="n">
+        <v>7</v>
+      </c>
+      <c r="C8" s="0" t="inlineStr">
+        <is>
+          <t>Sahiba</t>
+        </is>
+      </c>
+      <c r="D8" s="0" t="inlineStr">
+        <is>
+          <t>Aditya Rikhari</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="0" t="inlineStr">
+        <is>
+          <t>2026-04-05</t>
+        </is>
+      </c>
+      <c r="B9" s="0" t="n">
+        <v>8</v>
+      </c>
+      <c r="C9" s="0" t="inlineStr">
+        <is>
+          <t>Dooron Dooron</t>
+        </is>
+      </c>
+      <c r="D9" s="0" t="inlineStr">
+        <is>
+          <t>Paresh Pahuja</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="0" t="inlineStr">
+        <is>
+          <t>2026-04-05</t>
+        </is>
+      </c>
+      <c r="B10" s="0" t="n">
+        <v>9</v>
+      </c>
+      <c r="C10" s="0" t="inlineStr">
+        <is>
+          <t>Sitaare</t>
+        </is>
+      </c>
+      <c r="D10" s="0" t="inlineStr">
+        <is>
+          <t>Arijit Singh</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="0" t="inlineStr">
+        <is>
+          <t>2026-04-05</t>
+        </is>
+      </c>
+      <c r="B11" s="0" t="n">
+        <v>10</v>
+      </c>
+      <c r="C11" s="0" t="inlineStr">
+        <is>
+          <t>Apna Bana Le</t>
+        </is>
+      </c>
+      <c r="D11" s="0" t="inlineStr">
+        <is>
+          <t>Sachin-Jigar</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="0" t="inlineStr">
+        <is>
+          <t>2026-04-05</t>
+        </is>
+      </c>
+      <c r="B12" s="0" t="n">
+        <v>11</v>
+      </c>
+      <c r="C12" s="0" t="inlineStr">
+        <is>
+          <t>Jaan Se Guzarte Hain</t>
+        </is>
+      </c>
+      <c r="D12" s="0" t="inlineStr">
+        <is>
+          <t>Shashwat Sachdev</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="0" t="inlineStr">
+        <is>
+          <t>2026-04-05</t>
+        </is>
+      </c>
+      <c r="B13" s="0" t="n">
+        <v>12</v>
+      </c>
+      <c r="C13" s="0" t="inlineStr">
+        <is>
+          <t>Pavazha Malli</t>
+        </is>
+      </c>
+      <c r="D13" s="0" t="inlineStr">
+        <is>
+          <t>Sai Abhyankkar</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="0" t="inlineStr">
+        <is>
+          <t>2026-04-05</t>
+        </is>
+      </c>
+      <c r="B14" s="0" t="n">
+        <v>13</v>
+      </c>
+      <c r="C14" s="0" t="inlineStr">
+        <is>
+          <t>Finding Her</t>
+        </is>
+      </c>
+      <c r="D14" s="0" t="inlineStr">
+        <is>
+          <t>Kushagra</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="0" t="inlineStr">
+        <is>
+          <t>2026-04-05</t>
+        </is>
+      </c>
+      <c r="B15" s="0" t="n">
+        <v>14</v>
+      </c>
+      <c r="C15" s="0" t="inlineStr">
+        <is>
+          <t>Samjhawan</t>
+        </is>
+      </c>
+      <c r="D15" s="0" t="inlineStr">
+        <is>
+          <t>Jawad Ahmad</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="0" t="inlineStr">
+        <is>
+          <t>2026-04-05</t>
+        </is>
+      </c>
+      <c r="B16" s="0" t="n">
+        <v>15</v>
+      </c>
+      <c r="C16" s="0" t="inlineStr">
+        <is>
+          <t>Shararat</t>
+        </is>
+      </c>
+      <c r="D16" s="0" t="inlineStr">
+        <is>
+          <t>Shashwat Sachdev</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="0" t="inlineStr">
+        <is>
+          <t>2026-04-05</t>
+        </is>
+      </c>
+      <c r="B17" s="0" t="n">
+        <v>16</v>
+      </c>
+      <c r="C17" s="0" t="inlineStr">
+        <is>
+          <t>Arz Kiya Hai | Coke Studio Bharat</t>
+        </is>
+      </c>
+      <c r="D17" s="0" t="inlineStr">
+        <is>
+          <t>Anuv Jain</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="0" t="inlineStr">
+        <is>
+          <t>2026-04-05</t>
+        </is>
+      </c>
+      <c r="B18" s="0" t="n">
+        <v>17</v>
+      </c>
+      <c r="C18" s="0" t="inlineStr">
+        <is>
+          <t>Boyfriend</t>
+        </is>
+      </c>
+      <c r="D18" s="0" t="inlineStr">
+        <is>
+          <t>Karan Aujla</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="0" t="inlineStr">
+        <is>
+          <t>2026-04-05</t>
+        </is>
+      </c>
+      <c r="B19" s="0" t="n">
+        <v>18</v>
+      </c>
+      <c r="C19" s="0" t="inlineStr">
+        <is>
+          <t>Dhurandhar - Title Track</t>
+        </is>
+      </c>
+      <c r="D19" s="0" t="inlineStr">
+        <is>
+          <t>Shashwat Sachdev</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="0" t="inlineStr">
+        <is>
+          <t>2026-04-05</t>
+        </is>
+      </c>
+      <c r="B20" s="0" t="n">
+        <v>19</v>
+      </c>
+      <c r="C20" s="0" t="inlineStr">
+        <is>
+          <t>Ishq</t>
+        </is>
+      </c>
+      <c r="D20" s="0" t="inlineStr">
+        <is>
+          <t>Faheem Abdullah</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="0" t="inlineStr">
+        <is>
+          <t>2026-04-05</t>
+        </is>
+      </c>
+      <c r="B21" s="0" t="n">
+        <v>20</v>
+      </c>
+      <c r="C21" s="0" t="inlineStr">
+        <is>
+          <t>Mann Mera</t>
+        </is>
+      </c>
+      <c r="D21" s="0" t="inlineStr">
+        <is>
+          <t>Gajendra Verma</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="0" t="inlineStr">
+        <is>
+          <t>2026-04-05</t>
+        </is>
+      </c>
+      <c r="B22" s="0" t="n">
+        <v>21</v>
+      </c>
+      <c r="C22" s="0" t="inlineStr">
+        <is>
+          <t>Saiyaara</t>
+        </is>
+      </c>
+      <c r="D22" s="0" t="inlineStr">
+        <is>
+          <t>Tanishk Bagchi</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="0" t="inlineStr">
+        <is>
+          <t>2026-04-05</t>
+        </is>
+      </c>
+      <c r="B23" s="0" t="n">
+        <v>22</v>
+      </c>
+      <c r="C23" s="0" t="inlineStr">
+        <is>
+          <t>For A Reason</t>
+        </is>
+      </c>
+      <c r="D23" s="0" t="inlineStr">
+        <is>
+          <t>Karan Aujla</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="0" t="inlineStr">
+        <is>
+          <t>2026-04-05</t>
+        </is>
+      </c>
+      <c r="B24" s="0" t="n">
+        <v>23</v>
+      </c>
+      <c r="C24" s="0" t="inlineStr">
+        <is>
+          <t>Bairi</t>
+        </is>
+      </c>
+      <c r="D24" s="0" t="inlineStr">
+        <is>
+          <t>Virat</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="0" t="inlineStr">
+        <is>
+          <t>2026-04-05</t>
+        </is>
+      </c>
+      <c r="B25" s="0" t="n">
+        <v>24</v>
+      </c>
+      <c r="C25" s="0" t="inlineStr">
+        <is>
+          <t>Deewaana Deewaana</t>
+        </is>
+      </c>
+      <c r="D25" s="0" t="inlineStr">
+        <is>
+          <t>A.R. Rahman</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="0" t="inlineStr">
+        <is>
+          <t>2026-04-05</t>
+        </is>
+      </c>
+      <c r="B26" s="0" t="n">
+        <v>25</v>
+      </c>
+      <c r="C26" s="0" t="inlineStr">
+        <is>
+          <t>Raanjhan</t>
+        </is>
+      </c>
+      <c r="D26" s="0" t="inlineStr">
+        <is>
+          <t>Sachet-Parampara</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="0" t="inlineStr">
+        <is>
+          <t>2026-04-05</t>
+        </is>
+      </c>
+      <c r="B27" s="0" t="n">
+        <v>26</v>
+      </c>
+      <c r="C27" s="0" t="inlineStr">
+        <is>
+          <t>Naal Nachna</t>
+        </is>
+      </c>
+      <c r="D27" s="0" t="inlineStr">
+        <is>
+          <t>Shashwat Sachdev</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="0" t="inlineStr">
+        <is>
+          <t>2026-04-05</t>
+        </is>
+      </c>
+      <c r="B28" s="0" t="n">
+        <v>27</v>
+      </c>
+      <c r="C28" s="0" t="inlineStr">
+        <is>
+          <t>Ishqa Ve</t>
+        </is>
+      </c>
+      <c r="D28" s="0" t="inlineStr">
+        <is>
+          <t>Zeeshan Ali</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="0" t="inlineStr">
+        <is>
+          <t>2026-04-05</t>
+        </is>
+      </c>
+      <c r="B29" s="0" t="n">
+        <v>28</v>
+      </c>
+      <c r="C29" s="0" t="inlineStr">
+        <is>
+          <t>Phir Se</t>
+        </is>
+      </c>
+      <c r="D29" s="0" t="inlineStr">
+        <is>
+          <t>Shashwat Sachdev</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="0" t="inlineStr">
+        <is>
+          <t>2026-04-05</t>
+        </is>
+      </c>
+      <c r="B30" s="0" t="n">
+        <v>29</v>
+      </c>
+      <c r="C30" s="0" t="inlineStr">
+        <is>
+          <t>Tum Ho Toh</t>
+        </is>
+      </c>
+      <c r="D30" s="0" t="inlineStr">
+        <is>
+          <t>Vishal Mishra</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="0" t="inlineStr">
+        <is>
+          <t>2026-04-05</t>
+        </is>
+      </c>
+      <c r="B31" s="0" t="n">
+        <v>30</v>
+      </c>
+      <c r="C31" s="0" t="inlineStr">
+        <is>
+          <t>Tere Liye</t>
+        </is>
+      </c>
+      <c r="D31" s="0" t="inlineStr">
+        <is>
+          <t>Atif Aslam</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="0" t="inlineStr">
+        <is>
+          <t>2026-04-05</t>
+        </is>
+      </c>
+      <c r="B32" s="0" t="n">
+        <v>31</v>
+      </c>
+      <c r="C32" s="0" t="inlineStr">
+        <is>
+          <t>Darkhaast</t>
+        </is>
+      </c>
+      <c r="D32" s="0" t="inlineStr">
+        <is>
+          <t>Mithoon</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="0" t="inlineStr">
+        <is>
+          <t>2026-04-05</t>
+        </is>
+      </c>
+      <c r="B33" s="0" t="n">
+        <v>32</v>
+      </c>
+      <c r="C33" s="0" t="inlineStr">
+        <is>
+          <t>Run Down The City - Monica</t>
+        </is>
+      </c>
+      <c r="D33" s="0" t="inlineStr">
+        <is>
+          <t>Shashwat Sachdev</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="0" t="inlineStr">
+        <is>
+          <t>2026-04-05</t>
+        </is>
+      </c>
+      <c r="B34" s="0" t="n">
+        <v>33</v>
+      </c>
+      <c r="C34" s="0" t="inlineStr">
+        <is>
+          <t>Lutt Le Gaya</t>
+        </is>
+      </c>
+      <c r="D34" s="0" t="inlineStr">
+        <is>
+          <t>Shashwat Sachdev</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="0" t="inlineStr">
+        <is>
+          <t>2026-04-05</t>
+        </is>
+      </c>
+      <c r="B35" s="0" t="n">
+        <v>34</v>
+      </c>
+      <c r="C35" s="0" t="inlineStr">
+        <is>
+          <t>Haseen</t>
+        </is>
+      </c>
+      <c r="D35" s="0" t="inlineStr">
+        <is>
+          <t>Talwiinder</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="0" t="inlineStr">
+        <is>
+          <t>2026-04-05</t>
+        </is>
+      </c>
+      <c r="B36" s="0" t="n">
+        <v>35</v>
+      </c>
+      <c r="C36" s="0" t="inlineStr">
+        <is>
+          <t>Jo Tum Mere Ho</t>
+        </is>
+      </c>
+      <c r="D36" s="0" t="inlineStr">
+        <is>
+          <t>Anuv Jain</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="0" t="inlineStr">
+        <is>
+          <t>2026-04-05</t>
+        </is>
+      </c>
+      <c r="B37" s="0" t="n">
+        <v>36</v>
+      </c>
+      <c r="C37" s="0" t="inlineStr">
+        <is>
+          <t>Tere Bina</t>
+        </is>
+      </c>
+      <c r="D37" s="0" t="inlineStr">
+        <is>
+          <t>A.R. Rahman</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="0" t="inlineStr">
+        <is>
+          <t>2026-04-05</t>
+        </is>
+      </c>
+      <c r="B38" s="0" t="n">
+        <v>37</v>
+      </c>
+      <c r="C38" s="0" t="inlineStr">
+        <is>
+          <t>Agar Tum Saath Ho</t>
+        </is>
+      </c>
+      <c r="D38" s="0" t="inlineStr">
+        <is>
+          <t>Alka Yagnik</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="0" t="inlineStr">
+        <is>
+          <t>2026-04-05</t>
+        </is>
+      </c>
+      <c r="B39" s="0" t="n">
+        <v>38</v>
+      </c>
+      <c r="C39" s="0" t="inlineStr">
+        <is>
+          <t>Barbaad</t>
+        </is>
+      </c>
+      <c r="D39" s="0" t="inlineStr">
+        <is>
+          <t>The Rish</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="0" t="inlineStr">
+        <is>
+          <t>2026-04-05</t>
+        </is>
+      </c>
+      <c r="B40" s="0" t="n">
+        <v>39</v>
+      </c>
+      <c r="C40" s="0" t="inlineStr">
+        <is>
+          <t>Mutta Kalakki</t>
+        </is>
+      </c>
+      <c r="D40" s="0" t="inlineStr">
+        <is>
+          <t>G. V. Prakash</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" s="0" t="inlineStr">
+        <is>
+          <t>2026-04-05</t>
+        </is>
+      </c>
+      <c r="B41" s="0" t="n">
+        <v>40</v>
+      </c>
+      <c r="C41" s="0" t="inlineStr">
+        <is>
+          <t>Ishq Jalakar - Karvaan</t>
+        </is>
+      </c>
+      <c r="D41" s="0" t="inlineStr">
+        <is>
+          <t>Shashwat Sachdev</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" s="0" t="inlineStr">
+        <is>
+          <t>2026-04-05</t>
+        </is>
+      </c>
+      <c r="B42" s="0" t="n">
+        <v>41</v>
+      </c>
+      <c r="C42" s="0" t="inlineStr">
+        <is>
+          <t>Teri Deewani</t>
+        </is>
+      </c>
+      <c r="D42" s="0" t="inlineStr">
+        <is>
+          <t>Kailash Kher</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" s="0" t="inlineStr">
+        <is>
+          <t>2026-04-05</t>
+        </is>
+      </c>
+      <c r="B43" s="0" t="n">
+        <v>42</v>
+      </c>
+      <c r="C43" s="0" t="inlineStr">
+        <is>
+          <t>Mann Mera - Original Version</t>
+        </is>
+      </c>
+      <c r="D43" s="0" t="inlineStr">
+        <is>
+          <t>Gajendra Verma</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" s="0" t="inlineStr">
+        <is>
+          <t>2026-04-05</t>
+        </is>
+      </c>
+      <c r="B44" s="0" t="n">
+        <v>43</v>
+      </c>
+      <c r="C44" s="0" t="inlineStr">
+        <is>
+          <t>Ye Tune Kya Kiya</t>
+        </is>
+      </c>
+      <c r="D44" s="0" t="inlineStr">
+        <is>
+          <t>Pritam</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" s="0" t="inlineStr">
+        <is>
+          <t>2026-04-05</t>
+        </is>
+      </c>
+      <c r="B45" s="0" t="n">
+        <v>44</v>
+      </c>
+      <c r="C45" s="0" t="inlineStr">
+        <is>
+          <t>Ehsaas</t>
+        </is>
+      </c>
+      <c r="D45" s="0" t="inlineStr">
+        <is>
+          <t>Faheem Abdullah</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" s="0" t="inlineStr">
+        <is>
+          <t>2026-04-05</t>
+        </is>
+      </c>
+      <c r="B46" s="0" t="n">
+        <v>45</v>
+      </c>
+      <c r="C46" s="0" t="inlineStr">
+        <is>
+          <t>Aaya Sher</t>
+        </is>
+      </c>
+      <c r="D46" s="0" t="inlineStr">
+        <is>
+          <t>Anirudh Ravichander</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" s="0" t="inlineStr">
+        <is>
+          <t>2026-04-05</t>
+        </is>
+      </c>
+      <c r="B47" s="0" t="n">
+        <v>46</v>
+      </c>
+      <c r="C47" s="0" t="inlineStr">
+        <is>
+          <t>Main Aur Tu</t>
+        </is>
+      </c>
+      <c r="D47" s="0" t="inlineStr">
+        <is>
+          <t>Shashwat Sachdev</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" s="0" t="inlineStr">
+        <is>
+          <t>2026-04-05</t>
+        </is>
+      </c>
+      <c r="B48" s="0" t="n">
+        <v>47</v>
+      </c>
+      <c r="C48" s="0" t="inlineStr">
+        <is>
+          <t>Not Guilty</t>
+        </is>
+      </c>
+      <c r="D48" s="0" t="inlineStr">
+        <is>
+          <t>Dhanda Nyoliwala</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" s="0" t="inlineStr">
+        <is>
+          <t>2026-04-05</t>
+        </is>
+      </c>
+      <c r="B49" s="0" t="n">
+        <v>48</v>
+      </c>
+      <c r="C49" s="0" t="inlineStr">
+        <is>
+          <t>Dhun</t>
+        </is>
+      </c>
+      <c r="D49" s="0" t="inlineStr">
+        <is>
+          <t>Mithoon</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" s="0" t="inlineStr">
+        <is>
+          <t>2026-04-05</t>
+        </is>
+      </c>
+      <c r="B50" s="0" t="n">
+        <v>49</v>
+      </c>
+      <c r="C50" s="0" t="inlineStr">
+        <is>
+          <t>Zaalima</t>
+        </is>
+      </c>
+      <c r="D50" s="0" t="inlineStr">
+        <is>
+          <t>Arijit Singh</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" s="0" t="inlineStr">
+        <is>
+          <t>2026-04-05</t>
+        </is>
+      </c>
+      <c r="B51" s="0" t="n">
+        <v>50</v>
+      </c>
+      <c r="C51" s="0" t="inlineStr">
+        <is>
+          <t>Humdard</t>
+        </is>
+      </c>
+      <c r="D51" s="0" t="inlineStr">
+        <is>
+          <t>Arijit Singh</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet24.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:D51"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="24" t="inlineStr">
+        <is>
+          <t>Date</t>
+        </is>
+      </c>
+      <c r="B1" s="24" t="inlineStr">
+        <is>
+          <t>Rank</t>
+        </is>
+      </c>
+      <c r="C1" s="24" t="inlineStr">
+        <is>
+          <t>Song</t>
+        </is>
+      </c>
+      <c r="D1" s="24" t="inlineStr">
+        <is>
+          <t>Artist</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>2026-04-05</t>
+          <t>2026-04-06</t>
         </is>
       </c>
       <c r="B2" t="n">
@@ -17092,7 +18129,7 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>2026-04-05</t>
+          <t>2026-04-06</t>
         </is>
       </c>
       <c r="B3" t="n">
@@ -17112,7 +18149,7 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>2026-04-05</t>
+          <t>2026-04-06</t>
         </is>
       </c>
       <c r="B4" t="n">
@@ -17132,7 +18169,7 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>2026-04-05</t>
+          <t>2026-04-06</t>
         </is>
       </c>
       <c r="B5" t="n">
@@ -17152,7 +18189,7 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>2026-04-05</t>
+          <t>2026-04-06</t>
         </is>
       </c>
       <c r="B6" t="n">
@@ -17172,7 +18209,7 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>2026-04-05</t>
+          <t>2026-04-06</t>
         </is>
       </c>
       <c r="B7" t="n">
@@ -17192,7 +18229,7 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>2026-04-05</t>
+          <t>2026-04-06</t>
         </is>
       </c>
       <c r="B8" t="n">
@@ -17200,19 +18237,19 @@
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>Sahiba</t>
+          <t>Dooron Dooron</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>Aditya Rikhari</t>
+          <t>Paresh Pahuja</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>2026-04-05</t>
+          <t>2026-04-06</t>
         </is>
       </c>
       <c r="B9" t="n">
@@ -17220,19 +18257,19 @@
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>Dooron Dooron</t>
+          <t>Sahiba</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>Paresh Pahuja</t>
+          <t>Aditya Rikhari</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>2026-04-05</t>
+          <t>2026-04-06</t>
         </is>
       </c>
       <c r="B10" t="n">
@@ -17240,19 +18277,19 @@
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>Sitaare</t>
+          <t>Jaan Se Guzarte Hain</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>Arijit Singh</t>
+          <t>Shashwat Sachdev</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>2026-04-05</t>
+          <t>2026-04-06</t>
         </is>
       </c>
       <c r="B11" t="n">
@@ -17260,19 +18297,19 @@
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>Apna Bana Le</t>
+          <t>Sitaare</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>Sachin-Jigar</t>
+          <t>Arijit Singh</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>2026-04-05</t>
+          <t>2026-04-06</t>
         </is>
       </c>
       <c r="B12" t="n">
@@ -17280,19 +18317,19 @@
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>Jaan Se Guzarte Hain</t>
+          <t>Apna Bana Le</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>Shashwat Sachdev</t>
+          <t>Sachin-Jigar</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>2026-04-05</t>
+          <t>2026-04-06</t>
         </is>
       </c>
       <c r="B13" t="n">
@@ -17300,19 +18337,19 @@
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>Pavazha Malli</t>
+          <t>Samjhawan</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>Sai Abhyankkar</t>
+          <t>Jawad Ahmad</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>2026-04-05</t>
+          <t>2026-04-06</t>
         </is>
       </c>
       <c r="B14" t="n">
@@ -17320,19 +18357,19 @@
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>Finding Her</t>
+          <t>Pavazha Malli</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>Kushagra</t>
+          <t>Sai Abhyankkar</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>2026-04-05</t>
+          <t>2026-04-06</t>
         </is>
       </c>
       <c r="B15" t="n">
@@ -17340,19 +18377,19 @@
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>Samjhawan</t>
+          <t>Finding Her</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>Jawad Ahmad</t>
+          <t>Kushagra</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>2026-04-05</t>
+          <t>2026-04-06</t>
         </is>
       </c>
       <c r="B16" t="n">
@@ -17360,19 +18397,19 @@
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>Shararat</t>
+          <t>Arz Kiya Hai | Coke Studio Bharat</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>Shashwat Sachdev</t>
+          <t>Anuv Jain</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>2026-04-05</t>
+          <t>2026-04-06</t>
         </is>
       </c>
       <c r="B17" t="n">
@@ -17380,19 +18417,19 @@
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>Arz Kiya Hai | Coke Studio Bharat</t>
+          <t>Boyfriend</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>Anuv Jain</t>
+          <t>Karan Aujla</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>2026-04-05</t>
+          <t>2026-04-06</t>
         </is>
       </c>
       <c r="B18" t="n">
@@ -17400,19 +18437,19 @@
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>Boyfriend</t>
+          <t>Ishq</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>Karan Aujla</t>
+          <t>Faheem Abdullah</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>2026-04-05</t>
+          <t>2026-04-06</t>
         </is>
       </c>
       <c r="B19" t="n">
@@ -17420,7 +18457,7 @@
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>Dhurandhar - Title Track</t>
+          <t>Shararat</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
@@ -17432,7 +18469,7 @@
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>2026-04-05</t>
+          <t>2026-04-06</t>
         </is>
       </c>
       <c r="B20" t="n">
@@ -17440,19 +18477,19 @@
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>Ishq</t>
+          <t>Mann Mera</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>Faheem Abdullah</t>
+          <t>Gajendra Verma</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>2026-04-05</t>
+          <t>2026-04-06</t>
         </is>
       </c>
       <c r="B21" t="n">
@@ -17460,19 +18497,19 @@
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>Mann Mera</t>
+          <t>Dhurandhar - Title Track</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>Gajendra Verma</t>
+          <t>Shashwat Sachdev</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>2026-04-05</t>
+          <t>2026-04-06</t>
         </is>
       </c>
       <c r="B22" t="n">
@@ -17492,7 +18529,7 @@
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>2026-04-05</t>
+          <t>2026-04-06</t>
         </is>
       </c>
       <c r="B23" t="n">
@@ -17512,7 +18549,7 @@
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>2026-04-05</t>
+          <t>2026-04-06</t>
         </is>
       </c>
       <c r="B24" t="n">
@@ -17532,7 +18569,7 @@
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>2026-04-05</t>
+          <t>2026-04-06</t>
         </is>
       </c>
       <c r="B25" t="n">
@@ -17540,19 +18577,19 @@
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>Deewaana Deewaana</t>
+          <t>Phir Se</t>
         </is>
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>A.R. Rahman</t>
+          <t>Shashwat Sachdev</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>2026-04-05</t>
+          <t>2026-04-06</t>
         </is>
       </c>
       <c r="B26" t="n">
@@ -17560,19 +18597,19 @@
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>Raanjhan</t>
+          <t>Deewaana Deewaana</t>
         </is>
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>Sachet-Parampara</t>
+          <t>A.R. Rahman</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>2026-04-05</t>
+          <t>2026-04-06</t>
         </is>
       </c>
       <c r="B27" t="n">
@@ -17580,19 +18617,19 @@
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>Naal Nachna</t>
+          <t>Raanjhan</t>
         </is>
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t>Shashwat Sachdev</t>
+          <t>Sachet-Parampara</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>2026-04-05</t>
+          <t>2026-04-06</t>
         </is>
       </c>
       <c r="B28" t="n">
@@ -17600,19 +18637,19 @@
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>Ishqa Ve</t>
+          <t>Tere Liye</t>
         </is>
       </c>
       <c r="D28" t="inlineStr">
         <is>
-          <t>Zeeshan Ali</t>
+          <t>Atif Aslam</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>2026-04-05</t>
+          <t>2026-04-06</t>
         </is>
       </c>
       <c r="B29" t="n">
@@ -17620,7 +18657,7 @@
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>Phir Se</t>
+          <t>Naal Nachna</t>
         </is>
       </c>
       <c r="D29" t="inlineStr">
@@ -17632,7 +18669,7 @@
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>2026-04-05</t>
+          <t>2026-04-06</t>
         </is>
       </c>
       <c r="B30" t="n">
@@ -17652,7 +18689,7 @@
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>2026-04-05</t>
+          <t>2026-04-06</t>
         </is>
       </c>
       <c r="B31" t="n">
@@ -17660,19 +18697,19 @@
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>Tere Liye</t>
+          <t>Ishqa Ve</t>
         </is>
       </c>
       <c r="D31" t="inlineStr">
         <is>
-          <t>Atif Aslam</t>
+          <t>Zeeshan Ali</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>2026-04-05</t>
+          <t>2026-04-06</t>
         </is>
       </c>
       <c r="B32" t="n">
@@ -17692,7 +18729,7 @@
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>2026-04-05</t>
+          <t>2026-04-06</t>
         </is>
       </c>
       <c r="B33" t="n">
@@ -17712,7 +18749,7 @@
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>2026-04-05</t>
+          <t>2026-04-06</t>
         </is>
       </c>
       <c r="B34" t="n">
@@ -17732,7 +18769,7 @@
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>2026-04-05</t>
+          <t>2026-04-06</t>
         </is>
       </c>
       <c r="B35" t="n">
@@ -17740,19 +18777,19 @@
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>Haseen</t>
+          <t>Jo Tum Mere Ho</t>
         </is>
       </c>
       <c r="D35" t="inlineStr">
         <is>
-          <t>Talwiinder</t>
+          <t>Anuv Jain</t>
         </is>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>2026-04-05</t>
+          <t>2026-04-06</t>
         </is>
       </c>
       <c r="B36" t="n">
@@ -17760,19 +18797,19 @@
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>Jo Tum Mere Ho</t>
+          <t>Haseen</t>
         </is>
       </c>
       <c r="D36" t="inlineStr">
         <is>
-          <t>Anuv Jain</t>
+          <t>Talwiinder</t>
         </is>
       </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>2026-04-05</t>
+          <t>2026-04-06</t>
         </is>
       </c>
       <c r="B37" t="n">
@@ -17780,19 +18817,19 @@
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>Tere Bina</t>
+          <t>Barbaad</t>
         </is>
       </c>
       <c r="D37" t="inlineStr">
         <is>
-          <t>A.R. Rahman</t>
+          <t>The Rish</t>
         </is>
       </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>2026-04-05</t>
+          <t>2026-04-06</t>
         </is>
       </c>
       <c r="B38" t="n">
@@ -17812,7 +18849,7 @@
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>2026-04-05</t>
+          <t>2026-04-06</t>
         </is>
       </c>
       <c r="B39" t="n">
@@ -17820,19 +18857,19 @@
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>Barbaad</t>
+          <t>Tere Bina</t>
         </is>
       </c>
       <c r="D39" t="inlineStr">
         <is>
-          <t>The Rish</t>
+          <t>A.R. Rahman</t>
         </is>
       </c>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>2026-04-05</t>
+          <t>2026-04-06</t>
         </is>
       </c>
       <c r="B40" t="n">
@@ -17840,19 +18877,19 @@
       </c>
       <c r="C40" t="inlineStr">
         <is>
-          <t>Mutta Kalakki</t>
+          <t>Teri Deewani</t>
         </is>
       </c>
       <c r="D40" t="inlineStr">
         <is>
-          <t>G. V. Prakash</t>
+          <t>Kailash Kher</t>
         </is>
       </c>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>2026-04-05</t>
+          <t>2026-04-06</t>
         </is>
       </c>
       <c r="B41" t="n">
@@ -17860,19 +18897,19 @@
       </c>
       <c r="C41" t="inlineStr">
         <is>
-          <t>Ishq Jalakar - Karvaan</t>
+          <t>Not Guilty</t>
         </is>
       </c>
       <c r="D41" t="inlineStr">
         <is>
-          <t>Shashwat Sachdev</t>
+          <t>Dhanda Nyoliwala</t>
         </is>
       </c>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>2026-04-05</t>
+          <t>2026-04-06</t>
         </is>
       </c>
       <c r="B42" t="n">
@@ -17880,19 +18917,19 @@
       </c>
       <c r="C42" t="inlineStr">
         <is>
-          <t>Teri Deewani</t>
+          <t>Ye Tune Kya Kiya</t>
         </is>
       </c>
       <c r="D42" t="inlineStr">
         <is>
-          <t>Kailash Kher</t>
+          <t>Pritam</t>
         </is>
       </c>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>2026-04-05</t>
+          <t>2026-04-06</t>
         </is>
       </c>
       <c r="B43" t="n">
@@ -17912,7 +18949,7 @@
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>2026-04-05</t>
+          <t>2026-04-06</t>
         </is>
       </c>
       <c r="B44" t="n">
@@ -17920,19 +18957,19 @@
       </c>
       <c r="C44" t="inlineStr">
         <is>
-          <t>Ye Tune Kya Kiya</t>
+          <t>Main Aur Tu</t>
         </is>
       </c>
       <c r="D44" t="inlineStr">
         <is>
-          <t>Pritam</t>
+          <t>Shashwat Sachdev</t>
         </is>
       </c>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>2026-04-05</t>
+          <t>2026-04-06</t>
         </is>
       </c>
       <c r="B45" t="n">
@@ -17952,7 +18989,7 @@
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>2026-04-05</t>
+          <t>2026-04-06</t>
         </is>
       </c>
       <c r="B46" t="n">
@@ -17972,7 +19009,7 @@
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>2026-04-05</t>
+          <t>2026-04-06</t>
         </is>
       </c>
       <c r="B47" t="n">
@@ -17980,19 +19017,19 @@
       </c>
       <c r="C47" t="inlineStr">
         <is>
-          <t>Main Aur Tu</t>
+          <t>Mutta Kalakki</t>
         </is>
       </c>
       <c r="D47" t="inlineStr">
         <is>
-          <t>Shashwat Sachdev</t>
+          <t>G. V. Prakash</t>
         </is>
       </c>
     </row>
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>2026-04-05</t>
+          <t>2026-04-06</t>
         </is>
       </c>
       <c r="B48" t="n">
@@ -18000,19 +19037,19 @@
       </c>
       <c r="C48" t="inlineStr">
         <is>
-          <t>Not Guilty</t>
+          <t>Ishq Jalakar - Karvaan</t>
         </is>
       </c>
       <c r="D48" t="inlineStr">
         <is>
-          <t>Dhanda Nyoliwala</t>
+          <t>Shashwat Sachdev</t>
         </is>
       </c>
     </row>
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>2026-04-05</t>
+          <t>2026-04-06</t>
         </is>
       </c>
       <c r="B49" t="n">
@@ -18020,19 +19057,19 @@
       </c>
       <c r="C49" t="inlineStr">
         <is>
-          <t>Dhun</t>
+          <t>Jogi</t>
         </is>
       </c>
       <c r="D49" t="inlineStr">
         <is>
-          <t>Mithoon</t>
+          <t>thiarajxtt</t>
         </is>
       </c>
     </row>
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>2026-04-05</t>
+          <t>2026-04-06</t>
         </is>
       </c>
       <c r="B50" t="n">
@@ -18040,7 +19077,7 @@
       </c>
       <c r="C50" t="inlineStr">
         <is>
-          <t>Zaalima</t>
+          <t>Mast Magan</t>
         </is>
       </c>
       <c r="D50" t="inlineStr">
@@ -18052,7 +19089,7 @@
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>2026-04-05</t>
+          <t>2026-04-06</t>
         </is>
       </c>
       <c r="B51" t="n">
@@ -18060,12 +19097,12 @@
       </c>
       <c r="C51" t="inlineStr">
         <is>
-          <t>Humdard</t>
+          <t>Dhun</t>
         </is>
       </c>
       <c r="D51" t="inlineStr">
         <is>
-          <t>Arijit Singh</t>
+          <t>Mithoon</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
added data till 9th april, got predictions for 10th april
</commit_message>
<xml_diff>
--- a/Probability Project.xlsx
+++ b/Probability Project.xlsx
@@ -27,6 +27,9 @@
     <sheet name="AUTO_20260404" sheetId="22" state="visible" r:id="rId22"/>
     <sheet name="AUTO_20260405" sheetId="23" state="visible" r:id="rId23"/>
     <sheet name="AUTO_20260406" sheetId="24" state="visible" r:id="rId24"/>
+    <sheet name="AUTO_20260409" sheetId="25" state="visible" r:id="rId25"/>
+    <sheet name="AUTO_20260407" sheetId="26" state="visible" r:id="rId26"/>
+    <sheet name="AUTO_20260408" sheetId="27" state="visible" r:id="rId27"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -18107,9 +18110,3117 @@
       </c>
     </row>
     <row r="2">
+      <c r="A2" s="0" t="inlineStr">
+        <is>
+          <t>2026-04-06</t>
+        </is>
+      </c>
+      <c r="B2" s="0" t="n">
+        <v>1</v>
+      </c>
+      <c r="C2" s="0" t="inlineStr">
+        <is>
+          <t>Bairan</t>
+        </is>
+      </c>
+      <c r="D2" s="0" t="inlineStr">
+        <is>
+          <t>Banjaare</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="0" t="inlineStr">
+        <is>
+          <t>2026-04-06</t>
+        </is>
+      </c>
+      <c r="B3" s="0" t="n">
+        <v>2</v>
+      </c>
+      <c r="C3" s="0" t="inlineStr">
+        <is>
+          <t>Jaiye Sajana</t>
+        </is>
+      </c>
+      <c r="D3" s="0" t="inlineStr">
+        <is>
+          <t>Shashwat Sachdev</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="0" t="inlineStr">
+        <is>
+          <t>2026-04-06</t>
+        </is>
+      </c>
+      <c r="B4" s="0" t="n">
+        <v>3</v>
+      </c>
+      <c r="C4" s="0" t="inlineStr">
+        <is>
+          <t>Gehra Hua</t>
+        </is>
+      </c>
+      <c r="D4" s="0" t="inlineStr">
+        <is>
+          <t>Shashwat Sachdev</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="0" t="inlineStr">
+        <is>
+          <t>2026-04-06</t>
+        </is>
+      </c>
+      <c r="B5" s="0" t="n">
+        <v>4</v>
+      </c>
+      <c r="C5" s="0" t="inlineStr">
+        <is>
+          <t>Sheesha - Aakhya Mai Aakh Ghali Jo Bairan</t>
+        </is>
+      </c>
+      <c r="D5" s="0" t="inlineStr">
+        <is>
+          <t>Mitta Ror</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="0" t="inlineStr">
+        <is>
+          <t>2026-04-06</t>
+        </is>
+      </c>
+      <c r="B6" s="0" t="n">
+        <v>5</v>
+      </c>
+      <c r="C6" s="0" t="inlineStr">
+        <is>
+          <t>Khat</t>
+        </is>
+      </c>
+      <c r="D6" s="0" t="inlineStr">
+        <is>
+          <t>Navjot Ahuja</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="0" t="inlineStr">
+        <is>
+          <t>2026-04-06</t>
+        </is>
+      </c>
+      <c r="B7" s="0" t="n">
+        <v>6</v>
+      </c>
+      <c r="C7" s="0" t="inlineStr">
+        <is>
+          <t>Dhurandhar The Revenge - Aari Aari</t>
+        </is>
+      </c>
+      <c r="D7" s="0" t="inlineStr">
+        <is>
+          <t>Shashwat Sachdev</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="0" t="inlineStr">
+        <is>
+          <t>2026-04-06</t>
+        </is>
+      </c>
+      <c r="B8" s="0" t="n">
+        <v>7</v>
+      </c>
+      <c r="C8" s="0" t="inlineStr">
+        <is>
+          <t>Dooron Dooron</t>
+        </is>
+      </c>
+      <c r="D8" s="0" t="inlineStr">
+        <is>
+          <t>Paresh Pahuja</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="0" t="inlineStr">
+        <is>
+          <t>2026-04-06</t>
+        </is>
+      </c>
+      <c r="B9" s="0" t="n">
+        <v>8</v>
+      </c>
+      <c r="C9" s="0" t="inlineStr">
+        <is>
+          <t>Sahiba</t>
+        </is>
+      </c>
+      <c r="D9" s="0" t="inlineStr">
+        <is>
+          <t>Aditya Rikhari</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="0" t="inlineStr">
+        <is>
+          <t>2026-04-06</t>
+        </is>
+      </c>
+      <c r="B10" s="0" t="n">
+        <v>9</v>
+      </c>
+      <c r="C10" s="0" t="inlineStr">
+        <is>
+          <t>Jaan Se Guzarte Hain</t>
+        </is>
+      </c>
+      <c r="D10" s="0" t="inlineStr">
+        <is>
+          <t>Shashwat Sachdev</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="0" t="inlineStr">
+        <is>
+          <t>2026-04-06</t>
+        </is>
+      </c>
+      <c r="B11" s="0" t="n">
+        <v>10</v>
+      </c>
+      <c r="C11" s="0" t="inlineStr">
+        <is>
+          <t>Sitaare</t>
+        </is>
+      </c>
+      <c r="D11" s="0" t="inlineStr">
+        <is>
+          <t>Arijit Singh</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="0" t="inlineStr">
+        <is>
+          <t>2026-04-06</t>
+        </is>
+      </c>
+      <c r="B12" s="0" t="n">
+        <v>11</v>
+      </c>
+      <c r="C12" s="0" t="inlineStr">
+        <is>
+          <t>Apna Bana Le</t>
+        </is>
+      </c>
+      <c r="D12" s="0" t="inlineStr">
+        <is>
+          <t>Sachin-Jigar</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="0" t="inlineStr">
+        <is>
+          <t>2026-04-06</t>
+        </is>
+      </c>
+      <c r="B13" s="0" t="n">
+        <v>12</v>
+      </c>
+      <c r="C13" s="0" t="inlineStr">
+        <is>
+          <t>Samjhawan</t>
+        </is>
+      </c>
+      <c r="D13" s="0" t="inlineStr">
+        <is>
+          <t>Jawad Ahmad</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="0" t="inlineStr">
+        <is>
+          <t>2026-04-06</t>
+        </is>
+      </c>
+      <c r="B14" s="0" t="n">
+        <v>13</v>
+      </c>
+      <c r="C14" s="0" t="inlineStr">
+        <is>
+          <t>Pavazha Malli</t>
+        </is>
+      </c>
+      <c r="D14" s="0" t="inlineStr">
+        <is>
+          <t>Sai Abhyankkar</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="0" t="inlineStr">
+        <is>
+          <t>2026-04-06</t>
+        </is>
+      </c>
+      <c r="B15" s="0" t="n">
+        <v>14</v>
+      </c>
+      <c r="C15" s="0" t="inlineStr">
+        <is>
+          <t>Finding Her</t>
+        </is>
+      </c>
+      <c r="D15" s="0" t="inlineStr">
+        <is>
+          <t>Kushagra</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="0" t="inlineStr">
+        <is>
+          <t>2026-04-06</t>
+        </is>
+      </c>
+      <c r="B16" s="0" t="n">
+        <v>15</v>
+      </c>
+      <c r="C16" s="0" t="inlineStr">
+        <is>
+          <t>Arz Kiya Hai | Coke Studio Bharat</t>
+        </is>
+      </c>
+      <c r="D16" s="0" t="inlineStr">
+        <is>
+          <t>Anuv Jain</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="0" t="inlineStr">
+        <is>
+          <t>2026-04-06</t>
+        </is>
+      </c>
+      <c r="B17" s="0" t="n">
+        <v>16</v>
+      </c>
+      <c r="C17" s="0" t="inlineStr">
+        <is>
+          <t>Boyfriend</t>
+        </is>
+      </c>
+      <c r="D17" s="0" t="inlineStr">
+        <is>
+          <t>Karan Aujla</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="0" t="inlineStr">
+        <is>
+          <t>2026-04-06</t>
+        </is>
+      </c>
+      <c r="B18" s="0" t="n">
+        <v>17</v>
+      </c>
+      <c r="C18" s="0" t="inlineStr">
+        <is>
+          <t>Ishq</t>
+        </is>
+      </c>
+      <c r="D18" s="0" t="inlineStr">
+        <is>
+          <t>Faheem Abdullah</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="0" t="inlineStr">
+        <is>
+          <t>2026-04-06</t>
+        </is>
+      </c>
+      <c r="B19" s="0" t="n">
+        <v>18</v>
+      </c>
+      <c r="C19" s="0" t="inlineStr">
+        <is>
+          <t>Shararat</t>
+        </is>
+      </c>
+      <c r="D19" s="0" t="inlineStr">
+        <is>
+          <t>Shashwat Sachdev</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="0" t="inlineStr">
+        <is>
+          <t>2026-04-06</t>
+        </is>
+      </c>
+      <c r="B20" s="0" t="n">
+        <v>19</v>
+      </c>
+      <c r="C20" s="0" t="inlineStr">
+        <is>
+          <t>Mann Mera</t>
+        </is>
+      </c>
+      <c r="D20" s="0" t="inlineStr">
+        <is>
+          <t>Gajendra Verma</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="0" t="inlineStr">
+        <is>
+          <t>2026-04-06</t>
+        </is>
+      </c>
+      <c r="B21" s="0" t="n">
+        <v>20</v>
+      </c>
+      <c r="C21" s="0" t="inlineStr">
+        <is>
+          <t>Dhurandhar - Title Track</t>
+        </is>
+      </c>
+      <c r="D21" s="0" t="inlineStr">
+        <is>
+          <t>Shashwat Sachdev</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="0" t="inlineStr">
+        <is>
+          <t>2026-04-06</t>
+        </is>
+      </c>
+      <c r="B22" s="0" t="n">
+        <v>21</v>
+      </c>
+      <c r="C22" s="0" t="inlineStr">
+        <is>
+          <t>Saiyaara</t>
+        </is>
+      </c>
+      <c r="D22" s="0" t="inlineStr">
+        <is>
+          <t>Tanishk Bagchi</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="0" t="inlineStr">
+        <is>
+          <t>2026-04-06</t>
+        </is>
+      </c>
+      <c r="B23" s="0" t="n">
+        <v>22</v>
+      </c>
+      <c r="C23" s="0" t="inlineStr">
+        <is>
+          <t>For A Reason</t>
+        </is>
+      </c>
+      <c r="D23" s="0" t="inlineStr">
+        <is>
+          <t>Karan Aujla</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="0" t="inlineStr">
+        <is>
+          <t>2026-04-06</t>
+        </is>
+      </c>
+      <c r="B24" s="0" t="n">
+        <v>23</v>
+      </c>
+      <c r="C24" s="0" t="inlineStr">
+        <is>
+          <t>Bairi</t>
+        </is>
+      </c>
+      <c r="D24" s="0" t="inlineStr">
+        <is>
+          <t>Virat</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="0" t="inlineStr">
+        <is>
+          <t>2026-04-06</t>
+        </is>
+      </c>
+      <c r="B25" s="0" t="n">
+        <v>24</v>
+      </c>
+      <c r="C25" s="0" t="inlineStr">
+        <is>
+          <t>Phir Se</t>
+        </is>
+      </c>
+      <c r="D25" s="0" t="inlineStr">
+        <is>
+          <t>Shashwat Sachdev</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="0" t="inlineStr">
+        <is>
+          <t>2026-04-06</t>
+        </is>
+      </c>
+      <c r="B26" s="0" t="n">
+        <v>25</v>
+      </c>
+      <c r="C26" s="0" t="inlineStr">
+        <is>
+          <t>Deewaana Deewaana</t>
+        </is>
+      </c>
+      <c r="D26" s="0" t="inlineStr">
+        <is>
+          <t>A.R. Rahman</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="0" t="inlineStr">
+        <is>
+          <t>2026-04-06</t>
+        </is>
+      </c>
+      <c r="B27" s="0" t="n">
+        <v>26</v>
+      </c>
+      <c r="C27" s="0" t="inlineStr">
+        <is>
+          <t>Raanjhan</t>
+        </is>
+      </c>
+      <c r="D27" s="0" t="inlineStr">
+        <is>
+          <t>Sachet-Parampara</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="0" t="inlineStr">
+        <is>
+          <t>2026-04-06</t>
+        </is>
+      </c>
+      <c r="B28" s="0" t="n">
+        <v>27</v>
+      </c>
+      <c r="C28" s="0" t="inlineStr">
+        <is>
+          <t>Tere Liye</t>
+        </is>
+      </c>
+      <c r="D28" s="0" t="inlineStr">
+        <is>
+          <t>Atif Aslam</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="0" t="inlineStr">
+        <is>
+          <t>2026-04-06</t>
+        </is>
+      </c>
+      <c r="B29" s="0" t="n">
+        <v>28</v>
+      </c>
+      <c r="C29" s="0" t="inlineStr">
+        <is>
+          <t>Naal Nachna</t>
+        </is>
+      </c>
+      <c r="D29" s="0" t="inlineStr">
+        <is>
+          <t>Shashwat Sachdev</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="0" t="inlineStr">
+        <is>
+          <t>2026-04-06</t>
+        </is>
+      </c>
+      <c r="B30" s="0" t="n">
+        <v>29</v>
+      </c>
+      <c r="C30" s="0" t="inlineStr">
+        <is>
+          <t>Tum Ho Toh</t>
+        </is>
+      </c>
+      <c r="D30" s="0" t="inlineStr">
+        <is>
+          <t>Vishal Mishra</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="0" t="inlineStr">
+        <is>
+          <t>2026-04-06</t>
+        </is>
+      </c>
+      <c r="B31" s="0" t="n">
+        <v>30</v>
+      </c>
+      <c r="C31" s="0" t="inlineStr">
+        <is>
+          <t>Ishqa Ve</t>
+        </is>
+      </c>
+      <c r="D31" s="0" t="inlineStr">
+        <is>
+          <t>Zeeshan Ali</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="0" t="inlineStr">
+        <is>
+          <t>2026-04-06</t>
+        </is>
+      </c>
+      <c r="B32" s="0" t="n">
+        <v>31</v>
+      </c>
+      <c r="C32" s="0" t="inlineStr">
+        <is>
+          <t>Darkhaast</t>
+        </is>
+      </c>
+      <c r="D32" s="0" t="inlineStr">
+        <is>
+          <t>Mithoon</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="0" t="inlineStr">
+        <is>
+          <t>2026-04-06</t>
+        </is>
+      </c>
+      <c r="B33" s="0" t="n">
+        <v>32</v>
+      </c>
+      <c r="C33" s="0" t="inlineStr">
+        <is>
+          <t>Run Down The City - Monica</t>
+        </is>
+      </c>
+      <c r="D33" s="0" t="inlineStr">
+        <is>
+          <t>Shashwat Sachdev</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="0" t="inlineStr">
+        <is>
+          <t>2026-04-06</t>
+        </is>
+      </c>
+      <c r="B34" s="0" t="n">
+        <v>33</v>
+      </c>
+      <c r="C34" s="0" t="inlineStr">
+        <is>
+          <t>Lutt Le Gaya</t>
+        </is>
+      </c>
+      <c r="D34" s="0" t="inlineStr">
+        <is>
+          <t>Shashwat Sachdev</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="0" t="inlineStr">
+        <is>
+          <t>2026-04-06</t>
+        </is>
+      </c>
+      <c r="B35" s="0" t="n">
+        <v>34</v>
+      </c>
+      <c r="C35" s="0" t="inlineStr">
+        <is>
+          <t>Jo Tum Mere Ho</t>
+        </is>
+      </c>
+      <c r="D35" s="0" t="inlineStr">
+        <is>
+          <t>Anuv Jain</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="0" t="inlineStr">
+        <is>
+          <t>2026-04-06</t>
+        </is>
+      </c>
+      <c r="B36" s="0" t="n">
+        <v>35</v>
+      </c>
+      <c r="C36" s="0" t="inlineStr">
+        <is>
+          <t>Haseen</t>
+        </is>
+      </c>
+      <c r="D36" s="0" t="inlineStr">
+        <is>
+          <t>Talwiinder</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="0" t="inlineStr">
+        <is>
+          <t>2026-04-06</t>
+        </is>
+      </c>
+      <c r="B37" s="0" t="n">
+        <v>36</v>
+      </c>
+      <c r="C37" s="0" t="inlineStr">
+        <is>
+          <t>Barbaad</t>
+        </is>
+      </c>
+      <c r="D37" s="0" t="inlineStr">
+        <is>
+          <t>The Rish</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="0" t="inlineStr">
+        <is>
+          <t>2026-04-06</t>
+        </is>
+      </c>
+      <c r="B38" s="0" t="n">
+        <v>37</v>
+      </c>
+      <c r="C38" s="0" t="inlineStr">
+        <is>
+          <t>Agar Tum Saath Ho</t>
+        </is>
+      </c>
+      <c r="D38" s="0" t="inlineStr">
+        <is>
+          <t>Alka Yagnik</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="0" t="inlineStr">
+        <is>
+          <t>2026-04-06</t>
+        </is>
+      </c>
+      <c r="B39" s="0" t="n">
+        <v>38</v>
+      </c>
+      <c r="C39" s="0" t="inlineStr">
+        <is>
+          <t>Tere Bina</t>
+        </is>
+      </c>
+      <c r="D39" s="0" t="inlineStr">
+        <is>
+          <t>A.R. Rahman</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="0" t="inlineStr">
+        <is>
+          <t>2026-04-06</t>
+        </is>
+      </c>
+      <c r="B40" s="0" t="n">
+        <v>39</v>
+      </c>
+      <c r="C40" s="0" t="inlineStr">
+        <is>
+          <t>Teri Deewani</t>
+        </is>
+      </c>
+      <c r="D40" s="0" t="inlineStr">
+        <is>
+          <t>Kailash Kher</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" s="0" t="inlineStr">
+        <is>
+          <t>2026-04-06</t>
+        </is>
+      </c>
+      <c r="B41" s="0" t="n">
+        <v>40</v>
+      </c>
+      <c r="C41" s="0" t="inlineStr">
+        <is>
+          <t>Not Guilty</t>
+        </is>
+      </c>
+      <c r="D41" s="0" t="inlineStr">
+        <is>
+          <t>Dhanda Nyoliwala</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" s="0" t="inlineStr">
+        <is>
+          <t>2026-04-06</t>
+        </is>
+      </c>
+      <c r="B42" s="0" t="n">
+        <v>41</v>
+      </c>
+      <c r="C42" s="0" t="inlineStr">
+        <is>
+          <t>Ye Tune Kya Kiya</t>
+        </is>
+      </c>
+      <c r="D42" s="0" t="inlineStr">
+        <is>
+          <t>Pritam</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" s="0" t="inlineStr">
+        <is>
+          <t>2026-04-06</t>
+        </is>
+      </c>
+      <c r="B43" s="0" t="n">
+        <v>42</v>
+      </c>
+      <c r="C43" s="0" t="inlineStr">
+        <is>
+          <t>Mann Mera - Original Version</t>
+        </is>
+      </c>
+      <c r="D43" s="0" t="inlineStr">
+        <is>
+          <t>Gajendra Verma</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" s="0" t="inlineStr">
+        <is>
+          <t>2026-04-06</t>
+        </is>
+      </c>
+      <c r="B44" s="0" t="n">
+        <v>43</v>
+      </c>
+      <c r="C44" s="0" t="inlineStr">
+        <is>
+          <t>Main Aur Tu</t>
+        </is>
+      </c>
+      <c r="D44" s="0" t="inlineStr">
+        <is>
+          <t>Shashwat Sachdev</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" s="0" t="inlineStr">
+        <is>
+          <t>2026-04-06</t>
+        </is>
+      </c>
+      <c r="B45" s="0" t="n">
+        <v>44</v>
+      </c>
+      <c r="C45" s="0" t="inlineStr">
+        <is>
+          <t>Ehsaas</t>
+        </is>
+      </c>
+      <c r="D45" s="0" t="inlineStr">
+        <is>
+          <t>Faheem Abdullah</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" s="0" t="inlineStr">
+        <is>
+          <t>2026-04-06</t>
+        </is>
+      </c>
+      <c r="B46" s="0" t="n">
+        <v>45</v>
+      </c>
+      <c r="C46" s="0" t="inlineStr">
+        <is>
+          <t>Aaya Sher</t>
+        </is>
+      </c>
+      <c r="D46" s="0" t="inlineStr">
+        <is>
+          <t>Anirudh Ravichander</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" s="0" t="inlineStr">
+        <is>
+          <t>2026-04-06</t>
+        </is>
+      </c>
+      <c r="B47" s="0" t="n">
+        <v>46</v>
+      </c>
+      <c r="C47" s="0" t="inlineStr">
+        <is>
+          <t>Mutta Kalakki</t>
+        </is>
+      </c>
+      <c r="D47" s="0" t="inlineStr">
+        <is>
+          <t>G. V. Prakash</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" s="0" t="inlineStr">
+        <is>
+          <t>2026-04-06</t>
+        </is>
+      </c>
+      <c r="B48" s="0" t="n">
+        <v>47</v>
+      </c>
+      <c r="C48" s="0" t="inlineStr">
+        <is>
+          <t>Ishq Jalakar - Karvaan</t>
+        </is>
+      </c>
+      <c r="D48" s="0" t="inlineStr">
+        <is>
+          <t>Shashwat Sachdev</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" s="0" t="inlineStr">
+        <is>
+          <t>2026-04-06</t>
+        </is>
+      </c>
+      <c r="B49" s="0" t="n">
+        <v>48</v>
+      </c>
+      <c r="C49" s="0" t="inlineStr">
+        <is>
+          <t>Jogi</t>
+        </is>
+      </c>
+      <c r="D49" s="0" t="inlineStr">
+        <is>
+          <t>thiarajxtt</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" s="0" t="inlineStr">
+        <is>
+          <t>2026-04-06</t>
+        </is>
+      </c>
+      <c r="B50" s="0" t="n">
+        <v>49</v>
+      </c>
+      <c r="C50" s="0" t="inlineStr">
+        <is>
+          <t>Mast Magan</t>
+        </is>
+      </c>
+      <c r="D50" s="0" t="inlineStr">
+        <is>
+          <t>Arijit Singh</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" s="0" t="inlineStr">
+        <is>
+          <t>2026-04-06</t>
+        </is>
+      </c>
+      <c r="B51" s="0" t="n">
+        <v>50</v>
+      </c>
+      <c r="C51" s="0" t="inlineStr">
+        <is>
+          <t>Dhun</t>
+        </is>
+      </c>
+      <c r="D51" s="0" t="inlineStr">
+        <is>
+          <t>Mithoon</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet25.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:D51"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="24" t="inlineStr">
+        <is>
+          <t>Date</t>
+        </is>
+      </c>
+      <c r="B1" s="24" t="inlineStr">
+        <is>
+          <t>Rank</t>
+        </is>
+      </c>
+      <c r="C1" s="24" t="inlineStr">
+        <is>
+          <t>Song</t>
+        </is>
+      </c>
+      <c r="D1" s="24" t="inlineStr">
+        <is>
+          <t>Artist</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="0" t="inlineStr">
+        <is>
+          <t>2026-04-09</t>
+        </is>
+      </c>
+      <c r="B2" s="0" t="n">
+        <v>1</v>
+      </c>
+      <c r="C2" s="0" t="inlineStr">
+        <is>
+          <t>Bairan</t>
+        </is>
+      </c>
+      <c r="D2" s="0" t="inlineStr">
+        <is>
+          <t>Banjaare</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="0" t="inlineStr">
+        <is>
+          <t>2026-04-09</t>
+        </is>
+      </c>
+      <c r="B3" s="0" t="n">
+        <v>2</v>
+      </c>
+      <c r="C3" s="0" t="inlineStr">
+        <is>
+          <t>Jaiye Sajana</t>
+        </is>
+      </c>
+      <c r="D3" s="0" t="inlineStr">
+        <is>
+          <t>Shashwat Sachdev</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="0" t="inlineStr">
+        <is>
+          <t>2026-04-09</t>
+        </is>
+      </c>
+      <c r="B4" s="0" t="n">
+        <v>3</v>
+      </c>
+      <c r="C4" s="0" t="inlineStr">
+        <is>
+          <t>Gehra Hua</t>
+        </is>
+      </c>
+      <c r="D4" s="0" t="inlineStr">
+        <is>
+          <t>Shashwat Sachdev</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="0" t="inlineStr">
+        <is>
+          <t>2026-04-09</t>
+        </is>
+      </c>
+      <c r="B5" s="0" t="n">
+        <v>4</v>
+      </c>
+      <c r="C5" s="0" t="inlineStr">
+        <is>
+          <t>Sheesha - Aakhya Mai Aakh Ghali Jo Bairan</t>
+        </is>
+      </c>
+      <c r="D5" s="0" t="inlineStr">
+        <is>
+          <t>Mitta Ror</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="0" t="inlineStr">
+        <is>
+          <t>2026-04-09</t>
+        </is>
+      </c>
+      <c r="B6" s="0" t="n">
+        <v>5</v>
+      </c>
+      <c r="C6" s="0" t="inlineStr">
+        <is>
+          <t>Khat</t>
+        </is>
+      </c>
+      <c r="D6" s="0" t="inlineStr">
+        <is>
+          <t>Navjot Ahuja</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="0" t="inlineStr">
+        <is>
+          <t>2026-04-09</t>
+        </is>
+      </c>
+      <c r="B7" s="0" t="n">
+        <v>6</v>
+      </c>
+      <c r="C7" s="0" t="inlineStr">
+        <is>
+          <t>Dooron Dooron</t>
+        </is>
+      </c>
+      <c r="D7" s="0" t="inlineStr">
+        <is>
+          <t>Paresh Pahuja</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="0" t="inlineStr">
+        <is>
+          <t>2026-04-09</t>
+        </is>
+      </c>
+      <c r="B8" s="0" t="n">
+        <v>7</v>
+      </c>
+      <c r="C8" s="0" t="inlineStr">
+        <is>
+          <t>Dhurandhar The Revenge - Aari Aari</t>
+        </is>
+      </c>
+      <c r="D8" s="0" t="inlineStr">
+        <is>
+          <t>Shashwat Sachdev</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="0" t="inlineStr">
+        <is>
+          <t>2026-04-09</t>
+        </is>
+      </c>
+      <c r="B9" s="0" t="n">
+        <v>8</v>
+      </c>
+      <c r="C9" s="0" t="inlineStr">
+        <is>
+          <t>Apna Bana Le</t>
+        </is>
+      </c>
+      <c r="D9" s="0" t="inlineStr">
+        <is>
+          <t>Sachin-Jigar</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="0" t="inlineStr">
+        <is>
+          <t>2026-04-09</t>
+        </is>
+      </c>
+      <c r="B10" s="0" t="n">
+        <v>9</v>
+      </c>
+      <c r="C10" s="0" t="inlineStr">
+        <is>
+          <t>Samjhawan</t>
+        </is>
+      </c>
+      <c r="D10" s="0" t="inlineStr">
+        <is>
+          <t>Jawad Ahmad</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="0" t="inlineStr">
+        <is>
+          <t>2026-04-09</t>
+        </is>
+      </c>
+      <c r="B11" s="0" t="n">
+        <v>10</v>
+      </c>
+      <c r="C11" s="0" t="inlineStr">
+        <is>
+          <t>Sahiba</t>
+        </is>
+      </c>
+      <c r="D11" s="0" t="inlineStr">
+        <is>
+          <t>Aditya Rikhari</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="0" t="inlineStr">
+        <is>
+          <t>2026-04-09</t>
+        </is>
+      </c>
+      <c r="B12" s="0" t="n">
+        <v>11</v>
+      </c>
+      <c r="C12" s="0" t="inlineStr">
+        <is>
+          <t>Jaan Se Guzarte Hain</t>
+        </is>
+      </c>
+      <c r="D12" s="0" t="inlineStr">
+        <is>
+          <t>Shashwat Sachdev</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="0" t="inlineStr">
+        <is>
+          <t>2026-04-09</t>
+        </is>
+      </c>
+      <c r="B13" s="0" t="n">
+        <v>12</v>
+      </c>
+      <c r="C13" s="0" t="inlineStr">
+        <is>
+          <t>Finding Her</t>
+        </is>
+      </c>
+      <c r="D13" s="0" t="inlineStr">
+        <is>
+          <t>Kushagra</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="0" t="inlineStr">
+        <is>
+          <t>2026-04-09</t>
+        </is>
+      </c>
+      <c r="B14" s="0" t="n">
+        <v>13</v>
+      </c>
+      <c r="C14" s="0" t="inlineStr">
+        <is>
+          <t>Sitaare</t>
+        </is>
+      </c>
+      <c r="D14" s="0" t="inlineStr">
+        <is>
+          <t>Arijit Singh</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="0" t="inlineStr">
+        <is>
+          <t>2026-04-09</t>
+        </is>
+      </c>
+      <c r="B15" s="0" t="n">
+        <v>14</v>
+      </c>
+      <c r="C15" s="0" t="inlineStr">
+        <is>
+          <t>Pavazha Malli</t>
+        </is>
+      </c>
+      <c r="D15" s="0" t="inlineStr">
+        <is>
+          <t>Sai Abhyankkar</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="0" t="inlineStr">
+        <is>
+          <t>2026-04-09</t>
+        </is>
+      </c>
+      <c r="B16" s="0" t="n">
+        <v>15</v>
+      </c>
+      <c r="C16" s="0" t="inlineStr">
+        <is>
+          <t>Arz Kiya Hai | Coke Studio Bharat</t>
+        </is>
+      </c>
+      <c r="D16" s="0" t="inlineStr">
+        <is>
+          <t>Anuv Jain</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="0" t="inlineStr">
+        <is>
+          <t>2026-04-09</t>
+        </is>
+      </c>
+      <c r="B17" s="0" t="n">
+        <v>16</v>
+      </c>
+      <c r="C17" s="0" t="inlineStr">
+        <is>
+          <t>Boyfriend</t>
+        </is>
+      </c>
+      <c r="D17" s="0" t="inlineStr">
+        <is>
+          <t>Karan Aujla</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="0" t="inlineStr">
+        <is>
+          <t>2026-04-09</t>
+        </is>
+      </c>
+      <c r="B18" s="0" t="n">
+        <v>17</v>
+      </c>
+      <c r="C18" s="0" t="inlineStr">
+        <is>
+          <t>Mann Mera</t>
+        </is>
+      </c>
+      <c r="D18" s="0" t="inlineStr">
+        <is>
+          <t>Gajendra Verma</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="0" t="inlineStr">
+        <is>
+          <t>2026-04-09</t>
+        </is>
+      </c>
+      <c r="B19" s="0" t="n">
+        <v>18</v>
+      </c>
+      <c r="C19" s="0" t="inlineStr">
+        <is>
+          <t>Shararat</t>
+        </is>
+      </c>
+      <c r="D19" s="0" t="inlineStr">
+        <is>
+          <t>Shashwat Sachdev</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="0" t="inlineStr">
+        <is>
+          <t>2026-04-09</t>
+        </is>
+      </c>
+      <c r="B20" s="0" t="n">
+        <v>19</v>
+      </c>
+      <c r="C20" s="0" t="inlineStr">
+        <is>
+          <t>Ishq</t>
+        </is>
+      </c>
+      <c r="D20" s="0" t="inlineStr">
+        <is>
+          <t>Faheem Abdullah</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="0" t="inlineStr">
+        <is>
+          <t>2026-04-09</t>
+        </is>
+      </c>
+      <c r="B21" s="0" t="n">
+        <v>20</v>
+      </c>
+      <c r="C21" s="0" t="inlineStr">
+        <is>
+          <t>Saiyaara</t>
+        </is>
+      </c>
+      <c r="D21" s="0" t="inlineStr">
+        <is>
+          <t>Tanishk Bagchi</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="0" t="inlineStr">
+        <is>
+          <t>2026-04-09</t>
+        </is>
+      </c>
+      <c r="B22" s="0" t="n">
+        <v>21</v>
+      </c>
+      <c r="C22" s="0" t="inlineStr">
+        <is>
+          <t>Tere Liye</t>
+        </is>
+      </c>
+      <c r="D22" s="0" t="inlineStr">
+        <is>
+          <t>Atif Aslam</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="0" t="inlineStr">
+        <is>
+          <t>2026-04-09</t>
+        </is>
+      </c>
+      <c r="B23" s="0" t="n">
+        <v>22</v>
+      </c>
+      <c r="C23" s="0" t="inlineStr">
+        <is>
+          <t>Darkhaast</t>
+        </is>
+      </c>
+      <c r="D23" s="0" t="inlineStr">
+        <is>
+          <t>Mithoon</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="0" t="inlineStr">
+        <is>
+          <t>2026-04-09</t>
+        </is>
+      </c>
+      <c r="B24" s="0" t="n">
+        <v>23</v>
+      </c>
+      <c r="C24" s="0" t="inlineStr">
+        <is>
+          <t>Ishqa Ve</t>
+        </is>
+      </c>
+      <c r="D24" s="0" t="inlineStr">
+        <is>
+          <t>Zeeshan Ali</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="0" t="inlineStr">
+        <is>
+          <t>2026-04-09</t>
+        </is>
+      </c>
+      <c r="B25" s="0" t="n">
+        <v>24</v>
+      </c>
+      <c r="C25" s="0" t="inlineStr">
+        <is>
+          <t>For A Reason</t>
+        </is>
+      </c>
+      <c r="D25" s="0" t="inlineStr">
+        <is>
+          <t>Karan Aujla</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="0" t="inlineStr">
+        <is>
+          <t>2026-04-09</t>
+        </is>
+      </c>
+      <c r="B26" s="0" t="n">
+        <v>25</v>
+      </c>
+      <c r="C26" s="0" t="inlineStr">
+        <is>
+          <t>Dhurandhar - Title Track</t>
+        </is>
+      </c>
+      <c r="D26" s="0" t="inlineStr">
+        <is>
+          <t>Shashwat Sachdev</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="0" t="inlineStr">
+        <is>
+          <t>2026-04-09</t>
+        </is>
+      </c>
+      <c r="B27" s="0" t="n">
+        <v>26</v>
+      </c>
+      <c r="C27" s="0" t="inlineStr">
+        <is>
+          <t>Naal Nachna</t>
+        </is>
+      </c>
+      <c r="D27" s="0" t="inlineStr">
+        <is>
+          <t>Shashwat Sachdev</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="0" t="inlineStr">
+        <is>
+          <t>2026-04-09</t>
+        </is>
+      </c>
+      <c r="B28" s="0" t="n">
+        <v>27</v>
+      </c>
+      <c r="C28" s="0" t="inlineStr">
+        <is>
+          <t>Bairi</t>
+        </is>
+      </c>
+      <c r="D28" s="0" t="inlineStr">
+        <is>
+          <t>Virat</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="0" t="inlineStr">
+        <is>
+          <t>2026-04-09</t>
+        </is>
+      </c>
+      <c r="B29" s="0" t="n">
+        <v>28</v>
+      </c>
+      <c r="C29" s="0" t="inlineStr">
+        <is>
+          <t>Tum Ho Toh</t>
+        </is>
+      </c>
+      <c r="D29" s="0" t="inlineStr">
+        <is>
+          <t>Vishal Mishra</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="0" t="inlineStr">
+        <is>
+          <t>2026-04-09</t>
+        </is>
+      </c>
+      <c r="B30" s="0" t="n">
+        <v>29</v>
+      </c>
+      <c r="C30" s="0" t="inlineStr">
+        <is>
+          <t>Deewaana Deewaana</t>
+        </is>
+      </c>
+      <c r="D30" s="0" t="inlineStr">
+        <is>
+          <t>A.R. Rahman</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="0" t="inlineStr">
+        <is>
+          <t>2026-04-09</t>
+        </is>
+      </c>
+      <c r="B31" s="0" t="n">
+        <v>30</v>
+      </c>
+      <c r="C31" s="0" t="inlineStr">
+        <is>
+          <t>Phir Se</t>
+        </is>
+      </c>
+      <c r="D31" s="0" t="inlineStr">
+        <is>
+          <t>Shashwat Sachdev</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="0" t="inlineStr">
+        <is>
+          <t>2026-04-09</t>
+        </is>
+      </c>
+      <c r="B32" s="0" t="n">
+        <v>31</v>
+      </c>
+      <c r="C32" s="0" t="inlineStr">
+        <is>
+          <t>Raanjhan</t>
+        </is>
+      </c>
+      <c r="D32" s="0" t="inlineStr">
+        <is>
+          <t>Sachet-Parampara</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="0" t="inlineStr">
+        <is>
+          <t>2026-04-09</t>
+        </is>
+      </c>
+      <c r="B33" s="0" t="n">
+        <v>32</v>
+      </c>
+      <c r="C33" s="0" t="inlineStr">
+        <is>
+          <t>Agar Tum Saath Ho</t>
+        </is>
+      </c>
+      <c r="D33" s="0" t="inlineStr">
+        <is>
+          <t>Alka Yagnik</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="0" t="inlineStr">
+        <is>
+          <t>2026-04-09</t>
+        </is>
+      </c>
+      <c r="B34" s="0" t="n">
+        <v>33</v>
+      </c>
+      <c r="C34" s="0" t="inlineStr">
+        <is>
+          <t>Tere Bina</t>
+        </is>
+      </c>
+      <c r="D34" s="0" t="inlineStr">
+        <is>
+          <t>A.R. Rahman</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="0" t="inlineStr">
+        <is>
+          <t>2026-04-09</t>
+        </is>
+      </c>
+      <c r="B35" s="0" t="n">
+        <v>34</v>
+      </c>
+      <c r="C35" s="0" t="inlineStr">
+        <is>
+          <t>Jogi</t>
+        </is>
+      </c>
+      <c r="D35" s="0" t="inlineStr">
+        <is>
+          <t>thiarajxtt</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="0" t="inlineStr">
+        <is>
+          <t>2026-04-09</t>
+        </is>
+      </c>
+      <c r="B36" s="0" t="n">
+        <v>35</v>
+      </c>
+      <c r="C36" s="0" t="inlineStr">
+        <is>
+          <t>Jo Tum Mere Ho</t>
+        </is>
+      </c>
+      <c r="D36" s="0" t="inlineStr">
+        <is>
+          <t>Anuv Jain</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="0" t="inlineStr">
+        <is>
+          <t>2026-04-09</t>
+        </is>
+      </c>
+      <c r="B37" s="0" t="n">
+        <v>36</v>
+      </c>
+      <c r="C37" s="0" t="inlineStr">
+        <is>
+          <t>Haseen</t>
+        </is>
+      </c>
+      <c r="D37" s="0" t="inlineStr">
+        <is>
+          <t>Talwiinder</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="0" t="inlineStr">
+        <is>
+          <t>2026-04-09</t>
+        </is>
+      </c>
+      <c r="B38" s="0" t="n">
+        <v>37</v>
+      </c>
+      <c r="C38" s="0" t="inlineStr">
+        <is>
+          <t>Barbaad</t>
+        </is>
+      </c>
+      <c r="D38" s="0" t="inlineStr">
+        <is>
+          <t>The Rish</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="0" t="inlineStr">
+        <is>
+          <t>2026-04-09</t>
+        </is>
+      </c>
+      <c r="B39" s="0" t="n">
+        <v>38</v>
+      </c>
+      <c r="C39" s="0" t="inlineStr">
+        <is>
+          <t>Run Down The City - Monica</t>
+        </is>
+      </c>
+      <c r="D39" s="0" t="inlineStr">
+        <is>
+          <t>Shashwat Sachdev</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="0" t="inlineStr">
+        <is>
+          <t>2026-04-09</t>
+        </is>
+      </c>
+      <c r="B40" s="0" t="n">
+        <v>39</v>
+      </c>
+      <c r="C40" s="0" t="inlineStr">
+        <is>
+          <t>Lutt Le Gaya</t>
+        </is>
+      </c>
+      <c r="D40" s="0" t="inlineStr">
+        <is>
+          <t>Shashwat Sachdev</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" s="0" t="inlineStr">
+        <is>
+          <t>2026-04-09</t>
+        </is>
+      </c>
+      <c r="B41" s="0" t="n">
+        <v>40</v>
+      </c>
+      <c r="C41" s="0" t="inlineStr">
+        <is>
+          <t>Teri Deewani</t>
+        </is>
+      </c>
+      <c r="D41" s="0" t="inlineStr">
+        <is>
+          <t>Kailash Kher</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" s="0" t="inlineStr">
+        <is>
+          <t>2026-04-09</t>
+        </is>
+      </c>
+      <c r="B42" s="0" t="n">
+        <v>41</v>
+      </c>
+      <c r="C42" s="0" t="inlineStr">
+        <is>
+          <t>Mann Mera - Original Version</t>
+        </is>
+      </c>
+      <c r="D42" s="0" t="inlineStr">
+        <is>
+          <t>Gajendra Verma</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" s="0" t="inlineStr">
+        <is>
+          <t>2026-04-09</t>
+        </is>
+      </c>
+      <c r="B43" s="0" t="n">
+        <v>42</v>
+      </c>
+      <c r="C43" s="0" t="inlineStr">
+        <is>
+          <t>Ye Tune Kya Kiya</t>
+        </is>
+      </c>
+      <c r="D43" s="0" t="inlineStr">
+        <is>
+          <t>Pritam</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" s="0" t="inlineStr">
+        <is>
+          <t>2026-04-09</t>
+        </is>
+      </c>
+      <c r="B44" s="0" t="n">
+        <v>43</v>
+      </c>
+      <c r="C44" s="0" t="inlineStr">
+        <is>
+          <t>Ehsaas</t>
+        </is>
+      </c>
+      <c r="D44" s="0" t="inlineStr">
+        <is>
+          <t>Faheem Abdullah</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" s="0" t="inlineStr">
+        <is>
+          <t>2026-04-09</t>
+        </is>
+      </c>
+      <c r="B45" s="0" t="n">
+        <v>44</v>
+      </c>
+      <c r="C45" s="0" t="inlineStr">
+        <is>
+          <t>Not Guilty</t>
+        </is>
+      </c>
+      <c r="D45" s="0" t="inlineStr">
+        <is>
+          <t>Dhanda Nyoliwala</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" s="0" t="inlineStr">
+        <is>
+          <t>2026-04-09</t>
+        </is>
+      </c>
+      <c r="B46" s="0" t="n">
+        <v>45</v>
+      </c>
+      <c r="C46" s="0" t="inlineStr">
+        <is>
+          <t>Mast Magan</t>
+        </is>
+      </c>
+      <c r="D46" s="0" t="inlineStr">
+        <is>
+          <t>Arijit Singh</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" s="0" t="inlineStr">
+        <is>
+          <t>2026-04-09</t>
+        </is>
+      </c>
+      <c r="B47" s="0" t="n">
+        <v>46</v>
+      </c>
+      <c r="C47" s="0" t="inlineStr">
+        <is>
+          <t>Thodi Si Daaru</t>
+        </is>
+      </c>
+      <c r="D47" s="0" t="inlineStr">
+        <is>
+          <t>AP Dhillon</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" s="0" t="inlineStr">
+        <is>
+          <t>2026-04-09</t>
+        </is>
+      </c>
+      <c r="B48" s="0" t="n">
+        <v>47</v>
+      </c>
+      <c r="C48" s="0" t="inlineStr">
+        <is>
+          <t>High On You</t>
+        </is>
+      </c>
+      <c r="D48" s="0" t="inlineStr">
+        <is>
+          <t>Jind Universe</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" s="0" t="inlineStr">
+        <is>
+          <t>2026-04-09</t>
+        </is>
+      </c>
+      <c r="B49" s="0" t="n">
+        <v>48</v>
+      </c>
+      <c r="C49" s="0" t="inlineStr">
+        <is>
+          <t>Main Aur Tu</t>
+        </is>
+      </c>
+      <c r="D49" s="0" t="inlineStr">
+        <is>
+          <t>Shashwat Sachdev</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" s="0" t="inlineStr">
+        <is>
+          <t>2026-04-09</t>
+        </is>
+      </c>
+      <c r="B50" s="0" t="n">
+        <v>49</v>
+      </c>
+      <c r="C50" s="0" t="inlineStr">
+        <is>
+          <t>Aaya Sher</t>
+        </is>
+      </c>
+      <c r="D50" s="0" t="inlineStr">
+        <is>
+          <t>Anirudh Ravichander</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" s="0" t="inlineStr">
+        <is>
+          <t>2026-04-09</t>
+        </is>
+      </c>
+      <c r="B51" s="0" t="n">
+        <v>50</v>
+      </c>
+      <c r="C51" s="0" t="inlineStr">
+        <is>
+          <t>Ishq Jalakar - Karvaan</t>
+        </is>
+      </c>
+      <c r="D51" s="0" t="inlineStr">
+        <is>
+          <t>Shashwat Sachdev</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet26.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:D51"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="24" t="inlineStr">
+        <is>
+          <t>Date</t>
+        </is>
+      </c>
+      <c r="B1" s="24" t="inlineStr">
+        <is>
+          <t>Rank</t>
+        </is>
+      </c>
+      <c r="C1" s="24" t="inlineStr">
+        <is>
+          <t>Song</t>
+        </is>
+      </c>
+      <c r="D1" s="24" t="inlineStr">
+        <is>
+          <t>Artist</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="0" t="inlineStr">
+        <is>
+          <t>2026-04-07</t>
+        </is>
+      </c>
+      <c r="B2" s="0" t="n">
+        <v>1</v>
+      </c>
+      <c r="C2" s="0" t="inlineStr">
+        <is>
+          <t>Bairan</t>
+        </is>
+      </c>
+      <c r="D2" s="0" t="inlineStr">
+        <is>
+          <t>Banjaare</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="0" t="inlineStr">
+        <is>
+          <t>2026-04-07</t>
+        </is>
+      </c>
+      <c r="B3" s="0" t="n">
+        <v>2</v>
+      </c>
+      <c r="C3" s="0" t="inlineStr">
+        <is>
+          <t>Jaiye Sajana</t>
+        </is>
+      </c>
+      <c r="D3" s="0" t="inlineStr">
+        <is>
+          <t>Shashwat Sachdev</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="0" t="inlineStr">
+        <is>
+          <t>2026-04-07</t>
+        </is>
+      </c>
+      <c r="B4" s="0" t="n">
+        <v>3</v>
+      </c>
+      <c r="C4" s="0" t="inlineStr">
+        <is>
+          <t>Gehra Hua</t>
+        </is>
+      </c>
+      <c r="D4" s="0" t="inlineStr">
+        <is>
+          <t>Shashwat Sachdev</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="0" t="inlineStr">
+        <is>
+          <t>2026-04-07</t>
+        </is>
+      </c>
+      <c r="B5" s="0" t="n">
+        <v>4</v>
+      </c>
+      <c r="C5" s="0" t="inlineStr">
+        <is>
+          <t>Sheesha - Aakhya Mai Aakh Ghali Jo Bairan</t>
+        </is>
+      </c>
+      <c r="D5" s="0" t="inlineStr">
+        <is>
+          <t>Mitta Ror</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="0" t="inlineStr">
+        <is>
+          <t>2026-04-07</t>
+        </is>
+      </c>
+      <c r="B6" s="0" t="n">
+        <v>5</v>
+      </c>
+      <c r="C6" s="0" t="inlineStr">
+        <is>
+          <t>Khat</t>
+        </is>
+      </c>
+      <c r="D6" s="0" t="inlineStr">
+        <is>
+          <t>Navjot Ahuja</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="0" t="inlineStr">
+        <is>
+          <t>2026-04-07</t>
+        </is>
+      </c>
+      <c r="B7" s="0" t="n">
+        <v>6</v>
+      </c>
+      <c r="C7" s="0" t="inlineStr">
+        <is>
+          <t>Dhurandhar The Revenge - Aari Aari</t>
+        </is>
+      </c>
+      <c r="D7" s="0" t="inlineStr">
+        <is>
+          <t>Shashwat Sachdev</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="0" t="inlineStr">
+        <is>
+          <t>2026-04-07</t>
+        </is>
+      </c>
+      <c r="B8" s="0" t="n">
+        <v>7</v>
+      </c>
+      <c r="C8" s="0" t="inlineStr">
+        <is>
+          <t>Sahiba</t>
+        </is>
+      </c>
+      <c r="D8" s="0" t="inlineStr">
+        <is>
+          <t>Aditya Rikhari</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="0" t="inlineStr">
+        <is>
+          <t>2026-04-07</t>
+        </is>
+      </c>
+      <c r="B9" s="0" t="n">
+        <v>8</v>
+      </c>
+      <c r="C9" s="0" t="inlineStr">
+        <is>
+          <t>Dooron Dooron</t>
+        </is>
+      </c>
+      <c r="D9" s="0" t="inlineStr">
+        <is>
+          <t>Paresh Pahuja</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="0" t="inlineStr">
+        <is>
+          <t>2026-04-07</t>
+        </is>
+      </c>
+      <c r="B10" s="0" t="n">
+        <v>9</v>
+      </c>
+      <c r="C10" s="0" t="inlineStr">
+        <is>
+          <t>Apna Bana Le</t>
+        </is>
+      </c>
+      <c r="D10" s="0" t="inlineStr">
+        <is>
+          <t>Sachin-Jigar</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="0" t="inlineStr">
+        <is>
+          <t>2026-04-07</t>
+        </is>
+      </c>
+      <c r="B11" s="0" t="n">
+        <v>10</v>
+      </c>
+      <c r="C11" s="0" t="inlineStr">
+        <is>
+          <t>Sitaare</t>
+        </is>
+      </c>
+      <c r="D11" s="0" t="inlineStr">
+        <is>
+          <t>Arijit Singh</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="0" t="inlineStr">
+        <is>
+          <t>2026-04-07</t>
+        </is>
+      </c>
+      <c r="B12" s="0" t="n">
+        <v>11</v>
+      </c>
+      <c r="C12" s="0" t="inlineStr">
+        <is>
+          <t>Jaan Se Guzarte Hain</t>
+        </is>
+      </c>
+      <c r="D12" s="0" t="inlineStr">
+        <is>
+          <t>Shashwat Sachdev</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="0" t="inlineStr">
+        <is>
+          <t>2026-04-07</t>
+        </is>
+      </c>
+      <c r="B13" s="0" t="n">
+        <v>12</v>
+      </c>
+      <c r="C13" s="0" t="inlineStr">
+        <is>
+          <t>Samjhawan</t>
+        </is>
+      </c>
+      <c r="D13" s="0" t="inlineStr">
+        <is>
+          <t>Jawad Ahmad</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="0" t="inlineStr">
+        <is>
+          <t>2026-04-07</t>
+        </is>
+      </c>
+      <c r="B14" s="0" t="n">
+        <v>13</v>
+      </c>
+      <c r="C14" s="0" t="inlineStr">
+        <is>
+          <t>Finding Her</t>
+        </is>
+      </c>
+      <c r="D14" s="0" t="inlineStr">
+        <is>
+          <t>Kushagra</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="0" t="inlineStr">
+        <is>
+          <t>2026-04-07</t>
+        </is>
+      </c>
+      <c r="B15" s="0" t="n">
+        <v>14</v>
+      </c>
+      <c r="C15" s="0" t="inlineStr">
+        <is>
+          <t>Pavazha Malli</t>
+        </is>
+      </c>
+      <c r="D15" s="0" t="inlineStr">
+        <is>
+          <t>Sai Abhyankkar</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="0" t="inlineStr">
+        <is>
+          <t>2026-04-07</t>
+        </is>
+      </c>
+      <c r="B16" s="0" t="n">
+        <v>15</v>
+      </c>
+      <c r="C16" s="0" t="inlineStr">
+        <is>
+          <t>Arz Kiya Hai | Coke Studio Bharat</t>
+        </is>
+      </c>
+      <c r="D16" s="0" t="inlineStr">
+        <is>
+          <t>Anuv Jain</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="0" t="inlineStr">
+        <is>
+          <t>2026-04-07</t>
+        </is>
+      </c>
+      <c r="B17" s="0" t="n">
+        <v>16</v>
+      </c>
+      <c r="C17" s="0" t="inlineStr">
+        <is>
+          <t>Boyfriend</t>
+        </is>
+      </c>
+      <c r="D17" s="0" t="inlineStr">
+        <is>
+          <t>Karan Aujla</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="0" t="inlineStr">
+        <is>
+          <t>2026-04-07</t>
+        </is>
+      </c>
+      <c r="B18" s="0" t="n">
+        <v>17</v>
+      </c>
+      <c r="C18" s="0" t="inlineStr">
+        <is>
+          <t>Ishq</t>
+        </is>
+      </c>
+      <c r="D18" s="0" t="inlineStr">
+        <is>
+          <t>Faheem Abdullah</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="0" t="inlineStr">
+        <is>
+          <t>2026-04-07</t>
+        </is>
+      </c>
+      <c r="B19" s="0" t="n">
+        <v>18</v>
+      </c>
+      <c r="C19" s="0" t="inlineStr">
+        <is>
+          <t>Shararat</t>
+        </is>
+      </c>
+      <c r="D19" s="0" t="inlineStr">
+        <is>
+          <t>Shashwat Sachdev</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="0" t="inlineStr">
+        <is>
+          <t>2026-04-07</t>
+        </is>
+      </c>
+      <c r="B20" s="0" t="n">
+        <v>19</v>
+      </c>
+      <c r="C20" s="0" t="inlineStr">
+        <is>
+          <t>Dhurandhar - Title Track</t>
+        </is>
+      </c>
+      <c r="D20" s="0" t="inlineStr">
+        <is>
+          <t>Shashwat Sachdev</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="0" t="inlineStr">
+        <is>
+          <t>2026-04-07</t>
+        </is>
+      </c>
+      <c r="B21" s="0" t="n">
+        <v>20</v>
+      </c>
+      <c r="C21" s="0" t="inlineStr">
+        <is>
+          <t>Saiyaara</t>
+        </is>
+      </c>
+      <c r="D21" s="0" t="inlineStr">
+        <is>
+          <t>Tanishk Bagchi</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="0" t="inlineStr">
+        <is>
+          <t>2026-04-07</t>
+        </is>
+      </c>
+      <c r="B22" s="0" t="n">
+        <v>21</v>
+      </c>
+      <c r="C22" s="0" t="inlineStr">
+        <is>
+          <t>Mann Mera</t>
+        </is>
+      </c>
+      <c r="D22" s="0" t="inlineStr">
+        <is>
+          <t>Gajendra Verma</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="0" t="inlineStr">
+        <is>
+          <t>2026-04-07</t>
+        </is>
+      </c>
+      <c r="B23" s="0" t="n">
+        <v>22</v>
+      </c>
+      <c r="C23" s="0" t="inlineStr">
+        <is>
+          <t>Ishqa Ve</t>
+        </is>
+      </c>
+      <c r="D23" s="0" t="inlineStr">
+        <is>
+          <t>Zeeshan Ali</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="0" t="inlineStr">
+        <is>
+          <t>2026-04-07</t>
+        </is>
+      </c>
+      <c r="B24" s="0" t="n">
+        <v>23</v>
+      </c>
+      <c r="C24" s="0" t="inlineStr">
+        <is>
+          <t>Jogi</t>
+        </is>
+      </c>
+      <c r="D24" s="0" t="inlineStr">
+        <is>
+          <t>thiarajxtt</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="0" t="inlineStr">
+        <is>
+          <t>2026-04-07</t>
+        </is>
+      </c>
+      <c r="B25" s="0" t="n">
+        <v>24</v>
+      </c>
+      <c r="C25" s="0" t="inlineStr">
+        <is>
+          <t>Raanjhan</t>
+        </is>
+      </c>
+      <c r="D25" s="0" t="inlineStr">
+        <is>
+          <t>Sachet-Parampara</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="0" t="inlineStr">
+        <is>
+          <t>2026-04-07</t>
+        </is>
+      </c>
+      <c r="B26" s="0" t="n">
+        <v>25</v>
+      </c>
+      <c r="C26" s="0" t="inlineStr">
+        <is>
+          <t>Bairi</t>
+        </is>
+      </c>
+      <c r="D26" s="0" t="inlineStr">
+        <is>
+          <t>Virat</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="0" t="inlineStr">
+        <is>
+          <t>2026-04-07</t>
+        </is>
+      </c>
+      <c r="B27" s="0" t="n">
+        <v>26</v>
+      </c>
+      <c r="C27" s="0" t="inlineStr">
+        <is>
+          <t>For A Reason</t>
+        </is>
+      </c>
+      <c r="D27" s="0" t="inlineStr">
+        <is>
+          <t>Karan Aujla</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="0" t="inlineStr">
+        <is>
+          <t>2026-04-07</t>
+        </is>
+      </c>
+      <c r="B28" s="0" t="n">
+        <v>27</v>
+      </c>
+      <c r="C28" s="0" t="inlineStr">
+        <is>
+          <t>Jo Tum Mere Ho</t>
+        </is>
+      </c>
+      <c r="D28" s="0" t="inlineStr">
+        <is>
+          <t>Anuv Jain</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="0" t="inlineStr">
+        <is>
+          <t>2026-04-07</t>
+        </is>
+      </c>
+      <c r="B29" s="0" t="n">
+        <v>28</v>
+      </c>
+      <c r="C29" s="0" t="inlineStr">
+        <is>
+          <t>Tere Liye</t>
+        </is>
+      </c>
+      <c r="D29" s="0" t="inlineStr">
+        <is>
+          <t>Atif Aslam</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="0" t="inlineStr">
+        <is>
+          <t>2026-04-07</t>
+        </is>
+      </c>
+      <c r="B30" s="0" t="n">
+        <v>29</v>
+      </c>
+      <c r="C30" s="0" t="inlineStr">
+        <is>
+          <t>Phir Se</t>
+        </is>
+      </c>
+      <c r="D30" s="0" t="inlineStr">
+        <is>
+          <t>Shashwat Sachdev</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="0" t="inlineStr">
+        <is>
+          <t>2026-04-07</t>
+        </is>
+      </c>
+      <c r="B31" s="0" t="n">
+        <v>30</v>
+      </c>
+      <c r="C31" s="0" t="inlineStr">
+        <is>
+          <t>Naal Nachna</t>
+        </is>
+      </c>
+      <c r="D31" s="0" t="inlineStr">
+        <is>
+          <t>Shashwat Sachdev</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="0" t="inlineStr">
+        <is>
+          <t>2026-04-07</t>
+        </is>
+      </c>
+      <c r="B32" s="0" t="n">
+        <v>31</v>
+      </c>
+      <c r="C32" s="0" t="inlineStr">
+        <is>
+          <t>Darkhaast</t>
+        </is>
+      </c>
+      <c r="D32" s="0" t="inlineStr">
+        <is>
+          <t>Mithoon</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="0" t="inlineStr">
+        <is>
+          <t>2026-04-07</t>
+        </is>
+      </c>
+      <c r="B33" s="0" t="n">
+        <v>32</v>
+      </c>
+      <c r="C33" s="0" t="inlineStr">
+        <is>
+          <t>Deewaana Deewaana</t>
+        </is>
+      </c>
+      <c r="D33" s="0" t="inlineStr">
+        <is>
+          <t>A.R. Rahman</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="0" t="inlineStr">
+        <is>
+          <t>2026-04-07</t>
+        </is>
+      </c>
+      <c r="B34" s="0" t="n">
+        <v>33</v>
+      </c>
+      <c r="C34" s="0" t="inlineStr">
+        <is>
+          <t>Haseen</t>
+        </is>
+      </c>
+      <c r="D34" s="0" t="inlineStr">
+        <is>
+          <t>Talwiinder</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="0" t="inlineStr">
+        <is>
+          <t>2026-04-07</t>
+        </is>
+      </c>
+      <c r="B35" s="0" t="n">
+        <v>34</v>
+      </c>
+      <c r="C35" s="0" t="inlineStr">
+        <is>
+          <t>Run Down The City - Monica</t>
+        </is>
+      </c>
+      <c r="D35" s="0" t="inlineStr">
+        <is>
+          <t>Shashwat Sachdev</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="0" t="inlineStr">
+        <is>
+          <t>2026-04-07</t>
+        </is>
+      </c>
+      <c r="B36" s="0" t="n">
+        <v>35</v>
+      </c>
+      <c r="C36" s="0" t="inlineStr">
+        <is>
+          <t>Tum Ho Toh</t>
+        </is>
+      </c>
+      <c r="D36" s="0" t="inlineStr">
+        <is>
+          <t>Vishal Mishra</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="0" t="inlineStr">
+        <is>
+          <t>2026-04-07</t>
+        </is>
+      </c>
+      <c r="B37" s="0" t="n">
+        <v>36</v>
+      </c>
+      <c r="C37" s="0" t="inlineStr">
+        <is>
+          <t>Lutt Le Gaya</t>
+        </is>
+      </c>
+      <c r="D37" s="0" t="inlineStr">
+        <is>
+          <t>Shashwat Sachdev</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="0" t="inlineStr">
+        <is>
+          <t>2026-04-07</t>
+        </is>
+      </c>
+      <c r="B38" s="0" t="n">
+        <v>37</v>
+      </c>
+      <c r="C38" s="0" t="inlineStr">
+        <is>
+          <t>Agar Tum Saath Ho</t>
+        </is>
+      </c>
+      <c r="D38" s="0" t="inlineStr">
+        <is>
+          <t>Alka Yagnik</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="0" t="inlineStr">
+        <is>
+          <t>2026-04-07</t>
+        </is>
+      </c>
+      <c r="B39" s="0" t="n">
+        <v>38</v>
+      </c>
+      <c r="C39" s="0" t="inlineStr">
+        <is>
+          <t>Tere Bina</t>
+        </is>
+      </c>
+      <c r="D39" s="0" t="inlineStr">
+        <is>
+          <t>A.R. Rahman</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="0" t="inlineStr">
+        <is>
+          <t>2026-04-07</t>
+        </is>
+      </c>
+      <c r="B40" s="0" t="n">
+        <v>39</v>
+      </c>
+      <c r="C40" s="0" t="inlineStr">
+        <is>
+          <t>Barbaad</t>
+        </is>
+      </c>
+      <c r="D40" s="0" t="inlineStr">
+        <is>
+          <t>The Rish</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" s="0" t="inlineStr">
+        <is>
+          <t>2026-04-07</t>
+        </is>
+      </c>
+      <c r="B41" s="0" t="n">
+        <v>40</v>
+      </c>
+      <c r="C41" s="0" t="inlineStr">
+        <is>
+          <t>Ye Tune Kya Kiya</t>
+        </is>
+      </c>
+      <c r="D41" s="0" t="inlineStr">
+        <is>
+          <t>Pritam</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" s="0" t="inlineStr">
+        <is>
+          <t>2026-04-07</t>
+        </is>
+      </c>
+      <c r="B42" s="0" t="n">
+        <v>41</v>
+      </c>
+      <c r="C42" s="0" t="inlineStr">
+        <is>
+          <t>Teri Deewani</t>
+        </is>
+      </c>
+      <c r="D42" s="0" t="inlineStr">
+        <is>
+          <t>Kailash Kher</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" s="0" t="inlineStr">
+        <is>
+          <t>2026-04-07</t>
+        </is>
+      </c>
+      <c r="B43" s="0" t="n">
+        <v>42</v>
+      </c>
+      <c r="C43" s="0" t="inlineStr">
+        <is>
+          <t>Shree Hanuman Chalisa</t>
+        </is>
+      </c>
+      <c r="D43" s="0" t="inlineStr">
+        <is>
+          <t>Hariharan</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" s="0" t="inlineStr">
+        <is>
+          <t>2026-04-07</t>
+        </is>
+      </c>
+      <c r="B44" s="0" t="n">
+        <v>43</v>
+      </c>
+      <c r="C44" s="0" t="inlineStr">
+        <is>
+          <t>Zaalima</t>
+        </is>
+      </c>
+      <c r="D44" s="0" t="inlineStr">
+        <is>
+          <t>Arijit Singh</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" s="0" t="inlineStr">
+        <is>
+          <t>2026-04-07</t>
+        </is>
+      </c>
+      <c r="B45" s="0" t="n">
+        <v>44</v>
+      </c>
+      <c r="C45" s="0" t="inlineStr">
+        <is>
+          <t>Mann Mera - Original Version</t>
+        </is>
+      </c>
+      <c r="D45" s="0" t="inlineStr">
+        <is>
+          <t>Gajendra Verma</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" s="0" t="inlineStr">
+        <is>
+          <t>2026-04-07</t>
+        </is>
+      </c>
+      <c r="B46" s="0" t="n">
+        <v>45</v>
+      </c>
+      <c r="C46" s="0" t="inlineStr">
+        <is>
+          <t>Ishq Jalakar - Karvaan</t>
+        </is>
+      </c>
+      <c r="D46" s="0" t="inlineStr">
+        <is>
+          <t>Shashwat Sachdev</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" s="0" t="inlineStr">
+        <is>
+          <t>2026-04-07</t>
+        </is>
+      </c>
+      <c r="B47" s="0" t="n">
+        <v>46</v>
+      </c>
+      <c r="C47" s="0" t="inlineStr">
+        <is>
+          <t>Thodi Si Daaru</t>
+        </is>
+      </c>
+      <c r="D47" s="0" t="inlineStr">
+        <is>
+          <t>AP Dhillon</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" s="0" t="inlineStr">
+        <is>
+          <t>2026-04-07</t>
+        </is>
+      </c>
+      <c r="B48" s="0" t="n">
+        <v>47</v>
+      </c>
+      <c r="C48" s="0" t="inlineStr">
+        <is>
+          <t>Mast Magan</t>
+        </is>
+      </c>
+      <c r="D48" s="0" t="inlineStr">
+        <is>
+          <t>Arijit Singh</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" s="0" t="inlineStr">
+        <is>
+          <t>2026-04-07</t>
+        </is>
+      </c>
+      <c r="B49" s="0" t="n">
+        <v>48</v>
+      </c>
+      <c r="C49" s="0" t="inlineStr">
+        <is>
+          <t>Mutta Kalakki</t>
+        </is>
+      </c>
+      <c r="D49" s="0" t="inlineStr">
+        <is>
+          <t>G. V. Prakash</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" s="0" t="inlineStr">
+        <is>
+          <t>2026-04-07</t>
+        </is>
+      </c>
+      <c r="B50" s="0" t="n">
+        <v>49</v>
+      </c>
+      <c r="C50" s="0" t="inlineStr">
+        <is>
+          <t>Main Aur Tu</t>
+        </is>
+      </c>
+      <c r="D50" s="0" t="inlineStr">
+        <is>
+          <t>Shashwat Sachdev</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" s="0" t="inlineStr">
+        <is>
+          <t>2026-04-07</t>
+        </is>
+      </c>
+      <c r="B51" s="0" t="n">
+        <v>50</v>
+      </c>
+      <c r="C51" s="0" t="inlineStr">
+        <is>
+          <t>Aaya Sher</t>
+        </is>
+      </c>
+      <c r="D51" s="0" t="inlineStr">
+        <is>
+          <t>Anirudh Ravichander</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet27.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:D51"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="24" t="inlineStr">
+        <is>
+          <t>Date</t>
+        </is>
+      </c>
+      <c r="B1" s="24" t="inlineStr">
+        <is>
+          <t>Rank</t>
+        </is>
+      </c>
+      <c r="C1" s="24" t="inlineStr">
+        <is>
+          <t>Song</t>
+        </is>
+      </c>
+      <c r="D1" s="24" t="inlineStr">
+        <is>
+          <t>Artist</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>2026-04-06</t>
+          <t>2026-04-08</t>
         </is>
       </c>
       <c r="B2" t="n">
@@ -18129,7 +21240,7 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>2026-04-06</t>
+          <t>2026-04-08</t>
         </is>
       </c>
       <c r="B3" t="n">
@@ -18149,7 +21260,7 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>2026-04-06</t>
+          <t>2026-04-08</t>
         </is>
       </c>
       <c r="B4" t="n">
@@ -18169,7 +21280,7 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>2026-04-06</t>
+          <t>2026-04-08</t>
         </is>
       </c>
       <c r="B5" t="n">
@@ -18189,7 +21300,7 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>2026-04-06</t>
+          <t>2026-04-08</t>
         </is>
       </c>
       <c r="B6" t="n">
@@ -18209,7 +21320,7 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>2026-04-06</t>
+          <t>2026-04-08</t>
         </is>
       </c>
       <c r="B7" t="n">
@@ -18229,7 +21340,7 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>2026-04-06</t>
+          <t>2026-04-08</t>
         </is>
       </c>
       <c r="B8" t="n">
@@ -18249,7 +21360,7 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>2026-04-06</t>
+          <t>2026-04-08</t>
         </is>
       </c>
       <c r="B9" t="n">
@@ -18257,19 +21368,19 @@
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>Sahiba</t>
+          <t>Apna Bana Le</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>Aditya Rikhari</t>
+          <t>Sachin-Jigar</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>2026-04-06</t>
+          <t>2026-04-08</t>
         </is>
       </c>
       <c r="B10" t="n">
@@ -18277,19 +21388,19 @@
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>Jaan Se Guzarte Hain</t>
+          <t>Sahiba</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>Shashwat Sachdev</t>
+          <t>Aditya Rikhari</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>2026-04-06</t>
+          <t>2026-04-08</t>
         </is>
       </c>
       <c r="B11" t="n">
@@ -18309,7 +21420,7 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>2026-04-06</t>
+          <t>2026-04-08</t>
         </is>
       </c>
       <c r="B12" t="n">
@@ -18317,19 +21428,19 @@
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>Apna Bana Le</t>
+          <t>Samjhawan</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>Sachin-Jigar</t>
+          <t>Jawad Ahmad</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>2026-04-06</t>
+          <t>2026-04-08</t>
         </is>
       </c>
       <c r="B13" t="n">
@@ -18337,19 +21448,19 @@
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>Samjhawan</t>
+          <t>Jaan Se Guzarte Hain</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>Jawad Ahmad</t>
+          <t>Shashwat Sachdev</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>2026-04-06</t>
+          <t>2026-04-08</t>
         </is>
       </c>
       <c r="B14" t="n">
@@ -18357,19 +21468,19 @@
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>Pavazha Malli</t>
+          <t>Finding Her</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>Sai Abhyankkar</t>
+          <t>Kushagra</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>2026-04-06</t>
+          <t>2026-04-08</t>
         </is>
       </c>
       <c r="B15" t="n">
@@ -18377,19 +21488,19 @@
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>Finding Her</t>
+          <t>Boyfriend</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>Kushagra</t>
+          <t>Karan Aujla</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>2026-04-06</t>
+          <t>2026-04-08</t>
         </is>
       </c>
       <c r="B16" t="n">
@@ -18397,19 +21508,19 @@
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>Arz Kiya Hai | Coke Studio Bharat</t>
+          <t>Pavazha Malli</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>Anuv Jain</t>
+          <t>Sai Abhyankkar</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>2026-04-06</t>
+          <t>2026-04-08</t>
         </is>
       </c>
       <c r="B17" t="n">
@@ -18417,19 +21528,19 @@
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>Boyfriend</t>
+          <t>Arz Kiya Hai | Coke Studio Bharat</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>Karan Aujla</t>
+          <t>Anuv Jain</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>2026-04-06</t>
+          <t>2026-04-08</t>
         </is>
       </c>
       <c r="B18" t="n">
@@ -18437,19 +21548,19 @@
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>Ishq</t>
+          <t>Shararat</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>Faheem Abdullah</t>
+          <t>Shashwat Sachdev</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>2026-04-06</t>
+          <t>2026-04-08</t>
         </is>
       </c>
       <c r="B19" t="n">
@@ -18457,19 +21568,19 @@
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>Shararat</t>
+          <t>Ishq</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>Shashwat Sachdev</t>
+          <t>Faheem Abdullah</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>2026-04-06</t>
+          <t>2026-04-08</t>
         </is>
       </c>
       <c r="B20" t="n">
@@ -18489,7 +21600,7 @@
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>2026-04-06</t>
+          <t>2026-04-08</t>
         </is>
       </c>
       <c r="B21" t="n">
@@ -18497,19 +21608,19 @@
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>Dhurandhar - Title Track</t>
+          <t>Saiyaara</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>Shashwat Sachdev</t>
+          <t>Tanishk Bagchi</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>2026-04-06</t>
+          <t>2026-04-08</t>
         </is>
       </c>
       <c r="B22" t="n">
@@ -18517,19 +21628,19 @@
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>Saiyaara</t>
+          <t>Darkhaast</t>
         </is>
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>Tanishk Bagchi</t>
+          <t>Mithoon</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>2026-04-06</t>
+          <t>2026-04-08</t>
         </is>
       </c>
       <c r="B23" t="n">
@@ -18537,19 +21648,19 @@
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>For A Reason</t>
+          <t>Ishqa Ve</t>
         </is>
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>Karan Aujla</t>
+          <t>Zeeshan Ali</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>2026-04-06</t>
+          <t>2026-04-08</t>
         </is>
       </c>
       <c r="B24" t="n">
@@ -18557,19 +21668,19 @@
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>Bairi</t>
+          <t>Tum Ho Toh</t>
         </is>
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>Virat</t>
+          <t>Vishal Mishra</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>2026-04-06</t>
+          <t>2026-04-08</t>
         </is>
       </c>
       <c r="B25" t="n">
@@ -18577,7 +21688,7 @@
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>Phir Se</t>
+          <t>Dhurandhar - Title Track</t>
         </is>
       </c>
       <c r="D25" t="inlineStr">
@@ -18589,7 +21700,7 @@
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>2026-04-06</t>
+          <t>2026-04-08</t>
         </is>
       </c>
       <c r="B26" t="n">
@@ -18597,19 +21708,19 @@
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>Deewaana Deewaana</t>
+          <t>Naal Nachna</t>
         </is>
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>A.R. Rahman</t>
+          <t>Shashwat Sachdev</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>2026-04-06</t>
+          <t>2026-04-08</t>
         </is>
       </c>
       <c r="B27" t="n">
@@ -18617,19 +21728,19 @@
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>Raanjhan</t>
+          <t>For A Reason</t>
         </is>
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t>Sachet-Parampara</t>
+          <t>Karan Aujla</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>2026-04-06</t>
+          <t>2026-04-08</t>
         </is>
       </c>
       <c r="B28" t="n">
@@ -18637,19 +21748,19 @@
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>Tere Liye</t>
+          <t>Raanjhan</t>
         </is>
       </c>
       <c r="D28" t="inlineStr">
         <is>
-          <t>Atif Aslam</t>
+          <t>Sachet-Parampara</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>2026-04-06</t>
+          <t>2026-04-08</t>
         </is>
       </c>
       <c r="B29" t="n">
@@ -18657,19 +21768,19 @@
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>Naal Nachna</t>
+          <t>Deewaana Deewaana</t>
         </is>
       </c>
       <c r="D29" t="inlineStr">
         <is>
-          <t>Shashwat Sachdev</t>
+          <t>A.R. Rahman</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>2026-04-06</t>
+          <t>2026-04-08</t>
         </is>
       </c>
       <c r="B30" t="n">
@@ -18677,19 +21788,19 @@
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>Tum Ho Toh</t>
+          <t>Bairi</t>
         </is>
       </c>
       <c r="D30" t="inlineStr">
         <is>
-          <t>Vishal Mishra</t>
+          <t>Virat</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>2026-04-06</t>
+          <t>2026-04-08</t>
         </is>
       </c>
       <c r="B31" t="n">
@@ -18697,19 +21808,19 @@
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>Ishqa Ve</t>
+          <t>Jo Tum Mere Ho</t>
         </is>
       </c>
       <c r="D31" t="inlineStr">
         <is>
-          <t>Zeeshan Ali</t>
+          <t>Anuv Jain</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>2026-04-06</t>
+          <t>2026-04-08</t>
         </is>
       </c>
       <c r="B32" t="n">
@@ -18717,19 +21828,19 @@
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>Darkhaast</t>
+          <t>Tere Liye</t>
         </is>
       </c>
       <c r="D32" t="inlineStr">
         <is>
-          <t>Mithoon</t>
+          <t>Atif Aslam</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>2026-04-06</t>
+          <t>2026-04-08</t>
         </is>
       </c>
       <c r="B33" t="n">
@@ -18737,7 +21848,7 @@
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>Run Down The City - Monica</t>
+          <t>Phir Se</t>
         </is>
       </c>
       <c r="D33" t="inlineStr">
@@ -18749,7 +21860,7 @@
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>2026-04-06</t>
+          <t>2026-04-08</t>
         </is>
       </c>
       <c r="B34" t="n">
@@ -18757,19 +21868,19 @@
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>Lutt Le Gaya</t>
+          <t>Agar Tum Saath Ho</t>
         </is>
       </c>
       <c r="D34" t="inlineStr">
         <is>
-          <t>Shashwat Sachdev</t>
+          <t>Alka Yagnik</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>2026-04-06</t>
+          <t>2026-04-08</t>
         </is>
       </c>
       <c r="B35" t="n">
@@ -18777,19 +21888,19 @@
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>Jo Tum Mere Ho</t>
+          <t>Tere Bina</t>
         </is>
       </c>
       <c r="D35" t="inlineStr">
         <is>
-          <t>Anuv Jain</t>
+          <t>A.R. Rahman</t>
         </is>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>2026-04-06</t>
+          <t>2026-04-08</t>
         </is>
       </c>
       <c r="B36" t="n">
@@ -18797,19 +21908,19 @@
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>Haseen</t>
+          <t>Run Down The City - Monica</t>
         </is>
       </c>
       <c r="D36" t="inlineStr">
         <is>
-          <t>Talwiinder</t>
+          <t>Shashwat Sachdev</t>
         </is>
       </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>2026-04-06</t>
+          <t>2026-04-08</t>
         </is>
       </c>
       <c r="B37" t="n">
@@ -18817,19 +21928,19 @@
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>Barbaad</t>
+          <t>Haseen</t>
         </is>
       </c>
       <c r="D37" t="inlineStr">
         <is>
-          <t>The Rish</t>
+          <t>Talwiinder</t>
         </is>
       </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>2026-04-06</t>
+          <t>2026-04-08</t>
         </is>
       </c>
       <c r="B38" t="n">
@@ -18837,19 +21948,19 @@
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>Agar Tum Saath Ho</t>
+          <t>Barbaad</t>
         </is>
       </c>
       <c r="D38" t="inlineStr">
         <is>
-          <t>Alka Yagnik</t>
+          <t>The Rish</t>
         </is>
       </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>2026-04-06</t>
+          <t>2026-04-08</t>
         </is>
       </c>
       <c r="B39" t="n">
@@ -18857,19 +21968,19 @@
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>Tere Bina</t>
+          <t>Lutt Le Gaya</t>
         </is>
       </c>
       <c r="D39" t="inlineStr">
         <is>
-          <t>A.R. Rahman</t>
+          <t>Shashwat Sachdev</t>
         </is>
       </c>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>2026-04-06</t>
+          <t>2026-04-08</t>
         </is>
       </c>
       <c r="B40" t="n">
@@ -18889,7 +22000,7 @@
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>2026-04-06</t>
+          <t>2026-04-08</t>
         </is>
       </c>
       <c r="B41" t="n">
@@ -18897,19 +22008,19 @@
       </c>
       <c r="C41" t="inlineStr">
         <is>
-          <t>Not Guilty</t>
+          <t>Jogi</t>
         </is>
       </c>
       <c r="D41" t="inlineStr">
         <is>
-          <t>Dhanda Nyoliwala</t>
+          <t>thiarajxtt</t>
         </is>
       </c>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>2026-04-06</t>
+          <t>2026-04-08</t>
         </is>
       </c>
       <c r="B42" t="n">
@@ -18929,7 +22040,7 @@
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>2026-04-06</t>
+          <t>2026-04-08</t>
         </is>
       </c>
       <c r="B43" t="n">
@@ -18949,7 +22060,7 @@
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>2026-04-06</t>
+          <t>2026-04-08</t>
         </is>
       </c>
       <c r="B44" t="n">
@@ -18957,19 +22068,19 @@
       </c>
       <c r="C44" t="inlineStr">
         <is>
-          <t>Main Aur Tu</t>
+          <t>Ehsaas</t>
         </is>
       </c>
       <c r="D44" t="inlineStr">
         <is>
-          <t>Shashwat Sachdev</t>
+          <t>Faheem Abdullah</t>
         </is>
       </c>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>2026-04-06</t>
+          <t>2026-04-08</t>
         </is>
       </c>
       <c r="B45" t="n">
@@ -18977,19 +22088,19 @@
       </c>
       <c r="C45" t="inlineStr">
         <is>
-          <t>Ehsaas</t>
+          <t>Dhun</t>
         </is>
       </c>
       <c r="D45" t="inlineStr">
         <is>
-          <t>Faheem Abdullah</t>
+          <t>Mithoon</t>
         </is>
       </c>
     </row>
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>2026-04-06</t>
+          <t>2026-04-08</t>
         </is>
       </c>
       <c r="B46" t="n">
@@ -18997,19 +22108,19 @@
       </c>
       <c r="C46" t="inlineStr">
         <is>
-          <t>Aaya Sher</t>
+          <t>Zaalima</t>
         </is>
       </c>
       <c r="D46" t="inlineStr">
         <is>
-          <t>Anirudh Ravichander</t>
+          <t>Arijit Singh</t>
         </is>
       </c>
     </row>
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>2026-04-06</t>
+          <t>2026-04-08</t>
         </is>
       </c>
       <c r="B47" t="n">
@@ -19017,19 +22128,19 @@
       </c>
       <c r="C47" t="inlineStr">
         <is>
-          <t>Mutta Kalakki</t>
+          <t>Thodi Si Daaru</t>
         </is>
       </c>
       <c r="D47" t="inlineStr">
         <is>
-          <t>G. V. Prakash</t>
+          <t>AP Dhillon</t>
         </is>
       </c>
     </row>
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>2026-04-06</t>
+          <t>2026-04-08</t>
         </is>
       </c>
       <c r="B48" t="n">
@@ -19037,7 +22148,7 @@
       </c>
       <c r="C48" t="inlineStr">
         <is>
-          <t>Ishq Jalakar - Karvaan</t>
+          <t>Main Aur Tu</t>
         </is>
       </c>
       <c r="D48" t="inlineStr">
@@ -19049,7 +22160,7 @@
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>2026-04-06</t>
+          <t>2026-04-08</t>
         </is>
       </c>
       <c r="B49" t="n">
@@ -19057,19 +22168,19 @@
       </c>
       <c r="C49" t="inlineStr">
         <is>
-          <t>Jogi</t>
+          <t>Ishq Jalakar - Karvaan</t>
         </is>
       </c>
       <c r="D49" t="inlineStr">
         <is>
-          <t>thiarajxtt</t>
+          <t>Shashwat Sachdev</t>
         </is>
       </c>
     </row>
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>2026-04-06</t>
+          <t>2026-04-08</t>
         </is>
       </c>
       <c r="B50" t="n">
@@ -19089,7 +22200,7 @@
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>2026-04-06</t>
+          <t>2026-04-08</t>
         </is>
       </c>
       <c r="B51" t="n">
@@ -19097,12 +22208,12 @@
       </c>
       <c r="C51" t="inlineStr">
         <is>
-          <t>Dhun</t>
+          <t>Aaya Sher</t>
         </is>
       </c>
       <c r="D51" t="inlineStr">
         <is>
-          <t>Mithoon</t>
+          <t>Anirudh Ravichander</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
added data till 10th april, got predictions for 11th april
</commit_message>
<xml_diff>
--- a/Probability Project.xlsx
+++ b/Probability Project.xlsx
@@ -30,6 +30,7 @@
     <sheet name="AUTO_20260409" sheetId="25" state="visible" r:id="rId25"/>
     <sheet name="AUTO_20260407" sheetId="26" state="visible" r:id="rId26"/>
     <sheet name="AUTO_20260408" sheetId="27" state="visible" r:id="rId27"/>
+    <sheet name="AUTO_20260410" sheetId="28" state="visible" r:id="rId28"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -21218,9 +21219,1045 @@
       </c>
     </row>
     <row r="2">
+      <c r="A2" s="0" t="inlineStr">
+        <is>
+          <t>2026-04-08</t>
+        </is>
+      </c>
+      <c r="B2" s="0" t="n">
+        <v>1</v>
+      </c>
+      <c r="C2" s="0" t="inlineStr">
+        <is>
+          <t>Bairan</t>
+        </is>
+      </c>
+      <c r="D2" s="0" t="inlineStr">
+        <is>
+          <t>Banjaare</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="0" t="inlineStr">
+        <is>
+          <t>2026-04-08</t>
+        </is>
+      </c>
+      <c r="B3" s="0" t="n">
+        <v>2</v>
+      </c>
+      <c r="C3" s="0" t="inlineStr">
+        <is>
+          <t>Jaiye Sajana</t>
+        </is>
+      </c>
+      <c r="D3" s="0" t="inlineStr">
+        <is>
+          <t>Shashwat Sachdev</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="0" t="inlineStr">
+        <is>
+          <t>2026-04-08</t>
+        </is>
+      </c>
+      <c r="B4" s="0" t="n">
+        <v>3</v>
+      </c>
+      <c r="C4" s="0" t="inlineStr">
+        <is>
+          <t>Gehra Hua</t>
+        </is>
+      </c>
+      <c r="D4" s="0" t="inlineStr">
+        <is>
+          <t>Shashwat Sachdev</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="0" t="inlineStr">
+        <is>
+          <t>2026-04-08</t>
+        </is>
+      </c>
+      <c r="B5" s="0" t="n">
+        <v>4</v>
+      </c>
+      <c r="C5" s="0" t="inlineStr">
+        <is>
+          <t>Sheesha - Aakhya Mai Aakh Ghali Jo Bairan</t>
+        </is>
+      </c>
+      <c r="D5" s="0" t="inlineStr">
+        <is>
+          <t>Mitta Ror</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="0" t="inlineStr">
+        <is>
+          <t>2026-04-08</t>
+        </is>
+      </c>
+      <c r="B6" s="0" t="n">
+        <v>5</v>
+      </c>
+      <c r="C6" s="0" t="inlineStr">
+        <is>
+          <t>Khat</t>
+        </is>
+      </c>
+      <c r="D6" s="0" t="inlineStr">
+        <is>
+          <t>Navjot Ahuja</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="0" t="inlineStr">
+        <is>
+          <t>2026-04-08</t>
+        </is>
+      </c>
+      <c r="B7" s="0" t="n">
+        <v>6</v>
+      </c>
+      <c r="C7" s="0" t="inlineStr">
+        <is>
+          <t>Dhurandhar The Revenge - Aari Aari</t>
+        </is>
+      </c>
+      <c r="D7" s="0" t="inlineStr">
+        <is>
+          <t>Shashwat Sachdev</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="0" t="inlineStr">
+        <is>
+          <t>2026-04-08</t>
+        </is>
+      </c>
+      <c r="B8" s="0" t="n">
+        <v>7</v>
+      </c>
+      <c r="C8" s="0" t="inlineStr">
+        <is>
+          <t>Dooron Dooron</t>
+        </is>
+      </c>
+      <c r="D8" s="0" t="inlineStr">
+        <is>
+          <t>Paresh Pahuja</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="0" t="inlineStr">
+        <is>
+          <t>2026-04-08</t>
+        </is>
+      </c>
+      <c r="B9" s="0" t="n">
+        <v>8</v>
+      </c>
+      <c r="C9" s="0" t="inlineStr">
+        <is>
+          <t>Apna Bana Le</t>
+        </is>
+      </c>
+      <c r="D9" s="0" t="inlineStr">
+        <is>
+          <t>Sachin-Jigar</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="0" t="inlineStr">
+        <is>
+          <t>2026-04-08</t>
+        </is>
+      </c>
+      <c r="B10" s="0" t="n">
+        <v>9</v>
+      </c>
+      <c r="C10" s="0" t="inlineStr">
+        <is>
+          <t>Sahiba</t>
+        </is>
+      </c>
+      <c r="D10" s="0" t="inlineStr">
+        <is>
+          <t>Aditya Rikhari</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="0" t="inlineStr">
+        <is>
+          <t>2026-04-08</t>
+        </is>
+      </c>
+      <c r="B11" s="0" t="n">
+        <v>10</v>
+      </c>
+      <c r="C11" s="0" t="inlineStr">
+        <is>
+          <t>Sitaare</t>
+        </is>
+      </c>
+      <c r="D11" s="0" t="inlineStr">
+        <is>
+          <t>Arijit Singh</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="0" t="inlineStr">
+        <is>
+          <t>2026-04-08</t>
+        </is>
+      </c>
+      <c r="B12" s="0" t="n">
+        <v>11</v>
+      </c>
+      <c r="C12" s="0" t="inlineStr">
+        <is>
+          <t>Samjhawan</t>
+        </is>
+      </c>
+      <c r="D12" s="0" t="inlineStr">
+        <is>
+          <t>Jawad Ahmad</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="0" t="inlineStr">
+        <is>
+          <t>2026-04-08</t>
+        </is>
+      </c>
+      <c r="B13" s="0" t="n">
+        <v>12</v>
+      </c>
+      <c r="C13" s="0" t="inlineStr">
+        <is>
+          <t>Jaan Se Guzarte Hain</t>
+        </is>
+      </c>
+      <c r="D13" s="0" t="inlineStr">
+        <is>
+          <t>Shashwat Sachdev</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="0" t="inlineStr">
+        <is>
+          <t>2026-04-08</t>
+        </is>
+      </c>
+      <c r="B14" s="0" t="n">
+        <v>13</v>
+      </c>
+      <c r="C14" s="0" t="inlineStr">
+        <is>
+          <t>Finding Her</t>
+        </is>
+      </c>
+      <c r="D14" s="0" t="inlineStr">
+        <is>
+          <t>Kushagra</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="0" t="inlineStr">
+        <is>
+          <t>2026-04-08</t>
+        </is>
+      </c>
+      <c r="B15" s="0" t="n">
+        <v>14</v>
+      </c>
+      <c r="C15" s="0" t="inlineStr">
+        <is>
+          <t>Boyfriend</t>
+        </is>
+      </c>
+      <c r="D15" s="0" t="inlineStr">
+        <is>
+          <t>Karan Aujla</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="0" t="inlineStr">
+        <is>
+          <t>2026-04-08</t>
+        </is>
+      </c>
+      <c r="B16" s="0" t="n">
+        <v>15</v>
+      </c>
+      <c r="C16" s="0" t="inlineStr">
+        <is>
+          <t>Pavazha Malli</t>
+        </is>
+      </c>
+      <c r="D16" s="0" t="inlineStr">
+        <is>
+          <t>Sai Abhyankkar</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="0" t="inlineStr">
+        <is>
+          <t>2026-04-08</t>
+        </is>
+      </c>
+      <c r="B17" s="0" t="n">
+        <v>16</v>
+      </c>
+      <c r="C17" s="0" t="inlineStr">
+        <is>
+          <t>Arz Kiya Hai | Coke Studio Bharat</t>
+        </is>
+      </c>
+      <c r="D17" s="0" t="inlineStr">
+        <is>
+          <t>Anuv Jain</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="0" t="inlineStr">
+        <is>
+          <t>2026-04-08</t>
+        </is>
+      </c>
+      <c r="B18" s="0" t="n">
+        <v>17</v>
+      </c>
+      <c r="C18" s="0" t="inlineStr">
+        <is>
+          <t>Shararat</t>
+        </is>
+      </c>
+      <c r="D18" s="0" t="inlineStr">
+        <is>
+          <t>Shashwat Sachdev</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="0" t="inlineStr">
+        <is>
+          <t>2026-04-08</t>
+        </is>
+      </c>
+      <c r="B19" s="0" t="n">
+        <v>18</v>
+      </c>
+      <c r="C19" s="0" t="inlineStr">
+        <is>
+          <t>Ishq</t>
+        </is>
+      </c>
+      <c r="D19" s="0" t="inlineStr">
+        <is>
+          <t>Faheem Abdullah</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="0" t="inlineStr">
+        <is>
+          <t>2026-04-08</t>
+        </is>
+      </c>
+      <c r="B20" s="0" t="n">
+        <v>19</v>
+      </c>
+      <c r="C20" s="0" t="inlineStr">
+        <is>
+          <t>Mann Mera</t>
+        </is>
+      </c>
+      <c r="D20" s="0" t="inlineStr">
+        <is>
+          <t>Gajendra Verma</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="0" t="inlineStr">
+        <is>
+          <t>2026-04-08</t>
+        </is>
+      </c>
+      <c r="B21" s="0" t="n">
+        <v>20</v>
+      </c>
+      <c r="C21" s="0" t="inlineStr">
+        <is>
+          <t>Saiyaara</t>
+        </is>
+      </c>
+      <c r="D21" s="0" t="inlineStr">
+        <is>
+          <t>Tanishk Bagchi</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="0" t="inlineStr">
+        <is>
+          <t>2026-04-08</t>
+        </is>
+      </c>
+      <c r="B22" s="0" t="n">
+        <v>21</v>
+      </c>
+      <c r="C22" s="0" t="inlineStr">
+        <is>
+          <t>Darkhaast</t>
+        </is>
+      </c>
+      <c r="D22" s="0" t="inlineStr">
+        <is>
+          <t>Mithoon</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="0" t="inlineStr">
+        <is>
+          <t>2026-04-08</t>
+        </is>
+      </c>
+      <c r="B23" s="0" t="n">
+        <v>22</v>
+      </c>
+      <c r="C23" s="0" t="inlineStr">
+        <is>
+          <t>Ishqa Ve</t>
+        </is>
+      </c>
+      <c r="D23" s="0" t="inlineStr">
+        <is>
+          <t>Zeeshan Ali</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="0" t="inlineStr">
+        <is>
+          <t>2026-04-08</t>
+        </is>
+      </c>
+      <c r="B24" s="0" t="n">
+        <v>23</v>
+      </c>
+      <c r="C24" s="0" t="inlineStr">
+        <is>
+          <t>Tum Ho Toh</t>
+        </is>
+      </c>
+      <c r="D24" s="0" t="inlineStr">
+        <is>
+          <t>Vishal Mishra</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="0" t="inlineStr">
+        <is>
+          <t>2026-04-08</t>
+        </is>
+      </c>
+      <c r="B25" s="0" t="n">
+        <v>24</v>
+      </c>
+      <c r="C25" s="0" t="inlineStr">
+        <is>
+          <t>Dhurandhar - Title Track</t>
+        </is>
+      </c>
+      <c r="D25" s="0" t="inlineStr">
+        <is>
+          <t>Shashwat Sachdev</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="0" t="inlineStr">
+        <is>
+          <t>2026-04-08</t>
+        </is>
+      </c>
+      <c r="B26" s="0" t="n">
+        <v>25</v>
+      </c>
+      <c r="C26" s="0" t="inlineStr">
+        <is>
+          <t>Naal Nachna</t>
+        </is>
+      </c>
+      <c r="D26" s="0" t="inlineStr">
+        <is>
+          <t>Shashwat Sachdev</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="0" t="inlineStr">
+        <is>
+          <t>2026-04-08</t>
+        </is>
+      </c>
+      <c r="B27" s="0" t="n">
+        <v>26</v>
+      </c>
+      <c r="C27" s="0" t="inlineStr">
+        <is>
+          <t>For A Reason</t>
+        </is>
+      </c>
+      <c r="D27" s="0" t="inlineStr">
+        <is>
+          <t>Karan Aujla</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="0" t="inlineStr">
+        <is>
+          <t>2026-04-08</t>
+        </is>
+      </c>
+      <c r="B28" s="0" t="n">
+        <v>27</v>
+      </c>
+      <c r="C28" s="0" t="inlineStr">
+        <is>
+          <t>Raanjhan</t>
+        </is>
+      </c>
+      <c r="D28" s="0" t="inlineStr">
+        <is>
+          <t>Sachet-Parampara</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="0" t="inlineStr">
+        <is>
+          <t>2026-04-08</t>
+        </is>
+      </c>
+      <c r="B29" s="0" t="n">
+        <v>28</v>
+      </c>
+      <c r="C29" s="0" t="inlineStr">
+        <is>
+          <t>Deewaana Deewaana</t>
+        </is>
+      </c>
+      <c r="D29" s="0" t="inlineStr">
+        <is>
+          <t>A.R. Rahman</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="0" t="inlineStr">
+        <is>
+          <t>2026-04-08</t>
+        </is>
+      </c>
+      <c r="B30" s="0" t="n">
+        <v>29</v>
+      </c>
+      <c r="C30" s="0" t="inlineStr">
+        <is>
+          <t>Bairi</t>
+        </is>
+      </c>
+      <c r="D30" s="0" t="inlineStr">
+        <is>
+          <t>Virat</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="0" t="inlineStr">
+        <is>
+          <t>2026-04-08</t>
+        </is>
+      </c>
+      <c r="B31" s="0" t="n">
+        <v>30</v>
+      </c>
+      <c r="C31" s="0" t="inlineStr">
+        <is>
+          <t>Jo Tum Mere Ho</t>
+        </is>
+      </c>
+      <c r="D31" s="0" t="inlineStr">
+        <is>
+          <t>Anuv Jain</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="0" t="inlineStr">
+        <is>
+          <t>2026-04-08</t>
+        </is>
+      </c>
+      <c r="B32" s="0" t="n">
+        <v>31</v>
+      </c>
+      <c r="C32" s="0" t="inlineStr">
+        <is>
+          <t>Tere Liye</t>
+        </is>
+      </c>
+      <c r="D32" s="0" t="inlineStr">
+        <is>
+          <t>Atif Aslam</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="0" t="inlineStr">
+        <is>
+          <t>2026-04-08</t>
+        </is>
+      </c>
+      <c r="B33" s="0" t="n">
+        <v>32</v>
+      </c>
+      <c r="C33" s="0" t="inlineStr">
+        <is>
+          <t>Phir Se</t>
+        </is>
+      </c>
+      <c r="D33" s="0" t="inlineStr">
+        <is>
+          <t>Shashwat Sachdev</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="0" t="inlineStr">
+        <is>
+          <t>2026-04-08</t>
+        </is>
+      </c>
+      <c r="B34" s="0" t="n">
+        <v>33</v>
+      </c>
+      <c r="C34" s="0" t="inlineStr">
+        <is>
+          <t>Agar Tum Saath Ho</t>
+        </is>
+      </c>
+      <c r="D34" s="0" t="inlineStr">
+        <is>
+          <t>Alka Yagnik</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="0" t="inlineStr">
+        <is>
+          <t>2026-04-08</t>
+        </is>
+      </c>
+      <c r="B35" s="0" t="n">
+        <v>34</v>
+      </c>
+      <c r="C35" s="0" t="inlineStr">
+        <is>
+          <t>Tere Bina</t>
+        </is>
+      </c>
+      <c r="D35" s="0" t="inlineStr">
+        <is>
+          <t>A.R. Rahman</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="0" t="inlineStr">
+        <is>
+          <t>2026-04-08</t>
+        </is>
+      </c>
+      <c r="B36" s="0" t="n">
+        <v>35</v>
+      </c>
+      <c r="C36" s="0" t="inlineStr">
+        <is>
+          <t>Run Down The City - Monica</t>
+        </is>
+      </c>
+      <c r="D36" s="0" t="inlineStr">
+        <is>
+          <t>Shashwat Sachdev</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="0" t="inlineStr">
+        <is>
+          <t>2026-04-08</t>
+        </is>
+      </c>
+      <c r="B37" s="0" t="n">
+        <v>36</v>
+      </c>
+      <c r="C37" s="0" t="inlineStr">
+        <is>
+          <t>Haseen</t>
+        </is>
+      </c>
+      <c r="D37" s="0" t="inlineStr">
+        <is>
+          <t>Talwiinder</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="0" t="inlineStr">
+        <is>
+          <t>2026-04-08</t>
+        </is>
+      </c>
+      <c r="B38" s="0" t="n">
+        <v>37</v>
+      </c>
+      <c r="C38" s="0" t="inlineStr">
+        <is>
+          <t>Barbaad</t>
+        </is>
+      </c>
+      <c r="D38" s="0" t="inlineStr">
+        <is>
+          <t>The Rish</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="0" t="inlineStr">
+        <is>
+          <t>2026-04-08</t>
+        </is>
+      </c>
+      <c r="B39" s="0" t="n">
+        <v>38</v>
+      </c>
+      <c r="C39" s="0" t="inlineStr">
+        <is>
+          <t>Lutt Le Gaya</t>
+        </is>
+      </c>
+      <c r="D39" s="0" t="inlineStr">
+        <is>
+          <t>Shashwat Sachdev</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="0" t="inlineStr">
+        <is>
+          <t>2026-04-08</t>
+        </is>
+      </c>
+      <c r="B40" s="0" t="n">
+        <v>39</v>
+      </c>
+      <c r="C40" s="0" t="inlineStr">
+        <is>
+          <t>Teri Deewani</t>
+        </is>
+      </c>
+      <c r="D40" s="0" t="inlineStr">
+        <is>
+          <t>Kailash Kher</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" s="0" t="inlineStr">
+        <is>
+          <t>2026-04-08</t>
+        </is>
+      </c>
+      <c r="B41" s="0" t="n">
+        <v>40</v>
+      </c>
+      <c r="C41" s="0" t="inlineStr">
+        <is>
+          <t>Jogi</t>
+        </is>
+      </c>
+      <c r="D41" s="0" t="inlineStr">
+        <is>
+          <t>thiarajxtt</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" s="0" t="inlineStr">
+        <is>
+          <t>2026-04-08</t>
+        </is>
+      </c>
+      <c r="B42" s="0" t="n">
+        <v>41</v>
+      </c>
+      <c r="C42" s="0" t="inlineStr">
+        <is>
+          <t>Ye Tune Kya Kiya</t>
+        </is>
+      </c>
+      <c r="D42" s="0" t="inlineStr">
+        <is>
+          <t>Pritam</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" s="0" t="inlineStr">
+        <is>
+          <t>2026-04-08</t>
+        </is>
+      </c>
+      <c r="B43" s="0" t="n">
+        <v>42</v>
+      </c>
+      <c r="C43" s="0" t="inlineStr">
+        <is>
+          <t>Mann Mera - Original Version</t>
+        </is>
+      </c>
+      <c r="D43" s="0" t="inlineStr">
+        <is>
+          <t>Gajendra Verma</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" s="0" t="inlineStr">
+        <is>
+          <t>2026-04-08</t>
+        </is>
+      </c>
+      <c r="B44" s="0" t="n">
+        <v>43</v>
+      </c>
+      <c r="C44" s="0" t="inlineStr">
+        <is>
+          <t>Ehsaas</t>
+        </is>
+      </c>
+      <c r="D44" s="0" t="inlineStr">
+        <is>
+          <t>Faheem Abdullah</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" s="0" t="inlineStr">
+        <is>
+          <t>2026-04-08</t>
+        </is>
+      </c>
+      <c r="B45" s="0" t="n">
+        <v>44</v>
+      </c>
+      <c r="C45" s="0" t="inlineStr">
+        <is>
+          <t>Dhun</t>
+        </is>
+      </c>
+      <c r="D45" s="0" t="inlineStr">
+        <is>
+          <t>Mithoon</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" s="0" t="inlineStr">
+        <is>
+          <t>2026-04-08</t>
+        </is>
+      </c>
+      <c r="B46" s="0" t="n">
+        <v>45</v>
+      </c>
+      <c r="C46" s="0" t="inlineStr">
+        <is>
+          <t>Zaalima</t>
+        </is>
+      </c>
+      <c r="D46" s="0" t="inlineStr">
+        <is>
+          <t>Arijit Singh</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" s="0" t="inlineStr">
+        <is>
+          <t>2026-04-08</t>
+        </is>
+      </c>
+      <c r="B47" s="0" t="n">
+        <v>46</v>
+      </c>
+      <c r="C47" s="0" t="inlineStr">
+        <is>
+          <t>Thodi Si Daaru</t>
+        </is>
+      </c>
+      <c r="D47" s="0" t="inlineStr">
+        <is>
+          <t>AP Dhillon</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" s="0" t="inlineStr">
+        <is>
+          <t>2026-04-08</t>
+        </is>
+      </c>
+      <c r="B48" s="0" t="n">
+        <v>47</v>
+      </c>
+      <c r="C48" s="0" t="inlineStr">
+        <is>
+          <t>Main Aur Tu</t>
+        </is>
+      </c>
+      <c r="D48" s="0" t="inlineStr">
+        <is>
+          <t>Shashwat Sachdev</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" s="0" t="inlineStr">
+        <is>
+          <t>2026-04-08</t>
+        </is>
+      </c>
+      <c r="B49" s="0" t="n">
+        <v>48</v>
+      </c>
+      <c r="C49" s="0" t="inlineStr">
+        <is>
+          <t>Ishq Jalakar - Karvaan</t>
+        </is>
+      </c>
+      <c r="D49" s="0" t="inlineStr">
+        <is>
+          <t>Shashwat Sachdev</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" s="0" t="inlineStr">
+        <is>
+          <t>2026-04-08</t>
+        </is>
+      </c>
+      <c r="B50" s="0" t="n">
+        <v>49</v>
+      </c>
+      <c r="C50" s="0" t="inlineStr">
+        <is>
+          <t>Mast Magan</t>
+        </is>
+      </c>
+      <c r="D50" s="0" t="inlineStr">
+        <is>
+          <t>Arijit Singh</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" s="0" t="inlineStr">
+        <is>
+          <t>2026-04-08</t>
+        </is>
+      </c>
+      <c r="B51" s="0" t="n">
+        <v>50</v>
+      </c>
+      <c r="C51" s="0" t="inlineStr">
+        <is>
+          <t>Aaya Sher</t>
+        </is>
+      </c>
+      <c r="D51" s="0" t="inlineStr">
+        <is>
+          <t>Anirudh Ravichander</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet28.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:D51"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="24" t="inlineStr">
+        <is>
+          <t>Date</t>
+        </is>
+      </c>
+      <c r="B1" s="24" t="inlineStr">
+        <is>
+          <t>Rank</t>
+        </is>
+      </c>
+      <c r="C1" s="24" t="inlineStr">
+        <is>
+          <t>Song</t>
+        </is>
+      </c>
+      <c r="D1" s="24" t="inlineStr">
+        <is>
+          <t>Artist</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>2026-04-08</t>
+          <t>2026-04-10</t>
         </is>
       </c>
       <c r="B2" t="n">
@@ -21240,7 +22277,7 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>2026-04-08</t>
+          <t>2026-04-10</t>
         </is>
       </c>
       <c r="B3" t="n">
@@ -21260,7 +22297,7 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>2026-04-08</t>
+          <t>2026-04-10</t>
         </is>
       </c>
       <c r="B4" t="n">
@@ -21280,7 +22317,7 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>2026-04-08</t>
+          <t>2026-04-10</t>
         </is>
       </c>
       <c r="B5" t="n">
@@ -21300,7 +22337,7 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>2026-04-08</t>
+          <t>2026-04-10</t>
         </is>
       </c>
       <c r="B6" t="n">
@@ -21320,7 +22357,7 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>2026-04-08</t>
+          <t>2026-04-10</t>
         </is>
       </c>
       <c r="B7" t="n">
@@ -21340,7 +22377,7 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>2026-04-08</t>
+          <t>2026-04-10</t>
         </is>
       </c>
       <c r="B8" t="n">
@@ -21360,7 +22397,7 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>2026-04-08</t>
+          <t>2026-04-10</t>
         </is>
       </c>
       <c r="B9" t="n">
@@ -21380,7 +22417,7 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>2026-04-08</t>
+          <t>2026-04-10</t>
         </is>
       </c>
       <c r="B10" t="n">
@@ -21388,19 +22425,19 @@
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>Sahiba</t>
+          <t>Sitaare</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>Aditya Rikhari</t>
+          <t>Arijit Singh</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>2026-04-08</t>
+          <t>2026-04-10</t>
         </is>
       </c>
       <c r="B11" t="n">
@@ -21408,19 +22445,19 @@
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>Sitaare</t>
+          <t>Sahiba</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>Arijit Singh</t>
+          <t>Aditya Rikhari</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>2026-04-08</t>
+          <t>2026-04-10</t>
         </is>
       </c>
       <c r="B12" t="n">
@@ -21428,19 +22465,19 @@
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>Samjhawan</t>
+          <t>Jaan Se Guzarte Hain</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>Jawad Ahmad</t>
+          <t>Shashwat Sachdev</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>2026-04-08</t>
+          <t>2026-04-10</t>
         </is>
       </c>
       <c r="B13" t="n">
@@ -21448,19 +22485,19 @@
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>Jaan Se Guzarte Hain</t>
+          <t>Samjhawan</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>Shashwat Sachdev</t>
+          <t>Jawad Ahmad</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>2026-04-08</t>
+          <t>2026-04-10</t>
         </is>
       </c>
       <c r="B14" t="n">
@@ -21468,19 +22505,19 @@
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>Finding Her</t>
+          <t>Pavazha Malli</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>Kushagra</t>
+          <t>Sai Abhyankkar</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>2026-04-08</t>
+          <t>2026-04-10</t>
         </is>
       </c>
       <c r="B15" t="n">
@@ -21488,19 +22525,19 @@
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>Boyfriend</t>
+          <t>Finding Her</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>Karan Aujla</t>
+          <t>Kushagra</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>2026-04-08</t>
+          <t>2026-04-10</t>
         </is>
       </c>
       <c r="B16" t="n">
@@ -21508,19 +22545,19 @@
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>Pavazha Malli</t>
+          <t>Boyfriend</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>Sai Abhyankkar</t>
+          <t>Karan Aujla</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>2026-04-08</t>
+          <t>2026-04-10</t>
         </is>
       </c>
       <c r="B17" t="n">
@@ -21540,7 +22577,7 @@
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>2026-04-08</t>
+          <t>2026-04-10</t>
         </is>
       </c>
       <c r="B18" t="n">
@@ -21560,7 +22597,7 @@
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>2026-04-08</t>
+          <t>2026-04-10</t>
         </is>
       </c>
       <c r="B19" t="n">
@@ -21568,19 +22605,19 @@
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>Ishq</t>
+          <t>Mann Mera</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>Faheem Abdullah</t>
+          <t>Gajendra Verma</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>2026-04-08</t>
+          <t>2026-04-10</t>
         </is>
       </c>
       <c r="B20" t="n">
@@ -21588,19 +22625,19 @@
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>Mann Mera</t>
+          <t>Ishq</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>Gajendra Verma</t>
+          <t>Faheem Abdullah</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>2026-04-08</t>
+          <t>2026-04-10</t>
         </is>
       </c>
       <c r="B21" t="n">
@@ -21608,19 +22645,19 @@
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>Saiyaara</t>
+          <t>For A Reason</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>Tanishk Bagchi</t>
+          <t>Karan Aujla</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>2026-04-08</t>
+          <t>2026-04-10</t>
         </is>
       </c>
       <c r="B22" t="n">
@@ -21628,19 +22665,19 @@
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>Darkhaast</t>
+          <t>Saiyaara</t>
         </is>
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>Mithoon</t>
+          <t>Tanishk Bagchi</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>2026-04-08</t>
+          <t>2026-04-10</t>
         </is>
       </c>
       <c r="B23" t="n">
@@ -21660,7 +22697,7 @@
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>2026-04-08</t>
+          <t>2026-04-10</t>
         </is>
       </c>
       <c r="B24" t="n">
@@ -21668,19 +22705,19 @@
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>Tum Ho Toh</t>
+          <t>Naal Nachna</t>
         </is>
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>Vishal Mishra</t>
+          <t>Shashwat Sachdev</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>2026-04-08</t>
+          <t>2026-04-10</t>
         </is>
       </c>
       <c r="B25" t="n">
@@ -21688,19 +22725,19 @@
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>Dhurandhar - Title Track</t>
+          <t>Bairi</t>
         </is>
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>Shashwat Sachdev</t>
+          <t>Virat</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>2026-04-08</t>
+          <t>2026-04-10</t>
         </is>
       </c>
       <c r="B26" t="n">
@@ -21708,7 +22745,7 @@
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>Naal Nachna</t>
+          <t>Dhurandhar - Title Track</t>
         </is>
       </c>
       <c r="D26" t="inlineStr">
@@ -21720,7 +22757,7 @@
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>2026-04-08</t>
+          <t>2026-04-10</t>
         </is>
       </c>
       <c r="B27" t="n">
@@ -21728,19 +22765,19 @@
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>For A Reason</t>
+          <t>Tere Liye</t>
         </is>
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t>Karan Aujla</t>
+          <t>Atif Aslam</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>2026-04-08</t>
+          <t>2026-04-10</t>
         </is>
       </c>
       <c r="B28" t="n">
@@ -21748,19 +22785,19 @@
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>Raanjhan</t>
+          <t>Darkhaast</t>
         </is>
       </c>
       <c r="D28" t="inlineStr">
         <is>
-          <t>Sachet-Parampara</t>
+          <t>Mithoon</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>2026-04-08</t>
+          <t>2026-04-10</t>
         </is>
       </c>
       <c r="B29" t="n">
@@ -21780,7 +22817,7 @@
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>2026-04-08</t>
+          <t>2026-04-10</t>
         </is>
       </c>
       <c r="B30" t="n">
@@ -21788,19 +22825,19 @@
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>Bairi</t>
+          <t>Phir Se</t>
         </is>
       </c>
       <c r="D30" t="inlineStr">
         <is>
-          <t>Virat</t>
+          <t>Shashwat Sachdev</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>2026-04-08</t>
+          <t>2026-04-10</t>
         </is>
       </c>
       <c r="B31" t="n">
@@ -21808,19 +22845,19 @@
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>Jo Tum Mere Ho</t>
+          <t>Tum Ho Toh</t>
         </is>
       </c>
       <c r="D31" t="inlineStr">
         <is>
-          <t>Anuv Jain</t>
+          <t>Vishal Mishra</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>2026-04-08</t>
+          <t>2026-04-10</t>
         </is>
       </c>
       <c r="B32" t="n">
@@ -21828,19 +22865,19 @@
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>Tere Liye</t>
+          <t>Raanjhan</t>
         </is>
       </c>
       <c r="D32" t="inlineStr">
         <is>
-          <t>Atif Aslam</t>
+          <t>Sachet-Parampara</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>2026-04-08</t>
+          <t>2026-04-10</t>
         </is>
       </c>
       <c r="B33" t="n">
@@ -21848,19 +22885,19 @@
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>Phir Se</t>
+          <t>Agar Tum Saath Ho</t>
         </is>
       </c>
       <c r="D33" t="inlineStr">
         <is>
-          <t>Shashwat Sachdev</t>
+          <t>Alka Yagnik</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>2026-04-08</t>
+          <t>2026-04-10</t>
         </is>
       </c>
       <c r="B34" t="n">
@@ -21868,19 +22905,19 @@
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>Agar Tum Saath Ho</t>
+          <t>Jogi</t>
         </is>
       </c>
       <c r="D34" t="inlineStr">
         <is>
-          <t>Alka Yagnik</t>
+          <t>thiarajxtt</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>2026-04-08</t>
+          <t>2026-04-10</t>
         </is>
       </c>
       <c r="B35" t="n">
@@ -21900,7 +22937,7 @@
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>2026-04-08</t>
+          <t>2026-04-10</t>
         </is>
       </c>
       <c r="B36" t="n">
@@ -21908,19 +22945,19 @@
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>Run Down The City - Monica</t>
+          <t>Jo Tum Mere Ho</t>
         </is>
       </c>
       <c r="D36" t="inlineStr">
         <is>
-          <t>Shashwat Sachdev</t>
+          <t>Anuv Jain</t>
         </is>
       </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>2026-04-08</t>
+          <t>2026-04-10</t>
         </is>
       </c>
       <c r="B37" t="n">
@@ -21928,19 +22965,19 @@
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>Haseen</t>
+          <t>Lutt Le Gaya</t>
         </is>
       </c>
       <c r="D37" t="inlineStr">
         <is>
-          <t>Talwiinder</t>
+          <t>Shashwat Sachdev</t>
         </is>
       </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>2026-04-08</t>
+          <t>2026-04-10</t>
         </is>
       </c>
       <c r="B38" t="n">
@@ -21960,7 +22997,7 @@
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>2026-04-08</t>
+          <t>2026-04-10</t>
         </is>
       </c>
       <c r="B39" t="n">
@@ -21968,19 +23005,19 @@
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>Lutt Le Gaya</t>
+          <t>Teri Deewani</t>
         </is>
       </c>
       <c r="D39" t="inlineStr">
         <is>
-          <t>Shashwat Sachdev</t>
+          <t>Kailash Kher</t>
         </is>
       </c>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>2026-04-08</t>
+          <t>2026-04-10</t>
         </is>
       </c>
       <c r="B40" t="n">
@@ -21988,19 +23025,19 @@
       </c>
       <c r="C40" t="inlineStr">
         <is>
-          <t>Teri Deewani</t>
+          <t>Run Down The City - Monica</t>
         </is>
       </c>
       <c r="D40" t="inlineStr">
         <is>
-          <t>Kailash Kher</t>
+          <t>Shashwat Sachdev</t>
         </is>
       </c>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>2026-04-08</t>
+          <t>2026-04-10</t>
         </is>
       </c>
       <c r="B41" t="n">
@@ -22008,19 +23045,19 @@
       </c>
       <c r="C41" t="inlineStr">
         <is>
-          <t>Jogi</t>
+          <t>Haseen</t>
         </is>
       </c>
       <c r="D41" t="inlineStr">
         <is>
-          <t>thiarajxtt</t>
+          <t>Talwiinder</t>
         </is>
       </c>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>2026-04-08</t>
+          <t>2026-04-10</t>
         </is>
       </c>
       <c r="B42" t="n">
@@ -22040,7 +23077,7 @@
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>2026-04-08</t>
+          <t>2026-04-10</t>
         </is>
       </c>
       <c r="B43" t="n">
@@ -22048,19 +23085,19 @@
       </c>
       <c r="C43" t="inlineStr">
         <is>
-          <t>Mann Mera - Original Version</t>
+          <t>Zaalima</t>
         </is>
       </c>
       <c r="D43" t="inlineStr">
         <is>
-          <t>Gajendra Verma</t>
+          <t>Arijit Singh</t>
         </is>
       </c>
     </row>
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>2026-04-08</t>
+          <t>2026-04-10</t>
         </is>
       </c>
       <c r="B44" t="n">
@@ -22068,19 +23105,19 @@
       </c>
       <c r="C44" t="inlineStr">
         <is>
-          <t>Ehsaas</t>
+          <t>Mast Magan</t>
         </is>
       </c>
       <c r="D44" t="inlineStr">
         <is>
-          <t>Faheem Abdullah</t>
+          <t>Arijit Singh</t>
         </is>
       </c>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>2026-04-08</t>
+          <t>2026-04-10</t>
         </is>
       </c>
       <c r="B45" t="n">
@@ -22088,19 +23125,19 @@
       </c>
       <c r="C45" t="inlineStr">
         <is>
-          <t>Dhun</t>
+          <t>Ehsaas</t>
         </is>
       </c>
       <c r="D45" t="inlineStr">
         <is>
-          <t>Mithoon</t>
+          <t>Faheem Abdullah</t>
         </is>
       </c>
     </row>
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>2026-04-08</t>
+          <t>2026-04-10</t>
         </is>
       </c>
       <c r="B46" t="n">
@@ -22108,19 +23145,19 @@
       </c>
       <c r="C46" t="inlineStr">
         <is>
-          <t>Zaalima</t>
+          <t>Main Aur Tu</t>
         </is>
       </c>
       <c r="D46" t="inlineStr">
         <is>
-          <t>Arijit Singh</t>
+          <t>Shashwat Sachdev</t>
         </is>
       </c>
     </row>
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>2026-04-08</t>
+          <t>2026-04-10</t>
         </is>
       </c>
       <c r="B47" t="n">
@@ -22128,19 +23165,19 @@
       </c>
       <c r="C47" t="inlineStr">
         <is>
-          <t>Thodi Si Daaru</t>
+          <t>Not Guilty</t>
         </is>
       </c>
       <c r="D47" t="inlineStr">
         <is>
-          <t>AP Dhillon</t>
+          <t>Dhanda Nyoliwala</t>
         </is>
       </c>
     </row>
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>2026-04-08</t>
+          <t>2026-04-10</t>
         </is>
       </c>
       <c r="B48" t="n">
@@ -22148,19 +23185,19 @@
       </c>
       <c r="C48" t="inlineStr">
         <is>
-          <t>Main Aur Tu</t>
+          <t>Mann Mera - Original Version</t>
         </is>
       </c>
       <c r="D48" t="inlineStr">
         <is>
-          <t>Shashwat Sachdev</t>
+          <t>Gajendra Verma</t>
         </is>
       </c>
     </row>
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>2026-04-08</t>
+          <t>2026-04-10</t>
         </is>
       </c>
       <c r="B49" t="n">
@@ -22180,7 +23217,7 @@
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>2026-04-08</t>
+          <t>2026-04-10</t>
         </is>
       </c>
       <c r="B50" t="n">
@@ -22188,19 +23225,19 @@
       </c>
       <c r="C50" t="inlineStr">
         <is>
-          <t>Mast Magan</t>
+          <t>Mutta Kalakki</t>
         </is>
       </c>
       <c r="D50" t="inlineStr">
         <is>
-          <t>Arijit Singh</t>
+          <t>G. V. Prakash</t>
         </is>
       </c>
     </row>
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>2026-04-08</t>
+          <t>2026-04-10</t>
         </is>
       </c>
       <c r="B51" t="n">
@@ -22208,12 +23245,12 @@
       </c>
       <c r="C51" t="inlineStr">
         <is>
-          <t>Aaya Sher</t>
+          <t>Jhol - Acoustic</t>
         </is>
       </c>
       <c r="D51" t="inlineStr">
         <is>
-          <t>Anirudh Ravichander</t>
+          <t>Maanu</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
added data till 11th april, got predictions for 12th april
</commit_message>
<xml_diff>
--- a/Probability Project.xlsx
+++ b/Probability Project.xlsx
@@ -31,6 +31,7 @@
     <sheet name="AUTO_20260407" sheetId="26" state="visible" r:id="rId26"/>
     <sheet name="AUTO_20260408" sheetId="27" state="visible" r:id="rId27"/>
     <sheet name="AUTO_20260410" sheetId="28" state="visible" r:id="rId28"/>
+    <sheet name="AUTO_20260411" sheetId="29" state="visible" r:id="rId29"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -22255,9 +22256,1045 @@
       </c>
     </row>
     <row r="2">
+      <c r="A2" s="0" t="inlineStr">
+        <is>
+          <t>2026-04-10</t>
+        </is>
+      </c>
+      <c r="B2" s="0" t="n">
+        <v>1</v>
+      </c>
+      <c r="C2" s="0" t="inlineStr">
+        <is>
+          <t>Bairan</t>
+        </is>
+      </c>
+      <c r="D2" s="0" t="inlineStr">
+        <is>
+          <t>Banjaare</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="0" t="inlineStr">
+        <is>
+          <t>2026-04-10</t>
+        </is>
+      </c>
+      <c r="B3" s="0" t="n">
+        <v>2</v>
+      </c>
+      <c r="C3" s="0" t="inlineStr">
+        <is>
+          <t>Jaiye Sajana</t>
+        </is>
+      </c>
+      <c r="D3" s="0" t="inlineStr">
+        <is>
+          <t>Shashwat Sachdev</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="0" t="inlineStr">
+        <is>
+          <t>2026-04-10</t>
+        </is>
+      </c>
+      <c r="B4" s="0" t="n">
+        <v>3</v>
+      </c>
+      <c r="C4" s="0" t="inlineStr">
+        <is>
+          <t>Gehra Hua</t>
+        </is>
+      </c>
+      <c r="D4" s="0" t="inlineStr">
+        <is>
+          <t>Shashwat Sachdev</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="0" t="inlineStr">
+        <is>
+          <t>2026-04-10</t>
+        </is>
+      </c>
+      <c r="B5" s="0" t="n">
+        <v>4</v>
+      </c>
+      <c r="C5" s="0" t="inlineStr">
+        <is>
+          <t>Sheesha - Aakhya Mai Aakh Ghali Jo Bairan</t>
+        </is>
+      </c>
+      <c r="D5" s="0" t="inlineStr">
+        <is>
+          <t>Mitta Ror</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="0" t="inlineStr">
+        <is>
+          <t>2026-04-10</t>
+        </is>
+      </c>
+      <c r="B6" s="0" t="n">
+        <v>5</v>
+      </c>
+      <c r="C6" s="0" t="inlineStr">
+        <is>
+          <t>Khat</t>
+        </is>
+      </c>
+      <c r="D6" s="0" t="inlineStr">
+        <is>
+          <t>Navjot Ahuja</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="0" t="inlineStr">
+        <is>
+          <t>2026-04-10</t>
+        </is>
+      </c>
+      <c r="B7" s="0" t="n">
+        <v>6</v>
+      </c>
+      <c r="C7" s="0" t="inlineStr">
+        <is>
+          <t>Dhurandhar The Revenge - Aari Aari</t>
+        </is>
+      </c>
+      <c r="D7" s="0" t="inlineStr">
+        <is>
+          <t>Shashwat Sachdev</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="0" t="inlineStr">
+        <is>
+          <t>2026-04-10</t>
+        </is>
+      </c>
+      <c r="B8" s="0" t="n">
+        <v>7</v>
+      </c>
+      <c r="C8" s="0" t="inlineStr">
+        <is>
+          <t>Dooron Dooron</t>
+        </is>
+      </c>
+      <c r="D8" s="0" t="inlineStr">
+        <is>
+          <t>Paresh Pahuja</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="0" t="inlineStr">
+        <is>
+          <t>2026-04-10</t>
+        </is>
+      </c>
+      <c r="B9" s="0" t="n">
+        <v>8</v>
+      </c>
+      <c r="C9" s="0" t="inlineStr">
+        <is>
+          <t>Apna Bana Le</t>
+        </is>
+      </c>
+      <c r="D9" s="0" t="inlineStr">
+        <is>
+          <t>Sachin-Jigar</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="0" t="inlineStr">
+        <is>
+          <t>2026-04-10</t>
+        </is>
+      </c>
+      <c r="B10" s="0" t="n">
+        <v>9</v>
+      </c>
+      <c r="C10" s="0" t="inlineStr">
+        <is>
+          <t>Sitaare</t>
+        </is>
+      </c>
+      <c r="D10" s="0" t="inlineStr">
+        <is>
+          <t>Arijit Singh</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="0" t="inlineStr">
+        <is>
+          <t>2026-04-10</t>
+        </is>
+      </c>
+      <c r="B11" s="0" t="n">
+        <v>10</v>
+      </c>
+      <c r="C11" s="0" t="inlineStr">
+        <is>
+          <t>Sahiba</t>
+        </is>
+      </c>
+      <c r="D11" s="0" t="inlineStr">
+        <is>
+          <t>Aditya Rikhari</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="0" t="inlineStr">
+        <is>
+          <t>2026-04-10</t>
+        </is>
+      </c>
+      <c r="B12" s="0" t="n">
+        <v>11</v>
+      </c>
+      <c r="C12" s="0" t="inlineStr">
+        <is>
+          <t>Jaan Se Guzarte Hain</t>
+        </is>
+      </c>
+      <c r="D12" s="0" t="inlineStr">
+        <is>
+          <t>Shashwat Sachdev</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="0" t="inlineStr">
+        <is>
+          <t>2026-04-10</t>
+        </is>
+      </c>
+      <c r="B13" s="0" t="n">
+        <v>12</v>
+      </c>
+      <c r="C13" s="0" t="inlineStr">
+        <is>
+          <t>Samjhawan</t>
+        </is>
+      </c>
+      <c r="D13" s="0" t="inlineStr">
+        <is>
+          <t>Jawad Ahmad</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="0" t="inlineStr">
+        <is>
+          <t>2026-04-10</t>
+        </is>
+      </c>
+      <c r="B14" s="0" t="n">
+        <v>13</v>
+      </c>
+      <c r="C14" s="0" t="inlineStr">
+        <is>
+          <t>Pavazha Malli</t>
+        </is>
+      </c>
+      <c r="D14" s="0" t="inlineStr">
+        <is>
+          <t>Sai Abhyankkar</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="0" t="inlineStr">
+        <is>
+          <t>2026-04-10</t>
+        </is>
+      </c>
+      <c r="B15" s="0" t="n">
+        <v>14</v>
+      </c>
+      <c r="C15" s="0" t="inlineStr">
+        <is>
+          <t>Finding Her</t>
+        </is>
+      </c>
+      <c r="D15" s="0" t="inlineStr">
+        <is>
+          <t>Kushagra</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="0" t="inlineStr">
+        <is>
+          <t>2026-04-10</t>
+        </is>
+      </c>
+      <c r="B16" s="0" t="n">
+        <v>15</v>
+      </c>
+      <c r="C16" s="0" t="inlineStr">
+        <is>
+          <t>Boyfriend</t>
+        </is>
+      </c>
+      <c r="D16" s="0" t="inlineStr">
+        <is>
+          <t>Karan Aujla</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="0" t="inlineStr">
+        <is>
+          <t>2026-04-10</t>
+        </is>
+      </c>
+      <c r="B17" s="0" t="n">
+        <v>16</v>
+      </c>
+      <c r="C17" s="0" t="inlineStr">
+        <is>
+          <t>Arz Kiya Hai | Coke Studio Bharat</t>
+        </is>
+      </c>
+      <c r="D17" s="0" t="inlineStr">
+        <is>
+          <t>Anuv Jain</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="0" t="inlineStr">
+        <is>
+          <t>2026-04-10</t>
+        </is>
+      </c>
+      <c r="B18" s="0" t="n">
+        <v>17</v>
+      </c>
+      <c r="C18" s="0" t="inlineStr">
+        <is>
+          <t>Shararat</t>
+        </is>
+      </c>
+      <c r="D18" s="0" t="inlineStr">
+        <is>
+          <t>Shashwat Sachdev</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="0" t="inlineStr">
+        <is>
+          <t>2026-04-10</t>
+        </is>
+      </c>
+      <c r="B19" s="0" t="n">
+        <v>18</v>
+      </c>
+      <c r="C19" s="0" t="inlineStr">
+        <is>
+          <t>Mann Mera</t>
+        </is>
+      </c>
+      <c r="D19" s="0" t="inlineStr">
+        <is>
+          <t>Gajendra Verma</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="0" t="inlineStr">
+        <is>
+          <t>2026-04-10</t>
+        </is>
+      </c>
+      <c r="B20" s="0" t="n">
+        <v>19</v>
+      </c>
+      <c r="C20" s="0" t="inlineStr">
+        <is>
+          <t>Ishq</t>
+        </is>
+      </c>
+      <c r="D20" s="0" t="inlineStr">
+        <is>
+          <t>Faheem Abdullah</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="0" t="inlineStr">
+        <is>
+          <t>2026-04-10</t>
+        </is>
+      </c>
+      <c r="B21" s="0" t="n">
+        <v>20</v>
+      </c>
+      <c r="C21" s="0" t="inlineStr">
+        <is>
+          <t>For A Reason</t>
+        </is>
+      </c>
+      <c r="D21" s="0" t="inlineStr">
+        <is>
+          <t>Karan Aujla</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="0" t="inlineStr">
+        <is>
+          <t>2026-04-10</t>
+        </is>
+      </c>
+      <c r="B22" s="0" t="n">
+        <v>21</v>
+      </c>
+      <c r="C22" s="0" t="inlineStr">
+        <is>
+          <t>Saiyaara</t>
+        </is>
+      </c>
+      <c r="D22" s="0" t="inlineStr">
+        <is>
+          <t>Tanishk Bagchi</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="0" t="inlineStr">
+        <is>
+          <t>2026-04-10</t>
+        </is>
+      </c>
+      <c r="B23" s="0" t="n">
+        <v>22</v>
+      </c>
+      <c r="C23" s="0" t="inlineStr">
+        <is>
+          <t>Ishqa Ve</t>
+        </is>
+      </c>
+      <c r="D23" s="0" t="inlineStr">
+        <is>
+          <t>Zeeshan Ali</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="0" t="inlineStr">
+        <is>
+          <t>2026-04-10</t>
+        </is>
+      </c>
+      <c r="B24" s="0" t="n">
+        <v>23</v>
+      </c>
+      <c r="C24" s="0" t="inlineStr">
+        <is>
+          <t>Naal Nachna</t>
+        </is>
+      </c>
+      <c r="D24" s="0" t="inlineStr">
+        <is>
+          <t>Shashwat Sachdev</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="0" t="inlineStr">
+        <is>
+          <t>2026-04-10</t>
+        </is>
+      </c>
+      <c r="B25" s="0" t="n">
+        <v>24</v>
+      </c>
+      <c r="C25" s="0" t="inlineStr">
+        <is>
+          <t>Bairi</t>
+        </is>
+      </c>
+      <c r="D25" s="0" t="inlineStr">
+        <is>
+          <t>Virat</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="0" t="inlineStr">
+        <is>
+          <t>2026-04-10</t>
+        </is>
+      </c>
+      <c r="B26" s="0" t="n">
+        <v>25</v>
+      </c>
+      <c r="C26" s="0" t="inlineStr">
+        <is>
+          <t>Dhurandhar - Title Track</t>
+        </is>
+      </c>
+      <c r="D26" s="0" t="inlineStr">
+        <is>
+          <t>Shashwat Sachdev</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="0" t="inlineStr">
+        <is>
+          <t>2026-04-10</t>
+        </is>
+      </c>
+      <c r="B27" s="0" t="n">
+        <v>26</v>
+      </c>
+      <c r="C27" s="0" t="inlineStr">
+        <is>
+          <t>Tere Liye</t>
+        </is>
+      </c>
+      <c r="D27" s="0" t="inlineStr">
+        <is>
+          <t>Atif Aslam</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="0" t="inlineStr">
+        <is>
+          <t>2026-04-10</t>
+        </is>
+      </c>
+      <c r="B28" s="0" t="n">
+        <v>27</v>
+      </c>
+      <c r="C28" s="0" t="inlineStr">
+        <is>
+          <t>Darkhaast</t>
+        </is>
+      </c>
+      <c r="D28" s="0" t="inlineStr">
+        <is>
+          <t>Mithoon</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="0" t="inlineStr">
+        <is>
+          <t>2026-04-10</t>
+        </is>
+      </c>
+      <c r="B29" s="0" t="n">
+        <v>28</v>
+      </c>
+      <c r="C29" s="0" t="inlineStr">
+        <is>
+          <t>Deewaana Deewaana</t>
+        </is>
+      </c>
+      <c r="D29" s="0" t="inlineStr">
+        <is>
+          <t>A.R. Rahman</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="0" t="inlineStr">
+        <is>
+          <t>2026-04-10</t>
+        </is>
+      </c>
+      <c r="B30" s="0" t="n">
+        <v>29</v>
+      </c>
+      <c r="C30" s="0" t="inlineStr">
+        <is>
+          <t>Phir Se</t>
+        </is>
+      </c>
+      <c r="D30" s="0" t="inlineStr">
+        <is>
+          <t>Shashwat Sachdev</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="0" t="inlineStr">
+        <is>
+          <t>2026-04-10</t>
+        </is>
+      </c>
+      <c r="B31" s="0" t="n">
+        <v>30</v>
+      </c>
+      <c r="C31" s="0" t="inlineStr">
+        <is>
+          <t>Tum Ho Toh</t>
+        </is>
+      </c>
+      <c r="D31" s="0" t="inlineStr">
+        <is>
+          <t>Vishal Mishra</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="0" t="inlineStr">
+        <is>
+          <t>2026-04-10</t>
+        </is>
+      </c>
+      <c r="B32" s="0" t="n">
+        <v>31</v>
+      </c>
+      <c r="C32" s="0" t="inlineStr">
+        <is>
+          <t>Raanjhan</t>
+        </is>
+      </c>
+      <c r="D32" s="0" t="inlineStr">
+        <is>
+          <t>Sachet-Parampara</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="0" t="inlineStr">
+        <is>
+          <t>2026-04-10</t>
+        </is>
+      </c>
+      <c r="B33" s="0" t="n">
+        <v>32</v>
+      </c>
+      <c r="C33" s="0" t="inlineStr">
+        <is>
+          <t>Agar Tum Saath Ho</t>
+        </is>
+      </c>
+      <c r="D33" s="0" t="inlineStr">
+        <is>
+          <t>Alka Yagnik</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="0" t="inlineStr">
+        <is>
+          <t>2026-04-10</t>
+        </is>
+      </c>
+      <c r="B34" s="0" t="n">
+        <v>33</v>
+      </c>
+      <c r="C34" s="0" t="inlineStr">
+        <is>
+          <t>Jogi</t>
+        </is>
+      </c>
+      <c r="D34" s="0" t="inlineStr">
+        <is>
+          <t>thiarajxtt</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="0" t="inlineStr">
+        <is>
+          <t>2026-04-10</t>
+        </is>
+      </c>
+      <c r="B35" s="0" t="n">
+        <v>34</v>
+      </c>
+      <c r="C35" s="0" t="inlineStr">
+        <is>
+          <t>Tere Bina</t>
+        </is>
+      </c>
+      <c r="D35" s="0" t="inlineStr">
+        <is>
+          <t>A.R. Rahman</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="0" t="inlineStr">
+        <is>
+          <t>2026-04-10</t>
+        </is>
+      </c>
+      <c r="B36" s="0" t="n">
+        <v>35</v>
+      </c>
+      <c r="C36" s="0" t="inlineStr">
+        <is>
+          <t>Jo Tum Mere Ho</t>
+        </is>
+      </c>
+      <c r="D36" s="0" t="inlineStr">
+        <is>
+          <t>Anuv Jain</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="0" t="inlineStr">
+        <is>
+          <t>2026-04-10</t>
+        </is>
+      </c>
+      <c r="B37" s="0" t="n">
+        <v>36</v>
+      </c>
+      <c r="C37" s="0" t="inlineStr">
+        <is>
+          <t>Lutt Le Gaya</t>
+        </is>
+      </c>
+      <c r="D37" s="0" t="inlineStr">
+        <is>
+          <t>Shashwat Sachdev</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="0" t="inlineStr">
+        <is>
+          <t>2026-04-10</t>
+        </is>
+      </c>
+      <c r="B38" s="0" t="n">
+        <v>37</v>
+      </c>
+      <c r="C38" s="0" t="inlineStr">
+        <is>
+          <t>Barbaad</t>
+        </is>
+      </c>
+      <c r="D38" s="0" t="inlineStr">
+        <is>
+          <t>The Rish</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="0" t="inlineStr">
+        <is>
+          <t>2026-04-10</t>
+        </is>
+      </c>
+      <c r="B39" s="0" t="n">
+        <v>38</v>
+      </c>
+      <c r="C39" s="0" t="inlineStr">
+        <is>
+          <t>Teri Deewani</t>
+        </is>
+      </c>
+      <c r="D39" s="0" t="inlineStr">
+        <is>
+          <t>Kailash Kher</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="0" t="inlineStr">
+        <is>
+          <t>2026-04-10</t>
+        </is>
+      </c>
+      <c r="B40" s="0" t="n">
+        <v>39</v>
+      </c>
+      <c r="C40" s="0" t="inlineStr">
+        <is>
+          <t>Run Down The City - Monica</t>
+        </is>
+      </c>
+      <c r="D40" s="0" t="inlineStr">
+        <is>
+          <t>Shashwat Sachdev</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" s="0" t="inlineStr">
+        <is>
+          <t>2026-04-10</t>
+        </is>
+      </c>
+      <c r="B41" s="0" t="n">
+        <v>40</v>
+      </c>
+      <c r="C41" s="0" t="inlineStr">
+        <is>
+          <t>Haseen</t>
+        </is>
+      </c>
+      <c r="D41" s="0" t="inlineStr">
+        <is>
+          <t>Talwiinder</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" s="0" t="inlineStr">
+        <is>
+          <t>2026-04-10</t>
+        </is>
+      </c>
+      <c r="B42" s="0" t="n">
+        <v>41</v>
+      </c>
+      <c r="C42" s="0" t="inlineStr">
+        <is>
+          <t>Ye Tune Kya Kiya</t>
+        </is>
+      </c>
+      <c r="D42" s="0" t="inlineStr">
+        <is>
+          <t>Pritam</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" s="0" t="inlineStr">
+        <is>
+          <t>2026-04-10</t>
+        </is>
+      </c>
+      <c r="B43" s="0" t="n">
+        <v>42</v>
+      </c>
+      <c r="C43" s="0" t="inlineStr">
+        <is>
+          <t>Zaalima</t>
+        </is>
+      </c>
+      <c r="D43" s="0" t="inlineStr">
+        <is>
+          <t>Arijit Singh</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" s="0" t="inlineStr">
+        <is>
+          <t>2026-04-10</t>
+        </is>
+      </c>
+      <c r="B44" s="0" t="n">
+        <v>43</v>
+      </c>
+      <c r="C44" s="0" t="inlineStr">
+        <is>
+          <t>Mast Magan</t>
+        </is>
+      </c>
+      <c r="D44" s="0" t="inlineStr">
+        <is>
+          <t>Arijit Singh</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" s="0" t="inlineStr">
+        <is>
+          <t>2026-04-10</t>
+        </is>
+      </c>
+      <c r="B45" s="0" t="n">
+        <v>44</v>
+      </c>
+      <c r="C45" s="0" t="inlineStr">
+        <is>
+          <t>Ehsaas</t>
+        </is>
+      </c>
+      <c r="D45" s="0" t="inlineStr">
+        <is>
+          <t>Faheem Abdullah</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" s="0" t="inlineStr">
+        <is>
+          <t>2026-04-10</t>
+        </is>
+      </c>
+      <c r="B46" s="0" t="n">
+        <v>45</v>
+      </c>
+      <c r="C46" s="0" t="inlineStr">
+        <is>
+          <t>Main Aur Tu</t>
+        </is>
+      </c>
+      <c r="D46" s="0" t="inlineStr">
+        <is>
+          <t>Shashwat Sachdev</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" s="0" t="inlineStr">
+        <is>
+          <t>2026-04-10</t>
+        </is>
+      </c>
+      <c r="B47" s="0" t="n">
+        <v>46</v>
+      </c>
+      <c r="C47" s="0" t="inlineStr">
+        <is>
+          <t>Not Guilty</t>
+        </is>
+      </c>
+      <c r="D47" s="0" t="inlineStr">
+        <is>
+          <t>Dhanda Nyoliwala</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" s="0" t="inlineStr">
+        <is>
+          <t>2026-04-10</t>
+        </is>
+      </c>
+      <c r="B48" s="0" t="n">
+        <v>47</v>
+      </c>
+      <c r="C48" s="0" t="inlineStr">
+        <is>
+          <t>Mann Mera - Original Version</t>
+        </is>
+      </c>
+      <c r="D48" s="0" t="inlineStr">
+        <is>
+          <t>Gajendra Verma</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" s="0" t="inlineStr">
+        <is>
+          <t>2026-04-10</t>
+        </is>
+      </c>
+      <c r="B49" s="0" t="n">
+        <v>48</v>
+      </c>
+      <c r="C49" s="0" t="inlineStr">
+        <is>
+          <t>Ishq Jalakar - Karvaan</t>
+        </is>
+      </c>
+      <c r="D49" s="0" t="inlineStr">
+        <is>
+          <t>Shashwat Sachdev</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" s="0" t="inlineStr">
+        <is>
+          <t>2026-04-10</t>
+        </is>
+      </c>
+      <c r="B50" s="0" t="n">
+        <v>49</v>
+      </c>
+      <c r="C50" s="0" t="inlineStr">
+        <is>
+          <t>Mutta Kalakki</t>
+        </is>
+      </c>
+      <c r="D50" s="0" t="inlineStr">
+        <is>
+          <t>G. V. Prakash</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" s="0" t="inlineStr">
+        <is>
+          <t>2026-04-10</t>
+        </is>
+      </c>
+      <c r="B51" s="0" t="n">
+        <v>50</v>
+      </c>
+      <c r="C51" s="0" t="inlineStr">
+        <is>
+          <t>Jhol - Acoustic</t>
+        </is>
+      </c>
+      <c r="D51" s="0" t="inlineStr">
+        <is>
+          <t>Maanu</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet29.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:D51"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="24" t="inlineStr">
+        <is>
+          <t>Date</t>
+        </is>
+      </c>
+      <c r="B1" s="24" t="inlineStr">
+        <is>
+          <t>Rank</t>
+        </is>
+      </c>
+      <c r="C1" s="24" t="inlineStr">
+        <is>
+          <t>Song</t>
+        </is>
+      </c>
+      <c r="D1" s="24" t="inlineStr">
+        <is>
+          <t>Artist</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>2026-04-10</t>
+          <t>2026-04-11</t>
         </is>
       </c>
       <c r="B2" t="n">
@@ -22277,7 +23314,7 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>2026-04-10</t>
+          <t>2026-04-11</t>
         </is>
       </c>
       <c r="B3" t="n">
@@ -22297,7 +23334,7 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>2026-04-10</t>
+          <t>2026-04-11</t>
         </is>
       </c>
       <c r="B4" t="n">
@@ -22317,7 +23354,7 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>2026-04-10</t>
+          <t>2026-04-11</t>
         </is>
       </c>
       <c r="B5" t="n">
@@ -22337,7 +23374,7 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>2026-04-10</t>
+          <t>2026-04-11</t>
         </is>
       </c>
       <c r="B6" t="n">
@@ -22357,7 +23394,7 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>2026-04-10</t>
+          <t>2026-04-11</t>
         </is>
       </c>
       <c r="B7" t="n">
@@ -22365,19 +23402,19 @@
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>Dhurandhar The Revenge - Aari Aari</t>
+          <t>Sahiba</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>Shashwat Sachdev</t>
+          <t>Aditya Rikhari</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>2026-04-10</t>
+          <t>2026-04-11</t>
         </is>
       </c>
       <c r="B8" t="n">
@@ -22397,7 +23434,7 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>2026-04-10</t>
+          <t>2026-04-11</t>
         </is>
       </c>
       <c r="B9" t="n">
@@ -22405,19 +23442,19 @@
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>Apna Bana Le</t>
+          <t>Dhurandhar The Revenge - Aari Aari</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>Sachin-Jigar</t>
+          <t>Shashwat Sachdev</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>2026-04-10</t>
+          <t>2026-04-11</t>
         </is>
       </c>
       <c r="B10" t="n">
@@ -22425,19 +23462,19 @@
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>Sitaare</t>
+          <t>Apna Bana Le</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>Arijit Singh</t>
+          <t>Sachin-Jigar</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>2026-04-10</t>
+          <t>2026-04-11</t>
         </is>
       </c>
       <c r="B11" t="n">
@@ -22445,19 +23482,19 @@
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>Sahiba</t>
+          <t>Sitaare</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>Aditya Rikhari</t>
+          <t>Arijit Singh</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>2026-04-10</t>
+          <t>2026-04-11</t>
         </is>
       </c>
       <c r="B12" t="n">
@@ -22465,19 +23502,19 @@
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>Jaan Se Guzarte Hain</t>
+          <t>Samjhawan</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>Shashwat Sachdev</t>
+          <t>Jawad Ahmad</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>2026-04-10</t>
+          <t>2026-04-11</t>
         </is>
       </c>
       <c r="B13" t="n">
@@ -22485,19 +23522,19 @@
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>Samjhawan</t>
+          <t>Jaan Se Guzarte Hain</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>Jawad Ahmad</t>
+          <t>Shashwat Sachdev</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>2026-04-10</t>
+          <t>2026-04-11</t>
         </is>
       </c>
       <c r="B14" t="n">
@@ -22505,19 +23542,19 @@
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>Pavazha Malli</t>
+          <t>Boyfriend</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>Sai Abhyankkar</t>
+          <t>Karan Aujla</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>2026-04-10</t>
+          <t>2026-04-11</t>
         </is>
       </c>
       <c r="B15" t="n">
@@ -22525,19 +23562,19 @@
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>Finding Her</t>
+          <t>Pavazha Malli</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>Kushagra</t>
+          <t>Sai Abhyankkar</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>2026-04-10</t>
+          <t>2026-04-11</t>
         </is>
       </c>
       <c r="B16" t="n">
@@ -22545,19 +23582,19 @@
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>Boyfriend</t>
+          <t>Finding Her</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>Karan Aujla</t>
+          <t>Kushagra</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>2026-04-10</t>
+          <t>2026-04-11</t>
         </is>
       </c>
       <c r="B17" t="n">
@@ -22577,7 +23614,7 @@
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>2026-04-10</t>
+          <t>2026-04-11</t>
         </is>
       </c>
       <c r="B18" t="n">
@@ -22597,7 +23634,7 @@
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>2026-04-10</t>
+          <t>2026-04-11</t>
         </is>
       </c>
       <c r="B19" t="n">
@@ -22605,19 +23642,19 @@
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>Mann Mera</t>
+          <t>Ishq</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>Gajendra Verma</t>
+          <t>Faheem Abdullah</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>2026-04-10</t>
+          <t>2026-04-11</t>
         </is>
       </c>
       <c r="B20" t="n">
@@ -22625,19 +23662,19 @@
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>Ishq</t>
+          <t>Mann Mera</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>Faheem Abdullah</t>
+          <t>Gajendra Verma</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>2026-04-10</t>
+          <t>2026-04-11</t>
         </is>
       </c>
       <c r="B21" t="n">
@@ -22645,19 +23682,19 @@
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>For A Reason</t>
+          <t>Saiyaara</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>Karan Aujla</t>
+          <t>Tanishk Bagchi</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>2026-04-10</t>
+          <t>2026-04-11</t>
         </is>
       </c>
       <c r="B22" t="n">
@@ -22665,19 +23702,19 @@
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>Saiyaara</t>
+          <t>For A Reason</t>
         </is>
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>Tanishk Bagchi</t>
+          <t>Karan Aujla</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>2026-04-10</t>
+          <t>2026-04-11</t>
         </is>
       </c>
       <c r="B23" t="n">
@@ -22685,19 +23722,19 @@
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>Ishqa Ve</t>
+          <t>Dhurandhar - Title Track</t>
         </is>
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>Zeeshan Ali</t>
+          <t>Shashwat Sachdev</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>2026-04-10</t>
+          <t>2026-04-11</t>
         </is>
       </c>
       <c r="B24" t="n">
@@ -22705,19 +23742,19 @@
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>Naal Nachna</t>
+          <t>Ishqa Ve</t>
         </is>
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>Shashwat Sachdev</t>
+          <t>Zeeshan Ali</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>2026-04-10</t>
+          <t>2026-04-11</t>
         </is>
       </c>
       <c r="B25" t="n">
@@ -22737,7 +23774,7 @@
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>2026-04-10</t>
+          <t>2026-04-11</t>
         </is>
       </c>
       <c r="B26" t="n">
@@ -22745,7 +23782,7 @@
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>Dhurandhar - Title Track</t>
+          <t>Naal Nachna</t>
         </is>
       </c>
       <c r="D26" t="inlineStr">
@@ -22757,7 +23794,7 @@
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>2026-04-10</t>
+          <t>2026-04-11</t>
         </is>
       </c>
       <c r="B27" t="n">
@@ -22777,7 +23814,7 @@
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>2026-04-10</t>
+          <t>2026-04-11</t>
         </is>
       </c>
       <c r="B28" t="n">
@@ -22785,19 +23822,19 @@
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>Darkhaast</t>
+          <t>Tum Ho Toh</t>
         </is>
       </c>
       <c r="D28" t="inlineStr">
         <is>
-          <t>Mithoon</t>
+          <t>Vishal Mishra</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>2026-04-10</t>
+          <t>2026-04-11</t>
         </is>
       </c>
       <c r="B29" t="n">
@@ -22805,19 +23842,19 @@
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>Deewaana Deewaana</t>
+          <t>Jo Tum Mere Ho</t>
         </is>
       </c>
       <c r="D29" t="inlineStr">
         <is>
-          <t>A.R. Rahman</t>
+          <t>Anuv Jain</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>2026-04-10</t>
+          <t>2026-04-11</t>
         </is>
       </c>
       <c r="B30" t="n">
@@ -22825,19 +23862,19 @@
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>Phir Se</t>
+          <t>Raanjhan</t>
         </is>
       </c>
       <c r="D30" t="inlineStr">
         <is>
-          <t>Shashwat Sachdev</t>
+          <t>Sachet-Parampara</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>2026-04-10</t>
+          <t>2026-04-11</t>
         </is>
       </c>
       <c r="B31" t="n">
@@ -22845,19 +23882,19 @@
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>Tum Ho Toh</t>
+          <t>Deewaana Deewaana</t>
         </is>
       </c>
       <c r="D31" t="inlineStr">
         <is>
-          <t>Vishal Mishra</t>
+          <t>A.R. Rahman</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>2026-04-10</t>
+          <t>2026-04-11</t>
         </is>
       </c>
       <c r="B32" t="n">
@@ -22865,19 +23902,19 @@
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>Raanjhan</t>
+          <t>Darkhaast</t>
         </is>
       </c>
       <c r="D32" t="inlineStr">
         <is>
-          <t>Sachet-Parampara</t>
+          <t>Mithoon</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>2026-04-10</t>
+          <t>2026-04-11</t>
         </is>
       </c>
       <c r="B33" t="n">
@@ -22885,19 +23922,19 @@
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>Agar Tum Saath Ho</t>
+          <t>Tere Bina</t>
         </is>
       </c>
       <c r="D33" t="inlineStr">
         <is>
-          <t>Alka Yagnik</t>
+          <t>A.R. Rahman</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>2026-04-10</t>
+          <t>2026-04-11</t>
         </is>
       </c>
       <c r="B34" t="n">
@@ -22905,19 +23942,19 @@
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>Jogi</t>
+          <t>Agar Tum Saath Ho</t>
         </is>
       </c>
       <c r="D34" t="inlineStr">
         <is>
-          <t>thiarajxtt</t>
+          <t>Alka Yagnik</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>2026-04-10</t>
+          <t>2026-04-11</t>
         </is>
       </c>
       <c r="B35" t="n">
@@ -22925,19 +23962,19 @@
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>Tere Bina</t>
+          <t>Phir Se</t>
         </is>
       </c>
       <c r="D35" t="inlineStr">
         <is>
-          <t>A.R. Rahman</t>
+          <t>Shashwat Sachdev</t>
         </is>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>2026-04-10</t>
+          <t>2026-04-11</t>
         </is>
       </c>
       <c r="B36" t="n">
@@ -22945,19 +23982,19 @@
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>Jo Tum Mere Ho</t>
+          <t>Lutt Le Gaya</t>
         </is>
       </c>
       <c r="D36" t="inlineStr">
         <is>
-          <t>Anuv Jain</t>
+          <t>Shashwat Sachdev</t>
         </is>
       </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>2026-04-10</t>
+          <t>2026-04-11</t>
         </is>
       </c>
       <c r="B37" t="n">
@@ -22965,19 +24002,19 @@
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>Lutt Le Gaya</t>
+          <t>Teri Deewani</t>
         </is>
       </c>
       <c r="D37" t="inlineStr">
         <is>
-          <t>Shashwat Sachdev</t>
+          <t>Kailash Kher</t>
         </is>
       </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>2026-04-10</t>
+          <t>2026-04-11</t>
         </is>
       </c>
       <c r="B38" t="n">
@@ -22985,19 +24022,19 @@
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>Barbaad</t>
+          <t>Haseen</t>
         </is>
       </c>
       <c r="D38" t="inlineStr">
         <is>
-          <t>The Rish</t>
+          <t>Talwiinder</t>
         </is>
       </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>2026-04-10</t>
+          <t>2026-04-11</t>
         </is>
       </c>
       <c r="B39" t="n">
@@ -23005,19 +24042,19 @@
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>Teri Deewani</t>
+          <t>Ye Tune Kya Kiya</t>
         </is>
       </c>
       <c r="D39" t="inlineStr">
         <is>
-          <t>Kailash Kher</t>
+          <t>Pritam</t>
         </is>
       </c>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>2026-04-10</t>
+          <t>2026-04-11</t>
         </is>
       </c>
       <c r="B40" t="n">
@@ -23025,19 +24062,19 @@
       </c>
       <c r="C40" t="inlineStr">
         <is>
-          <t>Run Down The City - Monica</t>
+          <t>Barbaad</t>
         </is>
       </c>
       <c r="D40" t="inlineStr">
         <is>
-          <t>Shashwat Sachdev</t>
+          <t>The Rish</t>
         </is>
       </c>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>2026-04-10</t>
+          <t>2026-04-11</t>
         </is>
       </c>
       <c r="B41" t="n">
@@ -23045,19 +24082,19 @@
       </c>
       <c r="C41" t="inlineStr">
         <is>
-          <t>Haseen</t>
+          <t>Ehsaas</t>
         </is>
       </c>
       <c r="D41" t="inlineStr">
         <is>
-          <t>Talwiinder</t>
+          <t>Faheem Abdullah</t>
         </is>
       </c>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>2026-04-10</t>
+          <t>2026-04-11</t>
         </is>
       </c>
       <c r="B42" t="n">
@@ -23065,19 +24102,19 @@
       </c>
       <c r="C42" t="inlineStr">
         <is>
-          <t>Ye Tune Kya Kiya</t>
+          <t>Run Down The City - Monica</t>
         </is>
       </c>
       <c r="D42" t="inlineStr">
         <is>
-          <t>Pritam</t>
+          <t>Shashwat Sachdev</t>
         </is>
       </c>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>2026-04-10</t>
+          <t>2026-04-11</t>
         </is>
       </c>
       <c r="B43" t="n">
@@ -23085,7 +24122,7 @@
       </c>
       <c r="C43" t="inlineStr">
         <is>
-          <t>Zaalima</t>
+          <t>Mast Magan</t>
         </is>
       </c>
       <c r="D43" t="inlineStr">
@@ -23097,7 +24134,7 @@
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>2026-04-10</t>
+          <t>2026-04-11</t>
         </is>
       </c>
       <c r="B44" t="n">
@@ -23105,19 +24142,19 @@
       </c>
       <c r="C44" t="inlineStr">
         <is>
-          <t>Mast Magan</t>
+          <t>Thodi Si Daaru</t>
         </is>
       </c>
       <c r="D44" t="inlineStr">
         <is>
-          <t>Arijit Singh</t>
+          <t>AP Dhillon</t>
         </is>
       </c>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>2026-04-10</t>
+          <t>2026-04-11</t>
         </is>
       </c>
       <c r="B45" t="n">
@@ -23125,19 +24162,19 @@
       </c>
       <c r="C45" t="inlineStr">
         <is>
-          <t>Ehsaas</t>
+          <t>Ishq Jalakar - Karvaan</t>
         </is>
       </c>
       <c r="D45" t="inlineStr">
         <is>
-          <t>Faheem Abdullah</t>
+          <t>Shashwat Sachdev</t>
         </is>
       </c>
     </row>
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>2026-04-10</t>
+          <t>2026-04-11</t>
         </is>
       </c>
       <c r="B46" t="n">
@@ -23145,19 +24182,19 @@
       </c>
       <c r="C46" t="inlineStr">
         <is>
-          <t>Main Aur Tu</t>
+          <t>Mutta Kalakki</t>
         </is>
       </c>
       <c r="D46" t="inlineStr">
         <is>
-          <t>Shashwat Sachdev</t>
+          <t>G. V. Prakash</t>
         </is>
       </c>
     </row>
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>2026-04-10</t>
+          <t>2026-04-11</t>
         </is>
       </c>
       <c r="B47" t="n">
@@ -23165,19 +24202,19 @@
       </c>
       <c r="C47" t="inlineStr">
         <is>
-          <t>Not Guilty</t>
+          <t>Zaalima</t>
         </is>
       </c>
       <c r="D47" t="inlineStr">
         <is>
-          <t>Dhanda Nyoliwala</t>
+          <t>Arijit Singh</t>
         </is>
       </c>
     </row>
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>2026-04-10</t>
+          <t>2026-04-11</t>
         </is>
       </c>
       <c r="B48" t="n">
@@ -23185,19 +24222,19 @@
       </c>
       <c r="C48" t="inlineStr">
         <is>
-          <t>Mann Mera - Original Version</t>
+          <t>Not Guilty</t>
         </is>
       </c>
       <c r="D48" t="inlineStr">
         <is>
-          <t>Gajendra Verma</t>
+          <t>Dhanda Nyoliwala</t>
         </is>
       </c>
     </row>
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>2026-04-10</t>
+          <t>2026-04-11</t>
         </is>
       </c>
       <c r="B49" t="n">
@@ -23205,19 +24242,19 @@
       </c>
       <c r="C49" t="inlineStr">
         <is>
-          <t>Ishq Jalakar - Karvaan</t>
+          <t>Jogi</t>
         </is>
       </c>
       <c r="D49" t="inlineStr">
         <is>
-          <t>Shashwat Sachdev</t>
+          <t>thiarajxtt</t>
         </is>
       </c>
     </row>
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>2026-04-10</t>
+          <t>2026-04-11</t>
         </is>
       </c>
       <c r="B50" t="n">
@@ -23225,19 +24262,19 @@
       </c>
       <c r="C50" t="inlineStr">
         <is>
-          <t>Mutta Kalakki</t>
+          <t>Mann Mera - Original Version</t>
         </is>
       </c>
       <c r="D50" t="inlineStr">
         <is>
-          <t>G. V. Prakash</t>
+          <t>Gajendra Verma</t>
         </is>
       </c>
     </row>
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>2026-04-10</t>
+          <t>2026-04-11</t>
         </is>
       </c>
       <c r="B51" t="n">
@@ -23245,12 +24282,12 @@
       </c>
       <c r="C51" t="inlineStr">
         <is>
-          <t>Jhol - Acoustic</t>
+          <t>Humdard</t>
         </is>
       </c>
       <c r="D51" t="inlineStr">
         <is>
-          <t>Maanu</t>
+          <t>Arijit Singh</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
added data till 12th april, got predictions for 13th april
</commit_message>
<xml_diff>
--- a/Probability Project.xlsx
+++ b/Probability Project.xlsx
@@ -32,6 +32,7 @@
     <sheet name="AUTO_20260408" sheetId="27" state="visible" r:id="rId27"/>
     <sheet name="AUTO_20260410" sheetId="28" state="visible" r:id="rId28"/>
     <sheet name="AUTO_20260411" sheetId="29" state="visible" r:id="rId29"/>
+    <sheet name="AUTO_20260412" sheetId="30" state="visible" r:id="rId30"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -23292,1000 +23293,1000 @@
       </c>
     </row>
     <row r="2">
-      <c r="A2" t="inlineStr">
+      <c r="A2" s="0" t="inlineStr">
         <is>
           <t>2026-04-11</t>
         </is>
       </c>
-      <c r="B2" t="n">
+      <c r="B2" s="0" t="n">
         <v>1</v>
       </c>
-      <c r="C2" t="inlineStr">
+      <c r="C2" s="0" t="inlineStr">
         <is>
           <t>Bairan</t>
         </is>
       </c>
-      <c r="D2" t="inlineStr">
+      <c r="D2" s="0" t="inlineStr">
         <is>
           <t>Banjaare</t>
         </is>
       </c>
     </row>
     <row r="3">
-      <c r="A3" t="inlineStr">
+      <c r="A3" s="0" t="inlineStr">
         <is>
           <t>2026-04-11</t>
         </is>
       </c>
-      <c r="B3" t="n">
+      <c r="B3" s="0" t="n">
         <v>2</v>
       </c>
-      <c r="C3" t="inlineStr">
+      <c r="C3" s="0" t="inlineStr">
         <is>
           <t>Jaiye Sajana</t>
         </is>
       </c>
-      <c r="D3" t="inlineStr">
+      <c r="D3" s="0" t="inlineStr">
         <is>
           <t>Shashwat Sachdev</t>
         </is>
       </c>
     </row>
     <row r="4">
-      <c r="A4" t="inlineStr">
+      <c r="A4" s="0" t="inlineStr">
         <is>
           <t>2026-04-11</t>
         </is>
       </c>
-      <c r="B4" t="n">
+      <c r="B4" s="0" t="n">
         <v>3</v>
       </c>
-      <c r="C4" t="inlineStr">
+      <c r="C4" s="0" t="inlineStr">
         <is>
           <t>Gehra Hua</t>
         </is>
       </c>
-      <c r="D4" t="inlineStr">
+      <c r="D4" s="0" t="inlineStr">
         <is>
           <t>Shashwat Sachdev</t>
         </is>
       </c>
     </row>
     <row r="5">
-      <c r="A5" t="inlineStr">
+      <c r="A5" s="0" t="inlineStr">
         <is>
           <t>2026-04-11</t>
         </is>
       </c>
-      <c r="B5" t="n">
+      <c r="B5" s="0" t="n">
         <v>4</v>
       </c>
-      <c r="C5" t="inlineStr">
+      <c r="C5" s="0" t="inlineStr">
         <is>
           <t>Sheesha - Aakhya Mai Aakh Ghali Jo Bairan</t>
         </is>
       </c>
-      <c r="D5" t="inlineStr">
+      <c r="D5" s="0" t="inlineStr">
         <is>
           <t>Mitta Ror</t>
         </is>
       </c>
     </row>
     <row r="6">
-      <c r="A6" t="inlineStr">
+      <c r="A6" s="0" t="inlineStr">
         <is>
           <t>2026-04-11</t>
         </is>
       </c>
-      <c r="B6" t="n">
+      <c r="B6" s="0" t="n">
         <v>5</v>
       </c>
-      <c r="C6" t="inlineStr">
+      <c r="C6" s="0" t="inlineStr">
         <is>
           <t>Khat</t>
         </is>
       </c>
-      <c r="D6" t="inlineStr">
+      <c r="D6" s="0" t="inlineStr">
         <is>
           <t>Navjot Ahuja</t>
         </is>
       </c>
     </row>
     <row r="7">
-      <c r="A7" t="inlineStr">
+      <c r="A7" s="0" t="inlineStr">
         <is>
           <t>2026-04-11</t>
         </is>
       </c>
-      <c r="B7" t="n">
+      <c r="B7" s="0" t="n">
         <v>6</v>
       </c>
-      <c r="C7" t="inlineStr">
+      <c r="C7" s="0" t="inlineStr">
         <is>
           <t>Sahiba</t>
         </is>
       </c>
-      <c r="D7" t="inlineStr">
+      <c r="D7" s="0" t="inlineStr">
         <is>
           <t>Aditya Rikhari</t>
         </is>
       </c>
     </row>
     <row r="8">
-      <c r="A8" t="inlineStr">
+      <c r="A8" s="0" t="inlineStr">
         <is>
           <t>2026-04-11</t>
         </is>
       </c>
-      <c r="B8" t="n">
+      <c r="B8" s="0" t="n">
         <v>7</v>
       </c>
-      <c r="C8" t="inlineStr">
+      <c r="C8" s="0" t="inlineStr">
         <is>
           <t>Dooron Dooron</t>
         </is>
       </c>
-      <c r="D8" t="inlineStr">
+      <c r="D8" s="0" t="inlineStr">
         <is>
           <t>Paresh Pahuja</t>
         </is>
       </c>
     </row>
     <row r="9">
-      <c r="A9" t="inlineStr">
+      <c r="A9" s="0" t="inlineStr">
         <is>
           <t>2026-04-11</t>
         </is>
       </c>
-      <c r="B9" t="n">
+      <c r="B9" s="0" t="n">
         <v>8</v>
       </c>
-      <c r="C9" t="inlineStr">
+      <c r="C9" s="0" t="inlineStr">
         <is>
           <t>Dhurandhar The Revenge - Aari Aari</t>
         </is>
       </c>
-      <c r="D9" t="inlineStr">
+      <c r="D9" s="0" t="inlineStr">
         <is>
           <t>Shashwat Sachdev</t>
         </is>
       </c>
     </row>
     <row r="10">
-      <c r="A10" t="inlineStr">
+      <c r="A10" s="0" t="inlineStr">
         <is>
           <t>2026-04-11</t>
         </is>
       </c>
-      <c r="B10" t="n">
+      <c r="B10" s="0" t="n">
         <v>9</v>
       </c>
-      <c r="C10" t="inlineStr">
+      <c r="C10" s="0" t="inlineStr">
         <is>
           <t>Apna Bana Le</t>
         </is>
       </c>
-      <c r="D10" t="inlineStr">
+      <c r="D10" s="0" t="inlineStr">
         <is>
           <t>Sachin-Jigar</t>
         </is>
       </c>
     </row>
     <row r="11">
-      <c r="A11" t="inlineStr">
+      <c r="A11" s="0" t="inlineStr">
         <is>
           <t>2026-04-11</t>
         </is>
       </c>
-      <c r="B11" t="n">
+      <c r="B11" s="0" t="n">
         <v>10</v>
       </c>
-      <c r="C11" t="inlineStr">
+      <c r="C11" s="0" t="inlineStr">
         <is>
           <t>Sitaare</t>
         </is>
       </c>
-      <c r="D11" t="inlineStr">
+      <c r="D11" s="0" t="inlineStr">
         <is>
           <t>Arijit Singh</t>
         </is>
       </c>
     </row>
     <row r="12">
-      <c r="A12" t="inlineStr">
+      <c r="A12" s="0" t="inlineStr">
         <is>
           <t>2026-04-11</t>
         </is>
       </c>
-      <c r="B12" t="n">
+      <c r="B12" s="0" t="n">
         <v>11</v>
       </c>
-      <c r="C12" t="inlineStr">
+      <c r="C12" s="0" t="inlineStr">
         <is>
           <t>Samjhawan</t>
         </is>
       </c>
-      <c r="D12" t="inlineStr">
+      <c r="D12" s="0" t="inlineStr">
         <is>
           <t>Jawad Ahmad</t>
         </is>
       </c>
     </row>
     <row r="13">
-      <c r="A13" t="inlineStr">
+      <c r="A13" s="0" t="inlineStr">
         <is>
           <t>2026-04-11</t>
         </is>
       </c>
-      <c r="B13" t="n">
+      <c r="B13" s="0" t="n">
         <v>12</v>
       </c>
-      <c r="C13" t="inlineStr">
+      <c r="C13" s="0" t="inlineStr">
         <is>
           <t>Jaan Se Guzarte Hain</t>
         </is>
       </c>
-      <c r="D13" t="inlineStr">
+      <c r="D13" s="0" t="inlineStr">
         <is>
           <t>Shashwat Sachdev</t>
         </is>
       </c>
     </row>
     <row r="14">
-      <c r="A14" t="inlineStr">
+      <c r="A14" s="0" t="inlineStr">
         <is>
           <t>2026-04-11</t>
         </is>
       </c>
-      <c r="B14" t="n">
+      <c r="B14" s="0" t="n">
         <v>13</v>
       </c>
-      <c r="C14" t="inlineStr">
+      <c r="C14" s="0" t="inlineStr">
         <is>
           <t>Boyfriend</t>
         </is>
       </c>
-      <c r="D14" t="inlineStr">
+      <c r="D14" s="0" t="inlineStr">
         <is>
           <t>Karan Aujla</t>
         </is>
       </c>
     </row>
     <row r="15">
-      <c r="A15" t="inlineStr">
+      <c r="A15" s="0" t="inlineStr">
         <is>
           <t>2026-04-11</t>
         </is>
       </c>
-      <c r="B15" t="n">
+      <c r="B15" s="0" t="n">
         <v>14</v>
       </c>
-      <c r="C15" t="inlineStr">
+      <c r="C15" s="0" t="inlineStr">
         <is>
           <t>Pavazha Malli</t>
         </is>
       </c>
-      <c r="D15" t="inlineStr">
+      <c r="D15" s="0" t="inlineStr">
         <is>
           <t>Sai Abhyankkar</t>
         </is>
       </c>
     </row>
     <row r="16">
-      <c r="A16" t="inlineStr">
+      <c r="A16" s="0" t="inlineStr">
         <is>
           <t>2026-04-11</t>
         </is>
       </c>
-      <c r="B16" t="n">
+      <c r="B16" s="0" t="n">
         <v>15</v>
       </c>
-      <c r="C16" t="inlineStr">
+      <c r="C16" s="0" t="inlineStr">
         <is>
           <t>Finding Her</t>
         </is>
       </c>
-      <c r="D16" t="inlineStr">
+      <c r="D16" s="0" t="inlineStr">
         <is>
           <t>Kushagra</t>
         </is>
       </c>
     </row>
     <row r="17">
-      <c r="A17" t="inlineStr">
+      <c r="A17" s="0" t="inlineStr">
         <is>
           <t>2026-04-11</t>
         </is>
       </c>
-      <c r="B17" t="n">
+      <c r="B17" s="0" t="n">
         <v>16</v>
       </c>
-      <c r="C17" t="inlineStr">
+      <c r="C17" s="0" t="inlineStr">
         <is>
           <t>Arz Kiya Hai | Coke Studio Bharat</t>
         </is>
       </c>
-      <c r="D17" t="inlineStr">
+      <c r="D17" s="0" t="inlineStr">
         <is>
           <t>Anuv Jain</t>
         </is>
       </c>
     </row>
     <row r="18">
-      <c r="A18" t="inlineStr">
+      <c r="A18" s="0" t="inlineStr">
         <is>
           <t>2026-04-11</t>
         </is>
       </c>
-      <c r="B18" t="n">
+      <c r="B18" s="0" t="n">
         <v>17</v>
       </c>
-      <c r="C18" t="inlineStr">
+      <c r="C18" s="0" t="inlineStr">
         <is>
           <t>Shararat</t>
         </is>
       </c>
-      <c r="D18" t="inlineStr">
+      <c r="D18" s="0" t="inlineStr">
         <is>
           <t>Shashwat Sachdev</t>
         </is>
       </c>
     </row>
     <row r="19">
-      <c r="A19" t="inlineStr">
+      <c r="A19" s="0" t="inlineStr">
         <is>
           <t>2026-04-11</t>
         </is>
       </c>
-      <c r="B19" t="n">
+      <c r="B19" s="0" t="n">
         <v>18</v>
       </c>
-      <c r="C19" t="inlineStr">
+      <c r="C19" s="0" t="inlineStr">
         <is>
           <t>Ishq</t>
         </is>
       </c>
-      <c r="D19" t="inlineStr">
+      <c r="D19" s="0" t="inlineStr">
         <is>
           <t>Faheem Abdullah</t>
         </is>
       </c>
     </row>
     <row r="20">
-      <c r="A20" t="inlineStr">
+      <c r="A20" s="0" t="inlineStr">
         <is>
           <t>2026-04-11</t>
         </is>
       </c>
-      <c r="B20" t="n">
+      <c r="B20" s="0" t="n">
         <v>19</v>
       </c>
-      <c r="C20" t="inlineStr">
+      <c r="C20" s="0" t="inlineStr">
         <is>
           <t>Mann Mera</t>
         </is>
       </c>
-      <c r="D20" t="inlineStr">
+      <c r="D20" s="0" t="inlineStr">
         <is>
           <t>Gajendra Verma</t>
         </is>
       </c>
     </row>
     <row r="21">
-      <c r="A21" t="inlineStr">
+      <c r="A21" s="0" t="inlineStr">
         <is>
           <t>2026-04-11</t>
         </is>
       </c>
-      <c r="B21" t="n">
+      <c r="B21" s="0" t="n">
         <v>20</v>
       </c>
-      <c r="C21" t="inlineStr">
+      <c r="C21" s="0" t="inlineStr">
         <is>
           <t>Saiyaara</t>
         </is>
       </c>
-      <c r="D21" t="inlineStr">
+      <c r="D21" s="0" t="inlineStr">
         <is>
           <t>Tanishk Bagchi</t>
         </is>
       </c>
     </row>
     <row r="22">
-      <c r="A22" t="inlineStr">
+      <c r="A22" s="0" t="inlineStr">
         <is>
           <t>2026-04-11</t>
         </is>
       </c>
-      <c r="B22" t="n">
+      <c r="B22" s="0" t="n">
         <v>21</v>
       </c>
-      <c r="C22" t="inlineStr">
+      <c r="C22" s="0" t="inlineStr">
         <is>
           <t>For A Reason</t>
         </is>
       </c>
-      <c r="D22" t="inlineStr">
+      <c r="D22" s="0" t="inlineStr">
         <is>
           <t>Karan Aujla</t>
         </is>
       </c>
     </row>
     <row r="23">
-      <c r="A23" t="inlineStr">
+      <c r="A23" s="0" t="inlineStr">
         <is>
           <t>2026-04-11</t>
         </is>
       </c>
-      <c r="B23" t="n">
+      <c r="B23" s="0" t="n">
         <v>22</v>
       </c>
-      <c r="C23" t="inlineStr">
+      <c r="C23" s="0" t="inlineStr">
         <is>
           <t>Dhurandhar - Title Track</t>
         </is>
       </c>
-      <c r="D23" t="inlineStr">
+      <c r="D23" s="0" t="inlineStr">
         <is>
           <t>Shashwat Sachdev</t>
         </is>
       </c>
     </row>
     <row r="24">
-      <c r="A24" t="inlineStr">
+      <c r="A24" s="0" t="inlineStr">
         <is>
           <t>2026-04-11</t>
         </is>
       </c>
-      <c r="B24" t="n">
+      <c r="B24" s="0" t="n">
         <v>23</v>
       </c>
-      <c r="C24" t="inlineStr">
+      <c r="C24" s="0" t="inlineStr">
         <is>
           <t>Ishqa Ve</t>
         </is>
       </c>
-      <c r="D24" t="inlineStr">
+      <c r="D24" s="0" t="inlineStr">
         <is>
           <t>Zeeshan Ali</t>
         </is>
       </c>
     </row>
     <row r="25">
-      <c r="A25" t="inlineStr">
+      <c r="A25" s="0" t="inlineStr">
         <is>
           <t>2026-04-11</t>
         </is>
       </c>
-      <c r="B25" t="n">
+      <c r="B25" s="0" t="n">
         <v>24</v>
       </c>
-      <c r="C25" t="inlineStr">
+      <c r="C25" s="0" t="inlineStr">
         <is>
           <t>Bairi</t>
         </is>
       </c>
-      <c r="D25" t="inlineStr">
+      <c r="D25" s="0" t="inlineStr">
         <is>
           <t>Virat</t>
         </is>
       </c>
     </row>
     <row r="26">
-      <c r="A26" t="inlineStr">
+      <c r="A26" s="0" t="inlineStr">
         <is>
           <t>2026-04-11</t>
         </is>
       </c>
-      <c r="B26" t="n">
+      <c r="B26" s="0" t="n">
         <v>25</v>
       </c>
-      <c r="C26" t="inlineStr">
+      <c r="C26" s="0" t="inlineStr">
         <is>
           <t>Naal Nachna</t>
         </is>
       </c>
-      <c r="D26" t="inlineStr">
+      <c r="D26" s="0" t="inlineStr">
         <is>
           <t>Shashwat Sachdev</t>
         </is>
       </c>
     </row>
     <row r="27">
-      <c r="A27" t="inlineStr">
+      <c r="A27" s="0" t="inlineStr">
         <is>
           <t>2026-04-11</t>
         </is>
       </c>
-      <c r="B27" t="n">
+      <c r="B27" s="0" t="n">
         <v>26</v>
       </c>
-      <c r="C27" t="inlineStr">
+      <c r="C27" s="0" t="inlineStr">
         <is>
           <t>Tere Liye</t>
         </is>
       </c>
-      <c r="D27" t="inlineStr">
+      <c r="D27" s="0" t="inlineStr">
         <is>
           <t>Atif Aslam</t>
         </is>
       </c>
     </row>
     <row r="28">
-      <c r="A28" t="inlineStr">
+      <c r="A28" s="0" t="inlineStr">
         <is>
           <t>2026-04-11</t>
         </is>
       </c>
-      <c r="B28" t="n">
+      <c r="B28" s="0" t="n">
         <v>27</v>
       </c>
-      <c r="C28" t="inlineStr">
+      <c r="C28" s="0" t="inlineStr">
         <is>
           <t>Tum Ho Toh</t>
         </is>
       </c>
-      <c r="D28" t="inlineStr">
+      <c r="D28" s="0" t="inlineStr">
         <is>
           <t>Vishal Mishra</t>
         </is>
       </c>
     </row>
     <row r="29">
-      <c r="A29" t="inlineStr">
+      <c r="A29" s="0" t="inlineStr">
         <is>
           <t>2026-04-11</t>
         </is>
       </c>
-      <c r="B29" t="n">
+      <c r="B29" s="0" t="n">
         <v>28</v>
       </c>
-      <c r="C29" t="inlineStr">
+      <c r="C29" s="0" t="inlineStr">
         <is>
           <t>Jo Tum Mere Ho</t>
         </is>
       </c>
-      <c r="D29" t="inlineStr">
+      <c r="D29" s="0" t="inlineStr">
         <is>
           <t>Anuv Jain</t>
         </is>
       </c>
     </row>
     <row r="30">
-      <c r="A30" t="inlineStr">
+      <c r="A30" s="0" t="inlineStr">
         <is>
           <t>2026-04-11</t>
         </is>
       </c>
-      <c r="B30" t="n">
+      <c r="B30" s="0" t="n">
         <v>29</v>
       </c>
-      <c r="C30" t="inlineStr">
+      <c r="C30" s="0" t="inlineStr">
         <is>
           <t>Raanjhan</t>
         </is>
       </c>
-      <c r="D30" t="inlineStr">
+      <c r="D30" s="0" t="inlineStr">
         <is>
           <t>Sachet-Parampara</t>
         </is>
       </c>
     </row>
     <row r="31">
-      <c r="A31" t="inlineStr">
+      <c r="A31" s="0" t="inlineStr">
         <is>
           <t>2026-04-11</t>
         </is>
       </c>
-      <c r="B31" t="n">
+      <c r="B31" s="0" t="n">
         <v>30</v>
       </c>
-      <c r="C31" t="inlineStr">
+      <c r="C31" s="0" t="inlineStr">
         <is>
           <t>Deewaana Deewaana</t>
         </is>
       </c>
-      <c r="D31" t="inlineStr">
+      <c r="D31" s="0" t="inlineStr">
         <is>
           <t>A.R. Rahman</t>
         </is>
       </c>
     </row>
     <row r="32">
-      <c r="A32" t="inlineStr">
+      <c r="A32" s="0" t="inlineStr">
         <is>
           <t>2026-04-11</t>
         </is>
       </c>
-      <c r="B32" t="n">
+      <c r="B32" s="0" t="n">
         <v>31</v>
       </c>
-      <c r="C32" t="inlineStr">
+      <c r="C32" s="0" t="inlineStr">
         <is>
           <t>Darkhaast</t>
         </is>
       </c>
-      <c r="D32" t="inlineStr">
+      <c r="D32" s="0" t="inlineStr">
         <is>
           <t>Mithoon</t>
         </is>
       </c>
     </row>
     <row r="33">
-      <c r="A33" t="inlineStr">
+      <c r="A33" s="0" t="inlineStr">
         <is>
           <t>2026-04-11</t>
         </is>
       </c>
-      <c r="B33" t="n">
+      <c r="B33" s="0" t="n">
         <v>32</v>
       </c>
-      <c r="C33" t="inlineStr">
+      <c r="C33" s="0" t="inlineStr">
         <is>
           <t>Tere Bina</t>
         </is>
       </c>
-      <c r="D33" t="inlineStr">
+      <c r="D33" s="0" t="inlineStr">
         <is>
           <t>A.R. Rahman</t>
         </is>
       </c>
     </row>
     <row r="34">
-      <c r="A34" t="inlineStr">
+      <c r="A34" s="0" t="inlineStr">
         <is>
           <t>2026-04-11</t>
         </is>
       </c>
-      <c r="B34" t="n">
+      <c r="B34" s="0" t="n">
         <v>33</v>
       </c>
-      <c r="C34" t="inlineStr">
+      <c r="C34" s="0" t="inlineStr">
         <is>
           <t>Agar Tum Saath Ho</t>
         </is>
       </c>
-      <c r="D34" t="inlineStr">
+      <c r="D34" s="0" t="inlineStr">
         <is>
           <t>Alka Yagnik</t>
         </is>
       </c>
     </row>
     <row r="35">
-      <c r="A35" t="inlineStr">
+      <c r="A35" s="0" t="inlineStr">
         <is>
           <t>2026-04-11</t>
         </is>
       </c>
-      <c r="B35" t="n">
+      <c r="B35" s="0" t="n">
         <v>34</v>
       </c>
-      <c r="C35" t="inlineStr">
+      <c r="C35" s="0" t="inlineStr">
         <is>
           <t>Phir Se</t>
         </is>
       </c>
-      <c r="D35" t="inlineStr">
+      <c r="D35" s="0" t="inlineStr">
         <is>
           <t>Shashwat Sachdev</t>
         </is>
       </c>
     </row>
     <row r="36">
-      <c r="A36" t="inlineStr">
+      <c r="A36" s="0" t="inlineStr">
         <is>
           <t>2026-04-11</t>
         </is>
       </c>
-      <c r="B36" t="n">
+      <c r="B36" s="0" t="n">
         <v>35</v>
       </c>
-      <c r="C36" t="inlineStr">
+      <c r="C36" s="0" t="inlineStr">
         <is>
           <t>Lutt Le Gaya</t>
         </is>
       </c>
-      <c r="D36" t="inlineStr">
+      <c r="D36" s="0" t="inlineStr">
         <is>
           <t>Shashwat Sachdev</t>
         </is>
       </c>
     </row>
     <row r="37">
-      <c r="A37" t="inlineStr">
+      <c r="A37" s="0" t="inlineStr">
         <is>
           <t>2026-04-11</t>
         </is>
       </c>
-      <c r="B37" t="n">
+      <c r="B37" s="0" t="n">
         <v>36</v>
       </c>
-      <c r="C37" t="inlineStr">
+      <c r="C37" s="0" t="inlineStr">
         <is>
           <t>Teri Deewani</t>
         </is>
       </c>
-      <c r="D37" t="inlineStr">
+      <c r="D37" s="0" t="inlineStr">
         <is>
           <t>Kailash Kher</t>
         </is>
       </c>
     </row>
     <row r="38">
-      <c r="A38" t="inlineStr">
+      <c r="A38" s="0" t="inlineStr">
         <is>
           <t>2026-04-11</t>
         </is>
       </c>
-      <c r="B38" t="n">
+      <c r="B38" s="0" t="n">
         <v>37</v>
       </c>
-      <c r="C38" t="inlineStr">
+      <c r="C38" s="0" t="inlineStr">
         <is>
           <t>Haseen</t>
         </is>
       </c>
-      <c r="D38" t="inlineStr">
+      <c r="D38" s="0" t="inlineStr">
         <is>
           <t>Talwiinder</t>
         </is>
       </c>
     </row>
     <row r="39">
-      <c r="A39" t="inlineStr">
+      <c r="A39" s="0" t="inlineStr">
         <is>
           <t>2026-04-11</t>
         </is>
       </c>
-      <c r="B39" t="n">
+      <c r="B39" s="0" t="n">
         <v>38</v>
       </c>
-      <c r="C39" t="inlineStr">
+      <c r="C39" s="0" t="inlineStr">
         <is>
           <t>Ye Tune Kya Kiya</t>
         </is>
       </c>
-      <c r="D39" t="inlineStr">
+      <c r="D39" s="0" t="inlineStr">
         <is>
           <t>Pritam</t>
         </is>
       </c>
     </row>
     <row r="40">
-      <c r="A40" t="inlineStr">
+      <c r="A40" s="0" t="inlineStr">
         <is>
           <t>2026-04-11</t>
         </is>
       </c>
-      <c r="B40" t="n">
+      <c r="B40" s="0" t="n">
         <v>39</v>
       </c>
-      <c r="C40" t="inlineStr">
+      <c r="C40" s="0" t="inlineStr">
         <is>
           <t>Barbaad</t>
         </is>
       </c>
-      <c r="D40" t="inlineStr">
+      <c r="D40" s="0" t="inlineStr">
         <is>
           <t>The Rish</t>
         </is>
       </c>
     </row>
     <row r="41">
-      <c r="A41" t="inlineStr">
+      <c r="A41" s="0" t="inlineStr">
         <is>
           <t>2026-04-11</t>
         </is>
       </c>
-      <c r="B41" t="n">
+      <c r="B41" s="0" t="n">
         <v>40</v>
       </c>
-      <c r="C41" t="inlineStr">
+      <c r="C41" s="0" t="inlineStr">
         <is>
           <t>Ehsaas</t>
         </is>
       </c>
-      <c r="D41" t="inlineStr">
+      <c r="D41" s="0" t="inlineStr">
         <is>
           <t>Faheem Abdullah</t>
         </is>
       </c>
     </row>
     <row r="42">
-      <c r="A42" t="inlineStr">
+      <c r="A42" s="0" t="inlineStr">
         <is>
           <t>2026-04-11</t>
         </is>
       </c>
-      <c r="B42" t="n">
+      <c r="B42" s="0" t="n">
         <v>41</v>
       </c>
-      <c r="C42" t="inlineStr">
+      <c r="C42" s="0" t="inlineStr">
         <is>
           <t>Run Down The City - Monica</t>
         </is>
       </c>
-      <c r="D42" t="inlineStr">
+      <c r="D42" s="0" t="inlineStr">
         <is>
           <t>Shashwat Sachdev</t>
         </is>
       </c>
     </row>
     <row r="43">
-      <c r="A43" t="inlineStr">
+      <c r="A43" s="0" t="inlineStr">
         <is>
           <t>2026-04-11</t>
         </is>
       </c>
-      <c r="B43" t="n">
+      <c r="B43" s="0" t="n">
         <v>42</v>
       </c>
-      <c r="C43" t="inlineStr">
+      <c r="C43" s="0" t="inlineStr">
         <is>
           <t>Mast Magan</t>
         </is>
       </c>
-      <c r="D43" t="inlineStr">
+      <c r="D43" s="0" t="inlineStr">
         <is>
           <t>Arijit Singh</t>
         </is>
       </c>
     </row>
     <row r="44">
-      <c r="A44" t="inlineStr">
+      <c r="A44" s="0" t="inlineStr">
         <is>
           <t>2026-04-11</t>
         </is>
       </c>
-      <c r="B44" t="n">
+      <c r="B44" s="0" t="n">
         <v>43</v>
       </c>
-      <c r="C44" t="inlineStr">
+      <c r="C44" s="0" t="inlineStr">
         <is>
           <t>Thodi Si Daaru</t>
         </is>
       </c>
-      <c r="D44" t="inlineStr">
+      <c r="D44" s="0" t="inlineStr">
         <is>
           <t>AP Dhillon</t>
         </is>
       </c>
     </row>
     <row r="45">
-      <c r="A45" t="inlineStr">
+      <c r="A45" s="0" t="inlineStr">
         <is>
           <t>2026-04-11</t>
         </is>
       </c>
-      <c r="B45" t="n">
+      <c r="B45" s="0" t="n">
         <v>44</v>
       </c>
-      <c r="C45" t="inlineStr">
+      <c r="C45" s="0" t="inlineStr">
         <is>
           <t>Ishq Jalakar - Karvaan</t>
         </is>
       </c>
-      <c r="D45" t="inlineStr">
+      <c r="D45" s="0" t="inlineStr">
         <is>
           <t>Shashwat Sachdev</t>
         </is>
       </c>
     </row>
     <row r="46">
-      <c r="A46" t="inlineStr">
+      <c r="A46" s="0" t="inlineStr">
         <is>
           <t>2026-04-11</t>
         </is>
       </c>
-      <c r="B46" t="n">
+      <c r="B46" s="0" t="n">
         <v>45</v>
       </c>
-      <c r="C46" t="inlineStr">
+      <c r="C46" s="0" t="inlineStr">
         <is>
           <t>Mutta Kalakki</t>
         </is>
       </c>
-      <c r="D46" t="inlineStr">
+      <c r="D46" s="0" t="inlineStr">
         <is>
           <t>G. V. Prakash</t>
         </is>
       </c>
     </row>
     <row r="47">
-      <c r="A47" t="inlineStr">
+      <c r="A47" s="0" t="inlineStr">
         <is>
           <t>2026-04-11</t>
         </is>
       </c>
-      <c r="B47" t="n">
+      <c r="B47" s="0" t="n">
         <v>46</v>
       </c>
-      <c r="C47" t="inlineStr">
+      <c r="C47" s="0" t="inlineStr">
         <is>
           <t>Zaalima</t>
         </is>
       </c>
-      <c r="D47" t="inlineStr">
+      <c r="D47" s="0" t="inlineStr">
         <is>
           <t>Arijit Singh</t>
         </is>
       </c>
     </row>
     <row r="48">
-      <c r="A48" t="inlineStr">
+      <c r="A48" s="0" t="inlineStr">
         <is>
           <t>2026-04-11</t>
         </is>
       </c>
-      <c r="B48" t="n">
+      <c r="B48" s="0" t="n">
         <v>47</v>
       </c>
-      <c r="C48" t="inlineStr">
+      <c r="C48" s="0" t="inlineStr">
         <is>
           <t>Not Guilty</t>
         </is>
       </c>
-      <c r="D48" t="inlineStr">
+      <c r="D48" s="0" t="inlineStr">
         <is>
           <t>Dhanda Nyoliwala</t>
         </is>
       </c>
     </row>
     <row r="49">
-      <c r="A49" t="inlineStr">
+      <c r="A49" s="0" t="inlineStr">
         <is>
           <t>2026-04-11</t>
         </is>
       </c>
-      <c r="B49" t="n">
+      <c r="B49" s="0" t="n">
         <v>48</v>
       </c>
-      <c r="C49" t="inlineStr">
+      <c r="C49" s="0" t="inlineStr">
         <is>
           <t>Jogi</t>
         </is>
       </c>
-      <c r="D49" t="inlineStr">
+      <c r="D49" s="0" t="inlineStr">
         <is>
           <t>thiarajxtt</t>
         </is>
       </c>
     </row>
     <row r="50">
-      <c r="A50" t="inlineStr">
+      <c r="A50" s="0" t="inlineStr">
         <is>
           <t>2026-04-11</t>
         </is>
       </c>
-      <c r="B50" t="n">
+      <c r="B50" s="0" t="n">
         <v>49</v>
       </c>
-      <c r="C50" t="inlineStr">
+      <c r="C50" s="0" t="inlineStr">
         <is>
           <t>Mann Mera - Original Version</t>
         </is>
       </c>
-      <c r="D50" t="inlineStr">
+      <c r="D50" s="0" t="inlineStr">
         <is>
           <t>Gajendra Verma</t>
         </is>
       </c>
     </row>
     <row r="51">
-      <c r="A51" t="inlineStr">
+      <c r="A51" s="0" t="inlineStr">
         <is>
           <t>2026-04-11</t>
         </is>
       </c>
-      <c r="B51" t="n">
+      <c r="B51" s="0" t="n">
         <v>50</v>
       </c>
-      <c r="C51" t="inlineStr">
+      <c r="C51" s="0" t="inlineStr">
         <is>
           <t>Humdard</t>
         </is>
       </c>
-      <c r="D51" t="inlineStr">
+      <c r="D51" s="0" t="inlineStr">
         <is>
           <t>Arijit Singh</t>
         </is>
@@ -25332,6 +25333,1042 @@
 </worksheet>
 </file>
 
+<file path=xl/worksheets/sheet30.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:D51"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="24" t="inlineStr">
+        <is>
+          <t>Date</t>
+        </is>
+      </c>
+      <c r="B1" s="24" t="inlineStr">
+        <is>
+          <t>Rank</t>
+        </is>
+      </c>
+      <c r="C1" s="24" t="inlineStr">
+        <is>
+          <t>Song</t>
+        </is>
+      </c>
+      <c r="D1" s="24" t="inlineStr">
+        <is>
+          <t>Artist</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>2026-04-12</t>
+        </is>
+      </c>
+      <c r="B2" t="n">
+        <v>1</v>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>Bairan</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>Banjaare</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>2026-04-12</t>
+        </is>
+      </c>
+      <c r="B3" t="n">
+        <v>2</v>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>Gehra Hua</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>Shashwat Sachdev</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>2026-04-12</t>
+        </is>
+      </c>
+      <c r="B4" t="n">
+        <v>3</v>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>Jaiye Sajana</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>Shashwat Sachdev</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>2026-04-12</t>
+        </is>
+      </c>
+      <c r="B5" t="n">
+        <v>4</v>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>Sheesha - Aakhya Mai Aakh Ghali Jo Bairan</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>Mitta Ror</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>2026-04-12</t>
+        </is>
+      </c>
+      <c r="B6" t="n">
+        <v>5</v>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>Khat</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>Navjot Ahuja</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>2026-04-12</t>
+        </is>
+      </c>
+      <c r="B7" t="n">
+        <v>6</v>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>Dooron Dooron</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>Paresh Pahuja</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>2026-04-12</t>
+        </is>
+      </c>
+      <c r="B8" t="n">
+        <v>7</v>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>Sahiba</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>Aditya Rikhari</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>2026-04-12</t>
+        </is>
+      </c>
+      <c r="B9" t="n">
+        <v>8</v>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>Dhurandhar The Revenge - Aari Aari</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>Shashwat Sachdev</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>2026-04-12</t>
+        </is>
+      </c>
+      <c r="B10" t="n">
+        <v>9</v>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>Sitaare</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>Arijit Singh</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>2026-04-12</t>
+        </is>
+      </c>
+      <c r="B11" t="n">
+        <v>10</v>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>Samjhawan</t>
+        </is>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>Jawad Ahmad</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>2026-04-12</t>
+        </is>
+      </c>
+      <c r="B12" t="n">
+        <v>11</v>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>Apna Bana Le</t>
+        </is>
+      </c>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>Sachin-Jigar</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>2026-04-12</t>
+        </is>
+      </c>
+      <c r="B13" t="n">
+        <v>12</v>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>Finding Her</t>
+        </is>
+      </c>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t>Kushagra</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>2026-04-12</t>
+        </is>
+      </c>
+      <c r="B14" t="n">
+        <v>13</v>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>Pavazha Malli</t>
+        </is>
+      </c>
+      <c r="D14" t="inlineStr">
+        <is>
+          <t>Sai Abhyankkar</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>2026-04-12</t>
+        </is>
+      </c>
+      <c r="B15" t="n">
+        <v>14</v>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>Shararat</t>
+        </is>
+      </c>
+      <c r="D15" t="inlineStr">
+        <is>
+          <t>Shashwat Sachdev</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>2026-04-12</t>
+        </is>
+      </c>
+      <c r="B16" t="n">
+        <v>15</v>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>Jaan Se Guzarte Hain</t>
+        </is>
+      </c>
+      <c r="D16" t="inlineStr">
+        <is>
+          <t>Shashwat Sachdev</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>2026-04-12</t>
+        </is>
+      </c>
+      <c r="B17" t="n">
+        <v>16</v>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>Boyfriend</t>
+        </is>
+      </c>
+      <c r="D17" t="inlineStr">
+        <is>
+          <t>Karan Aujla</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>2026-04-12</t>
+        </is>
+      </c>
+      <c r="B18" t="n">
+        <v>17</v>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>Arz Kiya Hai | Coke Studio Bharat</t>
+        </is>
+      </c>
+      <c r="D18" t="inlineStr">
+        <is>
+          <t>Anuv Jain</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>2026-04-12</t>
+        </is>
+      </c>
+      <c r="B19" t="n">
+        <v>18</v>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>Mann Mera</t>
+        </is>
+      </c>
+      <c r="D19" t="inlineStr">
+        <is>
+          <t>Gajendra Verma</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>2026-04-12</t>
+        </is>
+      </c>
+      <c r="B20" t="n">
+        <v>19</v>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>Ishq</t>
+        </is>
+      </c>
+      <c r="D20" t="inlineStr">
+        <is>
+          <t>Faheem Abdullah</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>2026-04-12</t>
+        </is>
+      </c>
+      <c r="B21" t="n">
+        <v>20</v>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>Saiyaara</t>
+        </is>
+      </c>
+      <c r="D21" t="inlineStr">
+        <is>
+          <t>Tanishk Bagchi</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>2026-04-12</t>
+        </is>
+      </c>
+      <c r="B22" t="n">
+        <v>21</v>
+      </c>
+      <c r="C22" t="inlineStr">
+        <is>
+          <t>Bairi</t>
+        </is>
+      </c>
+      <c r="D22" t="inlineStr">
+        <is>
+          <t>Virat</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>2026-04-12</t>
+        </is>
+      </c>
+      <c r="B23" t="n">
+        <v>22</v>
+      </c>
+      <c r="C23" t="inlineStr">
+        <is>
+          <t>For A Reason</t>
+        </is>
+      </c>
+      <c r="D23" t="inlineStr">
+        <is>
+          <t>Karan Aujla</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>2026-04-12</t>
+        </is>
+      </c>
+      <c r="B24" t="n">
+        <v>23</v>
+      </c>
+      <c r="C24" t="inlineStr">
+        <is>
+          <t>Darkhaast</t>
+        </is>
+      </c>
+      <c r="D24" t="inlineStr">
+        <is>
+          <t>Mithoon</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>2026-04-12</t>
+        </is>
+      </c>
+      <c r="B25" t="n">
+        <v>24</v>
+      </c>
+      <c r="C25" t="inlineStr">
+        <is>
+          <t>Naal Nachna</t>
+        </is>
+      </c>
+      <c r="D25" t="inlineStr">
+        <is>
+          <t>Shashwat Sachdev</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>2026-04-12</t>
+        </is>
+      </c>
+      <c r="B26" t="n">
+        <v>25</v>
+      </c>
+      <c r="C26" t="inlineStr">
+        <is>
+          <t>Tum Ho Toh</t>
+        </is>
+      </c>
+      <c r="D26" t="inlineStr">
+        <is>
+          <t>Vishal Mishra</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>2026-04-12</t>
+        </is>
+      </c>
+      <c r="B27" t="n">
+        <v>26</v>
+      </c>
+      <c r="C27" t="inlineStr">
+        <is>
+          <t>Dhurandhar - Title Track</t>
+        </is>
+      </c>
+      <c r="D27" t="inlineStr">
+        <is>
+          <t>Shashwat Sachdev</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>2026-04-12</t>
+        </is>
+      </c>
+      <c r="B28" t="n">
+        <v>27</v>
+      </c>
+      <c r="C28" t="inlineStr">
+        <is>
+          <t>Ishqa Ve</t>
+        </is>
+      </c>
+      <c r="D28" t="inlineStr">
+        <is>
+          <t>Zeeshan Ali</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>2026-04-12</t>
+        </is>
+      </c>
+      <c r="B29" t="n">
+        <v>28</v>
+      </c>
+      <c r="C29" t="inlineStr">
+        <is>
+          <t>Tere Liye</t>
+        </is>
+      </c>
+      <c r="D29" t="inlineStr">
+        <is>
+          <t>Atif Aslam</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>2026-04-12</t>
+        </is>
+      </c>
+      <c r="B30" t="n">
+        <v>29</v>
+      </c>
+      <c r="C30" t="inlineStr">
+        <is>
+          <t>Raanjhan</t>
+        </is>
+      </c>
+      <c r="D30" t="inlineStr">
+        <is>
+          <t>Sachet-Parampara</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>2026-04-12</t>
+        </is>
+      </c>
+      <c r="B31" t="n">
+        <v>30</v>
+      </c>
+      <c r="C31" t="inlineStr">
+        <is>
+          <t>Deewaana Deewaana</t>
+        </is>
+      </c>
+      <c r="D31" t="inlineStr">
+        <is>
+          <t>A.R. Rahman</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="inlineStr">
+        <is>
+          <t>2026-04-12</t>
+        </is>
+      </c>
+      <c r="B32" t="n">
+        <v>31</v>
+      </c>
+      <c r="C32" t="inlineStr">
+        <is>
+          <t>Tere Bina</t>
+        </is>
+      </c>
+      <c r="D32" t="inlineStr">
+        <is>
+          <t>A.R. Rahman</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="inlineStr">
+        <is>
+          <t>2026-04-12</t>
+        </is>
+      </c>
+      <c r="B33" t="n">
+        <v>32</v>
+      </c>
+      <c r="C33" t="inlineStr">
+        <is>
+          <t>Jo Tum Mere Ho</t>
+        </is>
+      </c>
+      <c r="D33" t="inlineStr">
+        <is>
+          <t>Anuv Jain</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="inlineStr">
+        <is>
+          <t>2026-04-12</t>
+        </is>
+      </c>
+      <c r="B34" t="n">
+        <v>33</v>
+      </c>
+      <c r="C34" t="inlineStr">
+        <is>
+          <t>Agar Tum Saath Ho</t>
+        </is>
+      </c>
+      <c r="D34" t="inlineStr">
+        <is>
+          <t>Alka Yagnik</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="inlineStr">
+        <is>
+          <t>2026-04-12</t>
+        </is>
+      </c>
+      <c r="B35" t="n">
+        <v>34</v>
+      </c>
+      <c r="C35" t="inlineStr">
+        <is>
+          <t>Lutt Le Gaya</t>
+        </is>
+      </c>
+      <c r="D35" t="inlineStr">
+        <is>
+          <t>Shashwat Sachdev</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="inlineStr">
+        <is>
+          <t>2026-04-12</t>
+        </is>
+      </c>
+      <c r="B36" t="n">
+        <v>35</v>
+      </c>
+      <c r="C36" t="inlineStr">
+        <is>
+          <t>Teri Deewani</t>
+        </is>
+      </c>
+      <c r="D36" t="inlineStr">
+        <is>
+          <t>Kailash Kher</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="inlineStr">
+        <is>
+          <t>2026-04-12</t>
+        </is>
+      </c>
+      <c r="B37" t="n">
+        <v>36</v>
+      </c>
+      <c r="C37" t="inlineStr">
+        <is>
+          <t>Phir Se</t>
+        </is>
+      </c>
+      <c r="D37" t="inlineStr">
+        <is>
+          <t>Shashwat Sachdev</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="inlineStr">
+        <is>
+          <t>2026-04-12</t>
+        </is>
+      </c>
+      <c r="B38" t="n">
+        <v>37</v>
+      </c>
+      <c r="C38" t="inlineStr">
+        <is>
+          <t>Ehsaas</t>
+        </is>
+      </c>
+      <c r="D38" t="inlineStr">
+        <is>
+          <t>Faheem Abdullah</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="inlineStr">
+        <is>
+          <t>2026-04-12</t>
+        </is>
+      </c>
+      <c r="B39" t="n">
+        <v>38</v>
+      </c>
+      <c r="C39" t="inlineStr">
+        <is>
+          <t>Ye Tune Kya Kiya</t>
+        </is>
+      </c>
+      <c r="D39" t="inlineStr">
+        <is>
+          <t>Pritam</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" t="inlineStr">
+        <is>
+          <t>2026-04-12</t>
+        </is>
+      </c>
+      <c r="B40" t="n">
+        <v>39</v>
+      </c>
+      <c r="C40" t="inlineStr">
+        <is>
+          <t>Haseen</t>
+        </is>
+      </c>
+      <c r="D40" t="inlineStr">
+        <is>
+          <t>Talwiinder</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" t="inlineStr">
+        <is>
+          <t>2026-04-12</t>
+        </is>
+      </c>
+      <c r="B41" t="n">
+        <v>40</v>
+      </c>
+      <c r="C41" t="inlineStr">
+        <is>
+          <t>Run Down The City - Monica</t>
+        </is>
+      </c>
+      <c r="D41" t="inlineStr">
+        <is>
+          <t>Shashwat Sachdev</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" t="inlineStr">
+        <is>
+          <t>2026-04-12</t>
+        </is>
+      </c>
+      <c r="B42" t="n">
+        <v>41</v>
+      </c>
+      <c r="C42" t="inlineStr">
+        <is>
+          <t>Barbaad</t>
+        </is>
+      </c>
+      <c r="D42" t="inlineStr">
+        <is>
+          <t>The Rish</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" t="inlineStr">
+        <is>
+          <t>2026-04-12</t>
+        </is>
+      </c>
+      <c r="B43" t="n">
+        <v>42</v>
+      </c>
+      <c r="C43" t="inlineStr">
+        <is>
+          <t>Mutta Kalakki</t>
+        </is>
+      </c>
+      <c r="D43" t="inlineStr">
+        <is>
+          <t>G. V. Prakash</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" t="inlineStr">
+        <is>
+          <t>2026-04-12</t>
+        </is>
+      </c>
+      <c r="B44" t="n">
+        <v>43</v>
+      </c>
+      <c r="C44" t="inlineStr">
+        <is>
+          <t>Mast Magan</t>
+        </is>
+      </c>
+      <c r="D44" t="inlineStr">
+        <is>
+          <t>Arijit Singh</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" t="inlineStr">
+        <is>
+          <t>2026-04-12</t>
+        </is>
+      </c>
+      <c r="B45" t="n">
+        <v>44</v>
+      </c>
+      <c r="C45" t="inlineStr">
+        <is>
+          <t>Zaalima</t>
+        </is>
+      </c>
+      <c r="D45" t="inlineStr">
+        <is>
+          <t>Arijit Singh</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" t="inlineStr">
+        <is>
+          <t>2026-04-12</t>
+        </is>
+      </c>
+      <c r="B46" t="n">
+        <v>45</v>
+      </c>
+      <c r="C46" t="inlineStr">
+        <is>
+          <t>Thodi Si Daaru</t>
+        </is>
+      </c>
+      <c r="D46" t="inlineStr">
+        <is>
+          <t>AP Dhillon</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" t="inlineStr">
+        <is>
+          <t>2026-04-12</t>
+        </is>
+      </c>
+      <c r="B47" t="n">
+        <v>46</v>
+      </c>
+      <c r="C47" t="inlineStr">
+        <is>
+          <t>Ishq Jalakar - Karvaan</t>
+        </is>
+      </c>
+      <c r="D47" t="inlineStr">
+        <is>
+          <t>Shashwat Sachdev</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" t="inlineStr">
+        <is>
+          <t>2026-04-12</t>
+        </is>
+      </c>
+      <c r="B48" t="n">
+        <v>47</v>
+      </c>
+      <c r="C48" t="inlineStr">
+        <is>
+          <t>Humdard</t>
+        </is>
+      </c>
+      <c r="D48" t="inlineStr">
+        <is>
+          <t>Arijit Singh</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" t="inlineStr">
+        <is>
+          <t>2026-04-12</t>
+        </is>
+      </c>
+      <c r="B49" t="n">
+        <v>48</v>
+      </c>
+      <c r="C49" t="inlineStr">
+        <is>
+          <t>Mann Mera - Original Version</t>
+        </is>
+      </c>
+      <c r="D49" t="inlineStr">
+        <is>
+          <t>Gajendra Verma</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" t="inlineStr">
+        <is>
+          <t>2026-04-12</t>
+        </is>
+      </c>
+      <c r="B50" t="n">
+        <v>49</v>
+      </c>
+      <c r="C50" t="inlineStr">
+        <is>
+          <t>Jogi</t>
+        </is>
+      </c>
+      <c r="D50" t="inlineStr">
+        <is>
+          <t>thiarajxtt</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" t="inlineStr">
+        <is>
+          <t>2026-04-12</t>
+        </is>
+      </c>
+      <c r="B51" t="n">
+        <v>50</v>
+      </c>
+      <c r="C51" t="inlineStr">
+        <is>
+          <t>Aaya Sher</t>
+        </is>
+      </c>
+      <c r="D51" t="inlineStr">
+        <is>
+          <t>Anirudh Ravichander</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>

</xml_diff>

<commit_message>
got the data for 13th and 14th April, got the predictions for 15th April
</commit_message>
<xml_diff>
--- a/Probability Project.xlsx
+++ b/Probability Project.xlsx
@@ -33,6 +33,8 @@
     <sheet name="AUTO_20260410" sheetId="28" state="visible" r:id="rId28"/>
     <sheet name="AUTO_20260411" sheetId="29" state="visible" r:id="rId29"/>
     <sheet name="AUTO_20260412" sheetId="30" state="visible" r:id="rId30"/>
+    <sheet name="AUTO_20260414" sheetId="31" state="visible" r:id="rId31"/>
+    <sheet name="AUTO_20260413" sheetId="32" state="visible" r:id="rId32"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -21221,1000 +21223,1000 @@
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="0" t="inlineStr">
+      <c r="A2" t="inlineStr">
         <is>
           <t>2026-04-08</t>
         </is>
       </c>
-      <c r="B2" s="0" t="n">
+      <c r="B2" t="n">
         <v>1</v>
       </c>
-      <c r="C2" s="0" t="inlineStr">
+      <c r="C2" t="inlineStr">
         <is>
           <t>Bairan</t>
         </is>
       </c>
-      <c r="D2" s="0" t="inlineStr">
+      <c r="D2" t="inlineStr">
         <is>
           <t>Banjaare</t>
         </is>
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="0" t="inlineStr">
+      <c r="A3" t="inlineStr">
         <is>
           <t>2026-04-08</t>
         </is>
       </c>
-      <c r="B3" s="0" t="n">
+      <c r="B3" t="n">
         <v>2</v>
       </c>
-      <c r="C3" s="0" t="inlineStr">
+      <c r="C3" t="inlineStr">
         <is>
           <t>Jaiye Sajana</t>
         </is>
       </c>
-      <c r="D3" s="0" t="inlineStr">
+      <c r="D3" t="inlineStr">
         <is>
           <t>Shashwat Sachdev</t>
         </is>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="0" t="inlineStr">
+      <c r="A4" t="inlineStr">
         <is>
           <t>2026-04-08</t>
         </is>
       </c>
-      <c r="B4" s="0" t="n">
+      <c r="B4" t="n">
         <v>3</v>
       </c>
-      <c r="C4" s="0" t="inlineStr">
+      <c r="C4" t="inlineStr">
         <is>
           <t>Gehra Hua</t>
         </is>
       </c>
-      <c r="D4" s="0" t="inlineStr">
+      <c r="D4" t="inlineStr">
         <is>
           <t>Shashwat Sachdev</t>
         </is>
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="0" t="inlineStr">
+      <c r="A5" t="inlineStr">
         <is>
           <t>2026-04-08</t>
         </is>
       </c>
-      <c r="B5" s="0" t="n">
+      <c r="B5" t="n">
         <v>4</v>
       </c>
-      <c r="C5" s="0" t="inlineStr">
+      <c r="C5" t="inlineStr">
         <is>
           <t>Sheesha - Aakhya Mai Aakh Ghali Jo Bairan</t>
         </is>
       </c>
-      <c r="D5" s="0" t="inlineStr">
+      <c r="D5" t="inlineStr">
         <is>
           <t>Mitta Ror</t>
         </is>
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="0" t="inlineStr">
+      <c r="A6" t="inlineStr">
         <is>
           <t>2026-04-08</t>
         </is>
       </c>
-      <c r="B6" s="0" t="n">
+      <c r="B6" t="n">
         <v>5</v>
       </c>
-      <c r="C6" s="0" t="inlineStr">
+      <c r="C6" t="inlineStr">
         <is>
           <t>Khat</t>
         </is>
       </c>
-      <c r="D6" s="0" t="inlineStr">
+      <c r="D6" t="inlineStr">
         <is>
           <t>Navjot Ahuja</t>
         </is>
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="0" t="inlineStr">
+      <c r="A7" t="inlineStr">
         <is>
           <t>2026-04-08</t>
         </is>
       </c>
-      <c r="B7" s="0" t="n">
+      <c r="B7" t="n">
         <v>6</v>
       </c>
-      <c r="C7" s="0" t="inlineStr">
+      <c r="C7" t="inlineStr">
         <is>
           <t>Dhurandhar The Revenge - Aari Aari</t>
         </is>
       </c>
-      <c r="D7" s="0" t="inlineStr">
+      <c r="D7" t="inlineStr">
         <is>
           <t>Shashwat Sachdev</t>
         </is>
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="0" t="inlineStr">
+      <c r="A8" t="inlineStr">
         <is>
           <t>2026-04-08</t>
         </is>
       </c>
-      <c r="B8" s="0" t="n">
+      <c r="B8" t="n">
         <v>7</v>
       </c>
-      <c r="C8" s="0" t="inlineStr">
+      <c r="C8" t="inlineStr">
         <is>
           <t>Dooron Dooron</t>
         </is>
       </c>
-      <c r="D8" s="0" t="inlineStr">
+      <c r="D8" t="inlineStr">
         <is>
           <t>Paresh Pahuja</t>
         </is>
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="0" t="inlineStr">
+      <c r="A9" t="inlineStr">
         <is>
           <t>2026-04-08</t>
         </is>
       </c>
-      <c r="B9" s="0" t="n">
+      <c r="B9" t="n">
         <v>8</v>
       </c>
-      <c r="C9" s="0" t="inlineStr">
+      <c r="C9" t="inlineStr">
         <is>
           <t>Apna Bana Le</t>
         </is>
       </c>
-      <c r="D9" s="0" t="inlineStr">
+      <c r="D9" t="inlineStr">
         <is>
           <t>Sachin-Jigar</t>
         </is>
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="0" t="inlineStr">
+      <c r="A10" t="inlineStr">
         <is>
           <t>2026-04-08</t>
         </is>
       </c>
-      <c r="B10" s="0" t="n">
+      <c r="B10" t="n">
         <v>9</v>
       </c>
-      <c r="C10" s="0" t="inlineStr">
+      <c r="C10" t="inlineStr">
         <is>
           <t>Sahiba</t>
         </is>
       </c>
-      <c r="D10" s="0" t="inlineStr">
+      <c r="D10" t="inlineStr">
         <is>
           <t>Aditya Rikhari</t>
         </is>
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="0" t="inlineStr">
+      <c r="A11" t="inlineStr">
         <is>
           <t>2026-04-08</t>
         </is>
       </c>
-      <c r="B11" s="0" t="n">
+      <c r="B11" t="n">
         <v>10</v>
       </c>
-      <c r="C11" s="0" t="inlineStr">
+      <c r="C11" t="inlineStr">
         <is>
           <t>Sitaare</t>
         </is>
       </c>
-      <c r="D11" s="0" t="inlineStr">
+      <c r="D11" t="inlineStr">
         <is>
           <t>Arijit Singh</t>
         </is>
       </c>
     </row>
     <row r="12">
-      <c r="A12" s="0" t="inlineStr">
+      <c r="A12" t="inlineStr">
         <is>
           <t>2026-04-08</t>
         </is>
       </c>
-      <c r="B12" s="0" t="n">
+      <c r="B12" t="n">
         <v>11</v>
       </c>
-      <c r="C12" s="0" t="inlineStr">
+      <c r="C12" t="inlineStr">
         <is>
           <t>Samjhawan</t>
         </is>
       </c>
-      <c r="D12" s="0" t="inlineStr">
+      <c r="D12" t="inlineStr">
         <is>
           <t>Jawad Ahmad</t>
         </is>
       </c>
     </row>
     <row r="13">
-      <c r="A13" s="0" t="inlineStr">
+      <c r="A13" t="inlineStr">
         <is>
           <t>2026-04-08</t>
         </is>
       </c>
-      <c r="B13" s="0" t="n">
+      <c r="B13" t="n">
         <v>12</v>
       </c>
-      <c r="C13" s="0" t="inlineStr">
+      <c r="C13" t="inlineStr">
         <is>
           <t>Jaan Se Guzarte Hain</t>
         </is>
       </c>
-      <c r="D13" s="0" t="inlineStr">
+      <c r="D13" t="inlineStr">
         <is>
           <t>Shashwat Sachdev</t>
         </is>
       </c>
     </row>
     <row r="14">
-      <c r="A14" s="0" t="inlineStr">
+      <c r="A14" t="inlineStr">
         <is>
           <t>2026-04-08</t>
         </is>
       </c>
-      <c r="B14" s="0" t="n">
+      <c r="B14" t="n">
         <v>13</v>
       </c>
-      <c r="C14" s="0" t="inlineStr">
+      <c r="C14" t="inlineStr">
         <is>
           <t>Finding Her</t>
         </is>
       </c>
-      <c r="D14" s="0" t="inlineStr">
+      <c r="D14" t="inlineStr">
         <is>
           <t>Kushagra</t>
         </is>
       </c>
     </row>
     <row r="15">
-      <c r="A15" s="0" t="inlineStr">
+      <c r="A15" t="inlineStr">
         <is>
           <t>2026-04-08</t>
         </is>
       </c>
-      <c r="B15" s="0" t="n">
+      <c r="B15" t="n">
         <v>14</v>
       </c>
-      <c r="C15" s="0" t="inlineStr">
+      <c r="C15" t="inlineStr">
         <is>
           <t>Boyfriend</t>
         </is>
       </c>
-      <c r="D15" s="0" t="inlineStr">
+      <c r="D15" t="inlineStr">
         <is>
           <t>Karan Aujla</t>
         </is>
       </c>
     </row>
     <row r="16">
-      <c r="A16" s="0" t="inlineStr">
+      <c r="A16" t="inlineStr">
         <is>
           <t>2026-04-08</t>
         </is>
       </c>
-      <c r="B16" s="0" t="n">
+      <c r="B16" t="n">
         <v>15</v>
       </c>
-      <c r="C16" s="0" t="inlineStr">
+      <c r="C16" t="inlineStr">
         <is>
           <t>Pavazha Malli</t>
         </is>
       </c>
-      <c r="D16" s="0" t="inlineStr">
+      <c r="D16" t="inlineStr">
         <is>
           <t>Sai Abhyankkar</t>
         </is>
       </c>
     </row>
     <row r="17">
-      <c r="A17" s="0" t="inlineStr">
+      <c r="A17" t="inlineStr">
         <is>
           <t>2026-04-08</t>
         </is>
       </c>
-      <c r="B17" s="0" t="n">
+      <c r="B17" t="n">
         <v>16</v>
       </c>
-      <c r="C17" s="0" t="inlineStr">
+      <c r="C17" t="inlineStr">
         <is>
           <t>Arz Kiya Hai | Coke Studio Bharat</t>
         </is>
       </c>
-      <c r="D17" s="0" t="inlineStr">
+      <c r="D17" t="inlineStr">
         <is>
           <t>Anuv Jain</t>
         </is>
       </c>
     </row>
     <row r="18">
-      <c r="A18" s="0" t="inlineStr">
+      <c r="A18" t="inlineStr">
         <is>
           <t>2026-04-08</t>
         </is>
       </c>
-      <c r="B18" s="0" t="n">
+      <c r="B18" t="n">
         <v>17</v>
       </c>
-      <c r="C18" s="0" t="inlineStr">
+      <c r="C18" t="inlineStr">
         <is>
           <t>Shararat</t>
         </is>
       </c>
-      <c r="D18" s="0" t="inlineStr">
+      <c r="D18" t="inlineStr">
         <is>
           <t>Shashwat Sachdev</t>
         </is>
       </c>
     </row>
     <row r="19">
-      <c r="A19" s="0" t="inlineStr">
+      <c r="A19" t="inlineStr">
         <is>
           <t>2026-04-08</t>
         </is>
       </c>
-      <c r="B19" s="0" t="n">
+      <c r="B19" t="n">
         <v>18</v>
       </c>
-      <c r="C19" s="0" t="inlineStr">
+      <c r="C19" t="inlineStr">
         <is>
           <t>Ishq</t>
         </is>
       </c>
-      <c r="D19" s="0" t="inlineStr">
+      <c r="D19" t="inlineStr">
         <is>
           <t>Faheem Abdullah</t>
         </is>
       </c>
     </row>
     <row r="20">
-      <c r="A20" s="0" t="inlineStr">
+      <c r="A20" t="inlineStr">
         <is>
           <t>2026-04-08</t>
         </is>
       </c>
-      <c r="B20" s="0" t="n">
+      <c r="B20" t="n">
         <v>19</v>
       </c>
-      <c r="C20" s="0" t="inlineStr">
+      <c r="C20" t="inlineStr">
         <is>
           <t>Mann Mera</t>
         </is>
       </c>
-      <c r="D20" s="0" t="inlineStr">
+      <c r="D20" t="inlineStr">
         <is>
           <t>Gajendra Verma</t>
         </is>
       </c>
     </row>
     <row r="21">
-      <c r="A21" s="0" t="inlineStr">
+      <c r="A21" t="inlineStr">
         <is>
           <t>2026-04-08</t>
         </is>
       </c>
-      <c r="B21" s="0" t="n">
+      <c r="B21" t="n">
         <v>20</v>
       </c>
-      <c r="C21" s="0" t="inlineStr">
+      <c r="C21" t="inlineStr">
         <is>
           <t>Saiyaara</t>
         </is>
       </c>
-      <c r="D21" s="0" t="inlineStr">
+      <c r="D21" t="inlineStr">
         <is>
           <t>Tanishk Bagchi</t>
         </is>
       </c>
     </row>
     <row r="22">
-      <c r="A22" s="0" t="inlineStr">
+      <c r="A22" t="inlineStr">
         <is>
           <t>2026-04-08</t>
         </is>
       </c>
-      <c r="B22" s="0" t="n">
+      <c r="B22" t="n">
         <v>21</v>
       </c>
-      <c r="C22" s="0" t="inlineStr">
+      <c r="C22" t="inlineStr">
         <is>
           <t>Darkhaast</t>
         </is>
       </c>
-      <c r="D22" s="0" t="inlineStr">
+      <c r="D22" t="inlineStr">
         <is>
           <t>Mithoon</t>
         </is>
       </c>
     </row>
     <row r="23">
-      <c r="A23" s="0" t="inlineStr">
+      <c r="A23" t="inlineStr">
         <is>
           <t>2026-04-08</t>
         </is>
       </c>
-      <c r="B23" s="0" t="n">
+      <c r="B23" t="n">
         <v>22</v>
       </c>
-      <c r="C23" s="0" t="inlineStr">
+      <c r="C23" t="inlineStr">
         <is>
           <t>Ishqa Ve</t>
         </is>
       </c>
-      <c r="D23" s="0" t="inlineStr">
+      <c r="D23" t="inlineStr">
         <is>
           <t>Zeeshan Ali</t>
         </is>
       </c>
     </row>
     <row r="24">
-      <c r="A24" s="0" t="inlineStr">
+      <c r="A24" t="inlineStr">
         <is>
           <t>2026-04-08</t>
         </is>
       </c>
-      <c r="B24" s="0" t="n">
+      <c r="B24" t="n">
         <v>23</v>
       </c>
-      <c r="C24" s="0" t="inlineStr">
+      <c r="C24" t="inlineStr">
         <is>
           <t>Tum Ho Toh</t>
         </is>
       </c>
-      <c r="D24" s="0" t="inlineStr">
+      <c r="D24" t="inlineStr">
         <is>
           <t>Vishal Mishra</t>
         </is>
       </c>
     </row>
     <row r="25">
-      <c r="A25" s="0" t="inlineStr">
+      <c r="A25" t="inlineStr">
         <is>
           <t>2026-04-08</t>
         </is>
       </c>
-      <c r="B25" s="0" t="n">
+      <c r="B25" t="n">
         <v>24</v>
       </c>
-      <c r="C25" s="0" t="inlineStr">
+      <c r="C25" t="inlineStr">
         <is>
           <t>Dhurandhar - Title Track</t>
         </is>
       </c>
-      <c r="D25" s="0" t="inlineStr">
+      <c r="D25" t="inlineStr">
         <is>
           <t>Shashwat Sachdev</t>
         </is>
       </c>
     </row>
     <row r="26">
-      <c r="A26" s="0" t="inlineStr">
+      <c r="A26" t="inlineStr">
         <is>
           <t>2026-04-08</t>
         </is>
       </c>
-      <c r="B26" s="0" t="n">
+      <c r="B26" t="n">
         <v>25</v>
       </c>
-      <c r="C26" s="0" t="inlineStr">
+      <c r="C26" t="inlineStr">
         <is>
           <t>Naal Nachna</t>
         </is>
       </c>
-      <c r="D26" s="0" t="inlineStr">
+      <c r="D26" t="inlineStr">
         <is>
           <t>Shashwat Sachdev</t>
         </is>
       </c>
     </row>
     <row r="27">
-      <c r="A27" s="0" t="inlineStr">
+      <c r="A27" t="inlineStr">
         <is>
           <t>2026-04-08</t>
         </is>
       </c>
-      <c r="B27" s="0" t="n">
+      <c r="B27" t="n">
         <v>26</v>
       </c>
-      <c r="C27" s="0" t="inlineStr">
+      <c r="C27" t="inlineStr">
         <is>
           <t>For A Reason</t>
         </is>
       </c>
-      <c r="D27" s="0" t="inlineStr">
+      <c r="D27" t="inlineStr">
         <is>
           <t>Karan Aujla</t>
         </is>
       </c>
     </row>
     <row r="28">
-      <c r="A28" s="0" t="inlineStr">
+      <c r="A28" t="inlineStr">
         <is>
           <t>2026-04-08</t>
         </is>
       </c>
-      <c r="B28" s="0" t="n">
+      <c r="B28" t="n">
         <v>27</v>
       </c>
-      <c r="C28" s="0" t="inlineStr">
+      <c r="C28" t="inlineStr">
         <is>
           <t>Raanjhan</t>
         </is>
       </c>
-      <c r="D28" s="0" t="inlineStr">
+      <c r="D28" t="inlineStr">
         <is>
           <t>Sachet-Parampara</t>
         </is>
       </c>
     </row>
     <row r="29">
-      <c r="A29" s="0" t="inlineStr">
+      <c r="A29" t="inlineStr">
         <is>
           <t>2026-04-08</t>
         </is>
       </c>
-      <c r="B29" s="0" t="n">
+      <c r="B29" t="n">
         <v>28</v>
       </c>
-      <c r="C29" s="0" t="inlineStr">
+      <c r="C29" t="inlineStr">
         <is>
           <t>Deewaana Deewaana</t>
         </is>
       </c>
-      <c r="D29" s="0" t="inlineStr">
+      <c r="D29" t="inlineStr">
         <is>
           <t>A.R. Rahman</t>
         </is>
       </c>
     </row>
     <row r="30">
-      <c r="A30" s="0" t="inlineStr">
+      <c r="A30" t="inlineStr">
         <is>
           <t>2026-04-08</t>
         </is>
       </c>
-      <c r="B30" s="0" t="n">
+      <c r="B30" t="n">
         <v>29</v>
       </c>
-      <c r="C30" s="0" t="inlineStr">
+      <c r="C30" t="inlineStr">
         <is>
           <t>Bairi</t>
         </is>
       </c>
-      <c r="D30" s="0" t="inlineStr">
+      <c r="D30" t="inlineStr">
         <is>
           <t>Virat</t>
         </is>
       </c>
     </row>
     <row r="31">
-      <c r="A31" s="0" t="inlineStr">
+      <c r="A31" t="inlineStr">
         <is>
           <t>2026-04-08</t>
         </is>
       </c>
-      <c r="B31" s="0" t="n">
+      <c r="B31" t="n">
         <v>30</v>
       </c>
-      <c r="C31" s="0" t="inlineStr">
+      <c r="C31" t="inlineStr">
         <is>
           <t>Jo Tum Mere Ho</t>
         </is>
       </c>
-      <c r="D31" s="0" t="inlineStr">
+      <c r="D31" t="inlineStr">
         <is>
           <t>Anuv Jain</t>
         </is>
       </c>
     </row>
     <row r="32">
-      <c r="A32" s="0" t="inlineStr">
+      <c r="A32" t="inlineStr">
         <is>
           <t>2026-04-08</t>
         </is>
       </c>
-      <c r="B32" s="0" t="n">
+      <c r="B32" t="n">
         <v>31</v>
       </c>
-      <c r="C32" s="0" t="inlineStr">
+      <c r="C32" t="inlineStr">
         <is>
           <t>Tere Liye</t>
         </is>
       </c>
-      <c r="D32" s="0" t="inlineStr">
+      <c r="D32" t="inlineStr">
         <is>
           <t>Atif Aslam</t>
         </is>
       </c>
     </row>
     <row r="33">
-      <c r="A33" s="0" t="inlineStr">
+      <c r="A33" t="inlineStr">
         <is>
           <t>2026-04-08</t>
         </is>
       </c>
-      <c r="B33" s="0" t="n">
+      <c r="B33" t="n">
         <v>32</v>
       </c>
-      <c r="C33" s="0" t="inlineStr">
+      <c r="C33" t="inlineStr">
         <is>
           <t>Phir Se</t>
         </is>
       </c>
-      <c r="D33" s="0" t="inlineStr">
+      <c r="D33" t="inlineStr">
         <is>
           <t>Shashwat Sachdev</t>
         </is>
       </c>
     </row>
     <row r="34">
-      <c r="A34" s="0" t="inlineStr">
+      <c r="A34" t="inlineStr">
         <is>
           <t>2026-04-08</t>
         </is>
       </c>
-      <c r="B34" s="0" t="n">
+      <c r="B34" t="n">
         <v>33</v>
       </c>
-      <c r="C34" s="0" t="inlineStr">
+      <c r="C34" t="inlineStr">
         <is>
           <t>Agar Tum Saath Ho</t>
         </is>
       </c>
-      <c r="D34" s="0" t="inlineStr">
+      <c r="D34" t="inlineStr">
         <is>
           <t>Alka Yagnik</t>
         </is>
       </c>
     </row>
     <row r="35">
-      <c r="A35" s="0" t="inlineStr">
+      <c r="A35" t="inlineStr">
         <is>
           <t>2026-04-08</t>
         </is>
       </c>
-      <c r="B35" s="0" t="n">
+      <c r="B35" t="n">
         <v>34</v>
       </c>
-      <c r="C35" s="0" t="inlineStr">
+      <c r="C35" t="inlineStr">
         <is>
           <t>Tere Bina</t>
         </is>
       </c>
-      <c r="D35" s="0" t="inlineStr">
+      <c r="D35" t="inlineStr">
         <is>
           <t>A.R. Rahman</t>
         </is>
       </c>
     </row>
     <row r="36">
-      <c r="A36" s="0" t="inlineStr">
+      <c r="A36" t="inlineStr">
         <is>
           <t>2026-04-08</t>
         </is>
       </c>
-      <c r="B36" s="0" t="n">
+      <c r="B36" t="n">
         <v>35</v>
       </c>
-      <c r="C36" s="0" t="inlineStr">
+      <c r="C36" t="inlineStr">
         <is>
           <t>Run Down The City - Monica</t>
         </is>
       </c>
-      <c r="D36" s="0" t="inlineStr">
+      <c r="D36" t="inlineStr">
         <is>
           <t>Shashwat Sachdev</t>
         </is>
       </c>
     </row>
     <row r="37">
-      <c r="A37" s="0" t="inlineStr">
+      <c r="A37" t="inlineStr">
         <is>
           <t>2026-04-08</t>
         </is>
       </c>
-      <c r="B37" s="0" t="n">
+      <c r="B37" t="n">
         <v>36</v>
       </c>
-      <c r="C37" s="0" t="inlineStr">
+      <c r="C37" t="inlineStr">
         <is>
           <t>Haseen</t>
         </is>
       </c>
-      <c r="D37" s="0" t="inlineStr">
+      <c r="D37" t="inlineStr">
         <is>
           <t>Talwiinder</t>
         </is>
       </c>
     </row>
     <row r="38">
-      <c r="A38" s="0" t="inlineStr">
+      <c r="A38" t="inlineStr">
         <is>
           <t>2026-04-08</t>
         </is>
       </c>
-      <c r="B38" s="0" t="n">
+      <c r="B38" t="n">
         <v>37</v>
       </c>
-      <c r="C38" s="0" t="inlineStr">
+      <c r="C38" t="inlineStr">
         <is>
           <t>Barbaad</t>
         </is>
       </c>
-      <c r="D38" s="0" t="inlineStr">
+      <c r="D38" t="inlineStr">
         <is>
           <t>The Rish</t>
         </is>
       </c>
     </row>
     <row r="39">
-      <c r="A39" s="0" t="inlineStr">
+      <c r="A39" t="inlineStr">
         <is>
           <t>2026-04-08</t>
         </is>
       </c>
-      <c r="B39" s="0" t="n">
+      <c r="B39" t="n">
         <v>38</v>
       </c>
-      <c r="C39" s="0" t="inlineStr">
+      <c r="C39" t="inlineStr">
         <is>
           <t>Lutt Le Gaya</t>
         </is>
       </c>
-      <c r="D39" s="0" t="inlineStr">
+      <c r="D39" t="inlineStr">
         <is>
           <t>Shashwat Sachdev</t>
         </is>
       </c>
     </row>
     <row r="40">
-      <c r="A40" s="0" t="inlineStr">
+      <c r="A40" t="inlineStr">
         <is>
           <t>2026-04-08</t>
         </is>
       </c>
-      <c r="B40" s="0" t="n">
+      <c r="B40" t="n">
         <v>39</v>
       </c>
-      <c r="C40" s="0" t="inlineStr">
+      <c r="C40" t="inlineStr">
         <is>
           <t>Teri Deewani</t>
         </is>
       </c>
-      <c r="D40" s="0" t="inlineStr">
+      <c r="D40" t="inlineStr">
         <is>
           <t>Kailash Kher</t>
         </is>
       </c>
     </row>
     <row r="41">
-      <c r="A41" s="0" t="inlineStr">
+      <c r="A41" t="inlineStr">
         <is>
           <t>2026-04-08</t>
         </is>
       </c>
-      <c r="B41" s="0" t="n">
+      <c r="B41" t="n">
         <v>40</v>
       </c>
-      <c r="C41" s="0" t="inlineStr">
+      <c r="C41" t="inlineStr">
         <is>
           <t>Jogi</t>
         </is>
       </c>
-      <c r="D41" s="0" t="inlineStr">
+      <c r="D41" t="inlineStr">
         <is>
           <t>thiarajxtt</t>
         </is>
       </c>
     </row>
     <row r="42">
-      <c r="A42" s="0" t="inlineStr">
+      <c r="A42" t="inlineStr">
         <is>
           <t>2026-04-08</t>
         </is>
       </c>
-      <c r="B42" s="0" t="n">
+      <c r="B42" t="n">
         <v>41</v>
       </c>
-      <c r="C42" s="0" t="inlineStr">
+      <c r="C42" t="inlineStr">
         <is>
           <t>Ye Tune Kya Kiya</t>
         </is>
       </c>
-      <c r="D42" s="0" t="inlineStr">
+      <c r="D42" t="inlineStr">
         <is>
           <t>Pritam</t>
         </is>
       </c>
     </row>
     <row r="43">
-      <c r="A43" s="0" t="inlineStr">
+      <c r="A43" t="inlineStr">
         <is>
           <t>2026-04-08</t>
         </is>
       </c>
-      <c r="B43" s="0" t="n">
+      <c r="B43" t="n">
         <v>42</v>
       </c>
-      <c r="C43" s="0" t="inlineStr">
+      <c r="C43" t="inlineStr">
         <is>
           <t>Mann Mera - Original Version</t>
         </is>
       </c>
-      <c r="D43" s="0" t="inlineStr">
+      <c r="D43" t="inlineStr">
         <is>
           <t>Gajendra Verma</t>
         </is>
       </c>
     </row>
     <row r="44">
-      <c r="A44" s="0" t="inlineStr">
+      <c r="A44" t="inlineStr">
         <is>
           <t>2026-04-08</t>
         </is>
       </c>
-      <c r="B44" s="0" t="n">
+      <c r="B44" t="n">
         <v>43</v>
       </c>
-      <c r="C44" s="0" t="inlineStr">
+      <c r="C44" t="inlineStr">
         <is>
           <t>Ehsaas</t>
         </is>
       </c>
-      <c r="D44" s="0" t="inlineStr">
+      <c r="D44" t="inlineStr">
         <is>
           <t>Faheem Abdullah</t>
         </is>
       </c>
     </row>
     <row r="45">
-      <c r="A45" s="0" t="inlineStr">
+      <c r="A45" t="inlineStr">
         <is>
           <t>2026-04-08</t>
         </is>
       </c>
-      <c r="B45" s="0" t="n">
+      <c r="B45" t="n">
         <v>44</v>
       </c>
-      <c r="C45" s="0" t="inlineStr">
+      <c r="C45" t="inlineStr">
         <is>
           <t>Dhun</t>
         </is>
       </c>
-      <c r="D45" s="0" t="inlineStr">
+      <c r="D45" t="inlineStr">
         <is>
           <t>Mithoon</t>
         </is>
       </c>
     </row>
     <row r="46">
-      <c r="A46" s="0" t="inlineStr">
+      <c r="A46" t="inlineStr">
         <is>
           <t>2026-04-08</t>
         </is>
       </c>
-      <c r="B46" s="0" t="n">
+      <c r="B46" t="n">
         <v>45</v>
       </c>
-      <c r="C46" s="0" t="inlineStr">
+      <c r="C46" t="inlineStr">
         <is>
           <t>Zaalima</t>
         </is>
       </c>
-      <c r="D46" s="0" t="inlineStr">
+      <c r="D46" t="inlineStr">
         <is>
           <t>Arijit Singh</t>
         </is>
       </c>
     </row>
     <row r="47">
-      <c r="A47" s="0" t="inlineStr">
+      <c r="A47" t="inlineStr">
         <is>
           <t>2026-04-08</t>
         </is>
       </c>
-      <c r="B47" s="0" t="n">
+      <c r="B47" t="n">
         <v>46</v>
       </c>
-      <c r="C47" s="0" t="inlineStr">
+      <c r="C47" t="inlineStr">
         <is>
           <t>Thodi Si Daaru</t>
         </is>
       </c>
-      <c r="D47" s="0" t="inlineStr">
+      <c r="D47" t="inlineStr">
         <is>
           <t>AP Dhillon</t>
         </is>
       </c>
     </row>
     <row r="48">
-      <c r="A48" s="0" t="inlineStr">
+      <c r="A48" t="inlineStr">
         <is>
           <t>2026-04-08</t>
         </is>
       </c>
-      <c r="B48" s="0" t="n">
+      <c r="B48" t="n">
         <v>47</v>
       </c>
-      <c r="C48" s="0" t="inlineStr">
+      <c r="C48" t="inlineStr">
         <is>
           <t>Main Aur Tu</t>
         </is>
       </c>
-      <c r="D48" s="0" t="inlineStr">
+      <c r="D48" t="inlineStr">
         <is>
           <t>Shashwat Sachdev</t>
         </is>
       </c>
     </row>
     <row r="49">
-      <c r="A49" s="0" t="inlineStr">
+      <c r="A49" t="inlineStr">
         <is>
           <t>2026-04-08</t>
         </is>
       </c>
-      <c r="B49" s="0" t="n">
+      <c r="B49" t="n">
         <v>48</v>
       </c>
-      <c r="C49" s="0" t="inlineStr">
+      <c r="C49" t="inlineStr">
         <is>
           <t>Ishq Jalakar - Karvaan</t>
         </is>
       </c>
-      <c r="D49" s="0" t="inlineStr">
+      <c r="D49" t="inlineStr">
         <is>
           <t>Shashwat Sachdev</t>
         </is>
       </c>
     </row>
     <row r="50">
-      <c r="A50" s="0" t="inlineStr">
+      <c r="A50" t="inlineStr">
         <is>
           <t>2026-04-08</t>
         </is>
       </c>
-      <c r="B50" s="0" t="n">
+      <c r="B50" t="n">
         <v>49</v>
       </c>
-      <c r="C50" s="0" t="inlineStr">
+      <c r="C50" t="inlineStr">
         <is>
           <t>Mast Magan</t>
         </is>
       </c>
-      <c r="D50" s="0" t="inlineStr">
+      <c r="D50" t="inlineStr">
         <is>
           <t>Arijit Singh</t>
         </is>
       </c>
     </row>
     <row r="51">
-      <c r="A51" s="0" t="inlineStr">
+      <c r="A51" t="inlineStr">
         <is>
           <t>2026-04-08</t>
         </is>
       </c>
-      <c r="B51" s="0" t="n">
+      <c r="B51" t="n">
         <v>50</v>
       </c>
-      <c r="C51" s="0" t="inlineStr">
+      <c r="C51" t="inlineStr">
         <is>
           <t>Aaya Sher</t>
         </is>
       </c>
-      <c r="D51" s="0" t="inlineStr">
+      <c r="D51" t="inlineStr">
         <is>
           <t>Anirudh Ravichander</t>
         </is>
@@ -25365,1002 +25367,3074 @@
       </c>
     </row>
     <row r="2">
-      <c r="A2" t="inlineStr">
+      <c r="A2" s="0" t="inlineStr">
         <is>
           <t>2026-04-12</t>
         </is>
       </c>
-      <c r="B2" t="n">
+      <c r="B2" s="0" t="n">
         <v>1</v>
       </c>
-      <c r="C2" t="inlineStr">
+      <c r="C2" s="0" t="inlineStr">
         <is>
           <t>Bairan</t>
         </is>
       </c>
-      <c r="D2" t="inlineStr">
+      <c r="D2" s="0" t="inlineStr">
         <is>
           <t>Banjaare</t>
         </is>
       </c>
     </row>
     <row r="3">
-      <c r="A3" t="inlineStr">
+      <c r="A3" s="0" t="inlineStr">
         <is>
           <t>2026-04-12</t>
         </is>
       </c>
-      <c r="B3" t="n">
+      <c r="B3" s="0" t="n">
         <v>2</v>
       </c>
-      <c r="C3" t="inlineStr">
+      <c r="C3" s="0" t="inlineStr">
         <is>
           <t>Gehra Hua</t>
         </is>
       </c>
-      <c r="D3" t="inlineStr">
+      <c r="D3" s="0" t="inlineStr">
         <is>
           <t>Shashwat Sachdev</t>
         </is>
       </c>
     </row>
     <row r="4">
-      <c r="A4" t="inlineStr">
+      <c r="A4" s="0" t="inlineStr">
         <is>
           <t>2026-04-12</t>
         </is>
       </c>
-      <c r="B4" t="n">
+      <c r="B4" s="0" t="n">
         <v>3</v>
       </c>
-      <c r="C4" t="inlineStr">
+      <c r="C4" s="0" t="inlineStr">
         <is>
           <t>Jaiye Sajana</t>
         </is>
       </c>
-      <c r="D4" t="inlineStr">
+      <c r="D4" s="0" t="inlineStr">
         <is>
           <t>Shashwat Sachdev</t>
         </is>
       </c>
     </row>
     <row r="5">
-      <c r="A5" t="inlineStr">
+      <c r="A5" s="0" t="inlineStr">
         <is>
           <t>2026-04-12</t>
         </is>
       </c>
-      <c r="B5" t="n">
+      <c r="B5" s="0" t="n">
         <v>4</v>
       </c>
-      <c r="C5" t="inlineStr">
+      <c r="C5" s="0" t="inlineStr">
         <is>
           <t>Sheesha - Aakhya Mai Aakh Ghali Jo Bairan</t>
         </is>
       </c>
-      <c r="D5" t="inlineStr">
+      <c r="D5" s="0" t="inlineStr">
         <is>
           <t>Mitta Ror</t>
         </is>
       </c>
     </row>
     <row r="6">
-      <c r="A6" t="inlineStr">
+      <c r="A6" s="0" t="inlineStr">
         <is>
           <t>2026-04-12</t>
         </is>
       </c>
-      <c r="B6" t="n">
+      <c r="B6" s="0" t="n">
         <v>5</v>
       </c>
-      <c r="C6" t="inlineStr">
+      <c r="C6" s="0" t="inlineStr">
         <is>
           <t>Khat</t>
         </is>
       </c>
-      <c r="D6" t="inlineStr">
+      <c r="D6" s="0" t="inlineStr">
         <is>
           <t>Navjot Ahuja</t>
         </is>
       </c>
     </row>
     <row r="7">
-      <c r="A7" t="inlineStr">
+      <c r="A7" s="0" t="inlineStr">
         <is>
           <t>2026-04-12</t>
         </is>
       </c>
-      <c r="B7" t="n">
+      <c r="B7" s="0" t="n">
         <v>6</v>
       </c>
-      <c r="C7" t="inlineStr">
+      <c r="C7" s="0" t="inlineStr">
         <is>
           <t>Dooron Dooron</t>
         </is>
       </c>
-      <c r="D7" t="inlineStr">
+      <c r="D7" s="0" t="inlineStr">
         <is>
           <t>Paresh Pahuja</t>
         </is>
       </c>
     </row>
     <row r="8">
-      <c r="A8" t="inlineStr">
+      <c r="A8" s="0" t="inlineStr">
         <is>
           <t>2026-04-12</t>
         </is>
       </c>
-      <c r="B8" t="n">
+      <c r="B8" s="0" t="n">
         <v>7</v>
       </c>
-      <c r="C8" t="inlineStr">
+      <c r="C8" s="0" t="inlineStr">
         <is>
           <t>Sahiba</t>
         </is>
       </c>
-      <c r="D8" t="inlineStr">
+      <c r="D8" s="0" t="inlineStr">
         <is>
           <t>Aditya Rikhari</t>
         </is>
       </c>
     </row>
     <row r="9">
-      <c r="A9" t="inlineStr">
+      <c r="A9" s="0" t="inlineStr">
         <is>
           <t>2026-04-12</t>
         </is>
       </c>
-      <c r="B9" t="n">
+      <c r="B9" s="0" t="n">
         <v>8</v>
       </c>
-      <c r="C9" t="inlineStr">
+      <c r="C9" s="0" t="inlineStr">
         <is>
           <t>Dhurandhar The Revenge - Aari Aari</t>
         </is>
       </c>
-      <c r="D9" t="inlineStr">
+      <c r="D9" s="0" t="inlineStr">
         <is>
           <t>Shashwat Sachdev</t>
         </is>
       </c>
     </row>
     <row r="10">
-      <c r="A10" t="inlineStr">
+      <c r="A10" s="0" t="inlineStr">
         <is>
           <t>2026-04-12</t>
         </is>
       </c>
-      <c r="B10" t="n">
+      <c r="B10" s="0" t="n">
         <v>9</v>
       </c>
-      <c r="C10" t="inlineStr">
+      <c r="C10" s="0" t="inlineStr">
         <is>
           <t>Sitaare</t>
         </is>
       </c>
-      <c r="D10" t="inlineStr">
+      <c r="D10" s="0" t="inlineStr">
         <is>
           <t>Arijit Singh</t>
         </is>
       </c>
     </row>
     <row r="11">
-      <c r="A11" t="inlineStr">
+      <c r="A11" s="0" t="inlineStr">
         <is>
           <t>2026-04-12</t>
         </is>
       </c>
-      <c r="B11" t="n">
+      <c r="B11" s="0" t="n">
         <v>10</v>
       </c>
-      <c r="C11" t="inlineStr">
+      <c r="C11" s="0" t="inlineStr">
         <is>
           <t>Samjhawan</t>
         </is>
       </c>
-      <c r="D11" t="inlineStr">
+      <c r="D11" s="0" t="inlineStr">
         <is>
           <t>Jawad Ahmad</t>
         </is>
       </c>
     </row>
     <row r="12">
-      <c r="A12" t="inlineStr">
+      <c r="A12" s="0" t="inlineStr">
         <is>
           <t>2026-04-12</t>
         </is>
       </c>
-      <c r="B12" t="n">
+      <c r="B12" s="0" t="n">
         <v>11</v>
       </c>
-      <c r="C12" t="inlineStr">
+      <c r="C12" s="0" t="inlineStr">
         <is>
           <t>Apna Bana Le</t>
         </is>
       </c>
-      <c r="D12" t="inlineStr">
+      <c r="D12" s="0" t="inlineStr">
         <is>
           <t>Sachin-Jigar</t>
         </is>
       </c>
     </row>
     <row r="13">
-      <c r="A13" t="inlineStr">
+      <c r="A13" s="0" t="inlineStr">
         <is>
           <t>2026-04-12</t>
         </is>
       </c>
-      <c r="B13" t="n">
+      <c r="B13" s="0" t="n">
         <v>12</v>
       </c>
-      <c r="C13" t="inlineStr">
+      <c r="C13" s="0" t="inlineStr">
         <is>
           <t>Finding Her</t>
         </is>
       </c>
-      <c r="D13" t="inlineStr">
+      <c r="D13" s="0" t="inlineStr">
         <is>
           <t>Kushagra</t>
         </is>
       </c>
     </row>
     <row r="14">
-      <c r="A14" t="inlineStr">
+      <c r="A14" s="0" t="inlineStr">
         <is>
           <t>2026-04-12</t>
         </is>
       </c>
-      <c r="B14" t="n">
+      <c r="B14" s="0" t="n">
         <v>13</v>
       </c>
-      <c r="C14" t="inlineStr">
+      <c r="C14" s="0" t="inlineStr">
         <is>
           <t>Pavazha Malli</t>
         </is>
       </c>
-      <c r="D14" t="inlineStr">
+      <c r="D14" s="0" t="inlineStr">
         <is>
           <t>Sai Abhyankkar</t>
         </is>
       </c>
     </row>
     <row r="15">
-      <c r="A15" t="inlineStr">
+      <c r="A15" s="0" t="inlineStr">
         <is>
           <t>2026-04-12</t>
         </is>
       </c>
-      <c r="B15" t="n">
+      <c r="B15" s="0" t="n">
         <v>14</v>
       </c>
-      <c r="C15" t="inlineStr">
+      <c r="C15" s="0" t="inlineStr">
         <is>
           <t>Shararat</t>
         </is>
       </c>
-      <c r="D15" t="inlineStr">
+      <c r="D15" s="0" t="inlineStr">
         <is>
           <t>Shashwat Sachdev</t>
         </is>
       </c>
     </row>
     <row r="16">
-      <c r="A16" t="inlineStr">
+      <c r="A16" s="0" t="inlineStr">
         <is>
           <t>2026-04-12</t>
         </is>
       </c>
-      <c r="B16" t="n">
+      <c r="B16" s="0" t="n">
         <v>15</v>
       </c>
-      <c r="C16" t="inlineStr">
+      <c r="C16" s="0" t="inlineStr">
         <is>
           <t>Jaan Se Guzarte Hain</t>
         </is>
       </c>
-      <c r="D16" t="inlineStr">
+      <c r="D16" s="0" t="inlineStr">
         <is>
           <t>Shashwat Sachdev</t>
         </is>
       </c>
     </row>
     <row r="17">
-      <c r="A17" t="inlineStr">
+      <c r="A17" s="0" t="inlineStr">
         <is>
           <t>2026-04-12</t>
         </is>
       </c>
-      <c r="B17" t="n">
+      <c r="B17" s="0" t="n">
         <v>16</v>
       </c>
-      <c r="C17" t="inlineStr">
+      <c r="C17" s="0" t="inlineStr">
         <is>
           <t>Boyfriend</t>
         </is>
       </c>
-      <c r="D17" t="inlineStr">
+      <c r="D17" s="0" t="inlineStr">
         <is>
           <t>Karan Aujla</t>
         </is>
       </c>
     </row>
     <row r="18">
-      <c r="A18" t="inlineStr">
+      <c r="A18" s="0" t="inlineStr">
         <is>
           <t>2026-04-12</t>
         </is>
       </c>
-      <c r="B18" t="n">
+      <c r="B18" s="0" t="n">
         <v>17</v>
       </c>
-      <c r="C18" t="inlineStr">
+      <c r="C18" s="0" t="inlineStr">
         <is>
           <t>Arz Kiya Hai | Coke Studio Bharat</t>
         </is>
       </c>
-      <c r="D18" t="inlineStr">
+      <c r="D18" s="0" t="inlineStr">
         <is>
           <t>Anuv Jain</t>
         </is>
       </c>
     </row>
     <row r="19">
-      <c r="A19" t="inlineStr">
+      <c r="A19" s="0" t="inlineStr">
         <is>
           <t>2026-04-12</t>
         </is>
       </c>
-      <c r="B19" t="n">
+      <c r="B19" s="0" t="n">
         <v>18</v>
       </c>
-      <c r="C19" t="inlineStr">
+      <c r="C19" s="0" t="inlineStr">
         <is>
           <t>Mann Mera</t>
         </is>
       </c>
-      <c r="D19" t="inlineStr">
+      <c r="D19" s="0" t="inlineStr">
         <is>
           <t>Gajendra Verma</t>
         </is>
       </c>
     </row>
     <row r="20">
-      <c r="A20" t="inlineStr">
+      <c r="A20" s="0" t="inlineStr">
         <is>
           <t>2026-04-12</t>
         </is>
       </c>
-      <c r="B20" t="n">
+      <c r="B20" s="0" t="n">
         <v>19</v>
       </c>
-      <c r="C20" t="inlineStr">
+      <c r="C20" s="0" t="inlineStr">
         <is>
           <t>Ishq</t>
         </is>
       </c>
-      <c r="D20" t="inlineStr">
+      <c r="D20" s="0" t="inlineStr">
         <is>
           <t>Faheem Abdullah</t>
         </is>
       </c>
     </row>
     <row r="21">
-      <c r="A21" t="inlineStr">
+      <c r="A21" s="0" t="inlineStr">
         <is>
           <t>2026-04-12</t>
         </is>
       </c>
-      <c r="B21" t="n">
+      <c r="B21" s="0" t="n">
         <v>20</v>
       </c>
-      <c r="C21" t="inlineStr">
+      <c r="C21" s="0" t="inlineStr">
         <is>
           <t>Saiyaara</t>
         </is>
       </c>
-      <c r="D21" t="inlineStr">
+      <c r="D21" s="0" t="inlineStr">
         <is>
           <t>Tanishk Bagchi</t>
         </is>
       </c>
     </row>
     <row r="22">
-      <c r="A22" t="inlineStr">
+      <c r="A22" s="0" t="inlineStr">
         <is>
           <t>2026-04-12</t>
         </is>
       </c>
-      <c r="B22" t="n">
+      <c r="B22" s="0" t="n">
         <v>21</v>
       </c>
-      <c r="C22" t="inlineStr">
+      <c r="C22" s="0" t="inlineStr">
         <is>
           <t>Bairi</t>
         </is>
       </c>
-      <c r="D22" t="inlineStr">
+      <c r="D22" s="0" t="inlineStr">
         <is>
           <t>Virat</t>
         </is>
       </c>
     </row>
     <row r="23">
-      <c r="A23" t="inlineStr">
+      <c r="A23" s="0" t="inlineStr">
         <is>
           <t>2026-04-12</t>
         </is>
       </c>
-      <c r="B23" t="n">
+      <c r="B23" s="0" t="n">
         <v>22</v>
       </c>
-      <c r="C23" t="inlineStr">
+      <c r="C23" s="0" t="inlineStr">
         <is>
           <t>For A Reason</t>
         </is>
       </c>
-      <c r="D23" t="inlineStr">
+      <c r="D23" s="0" t="inlineStr">
         <is>
           <t>Karan Aujla</t>
         </is>
       </c>
     </row>
     <row r="24">
-      <c r="A24" t="inlineStr">
+      <c r="A24" s="0" t="inlineStr">
         <is>
           <t>2026-04-12</t>
         </is>
       </c>
-      <c r="B24" t="n">
+      <c r="B24" s="0" t="n">
         <v>23</v>
       </c>
-      <c r="C24" t="inlineStr">
+      <c r="C24" s="0" t="inlineStr">
         <is>
           <t>Darkhaast</t>
         </is>
       </c>
-      <c r="D24" t="inlineStr">
+      <c r="D24" s="0" t="inlineStr">
         <is>
           <t>Mithoon</t>
         </is>
       </c>
     </row>
     <row r="25">
-      <c r="A25" t="inlineStr">
+      <c r="A25" s="0" t="inlineStr">
         <is>
           <t>2026-04-12</t>
         </is>
       </c>
-      <c r="B25" t="n">
+      <c r="B25" s="0" t="n">
         <v>24</v>
       </c>
-      <c r="C25" t="inlineStr">
+      <c r="C25" s="0" t="inlineStr">
         <is>
           <t>Naal Nachna</t>
         </is>
       </c>
-      <c r="D25" t="inlineStr">
+      <c r="D25" s="0" t="inlineStr">
         <is>
           <t>Shashwat Sachdev</t>
         </is>
       </c>
     </row>
     <row r="26">
-      <c r="A26" t="inlineStr">
+      <c r="A26" s="0" t="inlineStr">
         <is>
           <t>2026-04-12</t>
         </is>
       </c>
-      <c r="B26" t="n">
+      <c r="B26" s="0" t="n">
         <v>25</v>
       </c>
-      <c r="C26" t="inlineStr">
+      <c r="C26" s="0" t="inlineStr">
         <is>
           <t>Tum Ho Toh</t>
         </is>
       </c>
-      <c r="D26" t="inlineStr">
+      <c r="D26" s="0" t="inlineStr">
         <is>
           <t>Vishal Mishra</t>
         </is>
       </c>
     </row>
     <row r="27">
-      <c r="A27" t="inlineStr">
+      <c r="A27" s="0" t="inlineStr">
         <is>
           <t>2026-04-12</t>
         </is>
       </c>
-      <c r="B27" t="n">
+      <c r="B27" s="0" t="n">
         <v>26</v>
       </c>
-      <c r="C27" t="inlineStr">
+      <c r="C27" s="0" t="inlineStr">
         <is>
           <t>Dhurandhar - Title Track</t>
         </is>
       </c>
-      <c r="D27" t="inlineStr">
+      <c r="D27" s="0" t="inlineStr">
         <is>
           <t>Shashwat Sachdev</t>
         </is>
       </c>
     </row>
     <row r="28">
-      <c r="A28" t="inlineStr">
+      <c r="A28" s="0" t="inlineStr">
         <is>
           <t>2026-04-12</t>
         </is>
       </c>
-      <c r="B28" t="n">
+      <c r="B28" s="0" t="n">
         <v>27</v>
       </c>
-      <c r="C28" t="inlineStr">
+      <c r="C28" s="0" t="inlineStr">
         <is>
           <t>Ishqa Ve</t>
         </is>
       </c>
-      <c r="D28" t="inlineStr">
+      <c r="D28" s="0" t="inlineStr">
         <is>
           <t>Zeeshan Ali</t>
         </is>
       </c>
     </row>
     <row r="29">
-      <c r="A29" t="inlineStr">
+      <c r="A29" s="0" t="inlineStr">
         <is>
           <t>2026-04-12</t>
         </is>
       </c>
-      <c r="B29" t="n">
+      <c r="B29" s="0" t="n">
         <v>28</v>
       </c>
-      <c r="C29" t="inlineStr">
+      <c r="C29" s="0" t="inlineStr">
         <is>
           <t>Tere Liye</t>
         </is>
       </c>
-      <c r="D29" t="inlineStr">
+      <c r="D29" s="0" t="inlineStr">
         <is>
           <t>Atif Aslam</t>
         </is>
       </c>
     </row>
     <row r="30">
-      <c r="A30" t="inlineStr">
+      <c r="A30" s="0" t="inlineStr">
         <is>
           <t>2026-04-12</t>
         </is>
       </c>
-      <c r="B30" t="n">
+      <c r="B30" s="0" t="n">
         <v>29</v>
       </c>
-      <c r="C30" t="inlineStr">
+      <c r="C30" s="0" t="inlineStr">
         <is>
           <t>Raanjhan</t>
         </is>
       </c>
-      <c r="D30" t="inlineStr">
+      <c r="D30" s="0" t="inlineStr">
         <is>
           <t>Sachet-Parampara</t>
         </is>
       </c>
     </row>
     <row r="31">
-      <c r="A31" t="inlineStr">
+      <c r="A31" s="0" t="inlineStr">
         <is>
           <t>2026-04-12</t>
         </is>
       </c>
-      <c r="B31" t="n">
+      <c r="B31" s="0" t="n">
         <v>30</v>
       </c>
-      <c r="C31" t="inlineStr">
+      <c r="C31" s="0" t="inlineStr">
         <is>
           <t>Deewaana Deewaana</t>
         </is>
       </c>
-      <c r="D31" t="inlineStr">
+      <c r="D31" s="0" t="inlineStr">
         <is>
           <t>A.R. Rahman</t>
         </is>
       </c>
     </row>
     <row r="32">
-      <c r="A32" t="inlineStr">
+      <c r="A32" s="0" t="inlineStr">
         <is>
           <t>2026-04-12</t>
         </is>
       </c>
-      <c r="B32" t="n">
+      <c r="B32" s="0" t="n">
         <v>31</v>
       </c>
-      <c r="C32" t="inlineStr">
+      <c r="C32" s="0" t="inlineStr">
         <is>
           <t>Tere Bina</t>
         </is>
       </c>
-      <c r="D32" t="inlineStr">
+      <c r="D32" s="0" t="inlineStr">
         <is>
           <t>A.R. Rahman</t>
         </is>
       </c>
     </row>
     <row r="33">
-      <c r="A33" t="inlineStr">
+      <c r="A33" s="0" t="inlineStr">
         <is>
           <t>2026-04-12</t>
         </is>
       </c>
-      <c r="B33" t="n">
+      <c r="B33" s="0" t="n">
         <v>32</v>
       </c>
-      <c r="C33" t="inlineStr">
+      <c r="C33" s="0" t="inlineStr">
         <is>
           <t>Jo Tum Mere Ho</t>
         </is>
       </c>
-      <c r="D33" t="inlineStr">
+      <c r="D33" s="0" t="inlineStr">
         <is>
           <t>Anuv Jain</t>
         </is>
       </c>
     </row>
     <row r="34">
-      <c r="A34" t="inlineStr">
+      <c r="A34" s="0" t="inlineStr">
         <is>
           <t>2026-04-12</t>
         </is>
       </c>
-      <c r="B34" t="n">
+      <c r="B34" s="0" t="n">
         <v>33</v>
       </c>
-      <c r="C34" t="inlineStr">
+      <c r="C34" s="0" t="inlineStr">
         <is>
           <t>Agar Tum Saath Ho</t>
         </is>
       </c>
-      <c r="D34" t="inlineStr">
+      <c r="D34" s="0" t="inlineStr">
         <is>
           <t>Alka Yagnik</t>
         </is>
       </c>
     </row>
     <row r="35">
-      <c r="A35" t="inlineStr">
+      <c r="A35" s="0" t="inlineStr">
         <is>
           <t>2026-04-12</t>
         </is>
       </c>
-      <c r="B35" t="n">
+      <c r="B35" s="0" t="n">
         <v>34</v>
       </c>
-      <c r="C35" t="inlineStr">
+      <c r="C35" s="0" t="inlineStr">
         <is>
           <t>Lutt Le Gaya</t>
         </is>
       </c>
-      <c r="D35" t="inlineStr">
+      <c r="D35" s="0" t="inlineStr">
         <is>
           <t>Shashwat Sachdev</t>
         </is>
       </c>
     </row>
     <row r="36">
-      <c r="A36" t="inlineStr">
+      <c r="A36" s="0" t="inlineStr">
         <is>
           <t>2026-04-12</t>
         </is>
       </c>
-      <c r="B36" t="n">
+      <c r="B36" s="0" t="n">
         <v>35</v>
       </c>
-      <c r="C36" t="inlineStr">
+      <c r="C36" s="0" t="inlineStr">
         <is>
           <t>Teri Deewani</t>
         </is>
       </c>
-      <c r="D36" t="inlineStr">
+      <c r="D36" s="0" t="inlineStr">
         <is>
           <t>Kailash Kher</t>
         </is>
       </c>
     </row>
     <row r="37">
-      <c r="A37" t="inlineStr">
+      <c r="A37" s="0" t="inlineStr">
         <is>
           <t>2026-04-12</t>
         </is>
       </c>
-      <c r="B37" t="n">
+      <c r="B37" s="0" t="n">
         <v>36</v>
       </c>
-      <c r="C37" t="inlineStr">
+      <c r="C37" s="0" t="inlineStr">
         <is>
           <t>Phir Se</t>
         </is>
       </c>
-      <c r="D37" t="inlineStr">
+      <c r="D37" s="0" t="inlineStr">
         <is>
           <t>Shashwat Sachdev</t>
         </is>
       </c>
     </row>
     <row r="38">
-      <c r="A38" t="inlineStr">
+      <c r="A38" s="0" t="inlineStr">
         <is>
           <t>2026-04-12</t>
         </is>
       </c>
-      <c r="B38" t="n">
+      <c r="B38" s="0" t="n">
         <v>37</v>
       </c>
-      <c r="C38" t="inlineStr">
+      <c r="C38" s="0" t="inlineStr">
         <is>
           <t>Ehsaas</t>
         </is>
       </c>
-      <c r="D38" t="inlineStr">
+      <c r="D38" s="0" t="inlineStr">
         <is>
           <t>Faheem Abdullah</t>
         </is>
       </c>
     </row>
     <row r="39">
-      <c r="A39" t="inlineStr">
+      <c r="A39" s="0" t="inlineStr">
         <is>
           <t>2026-04-12</t>
         </is>
       </c>
-      <c r="B39" t="n">
+      <c r="B39" s="0" t="n">
         <v>38</v>
       </c>
-      <c r="C39" t="inlineStr">
+      <c r="C39" s="0" t="inlineStr">
         <is>
           <t>Ye Tune Kya Kiya</t>
         </is>
       </c>
-      <c r="D39" t="inlineStr">
+      <c r="D39" s="0" t="inlineStr">
         <is>
           <t>Pritam</t>
         </is>
       </c>
     </row>
     <row r="40">
-      <c r="A40" t="inlineStr">
+      <c r="A40" s="0" t="inlineStr">
         <is>
           <t>2026-04-12</t>
         </is>
       </c>
-      <c r="B40" t="n">
+      <c r="B40" s="0" t="n">
         <v>39</v>
       </c>
-      <c r="C40" t="inlineStr">
+      <c r="C40" s="0" t="inlineStr">
         <is>
           <t>Haseen</t>
         </is>
       </c>
-      <c r="D40" t="inlineStr">
+      <c r="D40" s="0" t="inlineStr">
         <is>
           <t>Talwiinder</t>
         </is>
       </c>
     </row>
     <row r="41">
-      <c r="A41" t="inlineStr">
+      <c r="A41" s="0" t="inlineStr">
         <is>
           <t>2026-04-12</t>
         </is>
       </c>
-      <c r="B41" t="n">
+      <c r="B41" s="0" t="n">
         <v>40</v>
       </c>
-      <c r="C41" t="inlineStr">
+      <c r="C41" s="0" t="inlineStr">
         <is>
           <t>Run Down The City - Monica</t>
         </is>
       </c>
-      <c r="D41" t="inlineStr">
+      <c r="D41" s="0" t="inlineStr">
         <is>
           <t>Shashwat Sachdev</t>
         </is>
       </c>
     </row>
     <row r="42">
-      <c r="A42" t="inlineStr">
+      <c r="A42" s="0" t="inlineStr">
         <is>
           <t>2026-04-12</t>
         </is>
       </c>
-      <c r="B42" t="n">
+      <c r="B42" s="0" t="n">
         <v>41</v>
       </c>
-      <c r="C42" t="inlineStr">
+      <c r="C42" s="0" t="inlineStr">
         <is>
           <t>Barbaad</t>
         </is>
       </c>
-      <c r="D42" t="inlineStr">
+      <c r="D42" s="0" t="inlineStr">
         <is>
           <t>The Rish</t>
         </is>
       </c>
     </row>
     <row r="43">
-      <c r="A43" t="inlineStr">
+      <c r="A43" s="0" t="inlineStr">
         <is>
           <t>2026-04-12</t>
         </is>
       </c>
-      <c r="B43" t="n">
+      <c r="B43" s="0" t="n">
         <v>42</v>
       </c>
-      <c r="C43" t="inlineStr">
+      <c r="C43" s="0" t="inlineStr">
         <is>
           <t>Mutta Kalakki</t>
         </is>
       </c>
-      <c r="D43" t="inlineStr">
+      <c r="D43" s="0" t="inlineStr">
         <is>
           <t>G. V. Prakash</t>
         </is>
       </c>
     </row>
     <row r="44">
-      <c r="A44" t="inlineStr">
+      <c r="A44" s="0" t="inlineStr">
         <is>
           <t>2026-04-12</t>
         </is>
       </c>
-      <c r="B44" t="n">
+      <c r="B44" s="0" t="n">
         <v>43</v>
       </c>
-      <c r="C44" t="inlineStr">
+      <c r="C44" s="0" t="inlineStr">
         <is>
           <t>Mast Magan</t>
         </is>
       </c>
-      <c r="D44" t="inlineStr">
+      <c r="D44" s="0" t="inlineStr">
         <is>
           <t>Arijit Singh</t>
         </is>
       </c>
     </row>
     <row r="45">
-      <c r="A45" t="inlineStr">
+      <c r="A45" s="0" t="inlineStr">
         <is>
           <t>2026-04-12</t>
         </is>
       </c>
-      <c r="B45" t="n">
+      <c r="B45" s="0" t="n">
         <v>44</v>
       </c>
-      <c r="C45" t="inlineStr">
+      <c r="C45" s="0" t="inlineStr">
         <is>
           <t>Zaalima</t>
         </is>
       </c>
-      <c r="D45" t="inlineStr">
+      <c r="D45" s="0" t="inlineStr">
         <is>
           <t>Arijit Singh</t>
         </is>
       </c>
     </row>
     <row r="46">
-      <c r="A46" t="inlineStr">
+      <c r="A46" s="0" t="inlineStr">
         <is>
           <t>2026-04-12</t>
         </is>
       </c>
-      <c r="B46" t="n">
+      <c r="B46" s="0" t="n">
         <v>45</v>
       </c>
-      <c r="C46" t="inlineStr">
+      <c r="C46" s="0" t="inlineStr">
         <is>
           <t>Thodi Si Daaru</t>
         </is>
       </c>
-      <c r="D46" t="inlineStr">
+      <c r="D46" s="0" t="inlineStr">
         <is>
           <t>AP Dhillon</t>
         </is>
       </c>
     </row>
     <row r="47">
-      <c r="A47" t="inlineStr">
+      <c r="A47" s="0" t="inlineStr">
         <is>
           <t>2026-04-12</t>
         </is>
       </c>
-      <c r="B47" t="n">
+      <c r="B47" s="0" t="n">
         <v>46</v>
       </c>
-      <c r="C47" t="inlineStr">
+      <c r="C47" s="0" t="inlineStr">
         <is>
           <t>Ishq Jalakar - Karvaan</t>
         </is>
       </c>
-      <c r="D47" t="inlineStr">
+      <c r="D47" s="0" t="inlineStr">
         <is>
           <t>Shashwat Sachdev</t>
         </is>
       </c>
     </row>
     <row r="48">
-      <c r="A48" t="inlineStr">
+      <c r="A48" s="0" t="inlineStr">
         <is>
           <t>2026-04-12</t>
         </is>
       </c>
-      <c r="B48" t="n">
+      <c r="B48" s="0" t="n">
         <v>47</v>
       </c>
-      <c r="C48" t="inlineStr">
+      <c r="C48" s="0" t="inlineStr">
         <is>
           <t>Humdard</t>
         </is>
       </c>
-      <c r="D48" t="inlineStr">
+      <c r="D48" s="0" t="inlineStr">
         <is>
           <t>Arijit Singh</t>
         </is>
       </c>
     </row>
     <row r="49">
-      <c r="A49" t="inlineStr">
+      <c r="A49" s="0" t="inlineStr">
         <is>
           <t>2026-04-12</t>
         </is>
       </c>
-      <c r="B49" t="n">
+      <c r="B49" s="0" t="n">
         <v>48</v>
       </c>
-      <c r="C49" t="inlineStr">
+      <c r="C49" s="0" t="inlineStr">
         <is>
           <t>Mann Mera - Original Version</t>
         </is>
       </c>
-      <c r="D49" t="inlineStr">
+      <c r="D49" s="0" t="inlineStr">
         <is>
           <t>Gajendra Verma</t>
         </is>
       </c>
     </row>
     <row r="50">
-      <c r="A50" t="inlineStr">
+      <c r="A50" s="0" t="inlineStr">
         <is>
           <t>2026-04-12</t>
         </is>
       </c>
-      <c r="B50" t="n">
+      <c r="B50" s="0" t="n">
         <v>49</v>
       </c>
-      <c r="C50" t="inlineStr">
+      <c r="C50" s="0" t="inlineStr">
         <is>
           <t>Jogi</t>
         </is>
       </c>
-      <c r="D50" t="inlineStr">
+      <c r="D50" s="0" t="inlineStr">
         <is>
           <t>thiarajxtt</t>
         </is>
       </c>
     </row>
     <row r="51">
-      <c r="A51" t="inlineStr">
+      <c r="A51" s="0" t="inlineStr">
         <is>
           <t>2026-04-12</t>
         </is>
       </c>
-      <c r="B51" t="n">
+      <c r="B51" s="0" t="n">
         <v>50</v>
       </c>
-      <c r="C51" t="inlineStr">
+      <c r="C51" s="0" t="inlineStr">
         <is>
           <t>Aaya Sher</t>
         </is>
       </c>
-      <c r="D51" t="inlineStr">
+      <c r="D51" s="0" t="inlineStr">
         <is>
           <t>Anirudh Ravichander</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet31.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:D51"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="24" t="inlineStr">
+        <is>
+          <t>Date</t>
+        </is>
+      </c>
+      <c r="B1" s="24" t="inlineStr">
+        <is>
+          <t>Rank</t>
+        </is>
+      </c>
+      <c r="C1" s="24" t="inlineStr">
+        <is>
+          <t>Song</t>
+        </is>
+      </c>
+      <c r="D1" s="24" t="inlineStr">
+        <is>
+          <t>Artist</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="0" t="inlineStr">
+        <is>
+          <t>2026-04-14</t>
+        </is>
+      </c>
+      <c r="B2" s="0" t="n">
+        <v>1</v>
+      </c>
+      <c r="C2" s="0" t="inlineStr">
+        <is>
+          <t>Bairan</t>
+        </is>
+      </c>
+      <c r="D2" s="0" t="inlineStr">
+        <is>
+          <t>Banjaare</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="0" t="inlineStr">
+        <is>
+          <t>2026-04-14</t>
+        </is>
+      </c>
+      <c r="B3" s="0" t="n">
+        <v>2</v>
+      </c>
+      <c r="C3" s="0" t="inlineStr">
+        <is>
+          <t>Sheesha - Aakhya Mai Aakh Ghali Jo Bairan</t>
+        </is>
+      </c>
+      <c r="D3" s="0" t="inlineStr">
+        <is>
+          <t>Mitta Ror</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="0" t="inlineStr">
+        <is>
+          <t>2026-04-14</t>
+        </is>
+      </c>
+      <c r="B4" s="0" t="n">
+        <v>3</v>
+      </c>
+      <c r="C4" s="0" t="inlineStr">
+        <is>
+          <t>Gehra Hua</t>
+        </is>
+      </c>
+      <c r="D4" s="0" t="inlineStr">
+        <is>
+          <t>Shashwat Sachdev</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="0" t="inlineStr">
+        <is>
+          <t>2026-04-14</t>
+        </is>
+      </c>
+      <c r="B5" s="0" t="n">
+        <v>4</v>
+      </c>
+      <c r="C5" s="0" t="inlineStr">
+        <is>
+          <t>Jaiye Sajana</t>
+        </is>
+      </c>
+      <c r="D5" s="0" t="inlineStr">
+        <is>
+          <t>Shashwat Sachdev</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="0" t="inlineStr">
+        <is>
+          <t>2026-04-14</t>
+        </is>
+      </c>
+      <c r="B6" s="0" t="n">
+        <v>5</v>
+      </c>
+      <c r="C6" s="0" t="inlineStr">
+        <is>
+          <t>Khat</t>
+        </is>
+      </c>
+      <c r="D6" s="0" t="inlineStr">
+        <is>
+          <t>Navjot Ahuja</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="0" t="inlineStr">
+        <is>
+          <t>2026-04-14</t>
+        </is>
+      </c>
+      <c r="B7" s="0" t="n">
+        <v>6</v>
+      </c>
+      <c r="C7" s="0" t="inlineStr">
+        <is>
+          <t>Sahiba</t>
+        </is>
+      </c>
+      <c r="D7" s="0" t="inlineStr">
+        <is>
+          <t>Aditya Rikhari</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="0" t="inlineStr">
+        <is>
+          <t>2026-04-14</t>
+        </is>
+      </c>
+      <c r="B8" s="0" t="n">
+        <v>7</v>
+      </c>
+      <c r="C8" s="0" t="inlineStr">
+        <is>
+          <t>Sitaare</t>
+        </is>
+      </c>
+      <c r="D8" s="0" t="inlineStr">
+        <is>
+          <t>Arijit Singh</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="0" t="inlineStr">
+        <is>
+          <t>2026-04-14</t>
+        </is>
+      </c>
+      <c r="B9" s="0" t="n">
+        <v>8</v>
+      </c>
+      <c r="C9" s="0" t="inlineStr">
+        <is>
+          <t>Dooron Dooron</t>
+        </is>
+      </c>
+      <c r="D9" s="0" t="inlineStr">
+        <is>
+          <t>Paresh Pahuja</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="0" t="inlineStr">
+        <is>
+          <t>2026-04-14</t>
+        </is>
+      </c>
+      <c r="B10" s="0" t="n">
+        <v>9</v>
+      </c>
+      <c r="C10" s="0" t="inlineStr">
+        <is>
+          <t>Finding Her</t>
+        </is>
+      </c>
+      <c r="D10" s="0" t="inlineStr">
+        <is>
+          <t>Kushagra</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="0" t="inlineStr">
+        <is>
+          <t>2026-04-14</t>
+        </is>
+      </c>
+      <c r="B11" s="0" t="n">
+        <v>10</v>
+      </c>
+      <c r="C11" s="0" t="inlineStr">
+        <is>
+          <t>Samjhawan</t>
+        </is>
+      </c>
+      <c r="D11" s="0" t="inlineStr">
+        <is>
+          <t>Jawad Ahmad</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="0" t="inlineStr">
+        <is>
+          <t>2026-04-14</t>
+        </is>
+      </c>
+      <c r="B12" s="0" t="n">
+        <v>11</v>
+      </c>
+      <c r="C12" s="0" t="inlineStr">
+        <is>
+          <t>Arz Kiya Hai | Coke Studio Bharat</t>
+        </is>
+      </c>
+      <c r="D12" s="0" t="inlineStr">
+        <is>
+          <t>Anuv Jain</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="0" t="inlineStr">
+        <is>
+          <t>2026-04-14</t>
+        </is>
+      </c>
+      <c r="B13" s="0" t="n">
+        <v>12</v>
+      </c>
+      <c r="C13" s="0" t="inlineStr">
+        <is>
+          <t>Boyfriend</t>
+        </is>
+      </c>
+      <c r="D13" s="0" t="inlineStr">
+        <is>
+          <t>Karan Aujla</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="0" t="inlineStr">
+        <is>
+          <t>2026-04-14</t>
+        </is>
+      </c>
+      <c r="B14" s="0" t="n">
+        <v>13</v>
+      </c>
+      <c r="C14" s="0" t="inlineStr">
+        <is>
+          <t>Apna Bana Le</t>
+        </is>
+      </c>
+      <c r="D14" s="0" t="inlineStr">
+        <is>
+          <t>Sachin-Jigar</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="0" t="inlineStr">
+        <is>
+          <t>2026-04-14</t>
+        </is>
+      </c>
+      <c r="B15" s="0" t="n">
+        <v>14</v>
+      </c>
+      <c r="C15" s="0" t="inlineStr">
+        <is>
+          <t>Pavazha Malli</t>
+        </is>
+      </c>
+      <c r="D15" s="0" t="inlineStr">
+        <is>
+          <t>Sai Abhyankkar</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="0" t="inlineStr">
+        <is>
+          <t>2026-04-14</t>
+        </is>
+      </c>
+      <c r="B16" s="0" t="n">
+        <v>15</v>
+      </c>
+      <c r="C16" s="0" t="inlineStr">
+        <is>
+          <t>Dhurandhar The Revenge - Aari Aari</t>
+        </is>
+      </c>
+      <c r="D16" s="0" t="inlineStr">
+        <is>
+          <t>Shashwat Sachdev</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="0" t="inlineStr">
+        <is>
+          <t>2026-04-14</t>
+        </is>
+      </c>
+      <c r="B17" s="0" t="n">
+        <v>16</v>
+      </c>
+      <c r="C17" s="0" t="inlineStr">
+        <is>
+          <t>Jaan Se Guzarte Hain</t>
+        </is>
+      </c>
+      <c r="D17" s="0" t="inlineStr">
+        <is>
+          <t>Shashwat Sachdev</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="0" t="inlineStr">
+        <is>
+          <t>2026-04-14</t>
+        </is>
+      </c>
+      <c r="B18" s="0" t="n">
+        <v>17</v>
+      </c>
+      <c r="C18" s="0" t="inlineStr">
+        <is>
+          <t>Mann Mera</t>
+        </is>
+      </c>
+      <c r="D18" s="0" t="inlineStr">
+        <is>
+          <t>Gajendra Verma</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="0" t="inlineStr">
+        <is>
+          <t>2026-04-14</t>
+        </is>
+      </c>
+      <c r="B19" s="0" t="n">
+        <v>18</v>
+      </c>
+      <c r="C19" s="0" t="inlineStr">
+        <is>
+          <t>Shararat</t>
+        </is>
+      </c>
+      <c r="D19" s="0" t="inlineStr">
+        <is>
+          <t>Shashwat Sachdev</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="0" t="inlineStr">
+        <is>
+          <t>2026-04-14</t>
+        </is>
+      </c>
+      <c r="B20" s="0" t="n">
+        <v>19</v>
+      </c>
+      <c r="C20" s="0" t="inlineStr">
+        <is>
+          <t>Ishq</t>
+        </is>
+      </c>
+      <c r="D20" s="0" t="inlineStr">
+        <is>
+          <t>Faheem Abdullah</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="0" t="inlineStr">
+        <is>
+          <t>2026-04-14</t>
+        </is>
+      </c>
+      <c r="B21" s="0" t="n">
+        <v>20</v>
+      </c>
+      <c r="C21" s="0" t="inlineStr">
+        <is>
+          <t>For A Reason</t>
+        </is>
+      </c>
+      <c r="D21" s="0" t="inlineStr">
+        <is>
+          <t>Karan Aujla</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="0" t="inlineStr">
+        <is>
+          <t>2026-04-14</t>
+        </is>
+      </c>
+      <c r="B22" s="0" t="n">
+        <v>21</v>
+      </c>
+      <c r="C22" s="0" t="inlineStr">
+        <is>
+          <t>Ishqa Ve</t>
+        </is>
+      </c>
+      <c r="D22" s="0" t="inlineStr">
+        <is>
+          <t>Zeeshan Ali</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="0" t="inlineStr">
+        <is>
+          <t>2026-04-14</t>
+        </is>
+      </c>
+      <c r="B23" s="0" t="n">
+        <v>22</v>
+      </c>
+      <c r="C23" s="0" t="inlineStr">
+        <is>
+          <t>Saiyaara</t>
+        </is>
+      </c>
+      <c r="D23" s="0" t="inlineStr">
+        <is>
+          <t>Tanishk Bagchi</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="0" t="inlineStr">
+        <is>
+          <t>2026-04-14</t>
+        </is>
+      </c>
+      <c r="B24" s="0" t="n">
+        <v>23</v>
+      </c>
+      <c r="C24" s="0" t="inlineStr">
+        <is>
+          <t>Bairi</t>
+        </is>
+      </c>
+      <c r="D24" s="0" t="inlineStr">
+        <is>
+          <t>Virat</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="0" t="inlineStr">
+        <is>
+          <t>2026-04-14</t>
+        </is>
+      </c>
+      <c r="B25" s="0" t="n">
+        <v>24</v>
+      </c>
+      <c r="C25" s="0" t="inlineStr">
+        <is>
+          <t>Naal Nachna</t>
+        </is>
+      </c>
+      <c r="D25" s="0" t="inlineStr">
+        <is>
+          <t>Shashwat Sachdev</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="0" t="inlineStr">
+        <is>
+          <t>2026-04-14</t>
+        </is>
+      </c>
+      <c r="B26" s="0" t="n">
+        <v>25</v>
+      </c>
+      <c r="C26" s="0" t="inlineStr">
+        <is>
+          <t>Deewaana Deewaana</t>
+        </is>
+      </c>
+      <c r="D26" s="0" t="inlineStr">
+        <is>
+          <t>A.R. Rahman</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="0" t="inlineStr">
+        <is>
+          <t>2026-04-14</t>
+        </is>
+      </c>
+      <c r="B27" s="0" t="n">
+        <v>26</v>
+      </c>
+      <c r="C27" s="0" t="inlineStr">
+        <is>
+          <t>Tum Ho Toh</t>
+        </is>
+      </c>
+      <c r="D27" s="0" t="inlineStr">
+        <is>
+          <t>Vishal Mishra</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="0" t="inlineStr">
+        <is>
+          <t>2026-04-14</t>
+        </is>
+      </c>
+      <c r="B28" s="0" t="n">
+        <v>27</v>
+      </c>
+      <c r="C28" s="0" t="inlineStr">
+        <is>
+          <t>Tere Liye</t>
+        </is>
+      </c>
+      <c r="D28" s="0" t="inlineStr">
+        <is>
+          <t>Atif Aslam</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="0" t="inlineStr">
+        <is>
+          <t>2026-04-14</t>
+        </is>
+      </c>
+      <c r="B29" s="0" t="n">
+        <v>28</v>
+      </c>
+      <c r="C29" s="0" t="inlineStr">
+        <is>
+          <t>Dhurandhar - Title Track</t>
+        </is>
+      </c>
+      <c r="D29" s="0" t="inlineStr">
+        <is>
+          <t>Shashwat Sachdev</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="0" t="inlineStr">
+        <is>
+          <t>2026-04-14</t>
+        </is>
+      </c>
+      <c r="B30" s="0" t="n">
+        <v>29</v>
+      </c>
+      <c r="C30" s="0" t="inlineStr">
+        <is>
+          <t>Raanjhan</t>
+        </is>
+      </c>
+      <c r="D30" s="0" t="inlineStr">
+        <is>
+          <t>Sachet-Parampara</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="0" t="inlineStr">
+        <is>
+          <t>2026-04-14</t>
+        </is>
+      </c>
+      <c r="B31" s="0" t="n">
+        <v>30</v>
+      </c>
+      <c r="C31" s="0" t="inlineStr">
+        <is>
+          <t>Phir Se</t>
+        </is>
+      </c>
+      <c r="D31" s="0" t="inlineStr">
+        <is>
+          <t>Shashwat Sachdev</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="0" t="inlineStr">
+        <is>
+          <t>2026-04-14</t>
+        </is>
+      </c>
+      <c r="B32" s="0" t="n">
+        <v>31</v>
+      </c>
+      <c r="C32" s="0" t="inlineStr">
+        <is>
+          <t>Darkhaast</t>
+        </is>
+      </c>
+      <c r="D32" s="0" t="inlineStr">
+        <is>
+          <t>Mithoon</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="0" t="inlineStr">
+        <is>
+          <t>2026-04-14</t>
+        </is>
+      </c>
+      <c r="B33" s="0" t="n">
+        <v>32</v>
+      </c>
+      <c r="C33" s="0" t="inlineStr">
+        <is>
+          <t>Ehsaas</t>
+        </is>
+      </c>
+      <c r="D33" s="0" t="inlineStr">
+        <is>
+          <t>Faheem Abdullah</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="0" t="inlineStr">
+        <is>
+          <t>2026-04-14</t>
+        </is>
+      </c>
+      <c r="B34" s="0" t="n">
+        <v>33</v>
+      </c>
+      <c r="C34" s="0" t="inlineStr">
+        <is>
+          <t>Jo Tum Mere Ho</t>
+        </is>
+      </c>
+      <c r="D34" s="0" t="inlineStr">
+        <is>
+          <t>Anuv Jain</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="0" t="inlineStr">
+        <is>
+          <t>2026-04-14</t>
+        </is>
+      </c>
+      <c r="B35" s="0" t="n">
+        <v>34</v>
+      </c>
+      <c r="C35" s="0" t="inlineStr">
+        <is>
+          <t>Tere Bina</t>
+        </is>
+      </c>
+      <c r="D35" s="0" t="inlineStr">
+        <is>
+          <t>A.R. Rahman</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="0" t="inlineStr">
+        <is>
+          <t>2026-04-14</t>
+        </is>
+      </c>
+      <c r="B36" s="0" t="n">
+        <v>35</v>
+      </c>
+      <c r="C36" s="0" t="inlineStr">
+        <is>
+          <t>Agar Tum Saath Ho</t>
+        </is>
+      </c>
+      <c r="D36" s="0" t="inlineStr">
+        <is>
+          <t>Alka Yagnik</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="0" t="inlineStr">
+        <is>
+          <t>2026-04-14</t>
+        </is>
+      </c>
+      <c r="B37" s="0" t="n">
+        <v>36</v>
+      </c>
+      <c r="C37" s="0" t="inlineStr">
+        <is>
+          <t>Teri Deewani</t>
+        </is>
+      </c>
+      <c r="D37" s="0" t="inlineStr">
+        <is>
+          <t>Kailash Kher</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="0" t="inlineStr">
+        <is>
+          <t>2026-04-14</t>
+        </is>
+      </c>
+      <c r="B38" s="0" t="n">
+        <v>37</v>
+      </c>
+      <c r="C38" s="0" t="inlineStr">
+        <is>
+          <t>Run Down The City - Monica</t>
+        </is>
+      </c>
+      <c r="D38" s="0" t="inlineStr">
+        <is>
+          <t>Shashwat Sachdev</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="0" t="inlineStr">
+        <is>
+          <t>2026-04-14</t>
+        </is>
+      </c>
+      <c r="B39" s="0" t="n">
+        <v>38</v>
+      </c>
+      <c r="C39" s="0" t="inlineStr">
+        <is>
+          <t>Ye Tune Kya Kiya</t>
+        </is>
+      </c>
+      <c r="D39" s="0" t="inlineStr">
+        <is>
+          <t>Pritam</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="0" t="inlineStr">
+        <is>
+          <t>2026-04-14</t>
+        </is>
+      </c>
+      <c r="B40" s="0" t="n">
+        <v>39</v>
+      </c>
+      <c r="C40" s="0" t="inlineStr">
+        <is>
+          <t>Haseen</t>
+        </is>
+      </c>
+      <c r="D40" s="0" t="inlineStr">
+        <is>
+          <t>Talwiinder</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" s="0" t="inlineStr">
+        <is>
+          <t>2026-04-14</t>
+        </is>
+      </c>
+      <c r="B41" s="0" t="n">
+        <v>40</v>
+      </c>
+      <c r="C41" s="0" t="inlineStr">
+        <is>
+          <t>Lutt Le Gaya</t>
+        </is>
+      </c>
+      <c r="D41" s="0" t="inlineStr">
+        <is>
+          <t>Shashwat Sachdev</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" s="0" t="inlineStr">
+        <is>
+          <t>2026-04-14</t>
+        </is>
+      </c>
+      <c r="B42" s="0" t="n">
+        <v>41</v>
+      </c>
+      <c r="C42" s="0" t="inlineStr">
+        <is>
+          <t>Majboor</t>
+        </is>
+      </c>
+      <c r="D42" s="0" t="inlineStr">
+        <is>
+          <t>Sheheryar Rehan</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" s="0" t="inlineStr">
+        <is>
+          <t>2026-04-14</t>
+        </is>
+      </c>
+      <c r="B43" s="0" t="n">
+        <v>42</v>
+      </c>
+      <c r="C43" s="0" t="inlineStr">
+        <is>
+          <t>Barbaad</t>
+        </is>
+      </c>
+      <c r="D43" s="0" t="inlineStr">
+        <is>
+          <t>The Rish</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" s="0" t="inlineStr">
+        <is>
+          <t>2026-04-14</t>
+        </is>
+      </c>
+      <c r="B44" s="0" t="n">
+        <v>43</v>
+      </c>
+      <c r="C44" s="0" t="inlineStr">
+        <is>
+          <t>Jogi</t>
+        </is>
+      </c>
+      <c r="D44" s="0" t="inlineStr">
+        <is>
+          <t>thiarajxtt</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" s="0" t="inlineStr">
+        <is>
+          <t>2026-04-14</t>
+        </is>
+      </c>
+      <c r="B45" s="0" t="n">
+        <v>44</v>
+      </c>
+      <c r="C45" s="0" t="inlineStr">
+        <is>
+          <t>Mann Mera - Original Version</t>
+        </is>
+      </c>
+      <c r="D45" s="0" t="inlineStr">
+        <is>
+          <t>Gajendra Verma</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" s="0" t="inlineStr">
+        <is>
+          <t>2026-04-14</t>
+        </is>
+      </c>
+      <c r="B46" s="0" t="n">
+        <v>45</v>
+      </c>
+      <c r="C46" s="0" t="inlineStr">
+        <is>
+          <t>High On You</t>
+        </is>
+      </c>
+      <c r="D46" s="0" t="inlineStr">
+        <is>
+          <t>Jind Universe</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" s="0" t="inlineStr">
+        <is>
+          <t>2026-04-14</t>
+        </is>
+      </c>
+      <c r="B47" s="0" t="n">
+        <v>46</v>
+      </c>
+      <c r="C47" s="0" t="inlineStr">
+        <is>
+          <t>Thodi Si Daaru</t>
+        </is>
+      </c>
+      <c r="D47" s="0" t="inlineStr">
+        <is>
+          <t>AP Dhillon</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" s="0" t="inlineStr">
+        <is>
+          <t>2026-04-14</t>
+        </is>
+      </c>
+      <c r="B48" s="0" t="n">
+        <v>47</v>
+      </c>
+      <c r="C48" s="0" t="inlineStr">
+        <is>
+          <t>Mast Magan</t>
+        </is>
+      </c>
+      <c r="D48" s="0" t="inlineStr">
+        <is>
+          <t>Arijit Singh</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" s="0" t="inlineStr">
+        <is>
+          <t>2026-04-14</t>
+        </is>
+      </c>
+      <c r="B49" s="0" t="n">
+        <v>48</v>
+      </c>
+      <c r="C49" s="0" t="inlineStr">
+        <is>
+          <t>Not Guilty</t>
+        </is>
+      </c>
+      <c r="D49" s="0" t="inlineStr">
+        <is>
+          <t>Dhanda Nyoliwala</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" s="0" t="inlineStr">
+        <is>
+          <t>2026-04-14</t>
+        </is>
+      </c>
+      <c r="B50" s="0" t="n">
+        <v>49</v>
+      </c>
+      <c r="C50" s="0" t="inlineStr">
+        <is>
+          <t>Mutta Kalakki</t>
+        </is>
+      </c>
+      <c r="D50" s="0" t="inlineStr">
+        <is>
+          <t>G. V. Prakash</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" s="0" t="inlineStr">
+        <is>
+          <t>2026-04-14</t>
+        </is>
+      </c>
+      <c r="B51" s="0" t="n">
+        <v>50</v>
+      </c>
+      <c r="C51" s="0" t="inlineStr">
+        <is>
+          <t>Zaalima</t>
+        </is>
+      </c>
+      <c r="D51" s="0" t="inlineStr">
+        <is>
+          <t>Arijit Singh</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet32.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:D51"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="24" t="inlineStr">
+        <is>
+          <t>Date</t>
+        </is>
+      </c>
+      <c r="B1" s="24" t="inlineStr">
+        <is>
+          <t>Rank</t>
+        </is>
+      </c>
+      <c r="C1" s="24" t="inlineStr">
+        <is>
+          <t>Song</t>
+        </is>
+      </c>
+      <c r="D1" s="24" t="inlineStr">
+        <is>
+          <t>Artist</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="0" t="inlineStr">
+        <is>
+          <t>2026-04-13</t>
+        </is>
+      </c>
+      <c r="B2" s="0" t="n">
+        <v>1</v>
+      </c>
+      <c r="C2" s="0" t="inlineStr">
+        <is>
+          <t>Bairan</t>
+        </is>
+      </c>
+      <c r="D2" s="0" t="inlineStr">
+        <is>
+          <t>Banjaare</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="0" t="inlineStr">
+        <is>
+          <t>2026-04-13</t>
+        </is>
+      </c>
+      <c r="B3" s="0" t="n">
+        <v>2</v>
+      </c>
+      <c r="C3" s="0" t="inlineStr">
+        <is>
+          <t>Jaiye Sajana</t>
+        </is>
+      </c>
+      <c r="D3" s="0" t="inlineStr">
+        <is>
+          <t>Shashwat Sachdev</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="0" t="inlineStr">
+        <is>
+          <t>2026-04-13</t>
+        </is>
+      </c>
+      <c r="B4" s="0" t="n">
+        <v>3</v>
+      </c>
+      <c r="C4" s="0" t="inlineStr">
+        <is>
+          <t>Sheesha - Aakhya Mai Aakh Ghali Jo Bairan</t>
+        </is>
+      </c>
+      <c r="D4" s="0" t="inlineStr">
+        <is>
+          <t>Mitta Ror</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="0" t="inlineStr">
+        <is>
+          <t>2026-04-13</t>
+        </is>
+      </c>
+      <c r="B5" s="0" t="n">
+        <v>4</v>
+      </c>
+      <c r="C5" s="0" t="inlineStr">
+        <is>
+          <t>Gehra Hua</t>
+        </is>
+      </c>
+      <c r="D5" s="0" t="inlineStr">
+        <is>
+          <t>Shashwat Sachdev</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="0" t="inlineStr">
+        <is>
+          <t>2026-04-13</t>
+        </is>
+      </c>
+      <c r="B6" s="0" t="n">
+        <v>5</v>
+      </c>
+      <c r="C6" s="0" t="inlineStr">
+        <is>
+          <t>Khat</t>
+        </is>
+      </c>
+      <c r="D6" s="0" t="inlineStr">
+        <is>
+          <t>Navjot Ahuja</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="0" t="inlineStr">
+        <is>
+          <t>2026-04-13</t>
+        </is>
+      </c>
+      <c r="B7" s="0" t="n">
+        <v>6</v>
+      </c>
+      <c r="C7" s="0" t="inlineStr">
+        <is>
+          <t>Sitaare</t>
+        </is>
+      </c>
+      <c r="D7" s="0" t="inlineStr">
+        <is>
+          <t>Arijit Singh</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="0" t="inlineStr">
+        <is>
+          <t>2026-04-13</t>
+        </is>
+      </c>
+      <c r="B8" s="0" t="n">
+        <v>7</v>
+      </c>
+      <c r="C8" s="0" t="inlineStr">
+        <is>
+          <t>Dooron Dooron</t>
+        </is>
+      </c>
+      <c r="D8" s="0" t="inlineStr">
+        <is>
+          <t>Paresh Pahuja</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="0" t="inlineStr">
+        <is>
+          <t>2026-04-13</t>
+        </is>
+      </c>
+      <c r="B9" s="0" t="n">
+        <v>8</v>
+      </c>
+      <c r="C9" s="0" t="inlineStr">
+        <is>
+          <t>Sahiba</t>
+        </is>
+      </c>
+      <c r="D9" s="0" t="inlineStr">
+        <is>
+          <t>Aditya Rikhari</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="0" t="inlineStr">
+        <is>
+          <t>2026-04-13</t>
+        </is>
+      </c>
+      <c r="B10" s="0" t="n">
+        <v>9</v>
+      </c>
+      <c r="C10" s="0" t="inlineStr">
+        <is>
+          <t>Apna Bana Le</t>
+        </is>
+      </c>
+      <c r="D10" s="0" t="inlineStr">
+        <is>
+          <t>Sachin-Jigar</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="0" t="inlineStr">
+        <is>
+          <t>2026-04-13</t>
+        </is>
+      </c>
+      <c r="B11" s="0" t="n">
+        <v>10</v>
+      </c>
+      <c r="C11" s="0" t="inlineStr">
+        <is>
+          <t>Dhurandhar The Revenge - Aari Aari</t>
+        </is>
+      </c>
+      <c r="D11" s="0" t="inlineStr">
+        <is>
+          <t>Shashwat Sachdev</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="0" t="inlineStr">
+        <is>
+          <t>2026-04-13</t>
+        </is>
+      </c>
+      <c r="B12" s="0" t="n">
+        <v>11</v>
+      </c>
+      <c r="C12" s="0" t="inlineStr">
+        <is>
+          <t>Samjhawan</t>
+        </is>
+      </c>
+      <c r="D12" s="0" t="inlineStr">
+        <is>
+          <t>Jawad Ahmad</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="0" t="inlineStr">
+        <is>
+          <t>2026-04-13</t>
+        </is>
+      </c>
+      <c r="B13" s="0" t="n">
+        <v>12</v>
+      </c>
+      <c r="C13" s="0" t="inlineStr">
+        <is>
+          <t>Pavazha Malli</t>
+        </is>
+      </c>
+      <c r="D13" s="0" t="inlineStr">
+        <is>
+          <t>Sai Abhyankkar</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="0" t="inlineStr">
+        <is>
+          <t>2026-04-13</t>
+        </is>
+      </c>
+      <c r="B14" s="0" t="n">
+        <v>13</v>
+      </c>
+      <c r="C14" s="0" t="inlineStr">
+        <is>
+          <t>Finding Her</t>
+        </is>
+      </c>
+      <c r="D14" s="0" t="inlineStr">
+        <is>
+          <t>Kushagra</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="0" t="inlineStr">
+        <is>
+          <t>2026-04-13</t>
+        </is>
+      </c>
+      <c r="B15" s="0" t="n">
+        <v>14</v>
+      </c>
+      <c r="C15" s="0" t="inlineStr">
+        <is>
+          <t>Jaan Se Guzarte Hain</t>
+        </is>
+      </c>
+      <c r="D15" s="0" t="inlineStr">
+        <is>
+          <t>Shashwat Sachdev</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="0" t="inlineStr">
+        <is>
+          <t>2026-04-13</t>
+        </is>
+      </c>
+      <c r="B16" s="0" t="n">
+        <v>15</v>
+      </c>
+      <c r="C16" s="0" t="inlineStr">
+        <is>
+          <t>Arz Kiya Hai | Coke Studio Bharat</t>
+        </is>
+      </c>
+      <c r="D16" s="0" t="inlineStr">
+        <is>
+          <t>Anuv Jain</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="0" t="inlineStr">
+        <is>
+          <t>2026-04-13</t>
+        </is>
+      </c>
+      <c r="B17" s="0" t="n">
+        <v>16</v>
+      </c>
+      <c r="C17" s="0" t="inlineStr">
+        <is>
+          <t>Boyfriend</t>
+        </is>
+      </c>
+      <c r="D17" s="0" t="inlineStr">
+        <is>
+          <t>Karan Aujla</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="0" t="inlineStr">
+        <is>
+          <t>2026-04-13</t>
+        </is>
+      </c>
+      <c r="B18" s="0" t="n">
+        <v>17</v>
+      </c>
+      <c r="C18" s="0" t="inlineStr">
+        <is>
+          <t>Mann Mera</t>
+        </is>
+      </c>
+      <c r="D18" s="0" t="inlineStr">
+        <is>
+          <t>Gajendra Verma</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="0" t="inlineStr">
+        <is>
+          <t>2026-04-13</t>
+        </is>
+      </c>
+      <c r="B19" s="0" t="n">
+        <v>18</v>
+      </c>
+      <c r="C19" s="0" t="inlineStr">
+        <is>
+          <t>Ishq</t>
+        </is>
+      </c>
+      <c r="D19" s="0" t="inlineStr">
+        <is>
+          <t>Faheem Abdullah</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="0" t="inlineStr">
+        <is>
+          <t>2026-04-13</t>
+        </is>
+      </c>
+      <c r="B20" s="0" t="n">
+        <v>19</v>
+      </c>
+      <c r="C20" s="0" t="inlineStr">
+        <is>
+          <t>Shararat</t>
+        </is>
+      </c>
+      <c r="D20" s="0" t="inlineStr">
+        <is>
+          <t>Shashwat Sachdev</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="0" t="inlineStr">
+        <is>
+          <t>2026-04-13</t>
+        </is>
+      </c>
+      <c r="B21" s="0" t="n">
+        <v>20</v>
+      </c>
+      <c r="C21" s="0" t="inlineStr">
+        <is>
+          <t>Saiyaara</t>
+        </is>
+      </c>
+      <c r="D21" s="0" t="inlineStr">
+        <is>
+          <t>Tanishk Bagchi</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="0" t="inlineStr">
+        <is>
+          <t>2026-04-13</t>
+        </is>
+      </c>
+      <c r="B22" s="0" t="n">
+        <v>21</v>
+      </c>
+      <c r="C22" s="0" t="inlineStr">
+        <is>
+          <t>Darkhaast</t>
+        </is>
+      </c>
+      <c r="D22" s="0" t="inlineStr">
+        <is>
+          <t>Mithoon</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="0" t="inlineStr">
+        <is>
+          <t>2026-04-13</t>
+        </is>
+      </c>
+      <c r="B23" s="0" t="n">
+        <v>22</v>
+      </c>
+      <c r="C23" s="0" t="inlineStr">
+        <is>
+          <t>For A Reason</t>
+        </is>
+      </c>
+      <c r="D23" s="0" t="inlineStr">
+        <is>
+          <t>Karan Aujla</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="0" t="inlineStr">
+        <is>
+          <t>2026-04-13</t>
+        </is>
+      </c>
+      <c r="B24" s="0" t="n">
+        <v>23</v>
+      </c>
+      <c r="C24" s="0" t="inlineStr">
+        <is>
+          <t>Bairi</t>
+        </is>
+      </c>
+      <c r="D24" s="0" t="inlineStr">
+        <is>
+          <t>Virat</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="0" t="inlineStr">
+        <is>
+          <t>2026-04-13</t>
+        </is>
+      </c>
+      <c r="B25" s="0" t="n">
+        <v>24</v>
+      </c>
+      <c r="C25" s="0" t="inlineStr">
+        <is>
+          <t>Naal Nachna</t>
+        </is>
+      </c>
+      <c r="D25" s="0" t="inlineStr">
+        <is>
+          <t>Shashwat Sachdev</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="0" t="inlineStr">
+        <is>
+          <t>2026-04-13</t>
+        </is>
+      </c>
+      <c r="B26" s="0" t="n">
+        <v>25</v>
+      </c>
+      <c r="C26" s="0" t="inlineStr">
+        <is>
+          <t>Dhurandhar - Title Track</t>
+        </is>
+      </c>
+      <c r="D26" s="0" t="inlineStr">
+        <is>
+          <t>Shashwat Sachdev</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="0" t="inlineStr">
+        <is>
+          <t>2026-04-13</t>
+        </is>
+      </c>
+      <c r="B27" s="0" t="n">
+        <v>26</v>
+      </c>
+      <c r="C27" s="0" t="inlineStr">
+        <is>
+          <t>Tere Liye</t>
+        </is>
+      </c>
+      <c r="D27" s="0" t="inlineStr">
+        <is>
+          <t>Atif Aslam</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="0" t="inlineStr">
+        <is>
+          <t>2026-04-13</t>
+        </is>
+      </c>
+      <c r="B28" s="0" t="n">
+        <v>27</v>
+      </c>
+      <c r="C28" s="0" t="inlineStr">
+        <is>
+          <t>Tum Ho Toh</t>
+        </is>
+      </c>
+      <c r="D28" s="0" t="inlineStr">
+        <is>
+          <t>Vishal Mishra</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="0" t="inlineStr">
+        <is>
+          <t>2026-04-13</t>
+        </is>
+      </c>
+      <c r="B29" s="0" t="n">
+        <v>28</v>
+      </c>
+      <c r="C29" s="0" t="inlineStr">
+        <is>
+          <t>Ishqa Ve</t>
+        </is>
+      </c>
+      <c r="D29" s="0" t="inlineStr">
+        <is>
+          <t>Zeeshan Ali</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="0" t="inlineStr">
+        <is>
+          <t>2026-04-13</t>
+        </is>
+      </c>
+      <c r="B30" s="0" t="n">
+        <v>29</v>
+      </c>
+      <c r="C30" s="0" t="inlineStr">
+        <is>
+          <t>Deewaana Deewaana</t>
+        </is>
+      </c>
+      <c r="D30" s="0" t="inlineStr">
+        <is>
+          <t>A.R. Rahman</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="0" t="inlineStr">
+        <is>
+          <t>2026-04-13</t>
+        </is>
+      </c>
+      <c r="B31" s="0" t="n">
+        <v>30</v>
+      </c>
+      <c r="C31" s="0" t="inlineStr">
+        <is>
+          <t>Phir Se</t>
+        </is>
+      </c>
+      <c r="D31" s="0" t="inlineStr">
+        <is>
+          <t>Shashwat Sachdev</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="0" t="inlineStr">
+        <is>
+          <t>2026-04-13</t>
+        </is>
+      </c>
+      <c r="B32" s="0" t="n">
+        <v>31</v>
+      </c>
+      <c r="C32" s="0" t="inlineStr">
+        <is>
+          <t>Jo Tum Mere Ho</t>
+        </is>
+      </c>
+      <c r="D32" s="0" t="inlineStr">
+        <is>
+          <t>Anuv Jain</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="0" t="inlineStr">
+        <is>
+          <t>2026-04-13</t>
+        </is>
+      </c>
+      <c r="B33" s="0" t="n">
+        <v>32</v>
+      </c>
+      <c r="C33" s="0" t="inlineStr">
+        <is>
+          <t>Raanjhan</t>
+        </is>
+      </c>
+      <c r="D33" s="0" t="inlineStr">
+        <is>
+          <t>Sachet-Parampara</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="0" t="inlineStr">
+        <is>
+          <t>2026-04-13</t>
+        </is>
+      </c>
+      <c r="B34" s="0" t="n">
+        <v>33</v>
+      </c>
+      <c r="C34" s="0" t="inlineStr">
+        <is>
+          <t>Agar Tum Saath Ho</t>
+        </is>
+      </c>
+      <c r="D34" s="0" t="inlineStr">
+        <is>
+          <t>Alka Yagnik</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="0" t="inlineStr">
+        <is>
+          <t>2026-04-13</t>
+        </is>
+      </c>
+      <c r="B35" s="0" t="n">
+        <v>34</v>
+      </c>
+      <c r="C35" s="0" t="inlineStr">
+        <is>
+          <t>Tere Bina</t>
+        </is>
+      </c>
+      <c r="D35" s="0" t="inlineStr">
+        <is>
+          <t>A.R. Rahman</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="0" t="inlineStr">
+        <is>
+          <t>2026-04-13</t>
+        </is>
+      </c>
+      <c r="B36" s="0" t="n">
+        <v>35</v>
+      </c>
+      <c r="C36" s="0" t="inlineStr">
+        <is>
+          <t>Lutt Le Gaya</t>
+        </is>
+      </c>
+      <c r="D36" s="0" t="inlineStr">
+        <is>
+          <t>Shashwat Sachdev</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="0" t="inlineStr">
+        <is>
+          <t>2026-04-13</t>
+        </is>
+      </c>
+      <c r="B37" s="0" t="n">
+        <v>36</v>
+      </c>
+      <c r="C37" s="0" t="inlineStr">
+        <is>
+          <t>Ehsaas</t>
+        </is>
+      </c>
+      <c r="D37" s="0" t="inlineStr">
+        <is>
+          <t>Faheem Abdullah</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="0" t="inlineStr">
+        <is>
+          <t>2026-04-13</t>
+        </is>
+      </c>
+      <c r="B38" s="0" t="n">
+        <v>37</v>
+      </c>
+      <c r="C38" s="0" t="inlineStr">
+        <is>
+          <t>Ye Tune Kya Kiya</t>
+        </is>
+      </c>
+      <c r="D38" s="0" t="inlineStr">
+        <is>
+          <t>Pritam</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="0" t="inlineStr">
+        <is>
+          <t>2026-04-13</t>
+        </is>
+      </c>
+      <c r="B39" s="0" t="n">
+        <v>38</v>
+      </c>
+      <c r="C39" s="0" t="inlineStr">
+        <is>
+          <t>Barbaad</t>
+        </is>
+      </c>
+      <c r="D39" s="0" t="inlineStr">
+        <is>
+          <t>The Rish</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="0" t="inlineStr">
+        <is>
+          <t>2026-04-13</t>
+        </is>
+      </c>
+      <c r="B40" s="0" t="n">
+        <v>39</v>
+      </c>
+      <c r="C40" s="0" t="inlineStr">
+        <is>
+          <t>Teri Deewani</t>
+        </is>
+      </c>
+      <c r="D40" s="0" t="inlineStr">
+        <is>
+          <t>Kailash Kher</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" s="0" t="inlineStr">
+        <is>
+          <t>2026-04-13</t>
+        </is>
+      </c>
+      <c r="B41" s="0" t="n">
+        <v>40</v>
+      </c>
+      <c r="C41" s="0" t="inlineStr">
+        <is>
+          <t>Haseen</t>
+        </is>
+      </c>
+      <c r="D41" s="0" t="inlineStr">
+        <is>
+          <t>Talwiinder</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" s="0" t="inlineStr">
+        <is>
+          <t>2026-04-13</t>
+        </is>
+      </c>
+      <c r="B42" s="0" t="n">
+        <v>41</v>
+      </c>
+      <c r="C42" s="0" t="inlineStr">
+        <is>
+          <t>Run Down The City - Monica</t>
+        </is>
+      </c>
+      <c r="D42" s="0" t="inlineStr">
+        <is>
+          <t>Shashwat Sachdev</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" s="0" t="inlineStr">
+        <is>
+          <t>2026-04-13</t>
+        </is>
+      </c>
+      <c r="B43" s="0" t="n">
+        <v>42</v>
+      </c>
+      <c r="C43" s="0" t="inlineStr">
+        <is>
+          <t>Jogi</t>
+        </is>
+      </c>
+      <c r="D43" s="0" t="inlineStr">
+        <is>
+          <t>thiarajxtt</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" s="0" t="inlineStr">
+        <is>
+          <t>2026-04-13</t>
+        </is>
+      </c>
+      <c r="B44" s="0" t="n">
+        <v>43</v>
+      </c>
+      <c r="C44" s="0" t="inlineStr">
+        <is>
+          <t>Mast Magan</t>
+        </is>
+      </c>
+      <c r="D44" s="0" t="inlineStr">
+        <is>
+          <t>Arijit Singh</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" s="0" t="inlineStr">
+        <is>
+          <t>2026-04-13</t>
+        </is>
+      </c>
+      <c r="B45" s="0" t="n">
+        <v>44</v>
+      </c>
+      <c r="C45" s="0" t="inlineStr">
+        <is>
+          <t>Mann Mera - Original Version</t>
+        </is>
+      </c>
+      <c r="D45" s="0" t="inlineStr">
+        <is>
+          <t>Gajendra Verma</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" s="0" t="inlineStr">
+        <is>
+          <t>2026-04-13</t>
+        </is>
+      </c>
+      <c r="B46" s="0" t="n">
+        <v>45</v>
+      </c>
+      <c r="C46" s="0" t="inlineStr">
+        <is>
+          <t>Zaalima</t>
+        </is>
+      </c>
+      <c r="D46" s="0" t="inlineStr">
+        <is>
+          <t>Arijit Singh</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" s="0" t="inlineStr">
+        <is>
+          <t>2026-04-13</t>
+        </is>
+      </c>
+      <c r="B47" s="0" t="n">
+        <v>46</v>
+      </c>
+      <c r="C47" s="0" t="inlineStr">
+        <is>
+          <t>Not Guilty</t>
+        </is>
+      </c>
+      <c r="D47" s="0" t="inlineStr">
+        <is>
+          <t>Dhanda Nyoliwala</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" s="0" t="inlineStr">
+        <is>
+          <t>2026-04-13</t>
+        </is>
+      </c>
+      <c r="B48" s="0" t="n">
+        <v>47</v>
+      </c>
+      <c r="C48" s="0" t="inlineStr">
+        <is>
+          <t>Mutta Kalakki</t>
+        </is>
+      </c>
+      <c r="D48" s="0" t="inlineStr">
+        <is>
+          <t>G. V. Prakash</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" s="0" t="inlineStr">
+        <is>
+          <t>2026-04-13</t>
+        </is>
+      </c>
+      <c r="B49" s="0" t="n">
+        <v>48</v>
+      </c>
+      <c r="C49" s="0" t="inlineStr">
+        <is>
+          <t>Ishq Jalakar - Karvaan</t>
+        </is>
+      </c>
+      <c r="D49" s="0" t="inlineStr">
+        <is>
+          <t>Shashwat Sachdev</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" s="0" t="inlineStr">
+        <is>
+          <t>2026-04-13</t>
+        </is>
+      </c>
+      <c r="B50" s="0" t="n">
+        <v>49</v>
+      </c>
+      <c r="C50" s="0" t="inlineStr">
+        <is>
+          <t>Jhol - Acoustic</t>
+        </is>
+      </c>
+      <c r="D50" s="0" t="inlineStr">
+        <is>
+          <t>Maanu</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" s="0" t="inlineStr">
+        <is>
+          <t>2026-04-13</t>
+        </is>
+      </c>
+      <c r="B51" s="0" t="n">
+        <v>50</v>
+      </c>
+      <c r="C51" s="0" t="inlineStr">
+        <is>
+          <t>Thodi Si Daaru</t>
+        </is>
+      </c>
+      <c r="D51" s="0" t="inlineStr">
+        <is>
+          <t>AP Dhillon</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
got data for 15th and predictions for 16th
</commit_message>
<xml_diff>
--- a/Probability Project.xlsx
+++ b/Probability Project.xlsx
@@ -35,6 +35,7 @@
     <sheet name="AUTO_20260412" sheetId="30" state="visible" r:id="rId30"/>
     <sheet name="AUTO_20260414" sheetId="31" state="visible" r:id="rId31"/>
     <sheet name="AUTO_20260413" sheetId="32" state="visible" r:id="rId32"/>
+    <sheet name="AUTO_20260415" sheetId="33" state="visible" r:id="rId33"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -21223,1000 +21224,1000 @@
       </c>
     </row>
     <row r="2">
-      <c r="A2" t="inlineStr">
+      <c r="A2" s="0" t="inlineStr">
         <is>
           <t>2026-04-08</t>
         </is>
       </c>
-      <c r="B2" t="n">
+      <c r="B2" s="0" t="n">
         <v>1</v>
       </c>
-      <c r="C2" t="inlineStr">
+      <c r="C2" s="0" t="inlineStr">
         <is>
           <t>Bairan</t>
         </is>
       </c>
-      <c r="D2" t="inlineStr">
+      <c r="D2" s="0" t="inlineStr">
         <is>
           <t>Banjaare</t>
         </is>
       </c>
     </row>
     <row r="3">
-      <c r="A3" t="inlineStr">
+      <c r="A3" s="0" t="inlineStr">
         <is>
           <t>2026-04-08</t>
         </is>
       </c>
-      <c r="B3" t="n">
+      <c r="B3" s="0" t="n">
         <v>2</v>
       </c>
-      <c r="C3" t="inlineStr">
+      <c r="C3" s="0" t="inlineStr">
         <is>
           <t>Jaiye Sajana</t>
         </is>
       </c>
-      <c r="D3" t="inlineStr">
+      <c r="D3" s="0" t="inlineStr">
         <is>
           <t>Shashwat Sachdev</t>
         </is>
       </c>
     </row>
     <row r="4">
-      <c r="A4" t="inlineStr">
+      <c r="A4" s="0" t="inlineStr">
         <is>
           <t>2026-04-08</t>
         </is>
       </c>
-      <c r="B4" t="n">
+      <c r="B4" s="0" t="n">
         <v>3</v>
       </c>
-      <c r="C4" t="inlineStr">
+      <c r="C4" s="0" t="inlineStr">
         <is>
           <t>Gehra Hua</t>
         </is>
       </c>
-      <c r="D4" t="inlineStr">
+      <c r="D4" s="0" t="inlineStr">
         <is>
           <t>Shashwat Sachdev</t>
         </is>
       </c>
     </row>
     <row r="5">
-      <c r="A5" t="inlineStr">
+      <c r="A5" s="0" t="inlineStr">
         <is>
           <t>2026-04-08</t>
         </is>
       </c>
-      <c r="B5" t="n">
+      <c r="B5" s="0" t="n">
         <v>4</v>
       </c>
-      <c r="C5" t="inlineStr">
+      <c r="C5" s="0" t="inlineStr">
         <is>
           <t>Sheesha - Aakhya Mai Aakh Ghali Jo Bairan</t>
         </is>
       </c>
-      <c r="D5" t="inlineStr">
+      <c r="D5" s="0" t="inlineStr">
         <is>
           <t>Mitta Ror</t>
         </is>
       </c>
     </row>
     <row r="6">
-      <c r="A6" t="inlineStr">
+      <c r="A6" s="0" t="inlineStr">
         <is>
           <t>2026-04-08</t>
         </is>
       </c>
-      <c r="B6" t="n">
+      <c r="B6" s="0" t="n">
         <v>5</v>
       </c>
-      <c r="C6" t="inlineStr">
+      <c r="C6" s="0" t="inlineStr">
         <is>
           <t>Khat</t>
         </is>
       </c>
-      <c r="D6" t="inlineStr">
+      <c r="D6" s="0" t="inlineStr">
         <is>
           <t>Navjot Ahuja</t>
         </is>
       </c>
     </row>
     <row r="7">
-      <c r="A7" t="inlineStr">
+      <c r="A7" s="0" t="inlineStr">
         <is>
           <t>2026-04-08</t>
         </is>
       </c>
-      <c r="B7" t="n">
+      <c r="B7" s="0" t="n">
         <v>6</v>
       </c>
-      <c r="C7" t="inlineStr">
+      <c r="C7" s="0" t="inlineStr">
         <is>
           <t>Dhurandhar The Revenge - Aari Aari</t>
         </is>
       </c>
-      <c r="D7" t="inlineStr">
+      <c r="D7" s="0" t="inlineStr">
         <is>
           <t>Shashwat Sachdev</t>
         </is>
       </c>
     </row>
     <row r="8">
-      <c r="A8" t="inlineStr">
+      <c r="A8" s="0" t="inlineStr">
         <is>
           <t>2026-04-08</t>
         </is>
       </c>
-      <c r="B8" t="n">
+      <c r="B8" s="0" t="n">
         <v>7</v>
       </c>
-      <c r="C8" t="inlineStr">
+      <c r="C8" s="0" t="inlineStr">
         <is>
           <t>Dooron Dooron</t>
         </is>
       </c>
-      <c r="D8" t="inlineStr">
+      <c r="D8" s="0" t="inlineStr">
         <is>
           <t>Paresh Pahuja</t>
         </is>
       </c>
     </row>
     <row r="9">
-      <c r="A9" t="inlineStr">
+      <c r="A9" s="0" t="inlineStr">
         <is>
           <t>2026-04-08</t>
         </is>
       </c>
-      <c r="B9" t="n">
+      <c r="B9" s="0" t="n">
         <v>8</v>
       </c>
-      <c r="C9" t="inlineStr">
+      <c r="C9" s="0" t="inlineStr">
         <is>
           <t>Apna Bana Le</t>
         </is>
       </c>
-      <c r="D9" t="inlineStr">
+      <c r="D9" s="0" t="inlineStr">
         <is>
           <t>Sachin-Jigar</t>
         </is>
       </c>
     </row>
     <row r="10">
-      <c r="A10" t="inlineStr">
+      <c r="A10" s="0" t="inlineStr">
         <is>
           <t>2026-04-08</t>
         </is>
       </c>
-      <c r="B10" t="n">
+      <c r="B10" s="0" t="n">
         <v>9</v>
       </c>
-      <c r="C10" t="inlineStr">
+      <c r="C10" s="0" t="inlineStr">
         <is>
           <t>Sahiba</t>
         </is>
       </c>
-      <c r="D10" t="inlineStr">
+      <c r="D10" s="0" t="inlineStr">
         <is>
           <t>Aditya Rikhari</t>
         </is>
       </c>
     </row>
     <row r="11">
-      <c r="A11" t="inlineStr">
+      <c r="A11" s="0" t="inlineStr">
         <is>
           <t>2026-04-08</t>
         </is>
       </c>
-      <c r="B11" t="n">
+      <c r="B11" s="0" t="n">
         <v>10</v>
       </c>
-      <c r="C11" t="inlineStr">
+      <c r="C11" s="0" t="inlineStr">
         <is>
           <t>Sitaare</t>
         </is>
       </c>
-      <c r="D11" t="inlineStr">
+      <c r="D11" s="0" t="inlineStr">
         <is>
           <t>Arijit Singh</t>
         </is>
       </c>
     </row>
     <row r="12">
-      <c r="A12" t="inlineStr">
+      <c r="A12" s="0" t="inlineStr">
         <is>
           <t>2026-04-08</t>
         </is>
       </c>
-      <c r="B12" t="n">
+      <c r="B12" s="0" t="n">
         <v>11</v>
       </c>
-      <c r="C12" t="inlineStr">
+      <c r="C12" s="0" t="inlineStr">
         <is>
           <t>Samjhawan</t>
         </is>
       </c>
-      <c r="D12" t="inlineStr">
+      <c r="D12" s="0" t="inlineStr">
         <is>
           <t>Jawad Ahmad</t>
         </is>
       </c>
     </row>
     <row r="13">
-      <c r="A13" t="inlineStr">
+      <c r="A13" s="0" t="inlineStr">
         <is>
           <t>2026-04-08</t>
         </is>
       </c>
-      <c r="B13" t="n">
+      <c r="B13" s="0" t="n">
         <v>12</v>
       </c>
-      <c r="C13" t="inlineStr">
+      <c r="C13" s="0" t="inlineStr">
         <is>
           <t>Jaan Se Guzarte Hain</t>
         </is>
       </c>
-      <c r="D13" t="inlineStr">
+      <c r="D13" s="0" t="inlineStr">
         <is>
           <t>Shashwat Sachdev</t>
         </is>
       </c>
     </row>
     <row r="14">
-      <c r="A14" t="inlineStr">
+      <c r="A14" s="0" t="inlineStr">
         <is>
           <t>2026-04-08</t>
         </is>
       </c>
-      <c r="B14" t="n">
+      <c r="B14" s="0" t="n">
         <v>13</v>
       </c>
-      <c r="C14" t="inlineStr">
+      <c r="C14" s="0" t="inlineStr">
         <is>
           <t>Finding Her</t>
         </is>
       </c>
-      <c r="D14" t="inlineStr">
+      <c r="D14" s="0" t="inlineStr">
         <is>
           <t>Kushagra</t>
         </is>
       </c>
     </row>
     <row r="15">
-      <c r="A15" t="inlineStr">
+      <c r="A15" s="0" t="inlineStr">
         <is>
           <t>2026-04-08</t>
         </is>
       </c>
-      <c r="B15" t="n">
+      <c r="B15" s="0" t="n">
         <v>14</v>
       </c>
-      <c r="C15" t="inlineStr">
+      <c r="C15" s="0" t="inlineStr">
         <is>
           <t>Boyfriend</t>
         </is>
       </c>
-      <c r="D15" t="inlineStr">
+      <c r="D15" s="0" t="inlineStr">
         <is>
           <t>Karan Aujla</t>
         </is>
       </c>
     </row>
     <row r="16">
-      <c r="A16" t="inlineStr">
+      <c r="A16" s="0" t="inlineStr">
         <is>
           <t>2026-04-08</t>
         </is>
       </c>
-      <c r="B16" t="n">
+      <c r="B16" s="0" t="n">
         <v>15</v>
       </c>
-      <c r="C16" t="inlineStr">
+      <c r="C16" s="0" t="inlineStr">
         <is>
           <t>Pavazha Malli</t>
         </is>
       </c>
-      <c r="D16" t="inlineStr">
+      <c r="D16" s="0" t="inlineStr">
         <is>
           <t>Sai Abhyankkar</t>
         </is>
       </c>
     </row>
     <row r="17">
-      <c r="A17" t="inlineStr">
+      <c r="A17" s="0" t="inlineStr">
         <is>
           <t>2026-04-08</t>
         </is>
       </c>
-      <c r="B17" t="n">
+      <c r="B17" s="0" t="n">
         <v>16</v>
       </c>
-      <c r="C17" t="inlineStr">
+      <c r="C17" s="0" t="inlineStr">
         <is>
           <t>Arz Kiya Hai | Coke Studio Bharat</t>
         </is>
       </c>
-      <c r="D17" t="inlineStr">
+      <c r="D17" s="0" t="inlineStr">
         <is>
           <t>Anuv Jain</t>
         </is>
       </c>
     </row>
     <row r="18">
-      <c r="A18" t="inlineStr">
+      <c r="A18" s="0" t="inlineStr">
         <is>
           <t>2026-04-08</t>
         </is>
       </c>
-      <c r="B18" t="n">
+      <c r="B18" s="0" t="n">
         <v>17</v>
       </c>
-      <c r="C18" t="inlineStr">
+      <c r="C18" s="0" t="inlineStr">
         <is>
           <t>Shararat</t>
         </is>
       </c>
-      <c r="D18" t="inlineStr">
+      <c r="D18" s="0" t="inlineStr">
         <is>
           <t>Shashwat Sachdev</t>
         </is>
       </c>
     </row>
     <row r="19">
-      <c r="A19" t="inlineStr">
+      <c r="A19" s="0" t="inlineStr">
         <is>
           <t>2026-04-08</t>
         </is>
       </c>
-      <c r="B19" t="n">
+      <c r="B19" s="0" t="n">
         <v>18</v>
       </c>
-      <c r="C19" t="inlineStr">
+      <c r="C19" s="0" t="inlineStr">
         <is>
           <t>Ishq</t>
         </is>
       </c>
-      <c r="D19" t="inlineStr">
+      <c r="D19" s="0" t="inlineStr">
         <is>
           <t>Faheem Abdullah</t>
         </is>
       </c>
     </row>
     <row r="20">
-      <c r="A20" t="inlineStr">
+      <c r="A20" s="0" t="inlineStr">
         <is>
           <t>2026-04-08</t>
         </is>
       </c>
-      <c r="B20" t="n">
+      <c r="B20" s="0" t="n">
         <v>19</v>
       </c>
-      <c r="C20" t="inlineStr">
+      <c r="C20" s="0" t="inlineStr">
         <is>
           <t>Mann Mera</t>
         </is>
       </c>
-      <c r="D20" t="inlineStr">
+      <c r="D20" s="0" t="inlineStr">
         <is>
           <t>Gajendra Verma</t>
         </is>
       </c>
     </row>
     <row r="21">
-      <c r="A21" t="inlineStr">
+      <c r="A21" s="0" t="inlineStr">
         <is>
           <t>2026-04-08</t>
         </is>
       </c>
-      <c r="B21" t="n">
+      <c r="B21" s="0" t="n">
         <v>20</v>
       </c>
-      <c r="C21" t="inlineStr">
+      <c r="C21" s="0" t="inlineStr">
         <is>
           <t>Saiyaara</t>
         </is>
       </c>
-      <c r="D21" t="inlineStr">
+      <c r="D21" s="0" t="inlineStr">
         <is>
           <t>Tanishk Bagchi</t>
         </is>
       </c>
     </row>
     <row r="22">
-      <c r="A22" t="inlineStr">
+      <c r="A22" s="0" t="inlineStr">
         <is>
           <t>2026-04-08</t>
         </is>
       </c>
-      <c r="B22" t="n">
+      <c r="B22" s="0" t="n">
         <v>21</v>
       </c>
-      <c r="C22" t="inlineStr">
+      <c r="C22" s="0" t="inlineStr">
         <is>
           <t>Darkhaast</t>
         </is>
       </c>
-      <c r="D22" t="inlineStr">
+      <c r="D22" s="0" t="inlineStr">
         <is>
           <t>Mithoon</t>
         </is>
       </c>
     </row>
     <row r="23">
-      <c r="A23" t="inlineStr">
+      <c r="A23" s="0" t="inlineStr">
         <is>
           <t>2026-04-08</t>
         </is>
       </c>
-      <c r="B23" t="n">
+      <c r="B23" s="0" t="n">
         <v>22</v>
       </c>
-      <c r="C23" t="inlineStr">
+      <c r="C23" s="0" t="inlineStr">
         <is>
           <t>Ishqa Ve</t>
         </is>
       </c>
-      <c r="D23" t="inlineStr">
+      <c r="D23" s="0" t="inlineStr">
         <is>
           <t>Zeeshan Ali</t>
         </is>
       </c>
     </row>
     <row r="24">
-      <c r="A24" t="inlineStr">
+      <c r="A24" s="0" t="inlineStr">
         <is>
           <t>2026-04-08</t>
         </is>
       </c>
-      <c r="B24" t="n">
+      <c r="B24" s="0" t="n">
         <v>23</v>
       </c>
-      <c r="C24" t="inlineStr">
+      <c r="C24" s="0" t="inlineStr">
         <is>
           <t>Tum Ho Toh</t>
         </is>
       </c>
-      <c r="D24" t="inlineStr">
+      <c r="D24" s="0" t="inlineStr">
         <is>
           <t>Vishal Mishra</t>
         </is>
       </c>
     </row>
     <row r="25">
-      <c r="A25" t="inlineStr">
+      <c r="A25" s="0" t="inlineStr">
         <is>
           <t>2026-04-08</t>
         </is>
       </c>
-      <c r="B25" t="n">
+      <c r="B25" s="0" t="n">
         <v>24</v>
       </c>
-      <c r="C25" t="inlineStr">
+      <c r="C25" s="0" t="inlineStr">
         <is>
           <t>Dhurandhar - Title Track</t>
         </is>
       </c>
-      <c r="D25" t="inlineStr">
+      <c r="D25" s="0" t="inlineStr">
         <is>
           <t>Shashwat Sachdev</t>
         </is>
       </c>
     </row>
     <row r="26">
-      <c r="A26" t="inlineStr">
+      <c r="A26" s="0" t="inlineStr">
         <is>
           <t>2026-04-08</t>
         </is>
       </c>
-      <c r="B26" t="n">
+      <c r="B26" s="0" t="n">
         <v>25</v>
       </c>
-      <c r="C26" t="inlineStr">
+      <c r="C26" s="0" t="inlineStr">
         <is>
           <t>Naal Nachna</t>
         </is>
       </c>
-      <c r="D26" t="inlineStr">
+      <c r="D26" s="0" t="inlineStr">
         <is>
           <t>Shashwat Sachdev</t>
         </is>
       </c>
     </row>
     <row r="27">
-      <c r="A27" t="inlineStr">
+      <c r="A27" s="0" t="inlineStr">
         <is>
           <t>2026-04-08</t>
         </is>
       </c>
-      <c r="B27" t="n">
+      <c r="B27" s="0" t="n">
         <v>26</v>
       </c>
-      <c r="C27" t="inlineStr">
+      <c r="C27" s="0" t="inlineStr">
         <is>
           <t>For A Reason</t>
         </is>
       </c>
-      <c r="D27" t="inlineStr">
+      <c r="D27" s="0" t="inlineStr">
         <is>
           <t>Karan Aujla</t>
         </is>
       </c>
     </row>
     <row r="28">
-      <c r="A28" t="inlineStr">
+      <c r="A28" s="0" t="inlineStr">
         <is>
           <t>2026-04-08</t>
         </is>
       </c>
-      <c r="B28" t="n">
+      <c r="B28" s="0" t="n">
         <v>27</v>
       </c>
-      <c r="C28" t="inlineStr">
+      <c r="C28" s="0" t="inlineStr">
         <is>
           <t>Raanjhan</t>
         </is>
       </c>
-      <c r="D28" t="inlineStr">
+      <c r="D28" s="0" t="inlineStr">
         <is>
           <t>Sachet-Parampara</t>
         </is>
       </c>
     </row>
     <row r="29">
-      <c r="A29" t="inlineStr">
+      <c r="A29" s="0" t="inlineStr">
         <is>
           <t>2026-04-08</t>
         </is>
       </c>
-      <c r="B29" t="n">
+      <c r="B29" s="0" t="n">
         <v>28</v>
       </c>
-      <c r="C29" t="inlineStr">
+      <c r="C29" s="0" t="inlineStr">
         <is>
           <t>Deewaana Deewaana</t>
         </is>
       </c>
-      <c r="D29" t="inlineStr">
+      <c r="D29" s="0" t="inlineStr">
         <is>
           <t>A.R. Rahman</t>
         </is>
       </c>
     </row>
     <row r="30">
-      <c r="A30" t="inlineStr">
+      <c r="A30" s="0" t="inlineStr">
         <is>
           <t>2026-04-08</t>
         </is>
       </c>
-      <c r="B30" t="n">
+      <c r="B30" s="0" t="n">
         <v>29</v>
       </c>
-      <c r="C30" t="inlineStr">
+      <c r="C30" s="0" t="inlineStr">
         <is>
           <t>Bairi</t>
         </is>
       </c>
-      <c r="D30" t="inlineStr">
+      <c r="D30" s="0" t="inlineStr">
         <is>
           <t>Virat</t>
         </is>
       </c>
     </row>
     <row r="31">
-      <c r="A31" t="inlineStr">
+      <c r="A31" s="0" t="inlineStr">
         <is>
           <t>2026-04-08</t>
         </is>
       </c>
-      <c r="B31" t="n">
+      <c r="B31" s="0" t="n">
         <v>30</v>
       </c>
-      <c r="C31" t="inlineStr">
+      <c r="C31" s="0" t="inlineStr">
         <is>
           <t>Jo Tum Mere Ho</t>
         </is>
       </c>
-      <c r="D31" t="inlineStr">
+      <c r="D31" s="0" t="inlineStr">
         <is>
           <t>Anuv Jain</t>
         </is>
       </c>
     </row>
     <row r="32">
-      <c r="A32" t="inlineStr">
+      <c r="A32" s="0" t="inlineStr">
         <is>
           <t>2026-04-08</t>
         </is>
       </c>
-      <c r="B32" t="n">
+      <c r="B32" s="0" t="n">
         <v>31</v>
       </c>
-      <c r="C32" t="inlineStr">
+      <c r="C32" s="0" t="inlineStr">
         <is>
           <t>Tere Liye</t>
         </is>
       </c>
-      <c r="D32" t="inlineStr">
+      <c r="D32" s="0" t="inlineStr">
         <is>
           <t>Atif Aslam</t>
         </is>
       </c>
     </row>
     <row r="33">
-      <c r="A33" t="inlineStr">
+      <c r="A33" s="0" t="inlineStr">
         <is>
           <t>2026-04-08</t>
         </is>
       </c>
-      <c r="B33" t="n">
+      <c r="B33" s="0" t="n">
         <v>32</v>
       </c>
-      <c r="C33" t="inlineStr">
+      <c r="C33" s="0" t="inlineStr">
         <is>
           <t>Phir Se</t>
         </is>
       </c>
-      <c r="D33" t="inlineStr">
+      <c r="D33" s="0" t="inlineStr">
         <is>
           <t>Shashwat Sachdev</t>
         </is>
       </c>
     </row>
     <row r="34">
-      <c r="A34" t="inlineStr">
+      <c r="A34" s="0" t="inlineStr">
         <is>
           <t>2026-04-08</t>
         </is>
       </c>
-      <c r="B34" t="n">
+      <c r="B34" s="0" t="n">
         <v>33</v>
       </c>
-      <c r="C34" t="inlineStr">
+      <c r="C34" s="0" t="inlineStr">
         <is>
           <t>Agar Tum Saath Ho</t>
         </is>
       </c>
-      <c r="D34" t="inlineStr">
+      <c r="D34" s="0" t="inlineStr">
         <is>
           <t>Alka Yagnik</t>
         </is>
       </c>
     </row>
     <row r="35">
-      <c r="A35" t="inlineStr">
+      <c r="A35" s="0" t="inlineStr">
         <is>
           <t>2026-04-08</t>
         </is>
       </c>
-      <c r="B35" t="n">
+      <c r="B35" s="0" t="n">
         <v>34</v>
       </c>
-      <c r="C35" t="inlineStr">
+      <c r="C35" s="0" t="inlineStr">
         <is>
           <t>Tere Bina</t>
         </is>
       </c>
-      <c r="D35" t="inlineStr">
+      <c r="D35" s="0" t="inlineStr">
         <is>
           <t>A.R. Rahman</t>
         </is>
       </c>
     </row>
     <row r="36">
-      <c r="A36" t="inlineStr">
+      <c r="A36" s="0" t="inlineStr">
         <is>
           <t>2026-04-08</t>
         </is>
       </c>
-      <c r="B36" t="n">
+      <c r="B36" s="0" t="n">
         <v>35</v>
       </c>
-      <c r="C36" t="inlineStr">
+      <c r="C36" s="0" t="inlineStr">
         <is>
           <t>Run Down The City - Monica</t>
         </is>
       </c>
-      <c r="D36" t="inlineStr">
+      <c r="D36" s="0" t="inlineStr">
         <is>
           <t>Shashwat Sachdev</t>
         </is>
       </c>
     </row>
     <row r="37">
-      <c r="A37" t="inlineStr">
+      <c r="A37" s="0" t="inlineStr">
         <is>
           <t>2026-04-08</t>
         </is>
       </c>
-      <c r="B37" t="n">
+      <c r="B37" s="0" t="n">
         <v>36</v>
       </c>
-      <c r="C37" t="inlineStr">
+      <c r="C37" s="0" t="inlineStr">
         <is>
           <t>Haseen</t>
         </is>
       </c>
-      <c r="D37" t="inlineStr">
+      <c r="D37" s="0" t="inlineStr">
         <is>
           <t>Talwiinder</t>
         </is>
       </c>
     </row>
     <row r="38">
-      <c r="A38" t="inlineStr">
+      <c r="A38" s="0" t="inlineStr">
         <is>
           <t>2026-04-08</t>
         </is>
       </c>
-      <c r="B38" t="n">
+      <c r="B38" s="0" t="n">
         <v>37</v>
       </c>
-      <c r="C38" t="inlineStr">
+      <c r="C38" s="0" t="inlineStr">
         <is>
           <t>Barbaad</t>
         </is>
       </c>
-      <c r="D38" t="inlineStr">
+      <c r="D38" s="0" t="inlineStr">
         <is>
           <t>The Rish</t>
         </is>
       </c>
     </row>
     <row r="39">
-      <c r="A39" t="inlineStr">
+      <c r="A39" s="0" t="inlineStr">
         <is>
           <t>2026-04-08</t>
         </is>
       </c>
-      <c r="B39" t="n">
+      <c r="B39" s="0" t="n">
         <v>38</v>
       </c>
-      <c r="C39" t="inlineStr">
+      <c r="C39" s="0" t="inlineStr">
         <is>
           <t>Lutt Le Gaya</t>
         </is>
       </c>
-      <c r="D39" t="inlineStr">
+      <c r="D39" s="0" t="inlineStr">
         <is>
           <t>Shashwat Sachdev</t>
         </is>
       </c>
     </row>
     <row r="40">
-      <c r="A40" t="inlineStr">
+      <c r="A40" s="0" t="inlineStr">
         <is>
           <t>2026-04-08</t>
         </is>
       </c>
-      <c r="B40" t="n">
+      <c r="B40" s="0" t="n">
         <v>39</v>
       </c>
-      <c r="C40" t="inlineStr">
+      <c r="C40" s="0" t="inlineStr">
         <is>
           <t>Teri Deewani</t>
         </is>
       </c>
-      <c r="D40" t="inlineStr">
+      <c r="D40" s="0" t="inlineStr">
         <is>
           <t>Kailash Kher</t>
         </is>
       </c>
     </row>
     <row r="41">
-      <c r="A41" t="inlineStr">
+      <c r="A41" s="0" t="inlineStr">
         <is>
           <t>2026-04-08</t>
         </is>
       </c>
-      <c r="B41" t="n">
+      <c r="B41" s="0" t="n">
         <v>40</v>
       </c>
-      <c r="C41" t="inlineStr">
+      <c r="C41" s="0" t="inlineStr">
         <is>
           <t>Jogi</t>
         </is>
       </c>
-      <c r="D41" t="inlineStr">
+      <c r="D41" s="0" t="inlineStr">
         <is>
           <t>thiarajxtt</t>
         </is>
       </c>
     </row>
     <row r="42">
-      <c r="A42" t="inlineStr">
+      <c r="A42" s="0" t="inlineStr">
         <is>
           <t>2026-04-08</t>
         </is>
       </c>
-      <c r="B42" t="n">
+      <c r="B42" s="0" t="n">
         <v>41</v>
       </c>
-      <c r="C42" t="inlineStr">
+      <c r="C42" s="0" t="inlineStr">
         <is>
           <t>Ye Tune Kya Kiya</t>
         </is>
       </c>
-      <c r="D42" t="inlineStr">
+      <c r="D42" s="0" t="inlineStr">
         <is>
           <t>Pritam</t>
         </is>
       </c>
     </row>
     <row r="43">
-      <c r="A43" t="inlineStr">
+      <c r="A43" s="0" t="inlineStr">
         <is>
           <t>2026-04-08</t>
         </is>
       </c>
-      <c r="B43" t="n">
+      <c r="B43" s="0" t="n">
         <v>42</v>
       </c>
-      <c r="C43" t="inlineStr">
+      <c r="C43" s="0" t="inlineStr">
         <is>
           <t>Mann Mera - Original Version</t>
         </is>
       </c>
-      <c r="D43" t="inlineStr">
+      <c r="D43" s="0" t="inlineStr">
         <is>
           <t>Gajendra Verma</t>
         </is>
       </c>
     </row>
     <row r="44">
-      <c r="A44" t="inlineStr">
+      <c r="A44" s="0" t="inlineStr">
         <is>
           <t>2026-04-08</t>
         </is>
       </c>
-      <c r="B44" t="n">
+      <c r="B44" s="0" t="n">
         <v>43</v>
       </c>
-      <c r="C44" t="inlineStr">
+      <c r="C44" s="0" t="inlineStr">
         <is>
           <t>Ehsaas</t>
         </is>
       </c>
-      <c r="D44" t="inlineStr">
+      <c r="D44" s="0" t="inlineStr">
         <is>
           <t>Faheem Abdullah</t>
         </is>
       </c>
     </row>
     <row r="45">
-      <c r="A45" t="inlineStr">
+      <c r="A45" s="0" t="inlineStr">
         <is>
           <t>2026-04-08</t>
         </is>
       </c>
-      <c r="B45" t="n">
+      <c r="B45" s="0" t="n">
         <v>44</v>
       </c>
-      <c r="C45" t="inlineStr">
+      <c r="C45" s="0" t="inlineStr">
         <is>
           <t>Dhun</t>
         </is>
       </c>
-      <c r="D45" t="inlineStr">
+      <c r="D45" s="0" t="inlineStr">
         <is>
           <t>Mithoon</t>
         </is>
       </c>
     </row>
     <row r="46">
-      <c r="A46" t="inlineStr">
+      <c r="A46" s="0" t="inlineStr">
         <is>
           <t>2026-04-08</t>
         </is>
       </c>
-      <c r="B46" t="n">
+      <c r="B46" s="0" t="n">
         <v>45</v>
       </c>
-      <c r="C46" t="inlineStr">
+      <c r="C46" s="0" t="inlineStr">
         <is>
           <t>Zaalima</t>
         </is>
       </c>
-      <c r="D46" t="inlineStr">
+      <c r="D46" s="0" t="inlineStr">
         <is>
           <t>Arijit Singh</t>
         </is>
       </c>
     </row>
     <row r="47">
-      <c r="A47" t="inlineStr">
+      <c r="A47" s="0" t="inlineStr">
         <is>
           <t>2026-04-08</t>
         </is>
       </c>
-      <c r="B47" t="n">
+      <c r="B47" s="0" t="n">
         <v>46</v>
       </c>
-      <c r="C47" t="inlineStr">
+      <c r="C47" s="0" t="inlineStr">
         <is>
           <t>Thodi Si Daaru</t>
         </is>
       </c>
-      <c r="D47" t="inlineStr">
+      <c r="D47" s="0" t="inlineStr">
         <is>
           <t>AP Dhillon</t>
         </is>
       </c>
     </row>
     <row r="48">
-      <c r="A48" t="inlineStr">
+      <c r="A48" s="0" t="inlineStr">
         <is>
           <t>2026-04-08</t>
         </is>
       </c>
-      <c r="B48" t="n">
+      <c r="B48" s="0" t="n">
         <v>47</v>
       </c>
-      <c r="C48" t="inlineStr">
+      <c r="C48" s="0" t="inlineStr">
         <is>
           <t>Main Aur Tu</t>
         </is>
       </c>
-      <c r="D48" t="inlineStr">
+      <c r="D48" s="0" t="inlineStr">
         <is>
           <t>Shashwat Sachdev</t>
         </is>
       </c>
     </row>
     <row r="49">
-      <c r="A49" t="inlineStr">
+      <c r="A49" s="0" t="inlineStr">
         <is>
           <t>2026-04-08</t>
         </is>
       </c>
-      <c r="B49" t="n">
+      <c r="B49" s="0" t="n">
         <v>48</v>
       </c>
-      <c r="C49" t="inlineStr">
+      <c r="C49" s="0" t="inlineStr">
         <is>
           <t>Ishq Jalakar - Karvaan</t>
         </is>
       </c>
-      <c r="D49" t="inlineStr">
+      <c r="D49" s="0" t="inlineStr">
         <is>
           <t>Shashwat Sachdev</t>
         </is>
       </c>
     </row>
     <row r="50">
-      <c r="A50" t="inlineStr">
+      <c r="A50" s="0" t="inlineStr">
         <is>
           <t>2026-04-08</t>
         </is>
       </c>
-      <c r="B50" t="n">
+      <c r="B50" s="0" t="n">
         <v>49</v>
       </c>
-      <c r="C50" t="inlineStr">
+      <c r="C50" s="0" t="inlineStr">
         <is>
           <t>Mast Magan</t>
         </is>
       </c>
-      <c r="D50" t="inlineStr">
+      <c r="D50" s="0" t="inlineStr">
         <is>
           <t>Arijit Singh</t>
         </is>
       </c>
     </row>
     <row r="51">
-      <c r="A51" t="inlineStr">
+      <c r="A51" s="0" t="inlineStr">
         <is>
           <t>2026-04-08</t>
         </is>
       </c>
-      <c r="B51" t="n">
+      <c r="B51" s="0" t="n">
         <v>50</v>
       </c>
-      <c r="C51" t="inlineStr">
+      <c r="C51" s="0" t="inlineStr">
         <is>
           <t>Aaya Sher</t>
         </is>
       </c>
-      <c r="D51" t="inlineStr">
+      <c r="D51" s="0" t="inlineStr">
         <is>
           <t>Anirudh Ravichander</t>
         </is>
@@ -28443,6 +28444,1042 @@
 </worksheet>
 </file>
 
+<file path=xl/worksheets/sheet33.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:D51"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="24" t="inlineStr">
+        <is>
+          <t>Date</t>
+        </is>
+      </c>
+      <c r="B1" s="24" t="inlineStr">
+        <is>
+          <t>Rank</t>
+        </is>
+      </c>
+      <c r="C1" s="24" t="inlineStr">
+        <is>
+          <t>Song</t>
+        </is>
+      </c>
+      <c r="D1" s="24" t="inlineStr">
+        <is>
+          <t>Artist</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>2026-04-15</t>
+        </is>
+      </c>
+      <c r="B2" t="n">
+        <v>1</v>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>Bairan</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>Banjaare</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>2026-04-15</t>
+        </is>
+      </c>
+      <c r="B3" t="n">
+        <v>2</v>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>Gehra Hua</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>Shashwat Sachdev</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>2026-04-15</t>
+        </is>
+      </c>
+      <c r="B4" t="n">
+        <v>3</v>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>Sheesha - Aakhya Mai Aakh Ghali Jo Bairan</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>Mitta Ror</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>2026-04-15</t>
+        </is>
+      </c>
+      <c r="B5" t="n">
+        <v>4</v>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>Jaiye Sajana</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>Shashwat Sachdev</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>2026-04-15</t>
+        </is>
+      </c>
+      <c r="B6" t="n">
+        <v>5</v>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>Khat</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>Navjot Ahuja</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>2026-04-15</t>
+        </is>
+      </c>
+      <c r="B7" t="n">
+        <v>6</v>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>Sitaare</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>Arijit Singh</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>2026-04-15</t>
+        </is>
+      </c>
+      <c r="B8" t="n">
+        <v>7</v>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>Dooron Dooron</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>Paresh Pahuja</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>2026-04-15</t>
+        </is>
+      </c>
+      <c r="B9" t="n">
+        <v>8</v>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>Sahiba</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>Aditya Rikhari</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>2026-04-15</t>
+        </is>
+      </c>
+      <c r="B10" t="n">
+        <v>9</v>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>Finding Her</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>Kushagra</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>2026-04-15</t>
+        </is>
+      </c>
+      <c r="B11" t="n">
+        <v>10</v>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>Apna Bana Le</t>
+        </is>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>Sachin-Jigar</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>2026-04-15</t>
+        </is>
+      </c>
+      <c r="B12" t="n">
+        <v>11</v>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>Samjhawan</t>
+        </is>
+      </c>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>Jawad Ahmad</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>2026-04-15</t>
+        </is>
+      </c>
+      <c r="B13" t="n">
+        <v>12</v>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>Arz Kiya Hai | Coke Studio Bharat</t>
+        </is>
+      </c>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t>Anuv Jain</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>2026-04-15</t>
+        </is>
+      </c>
+      <c r="B14" t="n">
+        <v>13</v>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>Pavazha Malli</t>
+        </is>
+      </c>
+      <c r="D14" t="inlineStr">
+        <is>
+          <t>Sai Abhyankkar</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>2026-04-15</t>
+        </is>
+      </c>
+      <c r="B15" t="n">
+        <v>14</v>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>Dhurandhar The Revenge - Aari Aari</t>
+        </is>
+      </c>
+      <c r="D15" t="inlineStr">
+        <is>
+          <t>Shashwat Sachdev</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>2026-04-15</t>
+        </is>
+      </c>
+      <c r="B16" t="n">
+        <v>15</v>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>Boyfriend</t>
+        </is>
+      </c>
+      <c r="D16" t="inlineStr">
+        <is>
+          <t>Karan Aujla</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>2026-04-15</t>
+        </is>
+      </c>
+      <c r="B17" t="n">
+        <v>16</v>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>Mann Mera</t>
+        </is>
+      </c>
+      <c r="D17" t="inlineStr">
+        <is>
+          <t>Gajendra Verma</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>2026-04-15</t>
+        </is>
+      </c>
+      <c r="B18" t="n">
+        <v>17</v>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>Jaan Se Guzarte Hain</t>
+        </is>
+      </c>
+      <c r="D18" t="inlineStr">
+        <is>
+          <t>Shashwat Sachdev</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>2026-04-15</t>
+        </is>
+      </c>
+      <c r="B19" t="n">
+        <v>18</v>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>Ishq</t>
+        </is>
+      </c>
+      <c r="D19" t="inlineStr">
+        <is>
+          <t>Faheem Abdullah</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>2026-04-15</t>
+        </is>
+      </c>
+      <c r="B20" t="n">
+        <v>19</v>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>Shararat</t>
+        </is>
+      </c>
+      <c r="D20" t="inlineStr">
+        <is>
+          <t>Shashwat Sachdev</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>2026-04-15</t>
+        </is>
+      </c>
+      <c r="B21" t="n">
+        <v>20</v>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>Majboor</t>
+        </is>
+      </c>
+      <c r="D21" t="inlineStr">
+        <is>
+          <t>Sheheryar Rehan</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>2026-04-15</t>
+        </is>
+      </c>
+      <c r="B22" t="n">
+        <v>21</v>
+      </c>
+      <c r="C22" t="inlineStr">
+        <is>
+          <t>Saiyaara</t>
+        </is>
+      </c>
+      <c r="D22" t="inlineStr">
+        <is>
+          <t>Tanishk Bagchi</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>2026-04-15</t>
+        </is>
+      </c>
+      <c r="B23" t="n">
+        <v>22</v>
+      </c>
+      <c r="C23" t="inlineStr">
+        <is>
+          <t>For A Reason</t>
+        </is>
+      </c>
+      <c r="D23" t="inlineStr">
+        <is>
+          <t>Karan Aujla</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>2026-04-15</t>
+        </is>
+      </c>
+      <c r="B24" t="n">
+        <v>23</v>
+      </c>
+      <c r="C24" t="inlineStr">
+        <is>
+          <t>Tum Ho Toh</t>
+        </is>
+      </c>
+      <c r="D24" t="inlineStr">
+        <is>
+          <t>Vishal Mishra</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>2026-04-15</t>
+        </is>
+      </c>
+      <c r="B25" t="n">
+        <v>24</v>
+      </c>
+      <c r="C25" t="inlineStr">
+        <is>
+          <t>Darkhaast</t>
+        </is>
+      </c>
+      <c r="D25" t="inlineStr">
+        <is>
+          <t>Mithoon</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>2026-04-15</t>
+        </is>
+      </c>
+      <c r="B26" t="n">
+        <v>25</v>
+      </c>
+      <c r="C26" t="inlineStr">
+        <is>
+          <t>Ishqa Ve</t>
+        </is>
+      </c>
+      <c r="D26" t="inlineStr">
+        <is>
+          <t>Zeeshan Ali</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>2026-04-15</t>
+        </is>
+      </c>
+      <c r="B27" t="n">
+        <v>26</v>
+      </c>
+      <c r="C27" t="inlineStr">
+        <is>
+          <t>Raanjhan</t>
+        </is>
+      </c>
+      <c r="D27" t="inlineStr">
+        <is>
+          <t>Sachet-Parampara</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>2026-04-15</t>
+        </is>
+      </c>
+      <c r="B28" t="n">
+        <v>27</v>
+      </c>
+      <c r="C28" t="inlineStr">
+        <is>
+          <t>Naal Nachna</t>
+        </is>
+      </c>
+      <c r="D28" t="inlineStr">
+        <is>
+          <t>Shashwat Sachdev</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>2026-04-15</t>
+        </is>
+      </c>
+      <c r="B29" t="n">
+        <v>28</v>
+      </c>
+      <c r="C29" t="inlineStr">
+        <is>
+          <t>Phir Se</t>
+        </is>
+      </c>
+      <c r="D29" t="inlineStr">
+        <is>
+          <t>Shashwat Sachdev</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>2026-04-15</t>
+        </is>
+      </c>
+      <c r="B30" t="n">
+        <v>29</v>
+      </c>
+      <c r="C30" t="inlineStr">
+        <is>
+          <t>Deewaana Deewaana</t>
+        </is>
+      </c>
+      <c r="D30" t="inlineStr">
+        <is>
+          <t>A.R. Rahman</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>2026-04-15</t>
+        </is>
+      </c>
+      <c r="B31" t="n">
+        <v>30</v>
+      </c>
+      <c r="C31" t="inlineStr">
+        <is>
+          <t>Bairi</t>
+        </is>
+      </c>
+      <c r="D31" t="inlineStr">
+        <is>
+          <t>Virat</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="inlineStr">
+        <is>
+          <t>2026-04-15</t>
+        </is>
+      </c>
+      <c r="B32" t="n">
+        <v>31</v>
+      </c>
+      <c r="C32" t="inlineStr">
+        <is>
+          <t>Tere Liye</t>
+        </is>
+      </c>
+      <c r="D32" t="inlineStr">
+        <is>
+          <t>Atif Aslam</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="inlineStr">
+        <is>
+          <t>2026-04-15</t>
+        </is>
+      </c>
+      <c r="B33" t="n">
+        <v>32</v>
+      </c>
+      <c r="C33" t="inlineStr">
+        <is>
+          <t>Dhurandhar - Title Track</t>
+        </is>
+      </c>
+      <c r="D33" t="inlineStr">
+        <is>
+          <t>Shashwat Sachdev</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="inlineStr">
+        <is>
+          <t>2026-04-15</t>
+        </is>
+      </c>
+      <c r="B34" t="n">
+        <v>33</v>
+      </c>
+      <c r="C34" t="inlineStr">
+        <is>
+          <t>Ehsaas</t>
+        </is>
+      </c>
+      <c r="D34" t="inlineStr">
+        <is>
+          <t>Faheem Abdullah</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="inlineStr">
+        <is>
+          <t>2026-04-15</t>
+        </is>
+      </c>
+      <c r="B35" t="n">
+        <v>34</v>
+      </c>
+      <c r="C35" t="inlineStr">
+        <is>
+          <t>Jo Tum Mere Ho</t>
+        </is>
+      </c>
+      <c r="D35" t="inlineStr">
+        <is>
+          <t>Anuv Jain</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="inlineStr">
+        <is>
+          <t>2026-04-15</t>
+        </is>
+      </c>
+      <c r="B36" t="n">
+        <v>35</v>
+      </c>
+      <c r="C36" t="inlineStr">
+        <is>
+          <t>Agar Tum Saath Ho</t>
+        </is>
+      </c>
+      <c r="D36" t="inlineStr">
+        <is>
+          <t>Alka Yagnik</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="inlineStr">
+        <is>
+          <t>2026-04-15</t>
+        </is>
+      </c>
+      <c r="B37" t="n">
+        <v>36</v>
+      </c>
+      <c r="C37" t="inlineStr">
+        <is>
+          <t>Tere Bina</t>
+        </is>
+      </c>
+      <c r="D37" t="inlineStr">
+        <is>
+          <t>A.R. Rahman</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="inlineStr">
+        <is>
+          <t>2026-04-15</t>
+        </is>
+      </c>
+      <c r="B38" t="n">
+        <v>37</v>
+      </c>
+      <c r="C38" t="inlineStr">
+        <is>
+          <t>Run Down The City - Monica</t>
+        </is>
+      </c>
+      <c r="D38" t="inlineStr">
+        <is>
+          <t>Shashwat Sachdev</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="inlineStr">
+        <is>
+          <t>2026-04-15</t>
+        </is>
+      </c>
+      <c r="B39" t="n">
+        <v>38</v>
+      </c>
+      <c r="C39" t="inlineStr">
+        <is>
+          <t>Lutt Le Gaya</t>
+        </is>
+      </c>
+      <c r="D39" t="inlineStr">
+        <is>
+          <t>Shashwat Sachdev</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" t="inlineStr">
+        <is>
+          <t>2026-04-15</t>
+        </is>
+      </c>
+      <c r="B40" t="n">
+        <v>39</v>
+      </c>
+      <c r="C40" t="inlineStr">
+        <is>
+          <t>Teri Deewani</t>
+        </is>
+      </c>
+      <c r="D40" t="inlineStr">
+        <is>
+          <t>Kailash Kher</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" t="inlineStr">
+        <is>
+          <t>2026-04-15</t>
+        </is>
+      </c>
+      <c r="B41" t="n">
+        <v>40</v>
+      </c>
+      <c r="C41" t="inlineStr">
+        <is>
+          <t>Ye Tune Kya Kiya</t>
+        </is>
+      </c>
+      <c r="D41" t="inlineStr">
+        <is>
+          <t>Pritam</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" t="inlineStr">
+        <is>
+          <t>2026-04-15</t>
+        </is>
+      </c>
+      <c r="B42" t="n">
+        <v>41</v>
+      </c>
+      <c r="C42" t="inlineStr">
+        <is>
+          <t>Jogi</t>
+        </is>
+      </c>
+      <c r="D42" t="inlineStr">
+        <is>
+          <t>thiarajxtt</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" t="inlineStr">
+        <is>
+          <t>2026-04-15</t>
+        </is>
+      </c>
+      <c r="B43" t="n">
+        <v>42</v>
+      </c>
+      <c r="C43" t="inlineStr">
+        <is>
+          <t>Barbaad</t>
+        </is>
+      </c>
+      <c r="D43" t="inlineStr">
+        <is>
+          <t>The Rish</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" t="inlineStr">
+        <is>
+          <t>2026-04-15</t>
+        </is>
+      </c>
+      <c r="B44" t="n">
+        <v>43</v>
+      </c>
+      <c r="C44" t="inlineStr">
+        <is>
+          <t>Haseen</t>
+        </is>
+      </c>
+      <c r="D44" t="inlineStr">
+        <is>
+          <t>Talwiinder</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" t="inlineStr">
+        <is>
+          <t>2026-04-15</t>
+        </is>
+      </c>
+      <c r="B45" t="n">
+        <v>44</v>
+      </c>
+      <c r="C45" t="inlineStr">
+        <is>
+          <t>Not Guilty</t>
+        </is>
+      </c>
+      <c r="D45" t="inlineStr">
+        <is>
+          <t>Dhanda Nyoliwala</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" t="inlineStr">
+        <is>
+          <t>2026-04-15</t>
+        </is>
+      </c>
+      <c r="B46" t="n">
+        <v>45</v>
+      </c>
+      <c r="C46" t="inlineStr">
+        <is>
+          <t>High On You</t>
+        </is>
+      </c>
+      <c r="D46" t="inlineStr">
+        <is>
+          <t>Jind Universe</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" t="inlineStr">
+        <is>
+          <t>2026-04-15</t>
+        </is>
+      </c>
+      <c r="B47" t="n">
+        <v>46</v>
+      </c>
+      <c r="C47" t="inlineStr">
+        <is>
+          <t>Mann Mera - Original Version</t>
+        </is>
+      </c>
+      <c r="D47" t="inlineStr">
+        <is>
+          <t>Gajendra Verma</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" t="inlineStr">
+        <is>
+          <t>2026-04-15</t>
+        </is>
+      </c>
+      <c r="B48" t="n">
+        <v>47</v>
+      </c>
+      <c r="C48" t="inlineStr">
+        <is>
+          <t>Mast Magan</t>
+        </is>
+      </c>
+      <c r="D48" t="inlineStr">
+        <is>
+          <t>Arijit Singh</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" t="inlineStr">
+        <is>
+          <t>2026-04-15</t>
+        </is>
+      </c>
+      <c r="B49" t="n">
+        <v>48</v>
+      </c>
+      <c r="C49" t="inlineStr">
+        <is>
+          <t>Thodi Si Daaru</t>
+        </is>
+      </c>
+      <c r="D49" t="inlineStr">
+        <is>
+          <t>AP Dhillon</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" t="inlineStr">
+        <is>
+          <t>2026-04-15</t>
+        </is>
+      </c>
+      <c r="B50" t="n">
+        <v>49</v>
+      </c>
+      <c r="C50" t="inlineStr">
+        <is>
+          <t>Jhol - Acoustic</t>
+        </is>
+      </c>
+      <c r="D50" t="inlineStr">
+        <is>
+          <t>Maanu</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" t="inlineStr">
+        <is>
+          <t>2026-04-15</t>
+        </is>
+      </c>
+      <c r="B51" t="n">
+        <v>50</v>
+      </c>
+      <c r="C51" t="inlineStr">
+        <is>
+          <t>Dhun</t>
+        </is>
+      </c>
+      <c r="D51" t="inlineStr">
+        <is>
+          <t>Mithoon</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>

</xml_diff>

<commit_message>
got data for 16th and predictions for 17th april
</commit_message>
<xml_diff>
--- a/Probability Project.xlsx
+++ b/Probability Project.xlsx
@@ -36,6 +36,7 @@
     <sheet name="AUTO_20260414" sheetId="31" state="visible" r:id="rId31"/>
     <sheet name="AUTO_20260413" sheetId="32" state="visible" r:id="rId32"/>
     <sheet name="AUTO_20260415" sheetId="33" state="visible" r:id="rId33"/>
+    <sheet name="AUTO_20260416" sheetId="34" state="visible" r:id="rId34"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -28476,9 +28477,1045 @@
       </c>
     </row>
     <row r="2">
+      <c r="A2" s="0" t="inlineStr">
+        <is>
+          <t>2026-04-15</t>
+        </is>
+      </c>
+      <c r="B2" s="0" t="n">
+        <v>1</v>
+      </c>
+      <c r="C2" s="0" t="inlineStr">
+        <is>
+          <t>Bairan</t>
+        </is>
+      </c>
+      <c r="D2" s="0" t="inlineStr">
+        <is>
+          <t>Banjaare</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="0" t="inlineStr">
+        <is>
+          <t>2026-04-15</t>
+        </is>
+      </c>
+      <c r="B3" s="0" t="n">
+        <v>2</v>
+      </c>
+      <c r="C3" s="0" t="inlineStr">
+        <is>
+          <t>Gehra Hua</t>
+        </is>
+      </c>
+      <c r="D3" s="0" t="inlineStr">
+        <is>
+          <t>Shashwat Sachdev</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="0" t="inlineStr">
+        <is>
+          <t>2026-04-15</t>
+        </is>
+      </c>
+      <c r="B4" s="0" t="n">
+        <v>3</v>
+      </c>
+      <c r="C4" s="0" t="inlineStr">
+        <is>
+          <t>Sheesha - Aakhya Mai Aakh Ghali Jo Bairan</t>
+        </is>
+      </c>
+      <c r="D4" s="0" t="inlineStr">
+        <is>
+          <t>Mitta Ror</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="0" t="inlineStr">
+        <is>
+          <t>2026-04-15</t>
+        </is>
+      </c>
+      <c r="B5" s="0" t="n">
+        <v>4</v>
+      </c>
+      <c r="C5" s="0" t="inlineStr">
+        <is>
+          <t>Jaiye Sajana</t>
+        </is>
+      </c>
+      <c r="D5" s="0" t="inlineStr">
+        <is>
+          <t>Shashwat Sachdev</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="0" t="inlineStr">
+        <is>
+          <t>2026-04-15</t>
+        </is>
+      </c>
+      <c r="B6" s="0" t="n">
+        <v>5</v>
+      </c>
+      <c r="C6" s="0" t="inlineStr">
+        <is>
+          <t>Khat</t>
+        </is>
+      </c>
+      <c r="D6" s="0" t="inlineStr">
+        <is>
+          <t>Navjot Ahuja</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="0" t="inlineStr">
+        <is>
+          <t>2026-04-15</t>
+        </is>
+      </c>
+      <c r="B7" s="0" t="n">
+        <v>6</v>
+      </c>
+      <c r="C7" s="0" t="inlineStr">
+        <is>
+          <t>Sitaare</t>
+        </is>
+      </c>
+      <c r="D7" s="0" t="inlineStr">
+        <is>
+          <t>Arijit Singh</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="0" t="inlineStr">
+        <is>
+          <t>2026-04-15</t>
+        </is>
+      </c>
+      <c r="B8" s="0" t="n">
+        <v>7</v>
+      </c>
+      <c r="C8" s="0" t="inlineStr">
+        <is>
+          <t>Dooron Dooron</t>
+        </is>
+      </c>
+      <c r="D8" s="0" t="inlineStr">
+        <is>
+          <t>Paresh Pahuja</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="0" t="inlineStr">
+        <is>
+          <t>2026-04-15</t>
+        </is>
+      </c>
+      <c r="B9" s="0" t="n">
+        <v>8</v>
+      </c>
+      <c r="C9" s="0" t="inlineStr">
+        <is>
+          <t>Sahiba</t>
+        </is>
+      </c>
+      <c r="D9" s="0" t="inlineStr">
+        <is>
+          <t>Aditya Rikhari</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="0" t="inlineStr">
+        <is>
+          <t>2026-04-15</t>
+        </is>
+      </c>
+      <c r="B10" s="0" t="n">
+        <v>9</v>
+      </c>
+      <c r="C10" s="0" t="inlineStr">
+        <is>
+          <t>Finding Her</t>
+        </is>
+      </c>
+      <c r="D10" s="0" t="inlineStr">
+        <is>
+          <t>Kushagra</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="0" t="inlineStr">
+        <is>
+          <t>2026-04-15</t>
+        </is>
+      </c>
+      <c r="B11" s="0" t="n">
+        <v>10</v>
+      </c>
+      <c r="C11" s="0" t="inlineStr">
+        <is>
+          <t>Apna Bana Le</t>
+        </is>
+      </c>
+      <c r="D11" s="0" t="inlineStr">
+        <is>
+          <t>Sachin-Jigar</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="0" t="inlineStr">
+        <is>
+          <t>2026-04-15</t>
+        </is>
+      </c>
+      <c r="B12" s="0" t="n">
+        <v>11</v>
+      </c>
+      <c r="C12" s="0" t="inlineStr">
+        <is>
+          <t>Samjhawan</t>
+        </is>
+      </c>
+      <c r="D12" s="0" t="inlineStr">
+        <is>
+          <t>Jawad Ahmad</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="0" t="inlineStr">
+        <is>
+          <t>2026-04-15</t>
+        </is>
+      </c>
+      <c r="B13" s="0" t="n">
+        <v>12</v>
+      </c>
+      <c r="C13" s="0" t="inlineStr">
+        <is>
+          <t>Arz Kiya Hai | Coke Studio Bharat</t>
+        </is>
+      </c>
+      <c r="D13" s="0" t="inlineStr">
+        <is>
+          <t>Anuv Jain</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="0" t="inlineStr">
+        <is>
+          <t>2026-04-15</t>
+        </is>
+      </c>
+      <c r="B14" s="0" t="n">
+        <v>13</v>
+      </c>
+      <c r="C14" s="0" t="inlineStr">
+        <is>
+          <t>Pavazha Malli</t>
+        </is>
+      </c>
+      <c r="D14" s="0" t="inlineStr">
+        <is>
+          <t>Sai Abhyankkar</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="0" t="inlineStr">
+        <is>
+          <t>2026-04-15</t>
+        </is>
+      </c>
+      <c r="B15" s="0" t="n">
+        <v>14</v>
+      </c>
+      <c r="C15" s="0" t="inlineStr">
+        <is>
+          <t>Dhurandhar The Revenge - Aari Aari</t>
+        </is>
+      </c>
+      <c r="D15" s="0" t="inlineStr">
+        <is>
+          <t>Shashwat Sachdev</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="0" t="inlineStr">
+        <is>
+          <t>2026-04-15</t>
+        </is>
+      </c>
+      <c r="B16" s="0" t="n">
+        <v>15</v>
+      </c>
+      <c r="C16" s="0" t="inlineStr">
+        <is>
+          <t>Boyfriend</t>
+        </is>
+      </c>
+      <c r="D16" s="0" t="inlineStr">
+        <is>
+          <t>Karan Aujla</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="0" t="inlineStr">
+        <is>
+          <t>2026-04-15</t>
+        </is>
+      </c>
+      <c r="B17" s="0" t="n">
+        <v>16</v>
+      </c>
+      <c r="C17" s="0" t="inlineStr">
+        <is>
+          <t>Mann Mera</t>
+        </is>
+      </c>
+      <c r="D17" s="0" t="inlineStr">
+        <is>
+          <t>Gajendra Verma</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="0" t="inlineStr">
+        <is>
+          <t>2026-04-15</t>
+        </is>
+      </c>
+      <c r="B18" s="0" t="n">
+        <v>17</v>
+      </c>
+      <c r="C18" s="0" t="inlineStr">
+        <is>
+          <t>Jaan Se Guzarte Hain</t>
+        </is>
+      </c>
+      <c r="D18" s="0" t="inlineStr">
+        <is>
+          <t>Shashwat Sachdev</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="0" t="inlineStr">
+        <is>
+          <t>2026-04-15</t>
+        </is>
+      </c>
+      <c r="B19" s="0" t="n">
+        <v>18</v>
+      </c>
+      <c r="C19" s="0" t="inlineStr">
+        <is>
+          <t>Ishq</t>
+        </is>
+      </c>
+      <c r="D19" s="0" t="inlineStr">
+        <is>
+          <t>Faheem Abdullah</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="0" t="inlineStr">
+        <is>
+          <t>2026-04-15</t>
+        </is>
+      </c>
+      <c r="B20" s="0" t="n">
+        <v>19</v>
+      </c>
+      <c r="C20" s="0" t="inlineStr">
+        <is>
+          <t>Shararat</t>
+        </is>
+      </c>
+      <c r="D20" s="0" t="inlineStr">
+        <is>
+          <t>Shashwat Sachdev</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="0" t="inlineStr">
+        <is>
+          <t>2026-04-15</t>
+        </is>
+      </c>
+      <c r="B21" s="0" t="n">
+        <v>20</v>
+      </c>
+      <c r="C21" s="0" t="inlineStr">
+        <is>
+          <t>Majboor</t>
+        </is>
+      </c>
+      <c r="D21" s="0" t="inlineStr">
+        <is>
+          <t>Sheheryar Rehan</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="0" t="inlineStr">
+        <is>
+          <t>2026-04-15</t>
+        </is>
+      </c>
+      <c r="B22" s="0" t="n">
+        <v>21</v>
+      </c>
+      <c r="C22" s="0" t="inlineStr">
+        <is>
+          <t>Saiyaara</t>
+        </is>
+      </c>
+      <c r="D22" s="0" t="inlineStr">
+        <is>
+          <t>Tanishk Bagchi</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="0" t="inlineStr">
+        <is>
+          <t>2026-04-15</t>
+        </is>
+      </c>
+      <c r="B23" s="0" t="n">
+        <v>22</v>
+      </c>
+      <c r="C23" s="0" t="inlineStr">
+        <is>
+          <t>For A Reason</t>
+        </is>
+      </c>
+      <c r="D23" s="0" t="inlineStr">
+        <is>
+          <t>Karan Aujla</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="0" t="inlineStr">
+        <is>
+          <t>2026-04-15</t>
+        </is>
+      </c>
+      <c r="B24" s="0" t="n">
+        <v>23</v>
+      </c>
+      <c r="C24" s="0" t="inlineStr">
+        <is>
+          <t>Tum Ho Toh</t>
+        </is>
+      </c>
+      <c r="D24" s="0" t="inlineStr">
+        <is>
+          <t>Vishal Mishra</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="0" t="inlineStr">
+        <is>
+          <t>2026-04-15</t>
+        </is>
+      </c>
+      <c r="B25" s="0" t="n">
+        <v>24</v>
+      </c>
+      <c r="C25" s="0" t="inlineStr">
+        <is>
+          <t>Darkhaast</t>
+        </is>
+      </c>
+      <c r="D25" s="0" t="inlineStr">
+        <is>
+          <t>Mithoon</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="0" t="inlineStr">
+        <is>
+          <t>2026-04-15</t>
+        </is>
+      </c>
+      <c r="B26" s="0" t="n">
+        <v>25</v>
+      </c>
+      <c r="C26" s="0" t="inlineStr">
+        <is>
+          <t>Ishqa Ve</t>
+        </is>
+      </c>
+      <c r="D26" s="0" t="inlineStr">
+        <is>
+          <t>Zeeshan Ali</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="0" t="inlineStr">
+        <is>
+          <t>2026-04-15</t>
+        </is>
+      </c>
+      <c r="B27" s="0" t="n">
+        <v>26</v>
+      </c>
+      <c r="C27" s="0" t="inlineStr">
+        <is>
+          <t>Raanjhan</t>
+        </is>
+      </c>
+      <c r="D27" s="0" t="inlineStr">
+        <is>
+          <t>Sachet-Parampara</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="0" t="inlineStr">
+        <is>
+          <t>2026-04-15</t>
+        </is>
+      </c>
+      <c r="B28" s="0" t="n">
+        <v>27</v>
+      </c>
+      <c r="C28" s="0" t="inlineStr">
+        <is>
+          <t>Naal Nachna</t>
+        </is>
+      </c>
+      <c r="D28" s="0" t="inlineStr">
+        <is>
+          <t>Shashwat Sachdev</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="0" t="inlineStr">
+        <is>
+          <t>2026-04-15</t>
+        </is>
+      </c>
+      <c r="B29" s="0" t="n">
+        <v>28</v>
+      </c>
+      <c r="C29" s="0" t="inlineStr">
+        <is>
+          <t>Phir Se</t>
+        </is>
+      </c>
+      <c r="D29" s="0" t="inlineStr">
+        <is>
+          <t>Shashwat Sachdev</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="0" t="inlineStr">
+        <is>
+          <t>2026-04-15</t>
+        </is>
+      </c>
+      <c r="B30" s="0" t="n">
+        <v>29</v>
+      </c>
+      <c r="C30" s="0" t="inlineStr">
+        <is>
+          <t>Deewaana Deewaana</t>
+        </is>
+      </c>
+      <c r="D30" s="0" t="inlineStr">
+        <is>
+          <t>A.R. Rahman</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="0" t="inlineStr">
+        <is>
+          <t>2026-04-15</t>
+        </is>
+      </c>
+      <c r="B31" s="0" t="n">
+        <v>30</v>
+      </c>
+      <c r="C31" s="0" t="inlineStr">
+        <is>
+          <t>Bairi</t>
+        </is>
+      </c>
+      <c r="D31" s="0" t="inlineStr">
+        <is>
+          <t>Virat</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="0" t="inlineStr">
+        <is>
+          <t>2026-04-15</t>
+        </is>
+      </c>
+      <c r="B32" s="0" t="n">
+        <v>31</v>
+      </c>
+      <c r="C32" s="0" t="inlineStr">
+        <is>
+          <t>Tere Liye</t>
+        </is>
+      </c>
+      <c r="D32" s="0" t="inlineStr">
+        <is>
+          <t>Atif Aslam</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="0" t="inlineStr">
+        <is>
+          <t>2026-04-15</t>
+        </is>
+      </c>
+      <c r="B33" s="0" t="n">
+        <v>32</v>
+      </c>
+      <c r="C33" s="0" t="inlineStr">
+        <is>
+          <t>Dhurandhar - Title Track</t>
+        </is>
+      </c>
+      <c r="D33" s="0" t="inlineStr">
+        <is>
+          <t>Shashwat Sachdev</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="0" t="inlineStr">
+        <is>
+          <t>2026-04-15</t>
+        </is>
+      </c>
+      <c r="B34" s="0" t="n">
+        <v>33</v>
+      </c>
+      <c r="C34" s="0" t="inlineStr">
+        <is>
+          <t>Ehsaas</t>
+        </is>
+      </c>
+      <c r="D34" s="0" t="inlineStr">
+        <is>
+          <t>Faheem Abdullah</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="0" t="inlineStr">
+        <is>
+          <t>2026-04-15</t>
+        </is>
+      </c>
+      <c r="B35" s="0" t="n">
+        <v>34</v>
+      </c>
+      <c r="C35" s="0" t="inlineStr">
+        <is>
+          <t>Jo Tum Mere Ho</t>
+        </is>
+      </c>
+      <c r="D35" s="0" t="inlineStr">
+        <is>
+          <t>Anuv Jain</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="0" t="inlineStr">
+        <is>
+          <t>2026-04-15</t>
+        </is>
+      </c>
+      <c r="B36" s="0" t="n">
+        <v>35</v>
+      </c>
+      <c r="C36" s="0" t="inlineStr">
+        <is>
+          <t>Agar Tum Saath Ho</t>
+        </is>
+      </c>
+      <c r="D36" s="0" t="inlineStr">
+        <is>
+          <t>Alka Yagnik</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="0" t="inlineStr">
+        <is>
+          <t>2026-04-15</t>
+        </is>
+      </c>
+      <c r="B37" s="0" t="n">
+        <v>36</v>
+      </c>
+      <c r="C37" s="0" t="inlineStr">
+        <is>
+          <t>Tere Bina</t>
+        </is>
+      </c>
+      <c r="D37" s="0" t="inlineStr">
+        <is>
+          <t>A.R. Rahman</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="0" t="inlineStr">
+        <is>
+          <t>2026-04-15</t>
+        </is>
+      </c>
+      <c r="B38" s="0" t="n">
+        <v>37</v>
+      </c>
+      <c r="C38" s="0" t="inlineStr">
+        <is>
+          <t>Run Down The City - Monica</t>
+        </is>
+      </c>
+      <c r="D38" s="0" t="inlineStr">
+        <is>
+          <t>Shashwat Sachdev</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="0" t="inlineStr">
+        <is>
+          <t>2026-04-15</t>
+        </is>
+      </c>
+      <c r="B39" s="0" t="n">
+        <v>38</v>
+      </c>
+      <c r="C39" s="0" t="inlineStr">
+        <is>
+          <t>Lutt Le Gaya</t>
+        </is>
+      </c>
+      <c r="D39" s="0" t="inlineStr">
+        <is>
+          <t>Shashwat Sachdev</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="0" t="inlineStr">
+        <is>
+          <t>2026-04-15</t>
+        </is>
+      </c>
+      <c r="B40" s="0" t="n">
+        <v>39</v>
+      </c>
+      <c r="C40" s="0" t="inlineStr">
+        <is>
+          <t>Teri Deewani</t>
+        </is>
+      </c>
+      <c r="D40" s="0" t="inlineStr">
+        <is>
+          <t>Kailash Kher</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" s="0" t="inlineStr">
+        <is>
+          <t>2026-04-15</t>
+        </is>
+      </c>
+      <c r="B41" s="0" t="n">
+        <v>40</v>
+      </c>
+      <c r="C41" s="0" t="inlineStr">
+        <is>
+          <t>Ye Tune Kya Kiya</t>
+        </is>
+      </c>
+      <c r="D41" s="0" t="inlineStr">
+        <is>
+          <t>Pritam</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" s="0" t="inlineStr">
+        <is>
+          <t>2026-04-15</t>
+        </is>
+      </c>
+      <c r="B42" s="0" t="n">
+        <v>41</v>
+      </c>
+      <c r="C42" s="0" t="inlineStr">
+        <is>
+          <t>Jogi</t>
+        </is>
+      </c>
+      <c r="D42" s="0" t="inlineStr">
+        <is>
+          <t>thiarajxtt</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" s="0" t="inlineStr">
+        <is>
+          <t>2026-04-15</t>
+        </is>
+      </c>
+      <c r="B43" s="0" t="n">
+        <v>42</v>
+      </c>
+      <c r="C43" s="0" t="inlineStr">
+        <is>
+          <t>Barbaad</t>
+        </is>
+      </c>
+      <c r="D43" s="0" t="inlineStr">
+        <is>
+          <t>The Rish</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" s="0" t="inlineStr">
+        <is>
+          <t>2026-04-15</t>
+        </is>
+      </c>
+      <c r="B44" s="0" t="n">
+        <v>43</v>
+      </c>
+      <c r="C44" s="0" t="inlineStr">
+        <is>
+          <t>Haseen</t>
+        </is>
+      </c>
+      <c r="D44" s="0" t="inlineStr">
+        <is>
+          <t>Talwiinder</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" s="0" t="inlineStr">
+        <is>
+          <t>2026-04-15</t>
+        </is>
+      </c>
+      <c r="B45" s="0" t="n">
+        <v>44</v>
+      </c>
+      <c r="C45" s="0" t="inlineStr">
+        <is>
+          <t>Not Guilty</t>
+        </is>
+      </c>
+      <c r="D45" s="0" t="inlineStr">
+        <is>
+          <t>Dhanda Nyoliwala</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" s="0" t="inlineStr">
+        <is>
+          <t>2026-04-15</t>
+        </is>
+      </c>
+      <c r="B46" s="0" t="n">
+        <v>45</v>
+      </c>
+      <c r="C46" s="0" t="inlineStr">
+        <is>
+          <t>High On You</t>
+        </is>
+      </c>
+      <c r="D46" s="0" t="inlineStr">
+        <is>
+          <t>Jind Universe</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" s="0" t="inlineStr">
+        <is>
+          <t>2026-04-15</t>
+        </is>
+      </c>
+      <c r="B47" s="0" t="n">
+        <v>46</v>
+      </c>
+      <c r="C47" s="0" t="inlineStr">
+        <is>
+          <t>Mann Mera - Original Version</t>
+        </is>
+      </c>
+      <c r="D47" s="0" t="inlineStr">
+        <is>
+          <t>Gajendra Verma</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" s="0" t="inlineStr">
+        <is>
+          <t>2026-04-15</t>
+        </is>
+      </c>
+      <c r="B48" s="0" t="n">
+        <v>47</v>
+      </c>
+      <c r="C48" s="0" t="inlineStr">
+        <is>
+          <t>Mast Magan</t>
+        </is>
+      </c>
+      <c r="D48" s="0" t="inlineStr">
+        <is>
+          <t>Arijit Singh</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" s="0" t="inlineStr">
+        <is>
+          <t>2026-04-15</t>
+        </is>
+      </c>
+      <c r="B49" s="0" t="n">
+        <v>48</v>
+      </c>
+      <c r="C49" s="0" t="inlineStr">
+        <is>
+          <t>Thodi Si Daaru</t>
+        </is>
+      </c>
+      <c r="D49" s="0" t="inlineStr">
+        <is>
+          <t>AP Dhillon</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" s="0" t="inlineStr">
+        <is>
+          <t>2026-04-15</t>
+        </is>
+      </c>
+      <c r="B50" s="0" t="n">
+        <v>49</v>
+      </c>
+      <c r="C50" s="0" t="inlineStr">
+        <is>
+          <t>Jhol - Acoustic</t>
+        </is>
+      </c>
+      <c r="D50" s="0" t="inlineStr">
+        <is>
+          <t>Maanu</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" s="0" t="inlineStr">
+        <is>
+          <t>2026-04-15</t>
+        </is>
+      </c>
+      <c r="B51" s="0" t="n">
+        <v>50</v>
+      </c>
+      <c r="C51" s="0" t="inlineStr">
+        <is>
+          <t>Dhun</t>
+        </is>
+      </c>
+      <c r="D51" s="0" t="inlineStr">
+        <is>
+          <t>Mithoon</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet34.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:D51"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="24" t="inlineStr">
+        <is>
+          <t>Date</t>
+        </is>
+      </c>
+      <c r="B1" s="24" t="inlineStr">
+        <is>
+          <t>Rank</t>
+        </is>
+      </c>
+      <c r="C1" s="24" t="inlineStr">
+        <is>
+          <t>Song</t>
+        </is>
+      </c>
+      <c r="D1" s="24" t="inlineStr">
+        <is>
+          <t>Artist</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>2026-04-15</t>
+          <t>2026-04-16</t>
         </is>
       </c>
       <c r="B2" t="n">
@@ -28498,7 +29535,7 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>2026-04-15</t>
+          <t>2026-04-16</t>
         </is>
       </c>
       <c r="B3" t="n">
@@ -28506,19 +29543,19 @@
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>Gehra Hua</t>
+          <t>Sheesha - Aakhya Mai Aakh Ghali Jo Bairan</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>Shashwat Sachdev</t>
+          <t>Mitta Ror</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>2026-04-15</t>
+          <t>2026-04-16</t>
         </is>
       </c>
       <c r="B4" t="n">
@@ -28526,19 +29563,19 @@
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>Sheesha - Aakhya Mai Aakh Ghali Jo Bairan</t>
+          <t>Gehra Hua</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>Mitta Ror</t>
+          <t>Shashwat Sachdev</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>2026-04-15</t>
+          <t>2026-04-16</t>
         </is>
       </c>
       <c r="B5" t="n">
@@ -28558,7 +29595,7 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>2026-04-15</t>
+          <t>2026-04-16</t>
         </is>
       </c>
       <c r="B6" t="n">
@@ -28578,7 +29615,7 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>2026-04-15</t>
+          <t>2026-04-16</t>
         </is>
       </c>
       <c r="B7" t="n">
@@ -28586,19 +29623,19 @@
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>Sitaare</t>
+          <t>Dooron Dooron</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>Arijit Singh</t>
+          <t>Paresh Pahuja</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>2026-04-15</t>
+          <t>2026-04-16</t>
         </is>
       </c>
       <c r="B8" t="n">
@@ -28606,19 +29643,19 @@
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>Dooron Dooron</t>
+          <t>Sahiba</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>Paresh Pahuja</t>
+          <t>Aditya Rikhari</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>2026-04-15</t>
+          <t>2026-04-16</t>
         </is>
       </c>
       <c r="B9" t="n">
@@ -28626,19 +29663,19 @@
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>Sahiba</t>
+          <t>Sitaare</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>Aditya Rikhari</t>
+          <t>Arijit Singh</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>2026-04-15</t>
+          <t>2026-04-16</t>
         </is>
       </c>
       <c r="B10" t="n">
@@ -28658,7 +29695,7 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>2026-04-15</t>
+          <t>2026-04-16</t>
         </is>
       </c>
       <c r="B11" t="n">
@@ -28678,7 +29715,7 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>2026-04-15</t>
+          <t>2026-04-16</t>
         </is>
       </c>
       <c r="B12" t="n">
@@ -28686,19 +29723,19 @@
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>Samjhawan</t>
+          <t>Majboor</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>Jawad Ahmad</t>
+          <t>Sheheryar Rehan</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>2026-04-15</t>
+          <t>2026-04-16</t>
         </is>
       </c>
       <c r="B13" t="n">
@@ -28718,7 +29755,7 @@
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>2026-04-15</t>
+          <t>2026-04-16</t>
         </is>
       </c>
       <c r="B14" t="n">
@@ -28726,19 +29763,19 @@
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>Pavazha Malli</t>
+          <t>Dhurandhar The Revenge - Aari Aari</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>Sai Abhyankkar</t>
+          <t>Shashwat Sachdev</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>2026-04-15</t>
+          <t>2026-04-16</t>
         </is>
       </c>
       <c r="B15" t="n">
@@ -28746,19 +29783,19 @@
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>Dhurandhar The Revenge - Aari Aari</t>
+          <t>Pavazha Malli</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>Shashwat Sachdev</t>
+          <t>Sai Abhyankkar</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>2026-04-15</t>
+          <t>2026-04-16</t>
         </is>
       </c>
       <c r="B16" t="n">
@@ -28766,19 +29803,19 @@
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>Boyfriend</t>
+          <t>Samjhawan</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>Karan Aujla</t>
+          <t>Jawad Ahmad</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>2026-04-15</t>
+          <t>2026-04-16</t>
         </is>
       </c>
       <c r="B17" t="n">
@@ -28786,19 +29823,19 @@
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>Mann Mera</t>
+          <t>Boyfriend</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>Gajendra Verma</t>
+          <t>Karan Aujla</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>2026-04-15</t>
+          <t>2026-04-16</t>
         </is>
       </c>
       <c r="B18" t="n">
@@ -28818,7 +29855,7 @@
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>2026-04-15</t>
+          <t>2026-04-16</t>
         </is>
       </c>
       <c r="B19" t="n">
@@ -28826,19 +29863,19 @@
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>Ishq</t>
+          <t>Mann Mera</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>Faheem Abdullah</t>
+          <t>Gajendra Verma</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>2026-04-15</t>
+          <t>2026-04-16</t>
         </is>
       </c>
       <c r="B20" t="n">
@@ -28846,19 +29883,19 @@
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>Shararat</t>
+          <t>Ishq</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>Shashwat Sachdev</t>
+          <t>Faheem Abdullah</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>2026-04-15</t>
+          <t>2026-04-16</t>
         </is>
       </c>
       <c r="B21" t="n">
@@ -28866,19 +29903,19 @@
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>Majboor</t>
+          <t>Shararat</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>Sheheryar Rehan</t>
+          <t>Shashwat Sachdev</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>2026-04-15</t>
+          <t>2026-04-16</t>
         </is>
       </c>
       <c r="B22" t="n">
@@ -28886,19 +29923,19 @@
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>Saiyaara</t>
+          <t>Darkhaast</t>
         </is>
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>Tanishk Bagchi</t>
+          <t>Mithoon</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>2026-04-15</t>
+          <t>2026-04-16</t>
         </is>
       </c>
       <c r="B23" t="n">
@@ -28906,19 +29943,19 @@
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>For A Reason</t>
+          <t>Tum Ho Toh</t>
         </is>
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>Karan Aujla</t>
+          <t>Vishal Mishra</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>2026-04-15</t>
+          <t>2026-04-16</t>
         </is>
       </c>
       <c r="B24" t="n">
@@ -28926,19 +29963,19 @@
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>Tum Ho Toh</t>
+          <t>For A Reason</t>
         </is>
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>Vishal Mishra</t>
+          <t>Karan Aujla</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>2026-04-15</t>
+          <t>2026-04-16</t>
         </is>
       </c>
       <c r="B25" t="n">
@@ -28946,19 +29983,19 @@
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>Darkhaast</t>
+          <t>Ishqa Ve</t>
         </is>
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>Mithoon</t>
+          <t>Zeeshan Ali</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>2026-04-15</t>
+          <t>2026-04-16</t>
         </is>
       </c>
       <c r="B26" t="n">
@@ -28966,19 +30003,19 @@
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>Ishqa Ve</t>
+          <t>Deewaana Deewaana</t>
         </is>
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>Zeeshan Ali</t>
+          <t>A.R. Rahman</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>2026-04-15</t>
+          <t>2026-04-16</t>
         </is>
       </c>
       <c r="B27" t="n">
@@ -28986,19 +30023,19 @@
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>Raanjhan</t>
+          <t>Saiyaara</t>
         </is>
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t>Sachet-Parampara</t>
+          <t>Tanishk Bagchi</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>2026-04-15</t>
+          <t>2026-04-16</t>
         </is>
       </c>
       <c r="B28" t="n">
@@ -29006,19 +30043,19 @@
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>Naal Nachna</t>
+          <t>Bairi</t>
         </is>
       </c>
       <c r="D28" t="inlineStr">
         <is>
-          <t>Shashwat Sachdev</t>
+          <t>Virat</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>2026-04-15</t>
+          <t>2026-04-16</t>
         </is>
       </c>
       <c r="B29" t="n">
@@ -29026,19 +30063,19 @@
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>Phir Se</t>
+          <t>Raanjhan</t>
         </is>
       </c>
       <c r="D29" t="inlineStr">
         <is>
-          <t>Shashwat Sachdev</t>
+          <t>Sachet-Parampara</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>2026-04-15</t>
+          <t>2026-04-16</t>
         </is>
       </c>
       <c r="B30" t="n">
@@ -29046,19 +30083,19 @@
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>Deewaana Deewaana</t>
+          <t>Tere Liye</t>
         </is>
       </c>
       <c r="D30" t="inlineStr">
         <is>
-          <t>A.R. Rahman</t>
+          <t>Atif Aslam</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>2026-04-15</t>
+          <t>2026-04-16</t>
         </is>
       </c>
       <c r="B31" t="n">
@@ -29066,19 +30103,19 @@
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>Bairi</t>
+          <t>Dhurandhar - Title Track</t>
         </is>
       </c>
       <c r="D31" t="inlineStr">
         <is>
-          <t>Virat</t>
+          <t>Shashwat Sachdev</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>2026-04-15</t>
+          <t>2026-04-16</t>
         </is>
       </c>
       <c r="B32" t="n">
@@ -29086,19 +30123,19 @@
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>Tere Liye</t>
+          <t>Naal Nachna</t>
         </is>
       </c>
       <c r="D32" t="inlineStr">
         <is>
-          <t>Atif Aslam</t>
+          <t>Shashwat Sachdev</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>2026-04-15</t>
+          <t>2026-04-16</t>
         </is>
       </c>
       <c r="B33" t="n">
@@ -29106,19 +30143,19 @@
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>Dhurandhar - Title Track</t>
+          <t>Ehsaas</t>
         </is>
       </c>
       <c r="D33" t="inlineStr">
         <is>
-          <t>Shashwat Sachdev</t>
+          <t>Faheem Abdullah</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>2026-04-15</t>
+          <t>2026-04-16</t>
         </is>
       </c>
       <c r="B34" t="n">
@@ -29126,19 +30163,19 @@
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>Ehsaas</t>
+          <t>Phir Se</t>
         </is>
       </c>
       <c r="D34" t="inlineStr">
         <is>
-          <t>Faheem Abdullah</t>
+          <t>Shashwat Sachdev</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>2026-04-15</t>
+          <t>2026-04-16</t>
         </is>
       </c>
       <c r="B35" t="n">
@@ -29146,19 +30183,19 @@
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>Jo Tum Mere Ho</t>
+          <t>Tere Bina</t>
         </is>
       </c>
       <c r="D35" t="inlineStr">
         <is>
-          <t>Anuv Jain</t>
+          <t>A.R. Rahman</t>
         </is>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>2026-04-15</t>
+          <t>2026-04-16</t>
         </is>
       </c>
       <c r="B36" t="n">
@@ -29166,19 +30203,19 @@
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>Agar Tum Saath Ho</t>
+          <t>Jo Tum Mere Ho</t>
         </is>
       </c>
       <c r="D36" t="inlineStr">
         <is>
-          <t>Alka Yagnik</t>
+          <t>Anuv Jain</t>
         </is>
       </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>2026-04-15</t>
+          <t>2026-04-16</t>
         </is>
       </c>
       <c r="B37" t="n">
@@ -29186,19 +30223,19 @@
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>Tere Bina</t>
+          <t>Agar Tum Saath Ho</t>
         </is>
       </c>
       <c r="D37" t="inlineStr">
         <is>
-          <t>A.R. Rahman</t>
+          <t>Alka Yagnik</t>
         </is>
       </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>2026-04-15</t>
+          <t>2026-04-16</t>
         </is>
       </c>
       <c r="B38" t="n">
@@ -29206,19 +30243,19 @@
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>Run Down The City - Monica</t>
+          <t>Barbaad</t>
         </is>
       </c>
       <c r="D38" t="inlineStr">
         <is>
-          <t>Shashwat Sachdev</t>
+          <t>The Rish</t>
         </is>
       </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>2026-04-15</t>
+          <t>2026-04-16</t>
         </is>
       </c>
       <c r="B39" t="n">
@@ -29238,7 +30275,7 @@
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>2026-04-15</t>
+          <t>2026-04-16</t>
         </is>
       </c>
       <c r="B40" t="n">
@@ -29246,19 +30283,19 @@
       </c>
       <c r="C40" t="inlineStr">
         <is>
-          <t>Teri Deewani</t>
+          <t>Run Down The City - Monica</t>
         </is>
       </c>
       <c r="D40" t="inlineStr">
         <is>
-          <t>Kailash Kher</t>
+          <t>Shashwat Sachdev</t>
         </is>
       </c>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>2026-04-15</t>
+          <t>2026-04-16</t>
         </is>
       </c>
       <c r="B41" t="n">
@@ -29278,7 +30315,7 @@
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>2026-04-15</t>
+          <t>2026-04-16</t>
         </is>
       </c>
       <c r="B42" t="n">
@@ -29286,19 +30323,19 @@
       </c>
       <c r="C42" t="inlineStr">
         <is>
-          <t>Jogi</t>
+          <t>Haseen</t>
         </is>
       </c>
       <c r="D42" t="inlineStr">
         <is>
-          <t>thiarajxtt</t>
+          <t>Talwiinder</t>
         </is>
       </c>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>2026-04-15</t>
+          <t>2026-04-16</t>
         </is>
       </c>
       <c r="B43" t="n">
@@ -29306,19 +30343,19 @@
       </c>
       <c r="C43" t="inlineStr">
         <is>
-          <t>Barbaad</t>
+          <t>Teri Deewani</t>
         </is>
       </c>
       <c r="D43" t="inlineStr">
         <is>
-          <t>The Rish</t>
+          <t>Kailash Kher</t>
         </is>
       </c>
     </row>
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>2026-04-15</t>
+          <t>2026-04-16</t>
         </is>
       </c>
       <c r="B44" t="n">
@@ -29326,19 +30363,19 @@
       </c>
       <c r="C44" t="inlineStr">
         <is>
-          <t>Haseen</t>
+          <t>Jhol - Acoustic</t>
         </is>
       </c>
       <c r="D44" t="inlineStr">
         <is>
-          <t>Talwiinder</t>
+          <t>Maanu</t>
         </is>
       </c>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>2026-04-15</t>
+          <t>2026-04-16</t>
         </is>
       </c>
       <c r="B45" t="n">
@@ -29346,19 +30383,19 @@
       </c>
       <c r="C45" t="inlineStr">
         <is>
-          <t>Not Guilty</t>
+          <t>Zaalima</t>
         </is>
       </c>
       <c r="D45" t="inlineStr">
         <is>
-          <t>Dhanda Nyoliwala</t>
+          <t>Arijit Singh</t>
         </is>
       </c>
     </row>
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>2026-04-15</t>
+          <t>2026-04-16</t>
         </is>
       </c>
       <c r="B46" t="n">
@@ -29378,7 +30415,7 @@
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>2026-04-15</t>
+          <t>2026-04-16</t>
         </is>
       </c>
       <c r="B47" t="n">
@@ -29386,19 +30423,19 @@
       </c>
       <c r="C47" t="inlineStr">
         <is>
-          <t>Mann Mera - Original Version</t>
+          <t>Dhun</t>
         </is>
       </c>
       <c r="D47" t="inlineStr">
         <is>
-          <t>Gajendra Verma</t>
+          <t>Mithoon</t>
         </is>
       </c>
     </row>
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>2026-04-15</t>
+          <t>2026-04-16</t>
         </is>
       </c>
       <c r="B48" t="n">
@@ -29406,19 +30443,19 @@
       </c>
       <c r="C48" t="inlineStr">
         <is>
-          <t>Mast Magan</t>
+          <t>Jogi</t>
         </is>
       </c>
       <c r="D48" t="inlineStr">
         <is>
-          <t>Arijit Singh</t>
+          <t>thiarajxtt</t>
         </is>
       </c>
     </row>
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>2026-04-15</t>
+          <t>2026-04-16</t>
         </is>
       </c>
       <c r="B49" t="n">
@@ -29426,19 +30463,19 @@
       </c>
       <c r="C49" t="inlineStr">
         <is>
-          <t>Thodi Si Daaru</t>
+          <t>Not Guilty</t>
         </is>
       </c>
       <c r="D49" t="inlineStr">
         <is>
-          <t>AP Dhillon</t>
+          <t>Dhanda Nyoliwala</t>
         </is>
       </c>
     </row>
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>2026-04-15</t>
+          <t>2026-04-16</t>
         </is>
       </c>
       <c r="B50" t="n">
@@ -29446,19 +30483,19 @@
       </c>
       <c r="C50" t="inlineStr">
         <is>
-          <t>Jhol - Acoustic</t>
+          <t>Mann Mera - Original Version</t>
         </is>
       </c>
       <c r="D50" t="inlineStr">
         <is>
-          <t>Maanu</t>
+          <t>Gajendra Verma</t>
         </is>
       </c>
     </row>
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>2026-04-15</t>
+          <t>2026-04-16</t>
         </is>
       </c>
       <c r="B51" t="n">
@@ -29466,12 +30503,12 @@
       </c>
       <c r="C51" t="inlineStr">
         <is>
-          <t>Dhun</t>
+          <t>Mutta Kalakki</t>
         </is>
       </c>
       <c r="D51" t="inlineStr">
         <is>
-          <t>Mithoon</t>
+          <t>G. V. Prakash</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
got data for 18th and predictions for 19th april
</commit_message>
<xml_diff>
--- a/Probability Project.xlsx
+++ b/Probability Project.xlsx
@@ -37,6 +37,8 @@
     <sheet name="AUTO_20260413" sheetId="32" state="visible" r:id="rId32"/>
     <sheet name="AUTO_20260415" sheetId="33" state="visible" r:id="rId33"/>
     <sheet name="AUTO_20260416" sheetId="34" state="visible" r:id="rId34"/>
+    <sheet name="AUTO_20260418" sheetId="35" state="visible" r:id="rId35"/>
+    <sheet name="AUTO_20260417" sheetId="36" state="visible" r:id="rId36"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -29513,9 +29515,2081 @@
       </c>
     </row>
     <row r="2">
+      <c r="A2" s="0" t="inlineStr">
+        <is>
+          <t>2026-04-16</t>
+        </is>
+      </c>
+      <c r="B2" s="0" t="n">
+        <v>1</v>
+      </c>
+      <c r="C2" s="0" t="inlineStr">
+        <is>
+          <t>Bairan</t>
+        </is>
+      </c>
+      <c r="D2" s="0" t="inlineStr">
+        <is>
+          <t>Banjaare</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="0" t="inlineStr">
+        <is>
+          <t>2026-04-16</t>
+        </is>
+      </c>
+      <c r="B3" s="0" t="n">
+        <v>2</v>
+      </c>
+      <c r="C3" s="0" t="inlineStr">
+        <is>
+          <t>Sheesha - Aakhya Mai Aakh Ghali Jo Bairan</t>
+        </is>
+      </c>
+      <c r="D3" s="0" t="inlineStr">
+        <is>
+          <t>Mitta Ror</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="0" t="inlineStr">
+        <is>
+          <t>2026-04-16</t>
+        </is>
+      </c>
+      <c r="B4" s="0" t="n">
+        <v>3</v>
+      </c>
+      <c r="C4" s="0" t="inlineStr">
+        <is>
+          <t>Gehra Hua</t>
+        </is>
+      </c>
+      <c r="D4" s="0" t="inlineStr">
+        <is>
+          <t>Shashwat Sachdev</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="0" t="inlineStr">
+        <is>
+          <t>2026-04-16</t>
+        </is>
+      </c>
+      <c r="B5" s="0" t="n">
+        <v>4</v>
+      </c>
+      <c r="C5" s="0" t="inlineStr">
+        <is>
+          <t>Jaiye Sajana</t>
+        </is>
+      </c>
+      <c r="D5" s="0" t="inlineStr">
+        <is>
+          <t>Shashwat Sachdev</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="0" t="inlineStr">
+        <is>
+          <t>2026-04-16</t>
+        </is>
+      </c>
+      <c r="B6" s="0" t="n">
+        <v>5</v>
+      </c>
+      <c r="C6" s="0" t="inlineStr">
+        <is>
+          <t>Khat</t>
+        </is>
+      </c>
+      <c r="D6" s="0" t="inlineStr">
+        <is>
+          <t>Navjot Ahuja</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="0" t="inlineStr">
+        <is>
+          <t>2026-04-16</t>
+        </is>
+      </c>
+      <c r="B7" s="0" t="n">
+        <v>6</v>
+      </c>
+      <c r="C7" s="0" t="inlineStr">
+        <is>
+          <t>Dooron Dooron</t>
+        </is>
+      </c>
+      <c r="D7" s="0" t="inlineStr">
+        <is>
+          <t>Paresh Pahuja</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="0" t="inlineStr">
+        <is>
+          <t>2026-04-16</t>
+        </is>
+      </c>
+      <c r="B8" s="0" t="n">
+        <v>7</v>
+      </c>
+      <c r="C8" s="0" t="inlineStr">
+        <is>
+          <t>Sahiba</t>
+        </is>
+      </c>
+      <c r="D8" s="0" t="inlineStr">
+        <is>
+          <t>Aditya Rikhari</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="0" t="inlineStr">
+        <is>
+          <t>2026-04-16</t>
+        </is>
+      </c>
+      <c r="B9" s="0" t="n">
+        <v>8</v>
+      </c>
+      <c r="C9" s="0" t="inlineStr">
+        <is>
+          <t>Sitaare</t>
+        </is>
+      </c>
+      <c r="D9" s="0" t="inlineStr">
+        <is>
+          <t>Arijit Singh</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="0" t="inlineStr">
+        <is>
+          <t>2026-04-16</t>
+        </is>
+      </c>
+      <c r="B10" s="0" t="n">
+        <v>9</v>
+      </c>
+      <c r="C10" s="0" t="inlineStr">
+        <is>
+          <t>Finding Her</t>
+        </is>
+      </c>
+      <c r="D10" s="0" t="inlineStr">
+        <is>
+          <t>Kushagra</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="0" t="inlineStr">
+        <is>
+          <t>2026-04-16</t>
+        </is>
+      </c>
+      <c r="B11" s="0" t="n">
+        <v>10</v>
+      </c>
+      <c r="C11" s="0" t="inlineStr">
+        <is>
+          <t>Apna Bana Le</t>
+        </is>
+      </c>
+      <c r="D11" s="0" t="inlineStr">
+        <is>
+          <t>Sachin-Jigar</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="0" t="inlineStr">
+        <is>
+          <t>2026-04-16</t>
+        </is>
+      </c>
+      <c r="B12" s="0" t="n">
+        <v>11</v>
+      </c>
+      <c r="C12" s="0" t="inlineStr">
+        <is>
+          <t>Majboor</t>
+        </is>
+      </c>
+      <c r="D12" s="0" t="inlineStr">
+        <is>
+          <t>Sheheryar Rehan</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="0" t="inlineStr">
+        <is>
+          <t>2026-04-16</t>
+        </is>
+      </c>
+      <c r="B13" s="0" t="n">
+        <v>12</v>
+      </c>
+      <c r="C13" s="0" t="inlineStr">
+        <is>
+          <t>Arz Kiya Hai | Coke Studio Bharat</t>
+        </is>
+      </c>
+      <c r="D13" s="0" t="inlineStr">
+        <is>
+          <t>Anuv Jain</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="0" t="inlineStr">
+        <is>
+          <t>2026-04-16</t>
+        </is>
+      </c>
+      <c r="B14" s="0" t="n">
+        <v>13</v>
+      </c>
+      <c r="C14" s="0" t="inlineStr">
+        <is>
+          <t>Dhurandhar The Revenge - Aari Aari</t>
+        </is>
+      </c>
+      <c r="D14" s="0" t="inlineStr">
+        <is>
+          <t>Shashwat Sachdev</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="0" t="inlineStr">
+        <is>
+          <t>2026-04-16</t>
+        </is>
+      </c>
+      <c r="B15" s="0" t="n">
+        <v>14</v>
+      </c>
+      <c r="C15" s="0" t="inlineStr">
+        <is>
+          <t>Pavazha Malli</t>
+        </is>
+      </c>
+      <c r="D15" s="0" t="inlineStr">
+        <is>
+          <t>Sai Abhyankkar</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="0" t="inlineStr">
+        <is>
+          <t>2026-04-16</t>
+        </is>
+      </c>
+      <c r="B16" s="0" t="n">
+        <v>15</v>
+      </c>
+      <c r="C16" s="0" t="inlineStr">
+        <is>
+          <t>Samjhawan</t>
+        </is>
+      </c>
+      <c r="D16" s="0" t="inlineStr">
+        <is>
+          <t>Jawad Ahmad</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="0" t="inlineStr">
+        <is>
+          <t>2026-04-16</t>
+        </is>
+      </c>
+      <c r="B17" s="0" t="n">
+        <v>16</v>
+      </c>
+      <c r="C17" s="0" t="inlineStr">
+        <is>
+          <t>Boyfriend</t>
+        </is>
+      </c>
+      <c r="D17" s="0" t="inlineStr">
+        <is>
+          <t>Karan Aujla</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="0" t="inlineStr">
+        <is>
+          <t>2026-04-16</t>
+        </is>
+      </c>
+      <c r="B18" s="0" t="n">
+        <v>17</v>
+      </c>
+      <c r="C18" s="0" t="inlineStr">
+        <is>
+          <t>Jaan Se Guzarte Hain</t>
+        </is>
+      </c>
+      <c r="D18" s="0" t="inlineStr">
+        <is>
+          <t>Shashwat Sachdev</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="0" t="inlineStr">
+        <is>
+          <t>2026-04-16</t>
+        </is>
+      </c>
+      <c r="B19" s="0" t="n">
+        <v>18</v>
+      </c>
+      <c r="C19" s="0" t="inlineStr">
+        <is>
+          <t>Mann Mera</t>
+        </is>
+      </c>
+      <c r="D19" s="0" t="inlineStr">
+        <is>
+          <t>Gajendra Verma</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="0" t="inlineStr">
+        <is>
+          <t>2026-04-16</t>
+        </is>
+      </c>
+      <c r="B20" s="0" t="n">
+        <v>19</v>
+      </c>
+      <c r="C20" s="0" t="inlineStr">
+        <is>
+          <t>Ishq</t>
+        </is>
+      </c>
+      <c r="D20" s="0" t="inlineStr">
+        <is>
+          <t>Faheem Abdullah</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="0" t="inlineStr">
+        <is>
+          <t>2026-04-16</t>
+        </is>
+      </c>
+      <c r="B21" s="0" t="n">
+        <v>20</v>
+      </c>
+      <c r="C21" s="0" t="inlineStr">
+        <is>
+          <t>Shararat</t>
+        </is>
+      </c>
+      <c r="D21" s="0" t="inlineStr">
+        <is>
+          <t>Shashwat Sachdev</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="0" t="inlineStr">
+        <is>
+          <t>2026-04-16</t>
+        </is>
+      </c>
+      <c r="B22" s="0" t="n">
+        <v>21</v>
+      </c>
+      <c r="C22" s="0" t="inlineStr">
+        <is>
+          <t>Darkhaast</t>
+        </is>
+      </c>
+      <c r="D22" s="0" t="inlineStr">
+        <is>
+          <t>Mithoon</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="0" t="inlineStr">
+        <is>
+          <t>2026-04-16</t>
+        </is>
+      </c>
+      <c r="B23" s="0" t="n">
+        <v>22</v>
+      </c>
+      <c r="C23" s="0" t="inlineStr">
+        <is>
+          <t>Tum Ho Toh</t>
+        </is>
+      </c>
+      <c r="D23" s="0" t="inlineStr">
+        <is>
+          <t>Vishal Mishra</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="0" t="inlineStr">
+        <is>
+          <t>2026-04-16</t>
+        </is>
+      </c>
+      <c r="B24" s="0" t="n">
+        <v>23</v>
+      </c>
+      <c r="C24" s="0" t="inlineStr">
+        <is>
+          <t>For A Reason</t>
+        </is>
+      </c>
+      <c r="D24" s="0" t="inlineStr">
+        <is>
+          <t>Karan Aujla</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="0" t="inlineStr">
+        <is>
+          <t>2026-04-16</t>
+        </is>
+      </c>
+      <c r="B25" s="0" t="n">
+        <v>24</v>
+      </c>
+      <c r="C25" s="0" t="inlineStr">
+        <is>
+          <t>Ishqa Ve</t>
+        </is>
+      </c>
+      <c r="D25" s="0" t="inlineStr">
+        <is>
+          <t>Zeeshan Ali</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="0" t="inlineStr">
+        <is>
+          <t>2026-04-16</t>
+        </is>
+      </c>
+      <c r="B26" s="0" t="n">
+        <v>25</v>
+      </c>
+      <c r="C26" s="0" t="inlineStr">
+        <is>
+          <t>Deewaana Deewaana</t>
+        </is>
+      </c>
+      <c r="D26" s="0" t="inlineStr">
+        <is>
+          <t>A.R. Rahman</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="0" t="inlineStr">
+        <is>
+          <t>2026-04-16</t>
+        </is>
+      </c>
+      <c r="B27" s="0" t="n">
+        <v>26</v>
+      </c>
+      <c r="C27" s="0" t="inlineStr">
+        <is>
+          <t>Saiyaara</t>
+        </is>
+      </c>
+      <c r="D27" s="0" t="inlineStr">
+        <is>
+          <t>Tanishk Bagchi</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="0" t="inlineStr">
+        <is>
+          <t>2026-04-16</t>
+        </is>
+      </c>
+      <c r="B28" s="0" t="n">
+        <v>27</v>
+      </c>
+      <c r="C28" s="0" t="inlineStr">
+        <is>
+          <t>Bairi</t>
+        </is>
+      </c>
+      <c r="D28" s="0" t="inlineStr">
+        <is>
+          <t>Virat</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="0" t="inlineStr">
+        <is>
+          <t>2026-04-16</t>
+        </is>
+      </c>
+      <c r="B29" s="0" t="n">
+        <v>28</v>
+      </c>
+      <c r="C29" s="0" t="inlineStr">
+        <is>
+          <t>Raanjhan</t>
+        </is>
+      </c>
+      <c r="D29" s="0" t="inlineStr">
+        <is>
+          <t>Sachet-Parampara</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="0" t="inlineStr">
+        <is>
+          <t>2026-04-16</t>
+        </is>
+      </c>
+      <c r="B30" s="0" t="n">
+        <v>29</v>
+      </c>
+      <c r="C30" s="0" t="inlineStr">
+        <is>
+          <t>Tere Liye</t>
+        </is>
+      </c>
+      <c r="D30" s="0" t="inlineStr">
+        <is>
+          <t>Atif Aslam</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="0" t="inlineStr">
+        <is>
+          <t>2026-04-16</t>
+        </is>
+      </c>
+      <c r="B31" s="0" t="n">
+        <v>30</v>
+      </c>
+      <c r="C31" s="0" t="inlineStr">
+        <is>
+          <t>Dhurandhar - Title Track</t>
+        </is>
+      </c>
+      <c r="D31" s="0" t="inlineStr">
+        <is>
+          <t>Shashwat Sachdev</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="0" t="inlineStr">
+        <is>
+          <t>2026-04-16</t>
+        </is>
+      </c>
+      <c r="B32" s="0" t="n">
+        <v>31</v>
+      </c>
+      <c r="C32" s="0" t="inlineStr">
+        <is>
+          <t>Naal Nachna</t>
+        </is>
+      </c>
+      <c r="D32" s="0" t="inlineStr">
+        <is>
+          <t>Shashwat Sachdev</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="0" t="inlineStr">
+        <is>
+          <t>2026-04-16</t>
+        </is>
+      </c>
+      <c r="B33" s="0" t="n">
+        <v>32</v>
+      </c>
+      <c r="C33" s="0" t="inlineStr">
+        <is>
+          <t>Ehsaas</t>
+        </is>
+      </c>
+      <c r="D33" s="0" t="inlineStr">
+        <is>
+          <t>Faheem Abdullah</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="0" t="inlineStr">
+        <is>
+          <t>2026-04-16</t>
+        </is>
+      </c>
+      <c r="B34" s="0" t="n">
+        <v>33</v>
+      </c>
+      <c r="C34" s="0" t="inlineStr">
+        <is>
+          <t>Phir Se</t>
+        </is>
+      </c>
+      <c r="D34" s="0" t="inlineStr">
+        <is>
+          <t>Shashwat Sachdev</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="0" t="inlineStr">
+        <is>
+          <t>2026-04-16</t>
+        </is>
+      </c>
+      <c r="B35" s="0" t="n">
+        <v>34</v>
+      </c>
+      <c r="C35" s="0" t="inlineStr">
+        <is>
+          <t>Tere Bina</t>
+        </is>
+      </c>
+      <c r="D35" s="0" t="inlineStr">
+        <is>
+          <t>A.R. Rahman</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="0" t="inlineStr">
+        <is>
+          <t>2026-04-16</t>
+        </is>
+      </c>
+      <c r="B36" s="0" t="n">
+        <v>35</v>
+      </c>
+      <c r="C36" s="0" t="inlineStr">
+        <is>
+          <t>Jo Tum Mere Ho</t>
+        </is>
+      </c>
+      <c r="D36" s="0" t="inlineStr">
+        <is>
+          <t>Anuv Jain</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="0" t="inlineStr">
+        <is>
+          <t>2026-04-16</t>
+        </is>
+      </c>
+      <c r="B37" s="0" t="n">
+        <v>36</v>
+      </c>
+      <c r="C37" s="0" t="inlineStr">
+        <is>
+          <t>Agar Tum Saath Ho</t>
+        </is>
+      </c>
+      <c r="D37" s="0" t="inlineStr">
+        <is>
+          <t>Alka Yagnik</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="0" t="inlineStr">
+        <is>
+          <t>2026-04-16</t>
+        </is>
+      </c>
+      <c r="B38" s="0" t="n">
+        <v>37</v>
+      </c>
+      <c r="C38" s="0" t="inlineStr">
+        <is>
+          <t>Barbaad</t>
+        </is>
+      </c>
+      <c r="D38" s="0" t="inlineStr">
+        <is>
+          <t>The Rish</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="0" t="inlineStr">
+        <is>
+          <t>2026-04-16</t>
+        </is>
+      </c>
+      <c r="B39" s="0" t="n">
+        <v>38</v>
+      </c>
+      <c r="C39" s="0" t="inlineStr">
+        <is>
+          <t>Lutt Le Gaya</t>
+        </is>
+      </c>
+      <c r="D39" s="0" t="inlineStr">
+        <is>
+          <t>Shashwat Sachdev</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="0" t="inlineStr">
+        <is>
+          <t>2026-04-16</t>
+        </is>
+      </c>
+      <c r="B40" s="0" t="n">
+        <v>39</v>
+      </c>
+      <c r="C40" s="0" t="inlineStr">
+        <is>
+          <t>Run Down The City - Monica</t>
+        </is>
+      </c>
+      <c r="D40" s="0" t="inlineStr">
+        <is>
+          <t>Shashwat Sachdev</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" s="0" t="inlineStr">
+        <is>
+          <t>2026-04-16</t>
+        </is>
+      </c>
+      <c r="B41" s="0" t="n">
+        <v>40</v>
+      </c>
+      <c r="C41" s="0" t="inlineStr">
+        <is>
+          <t>Ye Tune Kya Kiya</t>
+        </is>
+      </c>
+      <c r="D41" s="0" t="inlineStr">
+        <is>
+          <t>Pritam</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" s="0" t="inlineStr">
+        <is>
+          <t>2026-04-16</t>
+        </is>
+      </c>
+      <c r="B42" s="0" t="n">
+        <v>41</v>
+      </c>
+      <c r="C42" s="0" t="inlineStr">
+        <is>
+          <t>Haseen</t>
+        </is>
+      </c>
+      <c r="D42" s="0" t="inlineStr">
+        <is>
+          <t>Talwiinder</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" s="0" t="inlineStr">
+        <is>
+          <t>2026-04-16</t>
+        </is>
+      </c>
+      <c r="B43" s="0" t="n">
+        <v>42</v>
+      </c>
+      <c r="C43" s="0" t="inlineStr">
+        <is>
+          <t>Teri Deewani</t>
+        </is>
+      </c>
+      <c r="D43" s="0" t="inlineStr">
+        <is>
+          <t>Kailash Kher</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" s="0" t="inlineStr">
+        <is>
+          <t>2026-04-16</t>
+        </is>
+      </c>
+      <c r="B44" s="0" t="n">
+        <v>43</v>
+      </c>
+      <c r="C44" s="0" t="inlineStr">
+        <is>
+          <t>Jhol - Acoustic</t>
+        </is>
+      </c>
+      <c r="D44" s="0" t="inlineStr">
+        <is>
+          <t>Maanu</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" s="0" t="inlineStr">
+        <is>
+          <t>2026-04-16</t>
+        </is>
+      </c>
+      <c r="B45" s="0" t="n">
+        <v>44</v>
+      </c>
+      <c r="C45" s="0" t="inlineStr">
+        <is>
+          <t>Zaalima</t>
+        </is>
+      </c>
+      <c r="D45" s="0" t="inlineStr">
+        <is>
+          <t>Arijit Singh</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" s="0" t="inlineStr">
+        <is>
+          <t>2026-04-16</t>
+        </is>
+      </c>
+      <c r="B46" s="0" t="n">
+        <v>45</v>
+      </c>
+      <c r="C46" s="0" t="inlineStr">
+        <is>
+          <t>High On You</t>
+        </is>
+      </c>
+      <c r="D46" s="0" t="inlineStr">
+        <is>
+          <t>Jind Universe</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" s="0" t="inlineStr">
+        <is>
+          <t>2026-04-16</t>
+        </is>
+      </c>
+      <c r="B47" s="0" t="n">
+        <v>46</v>
+      </c>
+      <c r="C47" s="0" t="inlineStr">
+        <is>
+          <t>Dhun</t>
+        </is>
+      </c>
+      <c r="D47" s="0" t="inlineStr">
+        <is>
+          <t>Mithoon</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" s="0" t="inlineStr">
+        <is>
+          <t>2026-04-16</t>
+        </is>
+      </c>
+      <c r="B48" s="0" t="n">
+        <v>47</v>
+      </c>
+      <c r="C48" s="0" t="inlineStr">
+        <is>
+          <t>Jogi</t>
+        </is>
+      </c>
+      <c r="D48" s="0" t="inlineStr">
+        <is>
+          <t>thiarajxtt</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" s="0" t="inlineStr">
+        <is>
+          <t>2026-04-16</t>
+        </is>
+      </c>
+      <c r="B49" s="0" t="n">
+        <v>48</v>
+      </c>
+      <c r="C49" s="0" t="inlineStr">
+        <is>
+          <t>Not Guilty</t>
+        </is>
+      </c>
+      <c r="D49" s="0" t="inlineStr">
+        <is>
+          <t>Dhanda Nyoliwala</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" s="0" t="inlineStr">
+        <is>
+          <t>2026-04-16</t>
+        </is>
+      </c>
+      <c r="B50" s="0" t="n">
+        <v>49</v>
+      </c>
+      <c r="C50" s="0" t="inlineStr">
+        <is>
+          <t>Mann Mera - Original Version</t>
+        </is>
+      </c>
+      <c r="D50" s="0" t="inlineStr">
+        <is>
+          <t>Gajendra Verma</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" s="0" t="inlineStr">
+        <is>
+          <t>2026-04-16</t>
+        </is>
+      </c>
+      <c r="B51" s="0" t="n">
+        <v>50</v>
+      </c>
+      <c r="C51" s="0" t="inlineStr">
+        <is>
+          <t>Mutta Kalakki</t>
+        </is>
+      </c>
+      <c r="D51" s="0" t="inlineStr">
+        <is>
+          <t>G. V. Prakash</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet35.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:D51"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="24" t="inlineStr">
+        <is>
+          <t>Date</t>
+        </is>
+      </c>
+      <c r="B1" s="24" t="inlineStr">
+        <is>
+          <t>Rank</t>
+        </is>
+      </c>
+      <c r="C1" s="24" t="inlineStr">
+        <is>
+          <t>Song</t>
+        </is>
+      </c>
+      <c r="D1" s="24" t="inlineStr">
+        <is>
+          <t>Artist</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="0" t="inlineStr">
+        <is>
+          <t>2026-04-18</t>
+        </is>
+      </c>
+      <c r="B2" s="0" t="n">
+        <v>1</v>
+      </c>
+      <c r="C2" s="0" t="inlineStr">
+        <is>
+          <t>Bairan</t>
+        </is>
+      </c>
+      <c r="D2" s="0" t="inlineStr">
+        <is>
+          <t>Banjaare</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="0" t="inlineStr">
+        <is>
+          <t>2026-04-18</t>
+        </is>
+      </c>
+      <c r="B3" s="0" t="n">
+        <v>2</v>
+      </c>
+      <c r="C3" s="0" t="inlineStr">
+        <is>
+          <t>Gehra Hua</t>
+        </is>
+      </c>
+      <c r="D3" s="0" t="inlineStr">
+        <is>
+          <t>Shashwat Sachdev</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="0" t="inlineStr">
+        <is>
+          <t>2026-04-18</t>
+        </is>
+      </c>
+      <c r="B4" s="0" t="n">
+        <v>3</v>
+      </c>
+      <c r="C4" s="0" t="inlineStr">
+        <is>
+          <t>Sheesha - Aakhya Mai Aakh Ghali Jo Bairan</t>
+        </is>
+      </c>
+      <c r="D4" s="0" t="inlineStr">
+        <is>
+          <t>Mitta Ror</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="0" t="inlineStr">
+        <is>
+          <t>2026-04-18</t>
+        </is>
+      </c>
+      <c r="B5" s="0" t="n">
+        <v>4</v>
+      </c>
+      <c r="C5" s="0" t="inlineStr">
+        <is>
+          <t>Jaiye Sajana</t>
+        </is>
+      </c>
+      <c r="D5" s="0" t="inlineStr">
+        <is>
+          <t>Shashwat Sachdev</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="0" t="inlineStr">
+        <is>
+          <t>2026-04-18</t>
+        </is>
+      </c>
+      <c r="B6" s="0" t="n">
+        <v>5</v>
+      </c>
+      <c r="C6" s="0" t="inlineStr">
+        <is>
+          <t>Khat</t>
+        </is>
+      </c>
+      <c r="D6" s="0" t="inlineStr">
+        <is>
+          <t>Navjot Ahuja</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="0" t="inlineStr">
+        <is>
+          <t>2026-04-18</t>
+        </is>
+      </c>
+      <c r="B7" s="0" t="n">
+        <v>6</v>
+      </c>
+      <c r="C7" s="0" t="inlineStr">
+        <is>
+          <t>Majboor</t>
+        </is>
+      </c>
+      <c r="D7" s="0" t="inlineStr">
+        <is>
+          <t>Sheheryar Rehan</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="0" t="inlineStr">
+        <is>
+          <t>2026-04-18</t>
+        </is>
+      </c>
+      <c r="B8" s="0" t="n">
+        <v>7</v>
+      </c>
+      <c r="C8" s="0" t="inlineStr">
+        <is>
+          <t>Sahiba</t>
+        </is>
+      </c>
+      <c r="D8" s="0" t="inlineStr">
+        <is>
+          <t>Aditya Rikhari</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="0" t="inlineStr">
+        <is>
+          <t>2026-04-18</t>
+        </is>
+      </c>
+      <c r="B9" s="0" t="n">
+        <v>8</v>
+      </c>
+      <c r="C9" s="0" t="inlineStr">
+        <is>
+          <t>Sitaare</t>
+        </is>
+      </c>
+      <c r="D9" s="0" t="inlineStr">
+        <is>
+          <t>Arijit Singh</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="0" t="inlineStr">
+        <is>
+          <t>2026-04-18</t>
+        </is>
+      </c>
+      <c r="B10" s="0" t="n">
+        <v>9</v>
+      </c>
+      <c r="C10" s="0" t="inlineStr">
+        <is>
+          <t>Dooron Dooron</t>
+        </is>
+      </c>
+      <c r="D10" s="0" t="inlineStr">
+        <is>
+          <t>Paresh Pahuja</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="0" t="inlineStr">
+        <is>
+          <t>2026-04-18</t>
+        </is>
+      </c>
+      <c r="B11" s="0" t="n">
+        <v>10</v>
+      </c>
+      <c r="C11" s="0" t="inlineStr">
+        <is>
+          <t>Finding Her</t>
+        </is>
+      </c>
+      <c r="D11" s="0" t="inlineStr">
+        <is>
+          <t>Kushagra</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="0" t="inlineStr">
+        <is>
+          <t>2026-04-18</t>
+        </is>
+      </c>
+      <c r="B12" s="0" t="n">
+        <v>11</v>
+      </c>
+      <c r="C12" s="0" t="inlineStr">
+        <is>
+          <t>Samjhawan</t>
+        </is>
+      </c>
+      <c r="D12" s="0" t="inlineStr">
+        <is>
+          <t>Jawad Ahmad</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="0" t="inlineStr">
+        <is>
+          <t>2026-04-18</t>
+        </is>
+      </c>
+      <c r="B13" s="0" t="n">
+        <v>12</v>
+      </c>
+      <c r="C13" s="0" t="inlineStr">
+        <is>
+          <t>Pavazha Malli</t>
+        </is>
+      </c>
+      <c r="D13" s="0" t="inlineStr">
+        <is>
+          <t>Sai Abhyankkar</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="0" t="inlineStr">
+        <is>
+          <t>2026-04-18</t>
+        </is>
+      </c>
+      <c r="B14" s="0" t="n">
+        <v>13</v>
+      </c>
+      <c r="C14" s="0" t="inlineStr">
+        <is>
+          <t>Apna Bana Le</t>
+        </is>
+      </c>
+      <c r="D14" s="0" t="inlineStr">
+        <is>
+          <t>Sachin-Jigar</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="0" t="inlineStr">
+        <is>
+          <t>2026-04-18</t>
+        </is>
+      </c>
+      <c r="B15" s="0" t="n">
+        <v>14</v>
+      </c>
+      <c r="C15" s="0" t="inlineStr">
+        <is>
+          <t>Arz Kiya Hai | Coke Studio Bharat</t>
+        </is>
+      </c>
+      <c r="D15" s="0" t="inlineStr">
+        <is>
+          <t>Anuv Jain</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="0" t="inlineStr">
+        <is>
+          <t>2026-04-18</t>
+        </is>
+      </c>
+      <c r="B16" s="0" t="n">
+        <v>15</v>
+      </c>
+      <c r="C16" s="0" t="inlineStr">
+        <is>
+          <t>Dhurandhar The Revenge - Aari Aari</t>
+        </is>
+      </c>
+      <c r="D16" s="0" t="inlineStr">
+        <is>
+          <t>Shashwat Sachdev</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="0" t="inlineStr">
+        <is>
+          <t>2026-04-18</t>
+        </is>
+      </c>
+      <c r="B17" s="0" t="n">
+        <v>16</v>
+      </c>
+      <c r="C17" s="0" t="inlineStr">
+        <is>
+          <t>Boyfriend</t>
+        </is>
+      </c>
+      <c r="D17" s="0" t="inlineStr">
+        <is>
+          <t>Karan Aujla</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="0" t="inlineStr">
+        <is>
+          <t>2026-04-18</t>
+        </is>
+      </c>
+      <c r="B18" s="0" t="n">
+        <v>17</v>
+      </c>
+      <c r="C18" s="0" t="inlineStr">
+        <is>
+          <t>Shararat</t>
+        </is>
+      </c>
+      <c r="D18" s="0" t="inlineStr">
+        <is>
+          <t>Shashwat Sachdev</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="0" t="inlineStr">
+        <is>
+          <t>2026-04-18</t>
+        </is>
+      </c>
+      <c r="B19" s="0" t="n">
+        <v>18</v>
+      </c>
+      <c r="C19" s="0" t="inlineStr">
+        <is>
+          <t>Mann Mera</t>
+        </is>
+      </c>
+      <c r="D19" s="0" t="inlineStr">
+        <is>
+          <t>Gajendra Verma</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="0" t="inlineStr">
+        <is>
+          <t>2026-04-18</t>
+        </is>
+      </c>
+      <c r="B20" s="0" t="n">
+        <v>19</v>
+      </c>
+      <c r="C20" s="0" t="inlineStr">
+        <is>
+          <t>Jaan Se Guzarte Hain</t>
+        </is>
+      </c>
+      <c r="D20" s="0" t="inlineStr">
+        <is>
+          <t>Shashwat Sachdev</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="0" t="inlineStr">
+        <is>
+          <t>2026-04-18</t>
+        </is>
+      </c>
+      <c r="B21" s="0" t="n">
+        <v>20</v>
+      </c>
+      <c r="C21" s="0" t="inlineStr">
+        <is>
+          <t>Ishq</t>
+        </is>
+      </c>
+      <c r="D21" s="0" t="inlineStr">
+        <is>
+          <t>Faheem Abdullah</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="0" t="inlineStr">
+        <is>
+          <t>2026-04-18</t>
+        </is>
+      </c>
+      <c r="B22" s="0" t="n">
+        <v>21</v>
+      </c>
+      <c r="C22" s="0" t="inlineStr">
+        <is>
+          <t>Tum Ho Toh</t>
+        </is>
+      </c>
+      <c r="D22" s="0" t="inlineStr">
+        <is>
+          <t>Vishal Mishra</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="0" t="inlineStr">
+        <is>
+          <t>2026-04-18</t>
+        </is>
+      </c>
+      <c r="B23" s="0" t="n">
+        <v>22</v>
+      </c>
+      <c r="C23" s="0" t="inlineStr">
+        <is>
+          <t>Ishqa Ve</t>
+        </is>
+      </c>
+      <c r="D23" s="0" t="inlineStr">
+        <is>
+          <t>Zeeshan Ali</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="0" t="inlineStr">
+        <is>
+          <t>2026-04-18</t>
+        </is>
+      </c>
+      <c r="B24" s="0" t="n">
+        <v>23</v>
+      </c>
+      <c r="C24" s="0" t="inlineStr">
+        <is>
+          <t>Saiyaara</t>
+        </is>
+      </c>
+      <c r="D24" s="0" t="inlineStr">
+        <is>
+          <t>Tanishk Bagchi</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="0" t="inlineStr">
+        <is>
+          <t>2026-04-18</t>
+        </is>
+      </c>
+      <c r="B25" s="0" t="n">
+        <v>24</v>
+      </c>
+      <c r="C25" s="0" t="inlineStr">
+        <is>
+          <t>For A Reason</t>
+        </is>
+      </c>
+      <c r="D25" s="0" t="inlineStr">
+        <is>
+          <t>Karan Aujla</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="0" t="inlineStr">
+        <is>
+          <t>2026-04-18</t>
+        </is>
+      </c>
+      <c r="B26" s="0" t="n">
+        <v>25</v>
+      </c>
+      <c r="C26" s="0" t="inlineStr">
+        <is>
+          <t>Raanjhan</t>
+        </is>
+      </c>
+      <c r="D26" s="0" t="inlineStr">
+        <is>
+          <t>Sachet-Parampara</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="0" t="inlineStr">
+        <is>
+          <t>2026-04-18</t>
+        </is>
+      </c>
+      <c r="B27" s="0" t="n">
+        <v>26</v>
+      </c>
+      <c r="C27" s="0" t="inlineStr">
+        <is>
+          <t>Tere Liye</t>
+        </is>
+      </c>
+      <c r="D27" s="0" t="inlineStr">
+        <is>
+          <t>Atif Aslam</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="0" t="inlineStr">
+        <is>
+          <t>2026-04-18</t>
+        </is>
+      </c>
+      <c r="B28" s="0" t="n">
+        <v>27</v>
+      </c>
+      <c r="C28" s="0" t="inlineStr">
+        <is>
+          <t>Darkhaast</t>
+        </is>
+      </c>
+      <c r="D28" s="0" t="inlineStr">
+        <is>
+          <t>Mithoon</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="0" t="inlineStr">
+        <is>
+          <t>2026-04-18</t>
+        </is>
+      </c>
+      <c r="B29" s="0" t="n">
+        <v>28</v>
+      </c>
+      <c r="C29" s="0" t="inlineStr">
+        <is>
+          <t>Dhurandhar - Title Track</t>
+        </is>
+      </c>
+      <c r="D29" s="0" t="inlineStr">
+        <is>
+          <t>Shashwat Sachdev</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="0" t="inlineStr">
+        <is>
+          <t>2026-04-18</t>
+        </is>
+      </c>
+      <c r="B30" s="0" t="n">
+        <v>29</v>
+      </c>
+      <c r="C30" s="0" t="inlineStr">
+        <is>
+          <t>Bairi</t>
+        </is>
+      </c>
+      <c r="D30" s="0" t="inlineStr">
+        <is>
+          <t>Virat</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="0" t="inlineStr">
+        <is>
+          <t>2026-04-18</t>
+        </is>
+      </c>
+      <c r="B31" s="0" t="n">
+        <v>30</v>
+      </c>
+      <c r="C31" s="0" t="inlineStr">
+        <is>
+          <t>Deewaana Deewaana</t>
+        </is>
+      </c>
+      <c r="D31" s="0" t="inlineStr">
+        <is>
+          <t>A.R. Rahman</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="0" t="inlineStr">
+        <is>
+          <t>2026-04-18</t>
+        </is>
+      </c>
+      <c r="B32" s="0" t="n">
+        <v>31</v>
+      </c>
+      <c r="C32" s="0" t="inlineStr">
+        <is>
+          <t>Naal Nachna</t>
+        </is>
+      </c>
+      <c r="D32" s="0" t="inlineStr">
+        <is>
+          <t>Shashwat Sachdev</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="0" t="inlineStr">
+        <is>
+          <t>2026-04-18</t>
+        </is>
+      </c>
+      <c r="B33" s="0" t="n">
+        <v>32</v>
+      </c>
+      <c r="C33" s="0" t="inlineStr">
+        <is>
+          <t>Agar Tum Saath Ho</t>
+        </is>
+      </c>
+      <c r="D33" s="0" t="inlineStr">
+        <is>
+          <t>Alka Yagnik</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="0" t="inlineStr">
+        <is>
+          <t>2026-04-18</t>
+        </is>
+      </c>
+      <c r="B34" s="0" t="n">
+        <v>33</v>
+      </c>
+      <c r="C34" s="0" t="inlineStr">
+        <is>
+          <t>Tere Bina</t>
+        </is>
+      </c>
+      <c r="D34" s="0" t="inlineStr">
+        <is>
+          <t>A.R. Rahman</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="0" t="inlineStr">
+        <is>
+          <t>2026-04-18</t>
+        </is>
+      </c>
+      <c r="B35" s="0" t="n">
+        <v>34</v>
+      </c>
+      <c r="C35" s="0" t="inlineStr">
+        <is>
+          <t>Jo Tum Mere Ho</t>
+        </is>
+      </c>
+      <c r="D35" s="0" t="inlineStr">
+        <is>
+          <t>Anuv Jain</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="0" t="inlineStr">
+        <is>
+          <t>2026-04-18</t>
+        </is>
+      </c>
+      <c r="B36" s="0" t="n">
+        <v>35</v>
+      </c>
+      <c r="C36" s="0" t="inlineStr">
+        <is>
+          <t>Ehsaas</t>
+        </is>
+      </c>
+      <c r="D36" s="0" t="inlineStr">
+        <is>
+          <t>Faheem Abdullah</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="0" t="inlineStr">
+        <is>
+          <t>2026-04-18</t>
+        </is>
+      </c>
+      <c r="B37" s="0" t="n">
+        <v>36</v>
+      </c>
+      <c r="C37" s="0" t="inlineStr">
+        <is>
+          <t>Phir Se</t>
+        </is>
+      </c>
+      <c r="D37" s="0" t="inlineStr">
+        <is>
+          <t>Shashwat Sachdev</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="0" t="inlineStr">
+        <is>
+          <t>2026-04-18</t>
+        </is>
+      </c>
+      <c r="B38" s="0" t="n">
+        <v>37</v>
+      </c>
+      <c r="C38" s="0" t="inlineStr">
+        <is>
+          <t>Ye Tune Kya Kiya</t>
+        </is>
+      </c>
+      <c r="D38" s="0" t="inlineStr">
+        <is>
+          <t>Pritam</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="0" t="inlineStr">
+        <is>
+          <t>2026-04-18</t>
+        </is>
+      </c>
+      <c r="B39" s="0" t="n">
+        <v>38</v>
+      </c>
+      <c r="C39" s="0" t="inlineStr">
+        <is>
+          <t>Run Down The City - Monica</t>
+        </is>
+      </c>
+      <c r="D39" s="0" t="inlineStr">
+        <is>
+          <t>Shashwat Sachdev</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="0" t="inlineStr">
+        <is>
+          <t>2026-04-18</t>
+        </is>
+      </c>
+      <c r="B40" s="0" t="n">
+        <v>39</v>
+      </c>
+      <c r="C40" s="0" t="inlineStr">
+        <is>
+          <t>Haseen</t>
+        </is>
+      </c>
+      <c r="D40" s="0" t="inlineStr">
+        <is>
+          <t>Talwiinder</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" s="0" t="inlineStr">
+        <is>
+          <t>2026-04-18</t>
+        </is>
+      </c>
+      <c r="B41" s="0" t="n">
+        <v>40</v>
+      </c>
+      <c r="C41" s="0" t="inlineStr">
+        <is>
+          <t>Lutt Le Gaya</t>
+        </is>
+      </c>
+      <c r="D41" s="0" t="inlineStr">
+        <is>
+          <t>Shashwat Sachdev</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" s="0" t="inlineStr">
+        <is>
+          <t>2026-04-18</t>
+        </is>
+      </c>
+      <c r="B42" s="0" t="n">
+        <v>41</v>
+      </c>
+      <c r="C42" s="0" t="inlineStr">
+        <is>
+          <t>Barbaad</t>
+        </is>
+      </c>
+      <c r="D42" s="0" t="inlineStr">
+        <is>
+          <t>The Rish</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" s="0" t="inlineStr">
+        <is>
+          <t>2026-04-18</t>
+        </is>
+      </c>
+      <c r="B43" s="0" t="n">
+        <v>42</v>
+      </c>
+      <c r="C43" s="0" t="inlineStr">
+        <is>
+          <t>Mast Magan</t>
+        </is>
+      </c>
+      <c r="D43" s="0" t="inlineStr">
+        <is>
+          <t>Arijit Singh</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" s="0" t="inlineStr">
+        <is>
+          <t>2026-04-18</t>
+        </is>
+      </c>
+      <c r="B44" s="0" t="n">
+        <v>43</v>
+      </c>
+      <c r="C44" s="0" t="inlineStr">
+        <is>
+          <t>Mutta Kalakki</t>
+        </is>
+      </c>
+      <c r="D44" s="0" t="inlineStr">
+        <is>
+          <t>G. V. Prakash</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" s="0" t="inlineStr">
+        <is>
+          <t>2026-04-18</t>
+        </is>
+      </c>
+      <c r="B45" s="0" t="n">
+        <v>44</v>
+      </c>
+      <c r="C45" s="0" t="inlineStr">
+        <is>
+          <t>Zaalima</t>
+        </is>
+      </c>
+      <c r="D45" s="0" t="inlineStr">
+        <is>
+          <t>Arijit Singh</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" s="0" t="inlineStr">
+        <is>
+          <t>2026-04-18</t>
+        </is>
+      </c>
+      <c r="B46" s="0" t="n">
+        <v>45</v>
+      </c>
+      <c r="C46" s="0" t="inlineStr">
+        <is>
+          <t>High On You</t>
+        </is>
+      </c>
+      <c r="D46" s="0" t="inlineStr">
+        <is>
+          <t>Jind Universe</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" s="0" t="inlineStr">
+        <is>
+          <t>2026-04-18</t>
+        </is>
+      </c>
+      <c r="B47" s="0" t="n">
+        <v>46</v>
+      </c>
+      <c r="C47" s="0" t="inlineStr">
+        <is>
+          <t>Teri Deewani</t>
+        </is>
+      </c>
+      <c r="D47" s="0" t="inlineStr">
+        <is>
+          <t>Kailash Kher</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" s="0" t="inlineStr">
+        <is>
+          <t>2026-04-18</t>
+        </is>
+      </c>
+      <c r="B48" s="0" t="n">
+        <v>47</v>
+      </c>
+      <c r="C48" s="0" t="inlineStr">
+        <is>
+          <t>Dhun</t>
+        </is>
+      </c>
+      <c r="D48" s="0" t="inlineStr">
+        <is>
+          <t>Mithoon</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" s="0" t="inlineStr">
+        <is>
+          <t>2026-04-18</t>
+        </is>
+      </c>
+      <c r="B49" s="0" t="n">
+        <v>48</v>
+      </c>
+      <c r="C49" s="0" t="inlineStr">
+        <is>
+          <t>Thodi Si Daaru</t>
+        </is>
+      </c>
+      <c r="D49" s="0" t="inlineStr">
+        <is>
+          <t>AP Dhillon</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" s="0" t="inlineStr">
+        <is>
+          <t>2026-04-18</t>
+        </is>
+      </c>
+      <c r="B50" s="0" t="n">
+        <v>49</v>
+      </c>
+      <c r="C50" s="0" t="inlineStr">
+        <is>
+          <t>Aaya Sher</t>
+        </is>
+      </c>
+      <c r="D50" s="0" t="inlineStr">
+        <is>
+          <t>Anirudh Ravichander</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" s="0" t="inlineStr">
+        <is>
+          <t>2026-04-18</t>
+        </is>
+      </c>
+      <c r="B51" s="0" t="n">
+        <v>50</v>
+      </c>
+      <c r="C51" s="0" t="inlineStr">
+        <is>
+          <t>Jhol - Acoustic</t>
+        </is>
+      </c>
+      <c r="D51" s="0" t="inlineStr">
+        <is>
+          <t>Maanu</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet36.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:D51"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="24" t="inlineStr">
+        <is>
+          <t>Date</t>
+        </is>
+      </c>
+      <c r="B1" s="24" t="inlineStr">
+        <is>
+          <t>Rank</t>
+        </is>
+      </c>
+      <c r="C1" s="24" t="inlineStr">
+        <is>
+          <t>Song</t>
+        </is>
+      </c>
+      <c r="D1" s="24" t="inlineStr">
+        <is>
+          <t>Artist</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>2026-04-16</t>
+          <t>2026-04-17</t>
         </is>
       </c>
       <c r="B2" t="n">
@@ -29535,7 +31609,7 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>2026-04-16</t>
+          <t>2026-04-17</t>
         </is>
       </c>
       <c r="B3" t="n">
@@ -29543,19 +31617,19 @@
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>Sheesha - Aakhya Mai Aakh Ghali Jo Bairan</t>
+          <t>Gehra Hua</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>Mitta Ror</t>
+          <t>Shashwat Sachdev</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>2026-04-16</t>
+          <t>2026-04-17</t>
         </is>
       </c>
       <c r="B4" t="n">
@@ -29563,7 +31637,7 @@
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>Gehra Hua</t>
+          <t>Jaiye Sajana</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
@@ -29575,7 +31649,7 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>2026-04-16</t>
+          <t>2026-04-17</t>
         </is>
       </c>
       <c r="B5" t="n">
@@ -29583,19 +31657,19 @@
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>Jaiye Sajana</t>
+          <t>Khat</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>Shashwat Sachdev</t>
+          <t>Navjot Ahuja</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>2026-04-16</t>
+          <t>2026-04-17</t>
         </is>
       </c>
       <c r="B6" t="n">
@@ -29603,19 +31677,19 @@
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>Khat</t>
+          <t>Sheesha - Aakhya Mai Aakh Ghali Jo Bairan</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>Navjot Ahuja</t>
+          <t>Mitta Ror</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>2026-04-16</t>
+          <t>2026-04-17</t>
         </is>
       </c>
       <c r="B7" t="n">
@@ -29623,19 +31697,19 @@
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>Dooron Dooron</t>
+          <t>Sitaare</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>Paresh Pahuja</t>
+          <t>Arijit Singh</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>2026-04-16</t>
+          <t>2026-04-17</t>
         </is>
       </c>
       <c r="B8" t="n">
@@ -29655,7 +31729,7 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>2026-04-16</t>
+          <t>2026-04-17</t>
         </is>
       </c>
       <c r="B9" t="n">
@@ -29663,19 +31737,19 @@
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>Sitaare</t>
+          <t>Dooron Dooron</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>Arijit Singh</t>
+          <t>Paresh Pahuja</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>2026-04-16</t>
+          <t>2026-04-17</t>
         </is>
       </c>
       <c r="B10" t="n">
@@ -29683,19 +31757,19 @@
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>Finding Her</t>
+          <t>Majboor</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>Kushagra</t>
+          <t>Sheheryar Rehan</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>2026-04-16</t>
+          <t>2026-04-17</t>
         </is>
       </c>
       <c r="B11" t="n">
@@ -29703,19 +31777,19 @@
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>Apna Bana Le</t>
+          <t>Finding Her</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>Sachin-Jigar</t>
+          <t>Kushagra</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>2026-04-16</t>
+          <t>2026-04-17</t>
         </is>
       </c>
       <c r="B12" t="n">
@@ -29723,19 +31797,19 @@
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>Majboor</t>
+          <t>Samjhawan</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>Sheheryar Rehan</t>
+          <t>Jawad Ahmad</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>2026-04-16</t>
+          <t>2026-04-17</t>
         </is>
       </c>
       <c r="B13" t="n">
@@ -29743,19 +31817,19 @@
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>Arz Kiya Hai | Coke Studio Bharat</t>
+          <t>Pavazha Malli</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>Anuv Jain</t>
+          <t>Sai Abhyankkar</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>2026-04-16</t>
+          <t>2026-04-17</t>
         </is>
       </c>
       <c r="B14" t="n">
@@ -29763,19 +31837,19 @@
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>Dhurandhar The Revenge - Aari Aari</t>
+          <t>Arz Kiya Hai | Coke Studio Bharat</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>Shashwat Sachdev</t>
+          <t>Anuv Jain</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>2026-04-16</t>
+          <t>2026-04-17</t>
         </is>
       </c>
       <c r="B15" t="n">
@@ -29783,19 +31857,19 @@
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>Pavazha Malli</t>
+          <t>Apna Bana Le</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>Sai Abhyankkar</t>
+          <t>Sachin-Jigar</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>2026-04-16</t>
+          <t>2026-04-17</t>
         </is>
       </c>
       <c r="B16" t="n">
@@ -29803,19 +31877,19 @@
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>Samjhawan</t>
+          <t>Boyfriend</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>Jawad Ahmad</t>
+          <t>Karan Aujla</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>2026-04-16</t>
+          <t>2026-04-17</t>
         </is>
       </c>
       <c r="B17" t="n">
@@ -29823,19 +31897,19 @@
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>Boyfriend</t>
+          <t>Dhurandhar The Revenge - Aari Aari</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>Karan Aujla</t>
+          <t>Shashwat Sachdev</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>2026-04-16</t>
+          <t>2026-04-17</t>
         </is>
       </c>
       <c r="B18" t="n">
@@ -29855,7 +31929,7 @@
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>2026-04-16</t>
+          <t>2026-04-17</t>
         </is>
       </c>
       <c r="B19" t="n">
@@ -29863,19 +31937,19 @@
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>Mann Mera</t>
+          <t>Ishq</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>Gajendra Verma</t>
+          <t>Faheem Abdullah</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>2026-04-16</t>
+          <t>2026-04-17</t>
         </is>
       </c>
       <c r="B20" t="n">
@@ -29883,19 +31957,19 @@
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>Ishq</t>
+          <t>Mann Mera</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>Faheem Abdullah</t>
+          <t>Gajendra Verma</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>2026-04-16</t>
+          <t>2026-04-17</t>
         </is>
       </c>
       <c r="B21" t="n">
@@ -29915,7 +31989,7 @@
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>2026-04-16</t>
+          <t>2026-04-17</t>
         </is>
       </c>
       <c r="B22" t="n">
@@ -29923,19 +31997,19 @@
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>Darkhaast</t>
+          <t>For A Reason</t>
         </is>
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>Mithoon</t>
+          <t>Karan Aujla</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>2026-04-16</t>
+          <t>2026-04-17</t>
         </is>
       </c>
       <c r="B23" t="n">
@@ -29943,19 +32017,19 @@
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>Tum Ho Toh</t>
+          <t>Saiyaara</t>
         </is>
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>Vishal Mishra</t>
+          <t>Tanishk Bagchi</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>2026-04-16</t>
+          <t>2026-04-17</t>
         </is>
       </c>
       <c r="B24" t="n">
@@ -29963,19 +32037,19 @@
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>For A Reason</t>
+          <t>Tum Ho Toh</t>
         </is>
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>Karan Aujla</t>
+          <t>Vishal Mishra</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>2026-04-16</t>
+          <t>2026-04-17</t>
         </is>
       </c>
       <c r="B25" t="n">
@@ -29995,7 +32069,7 @@
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>2026-04-16</t>
+          <t>2026-04-17</t>
         </is>
       </c>
       <c r="B26" t="n">
@@ -30015,7 +32089,7 @@
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>2026-04-16</t>
+          <t>2026-04-17</t>
         </is>
       </c>
       <c r="B27" t="n">
@@ -30023,19 +32097,19 @@
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>Saiyaara</t>
+          <t>Raanjhan</t>
         </is>
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t>Tanishk Bagchi</t>
+          <t>Sachet-Parampara</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>2026-04-16</t>
+          <t>2026-04-17</t>
         </is>
       </c>
       <c r="B28" t="n">
@@ -30043,19 +32117,19 @@
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>Bairi</t>
+          <t>Darkhaast</t>
         </is>
       </c>
       <c r="D28" t="inlineStr">
         <is>
-          <t>Virat</t>
+          <t>Mithoon</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>2026-04-16</t>
+          <t>2026-04-17</t>
         </is>
       </c>
       <c r="B29" t="n">
@@ -30063,19 +32137,19 @@
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>Raanjhan</t>
+          <t>Tere Liye</t>
         </is>
       </c>
       <c r="D29" t="inlineStr">
         <is>
-          <t>Sachet-Parampara</t>
+          <t>Atif Aslam</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>2026-04-16</t>
+          <t>2026-04-17</t>
         </is>
       </c>
       <c r="B30" t="n">
@@ -30083,19 +32157,19 @@
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>Tere Liye</t>
+          <t>Dhurandhar - Title Track</t>
         </is>
       </c>
       <c r="D30" t="inlineStr">
         <is>
-          <t>Atif Aslam</t>
+          <t>Shashwat Sachdev</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>2026-04-16</t>
+          <t>2026-04-17</t>
         </is>
       </c>
       <c r="B31" t="n">
@@ -30103,7 +32177,7 @@
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>Dhurandhar - Title Track</t>
+          <t>Naal Nachna</t>
         </is>
       </c>
       <c r="D31" t="inlineStr">
@@ -30115,7 +32189,7 @@
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>2026-04-16</t>
+          <t>2026-04-17</t>
         </is>
       </c>
       <c r="B32" t="n">
@@ -30123,19 +32197,19 @@
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>Naal Nachna</t>
+          <t>Tere Bina</t>
         </is>
       </c>
       <c r="D32" t="inlineStr">
         <is>
-          <t>Shashwat Sachdev</t>
+          <t>A.R. Rahman</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>2026-04-16</t>
+          <t>2026-04-17</t>
         </is>
       </c>
       <c r="B33" t="n">
@@ -30143,19 +32217,19 @@
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>Ehsaas</t>
+          <t>Agar Tum Saath Ho</t>
         </is>
       </c>
       <c r="D33" t="inlineStr">
         <is>
-          <t>Faheem Abdullah</t>
+          <t>Alka Yagnik</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>2026-04-16</t>
+          <t>2026-04-17</t>
         </is>
       </c>
       <c r="B34" t="n">
@@ -30175,7 +32249,7 @@
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>2026-04-16</t>
+          <t>2026-04-17</t>
         </is>
       </c>
       <c r="B35" t="n">
@@ -30183,19 +32257,19 @@
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>Tere Bina</t>
+          <t>Jo Tum Mere Ho</t>
         </is>
       </c>
       <c r="D35" t="inlineStr">
         <is>
-          <t>A.R. Rahman</t>
+          <t>Anuv Jain</t>
         </is>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>2026-04-16</t>
+          <t>2026-04-17</t>
         </is>
       </c>
       <c r="B36" t="n">
@@ -30203,19 +32277,19 @@
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>Jo Tum Mere Ho</t>
+          <t>Ehsaas</t>
         </is>
       </c>
       <c r="D36" t="inlineStr">
         <is>
-          <t>Anuv Jain</t>
+          <t>Faheem Abdullah</t>
         </is>
       </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>2026-04-16</t>
+          <t>2026-04-17</t>
         </is>
       </c>
       <c r="B37" t="n">
@@ -30223,19 +32297,19 @@
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>Agar Tum Saath Ho</t>
+          <t>Bairi</t>
         </is>
       </c>
       <c r="D37" t="inlineStr">
         <is>
-          <t>Alka Yagnik</t>
+          <t>Virat</t>
         </is>
       </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>2026-04-16</t>
+          <t>2026-04-17</t>
         </is>
       </c>
       <c r="B38" t="n">
@@ -30243,19 +32317,19 @@
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>Barbaad</t>
+          <t>Ye Tune Kya Kiya</t>
         </is>
       </c>
       <c r="D38" t="inlineStr">
         <is>
-          <t>The Rish</t>
+          <t>Pritam</t>
         </is>
       </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>2026-04-16</t>
+          <t>2026-04-17</t>
         </is>
       </c>
       <c r="B39" t="n">
@@ -30275,7 +32349,7 @@
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>2026-04-16</t>
+          <t>2026-04-17</t>
         </is>
       </c>
       <c r="B40" t="n">
@@ -30283,19 +32357,19 @@
       </c>
       <c r="C40" t="inlineStr">
         <is>
-          <t>Run Down The City - Monica</t>
+          <t>Barbaad</t>
         </is>
       </c>
       <c r="D40" t="inlineStr">
         <is>
-          <t>Shashwat Sachdev</t>
+          <t>The Rish</t>
         </is>
       </c>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>2026-04-16</t>
+          <t>2026-04-17</t>
         </is>
       </c>
       <c r="B41" t="n">
@@ -30303,19 +32377,19 @@
       </c>
       <c r="C41" t="inlineStr">
         <is>
-          <t>Ye Tune Kya Kiya</t>
+          <t>Haseen</t>
         </is>
       </c>
       <c r="D41" t="inlineStr">
         <is>
-          <t>Pritam</t>
+          <t>Talwiinder</t>
         </is>
       </c>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>2026-04-16</t>
+          <t>2026-04-17</t>
         </is>
       </c>
       <c r="B42" t="n">
@@ -30323,19 +32397,19 @@
       </c>
       <c r="C42" t="inlineStr">
         <is>
-          <t>Haseen</t>
+          <t>Run Down The City - Monica</t>
         </is>
       </c>
       <c r="D42" t="inlineStr">
         <is>
-          <t>Talwiinder</t>
+          <t>Shashwat Sachdev</t>
         </is>
       </c>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>2026-04-16</t>
+          <t>2026-04-17</t>
         </is>
       </c>
       <c r="B43" t="n">
@@ -30343,19 +32417,19 @@
       </c>
       <c r="C43" t="inlineStr">
         <is>
-          <t>Teri Deewani</t>
+          <t>Mast Magan</t>
         </is>
       </c>
       <c r="D43" t="inlineStr">
         <is>
-          <t>Kailash Kher</t>
+          <t>Arijit Singh</t>
         </is>
       </c>
     </row>
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>2026-04-16</t>
+          <t>2026-04-17</t>
         </is>
       </c>
       <c r="B44" t="n">
@@ -30363,19 +32437,19 @@
       </c>
       <c r="C44" t="inlineStr">
         <is>
-          <t>Jhol - Acoustic</t>
+          <t>Teri Deewani</t>
         </is>
       </c>
       <c r="D44" t="inlineStr">
         <is>
-          <t>Maanu</t>
+          <t>Kailash Kher</t>
         </is>
       </c>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>2026-04-16</t>
+          <t>2026-04-17</t>
         </is>
       </c>
       <c r="B45" t="n">
@@ -30383,19 +32457,19 @@
       </c>
       <c r="C45" t="inlineStr">
         <is>
-          <t>Zaalima</t>
+          <t>Jhol - Acoustic</t>
         </is>
       </c>
       <c r="D45" t="inlineStr">
         <is>
-          <t>Arijit Singh</t>
+          <t>Maanu</t>
         </is>
       </c>
     </row>
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>2026-04-16</t>
+          <t>2026-04-17</t>
         </is>
       </c>
       <c r="B46" t="n">
@@ -30403,19 +32477,19 @@
       </c>
       <c r="C46" t="inlineStr">
         <is>
-          <t>High On You</t>
+          <t>Mutta Kalakki</t>
         </is>
       </c>
       <c r="D46" t="inlineStr">
         <is>
-          <t>Jind Universe</t>
+          <t>G. V. Prakash</t>
         </is>
       </c>
     </row>
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>2026-04-16</t>
+          <t>2026-04-17</t>
         </is>
       </c>
       <c r="B47" t="n">
@@ -30423,19 +32497,19 @@
       </c>
       <c r="C47" t="inlineStr">
         <is>
-          <t>Dhun</t>
+          <t>Zaalima</t>
         </is>
       </c>
       <c r="D47" t="inlineStr">
         <is>
-          <t>Mithoon</t>
+          <t>Arijit Singh</t>
         </is>
       </c>
     </row>
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>2026-04-16</t>
+          <t>2026-04-17</t>
         </is>
       </c>
       <c r="B48" t="n">
@@ -30443,19 +32517,19 @@
       </c>
       <c r="C48" t="inlineStr">
         <is>
-          <t>Jogi</t>
+          <t>Aaya Sher</t>
         </is>
       </c>
       <c r="D48" t="inlineStr">
         <is>
-          <t>thiarajxtt</t>
+          <t>Anirudh Ravichander</t>
         </is>
       </c>
     </row>
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>2026-04-16</t>
+          <t>2026-04-17</t>
         </is>
       </c>
       <c r="B49" t="n">
@@ -30463,19 +32537,19 @@
       </c>
       <c r="C49" t="inlineStr">
         <is>
-          <t>Not Guilty</t>
+          <t>Dhun</t>
         </is>
       </c>
       <c r="D49" t="inlineStr">
         <is>
-          <t>Dhanda Nyoliwala</t>
+          <t>Mithoon</t>
         </is>
       </c>
     </row>
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>2026-04-16</t>
+          <t>2026-04-17</t>
         </is>
       </c>
       <c r="B50" t="n">
@@ -30495,7 +32569,7 @@
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>2026-04-16</t>
+          <t>2026-04-17</t>
         </is>
       </c>
       <c r="B51" t="n">
@@ -30503,12 +32577,12 @@
       </c>
       <c r="C51" t="inlineStr">
         <is>
-          <t>Mutta Kalakki</t>
+          <t>High On You</t>
         </is>
       </c>
       <c r="D51" t="inlineStr">
         <is>
-          <t>G. V. Prakash</t>
+          <t>Jind Universe</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
got data for 19th and predictions for 20th april
</commit_message>
<xml_diff>
--- a/Probability Project.xlsx
+++ b/Probability Project.xlsx
@@ -39,6 +39,7 @@
     <sheet name="AUTO_20260416" sheetId="34" state="visible" r:id="rId34"/>
     <sheet name="AUTO_20260418" sheetId="35" state="visible" r:id="rId35"/>
     <sheet name="AUTO_20260417" sheetId="36" state="visible" r:id="rId36"/>
+    <sheet name="AUTO_20260419" sheetId="37" state="visible" r:id="rId37"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -31587,9 +31588,1045 @@
       </c>
     </row>
     <row r="2">
+      <c r="A2" s="0" t="inlineStr">
+        <is>
+          <t>2026-04-17</t>
+        </is>
+      </c>
+      <c r="B2" s="0" t="n">
+        <v>1</v>
+      </c>
+      <c r="C2" s="0" t="inlineStr">
+        <is>
+          <t>Bairan</t>
+        </is>
+      </c>
+      <c r="D2" s="0" t="inlineStr">
+        <is>
+          <t>Banjaare</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="0" t="inlineStr">
+        <is>
+          <t>2026-04-17</t>
+        </is>
+      </c>
+      <c r="B3" s="0" t="n">
+        <v>2</v>
+      </c>
+      <c r="C3" s="0" t="inlineStr">
+        <is>
+          <t>Gehra Hua</t>
+        </is>
+      </c>
+      <c r="D3" s="0" t="inlineStr">
+        <is>
+          <t>Shashwat Sachdev</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="0" t="inlineStr">
+        <is>
+          <t>2026-04-17</t>
+        </is>
+      </c>
+      <c r="B4" s="0" t="n">
+        <v>3</v>
+      </c>
+      <c r="C4" s="0" t="inlineStr">
+        <is>
+          <t>Jaiye Sajana</t>
+        </is>
+      </c>
+      <c r="D4" s="0" t="inlineStr">
+        <is>
+          <t>Shashwat Sachdev</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="0" t="inlineStr">
+        <is>
+          <t>2026-04-17</t>
+        </is>
+      </c>
+      <c r="B5" s="0" t="n">
+        <v>4</v>
+      </c>
+      <c r="C5" s="0" t="inlineStr">
+        <is>
+          <t>Khat</t>
+        </is>
+      </c>
+      <c r="D5" s="0" t="inlineStr">
+        <is>
+          <t>Navjot Ahuja</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="0" t="inlineStr">
+        <is>
+          <t>2026-04-17</t>
+        </is>
+      </c>
+      <c r="B6" s="0" t="n">
+        <v>5</v>
+      </c>
+      <c r="C6" s="0" t="inlineStr">
+        <is>
+          <t>Sheesha - Aakhya Mai Aakh Ghali Jo Bairan</t>
+        </is>
+      </c>
+      <c r="D6" s="0" t="inlineStr">
+        <is>
+          <t>Mitta Ror</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="0" t="inlineStr">
+        <is>
+          <t>2026-04-17</t>
+        </is>
+      </c>
+      <c r="B7" s="0" t="n">
+        <v>6</v>
+      </c>
+      <c r="C7" s="0" t="inlineStr">
+        <is>
+          <t>Sitaare</t>
+        </is>
+      </c>
+      <c r="D7" s="0" t="inlineStr">
+        <is>
+          <t>Arijit Singh</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="0" t="inlineStr">
+        <is>
+          <t>2026-04-17</t>
+        </is>
+      </c>
+      <c r="B8" s="0" t="n">
+        <v>7</v>
+      </c>
+      <c r="C8" s="0" t="inlineStr">
+        <is>
+          <t>Sahiba</t>
+        </is>
+      </c>
+      <c r="D8" s="0" t="inlineStr">
+        <is>
+          <t>Aditya Rikhari</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="0" t="inlineStr">
+        <is>
+          <t>2026-04-17</t>
+        </is>
+      </c>
+      <c r="B9" s="0" t="n">
+        <v>8</v>
+      </c>
+      <c r="C9" s="0" t="inlineStr">
+        <is>
+          <t>Dooron Dooron</t>
+        </is>
+      </c>
+      <c r="D9" s="0" t="inlineStr">
+        <is>
+          <t>Paresh Pahuja</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="0" t="inlineStr">
+        <is>
+          <t>2026-04-17</t>
+        </is>
+      </c>
+      <c r="B10" s="0" t="n">
+        <v>9</v>
+      </c>
+      <c r="C10" s="0" t="inlineStr">
+        <is>
+          <t>Majboor</t>
+        </is>
+      </c>
+      <c r="D10" s="0" t="inlineStr">
+        <is>
+          <t>Sheheryar Rehan</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="0" t="inlineStr">
+        <is>
+          <t>2026-04-17</t>
+        </is>
+      </c>
+      <c r="B11" s="0" t="n">
+        <v>10</v>
+      </c>
+      <c r="C11" s="0" t="inlineStr">
+        <is>
+          <t>Finding Her</t>
+        </is>
+      </c>
+      <c r="D11" s="0" t="inlineStr">
+        <is>
+          <t>Kushagra</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="0" t="inlineStr">
+        <is>
+          <t>2026-04-17</t>
+        </is>
+      </c>
+      <c r="B12" s="0" t="n">
+        <v>11</v>
+      </c>
+      <c r="C12" s="0" t="inlineStr">
+        <is>
+          <t>Samjhawan</t>
+        </is>
+      </c>
+      <c r="D12" s="0" t="inlineStr">
+        <is>
+          <t>Jawad Ahmad</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="0" t="inlineStr">
+        <is>
+          <t>2026-04-17</t>
+        </is>
+      </c>
+      <c r="B13" s="0" t="n">
+        <v>12</v>
+      </c>
+      <c r="C13" s="0" t="inlineStr">
+        <is>
+          <t>Pavazha Malli</t>
+        </is>
+      </c>
+      <c r="D13" s="0" t="inlineStr">
+        <is>
+          <t>Sai Abhyankkar</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="0" t="inlineStr">
+        <is>
+          <t>2026-04-17</t>
+        </is>
+      </c>
+      <c r="B14" s="0" t="n">
+        <v>13</v>
+      </c>
+      <c r="C14" s="0" t="inlineStr">
+        <is>
+          <t>Arz Kiya Hai | Coke Studio Bharat</t>
+        </is>
+      </c>
+      <c r="D14" s="0" t="inlineStr">
+        <is>
+          <t>Anuv Jain</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="0" t="inlineStr">
+        <is>
+          <t>2026-04-17</t>
+        </is>
+      </c>
+      <c r="B15" s="0" t="n">
+        <v>14</v>
+      </c>
+      <c r="C15" s="0" t="inlineStr">
+        <is>
+          <t>Apna Bana Le</t>
+        </is>
+      </c>
+      <c r="D15" s="0" t="inlineStr">
+        <is>
+          <t>Sachin-Jigar</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="0" t="inlineStr">
+        <is>
+          <t>2026-04-17</t>
+        </is>
+      </c>
+      <c r="B16" s="0" t="n">
+        <v>15</v>
+      </c>
+      <c r="C16" s="0" t="inlineStr">
+        <is>
+          <t>Boyfriend</t>
+        </is>
+      </c>
+      <c r="D16" s="0" t="inlineStr">
+        <is>
+          <t>Karan Aujla</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="0" t="inlineStr">
+        <is>
+          <t>2026-04-17</t>
+        </is>
+      </c>
+      <c r="B17" s="0" t="n">
+        <v>16</v>
+      </c>
+      <c r="C17" s="0" t="inlineStr">
+        <is>
+          <t>Dhurandhar The Revenge - Aari Aari</t>
+        </is>
+      </c>
+      <c r="D17" s="0" t="inlineStr">
+        <is>
+          <t>Shashwat Sachdev</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="0" t="inlineStr">
+        <is>
+          <t>2026-04-17</t>
+        </is>
+      </c>
+      <c r="B18" s="0" t="n">
+        <v>17</v>
+      </c>
+      <c r="C18" s="0" t="inlineStr">
+        <is>
+          <t>Jaan Se Guzarte Hain</t>
+        </is>
+      </c>
+      <c r="D18" s="0" t="inlineStr">
+        <is>
+          <t>Shashwat Sachdev</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="0" t="inlineStr">
+        <is>
+          <t>2026-04-17</t>
+        </is>
+      </c>
+      <c r="B19" s="0" t="n">
+        <v>18</v>
+      </c>
+      <c r="C19" s="0" t="inlineStr">
+        <is>
+          <t>Ishq</t>
+        </is>
+      </c>
+      <c r="D19" s="0" t="inlineStr">
+        <is>
+          <t>Faheem Abdullah</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="0" t="inlineStr">
+        <is>
+          <t>2026-04-17</t>
+        </is>
+      </c>
+      <c r="B20" s="0" t="n">
+        <v>19</v>
+      </c>
+      <c r="C20" s="0" t="inlineStr">
+        <is>
+          <t>Mann Mera</t>
+        </is>
+      </c>
+      <c r="D20" s="0" t="inlineStr">
+        <is>
+          <t>Gajendra Verma</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="0" t="inlineStr">
+        <is>
+          <t>2026-04-17</t>
+        </is>
+      </c>
+      <c r="B21" s="0" t="n">
+        <v>20</v>
+      </c>
+      <c r="C21" s="0" t="inlineStr">
+        <is>
+          <t>Shararat</t>
+        </is>
+      </c>
+      <c r="D21" s="0" t="inlineStr">
+        <is>
+          <t>Shashwat Sachdev</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="0" t="inlineStr">
+        <is>
+          <t>2026-04-17</t>
+        </is>
+      </c>
+      <c r="B22" s="0" t="n">
+        <v>21</v>
+      </c>
+      <c r="C22" s="0" t="inlineStr">
+        <is>
+          <t>For A Reason</t>
+        </is>
+      </c>
+      <c r="D22" s="0" t="inlineStr">
+        <is>
+          <t>Karan Aujla</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="0" t="inlineStr">
+        <is>
+          <t>2026-04-17</t>
+        </is>
+      </c>
+      <c r="B23" s="0" t="n">
+        <v>22</v>
+      </c>
+      <c r="C23" s="0" t="inlineStr">
+        <is>
+          <t>Saiyaara</t>
+        </is>
+      </c>
+      <c r="D23" s="0" t="inlineStr">
+        <is>
+          <t>Tanishk Bagchi</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="0" t="inlineStr">
+        <is>
+          <t>2026-04-17</t>
+        </is>
+      </c>
+      <c r="B24" s="0" t="n">
+        <v>23</v>
+      </c>
+      <c r="C24" s="0" t="inlineStr">
+        <is>
+          <t>Tum Ho Toh</t>
+        </is>
+      </c>
+      <c r="D24" s="0" t="inlineStr">
+        <is>
+          <t>Vishal Mishra</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="0" t="inlineStr">
+        <is>
+          <t>2026-04-17</t>
+        </is>
+      </c>
+      <c r="B25" s="0" t="n">
+        <v>24</v>
+      </c>
+      <c r="C25" s="0" t="inlineStr">
+        <is>
+          <t>Ishqa Ve</t>
+        </is>
+      </c>
+      <c r="D25" s="0" t="inlineStr">
+        <is>
+          <t>Zeeshan Ali</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="0" t="inlineStr">
+        <is>
+          <t>2026-04-17</t>
+        </is>
+      </c>
+      <c r="B26" s="0" t="n">
+        <v>25</v>
+      </c>
+      <c r="C26" s="0" t="inlineStr">
+        <is>
+          <t>Deewaana Deewaana</t>
+        </is>
+      </c>
+      <c r="D26" s="0" t="inlineStr">
+        <is>
+          <t>A.R. Rahman</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="0" t="inlineStr">
+        <is>
+          <t>2026-04-17</t>
+        </is>
+      </c>
+      <c r="B27" s="0" t="n">
+        <v>26</v>
+      </c>
+      <c r="C27" s="0" t="inlineStr">
+        <is>
+          <t>Raanjhan</t>
+        </is>
+      </c>
+      <c r="D27" s="0" t="inlineStr">
+        <is>
+          <t>Sachet-Parampara</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="0" t="inlineStr">
+        <is>
+          <t>2026-04-17</t>
+        </is>
+      </c>
+      <c r="B28" s="0" t="n">
+        <v>27</v>
+      </c>
+      <c r="C28" s="0" t="inlineStr">
+        <is>
+          <t>Darkhaast</t>
+        </is>
+      </c>
+      <c r="D28" s="0" t="inlineStr">
+        <is>
+          <t>Mithoon</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="0" t="inlineStr">
+        <is>
+          <t>2026-04-17</t>
+        </is>
+      </c>
+      <c r="B29" s="0" t="n">
+        <v>28</v>
+      </c>
+      <c r="C29" s="0" t="inlineStr">
+        <is>
+          <t>Tere Liye</t>
+        </is>
+      </c>
+      <c r="D29" s="0" t="inlineStr">
+        <is>
+          <t>Atif Aslam</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="0" t="inlineStr">
+        <is>
+          <t>2026-04-17</t>
+        </is>
+      </c>
+      <c r="B30" s="0" t="n">
+        <v>29</v>
+      </c>
+      <c r="C30" s="0" t="inlineStr">
+        <is>
+          <t>Dhurandhar - Title Track</t>
+        </is>
+      </c>
+      <c r="D30" s="0" t="inlineStr">
+        <is>
+          <t>Shashwat Sachdev</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="0" t="inlineStr">
+        <is>
+          <t>2026-04-17</t>
+        </is>
+      </c>
+      <c r="B31" s="0" t="n">
+        <v>30</v>
+      </c>
+      <c r="C31" s="0" t="inlineStr">
+        <is>
+          <t>Naal Nachna</t>
+        </is>
+      </c>
+      <c r="D31" s="0" t="inlineStr">
+        <is>
+          <t>Shashwat Sachdev</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="0" t="inlineStr">
+        <is>
+          <t>2026-04-17</t>
+        </is>
+      </c>
+      <c r="B32" s="0" t="n">
+        <v>31</v>
+      </c>
+      <c r="C32" s="0" t="inlineStr">
+        <is>
+          <t>Tere Bina</t>
+        </is>
+      </c>
+      <c r="D32" s="0" t="inlineStr">
+        <is>
+          <t>A.R. Rahman</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="0" t="inlineStr">
+        <is>
+          <t>2026-04-17</t>
+        </is>
+      </c>
+      <c r="B33" s="0" t="n">
+        <v>32</v>
+      </c>
+      <c r="C33" s="0" t="inlineStr">
+        <is>
+          <t>Agar Tum Saath Ho</t>
+        </is>
+      </c>
+      <c r="D33" s="0" t="inlineStr">
+        <is>
+          <t>Alka Yagnik</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="0" t="inlineStr">
+        <is>
+          <t>2026-04-17</t>
+        </is>
+      </c>
+      <c r="B34" s="0" t="n">
+        <v>33</v>
+      </c>
+      <c r="C34" s="0" t="inlineStr">
+        <is>
+          <t>Phir Se</t>
+        </is>
+      </c>
+      <c r="D34" s="0" t="inlineStr">
+        <is>
+          <t>Shashwat Sachdev</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="0" t="inlineStr">
+        <is>
+          <t>2026-04-17</t>
+        </is>
+      </c>
+      <c r="B35" s="0" t="n">
+        <v>34</v>
+      </c>
+      <c r="C35" s="0" t="inlineStr">
+        <is>
+          <t>Jo Tum Mere Ho</t>
+        </is>
+      </c>
+      <c r="D35" s="0" t="inlineStr">
+        <is>
+          <t>Anuv Jain</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="0" t="inlineStr">
+        <is>
+          <t>2026-04-17</t>
+        </is>
+      </c>
+      <c r="B36" s="0" t="n">
+        <v>35</v>
+      </c>
+      <c r="C36" s="0" t="inlineStr">
+        <is>
+          <t>Ehsaas</t>
+        </is>
+      </c>
+      <c r="D36" s="0" t="inlineStr">
+        <is>
+          <t>Faheem Abdullah</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="0" t="inlineStr">
+        <is>
+          <t>2026-04-17</t>
+        </is>
+      </c>
+      <c r="B37" s="0" t="n">
+        <v>36</v>
+      </c>
+      <c r="C37" s="0" t="inlineStr">
+        <is>
+          <t>Bairi</t>
+        </is>
+      </c>
+      <c r="D37" s="0" t="inlineStr">
+        <is>
+          <t>Virat</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="0" t="inlineStr">
+        <is>
+          <t>2026-04-17</t>
+        </is>
+      </c>
+      <c r="B38" s="0" t="n">
+        <v>37</v>
+      </c>
+      <c r="C38" s="0" t="inlineStr">
+        <is>
+          <t>Ye Tune Kya Kiya</t>
+        </is>
+      </c>
+      <c r="D38" s="0" t="inlineStr">
+        <is>
+          <t>Pritam</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="0" t="inlineStr">
+        <is>
+          <t>2026-04-17</t>
+        </is>
+      </c>
+      <c r="B39" s="0" t="n">
+        <v>38</v>
+      </c>
+      <c r="C39" s="0" t="inlineStr">
+        <is>
+          <t>Lutt Le Gaya</t>
+        </is>
+      </c>
+      <c r="D39" s="0" t="inlineStr">
+        <is>
+          <t>Shashwat Sachdev</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="0" t="inlineStr">
+        <is>
+          <t>2026-04-17</t>
+        </is>
+      </c>
+      <c r="B40" s="0" t="n">
+        <v>39</v>
+      </c>
+      <c r="C40" s="0" t="inlineStr">
+        <is>
+          <t>Barbaad</t>
+        </is>
+      </c>
+      <c r="D40" s="0" t="inlineStr">
+        <is>
+          <t>The Rish</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" s="0" t="inlineStr">
+        <is>
+          <t>2026-04-17</t>
+        </is>
+      </c>
+      <c r="B41" s="0" t="n">
+        <v>40</v>
+      </c>
+      <c r="C41" s="0" t="inlineStr">
+        <is>
+          <t>Haseen</t>
+        </is>
+      </c>
+      <c r="D41" s="0" t="inlineStr">
+        <is>
+          <t>Talwiinder</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" s="0" t="inlineStr">
+        <is>
+          <t>2026-04-17</t>
+        </is>
+      </c>
+      <c r="B42" s="0" t="n">
+        <v>41</v>
+      </c>
+      <c r="C42" s="0" t="inlineStr">
+        <is>
+          <t>Run Down The City - Monica</t>
+        </is>
+      </c>
+      <c r="D42" s="0" t="inlineStr">
+        <is>
+          <t>Shashwat Sachdev</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" s="0" t="inlineStr">
+        <is>
+          <t>2026-04-17</t>
+        </is>
+      </c>
+      <c r="B43" s="0" t="n">
+        <v>42</v>
+      </c>
+      <c r="C43" s="0" t="inlineStr">
+        <is>
+          <t>Mast Magan</t>
+        </is>
+      </c>
+      <c r="D43" s="0" t="inlineStr">
+        <is>
+          <t>Arijit Singh</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" s="0" t="inlineStr">
+        <is>
+          <t>2026-04-17</t>
+        </is>
+      </c>
+      <c r="B44" s="0" t="n">
+        <v>43</v>
+      </c>
+      <c r="C44" s="0" t="inlineStr">
+        <is>
+          <t>Teri Deewani</t>
+        </is>
+      </c>
+      <c r="D44" s="0" t="inlineStr">
+        <is>
+          <t>Kailash Kher</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" s="0" t="inlineStr">
+        <is>
+          <t>2026-04-17</t>
+        </is>
+      </c>
+      <c r="B45" s="0" t="n">
+        <v>44</v>
+      </c>
+      <c r="C45" s="0" t="inlineStr">
+        <is>
+          <t>Jhol - Acoustic</t>
+        </is>
+      </c>
+      <c r="D45" s="0" t="inlineStr">
+        <is>
+          <t>Maanu</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" s="0" t="inlineStr">
+        <is>
+          <t>2026-04-17</t>
+        </is>
+      </c>
+      <c r="B46" s="0" t="n">
+        <v>45</v>
+      </c>
+      <c r="C46" s="0" t="inlineStr">
+        <is>
+          <t>Mutta Kalakki</t>
+        </is>
+      </c>
+      <c r="D46" s="0" t="inlineStr">
+        <is>
+          <t>G. V. Prakash</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" s="0" t="inlineStr">
+        <is>
+          <t>2026-04-17</t>
+        </is>
+      </c>
+      <c r="B47" s="0" t="n">
+        <v>46</v>
+      </c>
+      <c r="C47" s="0" t="inlineStr">
+        <is>
+          <t>Zaalima</t>
+        </is>
+      </c>
+      <c r="D47" s="0" t="inlineStr">
+        <is>
+          <t>Arijit Singh</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" s="0" t="inlineStr">
+        <is>
+          <t>2026-04-17</t>
+        </is>
+      </c>
+      <c r="B48" s="0" t="n">
+        <v>47</v>
+      </c>
+      <c r="C48" s="0" t="inlineStr">
+        <is>
+          <t>Aaya Sher</t>
+        </is>
+      </c>
+      <c r="D48" s="0" t="inlineStr">
+        <is>
+          <t>Anirudh Ravichander</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" s="0" t="inlineStr">
+        <is>
+          <t>2026-04-17</t>
+        </is>
+      </c>
+      <c r="B49" s="0" t="n">
+        <v>48</v>
+      </c>
+      <c r="C49" s="0" t="inlineStr">
+        <is>
+          <t>Dhun</t>
+        </is>
+      </c>
+      <c r="D49" s="0" t="inlineStr">
+        <is>
+          <t>Mithoon</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" s="0" t="inlineStr">
+        <is>
+          <t>2026-04-17</t>
+        </is>
+      </c>
+      <c r="B50" s="0" t="n">
+        <v>49</v>
+      </c>
+      <c r="C50" s="0" t="inlineStr">
+        <is>
+          <t>Mann Mera - Original Version</t>
+        </is>
+      </c>
+      <c r="D50" s="0" t="inlineStr">
+        <is>
+          <t>Gajendra Verma</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" s="0" t="inlineStr">
+        <is>
+          <t>2026-04-17</t>
+        </is>
+      </c>
+      <c r="B51" s="0" t="n">
+        <v>50</v>
+      </c>
+      <c r="C51" s="0" t="inlineStr">
+        <is>
+          <t>High On You</t>
+        </is>
+      </c>
+      <c r="D51" s="0" t="inlineStr">
+        <is>
+          <t>Jind Universe</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet37.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:D51"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="24" t="inlineStr">
+        <is>
+          <t>Date</t>
+        </is>
+      </c>
+      <c r="B1" s="24" t="inlineStr">
+        <is>
+          <t>Rank</t>
+        </is>
+      </c>
+      <c r="C1" s="24" t="inlineStr">
+        <is>
+          <t>Song</t>
+        </is>
+      </c>
+      <c r="D1" s="24" t="inlineStr">
+        <is>
+          <t>Artist</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>2026-04-17</t>
+          <t>2026-04-19</t>
         </is>
       </c>
       <c r="B2" t="n">
@@ -31609,7 +32646,7 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>2026-04-17</t>
+          <t>2026-04-19</t>
         </is>
       </c>
       <c r="B3" t="n">
@@ -31629,7 +32666,7 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>2026-04-17</t>
+          <t>2026-04-19</t>
         </is>
       </c>
       <c r="B4" t="n">
@@ -31637,19 +32674,19 @@
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>Jaiye Sajana</t>
+          <t>Sheesha - Aakhya Mai Aakh Ghali Jo Bairan</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>Shashwat Sachdev</t>
+          <t>Mitta Ror</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>2026-04-17</t>
+          <t>2026-04-19</t>
         </is>
       </c>
       <c r="B5" t="n">
@@ -31657,19 +32694,19 @@
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>Khat</t>
+          <t>Jaiye Sajana</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>Navjot Ahuja</t>
+          <t>Shashwat Sachdev</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>2026-04-17</t>
+          <t>2026-04-19</t>
         </is>
       </c>
       <c r="B6" t="n">
@@ -31677,19 +32714,19 @@
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>Sheesha - Aakhya Mai Aakh Ghali Jo Bairan</t>
+          <t>Khat</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>Mitta Ror</t>
+          <t>Navjot Ahuja</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>2026-04-17</t>
+          <t>2026-04-19</t>
         </is>
       </c>
       <c r="B7" t="n">
@@ -31697,19 +32734,19 @@
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>Sitaare</t>
+          <t>Majboor</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>Arijit Singh</t>
+          <t>Sheheryar Rehan</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>2026-04-17</t>
+          <t>2026-04-19</t>
         </is>
       </c>
       <c r="B8" t="n">
@@ -31717,19 +32754,19 @@
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>Sahiba</t>
+          <t>Finding Her</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>Aditya Rikhari</t>
+          <t>Kushagra</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>2026-04-17</t>
+          <t>2026-04-19</t>
         </is>
       </c>
       <c r="B9" t="n">
@@ -31737,19 +32774,19 @@
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>Dooron Dooron</t>
+          <t>Sitaare</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>Paresh Pahuja</t>
+          <t>Arijit Singh</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>2026-04-17</t>
+          <t>2026-04-19</t>
         </is>
       </c>
       <c r="B10" t="n">
@@ -31757,19 +32794,19 @@
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>Majboor</t>
+          <t>Sahiba</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>Sheheryar Rehan</t>
+          <t>Aditya Rikhari</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>2026-04-17</t>
+          <t>2026-04-19</t>
         </is>
       </c>
       <c r="B11" t="n">
@@ -31777,19 +32814,19 @@
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>Finding Her</t>
+          <t>Dooron Dooron</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>Kushagra</t>
+          <t>Paresh Pahuja</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>2026-04-17</t>
+          <t>2026-04-19</t>
         </is>
       </c>
       <c r="B12" t="n">
@@ -31797,19 +32834,19 @@
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>Samjhawan</t>
+          <t>Pavazha Malli</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>Jawad Ahmad</t>
+          <t>Sai Abhyankkar</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>2026-04-17</t>
+          <t>2026-04-19</t>
         </is>
       </c>
       <c r="B13" t="n">
@@ -31817,19 +32854,19 @@
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>Pavazha Malli</t>
+          <t>Samjhawan</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>Sai Abhyankkar</t>
+          <t>Jawad Ahmad</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>2026-04-17</t>
+          <t>2026-04-19</t>
         </is>
       </c>
       <c r="B14" t="n">
@@ -31849,7 +32886,7 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>2026-04-17</t>
+          <t>2026-04-19</t>
         </is>
       </c>
       <c r="B15" t="n">
@@ -31869,7 +32906,7 @@
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>2026-04-17</t>
+          <t>2026-04-19</t>
         </is>
       </c>
       <c r="B16" t="n">
@@ -31877,19 +32914,19 @@
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>Boyfriend</t>
+          <t>Dhurandhar The Revenge - Aari Aari</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>Karan Aujla</t>
+          <t>Shashwat Sachdev</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>2026-04-17</t>
+          <t>2026-04-19</t>
         </is>
       </c>
       <c r="B17" t="n">
@@ -31897,19 +32934,19 @@
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>Dhurandhar The Revenge - Aari Aari</t>
+          <t>Boyfriend</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>Shashwat Sachdev</t>
+          <t>Karan Aujla</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>2026-04-17</t>
+          <t>2026-04-19</t>
         </is>
       </c>
       <c r="B18" t="n">
@@ -31917,7 +32954,7 @@
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>Jaan Se Guzarte Hain</t>
+          <t>Shararat</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
@@ -31929,7 +32966,7 @@
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>2026-04-17</t>
+          <t>2026-04-19</t>
         </is>
       </c>
       <c r="B19" t="n">
@@ -31937,19 +32974,19 @@
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>Ishq</t>
+          <t>Mann Mera</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>Faheem Abdullah</t>
+          <t>Gajendra Verma</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>2026-04-17</t>
+          <t>2026-04-19</t>
         </is>
       </c>
       <c r="B20" t="n">
@@ -31957,19 +32994,19 @@
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>Mann Mera</t>
+          <t>Ishq</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>Gajendra Verma</t>
+          <t>Faheem Abdullah</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>2026-04-17</t>
+          <t>2026-04-19</t>
         </is>
       </c>
       <c r="B21" t="n">
@@ -31977,7 +33014,7 @@
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>Shararat</t>
+          <t>Jaan Se Guzarte Hain</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
@@ -31989,7 +33026,7 @@
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>2026-04-17</t>
+          <t>2026-04-19</t>
         </is>
       </c>
       <c r="B22" t="n">
@@ -31997,19 +33034,19 @@
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>For A Reason</t>
+          <t>Tum Ho Toh</t>
         </is>
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>Karan Aujla</t>
+          <t>Vishal Mishra</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>2026-04-17</t>
+          <t>2026-04-19</t>
         </is>
       </c>
       <c r="B23" t="n">
@@ -32029,7 +33066,7 @@
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>2026-04-17</t>
+          <t>2026-04-19</t>
         </is>
       </c>
       <c r="B24" t="n">
@@ -32037,19 +33074,19 @@
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>Tum Ho Toh</t>
+          <t>For A Reason</t>
         </is>
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>Vishal Mishra</t>
+          <t>Karan Aujla</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>2026-04-17</t>
+          <t>2026-04-19</t>
         </is>
       </c>
       <c r="B25" t="n">
@@ -32057,19 +33094,19 @@
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>Ishqa Ve</t>
+          <t>Raanjhan</t>
         </is>
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>Zeeshan Ali</t>
+          <t>Sachet-Parampara</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>2026-04-17</t>
+          <t>2026-04-19</t>
         </is>
       </c>
       <c r="B26" t="n">
@@ -32089,7 +33126,7 @@
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>2026-04-17</t>
+          <t>2026-04-19</t>
         </is>
       </c>
       <c r="B27" t="n">
@@ -32097,19 +33134,19 @@
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>Raanjhan</t>
+          <t>Darkhaast</t>
         </is>
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t>Sachet-Parampara</t>
+          <t>Mithoon</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>2026-04-17</t>
+          <t>2026-04-19</t>
         </is>
       </c>
       <c r="B28" t="n">
@@ -32117,19 +33154,19 @@
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>Darkhaast</t>
+          <t>Dhurandhar - Title Track</t>
         </is>
       </c>
       <c r="D28" t="inlineStr">
         <is>
-          <t>Mithoon</t>
+          <t>Shashwat Sachdev</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>2026-04-17</t>
+          <t>2026-04-19</t>
         </is>
       </c>
       <c r="B29" t="n">
@@ -32149,7 +33186,7 @@
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>2026-04-17</t>
+          <t>2026-04-19</t>
         </is>
       </c>
       <c r="B30" t="n">
@@ -32157,19 +33194,19 @@
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>Dhurandhar - Title Track</t>
+          <t>Ishqa Ve</t>
         </is>
       </c>
       <c r="D30" t="inlineStr">
         <is>
-          <t>Shashwat Sachdev</t>
+          <t>Zeeshan Ali</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>2026-04-17</t>
+          <t>2026-04-19</t>
         </is>
       </c>
       <c r="B31" t="n">
@@ -32177,19 +33214,19 @@
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>Naal Nachna</t>
+          <t>Ehsaas</t>
         </is>
       </c>
       <c r="D31" t="inlineStr">
         <is>
-          <t>Shashwat Sachdev</t>
+          <t>Faheem Abdullah</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>2026-04-17</t>
+          <t>2026-04-19</t>
         </is>
       </c>
       <c r="B32" t="n">
@@ -32197,19 +33234,19 @@
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>Tere Bina</t>
+          <t>Naal Nachna</t>
         </is>
       </c>
       <c r="D32" t="inlineStr">
         <is>
-          <t>A.R. Rahman</t>
+          <t>Shashwat Sachdev</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>2026-04-17</t>
+          <t>2026-04-19</t>
         </is>
       </c>
       <c r="B33" t="n">
@@ -32217,19 +33254,19 @@
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>Agar Tum Saath Ho</t>
+          <t>Bairi</t>
         </is>
       </c>
       <c r="D33" t="inlineStr">
         <is>
-          <t>Alka Yagnik</t>
+          <t>Virat</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>2026-04-17</t>
+          <t>2026-04-19</t>
         </is>
       </c>
       <c r="B34" t="n">
@@ -32237,19 +33274,19 @@
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>Phir Se</t>
+          <t>Jo Tum Mere Ho</t>
         </is>
       </c>
       <c r="D34" t="inlineStr">
         <is>
-          <t>Shashwat Sachdev</t>
+          <t>Anuv Jain</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>2026-04-17</t>
+          <t>2026-04-19</t>
         </is>
       </c>
       <c r="B35" t="n">
@@ -32257,19 +33294,19 @@
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>Jo Tum Mere Ho</t>
+          <t>Tere Bina</t>
         </is>
       </c>
       <c r="D35" t="inlineStr">
         <is>
-          <t>Anuv Jain</t>
+          <t>A.R. Rahman</t>
         </is>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>2026-04-17</t>
+          <t>2026-04-19</t>
         </is>
       </c>
       <c r="B36" t="n">
@@ -32277,19 +33314,19 @@
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>Ehsaas</t>
+          <t>Agar Tum Saath Ho</t>
         </is>
       </c>
       <c r="D36" t="inlineStr">
         <is>
-          <t>Faheem Abdullah</t>
+          <t>Alka Yagnik</t>
         </is>
       </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>2026-04-17</t>
+          <t>2026-04-19</t>
         </is>
       </c>
       <c r="B37" t="n">
@@ -32297,19 +33334,19 @@
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>Bairi</t>
+          <t>Phir Se</t>
         </is>
       </c>
       <c r="D37" t="inlineStr">
         <is>
-          <t>Virat</t>
+          <t>Shashwat Sachdev</t>
         </is>
       </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>2026-04-17</t>
+          <t>2026-04-19</t>
         </is>
       </c>
       <c r="B38" t="n">
@@ -32317,19 +33354,19 @@
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>Ye Tune Kya Kiya</t>
+          <t>Haseen</t>
         </is>
       </c>
       <c r="D38" t="inlineStr">
         <is>
-          <t>Pritam</t>
+          <t>Talwiinder</t>
         </is>
       </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>2026-04-17</t>
+          <t>2026-04-19</t>
         </is>
       </c>
       <c r="B39" t="n">
@@ -32337,19 +33374,19 @@
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>Lutt Le Gaya</t>
+          <t>Ye Tune Kya Kiya</t>
         </is>
       </c>
       <c r="D39" t="inlineStr">
         <is>
-          <t>Shashwat Sachdev</t>
+          <t>Pritam</t>
         </is>
       </c>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>2026-04-17</t>
+          <t>2026-04-19</t>
         </is>
       </c>
       <c r="B40" t="n">
@@ -32369,7 +33406,7 @@
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>2026-04-17</t>
+          <t>2026-04-19</t>
         </is>
       </c>
       <c r="B41" t="n">
@@ -32377,19 +33414,19 @@
       </c>
       <c r="C41" t="inlineStr">
         <is>
-          <t>Haseen</t>
+          <t>Lutt Le Gaya</t>
         </is>
       </c>
       <c r="D41" t="inlineStr">
         <is>
-          <t>Talwiinder</t>
+          <t>Shashwat Sachdev</t>
         </is>
       </c>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>2026-04-17</t>
+          <t>2026-04-19</t>
         </is>
       </c>
       <c r="B42" t="n">
@@ -32397,19 +33434,19 @@
       </c>
       <c r="C42" t="inlineStr">
         <is>
-          <t>Run Down The City - Monica</t>
+          <t>Mutta Kalakki</t>
         </is>
       </c>
       <c r="D42" t="inlineStr">
         <is>
-          <t>Shashwat Sachdev</t>
+          <t>G. V. Prakash</t>
         </is>
       </c>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>2026-04-17</t>
+          <t>2026-04-19</t>
         </is>
       </c>
       <c r="B43" t="n">
@@ -32417,7 +33454,7 @@
       </c>
       <c r="C43" t="inlineStr">
         <is>
-          <t>Mast Magan</t>
+          <t>Zaalima</t>
         </is>
       </c>
       <c r="D43" t="inlineStr">
@@ -32429,7 +33466,7 @@
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>2026-04-17</t>
+          <t>2026-04-19</t>
         </is>
       </c>
       <c r="B44" t="n">
@@ -32449,7 +33486,7 @@
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>2026-04-17</t>
+          <t>2026-04-19</t>
         </is>
       </c>
       <c r="B45" t="n">
@@ -32457,19 +33494,19 @@
       </c>
       <c r="C45" t="inlineStr">
         <is>
-          <t>Jhol - Acoustic</t>
+          <t>Run Down The City - Monica</t>
         </is>
       </c>
       <c r="D45" t="inlineStr">
         <is>
-          <t>Maanu</t>
+          <t>Shashwat Sachdev</t>
         </is>
       </c>
     </row>
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>2026-04-17</t>
+          <t>2026-04-19</t>
         </is>
       </c>
       <c r="B46" t="n">
@@ -32477,19 +33514,19 @@
       </c>
       <c r="C46" t="inlineStr">
         <is>
-          <t>Mutta Kalakki</t>
+          <t>Aaya Sher</t>
         </is>
       </c>
       <c r="D46" t="inlineStr">
         <is>
-          <t>G. V. Prakash</t>
+          <t>Anirudh Ravichander</t>
         </is>
       </c>
     </row>
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>2026-04-17</t>
+          <t>2026-04-19</t>
         </is>
       </c>
       <c r="B47" t="n">
@@ -32497,19 +33534,19 @@
       </c>
       <c r="C47" t="inlineStr">
         <is>
-          <t>Zaalima</t>
+          <t>Jhol - Acoustic</t>
         </is>
       </c>
       <c r="D47" t="inlineStr">
         <is>
-          <t>Arijit Singh</t>
+          <t>Maanu</t>
         </is>
       </c>
     </row>
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>2026-04-17</t>
+          <t>2026-04-19</t>
         </is>
       </c>
       <c r="B48" t="n">
@@ -32517,19 +33554,19 @@
       </c>
       <c r="C48" t="inlineStr">
         <is>
-          <t>Aaya Sher</t>
+          <t>Mast Magan</t>
         </is>
       </c>
       <c r="D48" t="inlineStr">
         <is>
-          <t>Anirudh Ravichander</t>
+          <t>Arijit Singh</t>
         </is>
       </c>
     </row>
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>2026-04-17</t>
+          <t>2026-04-19</t>
         </is>
       </c>
       <c r="B49" t="n">
@@ -32549,7 +33586,7 @@
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>2026-04-17</t>
+          <t>2026-04-19</t>
         </is>
       </c>
       <c r="B50" t="n">
@@ -32557,19 +33594,19 @@
       </c>
       <c r="C50" t="inlineStr">
         <is>
-          <t>Mann Mera - Original Version</t>
+          <t>High On You</t>
         </is>
       </c>
       <c r="D50" t="inlineStr">
         <is>
-          <t>Gajendra Verma</t>
+          <t>Jind Universe</t>
         </is>
       </c>
     </row>
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>2026-04-17</t>
+          <t>2026-04-19</t>
         </is>
       </c>
       <c r="B51" t="n">
@@ -32577,12 +33614,12 @@
       </c>
       <c r="C51" t="inlineStr">
         <is>
-          <t>High On You</t>
+          <t>Mann Mera - Original Version</t>
         </is>
       </c>
       <c r="D51" t="inlineStr">
         <is>
-          <t>Jind Universe</t>
+          <t>Gajendra Verma</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
got gthe data till 26th april, got preditions for 27th april
</commit_message>
<xml_diff>
--- a/Probability Project.xlsx
+++ b/Probability Project.xlsx
@@ -44,6 +44,9 @@
     <sheet name="AUTO_20260420" sheetId="39" state="visible" r:id="rId39"/>
     <sheet name="AUTO_20260421" sheetId="40" state="visible" r:id="rId40"/>
     <sheet name="AUTO_20260422" sheetId="41" state="visible" r:id="rId41"/>
+    <sheet name="AUTO_20260426" sheetId="42" state="visible" r:id="rId42"/>
+    <sheet name="AUTO_20260424" sheetId="43" state="visible" r:id="rId43"/>
+    <sheet name="AUTO_20260425" sheetId="44" state="visible" r:id="rId44"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -37808,9 +37811,3117 @@
       </c>
     </row>
     <row r="2">
+      <c r="A2" s="0" t="inlineStr">
+        <is>
+          <t>2026-04-22</t>
+        </is>
+      </c>
+      <c r="B2" s="0" t="n">
+        <v>1</v>
+      </c>
+      <c r="C2" s="0" t="inlineStr">
+        <is>
+          <t>Bairan</t>
+        </is>
+      </c>
+      <c r="D2" s="0" t="inlineStr">
+        <is>
+          <t>Banjaare</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="0" t="inlineStr">
+        <is>
+          <t>2026-04-22</t>
+        </is>
+      </c>
+      <c r="B3" s="0" t="n">
+        <v>2</v>
+      </c>
+      <c r="C3" s="0" t="inlineStr">
+        <is>
+          <t>Gehra Hua</t>
+        </is>
+      </c>
+      <c r="D3" s="0" t="inlineStr">
+        <is>
+          <t>Shashwat Sachdev</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="0" t="inlineStr">
+        <is>
+          <t>2026-04-22</t>
+        </is>
+      </c>
+      <c r="B4" s="0" t="n">
+        <v>3</v>
+      </c>
+      <c r="C4" s="0" t="inlineStr">
+        <is>
+          <t>Majboor</t>
+        </is>
+      </c>
+      <c r="D4" s="0" t="inlineStr">
+        <is>
+          <t>Sheheryar Rehan</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="0" t="inlineStr">
+        <is>
+          <t>2026-04-22</t>
+        </is>
+      </c>
+      <c r="B5" s="0" t="n">
+        <v>4</v>
+      </c>
+      <c r="C5" s="0" t="inlineStr">
+        <is>
+          <t>Khat</t>
+        </is>
+      </c>
+      <c r="D5" s="0" t="inlineStr">
+        <is>
+          <t>Navjot Ahuja</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="0" t="inlineStr">
+        <is>
+          <t>2026-04-22</t>
+        </is>
+      </c>
+      <c r="B6" s="0" t="n">
+        <v>5</v>
+      </c>
+      <c r="C6" s="0" t="inlineStr">
+        <is>
+          <t>Sheesha - Aakhya Mai Aakh Ghali Jo Bairan</t>
+        </is>
+      </c>
+      <c r="D6" s="0" t="inlineStr">
+        <is>
+          <t>Mitta Ror</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="0" t="inlineStr">
+        <is>
+          <t>2026-04-22</t>
+        </is>
+      </c>
+      <c r="B7" s="0" t="n">
+        <v>6</v>
+      </c>
+      <c r="C7" s="0" t="inlineStr">
+        <is>
+          <t>Jaiye Sajana</t>
+        </is>
+      </c>
+      <c r="D7" s="0" t="inlineStr">
+        <is>
+          <t>Shashwat Sachdev</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="0" t="inlineStr">
+        <is>
+          <t>2026-04-22</t>
+        </is>
+      </c>
+      <c r="B8" s="0" t="n">
+        <v>7</v>
+      </c>
+      <c r="C8" s="0" t="inlineStr">
+        <is>
+          <t>Pavazha Malli</t>
+        </is>
+      </c>
+      <c r="D8" s="0" t="inlineStr">
+        <is>
+          <t>Sai Abhyankkar</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="0" t="inlineStr">
+        <is>
+          <t>2026-04-22</t>
+        </is>
+      </c>
+      <c r="B9" s="0" t="n">
+        <v>8</v>
+      </c>
+      <c r="C9" s="0" t="inlineStr">
+        <is>
+          <t>Finding Her</t>
+        </is>
+      </c>
+      <c r="D9" s="0" t="inlineStr">
+        <is>
+          <t>Kushagra</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="0" t="inlineStr">
+        <is>
+          <t>2026-04-22</t>
+        </is>
+      </c>
+      <c r="B10" s="0" t="n">
+        <v>9</v>
+      </c>
+      <c r="C10" s="0" t="inlineStr">
+        <is>
+          <t>Sahiba</t>
+        </is>
+      </c>
+      <c r="D10" s="0" t="inlineStr">
+        <is>
+          <t>Aditya Rikhari</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="0" t="inlineStr">
+        <is>
+          <t>2026-04-22</t>
+        </is>
+      </c>
+      <c r="B11" s="0" t="n">
+        <v>10</v>
+      </c>
+      <c r="C11" s="0" t="inlineStr">
+        <is>
+          <t>Sitaare</t>
+        </is>
+      </c>
+      <c r="D11" s="0" t="inlineStr">
+        <is>
+          <t>Arijit Singh</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="0" t="inlineStr">
+        <is>
+          <t>2026-04-22</t>
+        </is>
+      </c>
+      <c r="B12" s="0" t="n">
+        <v>11</v>
+      </c>
+      <c r="C12" s="0" t="inlineStr">
+        <is>
+          <t>Arz Kiya Hai | Coke Studio Bharat</t>
+        </is>
+      </c>
+      <c r="D12" s="0" t="inlineStr">
+        <is>
+          <t>Anuv Jain</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="0" t="inlineStr">
+        <is>
+          <t>2026-04-22</t>
+        </is>
+      </c>
+      <c r="B13" s="0" t="n">
+        <v>12</v>
+      </c>
+      <c r="C13" s="0" t="inlineStr">
+        <is>
+          <t>Dooron Dooron</t>
+        </is>
+      </c>
+      <c r="D13" s="0" t="inlineStr">
+        <is>
+          <t>Paresh Pahuja</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="0" t="inlineStr">
+        <is>
+          <t>2026-04-22</t>
+        </is>
+      </c>
+      <c r="B14" s="0" t="n">
+        <v>13</v>
+      </c>
+      <c r="C14" s="0" t="inlineStr">
+        <is>
+          <t>Samjhawan</t>
+        </is>
+      </c>
+      <c r="D14" s="0" t="inlineStr">
+        <is>
+          <t>Jawad Ahmad</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="0" t="inlineStr">
+        <is>
+          <t>2026-04-22</t>
+        </is>
+      </c>
+      <c r="B15" s="0" t="n">
+        <v>14</v>
+      </c>
+      <c r="C15" s="0" t="inlineStr">
+        <is>
+          <t>Apna Bana Le</t>
+        </is>
+      </c>
+      <c r="D15" s="0" t="inlineStr">
+        <is>
+          <t>Sachin-Jigar</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="0" t="inlineStr">
+        <is>
+          <t>2026-04-22</t>
+        </is>
+      </c>
+      <c r="B16" s="0" t="n">
+        <v>15</v>
+      </c>
+      <c r="C16" s="0" t="inlineStr">
+        <is>
+          <t>Mann Mera</t>
+        </is>
+      </c>
+      <c r="D16" s="0" t="inlineStr">
+        <is>
+          <t>Gajendra Verma</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="0" t="inlineStr">
+        <is>
+          <t>2026-04-22</t>
+        </is>
+      </c>
+      <c r="B17" s="0" t="n">
+        <v>16</v>
+      </c>
+      <c r="C17" s="0" t="inlineStr">
+        <is>
+          <t>Boyfriend</t>
+        </is>
+      </c>
+      <c r="D17" s="0" t="inlineStr">
+        <is>
+          <t>Karan Aujla</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="0" t="inlineStr">
+        <is>
+          <t>2026-04-22</t>
+        </is>
+      </c>
+      <c r="B18" s="0" t="n">
+        <v>17</v>
+      </c>
+      <c r="C18" s="0" t="inlineStr">
+        <is>
+          <t>Dhurandhar The Revenge - Aari Aari</t>
+        </is>
+      </c>
+      <c r="D18" s="0" t="inlineStr">
+        <is>
+          <t>Shashwat Sachdev</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="0" t="inlineStr">
+        <is>
+          <t>2026-04-22</t>
+        </is>
+      </c>
+      <c r="B19" s="0" t="n">
+        <v>18</v>
+      </c>
+      <c r="C19" s="0" t="inlineStr">
+        <is>
+          <t>Ishq</t>
+        </is>
+      </c>
+      <c r="D19" s="0" t="inlineStr">
+        <is>
+          <t>Faheem Abdullah</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="0" t="inlineStr">
+        <is>
+          <t>2026-04-22</t>
+        </is>
+      </c>
+      <c r="B20" s="0" t="n">
+        <v>19</v>
+      </c>
+      <c r="C20" s="0" t="inlineStr">
+        <is>
+          <t>Shararat</t>
+        </is>
+      </c>
+      <c r="D20" s="0" t="inlineStr">
+        <is>
+          <t>Shashwat Sachdev</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="0" t="inlineStr">
+        <is>
+          <t>2026-04-22</t>
+        </is>
+      </c>
+      <c r="B21" s="0" t="n">
+        <v>20</v>
+      </c>
+      <c r="C21" s="0" t="inlineStr">
+        <is>
+          <t>Tum Ho Toh</t>
+        </is>
+      </c>
+      <c r="D21" s="0" t="inlineStr">
+        <is>
+          <t>Vishal Mishra</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="0" t="inlineStr">
+        <is>
+          <t>2026-04-22</t>
+        </is>
+      </c>
+      <c r="B22" s="0" t="n">
+        <v>21</v>
+      </c>
+      <c r="C22" s="0" t="inlineStr">
+        <is>
+          <t>Saiyaara</t>
+        </is>
+      </c>
+      <c r="D22" s="0" t="inlineStr">
+        <is>
+          <t>Tanishk Bagchi</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="0" t="inlineStr">
+        <is>
+          <t>2026-04-22</t>
+        </is>
+      </c>
+      <c r="B23" s="0" t="n">
+        <v>22</v>
+      </c>
+      <c r="C23" s="0" t="inlineStr">
+        <is>
+          <t>Jaan Se Guzarte Hain</t>
+        </is>
+      </c>
+      <c r="D23" s="0" t="inlineStr">
+        <is>
+          <t>Shashwat Sachdev</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="0" t="inlineStr">
+        <is>
+          <t>2026-04-22</t>
+        </is>
+      </c>
+      <c r="B24" s="0" t="n">
+        <v>23</v>
+      </c>
+      <c r="C24" s="0" t="inlineStr">
+        <is>
+          <t>Raanjhan</t>
+        </is>
+      </c>
+      <c r="D24" s="0" t="inlineStr">
+        <is>
+          <t>Sachet-Parampara</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="0" t="inlineStr">
+        <is>
+          <t>2026-04-22</t>
+        </is>
+      </c>
+      <c r="B25" s="0" t="n">
+        <v>24</v>
+      </c>
+      <c r="C25" s="0" t="inlineStr">
+        <is>
+          <t>Darkhaast</t>
+        </is>
+      </c>
+      <c r="D25" s="0" t="inlineStr">
+        <is>
+          <t>Mithoon</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="0" t="inlineStr">
+        <is>
+          <t>2026-04-22</t>
+        </is>
+      </c>
+      <c r="B26" s="0" t="n">
+        <v>25</v>
+      </c>
+      <c r="C26" s="0" t="inlineStr">
+        <is>
+          <t>Ishqa Ve</t>
+        </is>
+      </c>
+      <c r="D26" s="0" t="inlineStr">
+        <is>
+          <t>Zeeshan Ali</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="0" t="inlineStr">
+        <is>
+          <t>2026-04-22</t>
+        </is>
+      </c>
+      <c r="B27" s="0" t="n">
+        <v>26</v>
+      </c>
+      <c r="C27" s="0" t="inlineStr">
+        <is>
+          <t>For A Reason</t>
+        </is>
+      </c>
+      <c r="D27" s="0" t="inlineStr">
+        <is>
+          <t>Karan Aujla</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="0" t="inlineStr">
+        <is>
+          <t>2026-04-22</t>
+        </is>
+      </c>
+      <c r="B28" s="0" t="n">
+        <v>27</v>
+      </c>
+      <c r="C28" s="0" t="inlineStr">
+        <is>
+          <t>Tere Liye</t>
+        </is>
+      </c>
+      <c r="D28" s="0" t="inlineStr">
+        <is>
+          <t>Atif Aslam</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="0" t="inlineStr">
+        <is>
+          <t>2026-04-22</t>
+        </is>
+      </c>
+      <c r="B29" s="0" t="n">
+        <v>28</v>
+      </c>
+      <c r="C29" s="0" t="inlineStr">
+        <is>
+          <t>Deewaana Deewaana</t>
+        </is>
+      </c>
+      <c r="D29" s="0" t="inlineStr">
+        <is>
+          <t>A.R. Rahman</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="0" t="inlineStr">
+        <is>
+          <t>2026-04-22</t>
+        </is>
+      </c>
+      <c r="B30" s="0" t="n">
+        <v>29</v>
+      </c>
+      <c r="C30" s="0" t="inlineStr">
+        <is>
+          <t>Ehsaas</t>
+        </is>
+      </c>
+      <c r="D30" s="0" t="inlineStr">
+        <is>
+          <t>Faheem Abdullah</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="0" t="inlineStr">
+        <is>
+          <t>2026-04-22</t>
+        </is>
+      </c>
+      <c r="B31" s="0" t="n">
+        <v>30</v>
+      </c>
+      <c r="C31" s="0" t="inlineStr">
+        <is>
+          <t>Jo Tum Mere Ho</t>
+        </is>
+      </c>
+      <c r="D31" s="0" t="inlineStr">
+        <is>
+          <t>Anuv Jain</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="0" t="inlineStr">
+        <is>
+          <t>2026-04-22</t>
+        </is>
+      </c>
+      <c r="B32" s="0" t="n">
+        <v>31</v>
+      </c>
+      <c r="C32" s="0" t="inlineStr">
+        <is>
+          <t>Dhurandhar - Title Track</t>
+        </is>
+      </c>
+      <c r="D32" s="0" t="inlineStr">
+        <is>
+          <t>Shashwat Sachdev</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="0" t="inlineStr">
+        <is>
+          <t>2026-04-22</t>
+        </is>
+      </c>
+      <c r="B33" s="0" t="n">
+        <v>32</v>
+      </c>
+      <c r="C33" s="0" t="inlineStr">
+        <is>
+          <t>Agar Tum Saath Ho</t>
+        </is>
+      </c>
+      <c r="D33" s="0" t="inlineStr">
+        <is>
+          <t>Alka Yagnik</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="0" t="inlineStr">
+        <is>
+          <t>2026-04-22</t>
+        </is>
+      </c>
+      <c r="B34" s="0" t="n">
+        <v>33</v>
+      </c>
+      <c r="C34" s="0" t="inlineStr">
+        <is>
+          <t>Naal Nachna</t>
+        </is>
+      </c>
+      <c r="D34" s="0" t="inlineStr">
+        <is>
+          <t>Shashwat Sachdev</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="0" t="inlineStr">
+        <is>
+          <t>2026-04-22</t>
+        </is>
+      </c>
+      <c r="B35" s="0" t="n">
+        <v>34</v>
+      </c>
+      <c r="C35" s="0" t="inlineStr">
+        <is>
+          <t>Tere Bina</t>
+        </is>
+      </c>
+      <c r="D35" s="0" t="inlineStr">
+        <is>
+          <t>A.R. Rahman</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="0" t="inlineStr">
+        <is>
+          <t>2026-04-22</t>
+        </is>
+      </c>
+      <c r="B36" s="0" t="n">
+        <v>35</v>
+      </c>
+      <c r="C36" s="0" t="inlineStr">
+        <is>
+          <t>Mutta Kalakki</t>
+        </is>
+      </c>
+      <c r="D36" s="0" t="inlineStr">
+        <is>
+          <t>G. V. Prakash</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="0" t="inlineStr">
+        <is>
+          <t>2026-04-22</t>
+        </is>
+      </c>
+      <c r="B37" s="0" t="n">
+        <v>36</v>
+      </c>
+      <c r="C37" s="0" t="inlineStr">
+        <is>
+          <t>Phir Se</t>
+        </is>
+      </c>
+      <c r="D37" s="0" t="inlineStr">
+        <is>
+          <t>Shashwat Sachdev</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="0" t="inlineStr">
+        <is>
+          <t>2026-04-22</t>
+        </is>
+      </c>
+      <c r="B38" s="0" t="n">
+        <v>37</v>
+      </c>
+      <c r="C38" s="0" t="inlineStr">
+        <is>
+          <t>Bairi</t>
+        </is>
+      </c>
+      <c r="D38" s="0" t="inlineStr">
+        <is>
+          <t>Virat</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="0" t="inlineStr">
+        <is>
+          <t>2026-04-22</t>
+        </is>
+      </c>
+      <c r="B39" s="0" t="n">
+        <v>38</v>
+      </c>
+      <c r="C39" s="0" t="inlineStr">
+        <is>
+          <t>Barbaad</t>
+        </is>
+      </c>
+      <c r="D39" s="0" t="inlineStr">
+        <is>
+          <t>The Rish</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="0" t="inlineStr">
+        <is>
+          <t>2026-04-22</t>
+        </is>
+      </c>
+      <c r="B40" s="0" t="n">
+        <v>39</v>
+      </c>
+      <c r="C40" s="0" t="inlineStr">
+        <is>
+          <t>Ye Tune Kya Kiya</t>
+        </is>
+      </c>
+      <c r="D40" s="0" t="inlineStr">
+        <is>
+          <t>Pritam</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" s="0" t="inlineStr">
+        <is>
+          <t>2026-04-22</t>
+        </is>
+      </c>
+      <c r="B41" s="0" t="n">
+        <v>40</v>
+      </c>
+      <c r="C41" s="0" t="inlineStr">
+        <is>
+          <t>Teri Deewani</t>
+        </is>
+      </c>
+      <c r="D41" s="0" t="inlineStr">
+        <is>
+          <t>Kailash Kher</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" s="0" t="inlineStr">
+        <is>
+          <t>2026-04-22</t>
+        </is>
+      </c>
+      <c r="B42" s="0" t="n">
+        <v>41</v>
+      </c>
+      <c r="C42" s="0" t="inlineStr">
+        <is>
+          <t>Aaya Sher</t>
+        </is>
+      </c>
+      <c r="D42" s="0" t="inlineStr">
+        <is>
+          <t>Anirudh Ravichander</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" s="0" t="inlineStr">
+        <is>
+          <t>2026-04-22</t>
+        </is>
+      </c>
+      <c r="B43" s="0" t="n">
+        <v>42</v>
+      </c>
+      <c r="C43" s="0" t="inlineStr">
+        <is>
+          <t>Haseen</t>
+        </is>
+      </c>
+      <c r="D43" s="0" t="inlineStr">
+        <is>
+          <t>Talwiinder</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" s="0" t="inlineStr">
+        <is>
+          <t>2026-04-22</t>
+        </is>
+      </c>
+      <c r="B44" s="0" t="n">
+        <v>43</v>
+      </c>
+      <c r="C44" s="0" t="inlineStr">
+        <is>
+          <t>Mann Mera - Original Version</t>
+        </is>
+      </c>
+      <c r="D44" s="0" t="inlineStr">
+        <is>
+          <t>Gajendra Verma</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" s="0" t="inlineStr">
+        <is>
+          <t>2026-04-22</t>
+        </is>
+      </c>
+      <c r="B45" s="0" t="n">
+        <v>44</v>
+      </c>
+      <c r="C45" s="0" t="inlineStr">
+        <is>
+          <t>Mast Magan</t>
+        </is>
+      </c>
+      <c r="D45" s="0" t="inlineStr">
+        <is>
+          <t>Arijit Singh</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" s="0" t="inlineStr">
+        <is>
+          <t>2026-04-22</t>
+        </is>
+      </c>
+      <c r="B46" s="0" t="n">
+        <v>45</v>
+      </c>
+      <c r="C46" s="0" t="inlineStr">
+        <is>
+          <t>Oorum Blood</t>
+        </is>
+      </c>
+      <c r="D46" s="0" t="inlineStr">
+        <is>
+          <t>Sai Abhyankkar</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" s="0" t="inlineStr">
+        <is>
+          <t>2026-04-22</t>
+        </is>
+      </c>
+      <c r="B47" s="0" t="n">
+        <v>46</v>
+      </c>
+      <c r="C47" s="0" t="inlineStr">
+        <is>
+          <t>Jhol - Acoustic</t>
+        </is>
+      </c>
+      <c r="D47" s="0" t="inlineStr">
+        <is>
+          <t>Maanu</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" s="0" t="inlineStr">
+        <is>
+          <t>2026-04-22</t>
+        </is>
+      </c>
+      <c r="B48" s="0" t="n">
+        <v>47</v>
+      </c>
+      <c r="C48" s="0" t="inlineStr">
+        <is>
+          <t>Lutt Le Gaya</t>
+        </is>
+      </c>
+      <c r="D48" s="0" t="inlineStr">
+        <is>
+          <t>Shashwat Sachdev</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" s="0" t="inlineStr">
+        <is>
+          <t>2026-04-22</t>
+        </is>
+      </c>
+      <c r="B49" s="0" t="n">
+        <v>48</v>
+      </c>
+      <c r="C49" s="0" t="inlineStr">
+        <is>
+          <t>High On You</t>
+        </is>
+      </c>
+      <c r="D49" s="0" t="inlineStr">
+        <is>
+          <t>Jind Universe</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" s="0" t="inlineStr">
+        <is>
+          <t>2026-04-22</t>
+        </is>
+      </c>
+      <c r="B50" s="0" t="n">
+        <v>49</v>
+      </c>
+      <c r="C50" s="0" t="inlineStr">
+        <is>
+          <t>Zaalima</t>
+        </is>
+      </c>
+      <c r="D50" s="0" t="inlineStr">
+        <is>
+          <t>Arijit Singh</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" s="0" t="inlineStr">
+        <is>
+          <t>2026-04-22</t>
+        </is>
+      </c>
+      <c r="B51" s="0" t="n">
+        <v>50</v>
+      </c>
+      <c r="C51" s="0" t="inlineStr">
+        <is>
+          <t>Raabta</t>
+        </is>
+      </c>
+      <c r="D51" s="0" t="inlineStr">
+        <is>
+          <t>Pritam</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet42.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:D51"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="24" t="inlineStr">
+        <is>
+          <t>Date</t>
+        </is>
+      </c>
+      <c r="B1" s="24" t="inlineStr">
+        <is>
+          <t>Rank</t>
+        </is>
+      </c>
+      <c r="C1" s="24" t="inlineStr">
+        <is>
+          <t>Song</t>
+        </is>
+      </c>
+      <c r="D1" s="24" t="inlineStr">
+        <is>
+          <t>Artist</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="0" t="inlineStr">
+        <is>
+          <t>2026-04-26</t>
+        </is>
+      </c>
+      <c r="B2" s="0" t="n">
+        <v>1</v>
+      </c>
+      <c r="C2" s="0" t="inlineStr">
+        <is>
+          <t>Bairan</t>
+        </is>
+      </c>
+      <c r="D2" s="0" t="inlineStr">
+        <is>
+          <t>Banjaare</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="0" t="inlineStr">
+        <is>
+          <t>2026-04-26</t>
+        </is>
+      </c>
+      <c r="B3" s="0" t="n">
+        <v>2</v>
+      </c>
+      <c r="C3" s="0" t="inlineStr">
+        <is>
+          <t>Gehra Hua</t>
+        </is>
+      </c>
+      <c r="D3" s="0" t="inlineStr">
+        <is>
+          <t>Shashwat Sachdev</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="0" t="inlineStr">
+        <is>
+          <t>2026-04-26</t>
+        </is>
+      </c>
+      <c r="B4" s="0" t="n">
+        <v>3</v>
+      </c>
+      <c r="C4" s="0" t="inlineStr">
+        <is>
+          <t>Majboor</t>
+        </is>
+      </c>
+      <c r="D4" s="0" t="inlineStr">
+        <is>
+          <t>Sheheryar Rehan</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="0" t="inlineStr">
+        <is>
+          <t>2026-04-26</t>
+        </is>
+      </c>
+      <c r="B5" s="0" t="n">
+        <v>4</v>
+      </c>
+      <c r="C5" s="0" t="inlineStr">
+        <is>
+          <t>Khat</t>
+        </is>
+      </c>
+      <c r="D5" s="0" t="inlineStr">
+        <is>
+          <t>Navjot Ahuja</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="0" t="inlineStr">
+        <is>
+          <t>2026-04-26</t>
+        </is>
+      </c>
+      <c r="B6" s="0" t="n">
+        <v>5</v>
+      </c>
+      <c r="C6" s="0" t="inlineStr">
+        <is>
+          <t>Sheesha - Aakhya Mai Aakh Ghali Jo Bairan</t>
+        </is>
+      </c>
+      <c r="D6" s="0" t="inlineStr">
+        <is>
+          <t>Mitta Ror</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="0" t="inlineStr">
+        <is>
+          <t>2026-04-26</t>
+        </is>
+      </c>
+      <c r="B7" s="0" t="n">
+        <v>6</v>
+      </c>
+      <c r="C7" s="0" t="inlineStr">
+        <is>
+          <t>Jaiye Sajana</t>
+        </is>
+      </c>
+      <c r="D7" s="0" t="inlineStr">
+        <is>
+          <t>Shashwat Sachdev</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="0" t="inlineStr">
+        <is>
+          <t>2026-04-26</t>
+        </is>
+      </c>
+      <c r="B8" s="0" t="n">
+        <v>7</v>
+      </c>
+      <c r="C8" s="0" t="inlineStr">
+        <is>
+          <t>Pavazha Malli</t>
+        </is>
+      </c>
+      <c r="D8" s="0" t="inlineStr">
+        <is>
+          <t>Sai Abhyankkar</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="0" t="inlineStr">
+        <is>
+          <t>2026-04-26</t>
+        </is>
+      </c>
+      <c r="B9" s="0" t="n">
+        <v>8</v>
+      </c>
+      <c r="C9" s="0" t="inlineStr">
+        <is>
+          <t>Finding Her</t>
+        </is>
+      </c>
+      <c r="D9" s="0" t="inlineStr">
+        <is>
+          <t>Kushagra</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="0" t="inlineStr">
+        <is>
+          <t>2026-04-26</t>
+        </is>
+      </c>
+      <c r="B10" s="0" t="n">
+        <v>9</v>
+      </c>
+      <c r="C10" s="0" t="inlineStr">
+        <is>
+          <t>Sahiba</t>
+        </is>
+      </c>
+      <c r="D10" s="0" t="inlineStr">
+        <is>
+          <t>Aditya Rikhari</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="0" t="inlineStr">
+        <is>
+          <t>2026-04-26</t>
+        </is>
+      </c>
+      <c r="B11" s="0" t="n">
+        <v>10</v>
+      </c>
+      <c r="C11" s="0" t="inlineStr">
+        <is>
+          <t>Sitaare</t>
+        </is>
+      </c>
+      <c r="D11" s="0" t="inlineStr">
+        <is>
+          <t>Arijit Singh</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="0" t="inlineStr">
+        <is>
+          <t>2026-04-26</t>
+        </is>
+      </c>
+      <c r="B12" s="0" t="n">
+        <v>11</v>
+      </c>
+      <c r="C12" s="0" t="inlineStr">
+        <is>
+          <t>Arz Kiya Hai | Coke Studio Bharat</t>
+        </is>
+      </c>
+      <c r="D12" s="0" t="inlineStr">
+        <is>
+          <t>Anuv Jain</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="0" t="inlineStr">
+        <is>
+          <t>2026-04-26</t>
+        </is>
+      </c>
+      <c r="B13" s="0" t="n">
+        <v>12</v>
+      </c>
+      <c r="C13" s="0" t="inlineStr">
+        <is>
+          <t>Apna Bana Le</t>
+        </is>
+      </c>
+      <c r="D13" s="0" t="inlineStr">
+        <is>
+          <t>Sachin-Jigar</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="0" t="inlineStr">
+        <is>
+          <t>2026-04-26</t>
+        </is>
+      </c>
+      <c r="B14" s="0" t="n">
+        <v>13</v>
+      </c>
+      <c r="C14" s="0" t="inlineStr">
+        <is>
+          <t>Dooron Dooron</t>
+        </is>
+      </c>
+      <c r="D14" s="0" t="inlineStr">
+        <is>
+          <t>Paresh Pahuja</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="0" t="inlineStr">
+        <is>
+          <t>2026-04-26</t>
+        </is>
+      </c>
+      <c r="B15" s="0" t="n">
+        <v>14</v>
+      </c>
+      <c r="C15" s="0" t="inlineStr">
+        <is>
+          <t>Samjhawan</t>
+        </is>
+      </c>
+      <c r="D15" s="0" t="inlineStr">
+        <is>
+          <t>Jawad Ahmad</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="0" t="inlineStr">
+        <is>
+          <t>2026-04-26</t>
+        </is>
+      </c>
+      <c r="B16" s="0" t="n">
+        <v>15</v>
+      </c>
+      <c r="C16" s="0" t="inlineStr">
+        <is>
+          <t>Mann Mera</t>
+        </is>
+      </c>
+      <c r="D16" s="0" t="inlineStr">
+        <is>
+          <t>Gajendra Verma</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="0" t="inlineStr">
+        <is>
+          <t>2026-04-26</t>
+        </is>
+      </c>
+      <c r="B17" s="0" t="n">
+        <v>16</v>
+      </c>
+      <c r="C17" s="0" t="inlineStr">
+        <is>
+          <t>Shararat</t>
+        </is>
+      </c>
+      <c r="D17" s="0" t="inlineStr">
+        <is>
+          <t>Shashwat Sachdev</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="0" t="inlineStr">
+        <is>
+          <t>2026-04-26</t>
+        </is>
+      </c>
+      <c r="B18" s="0" t="n">
+        <v>17</v>
+      </c>
+      <c r="C18" s="0" t="inlineStr">
+        <is>
+          <t>Boyfriend</t>
+        </is>
+      </c>
+      <c r="D18" s="0" t="inlineStr">
+        <is>
+          <t>Karan Aujla</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="0" t="inlineStr">
+        <is>
+          <t>2026-04-26</t>
+        </is>
+      </c>
+      <c r="B19" s="0" t="n">
+        <v>18</v>
+      </c>
+      <c r="C19" s="0" t="inlineStr">
+        <is>
+          <t>Tum Ho Toh</t>
+        </is>
+      </c>
+      <c r="D19" s="0" t="inlineStr">
+        <is>
+          <t>Vishal Mishra</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="0" t="inlineStr">
+        <is>
+          <t>2026-04-26</t>
+        </is>
+      </c>
+      <c r="B20" s="0" t="n">
+        <v>19</v>
+      </c>
+      <c r="C20" s="0" t="inlineStr">
+        <is>
+          <t>Ishq</t>
+        </is>
+      </c>
+      <c r="D20" s="0" t="inlineStr">
+        <is>
+          <t>Faheem Abdullah</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="0" t="inlineStr">
+        <is>
+          <t>2026-04-26</t>
+        </is>
+      </c>
+      <c r="B21" s="0" t="n">
+        <v>20</v>
+      </c>
+      <c r="C21" s="0" t="inlineStr">
+        <is>
+          <t>Dhurandhar The Revenge - Aari Aari</t>
+        </is>
+      </c>
+      <c r="D21" s="0" t="inlineStr">
+        <is>
+          <t>Shashwat Sachdev</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="0" t="inlineStr">
+        <is>
+          <t>2026-04-26</t>
+        </is>
+      </c>
+      <c r="B22" s="0" t="n">
+        <v>21</v>
+      </c>
+      <c r="C22" s="0" t="inlineStr">
+        <is>
+          <t>Saiyaara</t>
+        </is>
+      </c>
+      <c r="D22" s="0" t="inlineStr">
+        <is>
+          <t>Tanishk Bagchi</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="0" t="inlineStr">
+        <is>
+          <t>2026-04-26</t>
+        </is>
+      </c>
+      <c r="B23" s="0" t="n">
+        <v>22</v>
+      </c>
+      <c r="C23" s="0" t="inlineStr">
+        <is>
+          <t>Deewaana Deewaana</t>
+        </is>
+      </c>
+      <c r="D23" s="0" t="inlineStr">
+        <is>
+          <t>A.R. Rahman</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="0" t="inlineStr">
+        <is>
+          <t>2026-04-26</t>
+        </is>
+      </c>
+      <c r="B24" s="0" t="n">
+        <v>23</v>
+      </c>
+      <c r="C24" s="0" t="inlineStr">
+        <is>
+          <t>Jaan Se Guzarte Hain</t>
+        </is>
+      </c>
+      <c r="D24" s="0" t="inlineStr">
+        <is>
+          <t>Shashwat Sachdev</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="0" t="inlineStr">
+        <is>
+          <t>2026-04-26</t>
+        </is>
+      </c>
+      <c r="B25" s="0" t="n">
+        <v>24</v>
+      </c>
+      <c r="C25" s="0" t="inlineStr">
+        <is>
+          <t>Darkhaast</t>
+        </is>
+      </c>
+      <c r="D25" s="0" t="inlineStr">
+        <is>
+          <t>Mithoon</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="0" t="inlineStr">
+        <is>
+          <t>2026-04-26</t>
+        </is>
+      </c>
+      <c r="B26" s="0" t="n">
+        <v>25</v>
+      </c>
+      <c r="C26" s="0" t="inlineStr">
+        <is>
+          <t>For A Reason</t>
+        </is>
+      </c>
+      <c r="D26" s="0" t="inlineStr">
+        <is>
+          <t>Karan Aujla</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="0" t="inlineStr">
+        <is>
+          <t>2026-04-26</t>
+        </is>
+      </c>
+      <c r="B27" s="0" t="n">
+        <v>26</v>
+      </c>
+      <c r="C27" s="0" t="inlineStr">
+        <is>
+          <t>Tere Liye</t>
+        </is>
+      </c>
+      <c r="D27" s="0" t="inlineStr">
+        <is>
+          <t>Atif Aslam</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="0" t="inlineStr">
+        <is>
+          <t>2026-04-26</t>
+        </is>
+      </c>
+      <c r="B28" s="0" t="n">
+        <v>27</v>
+      </c>
+      <c r="C28" s="0" t="inlineStr">
+        <is>
+          <t>Raanjhan</t>
+        </is>
+      </c>
+      <c r="D28" s="0" t="inlineStr">
+        <is>
+          <t>Sachet-Parampara</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="0" t="inlineStr">
+        <is>
+          <t>2026-04-26</t>
+        </is>
+      </c>
+      <c r="B29" s="0" t="n">
+        <v>28</v>
+      </c>
+      <c r="C29" s="0" t="inlineStr">
+        <is>
+          <t>Ishqa Ve</t>
+        </is>
+      </c>
+      <c r="D29" s="0" t="inlineStr">
+        <is>
+          <t>Zeeshan Ali</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="0" t="inlineStr">
+        <is>
+          <t>2026-04-26</t>
+        </is>
+      </c>
+      <c r="B30" s="0" t="n">
+        <v>29</v>
+      </c>
+      <c r="C30" s="0" t="inlineStr">
+        <is>
+          <t>Jo Tum Mere Ho</t>
+        </is>
+      </c>
+      <c r="D30" s="0" t="inlineStr">
+        <is>
+          <t>Anuv Jain</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="0" t="inlineStr">
+        <is>
+          <t>2026-04-26</t>
+        </is>
+      </c>
+      <c r="B31" s="0" t="n">
+        <v>30</v>
+      </c>
+      <c r="C31" s="0" t="inlineStr">
+        <is>
+          <t>Tere Bina</t>
+        </is>
+      </c>
+      <c r="D31" s="0" t="inlineStr">
+        <is>
+          <t>A.R. Rahman</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="0" t="inlineStr">
+        <is>
+          <t>2026-04-26</t>
+        </is>
+      </c>
+      <c r="B32" s="0" t="n">
+        <v>31</v>
+      </c>
+      <c r="C32" s="0" t="inlineStr">
+        <is>
+          <t>Ehsaas</t>
+        </is>
+      </c>
+      <c r="D32" s="0" t="inlineStr">
+        <is>
+          <t>Faheem Abdullah</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="0" t="inlineStr">
+        <is>
+          <t>2026-04-26</t>
+        </is>
+      </c>
+      <c r="B33" s="0" t="n">
+        <v>32</v>
+      </c>
+      <c r="C33" s="0" t="inlineStr">
+        <is>
+          <t>Dhurandhar - Title Track</t>
+        </is>
+      </c>
+      <c r="D33" s="0" t="inlineStr">
+        <is>
+          <t>Shashwat Sachdev</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="0" t="inlineStr">
+        <is>
+          <t>2026-04-26</t>
+        </is>
+      </c>
+      <c r="B34" s="0" t="n">
+        <v>33</v>
+      </c>
+      <c r="C34" s="0" t="inlineStr">
+        <is>
+          <t>Agar Tum Saath Ho</t>
+        </is>
+      </c>
+      <c r="D34" s="0" t="inlineStr">
+        <is>
+          <t>Alka Yagnik</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="0" t="inlineStr">
+        <is>
+          <t>2026-04-26</t>
+        </is>
+      </c>
+      <c r="B35" s="0" t="n">
+        <v>34</v>
+      </c>
+      <c r="C35" s="0" t="inlineStr">
+        <is>
+          <t>Bairi</t>
+        </is>
+      </c>
+      <c r="D35" s="0" t="inlineStr">
+        <is>
+          <t>Virat</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="0" t="inlineStr">
+        <is>
+          <t>2026-04-26</t>
+        </is>
+      </c>
+      <c r="B36" s="0" t="n">
+        <v>35</v>
+      </c>
+      <c r="C36" s="0" t="inlineStr">
+        <is>
+          <t>Ye Tune Kya Kiya</t>
+        </is>
+      </c>
+      <c r="D36" s="0" t="inlineStr">
+        <is>
+          <t>Pritam</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="0" t="inlineStr">
+        <is>
+          <t>2026-04-26</t>
+        </is>
+      </c>
+      <c r="B37" s="0" t="n">
+        <v>36</v>
+      </c>
+      <c r="C37" s="0" t="inlineStr">
+        <is>
+          <t>Barbaad</t>
+        </is>
+      </c>
+      <c r="D37" s="0" t="inlineStr">
+        <is>
+          <t>The Rish</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="0" t="inlineStr">
+        <is>
+          <t>2026-04-26</t>
+        </is>
+      </c>
+      <c r="B38" s="0" t="n">
+        <v>37</v>
+      </c>
+      <c r="C38" s="0" t="inlineStr">
+        <is>
+          <t>Mutta Kalakki</t>
+        </is>
+      </c>
+      <c r="D38" s="0" t="inlineStr">
+        <is>
+          <t>G. V. Prakash</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="0" t="inlineStr">
+        <is>
+          <t>2026-04-26</t>
+        </is>
+      </c>
+      <c r="B39" s="0" t="n">
+        <v>38</v>
+      </c>
+      <c r="C39" s="0" t="inlineStr">
+        <is>
+          <t>Naal Nachna</t>
+        </is>
+      </c>
+      <c r="D39" s="0" t="inlineStr">
+        <is>
+          <t>Shashwat Sachdev</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="0" t="inlineStr">
+        <is>
+          <t>2026-04-26</t>
+        </is>
+      </c>
+      <c r="B40" s="0" t="n">
+        <v>39</v>
+      </c>
+      <c r="C40" s="0" t="inlineStr">
+        <is>
+          <t>Haseen</t>
+        </is>
+      </c>
+      <c r="D40" s="0" t="inlineStr">
+        <is>
+          <t>Talwiinder</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" s="0" t="inlineStr">
+        <is>
+          <t>2026-04-26</t>
+        </is>
+      </c>
+      <c r="B41" s="0" t="n">
+        <v>40</v>
+      </c>
+      <c r="C41" s="0" t="inlineStr">
+        <is>
+          <t>Phir Se</t>
+        </is>
+      </c>
+      <c r="D41" s="0" t="inlineStr">
+        <is>
+          <t>Shashwat Sachdev</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" s="0" t="inlineStr">
+        <is>
+          <t>2026-04-26</t>
+        </is>
+      </c>
+      <c r="B42" s="0" t="n">
+        <v>41</v>
+      </c>
+      <c r="C42" s="0" t="inlineStr">
+        <is>
+          <t>Aaya Sher</t>
+        </is>
+      </c>
+      <c r="D42" s="0" t="inlineStr">
+        <is>
+          <t>Anirudh Ravichander</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" s="0" t="inlineStr">
+        <is>
+          <t>2026-04-26</t>
+        </is>
+      </c>
+      <c r="B43" s="0" t="n">
+        <v>42</v>
+      </c>
+      <c r="C43" s="0" t="inlineStr">
+        <is>
+          <t>Lutt Le Gaya</t>
+        </is>
+      </c>
+      <c r="D43" s="0" t="inlineStr">
+        <is>
+          <t>Shashwat Sachdev</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" s="0" t="inlineStr">
+        <is>
+          <t>2026-04-26</t>
+        </is>
+      </c>
+      <c r="B44" s="0" t="n">
+        <v>43</v>
+      </c>
+      <c r="C44" s="0" t="inlineStr">
+        <is>
+          <t>High On You</t>
+        </is>
+      </c>
+      <c r="D44" s="0" t="inlineStr">
+        <is>
+          <t>Jind Universe</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" s="0" t="inlineStr">
+        <is>
+          <t>2026-04-26</t>
+        </is>
+      </c>
+      <c r="B45" s="0" t="n">
+        <v>44</v>
+      </c>
+      <c r="C45" s="0" t="inlineStr">
+        <is>
+          <t>Jhol - Acoustic</t>
+        </is>
+      </c>
+      <c r="D45" s="0" t="inlineStr">
+        <is>
+          <t>Maanu</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" s="0" t="inlineStr">
+        <is>
+          <t>2026-04-26</t>
+        </is>
+      </c>
+      <c r="B46" s="0" t="n">
+        <v>45</v>
+      </c>
+      <c r="C46" s="0" t="inlineStr">
+        <is>
+          <t>Mast Magan</t>
+        </is>
+      </c>
+      <c r="D46" s="0" t="inlineStr">
+        <is>
+          <t>Arijit Singh</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" s="0" t="inlineStr">
+        <is>
+          <t>2026-04-26</t>
+        </is>
+      </c>
+      <c r="B47" s="0" t="n">
+        <v>46</v>
+      </c>
+      <c r="C47" s="0" t="inlineStr">
+        <is>
+          <t>Teri Deewani</t>
+        </is>
+      </c>
+      <c r="D47" s="0" t="inlineStr">
+        <is>
+          <t>Kailash Kher</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" s="0" t="inlineStr">
+        <is>
+          <t>2026-04-26</t>
+        </is>
+      </c>
+      <c r="B48" s="0" t="n">
+        <v>47</v>
+      </c>
+      <c r="C48" s="0" t="inlineStr">
+        <is>
+          <t>Mann Mera - Original Version</t>
+        </is>
+      </c>
+      <c r="D48" s="0" t="inlineStr">
+        <is>
+          <t>Gajendra Verma</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" s="0" t="inlineStr">
+        <is>
+          <t>2026-04-26</t>
+        </is>
+      </c>
+      <c r="B49" s="0" t="n">
+        <v>48</v>
+      </c>
+      <c r="C49" s="0" t="inlineStr">
+        <is>
+          <t>Zaalima</t>
+        </is>
+      </c>
+      <c r="D49" s="0" t="inlineStr">
+        <is>
+          <t>Arijit Singh</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" s="0" t="inlineStr">
+        <is>
+          <t>2026-04-26</t>
+        </is>
+      </c>
+      <c r="B50" s="0" t="n">
+        <v>49</v>
+      </c>
+      <c r="C50" s="0" t="inlineStr">
+        <is>
+          <t>Oorum Blood</t>
+        </is>
+      </c>
+      <c r="D50" s="0" t="inlineStr">
+        <is>
+          <t>Sai Abhyankkar</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" s="0" t="inlineStr">
+        <is>
+          <t>2026-04-26</t>
+        </is>
+      </c>
+      <c r="B51" s="0" t="n">
+        <v>50</v>
+      </c>
+      <c r="C51" s="0" t="inlineStr">
+        <is>
+          <t>Thodi Si Daaru</t>
+        </is>
+      </c>
+      <c r="D51" s="0" t="inlineStr">
+        <is>
+          <t>AP Dhillon</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet43.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:D51"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="24" t="inlineStr">
+        <is>
+          <t>Date</t>
+        </is>
+      </c>
+      <c r="B1" s="24" t="inlineStr">
+        <is>
+          <t>Rank</t>
+        </is>
+      </c>
+      <c r="C1" s="24" t="inlineStr">
+        <is>
+          <t>Song</t>
+        </is>
+      </c>
+      <c r="D1" s="24" t="inlineStr">
+        <is>
+          <t>Artist</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="0" t="inlineStr">
+        <is>
+          <t>2026-04-24</t>
+        </is>
+      </c>
+      <c r="B2" s="0" t="n">
+        <v>1</v>
+      </c>
+      <c r="C2" s="0" t="inlineStr">
+        <is>
+          <t>Bairan</t>
+        </is>
+      </c>
+      <c r="D2" s="0" t="inlineStr">
+        <is>
+          <t>Banjaare</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="0" t="inlineStr">
+        <is>
+          <t>2026-04-24</t>
+        </is>
+      </c>
+      <c r="B3" s="0" t="n">
+        <v>2</v>
+      </c>
+      <c r="C3" s="0" t="inlineStr">
+        <is>
+          <t>Gehra Hua</t>
+        </is>
+      </c>
+      <c r="D3" s="0" t="inlineStr">
+        <is>
+          <t>Shashwat Sachdev</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="0" t="inlineStr">
+        <is>
+          <t>2026-04-24</t>
+        </is>
+      </c>
+      <c r="B4" s="0" t="n">
+        <v>3</v>
+      </c>
+      <c r="C4" s="0" t="inlineStr">
+        <is>
+          <t>Majboor</t>
+        </is>
+      </c>
+      <c r="D4" s="0" t="inlineStr">
+        <is>
+          <t>Sheheryar Rehan</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="0" t="inlineStr">
+        <is>
+          <t>2026-04-24</t>
+        </is>
+      </c>
+      <c r="B5" s="0" t="n">
+        <v>4</v>
+      </c>
+      <c r="C5" s="0" t="inlineStr">
+        <is>
+          <t>Khat</t>
+        </is>
+      </c>
+      <c r="D5" s="0" t="inlineStr">
+        <is>
+          <t>Navjot Ahuja</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="0" t="inlineStr">
+        <is>
+          <t>2026-04-24</t>
+        </is>
+      </c>
+      <c r="B6" s="0" t="n">
+        <v>5</v>
+      </c>
+      <c r="C6" s="0" t="inlineStr">
+        <is>
+          <t>Sheesha - Aakhya Mai Aakh Ghali Jo Bairan</t>
+        </is>
+      </c>
+      <c r="D6" s="0" t="inlineStr">
+        <is>
+          <t>Mitta Ror</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="0" t="inlineStr">
+        <is>
+          <t>2026-04-24</t>
+        </is>
+      </c>
+      <c r="B7" s="0" t="n">
+        <v>6</v>
+      </c>
+      <c r="C7" s="0" t="inlineStr">
+        <is>
+          <t>Jaiye Sajana</t>
+        </is>
+      </c>
+      <c r="D7" s="0" t="inlineStr">
+        <is>
+          <t>Shashwat Sachdev</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="0" t="inlineStr">
+        <is>
+          <t>2026-04-24</t>
+        </is>
+      </c>
+      <c r="B8" s="0" t="n">
+        <v>7</v>
+      </c>
+      <c r="C8" s="0" t="inlineStr">
+        <is>
+          <t>Pavazha Malli</t>
+        </is>
+      </c>
+      <c r="D8" s="0" t="inlineStr">
+        <is>
+          <t>Sai Abhyankkar</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="0" t="inlineStr">
+        <is>
+          <t>2026-04-24</t>
+        </is>
+      </c>
+      <c r="B9" s="0" t="n">
+        <v>8</v>
+      </c>
+      <c r="C9" s="0" t="inlineStr">
+        <is>
+          <t>Finding Her</t>
+        </is>
+      </c>
+      <c r="D9" s="0" t="inlineStr">
+        <is>
+          <t>Kushagra</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="0" t="inlineStr">
+        <is>
+          <t>2026-04-24</t>
+        </is>
+      </c>
+      <c r="B10" s="0" t="n">
+        <v>9</v>
+      </c>
+      <c r="C10" s="0" t="inlineStr">
+        <is>
+          <t>Arz Kiya Hai | Coke Studio Bharat</t>
+        </is>
+      </c>
+      <c r="D10" s="0" t="inlineStr">
+        <is>
+          <t>Anuv Jain</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="0" t="inlineStr">
+        <is>
+          <t>2026-04-24</t>
+        </is>
+      </c>
+      <c r="B11" s="0" t="n">
+        <v>10</v>
+      </c>
+      <c r="C11" s="0" t="inlineStr">
+        <is>
+          <t>Sahiba</t>
+        </is>
+      </c>
+      <c r="D11" s="0" t="inlineStr">
+        <is>
+          <t>Aditya Rikhari</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="0" t="inlineStr">
+        <is>
+          <t>2026-04-24</t>
+        </is>
+      </c>
+      <c r="B12" s="0" t="n">
+        <v>11</v>
+      </c>
+      <c r="C12" s="0" t="inlineStr">
+        <is>
+          <t>Dooron Dooron</t>
+        </is>
+      </c>
+      <c r="D12" s="0" t="inlineStr">
+        <is>
+          <t>Paresh Pahuja</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="0" t="inlineStr">
+        <is>
+          <t>2026-04-24</t>
+        </is>
+      </c>
+      <c r="B13" s="0" t="n">
+        <v>12</v>
+      </c>
+      <c r="C13" s="0" t="inlineStr">
+        <is>
+          <t>Sitaare</t>
+        </is>
+      </c>
+      <c r="D13" s="0" t="inlineStr">
+        <is>
+          <t>Arijit Singh</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="0" t="inlineStr">
+        <is>
+          <t>2026-04-24</t>
+        </is>
+      </c>
+      <c r="B14" s="0" t="n">
+        <v>13</v>
+      </c>
+      <c r="C14" s="0" t="inlineStr">
+        <is>
+          <t>Apna Bana Le</t>
+        </is>
+      </c>
+      <c r="D14" s="0" t="inlineStr">
+        <is>
+          <t>Sachin-Jigar</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="0" t="inlineStr">
+        <is>
+          <t>2026-04-24</t>
+        </is>
+      </c>
+      <c r="B15" s="0" t="n">
+        <v>14</v>
+      </c>
+      <c r="C15" s="0" t="inlineStr">
+        <is>
+          <t>Samjhawan</t>
+        </is>
+      </c>
+      <c r="D15" s="0" t="inlineStr">
+        <is>
+          <t>Jawad Ahmad</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="0" t="inlineStr">
+        <is>
+          <t>2026-04-24</t>
+        </is>
+      </c>
+      <c r="B16" s="0" t="n">
+        <v>15</v>
+      </c>
+      <c r="C16" s="0" t="inlineStr">
+        <is>
+          <t>Mann Mera</t>
+        </is>
+      </c>
+      <c r="D16" s="0" t="inlineStr">
+        <is>
+          <t>Gajendra Verma</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="0" t="inlineStr">
+        <is>
+          <t>2026-04-24</t>
+        </is>
+      </c>
+      <c r="B17" s="0" t="n">
+        <v>16</v>
+      </c>
+      <c r="C17" s="0" t="inlineStr">
+        <is>
+          <t>Boyfriend</t>
+        </is>
+      </c>
+      <c r="D17" s="0" t="inlineStr">
+        <is>
+          <t>Karan Aujla</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="0" t="inlineStr">
+        <is>
+          <t>2026-04-24</t>
+        </is>
+      </c>
+      <c r="B18" s="0" t="n">
+        <v>17</v>
+      </c>
+      <c r="C18" s="0" t="inlineStr">
+        <is>
+          <t>Shararat</t>
+        </is>
+      </c>
+      <c r="D18" s="0" t="inlineStr">
+        <is>
+          <t>Shashwat Sachdev</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="0" t="inlineStr">
+        <is>
+          <t>2026-04-24</t>
+        </is>
+      </c>
+      <c r="B19" s="0" t="n">
+        <v>18</v>
+      </c>
+      <c r="C19" s="0" t="inlineStr">
+        <is>
+          <t>Dhurandhar The Revenge - Aari Aari</t>
+        </is>
+      </c>
+      <c r="D19" s="0" t="inlineStr">
+        <is>
+          <t>Shashwat Sachdev</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="0" t="inlineStr">
+        <is>
+          <t>2026-04-24</t>
+        </is>
+      </c>
+      <c r="B20" s="0" t="n">
+        <v>19</v>
+      </c>
+      <c r="C20" s="0" t="inlineStr">
+        <is>
+          <t>Ishq</t>
+        </is>
+      </c>
+      <c r="D20" s="0" t="inlineStr">
+        <is>
+          <t>Faheem Abdullah</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="0" t="inlineStr">
+        <is>
+          <t>2026-04-24</t>
+        </is>
+      </c>
+      <c r="B21" s="0" t="n">
+        <v>20</v>
+      </c>
+      <c r="C21" s="0" t="inlineStr">
+        <is>
+          <t>Tum Ho Toh</t>
+        </is>
+      </c>
+      <c r="D21" s="0" t="inlineStr">
+        <is>
+          <t>Vishal Mishra</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="0" t="inlineStr">
+        <is>
+          <t>2026-04-24</t>
+        </is>
+      </c>
+      <c r="B22" s="0" t="n">
+        <v>21</v>
+      </c>
+      <c r="C22" s="0" t="inlineStr">
+        <is>
+          <t>Saiyaara</t>
+        </is>
+      </c>
+      <c r="D22" s="0" t="inlineStr">
+        <is>
+          <t>Tanishk Bagchi</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="0" t="inlineStr">
+        <is>
+          <t>2026-04-24</t>
+        </is>
+      </c>
+      <c r="B23" s="0" t="n">
+        <v>22</v>
+      </c>
+      <c r="C23" s="0" t="inlineStr">
+        <is>
+          <t>Jaan Se Guzarte Hain</t>
+        </is>
+      </c>
+      <c r="D23" s="0" t="inlineStr">
+        <is>
+          <t>Shashwat Sachdev</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="0" t="inlineStr">
+        <is>
+          <t>2026-04-24</t>
+        </is>
+      </c>
+      <c r="B24" s="0" t="n">
+        <v>23</v>
+      </c>
+      <c r="C24" s="0" t="inlineStr">
+        <is>
+          <t>For A Reason</t>
+        </is>
+      </c>
+      <c r="D24" s="0" t="inlineStr">
+        <is>
+          <t>Karan Aujla</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="0" t="inlineStr">
+        <is>
+          <t>2026-04-24</t>
+        </is>
+      </c>
+      <c r="B25" s="0" t="n">
+        <v>24</v>
+      </c>
+      <c r="C25" s="0" t="inlineStr">
+        <is>
+          <t>Deewaana Deewaana</t>
+        </is>
+      </c>
+      <c r="D25" s="0" t="inlineStr">
+        <is>
+          <t>A.R. Rahman</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="0" t="inlineStr">
+        <is>
+          <t>2026-04-24</t>
+        </is>
+      </c>
+      <c r="B26" s="0" t="n">
+        <v>25</v>
+      </c>
+      <c r="C26" s="0" t="inlineStr">
+        <is>
+          <t>Raanjhan</t>
+        </is>
+      </c>
+      <c r="D26" s="0" t="inlineStr">
+        <is>
+          <t>Sachet-Parampara</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="0" t="inlineStr">
+        <is>
+          <t>2026-04-24</t>
+        </is>
+      </c>
+      <c r="B27" s="0" t="n">
+        <v>26</v>
+      </c>
+      <c r="C27" s="0" t="inlineStr">
+        <is>
+          <t>Darkhaast</t>
+        </is>
+      </c>
+      <c r="D27" s="0" t="inlineStr">
+        <is>
+          <t>Mithoon</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="0" t="inlineStr">
+        <is>
+          <t>2026-04-24</t>
+        </is>
+      </c>
+      <c r="B28" s="0" t="n">
+        <v>27</v>
+      </c>
+      <c r="C28" s="0" t="inlineStr">
+        <is>
+          <t>Tere Liye</t>
+        </is>
+      </c>
+      <c r="D28" s="0" t="inlineStr">
+        <is>
+          <t>Atif Aslam</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="0" t="inlineStr">
+        <is>
+          <t>2026-04-24</t>
+        </is>
+      </c>
+      <c r="B29" s="0" t="n">
+        <v>28</v>
+      </c>
+      <c r="C29" s="0" t="inlineStr">
+        <is>
+          <t>Ishqa Ve</t>
+        </is>
+      </c>
+      <c r="D29" s="0" t="inlineStr">
+        <is>
+          <t>Zeeshan Ali</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="0" t="inlineStr">
+        <is>
+          <t>2026-04-24</t>
+        </is>
+      </c>
+      <c r="B30" s="0" t="n">
+        <v>29</v>
+      </c>
+      <c r="C30" s="0" t="inlineStr">
+        <is>
+          <t>Dhurandhar - Title Track</t>
+        </is>
+      </c>
+      <c r="D30" s="0" t="inlineStr">
+        <is>
+          <t>Shashwat Sachdev</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="0" t="inlineStr">
+        <is>
+          <t>2026-04-24</t>
+        </is>
+      </c>
+      <c r="B31" s="0" t="n">
+        <v>30</v>
+      </c>
+      <c r="C31" s="0" t="inlineStr">
+        <is>
+          <t>Jo Tum Mere Ho</t>
+        </is>
+      </c>
+      <c r="D31" s="0" t="inlineStr">
+        <is>
+          <t>Anuv Jain</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="0" t="inlineStr">
+        <is>
+          <t>2026-04-24</t>
+        </is>
+      </c>
+      <c r="B32" s="0" t="n">
+        <v>31</v>
+      </c>
+      <c r="C32" s="0" t="inlineStr">
+        <is>
+          <t>Agar Tum Saath Ho</t>
+        </is>
+      </c>
+      <c r="D32" s="0" t="inlineStr">
+        <is>
+          <t>Alka Yagnik</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="0" t="inlineStr">
+        <is>
+          <t>2026-04-24</t>
+        </is>
+      </c>
+      <c r="B33" s="0" t="n">
+        <v>32</v>
+      </c>
+      <c r="C33" s="0" t="inlineStr">
+        <is>
+          <t>Ehsaas</t>
+        </is>
+      </c>
+      <c r="D33" s="0" t="inlineStr">
+        <is>
+          <t>Faheem Abdullah</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="0" t="inlineStr">
+        <is>
+          <t>2026-04-24</t>
+        </is>
+      </c>
+      <c r="B34" s="0" t="n">
+        <v>33</v>
+      </c>
+      <c r="C34" s="0" t="inlineStr">
+        <is>
+          <t>Tere Bina</t>
+        </is>
+      </c>
+      <c r="D34" s="0" t="inlineStr">
+        <is>
+          <t>A.R. Rahman</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="0" t="inlineStr">
+        <is>
+          <t>2026-04-24</t>
+        </is>
+      </c>
+      <c r="B35" s="0" t="n">
+        <v>34</v>
+      </c>
+      <c r="C35" s="0" t="inlineStr">
+        <is>
+          <t>Naal Nachna</t>
+        </is>
+      </c>
+      <c r="D35" s="0" t="inlineStr">
+        <is>
+          <t>Shashwat Sachdev</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="0" t="inlineStr">
+        <is>
+          <t>2026-04-24</t>
+        </is>
+      </c>
+      <c r="B36" s="0" t="n">
+        <v>35</v>
+      </c>
+      <c r="C36" s="0" t="inlineStr">
+        <is>
+          <t>Barbaad</t>
+        </is>
+      </c>
+      <c r="D36" s="0" t="inlineStr">
+        <is>
+          <t>The Rish</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="0" t="inlineStr">
+        <is>
+          <t>2026-04-24</t>
+        </is>
+      </c>
+      <c r="B37" s="0" t="n">
+        <v>36</v>
+      </c>
+      <c r="C37" s="0" t="inlineStr">
+        <is>
+          <t>Ye Tune Kya Kiya</t>
+        </is>
+      </c>
+      <c r="D37" s="0" t="inlineStr">
+        <is>
+          <t>Pritam</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="0" t="inlineStr">
+        <is>
+          <t>2026-04-24</t>
+        </is>
+      </c>
+      <c r="B38" s="0" t="n">
+        <v>37</v>
+      </c>
+      <c r="C38" s="0" t="inlineStr">
+        <is>
+          <t>Bairi</t>
+        </is>
+      </c>
+      <c r="D38" s="0" t="inlineStr">
+        <is>
+          <t>Virat</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="0" t="inlineStr">
+        <is>
+          <t>2026-04-24</t>
+        </is>
+      </c>
+      <c r="B39" s="0" t="n">
+        <v>38</v>
+      </c>
+      <c r="C39" s="0" t="inlineStr">
+        <is>
+          <t>Teri Deewani</t>
+        </is>
+      </c>
+      <c r="D39" s="0" t="inlineStr">
+        <is>
+          <t>Kailash Kher</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="0" t="inlineStr">
+        <is>
+          <t>2026-04-24</t>
+        </is>
+      </c>
+      <c r="B40" s="0" t="n">
+        <v>39</v>
+      </c>
+      <c r="C40" s="0" t="inlineStr">
+        <is>
+          <t>Phir Se</t>
+        </is>
+      </c>
+      <c r="D40" s="0" t="inlineStr">
+        <is>
+          <t>Shashwat Sachdev</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" s="0" t="inlineStr">
+        <is>
+          <t>2026-04-24</t>
+        </is>
+      </c>
+      <c r="B41" s="0" t="n">
+        <v>40</v>
+      </c>
+      <c r="C41" s="0" t="inlineStr">
+        <is>
+          <t>Mutta Kalakki</t>
+        </is>
+      </c>
+      <c r="D41" s="0" t="inlineStr">
+        <is>
+          <t>G. V. Prakash</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" s="0" t="inlineStr">
+        <is>
+          <t>2026-04-24</t>
+        </is>
+      </c>
+      <c r="B42" s="0" t="n">
+        <v>41</v>
+      </c>
+      <c r="C42" s="0" t="inlineStr">
+        <is>
+          <t>Haseen</t>
+        </is>
+      </c>
+      <c r="D42" s="0" t="inlineStr">
+        <is>
+          <t>Talwiinder</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" s="0" t="inlineStr">
+        <is>
+          <t>2026-04-24</t>
+        </is>
+      </c>
+      <c r="B43" s="0" t="n">
+        <v>42</v>
+      </c>
+      <c r="C43" s="0" t="inlineStr">
+        <is>
+          <t>Aaya Sher</t>
+        </is>
+      </c>
+      <c r="D43" s="0" t="inlineStr">
+        <is>
+          <t>Anirudh Ravichander</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" s="0" t="inlineStr">
+        <is>
+          <t>2026-04-24</t>
+        </is>
+      </c>
+      <c r="B44" s="0" t="n">
+        <v>43</v>
+      </c>
+      <c r="C44" s="0" t="inlineStr">
+        <is>
+          <t>Mast Magan</t>
+        </is>
+      </c>
+      <c r="D44" s="0" t="inlineStr">
+        <is>
+          <t>Arijit Singh</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" s="0" t="inlineStr">
+        <is>
+          <t>2026-04-24</t>
+        </is>
+      </c>
+      <c r="B45" s="0" t="n">
+        <v>44</v>
+      </c>
+      <c r="C45" s="0" t="inlineStr">
+        <is>
+          <t>Mann Mera - Original Version</t>
+        </is>
+      </c>
+      <c r="D45" s="0" t="inlineStr">
+        <is>
+          <t>Gajendra Verma</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" s="0" t="inlineStr">
+        <is>
+          <t>2026-04-24</t>
+        </is>
+      </c>
+      <c r="B46" s="0" t="n">
+        <v>45</v>
+      </c>
+      <c r="C46" s="0" t="inlineStr">
+        <is>
+          <t>High On You</t>
+        </is>
+      </c>
+      <c r="D46" s="0" t="inlineStr">
+        <is>
+          <t>Jind Universe</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" s="0" t="inlineStr">
+        <is>
+          <t>2026-04-24</t>
+        </is>
+      </c>
+      <c r="B47" s="0" t="n">
+        <v>46</v>
+      </c>
+      <c r="C47" s="0" t="inlineStr">
+        <is>
+          <t>Lutt Le Gaya</t>
+        </is>
+      </c>
+      <c r="D47" s="0" t="inlineStr">
+        <is>
+          <t>Shashwat Sachdev</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" s="0" t="inlineStr">
+        <is>
+          <t>2026-04-24</t>
+        </is>
+      </c>
+      <c r="B48" s="0" t="n">
+        <v>47</v>
+      </c>
+      <c r="C48" s="0" t="inlineStr">
+        <is>
+          <t>Jhol - Acoustic</t>
+        </is>
+      </c>
+      <c r="D48" s="0" t="inlineStr">
+        <is>
+          <t>Maanu</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" s="0" t="inlineStr">
+        <is>
+          <t>2026-04-24</t>
+        </is>
+      </c>
+      <c r="B49" s="0" t="n">
+        <v>48</v>
+      </c>
+      <c r="C49" s="0" t="inlineStr">
+        <is>
+          <t>Oorum Blood</t>
+        </is>
+      </c>
+      <c r="D49" s="0" t="inlineStr">
+        <is>
+          <t>Sai Abhyankkar</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" s="0" t="inlineStr">
+        <is>
+          <t>2026-04-24</t>
+        </is>
+      </c>
+      <c r="B50" s="0" t="n">
+        <v>49</v>
+      </c>
+      <c r="C50" s="0" t="inlineStr">
+        <is>
+          <t>Humsafar</t>
+        </is>
+      </c>
+      <c r="D50" s="0" t="inlineStr">
+        <is>
+          <t>Sachet-Parampara</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" s="0" t="inlineStr">
+        <is>
+          <t>2026-04-24</t>
+        </is>
+      </c>
+      <c r="B51" s="0" t="n">
+        <v>50</v>
+      </c>
+      <c r="C51" s="0" t="inlineStr">
+        <is>
+          <t>Thodi Si Daaru</t>
+        </is>
+      </c>
+      <c r="D51" s="0" t="inlineStr">
+        <is>
+          <t>AP Dhillon</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet44.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:D51"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="24" t="inlineStr">
+        <is>
+          <t>Date</t>
+        </is>
+      </c>
+      <c r="B1" s="24" t="inlineStr">
+        <is>
+          <t>Rank</t>
+        </is>
+      </c>
+      <c r="C1" s="24" t="inlineStr">
+        <is>
+          <t>Song</t>
+        </is>
+      </c>
+      <c r="D1" s="24" t="inlineStr">
+        <is>
+          <t>Artist</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>2026-04-22</t>
+          <t>2026-04-25</t>
         </is>
       </c>
       <c r="B2" t="n">
@@ -37830,7 +40941,7 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>2026-04-22</t>
+          <t>2026-04-25</t>
         </is>
       </c>
       <c r="B3" t="n">
@@ -37850,7 +40961,7 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>2026-04-22</t>
+          <t>2026-04-25</t>
         </is>
       </c>
       <c r="B4" t="n">
@@ -37870,7 +40981,7 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>2026-04-22</t>
+          <t>2026-04-25</t>
         </is>
       </c>
       <c r="B5" t="n">
@@ -37890,7 +41001,7 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>2026-04-22</t>
+          <t>2026-04-25</t>
         </is>
       </c>
       <c r="B6" t="n">
@@ -37910,7 +41021,7 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>2026-04-22</t>
+          <t>2026-04-25</t>
         </is>
       </c>
       <c r="B7" t="n">
@@ -37930,7 +41041,7 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>2026-04-22</t>
+          <t>2026-04-25</t>
         </is>
       </c>
       <c r="B8" t="n">
@@ -37950,7 +41061,7 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>2026-04-22</t>
+          <t>2026-04-25</t>
         </is>
       </c>
       <c r="B9" t="n">
@@ -37970,7 +41081,7 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>2026-04-22</t>
+          <t>2026-04-25</t>
         </is>
       </c>
       <c r="B10" t="n">
@@ -37990,7 +41101,7 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>2026-04-22</t>
+          <t>2026-04-25</t>
         </is>
       </c>
       <c r="B11" t="n">
@@ -37998,19 +41109,19 @@
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>Sitaare</t>
+          <t>Arz Kiya Hai | Coke Studio Bharat</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>Arijit Singh</t>
+          <t>Anuv Jain</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>2026-04-22</t>
+          <t>2026-04-25</t>
         </is>
       </c>
       <c r="B12" t="n">
@@ -38018,19 +41129,19 @@
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>Arz Kiya Hai | Coke Studio Bharat</t>
+          <t>Sitaare</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>Anuv Jain</t>
+          <t>Arijit Singh</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>2026-04-22</t>
+          <t>2026-04-25</t>
         </is>
       </c>
       <c r="B13" t="n">
@@ -38050,7 +41161,7 @@
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>2026-04-22</t>
+          <t>2026-04-25</t>
         </is>
       </c>
       <c r="B14" t="n">
@@ -38058,19 +41169,19 @@
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>Samjhawan</t>
+          <t>Apna Bana Le</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>Jawad Ahmad</t>
+          <t>Sachin-Jigar</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>2026-04-22</t>
+          <t>2026-04-25</t>
         </is>
       </c>
       <c r="B15" t="n">
@@ -38078,19 +41189,19 @@
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>Apna Bana Le</t>
+          <t>Samjhawan</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>Sachin-Jigar</t>
+          <t>Jawad Ahmad</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>2026-04-22</t>
+          <t>2026-04-25</t>
         </is>
       </c>
       <c r="B16" t="n">
@@ -38110,7 +41221,7 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>2026-04-22</t>
+          <t>2026-04-25</t>
         </is>
       </c>
       <c r="B17" t="n">
@@ -38118,19 +41229,19 @@
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>Boyfriend</t>
+          <t>Shararat</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>Karan Aujla</t>
+          <t>Shashwat Sachdev</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>2026-04-22</t>
+          <t>2026-04-25</t>
         </is>
       </c>
       <c r="B18" t="n">
@@ -38138,19 +41249,19 @@
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>Dhurandhar The Revenge - Aari Aari</t>
+          <t>Boyfriend</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>Shashwat Sachdev</t>
+          <t>Karan Aujla</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>2026-04-22</t>
+          <t>2026-04-25</t>
         </is>
       </c>
       <c r="B19" t="n">
@@ -38170,7 +41281,7 @@
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>2026-04-22</t>
+          <t>2026-04-25</t>
         </is>
       </c>
       <c r="B20" t="n">
@@ -38178,7 +41289,7 @@
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>Shararat</t>
+          <t>Dhurandhar The Revenge - Aari Aari</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
@@ -38190,7 +41301,7 @@
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>2026-04-22</t>
+          <t>2026-04-25</t>
         </is>
       </c>
       <c r="B21" t="n">
@@ -38210,7 +41321,7 @@
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>2026-04-22</t>
+          <t>2026-04-25</t>
         </is>
       </c>
       <c r="B22" t="n">
@@ -38230,7 +41341,7 @@
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>2026-04-22</t>
+          <t>2026-04-25</t>
         </is>
       </c>
       <c r="B23" t="n">
@@ -38250,7 +41361,7 @@
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>2026-04-22</t>
+          <t>2026-04-25</t>
         </is>
       </c>
       <c r="B24" t="n">
@@ -38270,7 +41381,7 @@
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>2026-04-22</t>
+          <t>2026-04-25</t>
         </is>
       </c>
       <c r="B25" t="n">
@@ -38290,7 +41401,7 @@
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>2026-04-22</t>
+          <t>2026-04-25</t>
         </is>
       </c>
       <c r="B26" t="n">
@@ -38298,19 +41409,19 @@
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>Ishqa Ve</t>
+          <t>Deewaana Deewaana</t>
         </is>
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>Zeeshan Ali</t>
+          <t>A.R. Rahman</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>2026-04-22</t>
+          <t>2026-04-25</t>
         </is>
       </c>
       <c r="B27" t="n">
@@ -38330,7 +41441,7 @@
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>2026-04-22</t>
+          <t>2026-04-25</t>
         </is>
       </c>
       <c r="B28" t="n">
@@ -38350,7 +41461,7 @@
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>2026-04-22</t>
+          <t>2026-04-25</t>
         </is>
       </c>
       <c r="B29" t="n">
@@ -38358,19 +41469,19 @@
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>Deewaana Deewaana</t>
+          <t>Ishqa Ve</t>
         </is>
       </c>
       <c r="D29" t="inlineStr">
         <is>
-          <t>A.R. Rahman</t>
+          <t>Zeeshan Ali</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>2026-04-22</t>
+          <t>2026-04-25</t>
         </is>
       </c>
       <c r="B30" t="n">
@@ -38378,19 +41489,19 @@
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>Ehsaas</t>
+          <t>Dhurandhar - Title Track</t>
         </is>
       </c>
       <c r="D30" t="inlineStr">
         <is>
-          <t>Faheem Abdullah</t>
+          <t>Shashwat Sachdev</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>2026-04-22</t>
+          <t>2026-04-25</t>
         </is>
       </c>
       <c r="B31" t="n">
@@ -38398,19 +41509,19 @@
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>Jo Tum Mere Ho</t>
+          <t>Agar Tum Saath Ho</t>
         </is>
       </c>
       <c r="D31" t="inlineStr">
         <is>
-          <t>Anuv Jain</t>
+          <t>Alka Yagnik</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>2026-04-22</t>
+          <t>2026-04-25</t>
         </is>
       </c>
       <c r="B32" t="n">
@@ -38418,19 +41529,19 @@
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>Dhurandhar - Title Track</t>
+          <t>Ehsaas</t>
         </is>
       </c>
       <c r="D32" t="inlineStr">
         <is>
-          <t>Shashwat Sachdev</t>
+          <t>Faheem Abdullah</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>2026-04-22</t>
+          <t>2026-04-25</t>
         </is>
       </c>
       <c r="B33" t="n">
@@ -38438,19 +41549,19 @@
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>Agar Tum Saath Ho</t>
+          <t>Jo Tum Mere Ho</t>
         </is>
       </c>
       <c r="D33" t="inlineStr">
         <is>
-          <t>Alka Yagnik</t>
+          <t>Anuv Jain</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>2026-04-22</t>
+          <t>2026-04-25</t>
         </is>
       </c>
       <c r="B34" t="n">
@@ -38458,19 +41569,19 @@
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>Naal Nachna</t>
+          <t>Tere Bina</t>
         </is>
       </c>
       <c r="D34" t="inlineStr">
         <is>
-          <t>Shashwat Sachdev</t>
+          <t>A.R. Rahman</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>2026-04-22</t>
+          <t>2026-04-25</t>
         </is>
       </c>
       <c r="B35" t="n">
@@ -38478,19 +41589,19 @@
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>Tere Bina</t>
+          <t>Ye Tune Kya Kiya</t>
         </is>
       </c>
       <c r="D35" t="inlineStr">
         <is>
-          <t>A.R. Rahman</t>
+          <t>Pritam</t>
         </is>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>2026-04-22</t>
+          <t>2026-04-25</t>
         </is>
       </c>
       <c r="B36" t="n">
@@ -38498,19 +41609,19 @@
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>Mutta Kalakki</t>
+          <t>Naal Nachna</t>
         </is>
       </c>
       <c r="D36" t="inlineStr">
         <is>
-          <t>G. V. Prakash</t>
+          <t>Shashwat Sachdev</t>
         </is>
       </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>2026-04-22</t>
+          <t>2026-04-25</t>
         </is>
       </c>
       <c r="B37" t="n">
@@ -38518,19 +41629,19 @@
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>Phir Se</t>
+          <t>Barbaad</t>
         </is>
       </c>
       <c r="D37" t="inlineStr">
         <is>
-          <t>Shashwat Sachdev</t>
+          <t>The Rish</t>
         </is>
       </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>2026-04-22</t>
+          <t>2026-04-25</t>
         </is>
       </c>
       <c r="B38" t="n">
@@ -38550,7 +41661,7 @@
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>2026-04-22</t>
+          <t>2026-04-25</t>
         </is>
       </c>
       <c r="B39" t="n">
@@ -38558,19 +41669,19 @@
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>Barbaad</t>
+          <t>Mutta Kalakki</t>
         </is>
       </c>
       <c r="D39" t="inlineStr">
         <is>
-          <t>The Rish</t>
+          <t>G. V. Prakash</t>
         </is>
       </c>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>2026-04-22</t>
+          <t>2026-04-25</t>
         </is>
       </c>
       <c r="B40" t="n">
@@ -38578,19 +41689,19 @@
       </c>
       <c r="C40" t="inlineStr">
         <is>
-          <t>Ye Tune Kya Kiya</t>
+          <t>Teri Deewani</t>
         </is>
       </c>
       <c r="D40" t="inlineStr">
         <is>
-          <t>Pritam</t>
+          <t>Kailash Kher</t>
         </is>
       </c>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>2026-04-22</t>
+          <t>2026-04-25</t>
         </is>
       </c>
       <c r="B41" t="n">
@@ -38598,19 +41709,19 @@
       </c>
       <c r="C41" t="inlineStr">
         <is>
-          <t>Teri Deewani</t>
+          <t>Phir Se</t>
         </is>
       </c>
       <c r="D41" t="inlineStr">
         <is>
-          <t>Kailash Kher</t>
+          <t>Shashwat Sachdev</t>
         </is>
       </c>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>2026-04-22</t>
+          <t>2026-04-25</t>
         </is>
       </c>
       <c r="B42" t="n">
@@ -38618,19 +41729,19 @@
       </c>
       <c r="C42" t="inlineStr">
         <is>
-          <t>Aaya Sher</t>
+          <t>Lutt Le Gaya</t>
         </is>
       </c>
       <c r="D42" t="inlineStr">
         <is>
-          <t>Anirudh Ravichander</t>
+          <t>Shashwat Sachdev</t>
         </is>
       </c>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>2026-04-22</t>
+          <t>2026-04-25</t>
         </is>
       </c>
       <c r="B43" t="n">
@@ -38638,19 +41749,19 @@
       </c>
       <c r="C43" t="inlineStr">
         <is>
-          <t>Haseen</t>
+          <t>Aaya Sher</t>
         </is>
       </c>
       <c r="D43" t="inlineStr">
         <is>
-          <t>Talwiinder</t>
+          <t>Anirudh Ravichander</t>
         </is>
       </c>
     </row>
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>2026-04-22</t>
+          <t>2026-04-25</t>
         </is>
       </c>
       <c r="B44" t="n">
@@ -38658,19 +41769,19 @@
       </c>
       <c r="C44" t="inlineStr">
         <is>
-          <t>Mann Mera - Original Version</t>
+          <t>Haseen</t>
         </is>
       </c>
       <c r="D44" t="inlineStr">
         <is>
-          <t>Gajendra Verma</t>
+          <t>Talwiinder</t>
         </is>
       </c>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>2026-04-22</t>
+          <t>2026-04-25</t>
         </is>
       </c>
       <c r="B45" t="n">
@@ -38678,19 +41789,19 @@
       </c>
       <c r="C45" t="inlineStr">
         <is>
-          <t>Mast Magan</t>
+          <t>High On You</t>
         </is>
       </c>
       <c r="D45" t="inlineStr">
         <is>
-          <t>Arijit Singh</t>
+          <t>Jind Universe</t>
         </is>
       </c>
     </row>
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>2026-04-22</t>
+          <t>2026-04-25</t>
         </is>
       </c>
       <c r="B46" t="n">
@@ -38698,19 +41809,19 @@
       </c>
       <c r="C46" t="inlineStr">
         <is>
-          <t>Oorum Blood</t>
+          <t>Mast Magan</t>
         </is>
       </c>
       <c r="D46" t="inlineStr">
         <is>
-          <t>Sai Abhyankkar</t>
+          <t>Arijit Singh</t>
         </is>
       </c>
     </row>
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>2026-04-22</t>
+          <t>2026-04-25</t>
         </is>
       </c>
       <c r="B47" t="n">
@@ -38718,19 +41829,19 @@
       </c>
       <c r="C47" t="inlineStr">
         <is>
-          <t>Jhol - Acoustic</t>
+          <t>Mann Mera - Original Version</t>
         </is>
       </c>
       <c r="D47" t="inlineStr">
         <is>
-          <t>Maanu</t>
+          <t>Gajendra Verma</t>
         </is>
       </c>
     </row>
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>2026-04-22</t>
+          <t>2026-04-25</t>
         </is>
       </c>
       <c r="B48" t="n">
@@ -38738,19 +41849,19 @@
       </c>
       <c r="C48" t="inlineStr">
         <is>
-          <t>Lutt Le Gaya</t>
+          <t>Oorum Blood</t>
         </is>
       </c>
       <c r="D48" t="inlineStr">
         <is>
-          <t>Shashwat Sachdev</t>
+          <t>Sai Abhyankkar</t>
         </is>
       </c>
     </row>
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>2026-04-22</t>
+          <t>2026-04-25</t>
         </is>
       </c>
       <c r="B49" t="n">
@@ -38758,19 +41869,19 @@
       </c>
       <c r="C49" t="inlineStr">
         <is>
-          <t>High On You</t>
+          <t>Jhol - Acoustic</t>
         </is>
       </c>
       <c r="D49" t="inlineStr">
         <is>
-          <t>Jind Universe</t>
+          <t>Maanu</t>
         </is>
       </c>
     </row>
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>2026-04-22</t>
+          <t>2026-04-25</t>
         </is>
       </c>
       <c r="B50" t="n">
@@ -38778,19 +41889,19 @@
       </c>
       <c r="C50" t="inlineStr">
         <is>
-          <t>Zaalima</t>
+          <t>Thodi Si Daaru</t>
         </is>
       </c>
       <c r="D50" t="inlineStr">
         <is>
-          <t>Arijit Singh</t>
+          <t>AP Dhillon</t>
         </is>
       </c>
     </row>
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>2026-04-22</t>
+          <t>2026-04-25</t>
         </is>
       </c>
       <c r="B51" t="n">
@@ -38798,12 +41909,12 @@
       </c>
       <c r="C51" t="inlineStr">
         <is>
-          <t>Raabta</t>
+          <t>Zaalima</t>
         </is>
       </c>
       <c r="D51" t="inlineStr">
         <is>
-          <t>Pritam</t>
+          <t>Arijit Singh</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
add all data till 28th april and got predictions for 29th april
</commit_message>
<xml_diff>
--- a/Probability Project.xlsx
+++ b/Probability Project.xlsx
@@ -47,6 +47,8 @@
     <sheet name="AUTO_20260426" sheetId="42" state="visible" r:id="rId42"/>
     <sheet name="AUTO_20260424" sheetId="43" state="visible" r:id="rId43"/>
     <sheet name="AUTO_20260425" sheetId="44" state="visible" r:id="rId44"/>
+    <sheet name="AUTO_20260428" sheetId="45" state="visible" r:id="rId45"/>
+    <sheet name="AUTO_20260427" sheetId="46" state="visible" r:id="rId46"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -40919,9 +40921,2081 @@
       </c>
     </row>
     <row r="2">
+      <c r="A2" s="0" t="inlineStr">
+        <is>
+          <t>2026-04-25</t>
+        </is>
+      </c>
+      <c r="B2" s="0" t="n">
+        <v>1</v>
+      </c>
+      <c r="C2" s="0" t="inlineStr">
+        <is>
+          <t>Bairan</t>
+        </is>
+      </c>
+      <c r="D2" s="0" t="inlineStr">
+        <is>
+          <t>Banjaare</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="0" t="inlineStr">
+        <is>
+          <t>2026-04-25</t>
+        </is>
+      </c>
+      <c r="B3" s="0" t="n">
+        <v>2</v>
+      </c>
+      <c r="C3" s="0" t="inlineStr">
+        <is>
+          <t>Gehra Hua</t>
+        </is>
+      </c>
+      <c r="D3" s="0" t="inlineStr">
+        <is>
+          <t>Shashwat Sachdev</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="0" t="inlineStr">
+        <is>
+          <t>2026-04-25</t>
+        </is>
+      </c>
+      <c r="B4" s="0" t="n">
+        <v>3</v>
+      </c>
+      <c r="C4" s="0" t="inlineStr">
+        <is>
+          <t>Majboor</t>
+        </is>
+      </c>
+      <c r="D4" s="0" t="inlineStr">
+        <is>
+          <t>Sheheryar Rehan</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="0" t="inlineStr">
+        <is>
+          <t>2026-04-25</t>
+        </is>
+      </c>
+      <c r="B5" s="0" t="n">
+        <v>4</v>
+      </c>
+      <c r="C5" s="0" t="inlineStr">
+        <is>
+          <t>Khat</t>
+        </is>
+      </c>
+      <c r="D5" s="0" t="inlineStr">
+        <is>
+          <t>Navjot Ahuja</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="0" t="inlineStr">
+        <is>
+          <t>2026-04-25</t>
+        </is>
+      </c>
+      <c r="B6" s="0" t="n">
+        <v>5</v>
+      </c>
+      <c r="C6" s="0" t="inlineStr">
+        <is>
+          <t>Sheesha - Aakhya Mai Aakh Ghali Jo Bairan</t>
+        </is>
+      </c>
+      <c r="D6" s="0" t="inlineStr">
+        <is>
+          <t>Mitta Ror</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="0" t="inlineStr">
+        <is>
+          <t>2026-04-25</t>
+        </is>
+      </c>
+      <c r="B7" s="0" t="n">
+        <v>6</v>
+      </c>
+      <c r="C7" s="0" t="inlineStr">
+        <is>
+          <t>Jaiye Sajana</t>
+        </is>
+      </c>
+      <c r="D7" s="0" t="inlineStr">
+        <is>
+          <t>Shashwat Sachdev</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="0" t="inlineStr">
+        <is>
+          <t>2026-04-25</t>
+        </is>
+      </c>
+      <c r="B8" s="0" t="n">
+        <v>7</v>
+      </c>
+      <c r="C8" s="0" t="inlineStr">
+        <is>
+          <t>Pavazha Malli</t>
+        </is>
+      </c>
+      <c r="D8" s="0" t="inlineStr">
+        <is>
+          <t>Sai Abhyankkar</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="0" t="inlineStr">
+        <is>
+          <t>2026-04-25</t>
+        </is>
+      </c>
+      <c r="B9" s="0" t="n">
+        <v>8</v>
+      </c>
+      <c r="C9" s="0" t="inlineStr">
+        <is>
+          <t>Finding Her</t>
+        </is>
+      </c>
+      <c r="D9" s="0" t="inlineStr">
+        <is>
+          <t>Kushagra</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="0" t="inlineStr">
+        <is>
+          <t>2026-04-25</t>
+        </is>
+      </c>
+      <c r="B10" s="0" t="n">
+        <v>9</v>
+      </c>
+      <c r="C10" s="0" t="inlineStr">
+        <is>
+          <t>Sahiba</t>
+        </is>
+      </c>
+      <c r="D10" s="0" t="inlineStr">
+        <is>
+          <t>Aditya Rikhari</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="0" t="inlineStr">
+        <is>
+          <t>2026-04-25</t>
+        </is>
+      </c>
+      <c r="B11" s="0" t="n">
+        <v>10</v>
+      </c>
+      <c r="C11" s="0" t="inlineStr">
+        <is>
+          <t>Arz Kiya Hai | Coke Studio Bharat</t>
+        </is>
+      </c>
+      <c r="D11" s="0" t="inlineStr">
+        <is>
+          <t>Anuv Jain</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="0" t="inlineStr">
+        <is>
+          <t>2026-04-25</t>
+        </is>
+      </c>
+      <c r="B12" s="0" t="n">
+        <v>11</v>
+      </c>
+      <c r="C12" s="0" t="inlineStr">
+        <is>
+          <t>Sitaare</t>
+        </is>
+      </c>
+      <c r="D12" s="0" t="inlineStr">
+        <is>
+          <t>Arijit Singh</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="0" t="inlineStr">
+        <is>
+          <t>2026-04-25</t>
+        </is>
+      </c>
+      <c r="B13" s="0" t="n">
+        <v>12</v>
+      </c>
+      <c r="C13" s="0" t="inlineStr">
+        <is>
+          <t>Dooron Dooron</t>
+        </is>
+      </c>
+      <c r="D13" s="0" t="inlineStr">
+        <is>
+          <t>Paresh Pahuja</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="0" t="inlineStr">
+        <is>
+          <t>2026-04-25</t>
+        </is>
+      </c>
+      <c r="B14" s="0" t="n">
+        <v>13</v>
+      </c>
+      <c r="C14" s="0" t="inlineStr">
+        <is>
+          <t>Apna Bana Le</t>
+        </is>
+      </c>
+      <c r="D14" s="0" t="inlineStr">
+        <is>
+          <t>Sachin-Jigar</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="0" t="inlineStr">
+        <is>
+          <t>2026-04-25</t>
+        </is>
+      </c>
+      <c r="B15" s="0" t="n">
+        <v>14</v>
+      </c>
+      <c r="C15" s="0" t="inlineStr">
+        <is>
+          <t>Samjhawan</t>
+        </is>
+      </c>
+      <c r="D15" s="0" t="inlineStr">
+        <is>
+          <t>Jawad Ahmad</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="0" t="inlineStr">
+        <is>
+          <t>2026-04-25</t>
+        </is>
+      </c>
+      <c r="B16" s="0" t="n">
+        <v>15</v>
+      </c>
+      <c r="C16" s="0" t="inlineStr">
+        <is>
+          <t>Mann Mera</t>
+        </is>
+      </c>
+      <c r="D16" s="0" t="inlineStr">
+        <is>
+          <t>Gajendra Verma</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="0" t="inlineStr">
+        <is>
+          <t>2026-04-25</t>
+        </is>
+      </c>
+      <c r="B17" s="0" t="n">
+        <v>16</v>
+      </c>
+      <c r="C17" s="0" t="inlineStr">
+        <is>
+          <t>Shararat</t>
+        </is>
+      </c>
+      <c r="D17" s="0" t="inlineStr">
+        <is>
+          <t>Shashwat Sachdev</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="0" t="inlineStr">
+        <is>
+          <t>2026-04-25</t>
+        </is>
+      </c>
+      <c r="B18" s="0" t="n">
+        <v>17</v>
+      </c>
+      <c r="C18" s="0" t="inlineStr">
+        <is>
+          <t>Boyfriend</t>
+        </is>
+      </c>
+      <c r="D18" s="0" t="inlineStr">
+        <is>
+          <t>Karan Aujla</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="0" t="inlineStr">
+        <is>
+          <t>2026-04-25</t>
+        </is>
+      </c>
+      <c r="B19" s="0" t="n">
+        <v>18</v>
+      </c>
+      <c r="C19" s="0" t="inlineStr">
+        <is>
+          <t>Ishq</t>
+        </is>
+      </c>
+      <c r="D19" s="0" t="inlineStr">
+        <is>
+          <t>Faheem Abdullah</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="0" t="inlineStr">
+        <is>
+          <t>2026-04-25</t>
+        </is>
+      </c>
+      <c r="B20" s="0" t="n">
+        <v>19</v>
+      </c>
+      <c r="C20" s="0" t="inlineStr">
+        <is>
+          <t>Dhurandhar The Revenge - Aari Aari</t>
+        </is>
+      </c>
+      <c r="D20" s="0" t="inlineStr">
+        <is>
+          <t>Shashwat Sachdev</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="0" t="inlineStr">
+        <is>
+          <t>2026-04-25</t>
+        </is>
+      </c>
+      <c r="B21" s="0" t="n">
+        <v>20</v>
+      </c>
+      <c r="C21" s="0" t="inlineStr">
+        <is>
+          <t>Tum Ho Toh</t>
+        </is>
+      </c>
+      <c r="D21" s="0" t="inlineStr">
+        <is>
+          <t>Vishal Mishra</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="0" t="inlineStr">
+        <is>
+          <t>2026-04-25</t>
+        </is>
+      </c>
+      <c r="B22" s="0" t="n">
+        <v>21</v>
+      </c>
+      <c r="C22" s="0" t="inlineStr">
+        <is>
+          <t>Saiyaara</t>
+        </is>
+      </c>
+      <c r="D22" s="0" t="inlineStr">
+        <is>
+          <t>Tanishk Bagchi</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="0" t="inlineStr">
+        <is>
+          <t>2026-04-25</t>
+        </is>
+      </c>
+      <c r="B23" s="0" t="n">
+        <v>22</v>
+      </c>
+      <c r="C23" s="0" t="inlineStr">
+        <is>
+          <t>Jaan Se Guzarte Hain</t>
+        </is>
+      </c>
+      <c r="D23" s="0" t="inlineStr">
+        <is>
+          <t>Shashwat Sachdev</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="0" t="inlineStr">
+        <is>
+          <t>2026-04-25</t>
+        </is>
+      </c>
+      <c r="B24" s="0" t="n">
+        <v>23</v>
+      </c>
+      <c r="C24" s="0" t="inlineStr">
+        <is>
+          <t>Raanjhan</t>
+        </is>
+      </c>
+      <c r="D24" s="0" t="inlineStr">
+        <is>
+          <t>Sachet-Parampara</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="0" t="inlineStr">
+        <is>
+          <t>2026-04-25</t>
+        </is>
+      </c>
+      <c r="B25" s="0" t="n">
+        <v>24</v>
+      </c>
+      <c r="C25" s="0" t="inlineStr">
+        <is>
+          <t>Darkhaast</t>
+        </is>
+      </c>
+      <c r="D25" s="0" t="inlineStr">
+        <is>
+          <t>Mithoon</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="0" t="inlineStr">
+        <is>
+          <t>2026-04-25</t>
+        </is>
+      </c>
+      <c r="B26" s="0" t="n">
+        <v>25</v>
+      </c>
+      <c r="C26" s="0" t="inlineStr">
+        <is>
+          <t>Deewaana Deewaana</t>
+        </is>
+      </c>
+      <c r="D26" s="0" t="inlineStr">
+        <is>
+          <t>A.R. Rahman</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="0" t="inlineStr">
+        <is>
+          <t>2026-04-25</t>
+        </is>
+      </c>
+      <c r="B27" s="0" t="n">
+        <v>26</v>
+      </c>
+      <c r="C27" s="0" t="inlineStr">
+        <is>
+          <t>For A Reason</t>
+        </is>
+      </c>
+      <c r="D27" s="0" t="inlineStr">
+        <is>
+          <t>Karan Aujla</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="0" t="inlineStr">
+        <is>
+          <t>2026-04-25</t>
+        </is>
+      </c>
+      <c r="B28" s="0" t="n">
+        <v>27</v>
+      </c>
+      <c r="C28" s="0" t="inlineStr">
+        <is>
+          <t>Tere Liye</t>
+        </is>
+      </c>
+      <c r="D28" s="0" t="inlineStr">
+        <is>
+          <t>Atif Aslam</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="0" t="inlineStr">
+        <is>
+          <t>2026-04-25</t>
+        </is>
+      </c>
+      <c r="B29" s="0" t="n">
+        <v>28</v>
+      </c>
+      <c r="C29" s="0" t="inlineStr">
+        <is>
+          <t>Ishqa Ve</t>
+        </is>
+      </c>
+      <c r="D29" s="0" t="inlineStr">
+        <is>
+          <t>Zeeshan Ali</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="0" t="inlineStr">
+        <is>
+          <t>2026-04-25</t>
+        </is>
+      </c>
+      <c r="B30" s="0" t="n">
+        <v>29</v>
+      </c>
+      <c r="C30" s="0" t="inlineStr">
+        <is>
+          <t>Dhurandhar - Title Track</t>
+        </is>
+      </c>
+      <c r="D30" s="0" t="inlineStr">
+        <is>
+          <t>Shashwat Sachdev</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="0" t="inlineStr">
+        <is>
+          <t>2026-04-25</t>
+        </is>
+      </c>
+      <c r="B31" s="0" t="n">
+        <v>30</v>
+      </c>
+      <c r="C31" s="0" t="inlineStr">
+        <is>
+          <t>Agar Tum Saath Ho</t>
+        </is>
+      </c>
+      <c r="D31" s="0" t="inlineStr">
+        <is>
+          <t>Alka Yagnik</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="0" t="inlineStr">
+        <is>
+          <t>2026-04-25</t>
+        </is>
+      </c>
+      <c r="B32" s="0" t="n">
+        <v>31</v>
+      </c>
+      <c r="C32" s="0" t="inlineStr">
+        <is>
+          <t>Ehsaas</t>
+        </is>
+      </c>
+      <c r="D32" s="0" t="inlineStr">
+        <is>
+          <t>Faheem Abdullah</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="0" t="inlineStr">
+        <is>
+          <t>2026-04-25</t>
+        </is>
+      </c>
+      <c r="B33" s="0" t="n">
+        <v>32</v>
+      </c>
+      <c r="C33" s="0" t="inlineStr">
+        <is>
+          <t>Jo Tum Mere Ho</t>
+        </is>
+      </c>
+      <c r="D33" s="0" t="inlineStr">
+        <is>
+          <t>Anuv Jain</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="0" t="inlineStr">
+        <is>
+          <t>2026-04-25</t>
+        </is>
+      </c>
+      <c r="B34" s="0" t="n">
+        <v>33</v>
+      </c>
+      <c r="C34" s="0" t="inlineStr">
+        <is>
+          <t>Tere Bina</t>
+        </is>
+      </c>
+      <c r="D34" s="0" t="inlineStr">
+        <is>
+          <t>A.R. Rahman</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="0" t="inlineStr">
+        <is>
+          <t>2026-04-25</t>
+        </is>
+      </c>
+      <c r="B35" s="0" t="n">
+        <v>34</v>
+      </c>
+      <c r="C35" s="0" t="inlineStr">
+        <is>
+          <t>Ye Tune Kya Kiya</t>
+        </is>
+      </c>
+      <c r="D35" s="0" t="inlineStr">
+        <is>
+          <t>Pritam</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="0" t="inlineStr">
+        <is>
+          <t>2026-04-25</t>
+        </is>
+      </c>
+      <c r="B36" s="0" t="n">
+        <v>35</v>
+      </c>
+      <c r="C36" s="0" t="inlineStr">
+        <is>
+          <t>Naal Nachna</t>
+        </is>
+      </c>
+      <c r="D36" s="0" t="inlineStr">
+        <is>
+          <t>Shashwat Sachdev</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="0" t="inlineStr">
+        <is>
+          <t>2026-04-25</t>
+        </is>
+      </c>
+      <c r="B37" s="0" t="n">
+        <v>36</v>
+      </c>
+      <c r="C37" s="0" t="inlineStr">
+        <is>
+          <t>Barbaad</t>
+        </is>
+      </c>
+      <c r="D37" s="0" t="inlineStr">
+        <is>
+          <t>The Rish</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="0" t="inlineStr">
+        <is>
+          <t>2026-04-25</t>
+        </is>
+      </c>
+      <c r="B38" s="0" t="n">
+        <v>37</v>
+      </c>
+      <c r="C38" s="0" t="inlineStr">
+        <is>
+          <t>Bairi</t>
+        </is>
+      </c>
+      <c r="D38" s="0" t="inlineStr">
+        <is>
+          <t>Virat</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="0" t="inlineStr">
+        <is>
+          <t>2026-04-25</t>
+        </is>
+      </c>
+      <c r="B39" s="0" t="n">
+        <v>38</v>
+      </c>
+      <c r="C39" s="0" t="inlineStr">
+        <is>
+          <t>Mutta Kalakki</t>
+        </is>
+      </c>
+      <c r="D39" s="0" t="inlineStr">
+        <is>
+          <t>G. V. Prakash</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="0" t="inlineStr">
+        <is>
+          <t>2026-04-25</t>
+        </is>
+      </c>
+      <c r="B40" s="0" t="n">
+        <v>39</v>
+      </c>
+      <c r="C40" s="0" t="inlineStr">
+        <is>
+          <t>Teri Deewani</t>
+        </is>
+      </c>
+      <c r="D40" s="0" t="inlineStr">
+        <is>
+          <t>Kailash Kher</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" s="0" t="inlineStr">
+        <is>
+          <t>2026-04-25</t>
+        </is>
+      </c>
+      <c r="B41" s="0" t="n">
+        <v>40</v>
+      </c>
+      <c r="C41" s="0" t="inlineStr">
+        <is>
+          <t>Phir Se</t>
+        </is>
+      </c>
+      <c r="D41" s="0" t="inlineStr">
+        <is>
+          <t>Shashwat Sachdev</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" s="0" t="inlineStr">
+        <is>
+          <t>2026-04-25</t>
+        </is>
+      </c>
+      <c r="B42" s="0" t="n">
+        <v>41</v>
+      </c>
+      <c r="C42" s="0" t="inlineStr">
+        <is>
+          <t>Lutt Le Gaya</t>
+        </is>
+      </c>
+      <c r="D42" s="0" t="inlineStr">
+        <is>
+          <t>Shashwat Sachdev</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" s="0" t="inlineStr">
+        <is>
+          <t>2026-04-25</t>
+        </is>
+      </c>
+      <c r="B43" s="0" t="n">
+        <v>42</v>
+      </c>
+      <c r="C43" s="0" t="inlineStr">
+        <is>
+          <t>Aaya Sher</t>
+        </is>
+      </c>
+      <c r="D43" s="0" t="inlineStr">
+        <is>
+          <t>Anirudh Ravichander</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" s="0" t="inlineStr">
+        <is>
+          <t>2026-04-25</t>
+        </is>
+      </c>
+      <c r="B44" s="0" t="n">
+        <v>43</v>
+      </c>
+      <c r="C44" s="0" t="inlineStr">
+        <is>
+          <t>Haseen</t>
+        </is>
+      </c>
+      <c r="D44" s="0" t="inlineStr">
+        <is>
+          <t>Talwiinder</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" s="0" t="inlineStr">
+        <is>
+          <t>2026-04-25</t>
+        </is>
+      </c>
+      <c r="B45" s="0" t="n">
+        <v>44</v>
+      </c>
+      <c r="C45" s="0" t="inlineStr">
+        <is>
+          <t>High On You</t>
+        </is>
+      </c>
+      <c r="D45" s="0" t="inlineStr">
+        <is>
+          <t>Jind Universe</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" s="0" t="inlineStr">
+        <is>
+          <t>2026-04-25</t>
+        </is>
+      </c>
+      <c r="B46" s="0" t="n">
+        <v>45</v>
+      </c>
+      <c r="C46" s="0" t="inlineStr">
+        <is>
+          <t>Mast Magan</t>
+        </is>
+      </c>
+      <c r="D46" s="0" t="inlineStr">
+        <is>
+          <t>Arijit Singh</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" s="0" t="inlineStr">
+        <is>
+          <t>2026-04-25</t>
+        </is>
+      </c>
+      <c r="B47" s="0" t="n">
+        <v>46</v>
+      </c>
+      <c r="C47" s="0" t="inlineStr">
+        <is>
+          <t>Mann Mera - Original Version</t>
+        </is>
+      </c>
+      <c r="D47" s="0" t="inlineStr">
+        <is>
+          <t>Gajendra Verma</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" s="0" t="inlineStr">
+        <is>
+          <t>2026-04-25</t>
+        </is>
+      </c>
+      <c r="B48" s="0" t="n">
+        <v>47</v>
+      </c>
+      <c r="C48" s="0" t="inlineStr">
+        <is>
+          <t>Oorum Blood</t>
+        </is>
+      </c>
+      <c r="D48" s="0" t="inlineStr">
+        <is>
+          <t>Sai Abhyankkar</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" s="0" t="inlineStr">
+        <is>
+          <t>2026-04-25</t>
+        </is>
+      </c>
+      <c r="B49" s="0" t="n">
+        <v>48</v>
+      </c>
+      <c r="C49" s="0" t="inlineStr">
+        <is>
+          <t>Jhol - Acoustic</t>
+        </is>
+      </c>
+      <c r="D49" s="0" t="inlineStr">
+        <is>
+          <t>Maanu</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" s="0" t="inlineStr">
+        <is>
+          <t>2026-04-25</t>
+        </is>
+      </c>
+      <c r="B50" s="0" t="n">
+        <v>49</v>
+      </c>
+      <c r="C50" s="0" t="inlineStr">
+        <is>
+          <t>Thodi Si Daaru</t>
+        </is>
+      </c>
+      <c r="D50" s="0" t="inlineStr">
+        <is>
+          <t>AP Dhillon</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" s="0" t="inlineStr">
+        <is>
+          <t>2026-04-25</t>
+        </is>
+      </c>
+      <c r="B51" s="0" t="n">
+        <v>50</v>
+      </c>
+      <c r="C51" s="0" t="inlineStr">
+        <is>
+          <t>Zaalima</t>
+        </is>
+      </c>
+      <c r="D51" s="0" t="inlineStr">
+        <is>
+          <t>Arijit Singh</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet45.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:D51"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="24" t="inlineStr">
+        <is>
+          <t>Date</t>
+        </is>
+      </c>
+      <c r="B1" s="24" t="inlineStr">
+        <is>
+          <t>Rank</t>
+        </is>
+      </c>
+      <c r="C1" s="24" t="inlineStr">
+        <is>
+          <t>Song</t>
+        </is>
+      </c>
+      <c r="D1" s="24" t="inlineStr">
+        <is>
+          <t>Artist</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="0" t="inlineStr">
+        <is>
+          <t>2026-04-28</t>
+        </is>
+      </c>
+      <c r="B2" s="0" t="n">
+        <v>1</v>
+      </c>
+      <c r="C2" s="0" t="inlineStr">
+        <is>
+          <t>Bairan</t>
+        </is>
+      </c>
+      <c r="D2" s="0" t="inlineStr">
+        <is>
+          <t>Banjaare</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="0" t="inlineStr">
+        <is>
+          <t>2026-04-28</t>
+        </is>
+      </c>
+      <c r="B3" s="0" t="n">
+        <v>2</v>
+      </c>
+      <c r="C3" s="0" t="inlineStr">
+        <is>
+          <t>Gehra Hua</t>
+        </is>
+      </c>
+      <c r="D3" s="0" t="inlineStr">
+        <is>
+          <t>Shashwat Sachdev</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="0" t="inlineStr">
+        <is>
+          <t>2026-04-28</t>
+        </is>
+      </c>
+      <c r="B4" s="0" t="n">
+        <v>3</v>
+      </c>
+      <c r="C4" s="0" t="inlineStr">
+        <is>
+          <t>Majboor</t>
+        </is>
+      </c>
+      <c r="D4" s="0" t="inlineStr">
+        <is>
+          <t>Sheheryar Rehan</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="0" t="inlineStr">
+        <is>
+          <t>2026-04-28</t>
+        </is>
+      </c>
+      <c r="B5" s="0" t="n">
+        <v>4</v>
+      </c>
+      <c r="C5" s="0" t="inlineStr">
+        <is>
+          <t>Khat</t>
+        </is>
+      </c>
+      <c r="D5" s="0" t="inlineStr">
+        <is>
+          <t>Navjot Ahuja</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="0" t="inlineStr">
+        <is>
+          <t>2026-04-28</t>
+        </is>
+      </c>
+      <c r="B6" s="0" t="n">
+        <v>5</v>
+      </c>
+      <c r="C6" s="0" t="inlineStr">
+        <is>
+          <t>Jaiye Sajana</t>
+        </is>
+      </c>
+      <c r="D6" s="0" t="inlineStr">
+        <is>
+          <t>Shashwat Sachdev</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="0" t="inlineStr">
+        <is>
+          <t>2026-04-28</t>
+        </is>
+      </c>
+      <c r="B7" s="0" t="n">
+        <v>6</v>
+      </c>
+      <c r="C7" s="0" t="inlineStr">
+        <is>
+          <t>Sheesha - Aakhya Mai Aakh Ghali Jo Bairan</t>
+        </is>
+      </c>
+      <c r="D7" s="0" t="inlineStr">
+        <is>
+          <t>Mitta Ror</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="0" t="inlineStr">
+        <is>
+          <t>2026-04-28</t>
+        </is>
+      </c>
+      <c r="B8" s="0" t="n">
+        <v>7</v>
+      </c>
+      <c r="C8" s="0" t="inlineStr">
+        <is>
+          <t>Finding Her</t>
+        </is>
+      </c>
+      <c r="D8" s="0" t="inlineStr">
+        <is>
+          <t>Kushagra</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="0" t="inlineStr">
+        <is>
+          <t>2026-04-28</t>
+        </is>
+      </c>
+      <c r="B9" s="0" t="n">
+        <v>8</v>
+      </c>
+      <c r="C9" s="0" t="inlineStr">
+        <is>
+          <t>Pavazha Malli</t>
+        </is>
+      </c>
+      <c r="D9" s="0" t="inlineStr">
+        <is>
+          <t>Sai Abhyankkar</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="0" t="inlineStr">
+        <is>
+          <t>2026-04-28</t>
+        </is>
+      </c>
+      <c r="B10" s="0" t="n">
+        <v>9</v>
+      </c>
+      <c r="C10" s="0" t="inlineStr">
+        <is>
+          <t>Sahiba</t>
+        </is>
+      </c>
+      <c r="D10" s="0" t="inlineStr">
+        <is>
+          <t>Aditya Rikhari</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="0" t="inlineStr">
+        <is>
+          <t>2026-04-28</t>
+        </is>
+      </c>
+      <c r="B11" s="0" t="n">
+        <v>10</v>
+      </c>
+      <c r="C11" s="0" t="inlineStr">
+        <is>
+          <t>Sitaare</t>
+        </is>
+      </c>
+      <c r="D11" s="0" t="inlineStr">
+        <is>
+          <t>Arijit Singh</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="0" t="inlineStr">
+        <is>
+          <t>2026-04-28</t>
+        </is>
+      </c>
+      <c r="B12" s="0" t="n">
+        <v>11</v>
+      </c>
+      <c r="C12" s="0" t="inlineStr">
+        <is>
+          <t>Arz Kiya Hai | Coke Studio Bharat</t>
+        </is>
+      </c>
+      <c r="D12" s="0" t="inlineStr">
+        <is>
+          <t>Anuv Jain</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="0" t="inlineStr">
+        <is>
+          <t>2026-04-28</t>
+        </is>
+      </c>
+      <c r="B13" s="0" t="n">
+        <v>12</v>
+      </c>
+      <c r="C13" s="0" t="inlineStr">
+        <is>
+          <t>Apna Bana Le</t>
+        </is>
+      </c>
+      <c r="D13" s="0" t="inlineStr">
+        <is>
+          <t>Sachin-Jigar</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="0" t="inlineStr">
+        <is>
+          <t>2026-04-28</t>
+        </is>
+      </c>
+      <c r="B14" s="0" t="n">
+        <v>13</v>
+      </c>
+      <c r="C14" s="0" t="inlineStr">
+        <is>
+          <t>Dooron Dooron</t>
+        </is>
+      </c>
+      <c r="D14" s="0" t="inlineStr">
+        <is>
+          <t>Paresh Pahuja</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="0" t="inlineStr">
+        <is>
+          <t>2026-04-28</t>
+        </is>
+      </c>
+      <c r="B15" s="0" t="n">
+        <v>14</v>
+      </c>
+      <c r="C15" s="0" t="inlineStr">
+        <is>
+          <t>Samjhawan</t>
+        </is>
+      </c>
+      <c r="D15" s="0" t="inlineStr">
+        <is>
+          <t>Jawad Ahmad</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="0" t="inlineStr">
+        <is>
+          <t>2026-04-28</t>
+        </is>
+      </c>
+      <c r="B16" s="0" t="n">
+        <v>15</v>
+      </c>
+      <c r="C16" s="0" t="inlineStr">
+        <is>
+          <t>Mann Mera</t>
+        </is>
+      </c>
+      <c r="D16" s="0" t="inlineStr">
+        <is>
+          <t>Gajendra Verma</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="0" t="inlineStr">
+        <is>
+          <t>2026-04-28</t>
+        </is>
+      </c>
+      <c r="B17" s="0" t="n">
+        <v>16</v>
+      </c>
+      <c r="C17" s="0" t="inlineStr">
+        <is>
+          <t>Ishq</t>
+        </is>
+      </c>
+      <c r="D17" s="0" t="inlineStr">
+        <is>
+          <t>Faheem Abdullah</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="0" t="inlineStr">
+        <is>
+          <t>2026-04-28</t>
+        </is>
+      </c>
+      <c r="B18" s="0" t="n">
+        <v>17</v>
+      </c>
+      <c r="C18" s="0" t="inlineStr">
+        <is>
+          <t>Tum Ho Toh</t>
+        </is>
+      </c>
+      <c r="D18" s="0" t="inlineStr">
+        <is>
+          <t>Vishal Mishra</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="0" t="inlineStr">
+        <is>
+          <t>2026-04-28</t>
+        </is>
+      </c>
+      <c r="B19" s="0" t="n">
+        <v>18</v>
+      </c>
+      <c r="C19" s="0" t="inlineStr">
+        <is>
+          <t>Boyfriend</t>
+        </is>
+      </c>
+      <c r="D19" s="0" t="inlineStr">
+        <is>
+          <t>Karan Aujla</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="0" t="inlineStr">
+        <is>
+          <t>2026-04-28</t>
+        </is>
+      </c>
+      <c r="B20" s="0" t="n">
+        <v>19</v>
+      </c>
+      <c r="C20" s="0" t="inlineStr">
+        <is>
+          <t>Shararat</t>
+        </is>
+      </c>
+      <c r="D20" s="0" t="inlineStr">
+        <is>
+          <t>Shashwat Sachdev</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="0" t="inlineStr">
+        <is>
+          <t>2026-04-28</t>
+        </is>
+      </c>
+      <c r="B21" s="0" t="n">
+        <v>20</v>
+      </c>
+      <c r="C21" s="0" t="inlineStr">
+        <is>
+          <t>Deewaana Deewaana</t>
+        </is>
+      </c>
+      <c r="D21" s="0" t="inlineStr">
+        <is>
+          <t>A.R. Rahman</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="0" t="inlineStr">
+        <is>
+          <t>2026-04-28</t>
+        </is>
+      </c>
+      <c r="B22" s="0" t="n">
+        <v>21</v>
+      </c>
+      <c r="C22" s="0" t="inlineStr">
+        <is>
+          <t>Darkhaast</t>
+        </is>
+      </c>
+      <c r="D22" s="0" t="inlineStr">
+        <is>
+          <t>Mithoon</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="0" t="inlineStr">
+        <is>
+          <t>2026-04-28</t>
+        </is>
+      </c>
+      <c r="B23" s="0" t="n">
+        <v>22</v>
+      </c>
+      <c r="C23" s="0" t="inlineStr">
+        <is>
+          <t>Dhurandhar The Revenge - Aari Aari</t>
+        </is>
+      </c>
+      <c r="D23" s="0" t="inlineStr">
+        <is>
+          <t>Shashwat Sachdev</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="0" t="inlineStr">
+        <is>
+          <t>2026-04-28</t>
+        </is>
+      </c>
+      <c r="B24" s="0" t="n">
+        <v>23</v>
+      </c>
+      <c r="C24" s="0" t="inlineStr">
+        <is>
+          <t>Saiyaara</t>
+        </is>
+      </c>
+      <c r="D24" s="0" t="inlineStr">
+        <is>
+          <t>Tanishk Bagchi</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="0" t="inlineStr">
+        <is>
+          <t>2026-04-28</t>
+        </is>
+      </c>
+      <c r="B25" s="0" t="n">
+        <v>24</v>
+      </c>
+      <c r="C25" s="0" t="inlineStr">
+        <is>
+          <t>Tere Liye</t>
+        </is>
+      </c>
+      <c r="D25" s="0" t="inlineStr">
+        <is>
+          <t>Atif Aslam</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="0" t="inlineStr">
+        <is>
+          <t>2026-04-28</t>
+        </is>
+      </c>
+      <c r="B26" s="0" t="n">
+        <v>25</v>
+      </c>
+      <c r="C26" s="0" t="inlineStr">
+        <is>
+          <t>Jo Tum Mere Ho</t>
+        </is>
+      </c>
+      <c r="D26" s="0" t="inlineStr">
+        <is>
+          <t>Anuv Jain</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="0" t="inlineStr">
+        <is>
+          <t>2026-04-28</t>
+        </is>
+      </c>
+      <c r="B27" s="0" t="n">
+        <v>26</v>
+      </c>
+      <c r="C27" s="0" t="inlineStr">
+        <is>
+          <t>Jaan Se Guzarte Hain</t>
+        </is>
+      </c>
+      <c r="D27" s="0" t="inlineStr">
+        <is>
+          <t>Shashwat Sachdev</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="0" t="inlineStr">
+        <is>
+          <t>2026-04-28</t>
+        </is>
+      </c>
+      <c r="B28" s="0" t="n">
+        <v>27</v>
+      </c>
+      <c r="C28" s="0" t="inlineStr">
+        <is>
+          <t>Raanjhan</t>
+        </is>
+      </c>
+      <c r="D28" s="0" t="inlineStr">
+        <is>
+          <t>Sachet-Parampara</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="0" t="inlineStr">
+        <is>
+          <t>2026-04-28</t>
+        </is>
+      </c>
+      <c r="B29" s="0" t="n">
+        <v>28</v>
+      </c>
+      <c r="C29" s="0" t="inlineStr">
+        <is>
+          <t>For A Reason</t>
+        </is>
+      </c>
+      <c r="D29" s="0" t="inlineStr">
+        <is>
+          <t>Karan Aujla</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="0" t="inlineStr">
+        <is>
+          <t>2026-04-28</t>
+        </is>
+      </c>
+      <c r="B30" s="0" t="n">
+        <v>29</v>
+      </c>
+      <c r="C30" s="0" t="inlineStr">
+        <is>
+          <t>Ishqa Ve</t>
+        </is>
+      </c>
+      <c r="D30" s="0" t="inlineStr">
+        <is>
+          <t>Zeeshan Ali</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="0" t="inlineStr">
+        <is>
+          <t>2026-04-28</t>
+        </is>
+      </c>
+      <c r="B31" s="0" t="n">
+        <v>30</v>
+      </c>
+      <c r="C31" s="0" t="inlineStr">
+        <is>
+          <t>Barbaad</t>
+        </is>
+      </c>
+      <c r="D31" s="0" t="inlineStr">
+        <is>
+          <t>The Rish</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="0" t="inlineStr">
+        <is>
+          <t>2026-04-28</t>
+        </is>
+      </c>
+      <c r="B32" s="0" t="n">
+        <v>31</v>
+      </c>
+      <c r="C32" s="0" t="inlineStr">
+        <is>
+          <t>Tere Bina</t>
+        </is>
+      </c>
+      <c r="D32" s="0" t="inlineStr">
+        <is>
+          <t>A.R. Rahman</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="0" t="inlineStr">
+        <is>
+          <t>2026-04-28</t>
+        </is>
+      </c>
+      <c r="B33" s="0" t="n">
+        <v>32</v>
+      </c>
+      <c r="C33" s="0" t="inlineStr">
+        <is>
+          <t>Ehsaas</t>
+        </is>
+      </c>
+      <c r="D33" s="0" t="inlineStr">
+        <is>
+          <t>Faheem Abdullah</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="0" t="inlineStr">
+        <is>
+          <t>2026-04-28</t>
+        </is>
+      </c>
+      <c r="B34" s="0" t="n">
+        <v>33</v>
+      </c>
+      <c r="C34" s="0" t="inlineStr">
+        <is>
+          <t>Agar Tum Saath Ho</t>
+        </is>
+      </c>
+      <c r="D34" s="0" t="inlineStr">
+        <is>
+          <t>Alka Yagnik</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="0" t="inlineStr">
+        <is>
+          <t>2026-04-28</t>
+        </is>
+      </c>
+      <c r="B35" s="0" t="n">
+        <v>34</v>
+      </c>
+      <c r="C35" s="0" t="inlineStr">
+        <is>
+          <t>Dhurandhar - Title Track</t>
+        </is>
+      </c>
+      <c r="D35" s="0" t="inlineStr">
+        <is>
+          <t>Shashwat Sachdev</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="0" t="inlineStr">
+        <is>
+          <t>2026-04-28</t>
+        </is>
+      </c>
+      <c r="B36" s="0" t="n">
+        <v>35</v>
+      </c>
+      <c r="C36" s="0" t="inlineStr">
+        <is>
+          <t>Ye Tune Kya Kiya</t>
+        </is>
+      </c>
+      <c r="D36" s="0" t="inlineStr">
+        <is>
+          <t>Pritam</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="0" t="inlineStr">
+        <is>
+          <t>2026-04-28</t>
+        </is>
+      </c>
+      <c r="B37" s="0" t="n">
+        <v>36</v>
+      </c>
+      <c r="C37" s="0" t="inlineStr">
+        <is>
+          <t>Teri Deewani</t>
+        </is>
+      </c>
+      <c r="D37" s="0" t="inlineStr">
+        <is>
+          <t>Kailash Kher</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="0" t="inlineStr">
+        <is>
+          <t>2026-04-28</t>
+        </is>
+      </c>
+      <c r="B38" s="0" t="n">
+        <v>37</v>
+      </c>
+      <c r="C38" s="0" t="inlineStr">
+        <is>
+          <t>Zaalima</t>
+        </is>
+      </c>
+      <c r="D38" s="0" t="inlineStr">
+        <is>
+          <t>Arijit Singh</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="0" t="inlineStr">
+        <is>
+          <t>2026-04-28</t>
+        </is>
+      </c>
+      <c r="B39" s="0" t="n">
+        <v>38</v>
+      </c>
+      <c r="C39" s="0" t="inlineStr">
+        <is>
+          <t>Naal Nachna</t>
+        </is>
+      </c>
+      <c r="D39" s="0" t="inlineStr">
+        <is>
+          <t>Shashwat Sachdev</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="0" t="inlineStr">
+        <is>
+          <t>2026-04-28</t>
+        </is>
+      </c>
+      <c r="B40" s="0" t="n">
+        <v>39</v>
+      </c>
+      <c r="C40" s="0" t="inlineStr">
+        <is>
+          <t>Bairi</t>
+        </is>
+      </c>
+      <c r="D40" s="0" t="inlineStr">
+        <is>
+          <t>Virat</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" s="0" t="inlineStr">
+        <is>
+          <t>2026-04-28</t>
+        </is>
+      </c>
+      <c r="B41" s="0" t="n">
+        <v>40</v>
+      </c>
+      <c r="C41" s="0" t="inlineStr">
+        <is>
+          <t>Shree Hanuman Chalisa</t>
+        </is>
+      </c>
+      <c r="D41" s="0" t="inlineStr">
+        <is>
+          <t>Hariharan</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" s="0" t="inlineStr">
+        <is>
+          <t>2026-04-28</t>
+        </is>
+      </c>
+      <c r="B42" s="0" t="n">
+        <v>41</v>
+      </c>
+      <c r="C42" s="0" t="inlineStr">
+        <is>
+          <t>Mutta Kalakki</t>
+        </is>
+      </c>
+      <c r="D42" s="0" t="inlineStr">
+        <is>
+          <t>G. V. Prakash</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" s="0" t="inlineStr">
+        <is>
+          <t>2026-04-28</t>
+        </is>
+      </c>
+      <c r="B43" s="0" t="n">
+        <v>42</v>
+      </c>
+      <c r="C43" s="0" t="inlineStr">
+        <is>
+          <t>Phir Se</t>
+        </is>
+      </c>
+      <c r="D43" s="0" t="inlineStr">
+        <is>
+          <t>Shashwat Sachdev</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" s="0" t="inlineStr">
+        <is>
+          <t>2026-04-28</t>
+        </is>
+      </c>
+      <c r="B44" s="0" t="n">
+        <v>43</v>
+      </c>
+      <c r="C44" s="0" t="inlineStr">
+        <is>
+          <t>Mast Magan</t>
+        </is>
+      </c>
+      <c r="D44" s="0" t="inlineStr">
+        <is>
+          <t>Arijit Singh</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" s="0" t="inlineStr">
+        <is>
+          <t>2026-04-28</t>
+        </is>
+      </c>
+      <c r="B45" s="0" t="n">
+        <v>44</v>
+      </c>
+      <c r="C45" s="0" t="inlineStr">
+        <is>
+          <t>Chahun Main Ya Naa</t>
+        </is>
+      </c>
+      <c r="D45" s="0" t="inlineStr">
+        <is>
+          <t>Palak Muchhal</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" s="0" t="inlineStr">
+        <is>
+          <t>2026-04-28</t>
+        </is>
+      </c>
+      <c r="B46" s="0" t="n">
+        <v>45</v>
+      </c>
+      <c r="C46" s="0" t="inlineStr">
+        <is>
+          <t>Eyes on Me</t>
+        </is>
+      </c>
+      <c r="D46" s="0" t="inlineStr">
+        <is>
+          <t>Sidhu Moose Wala</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" s="0" t="inlineStr">
+        <is>
+          <t>2026-04-28</t>
+        </is>
+      </c>
+      <c r="B47" s="0" t="n">
+        <v>46</v>
+      </c>
+      <c r="C47" s="0" t="inlineStr">
+        <is>
+          <t>Mann Mera - Original Version</t>
+        </is>
+      </c>
+      <c r="D47" s="0" t="inlineStr">
+        <is>
+          <t>Gajendra Verma</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" s="0" t="inlineStr">
+        <is>
+          <t>2026-04-28</t>
+        </is>
+      </c>
+      <c r="B48" s="0" t="n">
+        <v>47</v>
+      </c>
+      <c r="C48" s="0" t="inlineStr">
+        <is>
+          <t>Aaya Sher</t>
+        </is>
+      </c>
+      <c r="D48" s="0" t="inlineStr">
+        <is>
+          <t>Anirudh Ravichander</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" s="0" t="inlineStr">
+        <is>
+          <t>2026-04-28</t>
+        </is>
+      </c>
+      <c r="B49" s="0" t="n">
+        <v>48</v>
+      </c>
+      <c r="C49" s="0" t="inlineStr">
+        <is>
+          <t>Haseen</t>
+        </is>
+      </c>
+      <c r="D49" s="0" t="inlineStr">
+        <is>
+          <t>Talwiinder</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" s="0" t="inlineStr">
+        <is>
+          <t>2026-04-28</t>
+        </is>
+      </c>
+      <c r="B50" s="0" t="n">
+        <v>49</v>
+      </c>
+      <c r="C50" s="0" t="inlineStr">
+        <is>
+          <t>High On You</t>
+        </is>
+      </c>
+      <c r="D50" s="0" t="inlineStr">
+        <is>
+          <t>Jind Universe</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" s="0" t="inlineStr">
+        <is>
+          <t>2026-04-28</t>
+        </is>
+      </c>
+      <c r="B51" s="0" t="n">
+        <v>50</v>
+      </c>
+      <c r="C51" s="0" t="inlineStr">
+        <is>
+          <t>Thodi Si Daaru</t>
+        </is>
+      </c>
+      <c r="D51" s="0" t="inlineStr">
+        <is>
+          <t>AP Dhillon</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet46.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:D51"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="24" t="inlineStr">
+        <is>
+          <t>Date</t>
+        </is>
+      </c>
+      <c r="B1" s="24" t="inlineStr">
+        <is>
+          <t>Rank</t>
+        </is>
+      </c>
+      <c r="C1" s="24" t="inlineStr">
+        <is>
+          <t>Song</t>
+        </is>
+      </c>
+      <c r="D1" s="24" t="inlineStr">
+        <is>
+          <t>Artist</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>2026-04-25</t>
+          <t>2026-04-27</t>
         </is>
       </c>
       <c r="B2" t="n">
@@ -40941,7 +43015,7 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>2026-04-25</t>
+          <t>2026-04-27</t>
         </is>
       </c>
       <c r="B3" t="n">
@@ -40949,19 +43023,19 @@
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>Gehra Hua</t>
+          <t>Majboor</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>Shashwat Sachdev</t>
+          <t>Sheheryar Rehan</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>2026-04-25</t>
+          <t>2026-04-27</t>
         </is>
       </c>
       <c r="B4" t="n">
@@ -40969,19 +43043,19 @@
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>Majboor</t>
+          <t>Gehra Hua</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>Sheheryar Rehan</t>
+          <t>Shashwat Sachdev</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>2026-04-25</t>
+          <t>2026-04-27</t>
         </is>
       </c>
       <c r="B5" t="n">
@@ -41001,7 +43075,7 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>2026-04-25</t>
+          <t>2026-04-27</t>
         </is>
       </c>
       <c r="B6" t="n">
@@ -41021,7 +43095,7 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>2026-04-25</t>
+          <t>2026-04-27</t>
         </is>
       </c>
       <c r="B7" t="n">
@@ -41041,7 +43115,7 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>2026-04-25</t>
+          <t>2026-04-27</t>
         </is>
       </c>
       <c r="B8" t="n">
@@ -41061,7 +43135,7 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>2026-04-25</t>
+          <t>2026-04-27</t>
         </is>
       </c>
       <c r="B9" t="n">
@@ -41081,7 +43155,7 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>2026-04-25</t>
+          <t>2026-04-27</t>
         </is>
       </c>
       <c r="B10" t="n">
@@ -41101,7 +43175,7 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>2026-04-25</t>
+          <t>2026-04-27</t>
         </is>
       </c>
       <c r="B11" t="n">
@@ -41121,7 +43195,7 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>2026-04-25</t>
+          <t>2026-04-27</t>
         </is>
       </c>
       <c r="B12" t="n">
@@ -41141,7 +43215,7 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>2026-04-25</t>
+          <t>2026-04-27</t>
         </is>
       </c>
       <c r="B13" t="n">
@@ -41149,19 +43223,19 @@
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>Dooron Dooron</t>
+          <t>Apna Bana Le</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>Paresh Pahuja</t>
+          <t>Sachin-Jigar</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>2026-04-25</t>
+          <t>2026-04-27</t>
         </is>
       </c>
       <c r="B14" t="n">
@@ -41169,19 +43243,19 @@
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>Apna Bana Le</t>
+          <t>Dooron Dooron</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>Sachin-Jigar</t>
+          <t>Paresh Pahuja</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>2026-04-25</t>
+          <t>2026-04-27</t>
         </is>
       </c>
       <c r="B15" t="n">
@@ -41201,7 +43275,7 @@
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>2026-04-25</t>
+          <t>2026-04-27</t>
         </is>
       </c>
       <c r="B16" t="n">
@@ -41221,7 +43295,7 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>2026-04-25</t>
+          <t>2026-04-27</t>
         </is>
       </c>
       <c r="B17" t="n">
@@ -41229,19 +43303,19 @@
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>Shararat</t>
+          <t>Tum Ho Toh</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>Shashwat Sachdev</t>
+          <t>Vishal Mishra</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>2026-04-25</t>
+          <t>2026-04-27</t>
         </is>
       </c>
       <c r="B18" t="n">
@@ -41249,19 +43323,19 @@
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>Boyfriend</t>
+          <t>Ishq</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>Karan Aujla</t>
+          <t>Faheem Abdullah</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>2026-04-25</t>
+          <t>2026-04-27</t>
         </is>
       </c>
       <c r="B19" t="n">
@@ -41269,19 +43343,19 @@
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>Ishq</t>
+          <t>Boyfriend</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>Faheem Abdullah</t>
+          <t>Karan Aujla</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>2026-04-25</t>
+          <t>2026-04-27</t>
         </is>
       </c>
       <c r="B20" t="n">
@@ -41289,7 +43363,7 @@
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>Dhurandhar The Revenge - Aari Aari</t>
+          <t>Shararat</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
@@ -41301,7 +43375,7 @@
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>2026-04-25</t>
+          <t>2026-04-27</t>
         </is>
       </c>
       <c r="B21" t="n">
@@ -41309,19 +43383,19 @@
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>Tum Ho Toh</t>
+          <t>Deewaana Deewaana</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>Vishal Mishra</t>
+          <t>A.R. Rahman</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>2026-04-25</t>
+          <t>2026-04-27</t>
         </is>
       </c>
       <c r="B22" t="n">
@@ -41329,19 +43403,19 @@
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>Saiyaara</t>
+          <t>Dhurandhar The Revenge - Aari Aari</t>
         </is>
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>Tanishk Bagchi</t>
+          <t>Shashwat Sachdev</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>2026-04-25</t>
+          <t>2026-04-27</t>
         </is>
       </c>
       <c r="B23" t="n">
@@ -41349,19 +43423,19 @@
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>Jaan Se Guzarte Hain</t>
+          <t>Saiyaara</t>
         </is>
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>Shashwat Sachdev</t>
+          <t>Tanishk Bagchi</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>2026-04-25</t>
+          <t>2026-04-27</t>
         </is>
       </c>
       <c r="B24" t="n">
@@ -41369,19 +43443,19 @@
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>Raanjhan</t>
+          <t>Darkhaast</t>
         </is>
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>Sachet-Parampara</t>
+          <t>Mithoon</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>2026-04-25</t>
+          <t>2026-04-27</t>
         </is>
       </c>
       <c r="B25" t="n">
@@ -41389,19 +43463,19 @@
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>Darkhaast</t>
+          <t>Raanjhan</t>
         </is>
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>Mithoon</t>
+          <t>Sachet-Parampara</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>2026-04-25</t>
+          <t>2026-04-27</t>
         </is>
       </c>
       <c r="B26" t="n">
@@ -41409,19 +43483,19 @@
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>Deewaana Deewaana</t>
+          <t>Jo Tum Mere Ho</t>
         </is>
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>A.R. Rahman</t>
+          <t>Anuv Jain</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>2026-04-25</t>
+          <t>2026-04-27</t>
         </is>
       </c>
       <c r="B27" t="n">
@@ -41429,19 +43503,19 @@
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>For A Reason</t>
+          <t>Jaan Se Guzarte Hain</t>
         </is>
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t>Karan Aujla</t>
+          <t>Shashwat Sachdev</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>2026-04-25</t>
+          <t>2026-04-27</t>
         </is>
       </c>
       <c r="B28" t="n">
@@ -41461,7 +43535,7 @@
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>2026-04-25</t>
+          <t>2026-04-27</t>
         </is>
       </c>
       <c r="B29" t="n">
@@ -41469,19 +43543,19 @@
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>Ishqa Ve</t>
+          <t>For A Reason</t>
         </is>
       </c>
       <c r="D29" t="inlineStr">
         <is>
-          <t>Zeeshan Ali</t>
+          <t>Karan Aujla</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>2026-04-25</t>
+          <t>2026-04-27</t>
         </is>
       </c>
       <c r="B30" t="n">
@@ -41489,19 +43563,19 @@
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>Dhurandhar - Title Track</t>
+          <t>Barbaad</t>
         </is>
       </c>
       <c r="D30" t="inlineStr">
         <is>
-          <t>Shashwat Sachdev</t>
+          <t>The Rish</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>2026-04-25</t>
+          <t>2026-04-27</t>
         </is>
       </c>
       <c r="B31" t="n">
@@ -41509,19 +43583,19 @@
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>Agar Tum Saath Ho</t>
+          <t>Tere Bina</t>
         </is>
       </c>
       <c r="D31" t="inlineStr">
         <is>
-          <t>Alka Yagnik</t>
+          <t>A.R. Rahman</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>2026-04-25</t>
+          <t>2026-04-27</t>
         </is>
       </c>
       <c r="B32" t="n">
@@ -41529,19 +43603,19 @@
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>Ehsaas</t>
+          <t>Ishqa Ve</t>
         </is>
       </c>
       <c r="D32" t="inlineStr">
         <is>
-          <t>Faheem Abdullah</t>
+          <t>Zeeshan Ali</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>2026-04-25</t>
+          <t>2026-04-27</t>
         </is>
       </c>
       <c r="B33" t="n">
@@ -41549,19 +43623,19 @@
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>Jo Tum Mere Ho</t>
+          <t>Agar Tum Saath Ho</t>
         </is>
       </c>
       <c r="D33" t="inlineStr">
         <is>
-          <t>Anuv Jain</t>
+          <t>Alka Yagnik</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>2026-04-25</t>
+          <t>2026-04-27</t>
         </is>
       </c>
       <c r="B34" t="n">
@@ -41569,19 +43643,19 @@
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>Tere Bina</t>
+          <t>Ehsaas</t>
         </is>
       </c>
       <c r="D34" t="inlineStr">
         <is>
-          <t>A.R. Rahman</t>
+          <t>Faheem Abdullah</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>2026-04-25</t>
+          <t>2026-04-27</t>
         </is>
       </c>
       <c r="B35" t="n">
@@ -41589,19 +43663,19 @@
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>Ye Tune Kya Kiya</t>
+          <t>Dhurandhar - Title Track</t>
         </is>
       </c>
       <c r="D35" t="inlineStr">
         <is>
-          <t>Pritam</t>
+          <t>Shashwat Sachdev</t>
         </is>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>2026-04-25</t>
+          <t>2026-04-27</t>
         </is>
       </c>
       <c r="B36" t="n">
@@ -41609,19 +43683,19 @@
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>Naal Nachna</t>
+          <t>Ye Tune Kya Kiya</t>
         </is>
       </c>
       <c r="D36" t="inlineStr">
         <is>
-          <t>Shashwat Sachdev</t>
+          <t>Pritam</t>
         </is>
       </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>2026-04-25</t>
+          <t>2026-04-27</t>
         </is>
       </c>
       <c r="B37" t="n">
@@ -41629,19 +43703,19 @@
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>Barbaad</t>
+          <t>Zaalima</t>
         </is>
       </c>
       <c r="D37" t="inlineStr">
         <is>
-          <t>The Rish</t>
+          <t>Arijit Singh</t>
         </is>
       </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>2026-04-25</t>
+          <t>2026-04-27</t>
         </is>
       </c>
       <c r="B38" t="n">
@@ -41649,19 +43723,19 @@
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>Bairi</t>
+          <t>Naal Nachna</t>
         </is>
       </c>
       <c r="D38" t="inlineStr">
         <is>
-          <t>Virat</t>
+          <t>Shashwat Sachdev</t>
         </is>
       </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>2026-04-25</t>
+          <t>2026-04-27</t>
         </is>
       </c>
       <c r="B39" t="n">
@@ -41669,19 +43743,19 @@
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>Mutta Kalakki</t>
+          <t>Teri Deewani</t>
         </is>
       </c>
       <c r="D39" t="inlineStr">
         <is>
-          <t>G. V. Prakash</t>
+          <t>Kailash Kher</t>
         </is>
       </c>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>2026-04-25</t>
+          <t>2026-04-27</t>
         </is>
       </c>
       <c r="B40" t="n">
@@ -41689,19 +43763,19 @@
       </c>
       <c r="C40" t="inlineStr">
         <is>
-          <t>Teri Deewani</t>
+          <t>Bairi</t>
         </is>
       </c>
       <c r="D40" t="inlineStr">
         <is>
-          <t>Kailash Kher</t>
+          <t>Virat</t>
         </is>
       </c>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>2026-04-25</t>
+          <t>2026-04-27</t>
         </is>
       </c>
       <c r="B41" t="n">
@@ -41709,19 +43783,19 @@
       </c>
       <c r="C41" t="inlineStr">
         <is>
-          <t>Phir Se</t>
+          <t>Mutta Kalakki</t>
         </is>
       </c>
       <c r="D41" t="inlineStr">
         <is>
-          <t>Shashwat Sachdev</t>
+          <t>G. V. Prakash</t>
         </is>
       </c>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>2026-04-25</t>
+          <t>2026-04-27</t>
         </is>
       </c>
       <c r="B42" t="n">
@@ -41729,7 +43803,7 @@
       </c>
       <c r="C42" t="inlineStr">
         <is>
-          <t>Lutt Le Gaya</t>
+          <t>Phir Se</t>
         </is>
       </c>
       <c r="D42" t="inlineStr">
@@ -41741,7 +43815,7 @@
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>2026-04-25</t>
+          <t>2026-04-27</t>
         </is>
       </c>
       <c r="B43" t="n">
@@ -41761,7 +43835,7 @@
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>2026-04-25</t>
+          <t>2026-04-27</t>
         </is>
       </c>
       <c r="B44" t="n">
@@ -41781,7 +43855,7 @@
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>2026-04-25</t>
+          <t>2026-04-27</t>
         </is>
       </c>
       <c r="B45" t="n">
@@ -41789,19 +43863,19 @@
       </c>
       <c r="C45" t="inlineStr">
         <is>
-          <t>High On You</t>
+          <t>Mast Magan</t>
         </is>
       </c>
       <c r="D45" t="inlineStr">
         <is>
-          <t>Jind Universe</t>
+          <t>Arijit Singh</t>
         </is>
       </c>
     </row>
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>2026-04-25</t>
+          <t>2026-04-27</t>
         </is>
       </c>
       <c r="B46" t="n">
@@ -41809,19 +43883,19 @@
       </c>
       <c r="C46" t="inlineStr">
         <is>
-          <t>Mast Magan</t>
+          <t>Jhol - Acoustic</t>
         </is>
       </c>
       <c r="D46" t="inlineStr">
         <is>
-          <t>Arijit Singh</t>
+          <t>Maanu</t>
         </is>
       </c>
     </row>
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>2026-04-25</t>
+          <t>2026-04-27</t>
         </is>
       </c>
       <c r="B47" t="n">
@@ -41829,19 +43903,19 @@
       </c>
       <c r="C47" t="inlineStr">
         <is>
-          <t>Mann Mera - Original Version</t>
+          <t>Chahun Main Ya Naa</t>
         </is>
       </c>
       <c r="D47" t="inlineStr">
         <is>
-          <t>Gajendra Verma</t>
+          <t>Palak Muchhal</t>
         </is>
       </c>
     </row>
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>2026-04-25</t>
+          <t>2026-04-27</t>
         </is>
       </c>
       <c r="B48" t="n">
@@ -41849,19 +43923,19 @@
       </c>
       <c r="C48" t="inlineStr">
         <is>
-          <t>Oorum Blood</t>
+          <t>Thodi Si Daaru</t>
         </is>
       </c>
       <c r="D48" t="inlineStr">
         <is>
-          <t>Sai Abhyankkar</t>
+          <t>AP Dhillon</t>
         </is>
       </c>
     </row>
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>2026-04-25</t>
+          <t>2026-04-27</t>
         </is>
       </c>
       <c r="B49" t="n">
@@ -41869,19 +43943,19 @@
       </c>
       <c r="C49" t="inlineStr">
         <is>
-          <t>Jhol - Acoustic</t>
+          <t>Mann Mera - Original Version</t>
         </is>
       </c>
       <c r="D49" t="inlineStr">
         <is>
-          <t>Maanu</t>
+          <t>Gajendra Verma</t>
         </is>
       </c>
     </row>
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>2026-04-25</t>
+          <t>2026-04-27</t>
         </is>
       </c>
       <c r="B50" t="n">
@@ -41889,19 +43963,19 @@
       </c>
       <c r="C50" t="inlineStr">
         <is>
-          <t>Thodi Si Daaru</t>
+          <t>Humsafar</t>
         </is>
       </c>
       <c r="D50" t="inlineStr">
         <is>
-          <t>AP Dhillon</t>
+          <t>Sachet-Parampara</t>
         </is>
       </c>
     </row>
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>2026-04-25</t>
+          <t>2026-04-27</t>
         </is>
       </c>
       <c r="B51" t="n">
@@ -41909,7 +43983,7 @@
       </c>
       <c r="C51" t="inlineStr">
         <is>
-          <t>Zaalima</t>
+          <t>Tum Hi Ho</t>
         </is>
       </c>
       <c r="D51" t="inlineStr">

</xml_diff>